<commit_message>
auto: anime list update 2026-05-03
</commit_message>
<xml_diff>
--- a/data/anime_list.xlsx
+++ b/data/anime_list.xlsx
@@ -18,16 +18,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -38,7 +35,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -46,21 +43,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -430,67 +418,67 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>season_id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>season_label</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>order</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>title</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>is_rerun</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>broadcast_format</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>broadcast_start</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>animation_studio</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>op_title</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>op_artist</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>ed_title</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>ed_artist</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>detail_url</t>
         </is>
@@ -6163,62 +6151,62 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>season_id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>season_label</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>anime_title</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>is_rerun</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>kind</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>index</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>song_title</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>artist</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>youtube_url</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>youtube_views</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>youtube_channel</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>last_searched_at</t>
         </is>

</xml_diff>

<commit_message>
data: full youtube search for 2026春 (124/161 hits, master_video +115)
</commit_message>
<xml_diff>
--- a/data/anime_list.xlsx
+++ b/data/anime_list.xlsx
@@ -18,13 +18,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -35,7 +38,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -43,12 +46,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -418,67 +430,67 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>season_id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>season_label</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>order</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>title</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>is_rerun</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>broadcast_format</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>broadcast_start</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>animation_studio</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>op_title</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>op_artist</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>ed_title</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>ed_artist</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>detail_url</t>
         </is>
@@ -6151,62 +6163,62 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>season_id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>season_label</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>anime_title</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>is_rerun</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>kind</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>index</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>song_title</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>artist</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>youtube_url</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>youtube_views</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>youtube_channel</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>last_searched_at</t>
         </is>
@@ -7223,10 +7235,24 @@
         </is>
       </c>
       <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
-      <c r="L23" t="inlineStr"/>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=kh1PwoEsIf8</t>
+        </is>
+      </c>
+      <c r="J23" t="n">
+        <v>6842</v>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>おジャ魔女どれみ公式チャンネル</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:03:45</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -7263,10 +7289,24 @@
           <t>i-dle</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr"/>
-      <c r="L24" t="inlineStr"/>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=JCDGaA2sfi0</t>
+        </is>
+      </c>
+      <c r="J24" t="n">
+        <v>1260189</v>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>オタクに優しいギャルはいない!?</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:03:58</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -7303,10 +7343,24 @@
           <t>三四少女</t>
         </is>
       </c>
-      <c r="I25" t="inlineStr"/>
-      <c r="J25" t="inlineStr"/>
-      <c r="K25" t="inlineStr"/>
-      <c r="L25" t="inlineStr"/>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=JCDGaA2sfi0</t>
+        </is>
+      </c>
+      <c r="J25" t="n">
+        <v>1260189</v>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>オタクに優しいギャルはいない!?</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:04:11</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -7343,10 +7397,24 @@
           <t>子ザメちゃん(CV：花澤香菜)</t>
         </is>
       </c>
-      <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr"/>
-      <c r="L26" t="inlineStr"/>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=Laf46YXDt68</t>
+        </is>
+      </c>
+      <c r="J26" t="n">
+        <v>874040</v>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>アニメ『おでかけ子ザメ』チャンネル</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:04:24</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -7383,10 +7451,24 @@
           <t>オーイシマサヨシ</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr"/>
-      <c r="L27" t="inlineStr"/>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=8Gtb1uhjPKs</t>
+        </is>
+      </c>
+      <c r="J27" t="n">
+        <v>1174964</v>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>TOHO animation</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:04:38</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -7423,10 +7505,24 @@
           <t>おねがいかなえ隊</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr"/>
-      <c r="L28" t="inlineStr"/>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=j1J45v_al9s</t>
+        </is>
+      </c>
+      <c r="J28" t="n">
+        <v>140</v>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>真一チャンネル</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:04:51</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -7463,10 +7559,24 @@
           <t>いぎなり東北産</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr"/>
-      <c r="K29" t="inlineStr"/>
-      <c r="L29" t="inlineStr"/>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=bH8Ukl9BM0s</t>
+        </is>
+      </c>
+      <c r="J29" t="n">
+        <v>41469</v>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>【公式】アイプリちゅ〜ぶ</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:05:05</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -7503,10 +7613,24 @@
           <t>JAM Project</t>
         </is>
       </c>
-      <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr"/>
-      <c r="K30" t="inlineStr"/>
-      <c r="L30" t="inlineStr"/>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=1d_YJXQZUgQ</t>
+        </is>
+      </c>
+      <c r="J30" t="n">
+        <v>487771</v>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>ヴァンガードチャンネル【アニメ「Divinez 幻真星戦編」配信中!!】</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:05:13</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -7543,10 +7667,24 @@
           <t>JAM Project</t>
         </is>
       </c>
-      <c r="I31" t="inlineStr"/>
-      <c r="J31" t="inlineStr"/>
-      <c r="K31" t="inlineStr"/>
-      <c r="L31" t="inlineStr"/>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=1d_YJXQZUgQ</t>
+        </is>
+      </c>
+      <c r="J31" t="n">
+        <v>487771</v>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>ヴァンガードチャンネル【アニメ「Divinez 幻真星戦編」配信中!!】</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:05:20</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -7863,10 +8001,24 @@
           <t>Faulieu.</t>
         </is>
       </c>
-      <c r="I39" t="inlineStr"/>
-      <c r="J39" t="inlineStr"/>
-      <c r="K39" t="inlineStr"/>
-      <c r="L39" t="inlineStr"/>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=SGtyPSZqb5s</t>
+        </is>
+      </c>
+      <c r="J39" t="n">
+        <v>335542</v>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>Faulieu.</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:05:49</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -7903,10 +8055,24 @@
           <t>あおぎり高校</t>
         </is>
       </c>
-      <c r="I40" t="inlineStr"/>
-      <c r="J40" t="inlineStr"/>
-      <c r="K40" t="inlineStr"/>
-      <c r="L40" t="inlineStr"/>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=mHQi_a9MjkA</t>
+        </is>
+      </c>
+      <c r="J40" t="n">
+        <v>231842</v>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>あおぎり高校 - Aogiri Vtuber High School</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:06:02</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -7943,10 +8109,24 @@
           <t>雨宮天</t>
         </is>
       </c>
-      <c r="I41" t="inlineStr"/>
-      <c r="J41" t="inlineStr"/>
-      <c r="K41" t="inlineStr"/>
-      <c r="L41" t="inlineStr"/>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=R7u3ISKPujU</t>
+        </is>
+      </c>
+      <c r="J41" t="n">
+        <v>96474</v>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>雨宮天公式YouTubeチャンネル</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:06:15</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -8103,10 +8283,24 @@
           <t>yonige</t>
         </is>
       </c>
-      <c r="I45" t="inlineStr"/>
-      <c r="J45" t="inlineStr"/>
-      <c r="K45" t="inlineStr"/>
-      <c r="L45" t="inlineStr"/>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=XX90FklAWsc</t>
+        </is>
+      </c>
+      <c r="J45" t="n">
+        <v>151203</v>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>アニプレックス チャンネル</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:06:40</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -8139,10 +8333,24 @@
         </is>
       </c>
       <c r="H46" t="inlineStr"/>
-      <c r="I46" t="inlineStr"/>
-      <c r="J46" t="inlineStr"/>
-      <c r="K46" t="inlineStr"/>
-      <c r="L46" t="inlineStr"/>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=JEiHCjhKRYw</t>
+        </is>
+      </c>
+      <c r="J46" t="n">
+        <v>66168</v>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>アニプレックス チャンネル</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:06:53</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -8179,10 +8387,24 @@
           <t>HOKUTO</t>
         </is>
       </c>
-      <c r="I47" t="inlineStr"/>
-      <c r="J47" t="inlineStr"/>
-      <c r="K47" t="inlineStr"/>
-      <c r="L47" t="inlineStr"/>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=yxccM_weehk</t>
+        </is>
+      </c>
+      <c r="J47" t="n">
+        <v>135172</v>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>HOKUTO</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:07:06</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -8219,10 +8441,24 @@
           <t>内田真礼</t>
         </is>
       </c>
-      <c r="I48" t="inlineStr"/>
-      <c r="J48" t="inlineStr"/>
-      <c r="K48" t="inlineStr"/>
-      <c r="L48" t="inlineStr"/>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=Oz5EkYVJbBc</t>
+        </is>
+      </c>
+      <c r="J48" t="n">
+        <v>72088</v>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>アニメ『神の雫』official YouTube channel</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:07:19</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -8259,10 +8495,24 @@
           <t>入野自由</t>
         </is>
       </c>
-      <c r="I49" t="inlineStr"/>
-      <c r="J49" t="inlineStr"/>
-      <c r="K49" t="inlineStr"/>
-      <c r="L49" t="inlineStr"/>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=JMqsT9cPh1c</t>
+        </is>
+      </c>
+      <c r="J49" t="n">
+        <v>189836</v>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:07:31</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -8299,10 +8549,24 @@
           <t>JYOCHO</t>
         </is>
       </c>
-      <c r="I50" t="inlineStr"/>
-      <c r="J50" t="inlineStr"/>
-      <c r="K50" t="inlineStr"/>
-      <c r="L50" t="inlineStr"/>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=aDHno6PB5pM</t>
+        </is>
+      </c>
+      <c r="J50" t="n">
+        <v>20887</v>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>JYOCHO</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:07:43</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -8339,10 +8603,24 @@
           <t>岡村靖幸・中島健人</t>
         </is>
       </c>
-      <c r="I51" t="inlineStr"/>
-      <c r="J51" t="inlineStr"/>
-      <c r="K51" t="inlineStr"/>
-      <c r="L51" t="inlineStr"/>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=JNbh6RTyOaE</t>
+        </is>
+      </c>
+      <c r="J51" t="n">
+        <v>429432</v>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>アニプレックス チャンネル</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:07:55</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -8459,10 +8737,24 @@
           <t>IS:SUE</t>
         </is>
       </c>
-      <c r="I54" t="inlineStr"/>
-      <c r="J54" t="inlineStr"/>
-      <c r="K54" t="inlineStr"/>
-      <c r="L54" t="inlineStr"/>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=wM3E9LXHmu0</t>
+        </is>
+      </c>
+      <c r="J54" t="n">
+        <v>2689740</v>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>TVアニメ「キャンディーカリエス」</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:08:09</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -8499,10 +8791,24 @@
           <t>スカートとODD Foot Works</t>
         </is>
       </c>
-      <c r="I55" t="inlineStr"/>
-      <c r="J55" t="inlineStr"/>
-      <c r="K55" t="inlineStr"/>
-      <c r="L55" t="inlineStr"/>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=u5syUWK5d-8</t>
+        </is>
+      </c>
+      <c r="J55" t="n">
+        <v>58027</v>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>ぽにきゃん-Anime PONY CANYON</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:08:22</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -8539,10 +8845,24 @@
           <t>a子</t>
         </is>
       </c>
-      <c r="I56" t="inlineStr"/>
-      <c r="J56" t="inlineStr"/>
-      <c r="K56" t="inlineStr"/>
-      <c r="L56" t="inlineStr"/>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=n3c6bAOhVUg</t>
+        </is>
+      </c>
+      <c r="J56" t="n">
+        <v>464180</v>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>ぽにきゃん-Anime PONY CANYON</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:08:34</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -8579,10 +8899,24 @@
           <t>aespa</t>
         </is>
       </c>
-      <c r="I57" t="inlineStr"/>
-      <c r="J57" t="inlineStr"/>
-      <c r="K57" t="inlineStr"/>
-      <c r="L57" t="inlineStr"/>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=nMwSsHkjmfk</t>
+        </is>
+      </c>
+      <c r="J57" t="n">
+        <v>2326192</v>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>aespa</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:08:48</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -8619,10 +8953,24 @@
           <t>RIIZE</t>
         </is>
       </c>
-      <c r="I58" t="inlineStr"/>
-      <c r="J58" t="inlineStr"/>
-      <c r="K58" t="inlineStr"/>
-      <c r="L58" t="inlineStr"/>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=sfVO4X_xOu8</t>
+        </is>
+      </c>
+      <c r="J58" t="n">
+        <v>259210</v>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>RIIZE</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:09:00</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -8659,10 +9007,24 @@
           <t>Galileo Galilei</t>
         </is>
       </c>
-      <c r="I59" t="inlineStr"/>
-      <c r="J59" t="inlineStr"/>
-      <c r="K59" t="inlineStr"/>
-      <c r="L59" t="inlineStr"/>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=7ETgAcnUcro</t>
+        </is>
+      </c>
+      <c r="J59" t="n">
+        <v>51435</v>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>Galileo Galilei Official</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:09:13</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -8739,10 +9101,24 @@
           <t>reGretGirl</t>
         </is>
       </c>
-      <c r="I61" t="inlineStr"/>
-      <c r="J61" t="inlineStr"/>
-      <c r="K61" t="inlineStr"/>
-      <c r="L61" t="inlineStr"/>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=2hyWBr4hceY</t>
+        </is>
+      </c>
+      <c r="J61" t="n">
+        <v>207642</v>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>reGretGirl</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:09:37</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -8819,10 +9195,24 @@
           <t>ASCA</t>
         </is>
       </c>
-      <c r="I63" t="inlineStr"/>
-      <c r="J63" t="inlineStr"/>
-      <c r="K63" t="inlineStr"/>
-      <c r="L63" t="inlineStr"/>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=ATTWunJa4yc</t>
+        </is>
+      </c>
+      <c r="J63" t="n">
+        <v>36805</v>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>GOOD SMILE CHANNEL</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:10:02</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -8859,10 +9249,24 @@
           <t>スピラ・スピカ</t>
         </is>
       </c>
-      <c r="I64" t="inlineStr"/>
-      <c r="J64" t="inlineStr"/>
-      <c r="K64" t="inlineStr"/>
-      <c r="L64" t="inlineStr"/>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=L7t4Jsq51LE</t>
+        </is>
+      </c>
+      <c r="J64" t="n">
+        <v>24437</v>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">spira spica Official YouTube Channel (SMEJ) </t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:10:10</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -8899,10 +9303,24 @@
           <t>相葉芹亜（CV.藤寺美徳）</t>
         </is>
       </c>
-      <c r="I65" t="inlineStr"/>
-      <c r="J65" t="inlineStr"/>
-      <c r="K65" t="inlineStr"/>
-      <c r="L65" t="inlineStr"/>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=uN6qJzuCFtw</t>
+        </is>
+      </c>
+      <c r="J65" t="n">
+        <v>32753</v>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:10:23</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -8939,10 +9357,24 @@
           <t>オデッセウス（CV.寿美菜子）</t>
         </is>
       </c>
-      <c r="I66" t="inlineStr"/>
-      <c r="J66" t="inlineStr"/>
-      <c r="K66" t="inlineStr"/>
-      <c r="L66" t="inlineStr"/>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=KygwMir5i_U</t>
+        </is>
+      </c>
+      <c r="J66" t="n">
+        <v>10658</v>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:10:33</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -8979,10 +9411,24 @@
           <t>Novelbright</t>
         </is>
       </c>
-      <c r="I67" t="inlineStr"/>
-      <c r="J67" t="inlineStr"/>
-      <c r="K67" t="inlineStr"/>
-      <c r="L67" t="inlineStr"/>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=SAtVrwS86pE</t>
+        </is>
+      </c>
+      <c r="J67" t="n">
+        <v>2440838</v>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>Novelbright</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:10:46</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -9019,10 +9465,24 @@
           <t>ポルカドットスティングレイ</t>
         </is>
       </c>
-      <c r="I68" t="inlineStr"/>
-      <c r="J68" t="inlineStr"/>
-      <c r="K68" t="inlineStr"/>
-      <c r="L68" t="inlineStr"/>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=5ggfKnnQ-0Q</t>
+        </is>
+      </c>
+      <c r="J68" t="n">
+        <v>167421</v>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>TBSアニメ</t>
+        </is>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:10:59</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -9099,10 +9559,24 @@
           <t>22/7</t>
         </is>
       </c>
-      <c r="I70" t="inlineStr"/>
-      <c r="J70" t="inlineStr"/>
-      <c r="K70" t="inlineStr"/>
-      <c r="L70" t="inlineStr"/>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=gaPA7q3nd58</t>
+        </is>
+      </c>
+      <c r="J70" t="n">
+        <v>40260</v>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>22/7 OFFICIAL YouTube CHANNEL</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:11:22</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -9139,10 +9613,24 @@
           <t>緑仙</t>
         </is>
       </c>
-      <c r="I71" t="inlineStr"/>
-      <c r="J71" t="inlineStr"/>
-      <c r="K71" t="inlineStr"/>
-      <c r="L71" t="inlineStr"/>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=rm86UwJz8Ck</t>
+        </is>
+      </c>
+      <c r="J71" t="n">
+        <v>21883</v>
+      </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>NBCUniversal Anime/Music</t>
+        </is>
+      </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:11:35</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -9179,10 +9667,24 @@
           <t>ファントムシータ</t>
         </is>
       </c>
-      <c r="I72" t="inlineStr"/>
-      <c r="J72" t="inlineStr"/>
-      <c r="K72" t="inlineStr"/>
-      <c r="L72" t="inlineStr"/>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=WHkoz2tsc2s</t>
+        </is>
+      </c>
+      <c r="J72" t="n">
+        <v>3256</v>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>Yamashita Gakuen Anime Song Club</t>
+        </is>
+      </c>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:11:46</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -9219,10 +9721,24 @@
           <t>宮川愛李</t>
         </is>
       </c>
-      <c r="I73" t="inlineStr"/>
-      <c r="J73" t="inlineStr"/>
-      <c r="K73" t="inlineStr"/>
-      <c r="L73" t="inlineStr"/>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=zxS6lFQHiUc</t>
+        </is>
+      </c>
+      <c r="J73" t="n">
+        <v>112725</v>
+      </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>アルファポリス公式</t>
+        </is>
+      </c>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:11:59</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -9259,10 +9775,24 @@
           <t>RLOEVO</t>
         </is>
       </c>
-      <c r="I74" t="inlineStr"/>
-      <c r="J74" t="inlineStr"/>
-      <c r="K74" t="inlineStr"/>
-      <c r="L74" t="inlineStr"/>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=l0FE1UDC58U</t>
+        </is>
+      </c>
+      <c r="J74" t="n">
+        <v>271591</v>
+      </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>RLOEVO</t>
+        </is>
+      </c>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:12:10</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -9299,10 +9829,24 @@
           <t>ビバラッシュ</t>
         </is>
       </c>
-      <c r="I75" t="inlineStr"/>
-      <c r="J75" t="inlineStr"/>
-      <c r="K75" t="inlineStr"/>
-      <c r="L75" t="inlineStr"/>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=48pc58upFY4</t>
+        </is>
+      </c>
+      <c r="J75" t="n">
+        <v>21943</v>
+      </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>アニメ「自動販売機に生まれ変わった俺は迷宮を彷徨う」公式</t>
+        </is>
+      </c>
+      <c r="L75" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:12:21</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -9339,10 +9883,24 @@
           <t>FUWAMOCO</t>
         </is>
       </c>
-      <c r="I76" t="inlineStr"/>
-      <c r="J76" t="inlineStr"/>
-      <c r="K76" t="inlineStr"/>
-      <c r="L76" t="inlineStr"/>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=vSwxof0K8lk</t>
+        </is>
+      </c>
+      <c r="J76" t="n">
+        <v>274345</v>
+      </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>FUWAMOCO Ch. hololive-EN</t>
+        </is>
+      </c>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:12:33</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -9379,10 +9937,24 @@
           <t>GLAY</t>
         </is>
       </c>
-      <c r="I77" t="inlineStr"/>
-      <c r="J77" t="inlineStr"/>
-      <c r="K77" t="inlineStr"/>
-      <c r="L77" t="inlineStr"/>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=CqeuOBy-09U</t>
+        </is>
+      </c>
+      <c r="J77" t="n">
+        <v>2564203</v>
+      </c>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>GLAY</t>
+        </is>
+      </c>
+      <c r="L77" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:12:47</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -9419,10 +9991,24 @@
           <t>早見沙織</t>
         </is>
       </c>
-      <c r="I78" t="inlineStr"/>
-      <c r="J78" t="inlineStr"/>
-      <c r="K78" t="inlineStr"/>
-      <c r="L78" t="inlineStr"/>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=i8xvsTsbFfM</t>
+        </is>
+      </c>
+      <c r="J78" t="n">
+        <v>13560</v>
+      </c>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>早見沙織 Official YouTube Channel</t>
+        </is>
+      </c>
+      <c r="L78" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:13:00</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -9459,10 +10045,24 @@
           <t>Orangestar</t>
         </is>
       </c>
-      <c r="I79" t="inlineStr"/>
-      <c r="J79" t="inlineStr"/>
-      <c r="K79" t="inlineStr"/>
-      <c r="L79" t="inlineStr"/>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=WDeVDNg6lSE</t>
+        </is>
+      </c>
+      <c r="J79" t="n">
+        <v>875036</v>
+      </c>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>Orangestar</t>
+        </is>
+      </c>
+      <c r="L79" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:13:13</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -9499,10 +10099,24 @@
           <t>Orangestar</t>
         </is>
       </c>
-      <c r="I80" t="inlineStr"/>
-      <c r="J80" t="inlineStr"/>
-      <c r="K80" t="inlineStr"/>
-      <c r="L80" t="inlineStr"/>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=WDeVDNg6lSE</t>
+        </is>
+      </c>
+      <c r="J80" t="n">
+        <v>875036</v>
+      </c>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>Orangestar</t>
+        </is>
+      </c>
+      <c r="L80" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:13:27</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -9539,10 +10153,24 @@
           <t>Hey! Say! JUMP</t>
         </is>
       </c>
-      <c r="I81" t="inlineStr"/>
-      <c r="J81" t="inlineStr"/>
-      <c r="K81" t="inlineStr"/>
-      <c r="L81" t="inlineStr"/>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=cZftmR93acE</t>
+        </is>
+      </c>
+      <c r="J81" t="n">
+        <v>289023</v>
+      </c>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>アニメ小3アシベQQゴマちゃん公式チャンネル</t>
+        </is>
+      </c>
+      <c r="L81" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:13:40</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -9579,10 +10207,24 @@
           <t>BOYS AND MEN</t>
         </is>
       </c>
-      <c r="I82" t="inlineStr"/>
-      <c r="J82" t="inlineStr"/>
-      <c r="K82" t="inlineStr"/>
-      <c r="L82" t="inlineStr"/>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=gNZNdc5UbTE</t>
+        </is>
+      </c>
+      <c r="J82" t="n">
+        <v>4852025</v>
+      </c>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BOYS AND MEN ＜ボイメン＞ </t>
+        </is>
+      </c>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:13:52</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -9619,10 +10261,24 @@
           <t>村上佳佑</t>
         </is>
       </c>
-      <c r="I83" t="inlineStr"/>
-      <c r="J83" t="inlineStr"/>
-      <c r="K83" t="inlineStr"/>
-      <c r="L83" t="inlineStr"/>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=CGuw9xBuMVU</t>
+        </is>
+      </c>
+      <c r="J83" t="n">
+        <v>39427</v>
+      </c>
+      <c r="K83" t="inlineStr">
+        <is>
+          <t>アニメ・特撮ソング伴奏製作所</t>
+        </is>
+      </c>
+      <c r="L83" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:14:03</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -9659,10 +10315,24 @@
           <t>TETSUYA</t>
         </is>
       </c>
-      <c r="I84" t="inlineStr"/>
-      <c r="J84" t="inlineStr"/>
-      <c r="K84" t="inlineStr"/>
-      <c r="L84" t="inlineStr"/>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=KllomiQuM3Q</t>
+        </is>
+      </c>
+      <c r="J84" t="n">
+        <v>12495</v>
+      </c>
+      <c r="K84" t="inlineStr">
+        <is>
+          <t>アニメ・特撮ソング伴奏製作所</t>
+        </is>
+      </c>
+      <c r="L84" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:14:15</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="n">
@@ -9699,10 +10369,24 @@
           <t>SILENT SIREN</t>
         </is>
       </c>
-      <c r="I85" t="inlineStr"/>
-      <c r="J85" t="inlineStr"/>
-      <c r="K85" t="inlineStr"/>
-      <c r="L85" t="inlineStr"/>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=EItnl7wcQZk</t>
+        </is>
+      </c>
+      <c r="J85" t="n">
+        <v>1552645</v>
+      </c>
+      <c r="K85" t="inlineStr">
+        <is>
+          <t>SILENT_SIREN</t>
+        </is>
+      </c>
+      <c r="L85" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:14:26</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -9779,10 +10463,24 @@
           <t>ベリーグッドマン</t>
         </is>
       </c>
-      <c r="I87" t="inlineStr"/>
-      <c r="J87" t="inlineStr"/>
-      <c r="K87" t="inlineStr"/>
-      <c r="L87" t="inlineStr"/>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=3g-n6WbIcDA</t>
+        </is>
+      </c>
+      <c r="J87" t="n">
+        <v>8414</v>
+      </c>
+      <c r="K87" t="inlineStr">
+        <is>
+          <t>アニメ・特撮ソング伴奏製作所</t>
+        </is>
+      </c>
+      <c r="L87" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:14:49</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -9899,10 +10597,24 @@
           <t>tuki.</t>
         </is>
       </c>
-      <c r="I90" t="inlineStr"/>
-      <c r="J90" t="inlineStr"/>
-      <c r="K90" t="inlineStr"/>
-      <c r="L90" t="inlineStr"/>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=2splxp-qwH0</t>
+        </is>
+      </c>
+      <c r="J90" t="n">
+        <v>1001886</v>
+      </c>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>tuki.(17)</t>
+        </is>
+      </c>
+      <c r="L90" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:15:03</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -9939,10 +10651,24 @@
           <t>ヒグチアイ</t>
         </is>
       </c>
-      <c r="I91" t="inlineStr"/>
-      <c r="J91" t="inlineStr"/>
-      <c r="K91" t="inlineStr"/>
-      <c r="L91" t="inlineStr"/>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=0vTK8SWTgws</t>
+        </is>
+      </c>
+      <c r="J91" t="n">
+        <v>422037</v>
+      </c>
+      <c r="K91" t="inlineStr">
+        <is>
+          <t>TOHO animation</t>
+        </is>
+      </c>
+      <c r="L91" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:15:15</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -9979,10 +10705,24 @@
           <t>亜咲花</t>
         </is>
       </c>
-      <c r="I92" t="inlineStr"/>
-      <c r="J92" t="inlineStr"/>
-      <c r="K92" t="inlineStr"/>
-      <c r="L92" t="inlineStr"/>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=8XeyK9hI6WI</t>
+        </is>
+      </c>
+      <c r="J92" t="n">
+        <v>9657</v>
+      </c>
+      <c r="K92" t="inlineStr">
+        <is>
+          <t>亜咲花公式チャンネル</t>
+        </is>
+      </c>
+      <c r="L92" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:15:28</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -10019,10 +10759,24 @@
           <t>Baby Canta</t>
         </is>
       </c>
-      <c r="I93" t="inlineStr"/>
-      <c r="J93" t="inlineStr"/>
-      <c r="K93" t="inlineStr"/>
-      <c r="L93" t="inlineStr"/>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=dPWuN1uP09g</t>
+        </is>
+      </c>
+      <c r="J93" t="n">
+        <v>914861</v>
+      </c>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>TVアニメ「ダイヤのA」シリーズ</t>
+        </is>
+      </c>
+      <c r="L93" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:15:41</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -10059,10 +10813,24 @@
           <t>SUPER★DRAGON</t>
         </is>
       </c>
-      <c r="I94" t="inlineStr"/>
-      <c r="J94" t="inlineStr"/>
-      <c r="K94" t="inlineStr"/>
-      <c r="L94" t="inlineStr"/>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=dPWuN1uP09g</t>
+        </is>
+      </c>
+      <c r="J94" t="n">
+        <v>914861</v>
+      </c>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>TVアニメ「ダイヤのA」シリーズ</t>
+        </is>
+      </c>
+      <c r="L94" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:15:53</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -10099,10 +10867,24 @@
           <t>超特急</t>
         </is>
       </c>
-      <c r="I95" t="inlineStr"/>
-      <c r="J95" t="inlineStr"/>
-      <c r="K95" t="inlineStr"/>
-      <c r="L95" t="inlineStr"/>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=w8ltcHURKhc</t>
+        </is>
+      </c>
+      <c r="J95" t="n">
+        <v>190536</v>
+      </c>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>超特急</t>
+        </is>
+      </c>
+      <c r="L95" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:16:06</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -10139,10 +10921,24 @@
           <t>『ユイカ』</t>
         </is>
       </c>
-      <c r="I96" t="inlineStr"/>
-      <c r="J96" t="inlineStr"/>
-      <c r="K96" t="inlineStr"/>
-      <c r="L96" t="inlineStr"/>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=b92uylP2yCs</t>
+        </is>
+      </c>
+      <c r="J96" t="n">
+        <v>512594</v>
+      </c>
+      <c r="K96" t="inlineStr">
+        <is>
+          <t>『ユイカ』</t>
+        </is>
+      </c>
+      <c r="L96" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:16:19</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="n">
@@ -10179,10 +10975,24 @@
           <t>こっちのけんと</t>
         </is>
       </c>
-      <c r="I97" t="inlineStr"/>
-      <c r="J97" t="inlineStr"/>
-      <c r="K97" t="inlineStr"/>
-      <c r="L97" t="inlineStr"/>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=ffxN8II-Vic</t>
+        </is>
+      </c>
+      <c r="J97" t="n">
+        <v>1572114</v>
+      </c>
+      <c r="K97" t="inlineStr">
+        <is>
+          <t>こっちのけんと</t>
+        </is>
+      </c>
+      <c r="L97" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:16:33</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -10219,10 +11029,24 @@
           <t>ASH DA HERO</t>
         </is>
       </c>
-      <c r="I98" t="inlineStr"/>
-      <c r="J98" t="inlineStr"/>
-      <c r="K98" t="inlineStr"/>
-      <c r="L98" t="inlineStr"/>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=03eMtnVjiBk</t>
+        </is>
+      </c>
+      <c r="J98" t="n">
+        <v>1106840</v>
+      </c>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>isekai channel @バンダイナムコフィルムワークス</t>
+        </is>
+      </c>
+      <c r="L98" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:16:45</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="n">
@@ -10259,10 +11083,24 @@
           <t>シユイ</t>
         </is>
       </c>
-      <c r="I99" t="inlineStr"/>
-      <c r="J99" t="inlineStr"/>
-      <c r="K99" t="inlineStr"/>
-      <c r="L99" t="inlineStr"/>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=Pn0c9QIiqbo</t>
+        </is>
+      </c>
+      <c r="J99" t="n">
+        <v>174604</v>
+      </c>
+      <c r="K99" t="inlineStr">
+        <is>
+          <t>isekai channel @バンダイナムコフィルムワークス</t>
+        </is>
+      </c>
+      <c r="L99" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:16:57</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="n">
@@ -10339,10 +11177,24 @@
           <t>藍井エイル</t>
         </is>
       </c>
-      <c r="I101" t="inlineStr"/>
-      <c r="J101" t="inlineStr"/>
-      <c r="K101" t="inlineStr"/>
-      <c r="L101" t="inlineStr"/>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=ILfcwl8ZKDs</t>
+        </is>
+      </c>
+      <c r="J101" t="n">
+        <v>201532</v>
+      </c>
+      <c r="K101" t="inlineStr">
+        <is>
+          <t>Lantis Channel</t>
+        </is>
+      </c>
+      <c r="L101" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:17:21</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="n">
@@ -10379,10 +11231,24 @@
           <t>CiON</t>
         </is>
       </c>
-      <c r="I102" t="inlineStr"/>
-      <c r="J102" t="inlineStr"/>
-      <c r="K102" t="inlineStr"/>
-      <c r="L102" t="inlineStr"/>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=xdhkJtJcdEk</t>
+        </is>
+      </c>
+      <c r="J102" t="n">
+        <v>155173</v>
+      </c>
+      <c r="K102" t="inlineStr">
+        <is>
+          <t>CiON official YouTube Channel</t>
+        </is>
+      </c>
+      <c r="L102" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:17:34</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="n">
@@ -10419,10 +11285,24 @@
           <t>ALI</t>
         </is>
       </c>
-      <c r="I103" t="inlineStr"/>
-      <c r="J103" t="inlineStr"/>
-      <c r="K103" t="inlineStr"/>
-      <c r="L103" t="inlineStr"/>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=sPxXiXucYcM</t>
+        </is>
+      </c>
+      <c r="J103" t="n">
+        <v>7100246</v>
+      </c>
+      <c r="K103" t="inlineStr">
+        <is>
+          <t>ALI</t>
+        </is>
+      </c>
+      <c r="L103" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:17:47</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="n">
@@ -10459,10 +11339,24 @@
           <t>KANA-BOON</t>
         </is>
       </c>
-      <c r="I104" t="inlineStr"/>
-      <c r="J104" t="inlineStr"/>
-      <c r="K104" t="inlineStr"/>
-      <c r="L104" t="inlineStr"/>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=HNYp4T0kMNU</t>
+        </is>
+      </c>
+      <c r="J104" t="n">
+        <v>2456417</v>
+      </c>
+      <c r="K104" t="inlineStr">
+        <is>
+          <t>TOHO animation</t>
+        </is>
+      </c>
+      <c r="L104" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:18:01</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="n">
@@ -10499,10 +11393,24 @@
           <t>ASIAN KUNG-FU GENERATION</t>
         </is>
       </c>
-      <c r="I105" t="inlineStr"/>
-      <c r="J105" t="inlineStr"/>
-      <c r="K105" t="inlineStr"/>
-      <c r="L105" t="inlineStr"/>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=ycH4Twoq83I</t>
+        </is>
+      </c>
+      <c r="J105" t="n">
+        <v>807317</v>
+      </c>
+      <c r="K105" t="inlineStr">
+        <is>
+          <t>TOHO animation</t>
+        </is>
+      </c>
+      <c r="L105" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:18:14</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="n">
@@ -10539,10 +11447,24 @@
           <t>BREIMEN</t>
         </is>
       </c>
-      <c r="I106" t="inlineStr"/>
-      <c r="J106" t="inlineStr"/>
-      <c r="K106" t="inlineStr"/>
-      <c r="L106" t="inlineStr"/>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=5SGVXrvEK0o</t>
+        </is>
+      </c>
+      <c r="J106" t="n">
+        <v>1453819</v>
+      </c>
+      <c r="K106" t="inlineStr">
+        <is>
+          <t>BREIMEN _Channel</t>
+        </is>
+      </c>
+      <c r="L106" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:18:27</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="n">
@@ -10579,10 +11501,24 @@
           <t>音羽-otoha-</t>
         </is>
       </c>
-      <c r="I107" t="inlineStr"/>
-      <c r="J107" t="inlineStr"/>
-      <c r="K107" t="inlineStr"/>
-      <c r="L107" t="inlineStr"/>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=SZhcN4jVVzA</t>
+        </is>
+      </c>
+      <c r="J107" t="n">
+        <v>1122108</v>
+      </c>
+      <c r="K107" t="inlineStr">
+        <is>
+          <t>音羽-otoha-</t>
+        </is>
+      </c>
+      <c r="L107" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:18:40</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="n">
@@ -10619,10 +11555,24 @@
           <t>BURNOUT SYNDROMES</t>
         </is>
       </c>
-      <c r="I108" t="inlineStr"/>
-      <c r="J108" t="inlineStr"/>
-      <c r="K108" t="inlineStr"/>
-      <c r="L108" t="inlineStr"/>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=HXvZ7Y7uYbo</t>
+        </is>
+      </c>
+      <c r="J108" t="n">
+        <v>629266</v>
+      </c>
+      <c r="K108" t="inlineStr">
+        <is>
+          <t>TOHO animation</t>
+        </is>
+      </c>
+      <c r="L108" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:18:53</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="n">
@@ -10659,10 +11609,24 @@
           <t>(K)NoW_NAME</t>
         </is>
       </c>
-      <c r="I109" t="inlineStr"/>
-      <c r="J109" t="inlineStr"/>
-      <c r="K109" t="inlineStr"/>
-      <c r="L109" t="inlineStr"/>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=LWaqlY0Xqy0</t>
+        </is>
+      </c>
+      <c r="J109" t="n">
+        <v>911783</v>
+      </c>
+      <c r="K109" t="inlineStr">
+        <is>
+          <t>(K)NoW_NAME - Topic</t>
+        </is>
+      </c>
+      <c r="L109" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:19:05</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="n">
@@ -10699,10 +11663,24 @@
           <t>(K)NoW_NAME</t>
         </is>
       </c>
-      <c r="I110" t="inlineStr"/>
-      <c r="J110" t="inlineStr"/>
-      <c r="K110" t="inlineStr"/>
-      <c r="L110" t="inlineStr"/>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=6RnvqHkDI50</t>
+        </is>
+      </c>
+      <c r="J110" t="n">
+        <v>219181</v>
+      </c>
+      <c r="K110" t="inlineStr">
+        <is>
+          <t>(K)NoW_NAME - Topic</t>
+        </is>
+      </c>
+      <c r="L110" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:19:16</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="n">
@@ -10739,10 +11717,24 @@
           <t>Eve</t>
         </is>
       </c>
-      <c r="I111" t="inlineStr"/>
-      <c r="J111" t="inlineStr"/>
-      <c r="K111" t="inlineStr"/>
-      <c r="L111" t="inlineStr"/>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=ySpIrrCmiCU</t>
+        </is>
+      </c>
+      <c r="J111" t="n">
+        <v>2058400</v>
+      </c>
+      <c r="K111" t="inlineStr">
+        <is>
+          <t>Eve</t>
+        </is>
+      </c>
+      <c r="L111" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:19:30</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="n">
@@ -10779,10 +11771,24 @@
           <t>Nakamura Hak</t>
         </is>
       </c>
-      <c r="I112" t="inlineStr"/>
-      <c r="J112" t="inlineStr"/>
-      <c r="K112" t="inlineStr"/>
-      <c r="L112" t="inlineStr"/>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=rQ0S_0CepIo</t>
+        </is>
+      </c>
+      <c r="J112" t="n">
+        <v>1305856</v>
+      </c>
+      <c r="K112" t="inlineStr">
+        <is>
+          <t>TVアニメ「とんがり帽子のアトリエ」公式</t>
+        </is>
+      </c>
+      <c r="L112" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:19:42</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="n">
@@ -10819,10 +11825,24 @@
           <t>Aiobahn ＋81</t>
         </is>
       </c>
-      <c r="I113" t="inlineStr"/>
-      <c r="J113" t="inlineStr"/>
-      <c r="K113" t="inlineStr"/>
-      <c r="L113" t="inlineStr"/>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=BnkhBwzBqlQ</t>
+        </is>
+      </c>
+      <c r="J113" t="n">
+        <v>29176895</v>
+      </c>
+      <c r="K113" t="inlineStr">
+        <is>
+          <t>Aiobahn</t>
+        </is>
+      </c>
+      <c r="L113" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:19:55</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="n">
@@ -10859,10 +11879,24 @@
           <t>キタニタツヤ</t>
         </is>
       </c>
-      <c r="I114" t="inlineStr"/>
-      <c r="J114" t="inlineStr"/>
-      <c r="K114" t="inlineStr"/>
-      <c r="L114" t="inlineStr"/>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=l7hbIgnyhe0</t>
+        </is>
+      </c>
+      <c r="J114" t="n">
+        <v>579425</v>
+      </c>
+      <c r="K114" t="inlineStr">
+        <is>
+          <t>キタニタツヤ / Tatsuya Kitani</t>
+        </is>
+      </c>
+      <c r="L114" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:20:08</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="n">
@@ -10899,10 +11933,24 @@
           <t>HoneyWorks feat.鈴木愛理</t>
         </is>
       </c>
-      <c r="I115" t="inlineStr"/>
-      <c r="J115" t="inlineStr"/>
-      <c r="K115" t="inlineStr"/>
-      <c r="L115" t="inlineStr"/>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=_3aytoDQTHg</t>
+        </is>
+      </c>
+      <c r="J115" t="n">
+        <v>728377</v>
+      </c>
+      <c r="K115" t="inlineStr">
+        <is>
+          <t>MARUMOCHI from HoneyWorks</t>
+        </is>
+      </c>
+      <c r="L115" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:20:22</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="n">
@@ -10939,10 +11987,24 @@
           <t>吉乃</t>
         </is>
       </c>
-      <c r="I116" t="inlineStr"/>
-      <c r="J116" t="inlineStr"/>
-      <c r="K116" t="inlineStr"/>
-      <c r="L116" t="inlineStr"/>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=iouWS4pwX28</t>
+        </is>
+      </c>
+      <c r="J116" t="n">
+        <v>227515</v>
+      </c>
+      <c r="K116" t="inlineStr">
+        <is>
+          <t>吉乃</t>
+        </is>
+      </c>
+      <c r="L116" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:20:35</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="n">
@@ -11059,10 +12121,24 @@
           <t>キタニタツヤ</t>
         </is>
       </c>
-      <c r="I119" t="inlineStr"/>
-      <c r="J119" t="inlineStr"/>
-      <c r="K119" t="inlineStr"/>
-      <c r="L119" t="inlineStr"/>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=hA_9r-3jkSg</t>
+        </is>
+      </c>
+      <c r="J119" t="n">
+        <v>1806016</v>
+      </c>
+      <c r="K119" t="inlineStr">
+        <is>
+          <t>キタニタツヤ / Tatsuya Kitani</t>
+        </is>
+      </c>
+      <c r="L119" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:20:49</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="n">
@@ -11099,10 +12175,24 @@
           <t>Leina</t>
         </is>
       </c>
-      <c r="I120" t="inlineStr"/>
-      <c r="J120" t="inlineStr"/>
-      <c r="K120" t="inlineStr"/>
-      <c r="L120" t="inlineStr"/>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=1KnySdlZHJU</t>
+        </is>
+      </c>
+      <c r="J120" t="n">
+        <v>259162</v>
+      </c>
+      <c r="K120" t="inlineStr">
+        <is>
+          <t>Leina</t>
+        </is>
+      </c>
+      <c r="L120" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:21:02</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="n">
@@ -11139,10 +12229,24 @@
           <t>DARUMA Rollin’</t>
         </is>
       </c>
-      <c r="I121" t="inlineStr"/>
-      <c r="J121" t="inlineStr"/>
-      <c r="K121" t="inlineStr"/>
-      <c r="L121" t="inlineStr"/>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=mfBWkIIQE9w</t>
+        </is>
+      </c>
+      <c r="J121" t="n">
+        <v>267737</v>
+      </c>
+      <c r="K121" t="inlineStr">
+        <is>
+          <t>DARUMA Rollin'</t>
+        </is>
+      </c>
+      <c r="L121" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:21:14</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="n">
@@ -11179,10 +12283,24 @@
           <t>高橋哲也</t>
         </is>
       </c>
-      <c r="I122" t="inlineStr"/>
-      <c r="J122" t="inlineStr"/>
-      <c r="K122" t="inlineStr"/>
-      <c r="L122" t="inlineStr"/>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=muqyayR_9ts</t>
+        </is>
+      </c>
+      <c r="J122" t="n">
+        <v>8986</v>
+      </c>
+      <c r="K122" t="inlineStr">
+        <is>
+          <t>HERO'S Web公式チャンネル</t>
+        </is>
+      </c>
+      <c r="L122" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:21:29</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="n">
@@ -11339,10 +12457,24 @@
           <t>前島亜美</t>
         </is>
       </c>
-      <c r="I126" t="inlineStr"/>
-      <c r="J126" t="inlineStr"/>
-      <c r="K126" t="inlineStr"/>
-      <c r="L126" t="inlineStr"/>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=xuyA1jEiJ8c</t>
+        </is>
+      </c>
+      <c r="J126" t="n">
+        <v>193665</v>
+      </c>
+      <c r="K126" t="inlineStr">
+        <is>
+          <t>前島亜美</t>
+        </is>
+      </c>
+      <c r="L126" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:22:02</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="n">
@@ -11379,10 +12511,24 @@
           <t>愛美</t>
         </is>
       </c>
-      <c r="I127" t="inlineStr"/>
-      <c r="J127" t="inlineStr"/>
-      <c r="K127" t="inlineStr"/>
-      <c r="L127" t="inlineStr"/>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=ifutP5vX5TA</t>
+        </is>
+      </c>
+      <c r="J127" t="n">
+        <v>21547</v>
+      </c>
+      <c r="K127" t="inlineStr">
+        <is>
+          <t>AIMI official YouTube Channel</t>
+        </is>
+      </c>
+      <c r="L127" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:22:14</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="n">
@@ -11419,10 +12565,24 @@
           <t>issei</t>
         </is>
       </c>
-      <c r="I128" t="inlineStr"/>
-      <c r="J128" t="inlineStr"/>
-      <c r="K128" t="inlineStr"/>
-      <c r="L128" t="inlineStr"/>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=gOTNI5smH2E</t>
+        </is>
+      </c>
+      <c r="J128" t="n">
+        <v>1197894</v>
+      </c>
+      <c r="K128" t="inlineStr">
+        <is>
+          <t>TOHO animation</t>
+        </is>
+      </c>
+      <c r="L128" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:22:26</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="n">
@@ -11459,10 +12619,24 @@
           <t>神前暁</t>
         </is>
       </c>
-      <c r="I129" t="inlineStr"/>
-      <c r="J129" t="inlineStr"/>
-      <c r="K129" t="inlineStr"/>
-      <c r="L129" t="inlineStr"/>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=gOTNI5smH2E</t>
+        </is>
+      </c>
+      <c r="J129" t="n">
+        <v>1197894</v>
+      </c>
+      <c r="K129" t="inlineStr">
+        <is>
+          <t>TOHO animation</t>
+        </is>
+      </c>
+      <c r="L129" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:22:40</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="n">
@@ -11539,10 +12713,24 @@
           <t>SEVENTEEN</t>
         </is>
       </c>
-      <c r="I131" t="inlineStr"/>
-      <c r="J131" t="inlineStr"/>
-      <c r="K131" t="inlineStr"/>
-      <c r="L131" t="inlineStr"/>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=5A7qyhj-HjE</t>
+        </is>
+      </c>
+      <c r="J131" t="n">
+        <v>828219</v>
+      </c>
+      <c r="K131" t="inlineStr">
+        <is>
+          <t>SEVENTEEN</t>
+        </is>
+      </c>
+      <c r="L131" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:23:01</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="n">
@@ -11579,10 +12767,24 @@
           <t>レトロリロン</t>
         </is>
       </c>
-      <c r="I132" t="inlineStr"/>
-      <c r="J132" t="inlineStr"/>
-      <c r="K132" t="inlineStr"/>
-      <c r="L132" t="inlineStr"/>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=4cGnQ8gFCCs</t>
+        </is>
+      </c>
+      <c r="J132" t="n">
+        <v>117523</v>
+      </c>
+      <c r="K132" t="inlineStr">
+        <is>
+          <t>MBS animation 公式チャンネル</t>
+        </is>
+      </c>
+      <c r="L132" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:23:14</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="n">
@@ -11619,10 +12821,24 @@
           <t>ガラクタ</t>
         </is>
       </c>
-      <c r="I133" t="inlineStr"/>
-      <c r="J133" t="inlineStr"/>
-      <c r="K133" t="inlineStr"/>
-      <c r="L133" t="inlineStr"/>
+      <c r="I133" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=xSNhOhCEaC4</t>
+        </is>
+      </c>
+      <c r="J133" t="n">
+        <v>27686</v>
+      </c>
+      <c r="K133" t="inlineStr">
+        <is>
+          <t>MBS animation 公式チャンネル</t>
+        </is>
+      </c>
+      <c r="L133" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:23:27</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="n">
@@ -11659,10 +12875,24 @@
           <t>ALI</t>
         </is>
       </c>
-      <c r="I134" t="inlineStr"/>
-      <c r="J134" t="inlineStr"/>
-      <c r="K134" t="inlineStr"/>
-      <c r="L134" t="inlineStr"/>
+      <c r="I134" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=8V9cwO1ZxGk</t>
+        </is>
+      </c>
+      <c r="J134" t="n">
+        <v>80366</v>
+      </c>
+      <c r="K134" t="inlineStr">
+        <is>
+          <t>ALI</t>
+        </is>
+      </c>
+      <c r="L134" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:23:39</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="n">
@@ -11699,10 +12929,24 @@
           <t>紫 今</t>
         </is>
       </c>
-      <c r="I135" t="inlineStr"/>
-      <c r="J135" t="inlineStr"/>
-      <c r="K135" t="inlineStr"/>
-      <c r="L135" t="inlineStr"/>
+      <c r="I135" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=vlbobXEQLqY</t>
+        </is>
+      </c>
+      <c r="J135" t="n">
+        <v>125026</v>
+      </c>
+      <c r="K135" t="inlineStr">
+        <is>
+          <t>ギャガ公式チャンネル</t>
+        </is>
+      </c>
+      <c r="L135" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:23:50</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="n">
@@ -11979,10 +13223,24 @@
           <t>osage</t>
         </is>
       </c>
-      <c r="I142" t="inlineStr"/>
-      <c r="J142" t="inlineStr"/>
-      <c r="K142" t="inlineStr"/>
-      <c r="L142" t="inlineStr"/>
+      <c r="I142" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=0XwlRpvjbmY</t>
+        </is>
+      </c>
+      <c r="J142" t="n">
+        <v>3513</v>
+      </c>
+      <c r="K142" t="inlineStr">
+        <is>
+          <t>osage official</t>
+        </is>
+      </c>
+      <c r="L142" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:24:51</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="n">
@@ -12019,10 +13277,24 @@
           <t>ミーマイナー</t>
         </is>
       </c>
-      <c r="I143" t="inlineStr"/>
-      <c r="J143" t="inlineStr"/>
-      <c r="K143" t="inlineStr"/>
-      <c r="L143" t="inlineStr"/>
+      <c r="I143" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=6TOl476i5Q8</t>
+        </is>
+      </c>
+      <c r="J143" t="n">
+        <v>27410</v>
+      </c>
+      <c r="K143" t="inlineStr">
+        <is>
+          <t>ミーマイナー</t>
+        </is>
+      </c>
+      <c r="L143" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:25:04</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="n">
@@ -12059,10 +13331,24 @@
           <t>Little Glee Monster</t>
         </is>
       </c>
-      <c r="I144" t="inlineStr"/>
-      <c r="J144" t="inlineStr"/>
-      <c r="K144" t="inlineStr"/>
-      <c r="L144" t="inlineStr"/>
+      <c r="I144" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=DNa76ODisco</t>
+        </is>
+      </c>
+      <c r="J144" t="n">
+        <v>429127</v>
+      </c>
+      <c r="K144" t="inlineStr">
+        <is>
+          <t>Little Glee Monster</t>
+        </is>
+      </c>
+      <c r="L144" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:25:17</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="n">
@@ -12099,10 +13385,24 @@
           <t>生田絵梨花</t>
         </is>
       </c>
-      <c r="I145" t="inlineStr"/>
-      <c r="J145" t="inlineStr"/>
-      <c r="K145" t="inlineStr"/>
-      <c r="L145" t="inlineStr"/>
+      <c r="I145" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=kX0u1U7wMDk</t>
+        </is>
+      </c>
+      <c r="J145" t="n">
+        <v>705610</v>
+      </c>
+      <c r="K145" t="inlineStr">
+        <is>
+          <t>生田絵梨花 Official YouTube Channel</t>
+        </is>
+      </c>
+      <c r="L145" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:25:32</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="n">
@@ -12139,10 +13439,24 @@
           <t>Penthouse</t>
         </is>
       </c>
-      <c r="I146" t="inlineStr"/>
-      <c r="J146" t="inlineStr"/>
-      <c r="K146" t="inlineStr"/>
-      <c r="L146" t="inlineStr"/>
+      <c r="I146" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=m4yCXpCiXpk</t>
+        </is>
+      </c>
+      <c r="J146" t="n">
+        <v>705610</v>
+      </c>
+      <c r="K146" t="inlineStr">
+        <is>
+          <t>Penthouse</t>
+        </is>
+      </c>
+      <c r="L146" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:25:46</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="n">
@@ -12179,10 +13493,24 @@
           <t>CANDY TUNE</t>
         </is>
       </c>
-      <c r="I147" t="inlineStr"/>
-      <c r="J147" t="inlineStr"/>
-      <c r="K147" t="inlineStr"/>
-      <c r="L147" t="inlineStr"/>
+      <c r="I147" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=jMhzqfi9aPw</t>
+        </is>
+      </c>
+      <c r="J147" t="n">
+        <v>630585</v>
+      </c>
+      <c r="K147" t="inlineStr">
+        <is>
+          <t>アニメ「魔入りました!入間くん」公式Anime OFFICIAL</t>
+        </is>
+      </c>
+      <c r="L147" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:25:58</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="n">
@@ -12299,10 +13627,24 @@
           <t>Kis-My-Ft2</t>
         </is>
       </c>
-      <c r="I150" t="inlineStr"/>
-      <c r="J150" t="inlineStr"/>
-      <c r="K150" t="inlineStr"/>
-      <c r="L150" t="inlineStr"/>
+      <c r="I150" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=MGUp9RBrou4</t>
+        </is>
+      </c>
+      <c r="J150" t="n">
+        <v>10157104</v>
+      </c>
+      <c r="K150" t="inlineStr">
+        <is>
+          <t>Kis-My-Ft2</t>
+        </is>
+      </c>
+      <c r="L150" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:26:13</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="n">
@@ -12339,10 +13681,24 @@
           <t>TRUE</t>
         </is>
       </c>
-      <c r="I151" t="inlineStr"/>
-      <c r="J151" t="inlineStr"/>
-      <c r="K151" t="inlineStr"/>
-      <c r="L151" t="inlineStr"/>
+      <c r="I151" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=eVfpoS0rjw0</t>
+        </is>
+      </c>
+      <c r="J151" t="n">
+        <v>1659920</v>
+      </c>
+      <c r="K151" t="inlineStr">
+        <is>
+          <t>Bandai Namco Filmworks Channel</t>
+        </is>
+      </c>
+      <c r="L151" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:26:25</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="n">
@@ -12379,10 +13735,24 @@
           <t>多次元制御機構よだか</t>
         </is>
       </c>
-      <c r="I152" t="inlineStr"/>
-      <c r="J152" t="inlineStr"/>
-      <c r="K152" t="inlineStr"/>
-      <c r="L152" t="inlineStr"/>
+      <c r="I152" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=Z53w6cpG5GM</t>
+        </is>
+      </c>
+      <c r="J152" t="n">
+        <v>48053</v>
+      </c>
+      <c r="K152" t="inlineStr">
+        <is>
+          <t>TBSアニメ</t>
+        </is>
+      </c>
+      <c r="L152" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:26:35</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="n">
@@ -12419,10 +13789,24 @@
           <t>リリテア（CV.若山詩音）</t>
         </is>
       </c>
-      <c r="I153" t="inlineStr"/>
-      <c r="J153" t="inlineStr"/>
-      <c r="K153" t="inlineStr"/>
-      <c r="L153" t="inlineStr"/>
+      <c r="I153" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=ZvHOYO6tfvk</t>
+        </is>
+      </c>
+      <c r="J153" t="n">
+        <v>16033</v>
+      </c>
+      <c r="K153" t="inlineStr">
+        <is>
+          <t>リリテア（CV:若山詩音） - Topic</t>
+        </is>
+      </c>
+      <c r="L153" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:26:41</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="n">
@@ -12459,10 +13843,24 @@
           <t>ILLIT</t>
         </is>
       </c>
-      <c r="I154" t="inlineStr"/>
-      <c r="J154" t="inlineStr"/>
-      <c r="K154" t="inlineStr"/>
-      <c r="L154" t="inlineStr"/>
+      <c r="I154" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=OZ44P4JU87E</t>
+        </is>
+      </c>
+      <c r="J154" t="n">
+        <v>1544080</v>
+      </c>
+      <c r="K154" t="inlineStr">
+        <is>
+          <t>ILLIT</t>
+        </is>
+      </c>
+      <c r="L154" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:26:55</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="n">
@@ -12499,10 +13897,24 @@
           <t>ルルットリリィ（こんぺとリリィ（CV.橘めい）、ましゅールル（CV.小鹿なお））</t>
         </is>
       </c>
-      <c r="I155" t="inlineStr"/>
-      <c r="J155" t="inlineStr"/>
-      <c r="K155" t="inlineStr"/>
-      <c r="L155" t="inlineStr"/>
+      <c r="I155" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
+        </is>
+      </c>
+      <c r="J155" t="n">
+        <v>209352</v>
+      </c>
+      <c r="K155" t="inlineStr">
+        <is>
+          <t>Bandai Namco Filmworks Channel</t>
+        </is>
+      </c>
+      <c r="L155" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:27:07</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="n">
@@ -12539,10 +13951,24 @@
           <t>NEE</t>
         </is>
       </c>
-      <c r="I156" t="inlineStr"/>
-      <c r="J156" t="inlineStr"/>
-      <c r="K156" t="inlineStr"/>
-      <c r="L156" t="inlineStr"/>
+      <c r="I156" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=0j7O1Sw62Ms</t>
+        </is>
+      </c>
+      <c r="J156" t="n">
+        <v>39536</v>
+      </c>
+      <c r="K156" t="inlineStr">
+        <is>
+          <t>NEE</t>
+        </is>
+      </c>
+      <c r="L156" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:27:20</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="n">
@@ -12659,10 +14085,24 @@
           <t>平手友梨奈</t>
         </is>
       </c>
-      <c r="I159" t="inlineStr"/>
-      <c r="J159" t="inlineStr"/>
-      <c r="K159" t="inlineStr"/>
-      <c r="L159" t="inlineStr"/>
+      <c r="I159" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=QbNwgXAXq9M</t>
+        </is>
+      </c>
+      <c r="J159" t="n">
+        <v>964216</v>
+      </c>
+      <c r="K159" t="inlineStr">
+        <is>
+          <t>平手友梨奈</t>
+        </is>
+      </c>
+      <c r="L159" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:27:50</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="n">
@@ -12699,10 +14139,24 @@
           <t>AKASAKI</t>
         </is>
       </c>
-      <c r="I160" t="inlineStr"/>
-      <c r="J160" t="inlineStr"/>
-      <c r="K160" t="inlineStr"/>
-      <c r="L160" t="inlineStr"/>
+      <c r="I160" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=WwI7hPXZC-Y</t>
+        </is>
+      </c>
+      <c r="J160" t="n">
+        <v>2444210</v>
+      </c>
+      <c r="K160" t="inlineStr">
+        <is>
+          <t>AKASAKI (19)</t>
+        </is>
+      </c>
+      <c r="L160" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:28:02</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="n">
@@ -12739,10 +14193,24 @@
           <t>majiko</t>
         </is>
       </c>
-      <c r="I161" t="inlineStr"/>
-      <c r="J161" t="inlineStr"/>
-      <c r="K161" t="inlineStr"/>
-      <c r="L161" t="inlineStr"/>
+      <c r="I161" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=VHD2269UqdM</t>
+        </is>
+      </c>
+      <c r="J161" t="n">
+        <v>37559</v>
+      </c>
+      <c r="K161" t="inlineStr">
+        <is>
+          <t>ハピネット【アニメ公式】</t>
+        </is>
+      </c>
+      <c r="L161" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:28:14</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="n">
@@ -12779,10 +14247,24 @@
           <t>ARCANA PROJECT</t>
         </is>
       </c>
-      <c r="I162" t="inlineStr"/>
-      <c r="J162" t="inlineStr"/>
-      <c r="K162" t="inlineStr"/>
-      <c r="L162" t="inlineStr"/>
+      <c r="I162" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=vBSo4npKK9A</t>
+        </is>
+      </c>
+      <c r="J162" t="n">
+        <v>11878</v>
+      </c>
+      <c r="K162" t="inlineStr">
+        <is>
+          <t>ハピネット【アニメ公式】</t>
+        </is>
+      </c>
+      <c r="L162" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:28:25</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="n">
@@ -12819,10 +14301,24 @@
           <t>終活クラブ</t>
         </is>
       </c>
-      <c r="I163" t="inlineStr"/>
-      <c r="J163" t="inlineStr"/>
-      <c r="K163" t="inlineStr"/>
-      <c r="L163" t="inlineStr"/>
+      <c r="I163" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=suKjfBsH3UM</t>
+        </is>
+      </c>
+      <c r="J163" t="n">
+        <v>147879</v>
+      </c>
+      <c r="K163" t="inlineStr">
+        <is>
+          <t>アニメ『女神「異世界転生何になりたいですか」 俺「勇者の肋骨で」』</t>
+        </is>
+      </c>
+      <c r="L163" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:28:38</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="n">
@@ -12859,10 +14355,24 @@
           <t>shallm</t>
         </is>
       </c>
-      <c r="I164" t="inlineStr"/>
-      <c r="J164" t="inlineStr"/>
-      <c r="K164" t="inlineStr"/>
-      <c r="L164" t="inlineStr"/>
+      <c r="I164" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=suKjfBsH3UM</t>
+        </is>
+      </c>
+      <c r="J164" t="n">
+        <v>147879</v>
+      </c>
+      <c r="K164" t="inlineStr">
+        <is>
+          <t>アニメ『女神「異世界転生何になりたいですか」 俺「勇者の肋骨で」』</t>
+        </is>
+      </c>
+      <c r="L164" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:28:51</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="n">
@@ -12899,10 +14409,24 @@
           <t>藍井エイル</t>
         </is>
       </c>
-      <c r="I165" t="inlineStr"/>
-      <c r="J165" t="inlineStr"/>
-      <c r="K165" t="inlineStr"/>
-      <c r="L165" t="inlineStr"/>
+      <c r="I165" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=l78_JpSXfxw</t>
+        </is>
+      </c>
+      <c r="J165" t="n">
+        <v>358837</v>
+      </c>
+      <c r="K165" t="inlineStr">
+        <is>
+          <t>Lantis Channel</t>
+        </is>
+      </c>
+      <c r="L165" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:29:04</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" t="n">
@@ -12939,10 +14463,24 @@
           <t>ZAQ</t>
         </is>
       </c>
-      <c r="I166" t="inlineStr"/>
-      <c r="J166" t="inlineStr"/>
-      <c r="K166" t="inlineStr"/>
-      <c r="L166" t="inlineStr"/>
+      <c r="I166" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=jl7GmJBNxk4</t>
+        </is>
+      </c>
+      <c r="J166" t="n">
+        <v>89423</v>
+      </c>
+      <c r="K166" t="inlineStr">
+        <is>
+          <t>ZAQ Official Channel</t>
+        </is>
+      </c>
+      <c r="L166" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:29:16</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="n">
@@ -13059,10 +14597,24 @@
           <t>櫻坂46</t>
         </is>
       </c>
-      <c r="I169" t="inlineStr"/>
-      <c r="J169" t="inlineStr"/>
-      <c r="K169" t="inlineStr"/>
-      <c r="L169" t="inlineStr"/>
+      <c r="I169" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=AIspds2UVts</t>
+        </is>
+      </c>
+      <c r="J169" t="n">
+        <v>187933</v>
+      </c>
+      <c r="K169" t="inlineStr">
+        <is>
+          <t>NBCUniversal Anime/Music</t>
+        </is>
+      </c>
+      <c r="L169" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:29:28</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" t="n">
@@ -13099,10 +14651,24 @@
           <t>ピラフ星人</t>
         </is>
       </c>
-      <c r="I170" t="inlineStr"/>
-      <c r="J170" t="inlineStr"/>
-      <c r="K170" t="inlineStr"/>
-      <c r="L170" t="inlineStr"/>
+      <c r="I170" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=X6fNe1uPs9E</t>
+        </is>
+      </c>
+      <c r="J170" t="n">
+        <v>234792</v>
+      </c>
+      <c r="K170" t="inlineStr">
+        <is>
+          <t>NBCUniversal Anime/Music</t>
+        </is>
+      </c>
+      <c r="L170" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:29:40</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="n">
@@ -13139,10 +14705,24 @@
           <t>Vaundy</t>
         </is>
       </c>
-      <c r="I171" t="inlineStr"/>
-      <c r="J171" t="inlineStr"/>
-      <c r="K171" t="inlineStr"/>
-      <c r="L171" t="inlineStr"/>
+      <c r="I171" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=LVCwdZoUFQ8</t>
+        </is>
+      </c>
+      <c r="J171" t="n">
+        <v>3496214</v>
+      </c>
+      <c r="K171" t="inlineStr">
+        <is>
+          <t>Vaundy</t>
+        </is>
+      </c>
+      <c r="L171" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:29:53</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="n">
@@ -13179,10 +14759,24 @@
           <t>yama</t>
         </is>
       </c>
-      <c r="I172" t="inlineStr"/>
-      <c r="J172" t="inlineStr"/>
-      <c r="K172" t="inlineStr"/>
-      <c r="L172" t="inlineStr"/>
+      <c r="I172" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=8uRMfPTAhkU</t>
+        </is>
+      </c>
+      <c r="J172" t="n">
+        <v>373757</v>
+      </c>
+      <c r="K172" t="inlineStr">
+        <is>
+          <t>yama</t>
+        </is>
+      </c>
+      <c r="L172" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:30:06</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="n">
@@ -13219,10 +14813,24 @@
           <t>Daoko</t>
         </is>
       </c>
-      <c r="I173" t="inlineStr"/>
-      <c r="J173" t="inlineStr"/>
-      <c r="K173" t="inlineStr"/>
-      <c r="L173" t="inlineStr"/>
+      <c r="I173" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=0jO_isUIymg</t>
+        </is>
+      </c>
+      <c r="J173" t="n">
+        <v>129233</v>
+      </c>
+      <c r="K173" t="inlineStr">
+        <is>
+          <t>日活アニメチャンネル</t>
+        </is>
+      </c>
+      <c r="L173" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:30:19</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="n">
@@ -13259,10 +14867,24 @@
           <t>鶸村ひより(CV：高野麻里佳)、椋林瑞希(CV：伊駒ゆりえ)、雪下祐樹(CV：篠原侑)</t>
         </is>
       </c>
-      <c r="I174" t="inlineStr"/>
-      <c r="J174" t="inlineStr"/>
-      <c r="K174" t="inlineStr"/>
-      <c r="L174" t="inlineStr"/>
+      <c r="I174" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=LRPRccAPekk</t>
+        </is>
+      </c>
+      <c r="J174" t="n">
+        <v>132505</v>
+      </c>
+      <c r="K174" t="inlineStr">
+        <is>
+          <t>日活アニメチャンネル</t>
+        </is>
+      </c>
+      <c r="L174" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:30:33</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" t="n">
@@ -13299,10 +14921,24 @@
           <t>ヨルシカ</t>
         </is>
       </c>
-      <c r="I175" t="inlineStr"/>
-      <c r="J175" t="inlineStr"/>
-      <c r="K175" t="inlineStr"/>
-      <c r="L175" t="inlineStr"/>
+      <c r="I175" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=OHAjc-ayhus</t>
+        </is>
+      </c>
+      <c r="J175" t="n">
+        <v>6187955</v>
+      </c>
+      <c r="K175" t="inlineStr">
+        <is>
+          <t>ヨルシカ / n-buna Official</t>
+        </is>
+      </c>
+      <c r="L175" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:30:46</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" t="n">
@@ -13339,10 +14975,24 @@
           <t>Lucky Kilimanjaro</t>
         </is>
       </c>
-      <c r="I176" t="inlineStr"/>
-      <c r="J176" t="inlineStr"/>
-      <c r="K176" t="inlineStr"/>
-      <c r="L176" t="inlineStr"/>
+      <c r="I176" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=hyp8GGN7C1w</t>
+        </is>
+      </c>
+      <c r="J176" t="n">
+        <v>58183</v>
+      </c>
+      <c r="K176" t="inlineStr">
+        <is>
+          <t>Lucky Kilimanjaro</t>
+        </is>
+      </c>
+      <c r="L176" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:31:00</t>
+        </is>
+      </c>
     </row>
     <row r="177">
       <c r="A177" t="n">
@@ -13379,10 +15029,24 @@
           <t>eill</t>
         </is>
       </c>
-      <c r="I177" t="inlineStr"/>
-      <c r="J177" t="inlineStr"/>
-      <c r="K177" t="inlineStr"/>
-      <c r="L177" t="inlineStr"/>
+      <c r="I177" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=fsgD8mLRxwo</t>
+        </is>
+      </c>
+      <c r="J177" t="n">
+        <v>208770</v>
+      </c>
+      <c r="K177" t="inlineStr">
+        <is>
+          <t>eill official</t>
+        </is>
+      </c>
+      <c r="L177" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:31:16</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" t="n">
@@ -13419,10 +15083,24 @@
           <t>Sizuk</t>
         </is>
       </c>
-      <c r="I178" t="inlineStr"/>
-      <c r="J178" t="inlineStr"/>
-      <c r="K178" t="inlineStr"/>
-      <c r="L178" t="inlineStr"/>
+      <c r="I178" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=LimcX6xNEaY</t>
+        </is>
+      </c>
+      <c r="J178" t="n">
+        <v>59739</v>
+      </c>
+      <c r="K178" t="inlineStr">
+        <is>
+          <t>Sizuk / Shunryu</t>
+        </is>
+      </c>
+      <c r="L178" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:31:29</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" t="n">
@@ -13459,10 +15137,24 @@
           <t>鈴木このみ feat. Ashnikko</t>
         </is>
       </c>
-      <c r="I179" t="inlineStr"/>
-      <c r="J179" t="inlineStr"/>
-      <c r="K179" t="inlineStr"/>
-      <c r="L179" t="inlineStr"/>
+      <c r="I179" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=VDGG9zi53rQ</t>
+        </is>
+      </c>
+      <c r="J179" t="n">
+        <v>5097812</v>
+      </c>
+      <c r="K179" t="inlineStr">
+        <is>
+          <t>「Re:ゼロから始める異世界生活」チャンネル【公式】</t>
+        </is>
+      </c>
+      <c r="L179" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:31:42</t>
+        </is>
+      </c>
     </row>
     <row r="180">
       <c r="A180" t="n">
@@ -13499,10 +15191,24 @@
           <t>MYTH &amp; ROID feat. TK（凛として時雨）</t>
         </is>
       </c>
-      <c r="I180" t="inlineStr"/>
-      <c r="J180" t="inlineStr"/>
-      <c r="K180" t="inlineStr"/>
-      <c r="L180" t="inlineStr"/>
+      <c r="I180" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=iKLqlb_oX60</t>
+        </is>
+      </c>
+      <c r="J180" t="n">
+        <v>579546</v>
+      </c>
+      <c r="K180" t="inlineStr">
+        <is>
+          <t>「Re:ゼロから始める異世界生活」チャンネル【公式】</t>
+        </is>
+      </c>
+      <c r="L180" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:31:54</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" t="n">
@@ -13539,10 +15245,24 @@
           <t>幾田りら</t>
         </is>
       </c>
-      <c r="I181" t="inlineStr"/>
-      <c r="J181" t="inlineStr"/>
-      <c r="K181" t="inlineStr"/>
-      <c r="L181" t="inlineStr"/>
+      <c r="I181" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=JcDyAzbGA78</t>
+        </is>
+      </c>
+      <c r="J181" t="n">
+        <v>369868</v>
+      </c>
+      <c r="K181" t="inlineStr">
+        <is>
+          <t>幾田りら / Lilas Official</t>
+        </is>
+      </c>
+      <c r="L181" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:32:07</t>
+        </is>
+      </c>
     </row>
     <row r="182">
       <c r="A182" t="n">
@@ -13579,10 +15299,24 @@
           <t>シャイトープ</t>
         </is>
       </c>
-      <c r="I182" t="inlineStr"/>
-      <c r="J182" t="inlineStr"/>
-      <c r="K182" t="inlineStr"/>
-      <c r="L182" t="inlineStr"/>
+      <c r="I182" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=BEj-QbHC54M</t>
+        </is>
+      </c>
+      <c r="J182" t="n">
+        <v>34216</v>
+      </c>
+      <c r="K182" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="L182" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:32:18</t>
+        </is>
+      </c>
     </row>
     <row r="183">
       <c r="A183" t="n">
@@ -13619,10 +15353,24 @@
           <t>asmi</t>
         </is>
       </c>
-      <c r="I183" t="inlineStr"/>
-      <c r="J183" t="inlineStr"/>
-      <c r="K183" t="inlineStr"/>
-      <c r="L183" t="inlineStr"/>
+      <c r="I183" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=ikqz8riLe1M</t>
+        </is>
+      </c>
+      <c r="J183" t="n">
+        <v>24006</v>
+      </c>
+      <c r="K183" t="inlineStr">
+        <is>
+          <t>asmi Official Channel</t>
+        </is>
+      </c>
+      <c r="L183" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:32:31</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
auto: anime list update 2026-05-08
</commit_message>
<xml_diff>
--- a/data/anime_list.xlsx
+++ b/data/anime_list.xlsx
@@ -7132,7 +7132,7 @@
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t>2026年7月～ 日本テレビ系にて</t>
+          <t>2026年7月3日（金）～ 日本テレビ系にて</t>
         </is>
       </c>
       <c r="H123" t="inlineStr">
@@ -7140,8 +7140,16 @@
           <t>シンエイ動画</t>
         </is>
       </c>
-      <c r="I123" t="inlineStr"/>
-      <c r="J123" t="inlineStr"/>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>遺書</t>
+        </is>
+      </c>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t>キタニタツヤ</t>
+        </is>
+      </c>
       <c r="K123" t="inlineStr"/>
       <c r="L123" t="inlineStr"/>
       <c r="M123" t="inlineStr">
@@ -9297,7 +9305,7 @@
       </c>
       <c r="G168" t="inlineStr">
         <is>
-          <t>2026年7月～ TOKYO MX・BS朝日ほか</t>
+          <t>2026年7月2日（木）～ TOKYO MX・BS朝日ほか</t>
         </is>
       </c>
       <c r="H168" t="inlineStr">
@@ -9305,8 +9313,16 @@
           <t>サイピク</t>
         </is>
       </c>
-      <c r="I168" t="inlineStr"/>
-      <c r="J168" t="inlineStr"/>
+      <c r="I168" t="inlineStr">
+        <is>
+          <t>終宵</t>
+        </is>
+      </c>
+      <c r="J168" t="inlineStr">
+        <is>
+          <t>マカロニえんぴつ</t>
+        </is>
+      </c>
       <c r="K168" t="inlineStr"/>
       <c r="L168" t="inlineStr"/>
       <c r="M168" t="inlineStr">
@@ -9367,7 +9383,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L216"/>
+  <dimension ref="A1:L218"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18991,7 +19007,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>サイボーグ009 ネメシス</t>
+          <t>これ描いて死ね</t>
         </is>
       </c>
       <c r="D194" t="b">
@@ -18999,7 +19015,7 @@
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t>主題歌</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F194" t="n">
@@ -19007,12 +19023,12 @@
       </c>
       <c r="G194" t="inlineStr">
         <is>
-          <t>誰がために</t>
+          <t>遺書</t>
         </is>
       </c>
       <c r="H194" t="inlineStr">
         <is>
-          <t>杏子</t>
+          <t>キタニタツヤ</t>
         </is>
       </c>
       <c r="I194" t="inlineStr"/>
@@ -19031,7 +19047,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>さよならララ</t>
+          <t>サイボーグ009 ネメシス</t>
         </is>
       </c>
       <c r="D195" t="b">
@@ -19039,7 +19055,7 @@
       </c>
       <c r="E195" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>主題歌</t>
         </is>
       </c>
       <c r="F195" t="n">
@@ -19047,12 +19063,12 @@
       </c>
       <c r="G195" t="inlineStr">
         <is>
-          <t>さよならララ</t>
+          <t>誰がために</t>
         </is>
       </c>
       <c r="H195" t="inlineStr">
         <is>
-          <t>いきものがかり</t>
+          <t>杏子</t>
         </is>
       </c>
       <c r="I195" t="inlineStr"/>
@@ -19071,7 +19087,7 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>スーパーの裏でヤニ吸うふたり</t>
+          <t>さよならララ</t>
         </is>
       </c>
       <c r="D196" t="b">
@@ -19079,7 +19095,7 @@
       </c>
       <c r="E196" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F196" t="n">
@@ -19087,12 +19103,12 @@
       </c>
       <c r="G196" t="inlineStr">
         <is>
-          <t>Fiction</t>
+          <t>さよならララ</t>
         </is>
       </c>
       <c r="H196" t="inlineStr">
         <is>
-          <t>imase</t>
+          <t>いきものがかり</t>
         </is>
       </c>
       <c r="I196" t="inlineStr"/>
@@ -19111,7 +19127,7 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>正反対な君と僕 第2期</t>
+          <t>スーパーの裏でヤニ吸うふたり</t>
         </is>
       </c>
       <c r="D197" t="b">
@@ -19119,7 +19135,7 @@
       </c>
       <c r="E197" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F197" t="n">
@@ -19127,12 +19143,12 @@
       </c>
       <c r="G197" t="inlineStr">
         <is>
-          <t>メガネを外して</t>
+          <t>Fiction</t>
         </is>
       </c>
       <c r="H197" t="inlineStr">
         <is>
-          <t>乃紫</t>
+          <t>imase</t>
         </is>
       </c>
       <c r="I197" t="inlineStr"/>
@@ -19159,7 +19175,7 @@
       </c>
       <c r="E198" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F198" t="n">
@@ -19167,12 +19183,12 @@
       </c>
       <c r="G198" t="inlineStr">
         <is>
-          <t>ピュア feat. 橋本絵莉子</t>
+          <t>メガネを外して</t>
         </is>
       </c>
       <c r="H198" t="inlineStr">
         <is>
-          <t>PAS TASTA</t>
+          <t>乃紫</t>
         </is>
       </c>
       <c r="I198" t="inlineStr"/>
@@ -19191,7 +19207,7 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>対ありでした。～お嬢さまは格闘ゲームなんてしない～</t>
+          <t>正反対な君と僕 第2期</t>
         </is>
       </c>
       <c r="D199" t="b">
@@ -19199,7 +19215,7 @@
       </c>
       <c r="E199" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F199" t="n">
@@ -19207,12 +19223,12 @@
       </c>
       <c r="G199" t="inlineStr">
         <is>
-          <t>命短し対する乙女よ</t>
+          <t>ピュア feat. 橋本絵莉子</t>
         </is>
       </c>
       <c r="H199" t="inlineStr">
         <is>
-          <t>花冷え。</t>
+          <t>PAS TASTA</t>
         </is>
       </c>
       <c r="I199" t="inlineStr"/>
@@ -19231,7 +19247,7 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>手札が多めのビクトリア</t>
+          <t>対ありでした。～お嬢さまは格闘ゲームなんてしない～</t>
         </is>
       </c>
       <c r="D200" t="b">
@@ -19239,7 +19255,7 @@
       </c>
       <c r="E200" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F200" t="n">
@@ -19247,12 +19263,12 @@
       </c>
       <c r="G200" t="inlineStr">
         <is>
-          <t>縁のつき</t>
+          <t>命短し対する乙女よ</t>
         </is>
       </c>
       <c r="H200" t="inlineStr">
         <is>
-          <t>KI_EN</t>
+          <t>花冷え。</t>
         </is>
       </c>
       <c r="I200" t="inlineStr"/>
@@ -19271,7 +19287,7 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>転校先の清楚可憐な美少女が、昔男子と思って一緒に遊んだ幼馴染だった件</t>
+          <t>手札が多めのビクトリア</t>
         </is>
       </c>
       <c r="D201" t="b">
@@ -19279,7 +19295,7 @@
       </c>
       <c r="E201" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F201" t="n">
@@ -19287,12 +19303,12 @@
       </c>
       <c r="G201" t="inlineStr">
         <is>
-          <t>夏に重ねて</t>
+          <t>縁のつき</t>
         </is>
       </c>
       <c r="H201" t="inlineStr">
         <is>
-          <t>DIALOGUE+</t>
+          <t>KI_EN</t>
         </is>
       </c>
       <c r="I201" t="inlineStr"/>
@@ -19311,7 +19327,7 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>天は赤い河のほとり</t>
+          <t>転校先の清楚可憐な美少女が、昔男子と思って一緒に遊んだ幼馴染だった件</t>
         </is>
       </c>
       <c r="D202" t="b">
@@ -19327,12 +19343,12 @@
       </c>
       <c r="G202" t="inlineStr">
         <is>
-          <t>暁の空</t>
+          <t>夏に重ねて</t>
         </is>
       </c>
       <c r="H202" t="inlineStr">
         <is>
-          <t>七海ひろき</t>
+          <t>DIALOGUE+</t>
         </is>
       </c>
       <c r="I202" t="inlineStr"/>
@@ -19351,7 +19367,7 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>盗掘王</t>
+          <t>天は赤い河のほとり</t>
         </is>
       </c>
       <c r="D203" t="b">
@@ -19367,12 +19383,12 @@
       </c>
       <c r="G203" t="inlineStr">
         <is>
-          <t>SHOW DOWN</t>
+          <t>暁の空</t>
         </is>
       </c>
       <c r="H203" t="inlineStr">
         <is>
-          <t>QWER</t>
+          <t>七海ひろき</t>
         </is>
       </c>
       <c r="I203" t="inlineStr"/>
@@ -19391,7 +19407,7 @@
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>透明な夜に駆ける君と、目に見えない恋をした。</t>
+          <t>盗掘王</t>
         </is>
       </c>
       <c r="D204" t="b">
@@ -19399,7 +19415,7 @@
       </c>
       <c r="E204" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F204" t="n">
@@ -19407,12 +19423,12 @@
       </c>
       <c r="G204" t="inlineStr">
         <is>
-          <t>光</t>
+          <t>SHOW DOWN</t>
         </is>
       </c>
       <c r="H204" t="inlineStr">
         <is>
-          <t>櫻井優衣</t>
+          <t>QWER</t>
         </is>
       </c>
       <c r="I204" t="inlineStr"/>
@@ -19431,7 +19447,7 @@
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>二十世紀電氣目録-ユーレカ・エヴリカ-</t>
+          <t>透明な夜に駆ける君と、目に見えない恋をした。</t>
         </is>
       </c>
       <c r="D205" t="b">
@@ -19439,7 +19455,7 @@
       </c>
       <c r="E205" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F205" t="n">
@@ -19447,12 +19463,12 @@
       </c>
       <c r="G205" t="inlineStr">
         <is>
-          <t>ユーレカ・エヴリカ</t>
+          <t>光</t>
         </is>
       </c>
       <c r="H205" t="inlineStr">
         <is>
-          <t>五阿弥ルナ</t>
+          <t>櫻井優衣</t>
         </is>
       </c>
       <c r="I205" t="inlineStr"/>
@@ -19471,7 +19487,7 @@
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>ブチ切れ令嬢は報復を誓いました。 ～魔導書の力で祖国を叩き潰します～</t>
+          <t>二十世紀電氣目録-ユーレカ・エヴリカ-</t>
         </is>
       </c>
       <c r="D206" t="b">
@@ -19487,12 +19503,12 @@
       </c>
       <c r="G206" t="inlineStr">
         <is>
-          <t>Q.E.D.</t>
+          <t>ユーレカ・エヴリカ</t>
         </is>
       </c>
       <c r="H206" t="inlineStr">
         <is>
-          <t>小倉唯</t>
+          <t>五阿弥ルナ</t>
         </is>
       </c>
       <c r="I206" t="inlineStr"/>
@@ -19519,7 +19535,7 @@
       </c>
       <c r="E207" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F207" t="n">
@@ -19527,12 +19543,12 @@
       </c>
       <c r="G207" t="inlineStr">
         <is>
-          <t>グッバイ・ララバイ</t>
+          <t>Q.E.D.</t>
         </is>
       </c>
       <c r="H207" t="inlineStr">
         <is>
-          <t>大西亜玖璃</t>
+          <t>小倉唯</t>
         </is>
       </c>
       <c r="I207" t="inlineStr"/>
@@ -19551,7 +19567,7 @@
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>プラノサウルス ガチコセイブツ部</t>
+          <t>ブチ切れ令嬢は報復を誓いました。 ～魔導書の力で祖国を叩き潰します～</t>
         </is>
       </c>
       <c r="D208" t="b">
@@ -19559,7 +19575,7 @@
       </c>
       <c r="E208" t="inlineStr">
         <is>
-          <t>主題歌</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F208" t="n">
@@ -19567,12 +19583,12 @@
       </c>
       <c r="G208" t="inlineStr">
         <is>
-          <t>ガチde古生</t>
+          <t>グッバイ・ララバイ</t>
         </is>
       </c>
       <c r="H208" t="inlineStr">
         <is>
-          <t>リンクルプラネット</t>
+          <t>大西亜玖璃</t>
         </is>
       </c>
       <c r="I208" t="inlineStr"/>
@@ -19591,7 +19607,7 @@
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>炎の闘球女 ドッジ弾子</t>
+          <t>プラノサウルス ガチコセイブツ部</t>
         </is>
       </c>
       <c r="D209" t="b">
@@ -19599,7 +19615,7 @@
       </c>
       <c r="E209" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>主題歌</t>
         </is>
       </c>
       <c r="F209" t="n">
@@ -19607,12 +19623,12 @@
       </c>
       <c r="G209" t="inlineStr">
         <is>
-          <t>Welcome to あざとさワールド</t>
+          <t>ガチde古生</t>
         </is>
       </c>
       <c r="H209" t="inlineStr">
         <is>
-          <t>i☆Ris</t>
+          <t>リンクルプラネット</t>
         </is>
       </c>
       <c r="I209" t="inlineStr"/>
@@ -19631,7 +19647,7 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>魔法少女リリカルなのは EXCEEDS Gun Blaze Vengeance</t>
+          <t>炎の闘球女 ドッジ弾子</t>
         </is>
       </c>
       <c r="D210" t="b">
@@ -19647,12 +19663,12 @@
       </c>
       <c r="G210" t="inlineStr">
         <is>
-          <t>Ephemeral</t>
+          <t>Welcome to あざとさワールド</t>
         </is>
       </c>
       <c r="H210" t="inlineStr">
         <is>
-          <t>青木陽菜</t>
+          <t>i☆Ris</t>
         </is>
       </c>
       <c r="I210" t="inlineStr"/>
@@ -19671,7 +19687,7 @@
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>無自覚聖女は今日も無意識に力を垂れ流す</t>
+          <t>魔法少女リリカルなのは EXCEEDS Gun Blaze Vengeance</t>
         </is>
       </c>
       <c r="D211" t="b">
@@ -19679,7 +19695,7 @@
       </c>
       <c r="E211" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F211" t="n">
@@ -19687,12 +19703,12 @@
       </c>
       <c r="G211" t="inlineStr">
         <is>
-          <t>Windmaker</t>
+          <t>Ephemeral</t>
         </is>
       </c>
       <c r="H211" t="inlineStr">
         <is>
-          <t>花耶</t>
+          <t>青木陽菜</t>
         </is>
       </c>
       <c r="I211" t="inlineStr"/>
@@ -19711,7 +19727,7 @@
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>無職転生Ⅲ ～異世界行ったら本気だす～</t>
+          <t>無自覚聖女は今日も無意識に力を垂れ流す</t>
         </is>
       </c>
       <c r="D212" t="b">
@@ -19727,12 +19743,12 @@
       </c>
       <c r="G212" t="inlineStr">
         <is>
-          <t>決意の唄</t>
+          <t>Windmaker</t>
         </is>
       </c>
       <c r="H212" t="inlineStr">
         <is>
-          <t>大原ゆい子</t>
+          <t>花耶</t>
         </is>
       </c>
       <c r="I212" t="inlineStr"/>
@@ -19751,7 +19767,7 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>鎧真伝サムライトルーパー 第2クール</t>
+          <t>無職転生Ⅲ ～異世界行ったら本気だす～</t>
         </is>
       </c>
       <c r="D213" t="b">
@@ -19767,12 +19783,12 @@
       </c>
       <c r="G213" t="inlineStr">
         <is>
-          <t>YOAKE</t>
+          <t>決意の唄</t>
         </is>
       </c>
       <c r="H213" t="inlineStr">
         <is>
-          <t>blank paper</t>
+          <t>大原ゆい子</t>
         </is>
       </c>
       <c r="I213" t="inlineStr"/>
@@ -19799,7 +19815,7 @@
       </c>
       <c r="E214" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F214" t="n">
@@ -19807,12 +19823,12 @@
       </c>
       <c r="G214" t="inlineStr">
         <is>
-          <t>POWER</t>
+          <t>YOAKE</t>
         </is>
       </c>
       <c r="H214" t="inlineStr">
         <is>
-          <t>ONE OR EIGHT</t>
+          <t>blank paper</t>
         </is>
       </c>
       <c r="I214" t="inlineStr"/>
@@ -19831,7 +19847,7 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>令和のダラさん</t>
+          <t>鎧真伝サムライトルーパー 第2クール</t>
         </is>
       </c>
       <c r="D215" t="b">
@@ -19839,7 +19855,7 @@
       </c>
       <c r="E215" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F215" t="n">
@@ -19847,12 +19863,12 @@
       </c>
       <c r="G215" t="inlineStr">
         <is>
-          <t>ダラダラ♡ダンシング</t>
+          <t>POWER</t>
         </is>
       </c>
       <c r="H215" t="inlineStr">
         <is>
-          <t>ダラさん（CV：田村睦心） 三⼗⽊⾕⽇向（CV：津田美波） 三⼗⽊⾕薫（CV：寺澤百花） ナレーション（CV：てらそままさき）</t>
+          <t>ONE OR EIGHT</t>
         </is>
       </c>
       <c r="I215" t="inlineStr"/>
@@ -19871,7 +19887,7 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>LV999の村人</t>
+          <t>令和のダラさん</t>
         </is>
       </c>
       <c r="D216" t="b">
@@ -19887,12 +19903,12 @@
       </c>
       <c r="G216" t="inlineStr">
         <is>
-          <t>Not a Hero</t>
+          <t>ダラダラ♡ダンシング</t>
         </is>
       </c>
       <c r="H216" t="inlineStr">
         <is>
-          <t>藍月なくる&amp;棗いつき</t>
+          <t>ダラさん（CV：田村睦心） 三⼗⽊⾕⽇向（CV：津田美波） 三⼗⽊⾕薫（CV：寺澤百花） ナレーション（CV：てらそままさき）</t>
         </is>
       </c>
       <c r="I216" t="inlineStr"/>
@@ -19900,6 +19916,86 @@
       <c r="K216" t="inlineStr"/>
       <c r="L216" t="inlineStr"/>
     </row>
+    <row r="217">
+      <c r="A217" t="n">
+        <v>5806</v>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>2026夏アニメ</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>LV999の村人</t>
+        </is>
+      </c>
+      <c r="D217" t="b">
+        <v>0</v>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="F217" t="n">
+        <v>1</v>
+      </c>
+      <c r="G217" t="inlineStr">
+        <is>
+          <t>Not a Hero</t>
+        </is>
+      </c>
+      <c r="H217" t="inlineStr">
+        <is>
+          <t>藍月なくる&amp;棗いつき</t>
+        </is>
+      </c>
+      <c r="I217" t="inlineStr"/>
+      <c r="J217" t="inlineStr"/>
+      <c r="K217" t="inlineStr"/>
+      <c r="L217" t="inlineStr"/>
+    </row>
+    <row r="218">
+      <c r="A218" t="n">
+        <v>5806</v>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>2026夏アニメ</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>ワールド イズ ダンシング</t>
+        </is>
+      </c>
+      <c r="D218" t="b">
+        <v>0</v>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="F218" t="n">
+        <v>1</v>
+      </c>
+      <c r="G218" t="inlineStr">
+        <is>
+          <t>終宵</t>
+        </is>
+      </c>
+      <c r="H218" t="inlineStr">
+        <is>
+          <t>マカロニえんぴつ</t>
+        </is>
+      </c>
+      <c r="I218" t="inlineStr"/>
+      <c r="J218" t="inlineStr"/>
+      <c r="K218" t="inlineStr"/>
+      <c r="L218" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
auto: anime list update 2026-05-10
</commit_message>
<xml_diff>
--- a/data/anime_list.xlsx
+++ b/data/anime_list.xlsx
@@ -9483,24 +9483,10 @@
           <t>CHiCO with HoneyWorks</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=2tqTCYjznf0</t>
-        </is>
-      </c>
-      <c r="J2" t="n">
-        <v>46621</v>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>日活アニメチャンネル</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>2026-05-03T10:26:09</t>
-        </is>
-      </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -9537,24 +9523,10 @@
           <t>PompadollS</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=Idz-Bcjh95c</t>
-        </is>
-      </c>
-      <c r="J3" t="n">
-        <v>41037</v>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>PompadollS</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>2026-05-03T10:26:18</t>
-        </is>
-      </c>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -9751,24 +9723,10 @@
           <t>桑田佳祐</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=lBOmiR_1CGQ</t>
-        </is>
-      </c>
-      <c r="J8" t="n">
-        <v>2034617</v>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>桑田佳祐</t>
-        </is>
-      </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>2026-05-03T10:26:27</t>
-        </is>
-      </c>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -9805,24 +9763,10 @@
           <t>桑田佳祐</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=lBOmiR_1CGQ</t>
-        </is>
-      </c>
-      <c r="J9" t="n">
-        <v>2034617</v>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>桑田佳祐</t>
-        </is>
-      </c>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t>2026-05-03T10:26:37</t>
-        </is>
-      </c>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -9939,24 +9883,10 @@
           <t>HanaHope</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=eTeTEuwu_8c</t>
-        </is>
-      </c>
-      <c r="J12" t="n">
-        <v>115354</v>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>KADOKAWAanime</t>
-        </is>
-      </c>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>2026-05-03T10:26:46</t>
-        </is>
-      </c>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -9993,24 +9923,10 @@
           <t>中島美嘉</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=BNXqkwbfakg</t>
-        </is>
-      </c>
-      <c r="J13" t="n">
-        <v>44161</v>
-      </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>中島美嘉 Official YouTube Channel</t>
-        </is>
-      </c>
-      <c r="L13" t="inlineStr">
-        <is>
-          <t>2026-05-03T10:26:55</t>
-        </is>
-      </c>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -10127,24 +10043,10 @@
           <t>ルールーシー＝ルー（CV.下地紫野）＆ティア（CV.洲崎綾)</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=EMhgPcxCz9I</t>
-        </is>
-      </c>
-      <c r="J16" t="n">
-        <v>135897</v>
-      </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>ぽにきゃん-Anime PONY CANYON</t>
-        </is>
-      </c>
-      <c r="L16" t="inlineStr">
-        <is>
-          <t>2026-05-03T10:27:20</t>
-        </is>
-      </c>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -10181,24 +10083,10 @@
           <t>緋月ゆい</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=40K8d9oveiY</t>
-        </is>
-      </c>
-      <c r="J17" t="n">
-        <v>49858</v>
-      </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>ぽにきゃん-Anime PONY CANYON</t>
-        </is>
-      </c>
-      <c r="L17" t="inlineStr">
-        <is>
-          <t>2026-05-03T10:27:29</t>
-        </is>
-      </c>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -10235,24 +10123,10 @@
           <t>Sophià la Mode</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=3Psx5SclWFI</t>
-        </is>
-      </c>
-      <c r="J18" t="n">
-        <v>18119</v>
-      </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>NBCUniversal Anime/Music</t>
-        </is>
-      </c>
-      <c r="L18" t="inlineStr">
-        <is>
-          <t>2026-05-03T10:27:38</t>
-        </is>
-      </c>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -10289,24 +10163,10 @@
           <t>夢限大みゅーたいぷ</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=1ApeGKiI-FQ</t>
-        </is>
-      </c>
-      <c r="J19" t="n">
-        <v>6419</v>
-      </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>夢限大みゅーたいぷ</t>
-        </is>
-      </c>
-      <c r="L19" t="inlineStr">
-        <is>
-          <t>2026-05-03T10:27:45</t>
-        </is>
-      </c>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">

</xml_diff>

<commit_message>
auto: anime list update 2026-06-02
</commit_message>
<xml_diff>
--- a/data/anime_list.xlsx
+++ b/data/anime_list.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M119"/>
+  <dimension ref="A1:M122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2800,7 +2800,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>刃牙道 第2クール</t>
+          <t>パイの実 おしの森へようこそ！</t>
         </is>
       </c>
       <c r="E48" t="b">
@@ -2813,37 +2813,21 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>第1クール：2026年2月26日（木）〜 第2クール：2026年6月18日（木）～ Netflixにて 【TV放送】 2026年～</t>
+          <t>2026年6月4日（木）～ お口の恋人ロッテ【LOTTE】公式チャンネルにて</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>トムス・エンタテインメント</t>
-        </is>
-      </c>
-      <c r="I48" t="inlineStr">
-        <is>
-          <t>フルボコ</t>
-        </is>
-      </c>
-      <c r="J48" t="inlineStr">
-        <is>
-          <t>WANIMA</t>
-        </is>
-      </c>
-      <c r="K48" t="inlineStr">
-        <is>
-          <t>Mountain Top</t>
-        </is>
-      </c>
-      <c r="L48" t="inlineStr">
-        <is>
-          <t>Novel Core</t>
-        </is>
-      </c>
+          <t>TOHO animation STUDIO</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr"/>
+      <c r="J48" t="inlineStr"/>
+      <c r="K48" t="inlineStr"/>
+      <c r="L48" t="inlineStr"/>
       <c r="M48" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=23828</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28459</t>
         </is>
       </c>
     </row>
@@ -2861,7 +2845,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>花織さんは転生しても喧嘩がしたい</t>
+          <t>刃牙道 第2クール</t>
         </is>
       </c>
       <c r="E49" t="b">
@@ -2869,26 +2853,42 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>TVアニメ</t>
+          <t>配信</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>2026年7月～ ABCテレビ・テレビ朝日系・BS日テレにて</t>
+          <t>第1クール：2026年2月26日（木）〜 第2クール：2026年6月18日（木）～ Netflixにて 【TV放送】 2026年～</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>ライデンフィルム</t>
-        </is>
-      </c>
-      <c r="I49" t="inlineStr"/>
-      <c r="J49" t="inlineStr"/>
-      <c r="K49" t="inlineStr"/>
-      <c r="L49" t="inlineStr"/>
+          <t>トムス・エンタテインメント</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>フルボコ</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>WANIMA</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>Mountain Top</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>Novel Core</t>
+        </is>
+      </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26828</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=23828</t>
         </is>
       </c>
     </row>
@@ -2906,7 +2906,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>花ざかりの君たちへ 第2期</t>
+          <t>花織さんは転生しても喧嘩がしたい</t>
         </is>
       </c>
       <c r="E50" t="b">
@@ -2919,37 +2919,21 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>2026年7月1日（水）～ TOKYO MX・BS11ほか</t>
+          <t>2026年7月～ ABCテレビ・テレビ朝日系・BS日テレにて</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>シグナル・エムディ（</t>
-        </is>
-      </c>
-      <c r="I50" t="inlineStr">
-        <is>
-          <t>FLASHBULB</t>
-        </is>
-      </c>
-      <c r="J50" t="inlineStr">
-        <is>
-          <t>Omoinotake</t>
-        </is>
-      </c>
-      <c r="K50" t="inlineStr">
-        <is>
-          <t>花束</t>
-        </is>
-      </c>
-      <c r="L50" t="inlineStr">
-        <is>
-          <t>Omoinotake</t>
-        </is>
-      </c>
+          <t>ライデンフィルム</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr"/>
+      <c r="J50" t="inlineStr"/>
+      <c r="K50" t="inlineStr"/>
+      <c r="L50" t="inlineStr"/>
       <c r="M50" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27990</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26828</t>
         </is>
       </c>
     </row>
@@ -2967,7 +2951,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>バンドリ！ ゆめ∞みた</t>
+          <t>花ざかりの君たちへ 第2期</t>
         </is>
       </c>
       <c r="E51" t="b">
@@ -2980,21 +2964,37 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>2026年7月2日（木）～ TOKYO MXほか</t>
+          <t>2026年7月1日（水）～ TOKYO MX・BS11ほか</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>ニチカライン（</t>
-        </is>
-      </c>
-      <c r="I51" t="inlineStr"/>
-      <c r="J51" t="inlineStr"/>
-      <c r="K51" t="inlineStr"/>
-      <c r="L51" t="inlineStr"/>
+          <t>シグナル・エムディ（</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>FLASHBULB</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>Omoinotake</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>花束</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>Omoinotake</t>
+        </is>
+      </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26737</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27990</t>
         </is>
       </c>
     </row>
@@ -3012,7 +3012,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>パンの赤ちゃん</t>
+          <t>バンドリ！ ゆめ∞みた</t>
         </is>
       </c>
       <c r="E52" t="b">
@@ -3025,17 +3025,21 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>2026年7月4日（土）～ カンテレ・フジテレビ系列「土曜はナニする！？」にて</t>
-        </is>
-      </c>
-      <c r="H52" t="inlineStr"/>
+          <t>2026年7月2日（木）～ TOKYO MXほか</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>ニチカライン（</t>
+        </is>
+      </c>
       <c r="I52" t="inlineStr"/>
       <c r="J52" t="inlineStr"/>
       <c r="K52" t="inlineStr"/>
       <c r="L52" t="inlineStr"/>
       <c r="M52" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25145</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26737</t>
         </is>
       </c>
     </row>
@@ -3053,7 +3057,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>ヒロイン？聖女？いいえ、オールワークスメイドです（誇）！</t>
+          <t>パンの赤ちゃん</t>
         </is>
       </c>
       <c r="E53" t="b">
@@ -3066,37 +3070,17 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>2026年7月1日（水）～ TOKYO MX・BSフジほか</t>
-        </is>
-      </c>
-      <c r="H53" t="inlineStr">
-        <is>
-          <t>EMTスクエアード</t>
-        </is>
-      </c>
-      <c r="I53" t="inlineStr">
-        <is>
-          <t>マデュアル↔ハート</t>
-        </is>
-      </c>
-      <c r="J53" t="inlineStr">
-        <is>
-          <t>メロディ・ウェーブ(CV：宮本侑芽) ルシアナ・ルトルバーグ(CV：大久保瑠美)</t>
-        </is>
-      </c>
-      <c r="K53" t="inlineStr">
-        <is>
-          <t>ハンドメイド</t>
-        </is>
-      </c>
-      <c r="L53" t="inlineStr">
-        <is>
-          <t>仲村宗悟</t>
-        </is>
-      </c>
+          <t>2026年7月4日（土）～ カンテレ・フジテレビ系列「土曜はナニする！？」にて</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr"/>
+      <c r="I53" t="inlineStr"/>
+      <c r="J53" t="inlineStr"/>
+      <c r="K53" t="inlineStr"/>
+      <c r="L53" t="inlineStr"/>
       <c r="M53" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25936</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25145</t>
         </is>
       </c>
     </row>
@@ -3114,7 +3098,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>ブチ切れ令嬢は報復を誓いました。 ～魔導書の力で祖国を叩き潰します～</t>
+          <t>ヒロイン？聖女？いいえ、オールワークスメイドです（誇）！</t>
         </is>
       </c>
       <c r="E54" t="b">
@@ -3127,37 +3111,37 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>2026年7月〜 テレ東・BS11ほか</t>
+          <t>2026年7月1日（水）～ TOKYO MX・BSフジほか</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>スタジオコメット</t>
+          <t>EMTスクエアード</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>Q.E.D.</t>
+          <t>マデュアル↔ハート</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>小倉唯</t>
+          <t>メロディ・ウェーブ(CV：宮本侑芽) ルシアナ・ルトルバーグ(CV：大久保瑠美)</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>グッバイ・ララバイ</t>
+          <t>ハンドメイド</t>
         </is>
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>大西亜玖璃</t>
+          <t>仲村宗悟</t>
         </is>
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27366</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25936</t>
         </is>
       </c>
     </row>
@@ -3175,7 +3159,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>ふつつかな悪女ではございますが～雛宮蝶鼠とりかえ伝～</t>
+          <t>ブチ切れ令嬢は報復を誓いました。 ～魔導書の力で祖国を叩き潰します～</t>
         </is>
       </c>
       <c r="E55" t="b">
@@ -3188,21 +3172,37 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>2026年7月12日（日）〜 テレビ東京系列にて</t>
+          <t>2026年7月〜 テレ東・BS11ほか</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>動画工房</t>
-        </is>
-      </c>
-      <c r="I55" t="inlineStr"/>
-      <c r="J55" t="inlineStr"/>
-      <c r="K55" t="inlineStr"/>
-      <c r="L55" t="inlineStr"/>
+          <t>スタジオコメット</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>Q.E.D.</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>小倉唯</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>グッバイ・ララバイ</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>大西亜玖璃</t>
+        </is>
+      </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25702</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27366</t>
         </is>
       </c>
     </row>
@@ -3220,7 +3220,7 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>BLACK TORCH</t>
+          <t>ふつつかな悪女ではございますが～雛宮蝶鼠とりかえ伝～</t>
         </is>
       </c>
       <c r="E56" t="b">
@@ -3233,12 +3233,12 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>2026年7月4日（土）～ TOKYO MXほか</t>
+          <t>2026年7月12日（日）〜 テレビ東京系列にて</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>100studio</t>
+          <t>動画工房</t>
         </is>
       </c>
       <c r="I56" t="inlineStr"/>
@@ -3247,7 +3247,7 @@
       <c r="L56" t="inlineStr"/>
       <c r="M56" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25641</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25702</t>
         </is>
       </c>
     </row>
@@ -3265,7 +3265,7 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>プラノサウルス ガチコセイブツ部</t>
+          <t>BLACK TORCH</t>
         </is>
       </c>
       <c r="E57" t="b">
@@ -3278,12 +3278,12 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>2026年7月～ テレ東系列6局ネット「アニもり！」内にて</t>
+          <t>2026年7月4日（土）～ TOKYO MXほか</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>SMDE</t>
+          <t>100studio</t>
         </is>
       </c>
       <c r="I57" t="inlineStr"/>
@@ -3292,7 +3292,7 @@
       <c r="L57" t="inlineStr"/>
       <c r="M57" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27895</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25641</t>
         </is>
       </c>
     </row>
@@ -3310,7 +3310,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>BLEACH 千年血戦篇-禍進譚-</t>
+          <t>プラノサウルス ガチコセイブツ部</t>
         </is>
       </c>
       <c r="E58" t="b">
@@ -3323,12 +3323,12 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>2026年7月～ テレ東系列ほか</t>
+          <t>2026年7月～ テレ東系列6局ネット「アニもり！」内にて</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>PIERROT FILMS（</t>
+          <t>SMDE</t>
         </is>
       </c>
       <c r="I58" t="inlineStr"/>
@@ -3337,7 +3337,7 @@
       <c r="L58" t="inlineStr"/>
       <c r="M58" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25417</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27895</t>
         </is>
       </c>
     </row>
@@ -3355,7 +3355,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>文豪ストレイドッグス わん！２</t>
+          <t>BLEACH 千年血戦篇-禍進譚-</t>
         </is>
       </c>
       <c r="E59" t="b">
@@ -3368,12 +3368,12 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>2026年7月〜</t>
+          <t>2026年7月～ テレ東系列ほか</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>ボンズ</t>
+          <t>PIERROT FILMS（</t>
         </is>
       </c>
       <c r="I59" t="inlineStr"/>
@@ -3382,7 +3382,7 @@
       <c r="L59" t="inlineStr"/>
       <c r="M59" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27057</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25417</t>
         </is>
       </c>
     </row>
@@ -3400,7 +3400,7 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>ヘルモード ～やり込み好きのゲーマーは廃設定の異世界で無双する～ 2nd Season</t>
+          <t>文豪ストレイドッグス わん！２</t>
         </is>
       </c>
       <c r="E60" t="b">
@@ -3413,17 +3413,21 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>2026年7月～ TOKYO MX・MBS・BS日テレにて</t>
-        </is>
-      </c>
-      <c r="H60" t="inlineStr"/>
+          <t>2026年7月〜</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>ボンズ</t>
+        </is>
+      </c>
       <c r="I60" t="inlineStr"/>
       <c r="J60" t="inlineStr"/>
       <c r="K60" t="inlineStr"/>
       <c r="L60" t="inlineStr"/>
       <c r="M60" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28020</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27057</t>
         </is>
       </c>
     </row>
@@ -3441,7 +3445,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>炎の闘球女 ドッジ弾子</t>
+          <t>ヘルモード ～やり込み好きのゲーマーは廃設定の異世界で無双する～ 2nd Season</t>
         </is>
       </c>
       <c r="E61" t="b">
@@ -3454,29 +3458,17 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>2026年7月～ TOKYO MX・MBS・BS11にて</t>
-        </is>
-      </c>
-      <c r="H61" t="inlineStr">
-        <is>
-          <t>CUE</t>
-        </is>
-      </c>
+          <t>2026年7月～ TOKYO MX・MBS・BS日テレにて</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr"/>
       <c r="I61" t="inlineStr"/>
       <c r="J61" t="inlineStr"/>
-      <c r="K61" t="inlineStr">
-        <is>
-          <t>Welcome to あざとさワールド</t>
-        </is>
-      </c>
-      <c r="L61" t="inlineStr">
-        <is>
-          <t>i☆Ris</t>
-        </is>
-      </c>
+      <c r="K61" t="inlineStr"/>
+      <c r="L61" t="inlineStr"/>
       <c r="M61" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26401</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28020</t>
         </is>
       </c>
     </row>
@@ -3494,7 +3486,7 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>魔法少女リリカルなのは EXCEEDS Gun Blaze Vengeance</t>
+          <t>炎の闘球女 ドッジ弾子</t>
         </is>
       </c>
       <c r="E62" t="b">
@@ -3507,37 +3499,37 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>2026年7月4日（土）～ TOKYO MX・BS11にて</t>
+          <t>2026年7月6日（月）～ TOKYO MX・MBS・BS11にて</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>Seven Arcs</t>
+          <t>CUE</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>CRIMSON BULLET</t>
+          <t>会心の一劇</t>
         </is>
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>水樹奈々</t>
+          <t>ももいろクローバーZ</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
         <is>
-          <t>Ephemeral</t>
+          <t>Welcome to あざとさワールド</t>
         </is>
       </c>
       <c r="L62" t="inlineStr">
         <is>
-          <t>青木陽菜</t>
+          <t>i☆Ris</t>
         </is>
       </c>
       <c r="M62" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25418</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26401</t>
         </is>
       </c>
     </row>
@@ -3555,7 +3547,7 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>身代わり令嬢を救ったのは冷酷無慈悲な氷の王子の愛でした</t>
+          <t>魔法少女リリカルなのは EXCEEDS Gun Blaze Vengeance</t>
         </is>
       </c>
       <c r="E63" t="b">
@@ -3568,21 +3560,37 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>2026年7月～ TVKにて</t>
+          <t>2026年7月4日（土）～ TOKYO MX・BS11にて</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>Imagica Infos</t>
-        </is>
-      </c>
-      <c r="I63" t="inlineStr"/>
-      <c r="J63" t="inlineStr"/>
-      <c r="K63" t="inlineStr"/>
-      <c r="L63" t="inlineStr"/>
+          <t>Seven Arcs</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>CRIMSON BULLET</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>水樹奈々</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>Ephemeral</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>青木陽菜</t>
+        </is>
+      </c>
       <c r="M63" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28112</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25418</t>
         </is>
       </c>
     </row>
@@ -3600,7 +3608,7 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>無自覚聖女は今日も無意識に力を垂れ流す</t>
+          <t>身代わり令嬢を救ったのは冷酷無慈悲な氷の王子の愛でした</t>
         </is>
       </c>
       <c r="E64" t="b">
@@ -3613,37 +3621,21 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>2026年7月～ TOKYO MX・BS11・AT-Xにて</t>
+          <t>2026年7月～ TVKにて</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>マジックバス×ピカンテサーカス</t>
-        </is>
-      </c>
-      <c r="I64" t="inlineStr">
-        <is>
-          <t>Windmaker</t>
-        </is>
-      </c>
-      <c r="J64" t="inlineStr">
-        <is>
-          <t>花耶</t>
-        </is>
-      </c>
-      <c r="K64" t="inlineStr">
-        <is>
-          <t>アンノウンミー</t>
-        </is>
-      </c>
-      <c r="L64" t="inlineStr">
-        <is>
-          <t>ウタヒメドリーム オールスターズ【夢咲いぶき（CV:山﨑玲奈） 桜木舞華（CV:鈴木杏奈） 真白清美（CV:其原有沙） HiREN（CV:花耶） 水月ひかり（CV:礒部花凜） 高木凛（CV:鷲見友美ジェナ） 萩原ひまわり（CV:倉知玲鳳） SAKURAKO（CV:竹内夢）】</t>
-        </is>
-      </c>
+          <t>Imagica Infos</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr"/>
+      <c r="J64" t="inlineStr"/>
+      <c r="K64" t="inlineStr"/>
+      <c r="L64" t="inlineStr"/>
       <c r="M64" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26462</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28112</t>
         </is>
       </c>
     </row>
@@ -3661,7 +3653,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>無職転生Ⅲ ～異世界行ったら本気だす～</t>
+          <t>無自覚聖女は今日も無意識に力を垂れ流す</t>
         </is>
       </c>
       <c r="E65" t="b">
@@ -3674,25 +3666,37 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>2026年7月5日（日）～ TOKYO MX・BS11ほか</t>
-        </is>
-      </c>
-      <c r="H65" t="inlineStr"/>
+          <t>2026年7月～ TOKYO MX・BS11・AT-Xにて</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>マジックバス×ピカンテサーカス</t>
+        </is>
+      </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>決意の唄</t>
+          <t>Windmaker</t>
         </is>
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>大原ゆい子</t>
-        </is>
-      </c>
-      <c r="K65" t="inlineStr"/>
-      <c r="L65" t="inlineStr"/>
+          <t>花耶</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>アンノウンミー</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>ウタヒメドリーム オールスターズ【夢咲いぶき（CV:山﨑玲奈） 桜木舞華（CV:鈴木杏奈） 真白清美（CV:其原有沙） HiREN（CV:花耶） 水月ひかり（CV:礒部花凜） 高木凛（CV:鷲見友美ジェナ） 萩原ひまわり（CV:倉知玲鳳） SAKURAKO（CV:竹内夢）】</t>
+        </is>
+      </c>
       <c r="M65" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=24285</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26462</t>
         </is>
       </c>
     </row>
@@ -3710,7 +3714,7 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>メビウス・ダスト</t>
+          <t>無職転生Ⅲ ～異世界行ったら本気だす～</t>
         </is>
       </c>
       <c r="E66" t="b">
@@ -3723,29 +3727,25 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>2026年7月～</t>
-        </is>
-      </c>
-      <c r="H66" t="inlineStr">
-        <is>
-          <t>動画工房</t>
-        </is>
-      </c>
+          <t>2026年7月5日（日）～ TOKYO MX・BS11ほか</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr"/>
       <c r="I66" t="inlineStr">
         <is>
-          <t>メビウス</t>
+          <t>決意の唄</t>
         </is>
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>家入レオ</t>
+          <t>大原ゆい子</t>
         </is>
       </c>
       <c r="K66" t="inlineStr"/>
       <c r="L66" t="inlineStr"/>
       <c r="M66" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28016</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=24285</t>
         </is>
       </c>
     </row>
@@ -3763,7 +3763,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>ヤニねこ</t>
+          <t>メビウス・ダスト</t>
         </is>
       </c>
       <c r="E67" t="b">
@@ -3776,29 +3776,29 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>2026年7月2日（木）～ TOKYO MX・BS11にて</t>
+          <t>2026年7月～</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>バイブリーアニメーションスタジオ</t>
+          <t>動画工房</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>なんもねえ</t>
+          <t>メビウス</t>
         </is>
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>忘れらんねえよ</t>
+          <t>家入レオ</t>
         </is>
       </c>
       <c r="K67" t="inlineStr"/>
       <c r="L67" t="inlineStr"/>
       <c r="M67" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27571</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28016</t>
         </is>
       </c>
     </row>
@@ -3816,7 +3816,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>幼女戦記Ⅱ</t>
+          <t>ヤニねこ</t>
         </is>
       </c>
       <c r="E68" t="b">
@@ -3829,21 +3829,29 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>2026年7月～</t>
+          <t>2026年7月2日（木）～ TOKYO MX・BS11にて</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>NUT</t>
-        </is>
-      </c>
-      <c r="I68" t="inlineStr"/>
-      <c r="J68" t="inlineStr"/>
+          <t>バイブリーアニメーションスタジオ</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>なんもねえ</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>忘れらんねえよ</t>
+        </is>
+      </c>
       <c r="K68" t="inlineStr"/>
       <c r="L68" t="inlineStr"/>
       <c r="M68" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=14369</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27571</t>
         </is>
       </c>
     </row>
@@ -3861,7 +3869,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>鎧真伝サムライトルーパー 第2クール</t>
+          <t>幼女戦記Ⅱ</t>
         </is>
       </c>
       <c r="E69" t="b">
@@ -3874,37 +3882,21 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>【第1クール】 2026年1月6日（火）〜2026年3月24日（火） TOKYO MXほか 【第2クール】 2026年7月～</t>
+          <t>2026年7月～</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>サンライズ</t>
-        </is>
-      </c>
-      <c r="I69" t="inlineStr">
-        <is>
-          <t>YOAKE</t>
-        </is>
-      </c>
-      <c r="J69" t="inlineStr">
-        <is>
-          <t>blank paper</t>
-        </is>
-      </c>
-      <c r="K69" t="inlineStr">
-        <is>
-          <t>POWER</t>
-        </is>
-      </c>
-      <c r="L69" t="inlineStr">
-        <is>
-          <t>ONE OR EIGHT</t>
-        </is>
-      </c>
+          <t>NUT</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr"/>
+      <c r="J69" t="inlineStr"/>
+      <c r="K69" t="inlineStr"/>
+      <c r="L69" t="inlineStr"/>
       <c r="M69" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26202</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=14369</t>
         </is>
       </c>
     </row>
@@ -3922,7 +3914,7 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>落第賢者の学院無双～二度目の転生、Sランクチート魔術師冒険録～</t>
+          <t>鎧真伝サムライトルーパー 第2クール</t>
         </is>
       </c>
       <c r="E70" t="b">
@@ -3935,29 +3927,37 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>2026年7月～</t>
+          <t>第1クール：2026年1月6日（火）〜2026年3月24日（火） 第2クール：2026年7月7日（火）～ TOKYO MXほか</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>EMTスクエアード</t>
-        </is>
-      </c>
-      <c r="I70" t="inlineStr"/>
-      <c r="J70" t="inlineStr"/>
+          <t>サンライズ</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>YOAKE</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>blank paper</t>
+        </is>
+      </c>
       <c r="K70" t="inlineStr">
         <is>
-          <t>憧憬</t>
+          <t>POWER</t>
         </is>
       </c>
       <c r="L70" t="inlineStr">
         <is>
-          <t>TrySail</t>
+          <t>ONE OR EIGHT</t>
         </is>
       </c>
       <c r="M70" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27769</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26202</t>
         </is>
       </c>
     </row>
@@ -3975,7 +3975,7 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>領民0人スタートの辺境領主様</t>
+          <t>落第賢者の学院無双～二度目の転生、Sランクチート魔術師冒険録～</t>
         </is>
       </c>
       <c r="E71" t="b">
@@ -3988,37 +3988,29 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>2026年7月10日（金）～ TOKYO MXほか</t>
+          <t>2026年7月～</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>animation studio42</t>
-        </is>
-      </c>
-      <c r="I71" t="inlineStr">
-        <is>
-          <t>Wonder</t>
-        </is>
-      </c>
-      <c r="J71" t="inlineStr">
-        <is>
-          <t>CROWN HEAD</t>
-        </is>
-      </c>
+          <t>EMTスクエアード</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr"/>
+      <c r="J71" t="inlineStr"/>
       <c r="K71" t="inlineStr">
         <is>
-          <t>星降る夜の約束</t>
+          <t>憧憬</t>
         </is>
       </c>
       <c r="L71" t="inlineStr">
         <is>
-          <t>花耶</t>
+          <t>TrySail</t>
         </is>
       </c>
       <c r="M71" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26472</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27769</t>
         </is>
       </c>
     </row>
@@ -4036,7 +4028,7 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>令和のダラさん</t>
+          <t>領民0人スタートの辺境領主様</t>
         </is>
       </c>
       <c r="E72" t="b">
@@ -4049,29 +4041,37 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>2026年7月～</t>
+          <t>2026年7月10日（金）～ TOKYO MXほか</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>旭プロダクション</t>
+          <t>animation studio42</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>ダラダラ♡ダンシング</t>
+          <t>Wonder</t>
         </is>
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>ダラさん（CV：田村睦心） 三⼗⽊⾕⽇向（CV：津田美波） 三⼗⽊⾕薫（CV：寺澤百花） ナレーション（CV：てらそままさき）</t>
-        </is>
-      </c>
-      <c r="K72" t="inlineStr"/>
-      <c r="L72" t="inlineStr"/>
+          <t>CROWN HEAD</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>星降る夜の約束</t>
+        </is>
+      </c>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>花耶</t>
+        </is>
+      </c>
       <c r="M72" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27242</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26472</t>
         </is>
       </c>
     </row>
@@ -4089,7 +4089,7 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>レッツゴー怪奇組</t>
+          <t>令和のダラさん</t>
         </is>
       </c>
       <c r="E73" t="b">
@@ -4102,21 +4102,29 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>2026年7月5日（日）〜 TBS系全国28局ネットにて</t>
+          <t>2026年7月～</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>C-Station</t>
-        </is>
-      </c>
-      <c r="I73" t="inlineStr"/>
-      <c r="J73" t="inlineStr"/>
+          <t>旭プロダクション</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>ダラダラ♡ダンシング</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>ダラさん（CV：田村睦心） 三⼗⽊⾕⽇向（CV：津田美波） 三⼗⽊⾕薫（CV：寺澤百花） ナレーション（CV：てらそままさき）</t>
+        </is>
+      </c>
       <c r="K73" t="inlineStr"/>
       <c r="L73" t="inlineStr"/>
       <c r="M73" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28373</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27242</t>
         </is>
       </c>
     </row>
@@ -4134,7 +4142,7 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>LV999の村人</t>
+          <t>レッツゴー怪奇組</t>
         </is>
       </c>
       <c r="E74" t="b">
@@ -4147,29 +4155,21 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>2026年7月～ テレ東・BSフジほか</t>
+          <t>2026年7月5日（日）〜 TBS系全国28局ネットにて</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>ブレインズ・ベース</t>
-        </is>
-      </c>
-      <c r="I74" t="inlineStr">
-        <is>
-          <t>Not a Hero</t>
-        </is>
-      </c>
-      <c r="J74" t="inlineStr">
-        <is>
-          <t>藍月なくる&amp;棗いつき</t>
-        </is>
-      </c>
+          <t>C-Station</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr"/>
+      <c r="J74" t="inlineStr"/>
       <c r="K74" t="inlineStr"/>
       <c r="L74" t="inlineStr"/>
       <c r="M74" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26648</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28373</t>
         </is>
       </c>
     </row>
@@ -4187,7 +4187,7 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>ワールド イズ ダンシング</t>
+          <t>LV999の村人</t>
         </is>
       </c>
       <c r="E75" t="b">
@@ -4200,29 +4200,29 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>2026年7月2日（木）～ TOKYO MX・BS朝日ほか</t>
+          <t>2026年7月～ テレ東・BSフジほか</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>サイピク</t>
+          <t>ブレインズ・ベース</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>終宵</t>
+          <t>Not a Hero</t>
         </is>
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>マカロニえんぴつ</t>
+          <t>藍月なくる&amp;棗いつき</t>
         </is>
       </c>
       <c r="K75" t="inlineStr"/>
       <c r="L75" t="inlineStr"/>
       <c r="M75" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27472</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26648</t>
         </is>
       </c>
     </row>
@@ -4240,7 +4240,7 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>ONE PIECE HEROINES</t>
+          <t>ワールド イズ ダンシング</t>
         </is>
       </c>
       <c r="E76" t="b">
@@ -4253,35 +4253,47 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>2026年7月5日（日） 全国フジテレビ系にて</t>
-        </is>
-      </c>
-      <c r="H76" t="inlineStr"/>
-      <c r="I76" t="inlineStr"/>
-      <c r="J76" t="inlineStr"/>
+          <t>2026年7月2日（木）～ TOKYO MX・BS朝日ほか</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>サイピク</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>終宵</t>
+        </is>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>マカロニえんぴつ</t>
+        </is>
+      </c>
       <c r="K76" t="inlineStr"/>
       <c r="L76" t="inlineStr"/>
       <c r="M76" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26606</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27472</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
-        <v>5947</v>
+        <v>5806</v>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2026秋アニメ</t>
+          <t>2026夏アニメ</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>1</v>
+        <v>76</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>アオアシ Season2</t>
+          <t>ONE PIECE HEROINES</t>
         </is>
       </c>
       <c r="E77" t="b">
@@ -4294,21 +4306,17 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>2026年10月4日（日）～ NHK Eテレにて</t>
-        </is>
-      </c>
-      <c r="H77" t="inlineStr">
-        <is>
-          <t>トムス・エンタテインメント</t>
-        </is>
-      </c>
+          <t>2026年7月5日（日） 全国フジテレビ系にて</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr"/>
       <c r="I77" t="inlineStr"/>
       <c r="J77" t="inlineStr"/>
       <c r="K77" t="inlineStr"/>
       <c r="L77" t="inlineStr"/>
       <c r="M77" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25889</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26606</t>
         </is>
       </c>
     </row>
@@ -4322,11 +4330,11 @@
         </is>
       </c>
       <c r="C78" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>アオのハコ 第2期</t>
+          <t>アオアシ Season2</t>
         </is>
       </c>
       <c r="E78" t="b">
@@ -4339,12 +4347,12 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>2026年10月4日（日）～ TBS系にて</t>
+          <t>2026年10月4日（日）～ NHK Eテレにて</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>エレクトリックサーカス</t>
+          <t>トムス・エンタテインメント</t>
         </is>
       </c>
       <c r="I78" t="inlineStr"/>
@@ -4353,7 +4361,7 @@
       <c r="L78" t="inlineStr"/>
       <c r="M78" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25746</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25889</t>
         </is>
       </c>
     </row>
@@ -4367,11 +4375,11 @@
         </is>
       </c>
       <c r="C79" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>傷だらけ聖女より報復をこめて Season2</t>
+          <t>アオのハコ 第2期</t>
         </is>
       </c>
       <c r="E79" t="b">
@@ -4384,12 +4392,12 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>2026年10月〜</t>
+          <t>2026年10月4日（日）～ TBS系にて</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>Imagica Infos</t>
+          <t>エレクトリックサーカス</t>
         </is>
       </c>
       <c r="I79" t="inlineStr"/>
@@ -4398,7 +4406,7 @@
       <c r="L79" t="inlineStr"/>
       <c r="M79" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25118</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25746</t>
         </is>
       </c>
     </row>
@@ -4412,11 +4420,11 @@
         </is>
       </c>
       <c r="C80" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>恐怖コレクター</t>
+          <t>カードファイト!! ヴァンガード Divinez 運命星戦編</t>
         </is>
       </c>
       <c r="E80" t="b">
@@ -4429,17 +4437,21 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>2026年10月～ NHK総合にて</t>
-        </is>
-      </c>
-      <c r="H80" t="inlineStr"/>
+          <t>2026年11月7日（土）～2026年11月21日（土） テレビ愛知・テレ東系列6局ネットほか 【劇場先行】 2026年10月2日（金）</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>キネマシトラス</t>
+        </is>
+      </c>
       <c r="I80" t="inlineStr"/>
       <c r="J80" t="inlineStr"/>
       <c r="K80" t="inlineStr"/>
       <c r="L80" t="inlineStr"/>
       <c r="M80" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27214</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28214</t>
         </is>
       </c>
     </row>
@@ -4453,11 +4465,11 @@
         </is>
       </c>
       <c r="C81" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>凶乱令嬢ニア・リストン 病弱令嬢に転生した神殺しの武人の華麗なる無双録</t>
+          <t>傷だらけ聖女より報復をこめて Season2</t>
         </is>
       </c>
       <c r="E81" t="b">
@@ -4470,12 +4482,12 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
+          <t>2026年10月〜</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>KONAMI animation</t>
+          <t>Imagica Infos</t>
         </is>
       </c>
       <c r="I81" t="inlineStr"/>
@@ -4484,7 +4496,7 @@
       <c r="L81" t="inlineStr"/>
       <c r="M81" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27537</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25118</t>
         </is>
       </c>
     </row>
@@ -4498,11 +4510,11 @@
         </is>
       </c>
       <c r="C82" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>薬屋のひとりごと 第3期</t>
+          <t>恐怖コレクター</t>
         </is>
       </c>
       <c r="E82" t="b">
@@ -4515,7 +4527,7 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>第1クール：2026年10月～ 第2クール：2027年4月～ 日本テレビ系にて</t>
+          <t>2026年10月～ NHK総合にて</t>
         </is>
       </c>
       <c r="H82" t="inlineStr"/>
@@ -4525,7 +4537,7 @@
       <c r="L82" t="inlineStr"/>
       <c r="M82" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26369</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27214</t>
         </is>
       </c>
     </row>
@@ -4539,11 +4551,11 @@
         </is>
       </c>
       <c r="C83" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>ケロロ軍曹☆</t>
+          <t>凶乱令嬢ニア・リストン 病弱令嬢に転生した神殺しの武人の華麗なる無双録</t>
         </is>
       </c>
       <c r="E83" t="b">
@@ -4556,17 +4568,21 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>2026年秋</t>
-        </is>
-      </c>
-      <c r="H83" t="inlineStr"/>
+          <t>2026年10月～</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>KONAMI animation</t>
+        </is>
+      </c>
       <c r="I83" t="inlineStr"/>
       <c r="J83" t="inlineStr"/>
       <c r="K83" t="inlineStr"/>
       <c r="L83" t="inlineStr"/>
       <c r="M83" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27337</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27537</t>
         </is>
       </c>
     </row>
@@ -4580,11 +4596,11 @@
         </is>
       </c>
       <c r="C84" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>幻想水滸伝</t>
+          <t>薬屋のひとりごと 第3期</t>
         </is>
       </c>
       <c r="E84" t="b">
@@ -4597,7 +4613,7 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
+          <t>第1クール：2026年10月～ 第2クール：2027年4月～ 日本テレビ系にて</t>
         </is>
       </c>
       <c r="H84" t="inlineStr"/>
@@ -4607,7 +4623,7 @@
       <c r="L84" t="inlineStr"/>
       <c r="M84" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25616</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26369</t>
         </is>
       </c>
     </row>
@@ -4621,11 +4637,11 @@
         </is>
       </c>
       <c r="C85" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>PSYREN -サイレン-</t>
+          <t>ケロロ軍曹☆</t>
         </is>
       </c>
       <c r="E85" t="b">
@@ -4638,21 +4654,17 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
-        </is>
-      </c>
-      <c r="H85" t="inlineStr">
-        <is>
-          <t>サテライト</t>
-        </is>
-      </c>
+          <t>2026年秋</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr"/>
       <c r="I85" t="inlineStr"/>
       <c r="J85" t="inlineStr"/>
       <c r="K85" t="inlineStr"/>
       <c r="L85" t="inlineStr"/>
       <c r="M85" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27257</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27337</t>
         </is>
       </c>
     </row>
@@ -4666,11 +4678,11 @@
         </is>
       </c>
       <c r="C86" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>ジャンケットバンク</t>
+          <t>幻想水滸伝</t>
         </is>
       </c>
       <c r="E86" t="b">
@@ -4686,18 +4698,14 @@
           <t>2026年10月～</t>
         </is>
       </c>
-      <c r="H86" t="inlineStr">
-        <is>
-          <t>CUE</t>
-        </is>
-      </c>
+      <c r="H86" t="inlineStr"/>
       <c r="I86" t="inlineStr"/>
       <c r="J86" t="inlineStr"/>
       <c r="K86" t="inlineStr"/>
       <c r="L86" t="inlineStr"/>
       <c r="M86" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27908</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25616</t>
         </is>
       </c>
     </row>
@@ -4711,11 +4719,11 @@
         </is>
       </c>
       <c r="C87" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>朱色の仮面</t>
+          <t>PSYREN -サイレン-</t>
         </is>
       </c>
       <c r="E87" t="b">
@@ -4728,17 +4736,21 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>2026年10月～ 読売テレビ・日本テレビ系全国ネットにて</t>
-        </is>
-      </c>
-      <c r="H87" t="inlineStr"/>
+          <t>2026年10月～</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>サテライト</t>
+        </is>
+      </c>
       <c r="I87" t="inlineStr"/>
       <c r="J87" t="inlineStr"/>
       <c r="K87" t="inlineStr"/>
       <c r="L87" t="inlineStr"/>
       <c r="M87" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26362</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27257</t>
         </is>
       </c>
     </row>
@@ -4752,11 +4764,11 @@
         </is>
       </c>
       <c r="C88" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>しろたん</t>
+          <t>ジャンケットバンク</t>
         </is>
       </c>
       <c r="E88" t="b">
@@ -4769,12 +4781,12 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>2026年秋</t>
+          <t>2026年10月～</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>レスプリ</t>
+          <t>CUE</t>
         </is>
       </c>
       <c r="I88" t="inlineStr"/>
@@ -4783,7 +4795,7 @@
       <c r="L88" t="inlineStr"/>
       <c r="M88" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27989</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27908</t>
         </is>
       </c>
     </row>
@@ -4797,11 +4809,11 @@
         </is>
       </c>
       <c r="C89" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>新テニスの王子様 U-17 WORLD CUP 決勝メンバー決定戦</t>
+          <t>朱色の仮面</t>
         </is>
       </c>
       <c r="E89" t="b">
@@ -4814,7 +4826,7 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>2026年秋</t>
+          <t>2026年10月～ 読売テレビ・日本テレビ系全国ネットにて</t>
         </is>
       </c>
       <c r="H89" t="inlineStr"/>
@@ -4824,7 +4836,7 @@
       <c r="L89" t="inlineStr"/>
       <c r="M89" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26829</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26362</t>
         </is>
       </c>
     </row>
@@ -4838,11 +4850,11 @@
         </is>
       </c>
       <c r="C90" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>世界最強の魔女、始めました</t>
+          <t>しろたん</t>
         </is>
       </c>
       <c r="E90" t="b">
@@ -4855,12 +4867,12 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
+          <t>2026年秋</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>ブリッジ</t>
+          <t>レスプリ</t>
         </is>
       </c>
       <c r="I90" t="inlineStr"/>
@@ -4869,7 +4881,7 @@
       <c r="L90" t="inlineStr"/>
       <c r="M90" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28288</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27989</t>
         </is>
       </c>
     </row>
@@ -4883,11 +4895,11 @@
         </is>
       </c>
       <c r="C91" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>#ゾンビさがしてます</t>
+          <t>新テニスの王子様 U-17 WORLD CUP 決勝メンバー決定戦</t>
         </is>
       </c>
       <c r="E91" t="b">
@@ -4900,7 +4912,7 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>2026年10月〜 テレビ朝日系にて</t>
+          <t>2026年秋</t>
         </is>
       </c>
       <c r="H91" t="inlineStr"/>
@@ -4910,7 +4922,7 @@
       <c r="L91" t="inlineStr"/>
       <c r="M91" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26825</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26829</t>
         </is>
       </c>
     </row>
@@ -4924,11 +4936,11 @@
         </is>
       </c>
       <c r="C92" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>タヌキとキツネ</t>
+          <t>世界最強の魔女、始めました</t>
         </is>
       </c>
       <c r="E92" t="b">
@@ -4944,14 +4956,18 @@
           <t>2026年10月～</t>
         </is>
       </c>
-      <c r="H92" t="inlineStr"/>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>ブリッジ</t>
+        </is>
+      </c>
       <c r="I92" t="inlineStr"/>
       <c r="J92" t="inlineStr"/>
       <c r="K92" t="inlineStr"/>
       <c r="L92" t="inlineStr"/>
       <c r="M92" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=6380</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28288</t>
         </is>
       </c>
     </row>
@@ -4965,11 +4981,11 @@
         </is>
       </c>
       <c r="C93" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>TANK CHAIR-戦車椅子-</t>
+          <t>#ゾンビさがしてます</t>
         </is>
       </c>
       <c r="E93" t="b">
@@ -4982,21 +4998,17 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>2026年秋</t>
-        </is>
-      </c>
-      <c r="H93" t="inlineStr">
-        <is>
-          <t>ポリゴン・ピクチュアズ</t>
-        </is>
-      </c>
+          <t>2026年10月〜 テレビ朝日系にて</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr"/>
       <c r="I93" t="inlineStr"/>
       <c r="J93" t="inlineStr"/>
       <c r="K93" t="inlineStr"/>
       <c r="L93" t="inlineStr"/>
       <c r="M93" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27965</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26825</t>
         </is>
       </c>
     </row>
@@ -5010,11 +5022,11 @@
         </is>
       </c>
       <c r="C94" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>探偵はもう、死んでいる。Season2</t>
+          <t>タヌキとキツネ</t>
         </is>
       </c>
       <c r="E94" t="b">
@@ -5027,21 +5039,17 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>2026年10月〜</t>
-        </is>
-      </c>
-      <c r="H94" t="inlineStr">
-        <is>
-          <t>ENGI</t>
-        </is>
-      </c>
+          <t>2026年10月～</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr"/>
       <c r="I94" t="inlineStr"/>
       <c r="J94" t="inlineStr"/>
       <c r="K94" t="inlineStr"/>
       <c r="L94" t="inlineStr"/>
       <c r="M94" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=16348</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=6380</t>
         </is>
       </c>
     </row>
@@ -5055,11 +5063,11 @@
         </is>
       </c>
       <c r="C95" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>超巡！超条先輩</t>
+          <t>TANK CHAIR-戦車椅子-</t>
         </is>
       </c>
       <c r="E95" t="b">
@@ -5072,12 +5080,12 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
+          <t>2026年秋</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>アルボアニメーション</t>
+          <t>ポリゴン・ピクチュアズ</t>
         </is>
       </c>
       <c r="I95" t="inlineStr"/>
@@ -5086,7 +5094,7 @@
       <c r="L95" t="inlineStr"/>
       <c r="M95" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26933</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27965</t>
         </is>
       </c>
     </row>
@@ -5100,11 +5108,11 @@
         </is>
       </c>
       <c r="C96" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>てつりょー！meet with 鉄道むすめ</t>
+          <t>探偵はもう、死んでいる。Season2</t>
         </is>
       </c>
       <c r="E96" t="b">
@@ -5117,12 +5125,12 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>2026年秋</t>
+          <t>2026年10月〜</t>
         </is>
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>イーストフィッシュスタジオ</t>
+          <t>ENGI</t>
         </is>
       </c>
       <c r="I96" t="inlineStr"/>
@@ -5131,7 +5139,7 @@
       <c r="L96" t="inlineStr"/>
       <c r="M96" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26895</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=16348</t>
         </is>
       </c>
     </row>
@@ -5145,11 +5153,11 @@
         </is>
       </c>
       <c r="C97" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>転生貴族、鑑定スキルで成り上がる 第3期</t>
+          <t>超巡！超条先輩</t>
         </is>
       </c>
       <c r="E97" t="b">
@@ -5162,12 +5170,12 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>2026年秋 CBC/TBS系全国28局ネット「アガルアニメ」にて</t>
+          <t>2026年10月～</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>studio MOTHER</t>
+          <t>アルボアニメーション</t>
         </is>
       </c>
       <c r="I97" t="inlineStr"/>
@@ -5176,7 +5184,7 @@
       <c r="L97" t="inlineStr"/>
       <c r="M97" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25385</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26933</t>
         </is>
       </c>
     </row>
@@ -5190,11 +5198,11 @@
         </is>
       </c>
       <c r="C98" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>転生ゴブリンだけど質問ある？</t>
+          <t>てつりょー！meet with 鉄道むすめ</t>
         </is>
       </c>
       <c r="E98" t="b">
@@ -5207,12 +5215,12 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
+          <t>2026年秋</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>BAKKKA</t>
+          <t>イーストフィッシュスタジオ</t>
         </is>
       </c>
       <c r="I98" t="inlineStr"/>
@@ -5221,7 +5229,7 @@
       <c r="L98" t="inlineStr"/>
       <c r="M98" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27909</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26895</t>
         </is>
       </c>
     </row>
@@ -5235,11 +5243,11 @@
         </is>
       </c>
       <c r="C99" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>転生した大聖女は、聖女であることをひた隠す</t>
+          <t>転生貴族、鑑定スキルで成り上がる 第3期</t>
         </is>
       </c>
       <c r="E99" t="b">
@@ -5252,37 +5260,21 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
+          <t>2026年秋 CBC/TBS系全国28局ネット「アガルアニメ」にて</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>FelixFilm</t>
-        </is>
-      </c>
-      <c r="I99" t="inlineStr">
-        <is>
-          <t>Flare of Soul</t>
-        </is>
-      </c>
-      <c r="J99" t="inlineStr">
-        <is>
-          <t>花耶</t>
-        </is>
-      </c>
-      <c r="K99" t="inlineStr">
-        <is>
-          <t>STELLAR</t>
-        </is>
-      </c>
-      <c r="L99" t="inlineStr">
-        <is>
-          <t>ウタヒメドリーム オールスターズ</t>
-        </is>
-      </c>
+          <t>studio MOTHER</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr"/>
+      <c r="J99" t="inlineStr"/>
+      <c r="K99" t="inlineStr"/>
+      <c r="L99" t="inlineStr"/>
       <c r="M99" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25630</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25385</t>
         </is>
       </c>
     </row>
@@ -5296,11 +5288,11 @@
         </is>
       </c>
       <c r="C100" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>転生したら剣でした 第2期</t>
+          <t>転生ゴブリンだけど質問ある？</t>
         </is>
       </c>
       <c r="E100" t="b">
@@ -5318,7 +5310,7 @@
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>C2C</t>
+          <t>BAKKKA</t>
         </is>
       </c>
       <c r="I100" t="inlineStr"/>
@@ -5327,7 +5319,7 @@
       <c r="L100" t="inlineStr"/>
       <c r="M100" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=19149</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27909</t>
         </is>
       </c>
     </row>
@@ -5341,11 +5333,11 @@
         </is>
       </c>
       <c r="C101" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>とある暗部の少女共棲</t>
+          <t>転生した大聖女は、聖女であることをひた隠す</t>
         </is>
       </c>
       <c r="E101" t="b">
@@ -5358,21 +5350,37 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>2026年秋</t>
+          <t>2026年10月～</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>J.C.STAFF</t>
-        </is>
-      </c>
-      <c r="I101" t="inlineStr"/>
-      <c r="J101" t="inlineStr"/>
-      <c r="K101" t="inlineStr"/>
-      <c r="L101" t="inlineStr"/>
+          <t>FelixFilm</t>
+        </is>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>Flare of Soul</t>
+        </is>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>花耶</t>
+        </is>
+      </c>
+      <c r="K101" t="inlineStr">
+        <is>
+          <t>STELLAR</t>
+        </is>
+      </c>
+      <c r="L101" t="inlineStr">
+        <is>
+          <t>ウタヒメドリーム オールスターズ</t>
+        </is>
+      </c>
       <c r="M101" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25552</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25630</t>
         </is>
       </c>
     </row>
@@ -5386,11 +5394,11 @@
         </is>
       </c>
       <c r="C102" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>東京リベンジャーズ 三天戦争編</t>
+          <t>転生したら剣でした 第2期</t>
         </is>
       </c>
       <c r="E102" t="b">
@@ -5408,7 +5416,7 @@
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>ライデンフィルム</t>
+          <t>C2C</t>
         </is>
       </c>
       <c r="I102" t="inlineStr"/>
@@ -5417,7 +5425,7 @@
       <c r="L102" t="inlineStr"/>
       <c r="M102" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=24207</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=19149</t>
         </is>
       </c>
     </row>
@@ -5431,11 +5439,11 @@
         </is>
       </c>
       <c r="C103" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>桃源暗鬼 ～日光・華厳の滝編～</t>
+          <t>とある暗部の少女共棲</t>
         </is>
       </c>
       <c r="E103" t="b">
@@ -5448,17 +5456,21 @@
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>2026年10月～ 日本テレビ系「FRIDAY ANIME NIGHT（フラアニ）」枠にて</t>
-        </is>
-      </c>
-      <c r="H103" t="inlineStr"/>
+          <t>2026年秋</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>J.C.STAFF</t>
+        </is>
+      </c>
       <c r="I103" t="inlineStr"/>
       <c r="J103" t="inlineStr"/>
       <c r="K103" t="inlineStr"/>
       <c r="L103" t="inlineStr"/>
       <c r="M103" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27376</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25552</t>
         </is>
       </c>
     </row>
@@ -5472,11 +5484,11 @@
         </is>
       </c>
       <c r="C104" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>ドラゴンボール超 ビルス</t>
+          <t>東京リベンジャーズ 三天戦争編</t>
         </is>
       </c>
       <c r="E104" t="b">
@@ -5489,17 +5501,21 @@
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>2026年秋 フジテレビにて</t>
-        </is>
-      </c>
-      <c r="H104" t="inlineStr"/>
+          <t>2026年10月～</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>ライデンフィルム</t>
+        </is>
+      </c>
       <c r="I104" t="inlineStr"/>
       <c r="J104" t="inlineStr"/>
       <c r="K104" t="inlineStr"/>
       <c r="L104" t="inlineStr"/>
       <c r="M104" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27491</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=24207</t>
         </is>
       </c>
     </row>
@@ -5513,11 +5529,11 @@
         </is>
       </c>
       <c r="C105" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>バーテックスフォース</t>
+          <t>桃源暗鬼 ～日光・華厳の滝編～</t>
         </is>
       </c>
       <c r="E105" t="b">
@@ -5530,21 +5546,17 @@
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>2026年10月〜</t>
-        </is>
-      </c>
-      <c r="H105" t="inlineStr">
-        <is>
-          <t>SMDE</t>
-        </is>
-      </c>
+          <t>2026年10月～ 日本テレビ系「FRIDAY ANIME NIGHT（フラアニ）」枠にて</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr"/>
       <c r="I105" t="inlineStr"/>
       <c r="J105" t="inlineStr"/>
       <c r="K105" t="inlineStr"/>
       <c r="L105" t="inlineStr"/>
       <c r="M105" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27988</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27376</t>
         </is>
       </c>
     </row>
@@ -5558,11 +5570,11 @@
         </is>
       </c>
       <c r="C106" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Battle Spirits [Re] 絶界の空</t>
+          <t>ドラゴンボール超 ビルス</t>
         </is>
       </c>
       <c r="E106" t="b">
@@ -5575,7 +5587,7 @@
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>2026年秋</t>
+          <t>2026年秋 フジテレビにて</t>
         </is>
       </c>
       <c r="H106" t="inlineStr"/>
@@ -5585,7 +5597,7 @@
       <c r="L106" t="inlineStr"/>
       <c r="M106" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27954</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27491</t>
         </is>
       </c>
     </row>
@@ -5599,11 +5611,11 @@
         </is>
       </c>
       <c r="C107" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>パンどろぼう</t>
+          <t>バーテックスフォース</t>
         </is>
       </c>
       <c r="E107" t="b">
@@ -5616,17 +5628,21 @@
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>2026年10月〜 NHK Eテレにて</t>
-        </is>
-      </c>
-      <c r="H107" t="inlineStr"/>
+          <t>2026年10月〜</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>SMDE</t>
+        </is>
+      </c>
       <c r="I107" t="inlineStr"/>
       <c r="J107" t="inlineStr"/>
       <c r="K107" t="inlineStr"/>
       <c r="L107" t="inlineStr"/>
       <c r="M107" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26163</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27988</t>
         </is>
       </c>
     </row>
@@ -5640,11 +5656,11 @@
         </is>
       </c>
       <c r="C108" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>百妖譜 京師篇</t>
+          <t>Battle Spirits [Re] 絶界の空</t>
         </is>
       </c>
       <c r="E108" t="b">
@@ -5657,7 +5673,7 @@
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>2026年10月〜 フジテレビ「B8station」にて</t>
+          <t>2026年秋</t>
         </is>
       </c>
       <c r="H108" t="inlineStr"/>
@@ -5667,7 +5683,7 @@
       <c r="L108" t="inlineStr"/>
       <c r="M108" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27781</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27954</t>
         </is>
       </c>
     </row>
@@ -5681,11 +5697,11 @@
         </is>
       </c>
       <c r="C109" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>冰剣の魔術師が世界を統べるⅡ</t>
+          <t>パンどろぼう</t>
         </is>
       </c>
       <c r="E109" t="b">
@@ -5698,21 +5714,17 @@
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>2026年10月〜</t>
-        </is>
-      </c>
-      <c r="H109" t="inlineStr">
-        <is>
-          <t>ゼロジー</t>
-        </is>
-      </c>
+          <t>2026年10月〜 NHK Eテレにて</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr"/>
       <c r="I109" t="inlineStr"/>
       <c r="J109" t="inlineStr"/>
       <c r="K109" t="inlineStr"/>
       <c r="L109" t="inlineStr"/>
       <c r="M109" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28403</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26163</t>
         </is>
       </c>
     </row>
@@ -5726,11 +5738,11 @@
         </is>
       </c>
       <c r="C110" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>ホタルの嫁入り</t>
+          <t>百妖譜 京師篇</t>
         </is>
       </c>
       <c r="E110" t="b">
@@ -5743,21 +5755,17 @@
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>2026年10月～ 全国フジテレビ系“ ノイタミナ ”にて</t>
-        </is>
-      </c>
-      <c r="H110" t="inlineStr">
-        <is>
-          <t>david production</t>
-        </is>
-      </c>
+          <t>2026年10月〜 フジテレビ「B8station」にて</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr"/>
       <c r="I110" t="inlineStr"/>
       <c r="J110" t="inlineStr"/>
       <c r="K110" t="inlineStr"/>
       <c r="L110" t="inlineStr"/>
       <c r="M110" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27415</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27781</t>
         </is>
       </c>
     </row>
@@ -5771,11 +5779,11 @@
         </is>
       </c>
       <c r="C111" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>ポップパップポルターズ</t>
+          <t>冰剣の魔術師が世界を統べるⅡ</t>
         </is>
       </c>
       <c r="E111" t="b">
@@ -5788,12 +5796,12 @@
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>2026年秋 テレビ朝日にて</t>
+          <t>2026年10月〜</t>
         </is>
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>MOZU STUDIOS</t>
+          <t>ゼロジー</t>
         </is>
       </c>
       <c r="I111" t="inlineStr"/>
@@ -5802,7 +5810,7 @@
       <c r="L111" t="inlineStr"/>
       <c r="M111" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27823</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28403</t>
         </is>
       </c>
     </row>
@@ -5816,11 +5824,11 @@
         </is>
       </c>
       <c r="C112" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>ホテル・インヒューマンズ 第2期</t>
+          <t>ホタルの嫁入り</t>
         </is>
       </c>
       <c r="E112" t="b">
@@ -5833,12 +5841,12 @@
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>2026年10月～ テレ東系列ほか</t>
+          <t>2026年10月～ 全国フジテレビ系“ ノイタミナ ”にて</t>
         </is>
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>ブリッジ</t>
+          <t>david production</t>
         </is>
       </c>
       <c r="I112" t="inlineStr"/>
@@ -5847,7 +5855,7 @@
       <c r="L112" t="inlineStr"/>
       <c r="M112" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26870</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27415</t>
         </is>
       </c>
     </row>
@@ -5861,11 +5869,11 @@
         </is>
       </c>
       <c r="C113" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>マジカル★エクスプローラー</t>
+          <t>ポップパップポルターズ</t>
         </is>
       </c>
       <c r="E113" t="b">
@@ -5878,12 +5886,12 @@
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>2026年秋</t>
+          <t>2026年秋 テレビ朝日にて</t>
         </is>
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>WHITE FOX</t>
+          <t>MOZU STUDIOS</t>
         </is>
       </c>
       <c r="I113" t="inlineStr"/>
@@ -5892,7 +5900,7 @@
       <c r="L113" t="inlineStr"/>
       <c r="M113" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=23375</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27823</t>
         </is>
       </c>
     </row>
@@ -5906,11 +5914,11 @@
         </is>
       </c>
       <c r="C114" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>魔法騎士レイアース</t>
+          <t>ホテル・インヒューマンズ 第2期</t>
         </is>
       </c>
       <c r="E114" t="b">
@@ -5923,12 +5931,12 @@
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>2026年10月～ テレビ朝日系列にて</t>
+          <t>2026年10月～ テレ東系列ほか</t>
         </is>
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>E&amp;H production</t>
+          <t>ブリッジ</t>
         </is>
       </c>
       <c r="I114" t="inlineStr"/>
@@ -5937,7 +5945,7 @@
       <c r="L114" t="inlineStr"/>
       <c r="M114" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=24301</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26870</t>
         </is>
       </c>
     </row>
@@ -5951,11 +5959,11 @@
         </is>
       </c>
       <c r="C115" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>魔法少女育成計画restart</t>
+          <t>マジカル★エクスプローラー</t>
         </is>
       </c>
       <c r="E115" t="b">
@@ -5973,24 +5981,16 @@
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>SynergySP</t>
-        </is>
-      </c>
-      <c r="I115" t="inlineStr">
-        <is>
-          <t>No tears here</t>
-        </is>
-      </c>
-      <c r="J115" t="inlineStr">
-        <is>
-          <t>茅原実里</t>
-        </is>
-      </c>
+          <t>WHITE FOX</t>
+        </is>
+      </c>
+      <c r="I115" t="inlineStr"/>
+      <c r="J115" t="inlineStr"/>
       <c r="K115" t="inlineStr"/>
       <c r="L115" t="inlineStr"/>
       <c r="M115" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26693</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=23375</t>
         </is>
       </c>
     </row>
@@ -6004,11 +6004,11 @@
         </is>
       </c>
       <c r="C116" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>目覚めたら最強装備と宇宙船持ちだったので、一戸建て目指して傭兵として自由に生きたい</t>
+          <t>魔法騎士レイアース</t>
         </is>
       </c>
       <c r="E116" t="b">
@@ -6021,12 +6021,12 @@
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>2026年10月〜</t>
+          <t>2026年10月～ テレビ朝日系列にて</t>
         </is>
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>studio A-CAT</t>
+          <t>E&amp;H production</t>
         </is>
       </c>
       <c r="I116" t="inlineStr"/>
@@ -6035,7 +6035,7 @@
       <c r="L116" t="inlineStr"/>
       <c r="M116" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25525</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=24301</t>
         </is>
       </c>
     </row>
@@ -6049,11 +6049,11 @@
         </is>
       </c>
       <c r="C117" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>弱気MAX令嬢なのに、辣腕婚約者様の賭けに乗ってしまった</t>
+          <t>魔法少女育成計画restart</t>
         </is>
       </c>
       <c r="E117" t="b">
@@ -6066,21 +6066,29 @@
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
+          <t>2026年秋</t>
         </is>
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>寿門堂</t>
-        </is>
-      </c>
-      <c r="I117" t="inlineStr"/>
-      <c r="J117" t="inlineStr"/>
+          <t>SynergySP</t>
+        </is>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>No tears here</t>
+        </is>
+      </c>
+      <c r="J117" t="inlineStr">
+        <is>
+          <t>茅原実里</t>
+        </is>
+      </c>
       <c r="K117" t="inlineStr"/>
       <c r="L117" t="inlineStr"/>
       <c r="M117" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26947</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26693</t>
         </is>
       </c>
     </row>
@@ -6094,11 +6102,11 @@
         </is>
       </c>
       <c r="C118" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>らんま1/2 第3期</t>
+          <t>マロニエ王国の七人の騎士</t>
         </is>
       </c>
       <c r="E118" t="b">
@@ -6111,17 +6119,21 @@
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>2026年10月～ 日本テレビ系にて</t>
-        </is>
-      </c>
-      <c r="H118" t="inlineStr"/>
+          <t>2026年10月～ NHK Eテレにて</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>J.C.STAFF</t>
+        </is>
+      </c>
       <c r="I118" t="inlineStr"/>
       <c r="J118" t="inlineStr"/>
       <c r="K118" t="inlineStr"/>
       <c r="L118" t="inlineStr"/>
       <c r="M118" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28013</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28456</t>
         </is>
       </c>
     </row>
@@ -6135,11 +6147,11 @@
         </is>
       </c>
       <c r="C119" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>LEGO® ONE PIECE</t>
+          <t>目覚めたら最強装備と宇宙船持ちだったので、一戸建て目指して傭兵として自由に生きたい</t>
         </is>
       </c>
       <c r="E119" t="b">
@@ -6147,20 +6159,151 @@
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>配信</t>
+          <t>TVアニメ</t>
         </is>
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>2026年9月29日（火） Netflixにて</t>
-        </is>
-      </c>
-      <c r="H119" t="inlineStr"/>
+          <t>2026年10月〜</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>studio A-CAT</t>
+        </is>
+      </c>
       <c r="I119" t="inlineStr"/>
       <c r="J119" t="inlineStr"/>
       <c r="K119" t="inlineStr"/>
       <c r="L119" t="inlineStr"/>
       <c r="M119" t="inlineStr">
+        <is>
+          <t>https://www.animatetimes.com/tag/details.php?id=25525</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C120" t="n">
+        <v>43</v>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>弱気MAX令嬢なのに、辣腕婚約者様の賭けに乗ってしまった</t>
+        </is>
+      </c>
+      <c r="E120" t="b">
+        <v>0</v>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>TVアニメ</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>2026年10月～</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>寿門堂</t>
+        </is>
+      </c>
+      <c r="I120" t="inlineStr"/>
+      <c r="J120" t="inlineStr"/>
+      <c r="K120" t="inlineStr"/>
+      <c r="L120" t="inlineStr"/>
+      <c r="M120" t="inlineStr">
+        <is>
+          <t>https://www.animatetimes.com/tag/details.php?id=26947</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C121" t="n">
+        <v>44</v>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>らんま1/2 第3期</t>
+        </is>
+      </c>
+      <c r="E121" t="b">
+        <v>0</v>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>TVアニメ</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>2026年10月～ 日本テレビ系にて</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr"/>
+      <c r="I121" t="inlineStr"/>
+      <c r="J121" t="inlineStr"/>
+      <c r="K121" t="inlineStr"/>
+      <c r="L121" t="inlineStr"/>
+      <c r="M121" t="inlineStr">
+        <is>
+          <t>https://www.animatetimes.com/tag/details.php?id=28013</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C122" t="n">
+        <v>45</v>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>LEGO® ONE PIECE</t>
+        </is>
+      </c>
+      <c r="E122" t="b">
+        <v>0</v>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>配信</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>2026年9月29日（火） Netflixにて</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr"/>
+      <c r="I122" t="inlineStr"/>
+      <c r="J122" t="inlineStr"/>
+      <c r="K122" t="inlineStr"/>
+      <c r="L122" t="inlineStr"/>
+      <c r="M122" t="inlineStr">
         <is>
           <t>https://www.animatetimes.com/tag/details.php?id=28168</t>
         </is>
@@ -6177,7 +6320,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L68"/>
+  <dimension ref="A1:L72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7813,7 +7956,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>刃牙道 第2クール</t>
+          <t>パイの実 おしの森へようこそ！</t>
         </is>
       </c>
       <c r="D41" t="b">
@@ -7821,7 +7964,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>主題歌</t>
         </is>
       </c>
       <c r="F41" t="n">
@@ -7829,12 +7972,12 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>フルボコ</t>
+          <t>パイしか勝たん！推しの森活</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>WANIMA</t>
+          <t>安保心結</t>
         </is>
       </c>
       <c r="I41" t="inlineStr"/>
@@ -7861,7 +8004,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F42" t="n">
@@ -7869,12 +8012,12 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Mountain Top</t>
+          <t>フルボコ</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>Novel Core</t>
+          <t>WANIMA</t>
         </is>
       </c>
       <c r="I42" t="inlineStr"/>
@@ -7893,7 +8036,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>花ざかりの君たちへ 第2期</t>
+          <t>刃牙道 第2クール</t>
         </is>
       </c>
       <c r="D43" t="b">
@@ -7901,7 +8044,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F43" t="n">
@@ -7909,12 +8052,12 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>FLASHBULB</t>
+          <t>Mountain Top</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>Omoinotake</t>
+          <t>Novel Core</t>
         </is>
       </c>
       <c r="I43" t="inlineStr"/>
@@ -7941,7 +8084,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F44" t="n">
@@ -7949,7 +8092,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>花束</t>
+          <t>FLASHBULB</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -7973,7 +8116,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>ヒロイン？聖女？いいえ、オールワークスメイドです（誇）！</t>
+          <t>花ざかりの君たちへ 第2期</t>
         </is>
       </c>
       <c r="D45" t="b">
@@ -7981,7 +8124,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F45" t="n">
@@ -7989,12 +8132,12 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>マデュアル↔ハート</t>
+          <t>花束</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>メロディ・ウェーブ(CV：宮本侑芽) ルシアナ・ルトルバーグ(CV：大久保瑠美)</t>
+          <t>Omoinotake</t>
         </is>
       </c>
       <c r="I45" t="inlineStr"/>
@@ -8021,7 +8164,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F46" t="n">
@@ -8029,12 +8172,12 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>ハンドメイド</t>
+          <t>マデュアル↔ハート</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>仲村宗悟</t>
+          <t>メロディ・ウェーブ(CV：宮本侑芽) ルシアナ・ルトルバーグ(CV：大久保瑠美)</t>
         </is>
       </c>
       <c r="I46" t="inlineStr"/>
@@ -8053,7 +8196,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>ブチ切れ令嬢は報復を誓いました。 ～魔導書の力で祖国を叩き潰します～</t>
+          <t>ヒロイン？聖女？いいえ、オールワークスメイドです（誇）！</t>
         </is>
       </c>
       <c r="D47" t="b">
@@ -8061,7 +8204,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F47" t="n">
@@ -8069,12 +8212,12 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Q.E.D.</t>
+          <t>ハンドメイド</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>小倉唯</t>
+          <t>仲村宗悟</t>
         </is>
       </c>
       <c r="I47" t="inlineStr"/>
@@ -8101,7 +8244,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F48" t="n">
@@ -8109,12 +8252,12 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>グッバイ・ララバイ</t>
+          <t>Q.E.D.</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>大西亜玖璃</t>
+          <t>小倉唯</t>
         </is>
       </c>
       <c r="I48" t="inlineStr"/>
@@ -8133,7 +8276,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>プラノサウルス ガチコセイブツ部</t>
+          <t>ブチ切れ令嬢は報復を誓いました。 ～魔導書の力で祖国を叩き潰します～</t>
         </is>
       </c>
       <c r="D49" t="b">
@@ -8141,7 +8284,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>主題歌</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F49" t="n">
@@ -8149,12 +8292,12 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>ガチde古生</t>
+          <t>グッバイ・ララバイ</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>リンクルプラネット</t>
+          <t>大西亜玖璃</t>
         </is>
       </c>
       <c r="I49" t="inlineStr"/>
@@ -8173,7 +8316,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>炎の闘球女 ドッジ弾子</t>
+          <t>プラノサウルス ガチコセイブツ部</t>
         </is>
       </c>
       <c r="D50" t="b">
@@ -8181,7 +8324,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>主題歌</t>
         </is>
       </c>
       <c r="F50" t="n">
@@ -8189,12 +8332,12 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Welcome to あざとさワールド</t>
+          <t>ガチde古生</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>i☆Ris</t>
+          <t>リンクルプラネット</t>
         </is>
       </c>
       <c r="I50" t="inlineStr"/>
@@ -8213,7 +8356,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>魔法少女リリカルなのは EXCEEDS Gun Blaze Vengeance</t>
+          <t>炎の闘球女 ドッジ弾子</t>
         </is>
       </c>
       <c r="D51" t="b">
@@ -8229,12 +8372,12 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>CRIMSON BULLET</t>
+          <t>会心の一劇</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>水樹奈々</t>
+          <t>ももいろクローバーZ</t>
         </is>
       </c>
       <c r="I51" t="inlineStr"/>
@@ -8253,7 +8396,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>魔法少女リリカルなのは EXCEEDS Gun Blaze Vengeance</t>
+          <t>炎の闘球女 ドッジ弾子</t>
         </is>
       </c>
       <c r="D52" t="b">
@@ -8269,12 +8412,12 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Ephemeral</t>
+          <t>Welcome to あざとさワールド</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>青木陽菜</t>
+          <t>i☆Ris</t>
         </is>
       </c>
       <c r="I52" t="inlineStr"/>
@@ -8293,7 +8436,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>無自覚聖女は今日も無意識に力を垂れ流す</t>
+          <t>魔法少女リリカルなのは EXCEEDS Gun Blaze Vengeance</t>
         </is>
       </c>
       <c r="D53" t="b">
@@ -8309,12 +8452,12 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>Windmaker</t>
+          <t>CRIMSON BULLET</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>花耶</t>
+          <t>水樹奈々</t>
         </is>
       </c>
       <c r="I53" t="inlineStr"/>
@@ -8333,7 +8476,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>無自覚聖女は今日も無意識に力を垂れ流す</t>
+          <t>魔法少女リリカルなのは EXCEEDS Gun Blaze Vengeance</t>
         </is>
       </c>
       <c r="D54" t="b">
@@ -8349,12 +8492,12 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>アンノウンミー</t>
+          <t>Ephemeral</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>ウタヒメドリーム オールスターズ【夢咲いぶき（CV:山﨑玲奈） 桜木舞華（CV:鈴木杏奈） 真白清美（CV:其原有沙） HiREN（CV:花耶） 水月ひかり（CV:礒部花凜） 高木凛（CV:鷲見友美ジェナ） 萩原ひまわり（CV:倉知玲鳳） SAKURAKO（CV:竹内夢）】</t>
+          <t>青木陽菜</t>
         </is>
       </c>
       <c r="I54" t="inlineStr"/>
@@ -8373,7 +8516,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>無職転生Ⅲ ～異世界行ったら本気だす～</t>
+          <t>無自覚聖女は今日も無意識に力を垂れ流す</t>
         </is>
       </c>
       <c r="D55" t="b">
@@ -8389,12 +8532,12 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>決意の唄</t>
+          <t>Windmaker</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>大原ゆい子</t>
+          <t>花耶</t>
         </is>
       </c>
       <c r="I55" t="inlineStr"/>
@@ -8413,7 +8556,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>メビウス・ダスト</t>
+          <t>無自覚聖女は今日も無意識に力を垂れ流す</t>
         </is>
       </c>
       <c r="D56" t="b">
@@ -8421,7 +8564,7 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F56" t="n">
@@ -8429,12 +8572,12 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>メビウス</t>
+          <t>アンノウンミー</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>家入レオ</t>
+          <t>ウタヒメドリーム オールスターズ【夢咲いぶき（CV:山﨑玲奈） 桜木舞華（CV:鈴木杏奈） 真白清美（CV:其原有沙） HiREN（CV:花耶） 水月ひかり（CV:礒部花凜） 高木凛（CV:鷲見友美ジェナ） 萩原ひまわり（CV:倉知玲鳳） SAKURAKO（CV:竹内夢）】</t>
         </is>
       </c>
       <c r="I56" t="inlineStr"/>
@@ -8453,7 +8596,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>ヤニねこ</t>
+          <t>無職転生Ⅲ ～異世界行ったら本気だす～</t>
         </is>
       </c>
       <c r="D57" t="b">
@@ -8469,12 +8612,12 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>なんもねえ</t>
+          <t>決意の唄</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>忘れらんねえよ</t>
+          <t>大原ゆい子</t>
         </is>
       </c>
       <c r="I57" t="inlineStr"/>
@@ -8493,7 +8636,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>鎧真伝サムライトルーパー 第2クール</t>
+          <t>メビウス・ダスト</t>
         </is>
       </c>
       <c r="D58" t="b">
@@ -8509,12 +8652,12 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>YOAKE</t>
+          <t>メビウス</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>blank paper</t>
+          <t>家入レオ</t>
         </is>
       </c>
       <c r="I58" t="inlineStr"/>
@@ -8533,7 +8676,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>鎧真伝サムライトルーパー 第2クール</t>
+          <t>ヤニねこ</t>
         </is>
       </c>
       <c r="D59" t="b">
@@ -8541,7 +8684,7 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F59" t="n">
@@ -8549,12 +8692,12 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>POWER</t>
+          <t>なんもねえ</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>ONE OR EIGHT</t>
+          <t>忘れらんねえよ</t>
         </is>
       </c>
       <c r="I59" t="inlineStr"/>
@@ -8573,7 +8716,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>落第賢者の学院無双～二度目の転生、Sランクチート魔術師冒険録～</t>
+          <t>鎧真伝サムライトルーパー 第2クール</t>
         </is>
       </c>
       <c r="D60" t="b">
@@ -8581,7 +8724,7 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F60" t="n">
@@ -8589,12 +8732,12 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>憧憬</t>
+          <t>YOAKE</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>TrySail</t>
+          <t>blank paper</t>
         </is>
       </c>
       <c r="I60" t="inlineStr"/>
@@ -8613,7 +8756,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>領民0人スタートの辺境領主様</t>
+          <t>鎧真伝サムライトルーパー 第2クール</t>
         </is>
       </c>
       <c r="D61" t="b">
@@ -8625,16 +8768,16 @@
         </is>
       </c>
       <c r="F61" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>Wonder</t>
+          <t>BAD遺伝子</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>CROWN HEAD</t>
+          <t>Dannie May</t>
         </is>
       </c>
       <c r="I61" t="inlineStr"/>
@@ -8653,7 +8796,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>領民0人スタートの辺境領主様</t>
+          <t>鎧真伝サムライトルーパー 第2クール</t>
         </is>
       </c>
       <c r="D62" t="b">
@@ -8669,12 +8812,12 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>星降る夜の約束</t>
+          <t>POWER</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>花耶</t>
+          <t>ONE OR EIGHT</t>
         </is>
       </c>
       <c r="I62" t="inlineStr"/>
@@ -8693,7 +8836,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>令和のダラさん</t>
+          <t>鎧真伝サムライトルーパー 第2クール</t>
         </is>
       </c>
       <c r="D63" t="b">
@@ -8701,20 +8844,20 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F63" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>ダラダラ♡ダンシング</t>
+          <t>ばけもん</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>ダラさん（CV：田村睦心） 三⼗⽊⾕⽇向（CV：津田美波） 三⼗⽊⾕薫（CV：寺澤百花） ナレーション（CV：てらそままさき）</t>
+          <t>カラノア</t>
         </is>
       </c>
       <c r="I63" t="inlineStr"/>
@@ -8733,7 +8876,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>LV999の村人</t>
+          <t>落第賢者の学院無双～二度目の転生、Sランクチート魔術師冒険録～</t>
         </is>
       </c>
       <c r="D64" t="b">
@@ -8741,7 +8884,7 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F64" t="n">
@@ -8749,12 +8892,12 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>Not a Hero</t>
+          <t>憧憬</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>藍月なくる&amp;棗いつき</t>
+          <t>TrySail</t>
         </is>
       </c>
       <c r="I64" t="inlineStr"/>
@@ -8773,7 +8916,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>ワールド イズ ダンシング</t>
+          <t>領民0人スタートの辺境領主様</t>
         </is>
       </c>
       <c r="D65" t="b">
@@ -8789,12 +8932,12 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>終宵</t>
+          <t>Wonder</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>マカロニえんぴつ</t>
+          <t>CROWN HEAD</t>
         </is>
       </c>
       <c r="I65" t="inlineStr"/>
@@ -8804,16 +8947,16 @@
     </row>
     <row r="66">
       <c r="A66" t="n">
-        <v>5947</v>
+        <v>5806</v>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2026秋アニメ</t>
+          <t>2026夏アニメ</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>転生した大聖女は、聖女であることをひた隠す</t>
+          <t>領民0人スタートの辺境領主様</t>
         </is>
       </c>
       <c r="D66" t="b">
@@ -8821,7 +8964,7 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F66" t="n">
@@ -8829,7 +8972,7 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>Flare of Soul</t>
+          <t>星降る夜の約束</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
@@ -8844,16 +8987,16 @@
     </row>
     <row r="67">
       <c r="A67" t="n">
-        <v>5947</v>
+        <v>5806</v>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2026秋アニメ</t>
+          <t>2026夏アニメ</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>転生した大聖女は、聖女であることをひた隠す</t>
+          <t>令和のダラさん</t>
         </is>
       </c>
       <c r="D67" t="b">
@@ -8861,7 +9004,7 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F67" t="n">
@@ -8869,12 +9012,12 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>STELLAR</t>
+          <t>ダラダラ♡ダンシング</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>ウタヒメドリーム オールスターズ</t>
+          <t>ダラさん（CV：田村睦心） 三⼗⽊⾕⽇向（CV：津田美波） 三⼗⽊⾕薫（CV：寺澤百花） ナレーション（CV：てらそままさき）</t>
         </is>
       </c>
       <c r="I67" t="inlineStr"/>
@@ -8884,16 +9027,16 @@
     </row>
     <row r="68">
       <c r="A68" t="n">
-        <v>5947</v>
+        <v>5806</v>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>2026秋アニメ</t>
+          <t>2026夏アニメ</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>魔法少女育成計画restart</t>
+          <t>LV999の村人</t>
         </is>
       </c>
       <c r="D68" t="b">
@@ -8909,12 +9052,12 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>No tears here</t>
+          <t>Not a Hero</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>茅原実里</t>
+          <t>藍月なくる&amp;棗いつき</t>
         </is>
       </c>
       <c r="I68" t="inlineStr"/>
@@ -8922,6 +9065,166 @@
       <c r="K68" t="inlineStr"/>
       <c r="L68" t="inlineStr"/>
     </row>
+    <row r="69">
+      <c r="A69" t="n">
+        <v>5806</v>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>2026夏アニメ</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>ワールド イズ ダンシング</t>
+        </is>
+      </c>
+      <c r="D69" t="b">
+        <v>0</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="F69" t="n">
+        <v>1</v>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>終宵</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>マカロニえんぴつ</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr"/>
+      <c r="J69" t="inlineStr"/>
+      <c r="K69" t="inlineStr"/>
+      <c r="L69" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>転生した大聖女は、聖女であることをひた隠す</t>
+        </is>
+      </c>
+      <c r="D70" t="b">
+        <v>0</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="F70" t="n">
+        <v>1</v>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>Flare of Soul</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>花耶</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr"/>
+      <c r="J70" t="inlineStr"/>
+      <c r="K70" t="inlineStr"/>
+      <c r="L70" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>転生した大聖女は、聖女であることをひた隠す</t>
+        </is>
+      </c>
+      <c r="D71" t="b">
+        <v>0</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>ED</t>
+        </is>
+      </c>
+      <c r="F71" t="n">
+        <v>1</v>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>STELLAR</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>ウタヒメドリーム オールスターズ</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr"/>
+      <c r="J71" t="inlineStr"/>
+      <c r="K71" t="inlineStr"/>
+      <c r="L71" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>魔法少女育成計画restart</t>
+        </is>
+      </c>
+      <c r="D72" t="b">
+        <v>0</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="F72" t="n">
+        <v>1</v>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>No tears here</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>茅原実里</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr"/>
+      <c r="J72" t="inlineStr"/>
+      <c r="K72" t="inlineStr"/>
+      <c r="L72" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
auto: anime list update 2026-06-03
</commit_message>
<xml_diff>
--- a/data/anime_list.xlsx
+++ b/data/anime_list.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M122"/>
+  <dimension ref="A1:M123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1246,14 +1246,30 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2026年7月～ テレビ朝日系列・BS朝日にて</t>
+          <t>2026年7月4日（土）～ テレビ朝日系列・BS朝日にて</t>
         </is>
       </c>
       <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr"/>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>いつかちゃんと。</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>りりあ。</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>最終回</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>sorato</t>
+        </is>
+      </c>
       <c r="M17" t="inlineStr">
         <is>
           <t>https://www.animatetimes.com/tag/details.php?id=27779</t>
@@ -5615,7 +5631,7 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>バーテックスフォース</t>
+          <t>鳴海の平日</t>
         </is>
       </c>
       <c r="E107" t="b">
@@ -5623,17 +5639,17 @@
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>TVアニメ</t>
+          <t>配信</t>
         </is>
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>2026年10月〜</t>
+          <t>2026年秋</t>
         </is>
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>SMDE</t>
+          <t>Production I.G</t>
         </is>
       </c>
       <c r="I107" t="inlineStr"/>
@@ -5642,7 +5658,7 @@
       <c r="L107" t="inlineStr"/>
       <c r="M107" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27988</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28465</t>
         </is>
       </c>
     </row>
@@ -5660,7 +5676,7 @@
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Battle Spirits [Re] 絶界の空</t>
+          <t>バーテックスフォース</t>
         </is>
       </c>
       <c r="E108" t="b">
@@ -5673,17 +5689,21 @@
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>2026年秋</t>
-        </is>
-      </c>
-      <c r="H108" t="inlineStr"/>
+          <t>2026年10月〜</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>SMDE</t>
+        </is>
+      </c>
       <c r="I108" t="inlineStr"/>
       <c r="J108" t="inlineStr"/>
       <c r="K108" t="inlineStr"/>
       <c r="L108" t="inlineStr"/>
       <c r="M108" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27954</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27988</t>
         </is>
       </c>
     </row>
@@ -5701,7 +5721,7 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>パンどろぼう</t>
+          <t>Battle Spirits [Re] 絶界の空</t>
         </is>
       </c>
       <c r="E109" t="b">
@@ -5714,7 +5734,7 @@
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>2026年10月〜 NHK Eテレにて</t>
+          <t>2026年秋</t>
         </is>
       </c>
       <c r="H109" t="inlineStr"/>
@@ -5724,7 +5744,7 @@
       <c r="L109" t="inlineStr"/>
       <c r="M109" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26163</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27954</t>
         </is>
       </c>
     </row>
@@ -5742,7 +5762,7 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>百妖譜 京師篇</t>
+          <t>パンどろぼう</t>
         </is>
       </c>
       <c r="E110" t="b">
@@ -5755,7 +5775,7 @@
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>2026年10月〜 フジテレビ「B8station」にて</t>
+          <t>2026年10月〜 NHK Eテレにて</t>
         </is>
       </c>
       <c r="H110" t="inlineStr"/>
@@ -5765,7 +5785,7 @@
       <c r="L110" t="inlineStr"/>
       <c r="M110" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27781</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26163</t>
         </is>
       </c>
     </row>
@@ -5783,7 +5803,7 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>冰剣の魔術師が世界を統べるⅡ</t>
+          <t>百妖譜 京師篇</t>
         </is>
       </c>
       <c r="E111" t="b">
@@ -5796,21 +5816,17 @@
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>2026年10月〜</t>
-        </is>
-      </c>
-      <c r="H111" t="inlineStr">
-        <is>
-          <t>ゼロジー</t>
-        </is>
-      </c>
+          <t>2026年10月〜 フジテレビ「B8station」にて</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr"/>
       <c r="I111" t="inlineStr"/>
       <c r="J111" t="inlineStr"/>
       <c r="K111" t="inlineStr"/>
       <c r="L111" t="inlineStr"/>
       <c r="M111" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28403</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27781</t>
         </is>
       </c>
     </row>
@@ -5828,7 +5844,7 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>ホタルの嫁入り</t>
+          <t>冰剣の魔術師が世界を統べるⅡ</t>
         </is>
       </c>
       <c r="E112" t="b">
@@ -5841,12 +5857,12 @@
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>2026年10月～ 全国フジテレビ系“ ノイタミナ ”にて</t>
+          <t>2026年10月〜</t>
         </is>
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>david production</t>
+          <t>ゼロジー</t>
         </is>
       </c>
       <c r="I112" t="inlineStr"/>
@@ -5855,7 +5871,7 @@
       <c r="L112" t="inlineStr"/>
       <c r="M112" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27415</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28403</t>
         </is>
       </c>
     </row>
@@ -5873,7 +5889,7 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>ポップパップポルターズ</t>
+          <t>ホタルの嫁入り</t>
         </is>
       </c>
       <c r="E113" t="b">
@@ -5886,12 +5902,12 @@
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>2026年秋 テレビ朝日にて</t>
+          <t>2026年10月～ 全国フジテレビ系“ ノイタミナ ”にて</t>
         </is>
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>MOZU STUDIOS</t>
+          <t>david production</t>
         </is>
       </c>
       <c r="I113" t="inlineStr"/>
@@ -5900,7 +5916,7 @@
       <c r="L113" t="inlineStr"/>
       <c r="M113" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27823</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27415</t>
         </is>
       </c>
     </row>
@@ -5918,7 +5934,7 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>ホテル・インヒューマンズ 第2期</t>
+          <t>ポップパップポルターズ</t>
         </is>
       </c>
       <c r="E114" t="b">
@@ -5931,12 +5947,12 @@
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>2026年10月～ テレ東系列ほか</t>
+          <t>2026年秋 テレビ朝日にて</t>
         </is>
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>ブリッジ</t>
+          <t>MOZU STUDIOS</t>
         </is>
       </c>
       <c r="I114" t="inlineStr"/>
@@ -5945,7 +5961,7 @@
       <c r="L114" t="inlineStr"/>
       <c r="M114" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26870</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27823</t>
         </is>
       </c>
     </row>
@@ -5963,7 +5979,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>マジカル★エクスプローラー</t>
+          <t>ホテル・インヒューマンズ 第2期</t>
         </is>
       </c>
       <c r="E115" t="b">
@@ -5976,12 +5992,12 @@
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>2026年秋</t>
+          <t>2026年10月～ テレ東系列ほか</t>
         </is>
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>WHITE FOX</t>
+          <t>ブリッジ</t>
         </is>
       </c>
       <c r="I115" t="inlineStr"/>
@@ -5990,7 +6006,7 @@
       <c r="L115" t="inlineStr"/>
       <c r="M115" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=23375</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26870</t>
         </is>
       </c>
     </row>
@@ -6008,7 +6024,7 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>魔法騎士レイアース</t>
+          <t>マジカル★エクスプローラー</t>
         </is>
       </c>
       <c r="E116" t="b">
@@ -6021,12 +6037,12 @@
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>2026年10月～ テレビ朝日系列にて</t>
+          <t>2026年秋</t>
         </is>
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>E&amp;H production</t>
+          <t>WHITE FOX</t>
         </is>
       </c>
       <c r="I116" t="inlineStr"/>
@@ -6035,7 +6051,7 @@
       <c r="L116" t="inlineStr"/>
       <c r="M116" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=24301</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=23375</t>
         </is>
       </c>
     </row>
@@ -6053,7 +6069,7 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>魔法少女育成計画restart</t>
+          <t>魔法騎士レイアース</t>
         </is>
       </c>
       <c r="E117" t="b">
@@ -6066,29 +6082,21 @@
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>2026年秋</t>
+          <t>2026年10月～ テレビ朝日系列にて</t>
         </is>
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>SynergySP</t>
-        </is>
-      </c>
-      <c r="I117" t="inlineStr">
-        <is>
-          <t>No tears here</t>
-        </is>
-      </c>
-      <c r="J117" t="inlineStr">
-        <is>
-          <t>茅原実里</t>
-        </is>
-      </c>
+          <t>E&amp;H production</t>
+        </is>
+      </c>
+      <c r="I117" t="inlineStr"/>
+      <c r="J117" t="inlineStr"/>
       <c r="K117" t="inlineStr"/>
       <c r="L117" t="inlineStr"/>
       <c r="M117" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26693</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=24301</t>
         </is>
       </c>
     </row>
@@ -6106,7 +6114,7 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>マロニエ王国の七人の騎士</t>
+          <t>魔法少女育成計画restart</t>
         </is>
       </c>
       <c r="E118" t="b">
@@ -6119,21 +6127,29 @@
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>2026年10月～ NHK Eテレにて</t>
+          <t>2026年秋</t>
         </is>
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>J.C.STAFF</t>
-        </is>
-      </c>
-      <c r="I118" t="inlineStr"/>
-      <c r="J118" t="inlineStr"/>
+          <t>SynergySP</t>
+        </is>
+      </c>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>No tears here</t>
+        </is>
+      </c>
+      <c r="J118" t="inlineStr">
+        <is>
+          <t>茅原実里</t>
+        </is>
+      </c>
       <c r="K118" t="inlineStr"/>
       <c r="L118" t="inlineStr"/>
       <c r="M118" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28456</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26693</t>
         </is>
       </c>
     </row>
@@ -6151,7 +6167,7 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>目覚めたら最強装備と宇宙船持ちだったので、一戸建て目指して傭兵として自由に生きたい</t>
+          <t>マロニエ王国の七人の騎士</t>
         </is>
       </c>
       <c r="E119" t="b">
@@ -6164,12 +6180,12 @@
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>2026年10月〜</t>
+          <t>2026年10月～ NHK Eテレにて</t>
         </is>
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>studio A-CAT</t>
+          <t>J.C.STAFF</t>
         </is>
       </c>
       <c r="I119" t="inlineStr"/>
@@ -6178,7 +6194,7 @@
       <c r="L119" t="inlineStr"/>
       <c r="M119" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25525</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28456</t>
         </is>
       </c>
     </row>
@@ -6196,7 +6212,7 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>弱気MAX令嬢なのに、辣腕婚約者様の賭けに乗ってしまった</t>
+          <t>目覚めたら最強装備と宇宙船持ちだったので、一戸建て目指して傭兵として自由に生きたい</t>
         </is>
       </c>
       <c r="E120" t="b">
@@ -6209,12 +6225,12 @@
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
+          <t>2026年10月〜</t>
         </is>
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>寿門堂</t>
+          <t>studio A-CAT</t>
         </is>
       </c>
       <c r="I120" t="inlineStr"/>
@@ -6223,7 +6239,7 @@
       <c r="L120" t="inlineStr"/>
       <c r="M120" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26947</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25525</t>
         </is>
       </c>
     </row>
@@ -6241,7 +6257,7 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>らんま1/2 第3期</t>
+          <t>弱気MAX令嬢なのに、辣腕婚約者様の賭けに乗ってしまった</t>
         </is>
       </c>
       <c r="E121" t="b">
@@ -6254,17 +6270,21 @@
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>2026年10月～ 日本テレビ系にて</t>
-        </is>
-      </c>
-      <c r="H121" t="inlineStr"/>
+          <t>2026年10月～</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>寿門堂</t>
+        </is>
+      </c>
       <c r="I121" t="inlineStr"/>
       <c r="J121" t="inlineStr"/>
       <c r="K121" t="inlineStr"/>
       <c r="L121" t="inlineStr"/>
       <c r="M121" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28013</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26947</t>
         </is>
       </c>
     </row>
@@ -6282,7 +6302,7 @@
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>LEGO® ONE PIECE</t>
+          <t>らんま1/2 第3期</t>
         </is>
       </c>
       <c r="E122" t="b">
@@ -6290,12 +6310,12 @@
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>配信</t>
+          <t>TVアニメ</t>
         </is>
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>2026年9月29日（火） Netflixにて</t>
+          <t>2026年10月～ 日本テレビ系にて</t>
         </is>
       </c>
       <c r="H122" t="inlineStr"/>
@@ -6304,6 +6324,47 @@
       <c r="K122" t="inlineStr"/>
       <c r="L122" t="inlineStr"/>
       <c r="M122" t="inlineStr">
+        <is>
+          <t>https://www.animatetimes.com/tag/details.php?id=28013</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C123" t="n">
+        <v>46</v>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>LEGO® ONE PIECE</t>
+        </is>
+      </c>
+      <c r="E123" t="b">
+        <v>0</v>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>配信</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>2026年9月29日（火） Netflixにて</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr"/>
+      <c r="I123" t="inlineStr"/>
+      <c r="J123" t="inlineStr"/>
+      <c r="K123" t="inlineStr"/>
+      <c r="L123" t="inlineStr"/>
+      <c r="M123" t="inlineStr">
         <is>
           <t>https://www.animatetimes.com/tag/details.php?id=28168</t>
         </is>
@@ -6320,7 +6381,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L72"/>
+  <dimension ref="A1:L74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6916,7 +6977,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>ぐらんぶる Season 3</t>
+          <t>「きみを愛する気はない」と言った次期公爵様がなぜか溺愛してきます</t>
         </is>
       </c>
       <c r="D15" t="b">
@@ -6932,12 +6993,12 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>夏子</t>
+          <t>いつかちゃんと。</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>FUNKY MONKEY BΛBY'S</t>
+          <t>りりあ。</t>
         </is>
       </c>
       <c r="I15" t="inlineStr"/>
@@ -6956,7 +7017,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>ぐらんぶる Season 3</t>
+          <t>「きみを愛する気はない」と言った次期公爵様がなぜか溺愛してきます</t>
         </is>
       </c>
       <c r="D16" t="b">
@@ -6972,12 +7033,12 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>裸のマーメード</t>
+          <t>最終回</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>豆柴の大群</t>
+          <t>sorato</t>
         </is>
       </c>
       <c r="I16" t="inlineStr"/>
@@ -6996,7 +7057,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>クレバテスII-魔獣の王と偽りの勇者伝承-</t>
+          <t>ぐらんぶる Season 3</t>
         </is>
       </c>
       <c r="D17" t="b">
@@ -7004,7 +7065,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F17" t="n">
@@ -7012,12 +7073,12 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Awake Anew</t>
+          <t>夏子</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>MYTH &amp; ROID</t>
+          <t>FUNKY MONKEY BΛBY'S</t>
         </is>
       </c>
       <c r="I17" t="inlineStr"/>
@@ -7036,7 +7097,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>コードギアス 奪還のロゼ TV放送</t>
+          <t>ぐらんぶる Season 3</t>
         </is>
       </c>
       <c r="D18" t="b">
@@ -7044,7 +7105,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F18" t="n">
@@ -7052,12 +7113,12 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Running In My Head</t>
+          <t>裸のマーメード</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>MIYAVI</t>
+          <t>豆柴の大群</t>
         </is>
       </c>
       <c r="I18" t="inlineStr"/>
@@ -7076,7 +7137,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>コードギアス 奪還のロゼ TV放送</t>
+          <t>クレバテスII-魔獣の王と偽りの勇者伝承-</t>
         </is>
       </c>
       <c r="D19" t="b">
@@ -7092,12 +7153,12 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>ロゼ (Prod.TeddyLoid)</t>
+          <t>Awake Anew</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>満島ひかり</t>
+          <t>MYTH &amp; ROID</t>
         </is>
       </c>
       <c r="I19" t="inlineStr"/>
@@ -7116,7 +7177,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>これ描いて死ね</t>
+          <t>コードギアス 奪還のロゼ TV放送</t>
         </is>
       </c>
       <c r="D20" t="b">
@@ -7132,12 +7193,12 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>遺書</t>
+          <t>Running In My Head</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>キタニタツヤ</t>
+          <t>MIYAVI</t>
         </is>
       </c>
       <c r="I20" t="inlineStr"/>
@@ -7156,7 +7217,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>才女のお世話 高嶺の花だらけな名門校で、学院一のお嬢様(生活能力皆無)を陰ながらお世話することになりました</t>
+          <t>コードギアス 奪還のロゼ TV放送</t>
         </is>
       </c>
       <c r="D21" t="b">
@@ -7164,7 +7225,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F21" t="n">
@@ -7172,12 +7233,12 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>最最最高級のお世話して</t>
+          <t>ロゼ (Prod.TeddyLoid)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>angela</t>
+          <t>満島ひかり</t>
         </is>
       </c>
       <c r="I21" t="inlineStr"/>
@@ -7196,7 +7257,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>サイボーグ009 ネメシス</t>
+          <t>これ描いて死ね</t>
         </is>
       </c>
       <c r="D22" t="b">
@@ -7212,12 +7273,12 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>誰がために</t>
+          <t>遺書</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>杏子</t>
+          <t>キタニタツヤ</t>
         </is>
       </c>
       <c r="I22" t="inlineStr"/>
@@ -7236,7 +7297,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>さよならララ</t>
+          <t>才女のお世話 高嶺の花だらけな名門校で、学院一のお嬢様(生活能力皆無)を陰ながらお世話することになりました</t>
         </is>
       </c>
       <c r="D23" t="b">
@@ -7252,12 +7313,12 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>さよならララ</t>
+          <t>最最最高級のお世話して</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>いきものがかり</t>
+          <t>angela</t>
         </is>
       </c>
       <c r="I23" t="inlineStr"/>
@@ -7276,7 +7337,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>スーパーの裏でヤニ吸うふたり</t>
+          <t>サイボーグ009 ネメシス</t>
         </is>
       </c>
       <c r="D24" t="b">
@@ -7292,12 +7353,12 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>イチジク煙</t>
+          <t>誰がために</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>ずっと真夜中でいいのに。</t>
+          <t>杏子</t>
         </is>
       </c>
       <c r="I24" t="inlineStr"/>
@@ -7316,7 +7377,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>スーパーの裏でヤニ吸うふたり</t>
+          <t>さよならララ</t>
         </is>
       </c>
       <c r="D25" t="b">
@@ -7324,7 +7385,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F25" t="n">
@@ -7332,12 +7393,12 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Fiction</t>
+          <t>さよならララ</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>imase</t>
+          <t>いきものがかり</t>
         </is>
       </c>
       <c r="I25" t="inlineStr"/>
@@ -7356,7 +7417,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>捨てられ聖女の異世界ごはん旅 隠れスキルでキャンピングカーを召喚しました</t>
+          <t>スーパーの裏でヤニ吸うふたり</t>
         </is>
       </c>
       <c r="D26" t="b">
@@ -7372,12 +7433,12 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Butterfly</t>
+          <t>イチジク煙</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>INUWASI</t>
+          <t>ずっと真夜中でいいのに。</t>
         </is>
       </c>
       <c r="I26" t="inlineStr"/>
@@ -7396,7 +7457,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>捨てられ聖女の異世界ごはん旅 隠れスキルでキャンピングカーを召喚しました</t>
+          <t>スーパーの裏でヤニ吸うふたり</t>
         </is>
       </c>
       <c r="D27" t="b">
@@ -7412,12 +7473,12 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Holy Sweet Home</t>
+          <t>Fiction</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>音感れもねゐど</t>
+          <t>imase</t>
         </is>
       </c>
       <c r="I27" t="inlineStr"/>
@@ -7436,7 +7497,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>正反対な君と僕 第2期</t>
+          <t>捨てられ聖女の異世界ごはん旅 隠れスキルでキャンピングカーを召喚しました</t>
         </is>
       </c>
       <c r="D28" t="b">
@@ -7452,12 +7513,12 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>メガネを外して</t>
+          <t>Butterfly</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>乃紫</t>
+          <t>INUWASI</t>
         </is>
       </c>
       <c r="I28" t="inlineStr"/>
@@ -7476,7 +7537,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>正反対な君と僕 第2期</t>
+          <t>捨てられ聖女の異世界ごはん旅 隠れスキルでキャンピングカーを召喚しました</t>
         </is>
       </c>
       <c r="D29" t="b">
@@ -7484,20 +7545,20 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F29" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>猫じゃらし</t>
+          <t>Holy Sweet Home</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>7co</t>
+          <t>音感れもねゐど</t>
         </is>
       </c>
       <c r="I29" t="inlineStr"/>
@@ -7524,7 +7585,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F30" t="n">
@@ -7532,12 +7593,12 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>ピュア feat. 橋本絵莉子</t>
+          <t>メガネを外して</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>PAS TASTA</t>
+          <t>乃紫</t>
         </is>
       </c>
       <c r="I30" t="inlineStr"/>
@@ -7556,7 +7617,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>対ありでした。～お嬢さまは格闘ゲームなんてしない～</t>
+          <t>正反対な君と僕 第2期</t>
         </is>
       </c>
       <c r="D31" t="b">
@@ -7568,16 +7629,16 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>命短し対する乙女よ</t>
+          <t>猫じゃらし</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>花冷え。</t>
+          <t>7co</t>
         </is>
       </c>
       <c r="I31" t="inlineStr"/>
@@ -7596,7 +7657,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>追放された転生重騎士はゲーム知識で無双する</t>
+          <t>正反対な君と僕 第2期</t>
         </is>
       </c>
       <c r="D32" t="b">
@@ -7604,7 +7665,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F32" t="n">
@@ -7612,12 +7673,12 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Awake</t>
+          <t>ピュア feat. 橋本絵莉子</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>SPYAIR</t>
+          <t>PAS TASTA</t>
         </is>
       </c>
       <c r="I32" t="inlineStr"/>
@@ -7636,7 +7697,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>鉄鍋のジャン！</t>
+          <t>対ありでした。～お嬢さまは格闘ゲームなんてしない～</t>
         </is>
       </c>
       <c r="D33" t="b">
@@ -7652,12 +7713,12 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>火宴</t>
+          <t>命短し対する乙女よ</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>原因は自分にある。</t>
+          <t>花冷え。</t>
         </is>
       </c>
       <c r="I33" t="inlineStr"/>
@@ -7676,7 +7737,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>手札が多めのビクトリア</t>
+          <t>追放された転生重騎士はゲーム知識で無双する</t>
         </is>
       </c>
       <c r="D34" t="b">
@@ -7684,7 +7745,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F34" t="n">
@@ -7692,12 +7753,12 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>縁のつき</t>
+          <t>Awake</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>KI_EN</t>
+          <t>SPYAIR</t>
         </is>
       </c>
       <c r="I34" t="inlineStr"/>
@@ -7716,7 +7777,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>転校先の清楚可憐な美少女が、昔男子と思って一緒に遊んだ幼馴染だった件</t>
+          <t>鉄鍋のジャン！</t>
         </is>
       </c>
       <c r="D35" t="b">
@@ -7732,12 +7793,12 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>夏に重ねて</t>
+          <t>火宴</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>DIALOGUE+</t>
+          <t>原因は自分にある。</t>
         </is>
       </c>
       <c r="I35" t="inlineStr"/>
@@ -7756,7 +7817,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>天は赤い河のほとり</t>
+          <t>手札が多めのビクトリア</t>
         </is>
       </c>
       <c r="D36" t="b">
@@ -7764,7 +7825,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F36" t="n">
@@ -7772,12 +7833,12 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>暁の空</t>
+          <t>縁のつき</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>七海ひろき</t>
+          <t>KI_EN</t>
         </is>
       </c>
       <c r="I36" t="inlineStr"/>
@@ -7796,7 +7857,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>天幕のジャードゥーガル</t>
+          <t>転校先の清楚可憐な美少女が、昔男子と思って一緒に遊んだ幼馴染だった件</t>
         </is>
       </c>
       <c r="D37" t="b">
@@ -7812,12 +7873,12 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Stella</t>
+          <t>夏に重ねて</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>SEKAI NO OWARI</t>
+          <t>DIALOGUE+</t>
         </is>
       </c>
       <c r="I37" t="inlineStr"/>
@@ -7836,7 +7897,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>盗掘王</t>
+          <t>天は赤い河のほとり</t>
         </is>
       </c>
       <c r="D38" t="b">
@@ -7852,12 +7913,12 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>SHOW DOWN</t>
+          <t>暁の空</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>QWER</t>
+          <t>七海ひろき</t>
         </is>
       </c>
       <c r="I38" t="inlineStr"/>
@@ -7876,7 +7937,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>透明な夜に駆ける君と、目に見えない恋をした。</t>
+          <t>天幕のジャードゥーガル</t>
         </is>
       </c>
       <c r="D39" t="b">
@@ -7884,7 +7945,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F39" t="n">
@@ -7892,12 +7953,12 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>光</t>
+          <t>Stella</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>櫻井優衣</t>
+          <t>SEKAI NO OWARI</t>
         </is>
       </c>
       <c r="I39" t="inlineStr"/>
@@ -7916,7 +7977,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>二十世紀電氣目録-ユーレカ・エヴリカ-</t>
+          <t>盗掘王</t>
         </is>
       </c>
       <c r="D40" t="b">
@@ -7932,12 +7993,12 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>ユーレカ・エヴリカ</t>
+          <t>SHOW DOWN</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>五阿弥ルナ</t>
+          <t>QWER</t>
         </is>
       </c>
       <c r="I40" t="inlineStr"/>
@@ -7956,7 +8017,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>パイの実 おしの森へようこそ！</t>
+          <t>透明な夜に駆ける君と、目に見えない恋をした。</t>
         </is>
       </c>
       <c r="D41" t="b">
@@ -7964,7 +8025,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>主題歌</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F41" t="n">
@@ -7972,12 +8033,12 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>パイしか勝たん！推しの森活</t>
+          <t>光</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>安保心結</t>
+          <t>櫻井優衣</t>
         </is>
       </c>
       <c r="I41" t="inlineStr"/>
@@ -7996,7 +8057,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>刃牙道 第2クール</t>
+          <t>二十世紀電氣目録-ユーレカ・エヴリカ-</t>
         </is>
       </c>
       <c r="D42" t="b">
@@ -8012,12 +8073,12 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>フルボコ</t>
+          <t>ユーレカ・エヴリカ</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>WANIMA</t>
+          <t>五阿弥ルナ</t>
         </is>
       </c>
       <c r="I42" t="inlineStr"/>
@@ -8036,7 +8097,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>刃牙道 第2クール</t>
+          <t>パイの実 おしの森へようこそ！</t>
         </is>
       </c>
       <c r="D43" t="b">
@@ -8044,7 +8105,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>主題歌</t>
         </is>
       </c>
       <c r="F43" t="n">
@@ -8052,12 +8113,12 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Mountain Top</t>
+          <t>パイしか勝たん！推しの森活</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>Novel Core</t>
+          <t>安保心結</t>
         </is>
       </c>
       <c r="I43" t="inlineStr"/>
@@ -8076,7 +8137,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>花ざかりの君たちへ 第2期</t>
+          <t>刃牙道 第2クール</t>
         </is>
       </c>
       <c r="D44" t="b">
@@ -8092,12 +8153,12 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>FLASHBULB</t>
+          <t>フルボコ</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>Omoinotake</t>
+          <t>WANIMA</t>
         </is>
       </c>
       <c r="I44" t="inlineStr"/>
@@ -8116,7 +8177,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>花ざかりの君たちへ 第2期</t>
+          <t>刃牙道 第2クール</t>
         </is>
       </c>
       <c r="D45" t="b">
@@ -8132,12 +8193,12 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>花束</t>
+          <t>Mountain Top</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>Omoinotake</t>
+          <t>Novel Core</t>
         </is>
       </c>
       <c r="I45" t="inlineStr"/>
@@ -8156,7 +8217,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>ヒロイン？聖女？いいえ、オールワークスメイドです（誇）！</t>
+          <t>花ざかりの君たちへ 第2期</t>
         </is>
       </c>
       <c r="D46" t="b">
@@ -8172,12 +8233,12 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>マデュアル↔ハート</t>
+          <t>FLASHBULB</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>メロディ・ウェーブ(CV：宮本侑芽) ルシアナ・ルトルバーグ(CV：大久保瑠美)</t>
+          <t>Omoinotake</t>
         </is>
       </c>
       <c r="I46" t="inlineStr"/>
@@ -8196,7 +8257,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>ヒロイン？聖女？いいえ、オールワークスメイドです（誇）！</t>
+          <t>花ざかりの君たちへ 第2期</t>
         </is>
       </c>
       <c r="D47" t="b">
@@ -8212,12 +8273,12 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>ハンドメイド</t>
+          <t>花束</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>仲村宗悟</t>
+          <t>Omoinotake</t>
         </is>
       </c>
       <c r="I47" t="inlineStr"/>
@@ -8236,7 +8297,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>ブチ切れ令嬢は報復を誓いました。 ～魔導書の力で祖国を叩き潰します～</t>
+          <t>ヒロイン？聖女？いいえ、オールワークスメイドです（誇）！</t>
         </is>
       </c>
       <c r="D48" t="b">
@@ -8252,12 +8313,12 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Q.E.D.</t>
+          <t>マデュアル↔ハート</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>小倉唯</t>
+          <t>メロディ・ウェーブ(CV：宮本侑芽) ルシアナ・ルトルバーグ(CV：大久保瑠美)</t>
         </is>
       </c>
       <c r="I48" t="inlineStr"/>
@@ -8276,7 +8337,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>ブチ切れ令嬢は報復を誓いました。 ～魔導書の力で祖国を叩き潰します～</t>
+          <t>ヒロイン？聖女？いいえ、オールワークスメイドです（誇）！</t>
         </is>
       </c>
       <c r="D49" t="b">
@@ -8292,12 +8353,12 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>グッバイ・ララバイ</t>
+          <t>ハンドメイド</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>大西亜玖璃</t>
+          <t>仲村宗悟</t>
         </is>
       </c>
       <c r="I49" t="inlineStr"/>
@@ -8316,7 +8377,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>プラノサウルス ガチコセイブツ部</t>
+          <t>ブチ切れ令嬢は報復を誓いました。 ～魔導書の力で祖国を叩き潰します～</t>
         </is>
       </c>
       <c r="D50" t="b">
@@ -8324,7 +8385,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>主題歌</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F50" t="n">
@@ -8332,12 +8393,12 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>ガチde古生</t>
+          <t>Q.E.D.</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>リンクルプラネット</t>
+          <t>小倉唯</t>
         </is>
       </c>
       <c r="I50" t="inlineStr"/>
@@ -8356,7 +8417,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>炎の闘球女 ドッジ弾子</t>
+          <t>ブチ切れ令嬢は報復を誓いました。 ～魔導書の力で祖国を叩き潰します～</t>
         </is>
       </c>
       <c r="D51" t="b">
@@ -8364,7 +8425,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F51" t="n">
@@ -8372,12 +8433,12 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>会心の一劇</t>
+          <t>グッバイ・ララバイ</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>ももいろクローバーZ</t>
+          <t>大西亜玖璃</t>
         </is>
       </c>
       <c r="I51" t="inlineStr"/>
@@ -8396,7 +8457,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>炎の闘球女 ドッジ弾子</t>
+          <t>プラノサウルス ガチコセイブツ部</t>
         </is>
       </c>
       <c r="D52" t="b">
@@ -8404,7 +8465,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>主題歌</t>
         </is>
       </c>
       <c r="F52" t="n">
@@ -8412,12 +8473,12 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Welcome to あざとさワールド</t>
+          <t>ガチde古生</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>i☆Ris</t>
+          <t>リンクルプラネット</t>
         </is>
       </c>
       <c r="I52" t="inlineStr"/>
@@ -8436,7 +8497,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>魔法少女リリカルなのは EXCEEDS Gun Blaze Vengeance</t>
+          <t>炎の闘球女 ドッジ弾子</t>
         </is>
       </c>
       <c r="D53" t="b">
@@ -8452,12 +8513,12 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>CRIMSON BULLET</t>
+          <t>会心の一劇</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>水樹奈々</t>
+          <t>ももいろクローバーZ</t>
         </is>
       </c>
       <c r="I53" t="inlineStr"/>
@@ -8476,7 +8537,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>魔法少女リリカルなのは EXCEEDS Gun Blaze Vengeance</t>
+          <t>炎の闘球女 ドッジ弾子</t>
         </is>
       </c>
       <c r="D54" t="b">
@@ -8492,12 +8553,12 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Ephemeral</t>
+          <t>Welcome to あざとさワールド</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>青木陽菜</t>
+          <t>i☆Ris</t>
         </is>
       </c>
       <c r="I54" t="inlineStr"/>
@@ -8516,7 +8577,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>無自覚聖女は今日も無意識に力を垂れ流す</t>
+          <t>魔法少女リリカルなのは EXCEEDS Gun Blaze Vengeance</t>
         </is>
       </c>
       <c r="D55" t="b">
@@ -8532,12 +8593,12 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>Windmaker</t>
+          <t>CRIMSON BULLET</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>花耶</t>
+          <t>水樹奈々</t>
         </is>
       </c>
       <c r="I55" t="inlineStr"/>
@@ -8556,7 +8617,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>無自覚聖女は今日も無意識に力を垂れ流す</t>
+          <t>魔法少女リリカルなのは EXCEEDS Gun Blaze Vengeance</t>
         </is>
       </c>
       <c r="D56" t="b">
@@ -8572,12 +8633,12 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>アンノウンミー</t>
+          <t>Ephemeral</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>ウタヒメドリーム オールスターズ【夢咲いぶき（CV:山﨑玲奈） 桜木舞華（CV:鈴木杏奈） 真白清美（CV:其原有沙） HiREN（CV:花耶） 水月ひかり（CV:礒部花凜） 高木凛（CV:鷲見友美ジェナ） 萩原ひまわり（CV:倉知玲鳳） SAKURAKO（CV:竹内夢）】</t>
+          <t>青木陽菜</t>
         </is>
       </c>
       <c r="I56" t="inlineStr"/>
@@ -8596,7 +8657,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>無職転生Ⅲ ～異世界行ったら本気だす～</t>
+          <t>無自覚聖女は今日も無意識に力を垂れ流す</t>
         </is>
       </c>
       <c r="D57" t="b">
@@ -8612,12 +8673,12 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>決意の唄</t>
+          <t>Windmaker</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>大原ゆい子</t>
+          <t>花耶</t>
         </is>
       </c>
       <c r="I57" t="inlineStr"/>
@@ -8636,7 +8697,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>メビウス・ダスト</t>
+          <t>無自覚聖女は今日も無意識に力を垂れ流す</t>
         </is>
       </c>
       <c r="D58" t="b">
@@ -8644,7 +8705,7 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F58" t="n">
@@ -8652,12 +8713,12 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>メビウス</t>
+          <t>アンノウンミー</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>家入レオ</t>
+          <t>ウタヒメドリーム オールスターズ【夢咲いぶき（CV:山﨑玲奈） 桜木舞華（CV:鈴木杏奈） 真白清美（CV:其原有沙） HiREN（CV:花耶） 水月ひかり（CV:礒部花凜） 高木凛（CV:鷲見友美ジェナ） 萩原ひまわり（CV:倉知玲鳳） SAKURAKO（CV:竹内夢）】</t>
         </is>
       </c>
       <c r="I58" t="inlineStr"/>
@@ -8676,7 +8737,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>ヤニねこ</t>
+          <t>無職転生Ⅲ ～異世界行ったら本気だす～</t>
         </is>
       </c>
       <c r="D59" t="b">
@@ -8692,12 +8753,12 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>なんもねえ</t>
+          <t>決意の唄</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>忘れらんねえよ</t>
+          <t>大原ゆい子</t>
         </is>
       </c>
       <c r="I59" t="inlineStr"/>
@@ -8716,7 +8777,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>鎧真伝サムライトルーパー 第2クール</t>
+          <t>メビウス・ダスト</t>
         </is>
       </c>
       <c r="D60" t="b">
@@ -8732,12 +8793,12 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>YOAKE</t>
+          <t>メビウス</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>blank paper</t>
+          <t>家入レオ</t>
         </is>
       </c>
       <c r="I60" t="inlineStr"/>
@@ -8756,7 +8817,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>鎧真伝サムライトルーパー 第2クール</t>
+          <t>ヤニねこ</t>
         </is>
       </c>
       <c r="D61" t="b">
@@ -8768,16 +8829,16 @@
         </is>
       </c>
       <c r="F61" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>BAD遺伝子</t>
+          <t>なんもねえ</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>Dannie May</t>
+          <t>忘れらんねえよ</t>
         </is>
       </c>
       <c r="I61" t="inlineStr"/>
@@ -8804,7 +8865,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F62" t="n">
@@ -8812,12 +8873,12 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>POWER</t>
+          <t>YOAKE</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>ONE OR EIGHT</t>
+          <t>blank paper</t>
         </is>
       </c>
       <c r="I62" t="inlineStr"/>
@@ -8844,7 +8905,7 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F63" t="n">
@@ -8852,12 +8913,12 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>ばけもん</t>
+          <t>BAD遺伝子</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>カラノア</t>
+          <t>Dannie May</t>
         </is>
       </c>
       <c r="I63" t="inlineStr"/>
@@ -8876,7 +8937,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>落第賢者の学院無双～二度目の転生、Sランクチート魔術師冒険録～</t>
+          <t>鎧真伝サムライトルーパー 第2クール</t>
         </is>
       </c>
       <c r="D64" t="b">
@@ -8892,12 +8953,12 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>憧憬</t>
+          <t>POWER</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>TrySail</t>
+          <t>ONE OR EIGHT</t>
         </is>
       </c>
       <c r="I64" t="inlineStr"/>
@@ -8916,7 +8977,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>領民0人スタートの辺境領主様</t>
+          <t>鎧真伝サムライトルーパー 第2クール</t>
         </is>
       </c>
       <c r="D65" t="b">
@@ -8924,20 +8985,20 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F65" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>Wonder</t>
+          <t>ばけもん</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>CROWN HEAD</t>
+          <t>カラノア</t>
         </is>
       </c>
       <c r="I65" t="inlineStr"/>
@@ -8956,7 +9017,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>領民0人スタートの辺境領主様</t>
+          <t>落第賢者の学院無双～二度目の転生、Sランクチート魔術師冒険録～</t>
         </is>
       </c>
       <c r="D66" t="b">
@@ -8972,12 +9033,12 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>星降る夜の約束</t>
+          <t>憧憬</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>花耶</t>
+          <t>TrySail</t>
         </is>
       </c>
       <c r="I66" t="inlineStr"/>
@@ -8996,7 +9057,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>令和のダラさん</t>
+          <t>領民0人スタートの辺境領主様</t>
         </is>
       </c>
       <c r="D67" t="b">
@@ -9012,12 +9073,12 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>ダラダラ♡ダンシング</t>
+          <t>Wonder</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>ダラさん（CV：田村睦心） 三⼗⽊⾕⽇向（CV：津田美波） 三⼗⽊⾕薫（CV：寺澤百花） ナレーション（CV：てらそままさき）</t>
+          <t>CROWN HEAD</t>
         </is>
       </c>
       <c r="I67" t="inlineStr"/>
@@ -9036,7 +9097,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>LV999の村人</t>
+          <t>領民0人スタートの辺境領主様</t>
         </is>
       </c>
       <c r="D68" t="b">
@@ -9044,7 +9105,7 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F68" t="n">
@@ -9052,12 +9113,12 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>Not a Hero</t>
+          <t>星降る夜の約束</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>藍月なくる&amp;棗いつき</t>
+          <t>花耶</t>
         </is>
       </c>
       <c r="I68" t="inlineStr"/>
@@ -9076,7 +9137,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>ワールド イズ ダンシング</t>
+          <t>令和のダラさん</t>
         </is>
       </c>
       <c r="D69" t="b">
@@ -9092,12 +9153,12 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>終宵</t>
+          <t>ダラダラ♡ダンシング</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>マカロニえんぴつ</t>
+          <t>ダラさん（CV：田村睦心） 三⼗⽊⾕⽇向（CV：津田美波） 三⼗⽊⾕薫（CV：寺澤百花） ナレーション（CV：てらそままさき）</t>
         </is>
       </c>
       <c r="I69" t="inlineStr"/>
@@ -9107,16 +9168,16 @@
     </row>
     <row r="70">
       <c r="A70" t="n">
-        <v>5947</v>
+        <v>5806</v>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2026秋アニメ</t>
+          <t>2026夏アニメ</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>転生した大聖女は、聖女であることをひた隠す</t>
+          <t>LV999の村人</t>
         </is>
       </c>
       <c r="D70" t="b">
@@ -9132,12 +9193,12 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>Flare of Soul</t>
+          <t>Not a Hero</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>花耶</t>
+          <t>藍月なくる&amp;棗いつき</t>
         </is>
       </c>
       <c r="I70" t="inlineStr"/>
@@ -9147,16 +9208,16 @@
     </row>
     <row r="71">
       <c r="A71" t="n">
-        <v>5947</v>
+        <v>5806</v>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2026秋アニメ</t>
+          <t>2026夏アニメ</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>転生した大聖女は、聖女であることをひた隠す</t>
+          <t>ワールド イズ ダンシング</t>
         </is>
       </c>
       <c r="D71" t="b">
@@ -9164,7 +9225,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F71" t="n">
@@ -9172,12 +9233,12 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>STELLAR</t>
+          <t>終宵</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>ウタヒメドリーム オールスターズ</t>
+          <t>マカロニえんぴつ</t>
         </is>
       </c>
       <c r="I71" t="inlineStr"/>
@@ -9196,7 +9257,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>魔法少女育成計画restart</t>
+          <t>転生した大聖女は、聖女であることをひた隠す</t>
         </is>
       </c>
       <c r="D72" t="b">
@@ -9212,12 +9273,12 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>No tears here</t>
+          <t>Flare of Soul</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>茅原実里</t>
+          <t>花耶</t>
         </is>
       </c>
       <c r="I72" t="inlineStr"/>
@@ -9225,6 +9286,86 @@
       <c r="K72" t="inlineStr"/>
       <c r="L72" t="inlineStr"/>
     </row>
+    <row r="73">
+      <c r="A73" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>転生した大聖女は、聖女であることをひた隠す</t>
+        </is>
+      </c>
+      <c r="D73" t="b">
+        <v>0</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>ED</t>
+        </is>
+      </c>
+      <c r="F73" t="n">
+        <v>1</v>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>STELLAR</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>ウタヒメドリーム オールスターズ</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr"/>
+      <c r="J73" t="inlineStr"/>
+      <c r="K73" t="inlineStr"/>
+      <c r="L73" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>魔法少女育成計画restart</t>
+        </is>
+      </c>
+      <c r="D74" t="b">
+        <v>0</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="F74" t="n">
+        <v>1</v>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>No tears here</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>茅原実里</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr"/>
+      <c r="J74" t="inlineStr"/>
+      <c r="K74" t="inlineStr"/>
+      <c r="L74" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
auto: anime list update 2026-06-04
</commit_message>
<xml_diff>
--- a/data/anime_list.xlsx
+++ b/data/anime_list.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M123"/>
+  <dimension ref="A1:M126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -862,7 +862,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026年7月～</t>
+          <t>2026年7月8日（水）～ AT-X・TOKYO MXほか</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -989,7 +989,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026年7月～</t>
+          <t>2026年7月6日（月）～ AT-X・TOKYO MXほか</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -2145,8 +2145,16 @@
           <t>花冷え。</t>
         </is>
       </c>
-      <c r="K34" t="inlineStr"/>
-      <c r="L34" t="inlineStr"/>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>NEW GAME</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>halca</t>
+        </is>
+      </c>
       <c r="M34" t="inlineStr">
         <is>
           <t>https://www.animatetimes.com/tag/details.php?id=11593</t>
@@ -2861,7 +2869,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>刃牙道 第2クール</t>
+          <t>刃牙道 第1クール（TV放送）</t>
         </is>
       </c>
       <c r="E49" t="b">
@@ -2874,7 +2882,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>第1クール：2026年2月26日（木）〜 第2クール：2026年6月18日（木）～ Netflixにて 【TV放送】 2026年～</t>
+          <t>第1クール：2026年2月26日（木）〜 第2クール：2026年6月18日（木）～ Netflixにて 【TV放送】 第1クール：2026年7月5日（日）～ TOKYO MXほか</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
@@ -2922,7 +2930,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>花織さんは転生しても喧嘩がしたい</t>
+          <t>刃牙道 第2クール</t>
         </is>
       </c>
       <c r="E50" t="b">
@@ -2930,26 +2938,42 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>TVアニメ</t>
+          <t>配信</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>2026年7月～ ABCテレビ・テレビ朝日系・BS日テレにて</t>
+          <t>第1クール：2026年2月26日（木）〜 第2クール：2026年6月18日（木）～ Netflixにて 【TV放送】 第1クール：2026年7月5日（日）～ TOKYO MXほか</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>ライデンフィルム</t>
-        </is>
-      </c>
-      <c r="I50" t="inlineStr"/>
-      <c r="J50" t="inlineStr"/>
-      <c r="K50" t="inlineStr"/>
-      <c r="L50" t="inlineStr"/>
+          <t>トムス・エンタテインメント</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>フルボコ</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>WANIMA</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>Mountain Top</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>Novel Core</t>
+        </is>
+      </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26828</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=23828</t>
         </is>
       </c>
     </row>
@@ -2967,7 +2991,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>花ざかりの君たちへ 第2期</t>
+          <t>花織さんは転生しても喧嘩がしたい</t>
         </is>
       </c>
       <c r="E51" t="b">
@@ -2980,37 +3004,21 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>2026年7月1日（水）～ TOKYO MX・BS11ほか</t>
+          <t>2026年7月～ ABCテレビ・テレビ朝日系・BS日テレにて</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>シグナル・エムディ（</t>
-        </is>
-      </c>
-      <c r="I51" t="inlineStr">
-        <is>
-          <t>FLASHBULB</t>
-        </is>
-      </c>
-      <c r="J51" t="inlineStr">
-        <is>
-          <t>Omoinotake</t>
-        </is>
-      </c>
-      <c r="K51" t="inlineStr">
-        <is>
-          <t>花束</t>
-        </is>
-      </c>
-      <c r="L51" t="inlineStr">
-        <is>
-          <t>Omoinotake</t>
-        </is>
-      </c>
+          <t>ライデンフィルム</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr"/>
+      <c r="J51" t="inlineStr"/>
+      <c r="K51" t="inlineStr"/>
+      <c r="L51" t="inlineStr"/>
       <c r="M51" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27990</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26828</t>
         </is>
       </c>
     </row>
@@ -3028,7 +3036,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>バンドリ！ ゆめ∞みた</t>
+          <t>花ざかりの君たちへ 第2期</t>
         </is>
       </c>
       <c r="E52" t="b">
@@ -3041,21 +3049,37 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>2026年7月2日（木）～ TOKYO MXほか</t>
+          <t>2026年7月1日（水）～ TOKYO MX・BS11ほか</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>ニチカライン（</t>
-        </is>
-      </c>
-      <c r="I52" t="inlineStr"/>
-      <c r="J52" t="inlineStr"/>
-      <c r="K52" t="inlineStr"/>
-      <c r="L52" t="inlineStr"/>
+          <t>シグナル・エムディ（</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>FLASHBULB</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>Omoinotake</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>花束</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>Omoinotake</t>
+        </is>
+      </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26737</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27990</t>
         </is>
       </c>
     </row>
@@ -3073,7 +3097,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>パンの赤ちゃん</t>
+          <t>バンドリ！ ゆめ∞みた</t>
         </is>
       </c>
       <c r="E53" t="b">
@@ -3086,17 +3110,21 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>2026年7月4日（土）～ カンテレ・フジテレビ系列「土曜はナニする！？」にて</t>
-        </is>
-      </c>
-      <c r="H53" t="inlineStr"/>
+          <t>2026年7月2日（木）～ TOKYO MXほか</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>ニチカライン（</t>
+        </is>
+      </c>
       <c r="I53" t="inlineStr"/>
       <c r="J53" t="inlineStr"/>
       <c r="K53" t="inlineStr"/>
       <c r="L53" t="inlineStr"/>
       <c r="M53" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25145</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26737</t>
         </is>
       </c>
     </row>
@@ -3114,7 +3142,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>ヒロイン？聖女？いいえ、オールワークスメイドです（誇）！</t>
+          <t>パンの赤ちゃん</t>
         </is>
       </c>
       <c r="E54" t="b">
@@ -3127,37 +3155,17 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>2026年7月1日（水）～ TOKYO MX・BSフジほか</t>
-        </is>
-      </c>
-      <c r="H54" t="inlineStr">
-        <is>
-          <t>EMTスクエアード</t>
-        </is>
-      </c>
-      <c r="I54" t="inlineStr">
-        <is>
-          <t>マデュアル↔ハート</t>
-        </is>
-      </c>
-      <c r="J54" t="inlineStr">
-        <is>
-          <t>メロディ・ウェーブ(CV：宮本侑芽) ルシアナ・ルトルバーグ(CV：大久保瑠美)</t>
-        </is>
-      </c>
-      <c r="K54" t="inlineStr">
-        <is>
-          <t>ハンドメイド</t>
-        </is>
-      </c>
-      <c r="L54" t="inlineStr">
-        <is>
-          <t>仲村宗悟</t>
-        </is>
-      </c>
+          <t>2026年7月4日（土）～ カンテレ・フジテレビ系列「土曜はナニする！？」にて</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr"/>
+      <c r="I54" t="inlineStr"/>
+      <c r="J54" t="inlineStr"/>
+      <c r="K54" t="inlineStr"/>
+      <c r="L54" t="inlineStr"/>
       <c r="M54" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25936</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25145</t>
         </is>
       </c>
     </row>
@@ -3175,7 +3183,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>ブチ切れ令嬢は報復を誓いました。 ～魔導書の力で祖国を叩き潰します～</t>
+          <t>ヒロイン？聖女？いいえ、オールワークスメイドです（誇）！</t>
         </is>
       </c>
       <c r="E55" t="b">
@@ -3188,37 +3196,37 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>2026年7月〜 テレ東・BS11ほか</t>
+          <t>2026年7月1日（水）～ TOKYO MX・BSフジほか</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>スタジオコメット</t>
+          <t>EMTスクエアード</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>Q.E.D.</t>
+          <t>マデュアル↔ハート</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>小倉唯</t>
+          <t>メロディ・ウェーブ(CV：宮本侑芽) ルシアナ・ルトルバーグ(CV：大久保瑠美)</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
         <is>
-          <t>グッバイ・ララバイ</t>
+          <t>ハンドメイド</t>
         </is>
       </c>
       <c r="L55" t="inlineStr">
         <is>
-          <t>大西亜玖璃</t>
+          <t>仲村宗悟</t>
         </is>
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27366</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25936</t>
         </is>
       </c>
     </row>
@@ -3236,7 +3244,7 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>ふつつかな悪女ではございますが～雛宮蝶鼠とりかえ伝～</t>
+          <t>ブチ切れ令嬢は報復を誓いました。 ～魔導書の力で祖国を叩き潰します～</t>
         </is>
       </c>
       <c r="E56" t="b">
@@ -3249,21 +3257,37 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>2026年7月12日（日）〜 テレビ東京系列にて</t>
+          <t>2026年7月〜 テレ東・BS11ほか</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>動画工房</t>
-        </is>
-      </c>
-      <c r="I56" t="inlineStr"/>
-      <c r="J56" t="inlineStr"/>
-      <c r="K56" t="inlineStr"/>
-      <c r="L56" t="inlineStr"/>
+          <t>スタジオコメット</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>Q.E.D.</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>小倉唯</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>グッバイ・ララバイ</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>大西亜玖璃</t>
+        </is>
+      </c>
       <c r="M56" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25702</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27366</t>
         </is>
       </c>
     </row>
@@ -3281,7 +3305,7 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>BLACK TORCH</t>
+          <t>ふつつかな悪女ではございますが～雛宮蝶鼠とりかえ伝～</t>
         </is>
       </c>
       <c r="E57" t="b">
@@ -3294,12 +3318,12 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>2026年7月4日（土）～ TOKYO MXほか</t>
+          <t>2026年7月12日（日）〜 テレビ東京系列にて</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>100studio</t>
+          <t>動画工房</t>
         </is>
       </c>
       <c r="I57" t="inlineStr"/>
@@ -3308,7 +3332,7 @@
       <c r="L57" t="inlineStr"/>
       <c r="M57" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25641</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25702</t>
         </is>
       </c>
     </row>
@@ -3326,7 +3350,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>プラノサウルス ガチコセイブツ部</t>
+          <t>BLACK TORCH</t>
         </is>
       </c>
       <c r="E58" t="b">
@@ -3339,12 +3363,12 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>2026年7月～ テレ東系列6局ネット「アニもり！」内にて</t>
+          <t>2026年7月4日（土）～ TOKYO MXほか</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>SMDE</t>
+          <t>100studio</t>
         </is>
       </c>
       <c r="I58" t="inlineStr"/>
@@ -3353,7 +3377,7 @@
       <c r="L58" t="inlineStr"/>
       <c r="M58" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27895</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25641</t>
         </is>
       </c>
     </row>
@@ -3371,7 +3395,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>BLEACH 千年血戦篇-禍進譚-</t>
+          <t>プラノサウルス ガチコセイブツ部</t>
         </is>
       </c>
       <c r="E59" t="b">
@@ -3384,12 +3408,12 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>2026年7月～ テレ東系列ほか</t>
+          <t>2026年7月～ テレ東系列6局ネット「アニもり！」内にて</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>PIERROT FILMS（</t>
+          <t>SMDE</t>
         </is>
       </c>
       <c r="I59" t="inlineStr"/>
@@ -3398,7 +3422,7 @@
       <c r="L59" t="inlineStr"/>
       <c r="M59" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25417</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27895</t>
         </is>
       </c>
     </row>
@@ -3416,7 +3440,7 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>文豪ストレイドッグス わん！２</t>
+          <t>BLEACH 千年血戦篇-禍進譚-</t>
         </is>
       </c>
       <c r="E60" t="b">
@@ -3429,12 +3453,12 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>2026年7月〜</t>
+          <t>2026年7月～ テレ東系列ほか</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>ボンズ</t>
+          <t>PIERROT FILMS（</t>
         </is>
       </c>
       <c r="I60" t="inlineStr"/>
@@ -3443,7 +3467,7 @@
       <c r="L60" t="inlineStr"/>
       <c r="M60" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27057</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25417</t>
         </is>
       </c>
     </row>
@@ -3461,7 +3485,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>ヘルモード ～やり込み好きのゲーマーは廃設定の異世界で無双する～ 2nd Season</t>
+          <t>文豪ストレイドッグス わん！２</t>
         </is>
       </c>
       <c r="E61" t="b">
@@ -3474,17 +3498,21 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>2026年7月～ TOKYO MX・MBS・BS日テレにて</t>
-        </is>
-      </c>
-      <c r="H61" t="inlineStr"/>
+          <t>2026年7月〜</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>ボンズ</t>
+        </is>
+      </c>
       <c r="I61" t="inlineStr"/>
       <c r="J61" t="inlineStr"/>
       <c r="K61" t="inlineStr"/>
       <c r="L61" t="inlineStr"/>
       <c r="M61" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28020</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27057</t>
         </is>
       </c>
     </row>
@@ -3502,7 +3530,7 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>炎の闘球女 ドッジ弾子</t>
+          <t>ヘルモード ～やり込み好きのゲーマーは廃設定の異世界で無双する～ 2nd Season</t>
         </is>
       </c>
       <c r="E62" t="b">
@@ -3515,37 +3543,17 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>2026年7月6日（月）～ TOKYO MX・MBS・BS11にて</t>
-        </is>
-      </c>
-      <c r="H62" t="inlineStr">
-        <is>
-          <t>CUE</t>
-        </is>
-      </c>
-      <c r="I62" t="inlineStr">
-        <is>
-          <t>会心の一劇</t>
-        </is>
-      </c>
-      <c r="J62" t="inlineStr">
-        <is>
-          <t>ももいろクローバーZ</t>
-        </is>
-      </c>
-      <c r="K62" t="inlineStr">
-        <is>
-          <t>Welcome to あざとさワールド</t>
-        </is>
-      </c>
-      <c r="L62" t="inlineStr">
-        <is>
-          <t>i☆Ris</t>
-        </is>
-      </c>
+          <t>2026年7月～ TOKYO MX・MBS・BS日テレにて</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr"/>
+      <c r="I62" t="inlineStr"/>
+      <c r="J62" t="inlineStr"/>
+      <c r="K62" t="inlineStr"/>
+      <c r="L62" t="inlineStr"/>
       <c r="M62" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26401</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28020</t>
         </is>
       </c>
     </row>
@@ -3563,7 +3571,7 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>魔法少女リリカルなのは EXCEEDS Gun Blaze Vengeance</t>
+          <t>炎の闘球女 ドッジ弾子</t>
         </is>
       </c>
       <c r="E63" t="b">
@@ -3576,37 +3584,37 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>2026年7月4日（土）～ TOKYO MX・BS11にて</t>
+          <t>2026年7月6日（月）～ TOKYO MX・MBS・BS11にて</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>Seven Arcs</t>
+          <t>CUE</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>CRIMSON BULLET</t>
+          <t>会心の一劇</t>
         </is>
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>水樹奈々</t>
+          <t>ももいろクローバーZ</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
         <is>
-          <t>Ephemeral</t>
+          <t>Welcome to あざとさワールド</t>
         </is>
       </c>
       <c r="L63" t="inlineStr">
         <is>
-          <t>青木陽菜</t>
+          <t>i☆Ris</t>
         </is>
       </c>
       <c r="M63" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25418</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26401</t>
         </is>
       </c>
     </row>
@@ -3624,7 +3632,7 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>身代わり令嬢を救ったのは冷酷無慈悲な氷の王子の愛でした</t>
+          <t>魔法少女リリカルなのは EXCEEDS Gun Blaze Vengeance</t>
         </is>
       </c>
       <c r="E64" t="b">
@@ -3637,21 +3645,37 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>2026年7月～ TVKにて</t>
+          <t>2026年7月4日（土）～ TOKYO MX・BS11にて</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>Imagica Infos</t>
-        </is>
-      </c>
-      <c r="I64" t="inlineStr"/>
-      <c r="J64" t="inlineStr"/>
-      <c r="K64" t="inlineStr"/>
-      <c r="L64" t="inlineStr"/>
+          <t>Seven Arcs</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>CRIMSON BULLET</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>水樹奈々</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>Ephemeral</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>青木陽菜</t>
+        </is>
+      </c>
       <c r="M64" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28112</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25418</t>
         </is>
       </c>
     </row>
@@ -3669,7 +3693,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>無自覚聖女は今日も無意識に力を垂れ流す</t>
+          <t>身代わり令嬢を救ったのは冷酷無慈悲な氷の王子の愛でした</t>
         </is>
       </c>
       <c r="E65" t="b">
@@ -3682,37 +3706,21 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>2026年7月～ TOKYO MX・BS11・AT-Xにて</t>
+          <t>2026年7月～ TVKにて</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>マジックバス×ピカンテサーカス</t>
-        </is>
-      </c>
-      <c r="I65" t="inlineStr">
-        <is>
-          <t>Windmaker</t>
-        </is>
-      </c>
-      <c r="J65" t="inlineStr">
-        <is>
-          <t>花耶</t>
-        </is>
-      </c>
-      <c r="K65" t="inlineStr">
-        <is>
-          <t>アンノウンミー</t>
-        </is>
-      </c>
-      <c r="L65" t="inlineStr">
-        <is>
-          <t>ウタヒメドリーム オールスターズ【夢咲いぶき（CV:山﨑玲奈） 桜木舞華（CV:鈴木杏奈） 真白清美（CV:其原有沙） HiREN（CV:花耶） 水月ひかり（CV:礒部花凜） 高木凛（CV:鷲見友美ジェナ） 萩原ひまわり（CV:倉知玲鳳） SAKURAKO（CV:竹内夢）】</t>
-        </is>
-      </c>
+          <t>Imagica Infos</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr"/>
+      <c r="J65" t="inlineStr"/>
+      <c r="K65" t="inlineStr"/>
+      <c r="L65" t="inlineStr"/>
       <c r="M65" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26462</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28112</t>
         </is>
       </c>
     </row>
@@ -3730,7 +3738,7 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>無職転生Ⅲ ～異世界行ったら本気だす～</t>
+          <t>無自覚聖女は今日も無意識に力を垂れ流す</t>
         </is>
       </c>
       <c r="E66" t="b">
@@ -3743,25 +3751,37 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>2026年7月5日（日）～ TOKYO MX・BS11ほか</t>
-        </is>
-      </c>
-      <c r="H66" t="inlineStr"/>
+          <t>2026年7月～ TOKYO MX・BS11・AT-Xにて</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>マジックバス×ピカンテサーカス</t>
+        </is>
+      </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>決意の唄</t>
+          <t>Windmaker</t>
         </is>
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>大原ゆい子</t>
-        </is>
-      </c>
-      <c r="K66" t="inlineStr"/>
-      <c r="L66" t="inlineStr"/>
+          <t>花耶</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>アンノウンミー</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>ウタヒメドリーム オールスターズ【夢咲いぶき（CV:山﨑玲奈） 桜木舞華（CV:鈴木杏奈） 真白清美（CV:其原有沙） HiREN（CV:花耶） 水月ひかり（CV:礒部花凜） 高木凛（CV:鷲見友美ジェナ） 萩原ひまわり（CV:倉知玲鳳） SAKURAKO（CV:竹内夢）】</t>
+        </is>
+      </c>
       <c r="M66" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=24285</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26462</t>
         </is>
       </c>
     </row>
@@ -3779,7 +3799,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>メビウス・ダスト</t>
+          <t>無職転生Ⅲ ～異世界行ったら本気だす～</t>
         </is>
       </c>
       <c r="E67" t="b">
@@ -3792,29 +3812,25 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>2026年7月～</t>
-        </is>
-      </c>
-      <c r="H67" t="inlineStr">
-        <is>
-          <t>動画工房</t>
-        </is>
-      </c>
+          <t>2026年7月5日（日）～ TOKYO MX・BS11ほか</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr"/>
       <c r="I67" t="inlineStr">
         <is>
-          <t>メビウス</t>
+          <t>決意の唄</t>
         </is>
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>家入レオ</t>
+          <t>大原ゆい子</t>
         </is>
       </c>
       <c r="K67" t="inlineStr"/>
       <c r="L67" t="inlineStr"/>
       <c r="M67" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28016</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=24285</t>
         </is>
       </c>
     </row>
@@ -3832,7 +3848,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>ヤニねこ</t>
+          <t>メビウス・ダスト</t>
         </is>
       </c>
       <c r="E68" t="b">
@@ -3845,29 +3861,29 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>2026年7月2日（木）～ TOKYO MX・BS11にて</t>
+          <t>2026年7月～</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>バイブリーアニメーションスタジオ</t>
+          <t>動画工房</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>なんもねえ</t>
+          <t>メビウス</t>
         </is>
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>忘れらんねえよ</t>
+          <t>家入レオ</t>
         </is>
       </c>
       <c r="K68" t="inlineStr"/>
       <c r="L68" t="inlineStr"/>
       <c r="M68" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27571</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28016</t>
         </is>
       </c>
     </row>
@@ -3885,7 +3901,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>幼女戦記Ⅱ</t>
+          <t>ヤニねこ</t>
         </is>
       </c>
       <c r="E69" t="b">
@@ -3898,21 +3914,29 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>2026年7月～</t>
+          <t>2026年7月2日（木）～ TOKYO MX・BS11にて</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>NUT</t>
-        </is>
-      </c>
-      <c r="I69" t="inlineStr"/>
-      <c r="J69" t="inlineStr"/>
+          <t>バイブリーアニメーションスタジオ</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>なんもねえ</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>忘れらんねえよ</t>
+        </is>
+      </c>
       <c r="K69" t="inlineStr"/>
       <c r="L69" t="inlineStr"/>
       <c r="M69" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=14369</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27571</t>
         </is>
       </c>
     </row>
@@ -3930,7 +3954,7 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>鎧真伝サムライトルーパー 第2クール</t>
+          <t>幼女戦記Ⅱ</t>
         </is>
       </c>
       <c r="E70" t="b">
@@ -3943,37 +3967,21 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>第1クール：2026年1月6日（火）〜2026年3月24日（火） 第2クール：2026年7月7日（火）～ TOKYO MXほか</t>
+          <t>2026年7月～</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>サンライズ</t>
-        </is>
-      </c>
-      <c r="I70" t="inlineStr">
-        <is>
-          <t>YOAKE</t>
-        </is>
-      </c>
-      <c r="J70" t="inlineStr">
-        <is>
-          <t>blank paper</t>
-        </is>
-      </c>
-      <c r="K70" t="inlineStr">
-        <is>
-          <t>POWER</t>
-        </is>
-      </c>
-      <c r="L70" t="inlineStr">
-        <is>
-          <t>ONE OR EIGHT</t>
-        </is>
-      </c>
+          <t>NUT</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr"/>
+      <c r="J70" t="inlineStr"/>
+      <c r="K70" t="inlineStr"/>
+      <c r="L70" t="inlineStr"/>
       <c r="M70" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26202</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=14369</t>
         </is>
       </c>
     </row>
@@ -3991,7 +3999,7 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>落第賢者の学院無双～二度目の転生、Sランクチート魔術師冒険録～</t>
+          <t>鎧真伝サムライトルーパー 第2クール</t>
         </is>
       </c>
       <c r="E71" t="b">
@@ -4004,29 +4012,37 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>2026年7月～</t>
+          <t>第1クール：2026年1月6日（火）〜2026年3月24日（火） 第2クール：2026年7月7日（火）～ TOKYO MXほか</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>EMTスクエアード</t>
-        </is>
-      </c>
-      <c r="I71" t="inlineStr"/>
-      <c r="J71" t="inlineStr"/>
+          <t>サンライズ</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>YOAKE</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>blank paper</t>
+        </is>
+      </c>
       <c r="K71" t="inlineStr">
         <is>
-          <t>憧憬</t>
+          <t>POWER</t>
         </is>
       </c>
       <c r="L71" t="inlineStr">
         <is>
-          <t>TrySail</t>
+          <t>ONE OR EIGHT</t>
         </is>
       </c>
       <c r="M71" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27769</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26202</t>
         </is>
       </c>
     </row>
@@ -4044,7 +4060,7 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>領民0人スタートの辺境領主様</t>
+          <t>落第賢者の学院無双～二度目の転生、Sランクチート魔術師冒険録～</t>
         </is>
       </c>
       <c r="E72" t="b">
@@ -4057,37 +4073,29 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>2026年7月10日（金）～ TOKYO MXほか</t>
+          <t>2026年7月～</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>animation studio42</t>
-        </is>
-      </c>
-      <c r="I72" t="inlineStr">
-        <is>
-          <t>Wonder</t>
-        </is>
-      </c>
-      <c r="J72" t="inlineStr">
-        <is>
-          <t>CROWN HEAD</t>
-        </is>
-      </c>
+          <t>EMTスクエアード</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr"/>
+      <c r="J72" t="inlineStr"/>
       <c r="K72" t="inlineStr">
         <is>
-          <t>星降る夜の約束</t>
+          <t>憧憬</t>
         </is>
       </c>
       <c r="L72" t="inlineStr">
         <is>
-          <t>花耶</t>
+          <t>TrySail</t>
         </is>
       </c>
       <c r="M72" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26472</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27769</t>
         </is>
       </c>
     </row>
@@ -4105,7 +4113,7 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>令和のダラさん</t>
+          <t>領民0人スタートの辺境領主様</t>
         </is>
       </c>
       <c r="E73" t="b">
@@ -4118,29 +4126,37 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>2026年7月～</t>
+          <t>2026年7月10日（金）～ TOKYO MXほか</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>旭プロダクション</t>
+          <t>animation studio42</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>ダラダラ♡ダンシング</t>
+          <t>Wonder</t>
         </is>
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>ダラさん（CV：田村睦心） 三⼗⽊⾕⽇向（CV：津田美波） 三⼗⽊⾕薫（CV：寺澤百花） ナレーション（CV：てらそままさき）</t>
-        </is>
-      </c>
-      <c r="K73" t="inlineStr"/>
-      <c r="L73" t="inlineStr"/>
+          <t>CROWN HEAD</t>
+        </is>
+      </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>星降る夜の約束</t>
+        </is>
+      </c>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>花耶</t>
+        </is>
+      </c>
       <c r="M73" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27242</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26472</t>
         </is>
       </c>
     </row>
@@ -4158,7 +4174,7 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>レッツゴー怪奇組</t>
+          <t>令和のダラさん</t>
         </is>
       </c>
       <c r="E74" t="b">
@@ -4171,21 +4187,29 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>2026年7月5日（日）〜 TBS系全国28局ネットにて</t>
+          <t>2026年7月～</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>C-Station</t>
-        </is>
-      </c>
-      <c r="I74" t="inlineStr"/>
-      <c r="J74" t="inlineStr"/>
+          <t>旭プロダクション</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>ダラダラ♡ダンシング</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>ダラさん（CV：田村睦心） 三⼗⽊⾕⽇向（CV：津田美波） 三⼗⽊⾕薫（CV：寺澤百花） ナレーション（CV：てらそままさき）</t>
+        </is>
+      </c>
       <c r="K74" t="inlineStr"/>
       <c r="L74" t="inlineStr"/>
       <c r="M74" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28373</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27242</t>
         </is>
       </c>
     </row>
@@ -4203,7 +4227,7 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>LV999の村人</t>
+          <t>レッツゴー怪奇組</t>
         </is>
       </c>
       <c r="E75" t="b">
@@ -4216,29 +4240,21 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>2026年7月～ テレ東・BSフジほか</t>
+          <t>2026年7月5日（日）〜 TBS系全国28局ネットにて</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>ブレインズ・ベース</t>
-        </is>
-      </c>
-      <c r="I75" t="inlineStr">
-        <is>
-          <t>Not a Hero</t>
-        </is>
-      </c>
-      <c r="J75" t="inlineStr">
-        <is>
-          <t>藍月なくる&amp;棗いつき</t>
-        </is>
-      </c>
+          <t>C-Station</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr"/>
+      <c r="J75" t="inlineStr"/>
       <c r="K75" t="inlineStr"/>
       <c r="L75" t="inlineStr"/>
       <c r="M75" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26648</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28373</t>
         </is>
       </c>
     </row>
@@ -4256,7 +4272,7 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>ワールド イズ ダンシング</t>
+          <t>LV999の村人</t>
         </is>
       </c>
       <c r="E76" t="b">
@@ -4269,29 +4285,29 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>2026年7月2日（木）～ TOKYO MX・BS朝日ほか</t>
+          <t>2026年7月～ テレ東・BSフジほか</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>サイピク</t>
+          <t>ブレインズ・ベース</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>終宵</t>
+          <t>Not a Hero</t>
         </is>
       </c>
       <c r="J76" t="inlineStr">
         <is>
-          <t>マカロニえんぴつ</t>
+          <t>藍月なくる&amp;棗いつき</t>
         </is>
       </c>
       <c r="K76" t="inlineStr"/>
       <c r="L76" t="inlineStr"/>
       <c r="M76" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27472</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26648</t>
         </is>
       </c>
     </row>
@@ -4309,7 +4325,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>ONE PIECE HEROINES</t>
+          <t>ワールド イズ ダンシング</t>
         </is>
       </c>
       <c r="E77" t="b">
@@ -4322,35 +4338,47 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>2026年7月5日（日） 全国フジテレビ系にて</t>
-        </is>
-      </c>
-      <c r="H77" t="inlineStr"/>
-      <c r="I77" t="inlineStr"/>
-      <c r="J77" t="inlineStr"/>
+          <t>2026年7月2日（木）～ TOKYO MX・BS朝日ほか</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>サイピク</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>終宵</t>
+        </is>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>マカロニえんぴつ</t>
+        </is>
+      </c>
       <c r="K77" t="inlineStr"/>
       <c r="L77" t="inlineStr"/>
       <c r="M77" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26606</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27472</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="n">
-        <v>5947</v>
+        <v>5806</v>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>2026秋アニメ</t>
+          <t>2026夏アニメ</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>1</v>
+        <v>77</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>アオアシ Season2</t>
+          <t>ONE PIECE HEROINES</t>
         </is>
       </c>
       <c r="E78" t="b">
@@ -4363,21 +4391,17 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>2026年10月4日（日）～ NHK Eテレにて</t>
-        </is>
-      </c>
-      <c r="H78" t="inlineStr">
-        <is>
-          <t>トムス・エンタテインメント</t>
-        </is>
-      </c>
+          <t>2026年7月5日（日） 全国フジテレビ系にて</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr"/>
       <c r="I78" t="inlineStr"/>
       <c r="J78" t="inlineStr"/>
       <c r="K78" t="inlineStr"/>
       <c r="L78" t="inlineStr"/>
       <c r="M78" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25889</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26606</t>
         </is>
       </c>
     </row>
@@ -4391,11 +4415,11 @@
         </is>
       </c>
       <c r="C79" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>アオのハコ 第2期</t>
+          <t>アオアシ Season2</t>
         </is>
       </c>
       <c r="E79" t="b">
@@ -4408,12 +4432,12 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>2026年10月4日（日）～ TBS系にて</t>
+          <t>2026年10月4日（日）～ NHK Eテレにて</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>エレクトリックサーカス</t>
+          <t>トムス・エンタテインメント</t>
         </is>
       </c>
       <c r="I79" t="inlineStr"/>
@@ -4422,7 +4446,7 @@
       <c r="L79" t="inlineStr"/>
       <c r="M79" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25746</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25889</t>
         </is>
       </c>
     </row>
@@ -4436,11 +4460,11 @@
         </is>
       </c>
       <c r="C80" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>カードファイト!! ヴァンガード Divinez 運命星戦編</t>
+          <t>アオのハコ 第2期</t>
         </is>
       </c>
       <c r="E80" t="b">
@@ -4453,12 +4477,12 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>2026年11月7日（土）～2026年11月21日（土） テレビ愛知・テレ東系列6局ネットほか 【劇場先行】 2026年10月2日（金）</t>
+          <t>2026年10月4日（日）～ TBS系にて</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>キネマシトラス</t>
+          <t>エレクトリックサーカス</t>
         </is>
       </c>
       <c r="I80" t="inlineStr"/>
@@ -4467,7 +4491,7 @@
       <c r="L80" t="inlineStr"/>
       <c r="M80" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28214</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25746</t>
         </is>
       </c>
     </row>
@@ -4481,11 +4505,11 @@
         </is>
       </c>
       <c r="C81" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>傷だらけ聖女より報復をこめて Season2</t>
+          <t>カードファイト!! ヴァンガード Divinez 運命星戦編</t>
         </is>
       </c>
       <c r="E81" t="b">
@@ -4498,12 +4522,12 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>2026年10月〜</t>
+          <t>2026年11月7日（土）～2026年11月21日（土） テレビ愛知・テレ東系列6局ネットほか 【劇場先行】 2026年10月2日（金）</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>Imagica Infos</t>
+          <t>キネマシトラス</t>
         </is>
       </c>
       <c r="I81" t="inlineStr"/>
@@ -4512,7 +4536,7 @@
       <c r="L81" t="inlineStr"/>
       <c r="M81" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25118</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28214</t>
         </is>
       </c>
     </row>
@@ -4526,11 +4550,11 @@
         </is>
       </c>
       <c r="C82" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>恐怖コレクター</t>
+          <t>傷だらけ聖女より報復をこめて Season2</t>
         </is>
       </c>
       <c r="E82" t="b">
@@ -4543,17 +4567,21 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>2026年10月～ NHK総合にて</t>
-        </is>
-      </c>
-      <c r="H82" t="inlineStr"/>
+          <t>2026年10月〜</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>Imagica Infos</t>
+        </is>
+      </c>
       <c r="I82" t="inlineStr"/>
       <c r="J82" t="inlineStr"/>
       <c r="K82" t="inlineStr"/>
       <c r="L82" t="inlineStr"/>
       <c r="M82" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27214</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25118</t>
         </is>
       </c>
     </row>
@@ -4567,11 +4595,11 @@
         </is>
       </c>
       <c r="C83" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>凶乱令嬢ニア・リストン 病弱令嬢に転生した神殺しの武人の華麗なる無双録</t>
+          <t>恐怖コレクター</t>
         </is>
       </c>
       <c r="E83" t="b">
@@ -4584,21 +4612,17 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
-        </is>
-      </c>
-      <c r="H83" t="inlineStr">
-        <is>
-          <t>KONAMI animation</t>
-        </is>
-      </c>
+          <t>2026年10月～ NHK総合にて</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr"/>
       <c r="I83" t="inlineStr"/>
       <c r="J83" t="inlineStr"/>
       <c r="K83" t="inlineStr"/>
       <c r="L83" t="inlineStr"/>
       <c r="M83" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27537</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27214</t>
         </is>
       </c>
     </row>
@@ -4612,11 +4636,11 @@
         </is>
       </c>
       <c r="C84" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>薬屋のひとりごと 第3期</t>
+          <t>凶乱令嬢ニア・リストン 病弱令嬢に転生した神殺しの武人の華麗なる無双録</t>
         </is>
       </c>
       <c r="E84" t="b">
@@ -4629,17 +4653,21 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>第1クール：2026年10月～ 第2クール：2027年4月～ 日本テレビ系にて</t>
-        </is>
-      </c>
-      <c r="H84" t="inlineStr"/>
+          <t>2026年10月～</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>KONAMI animation</t>
+        </is>
+      </c>
       <c r="I84" t="inlineStr"/>
       <c r="J84" t="inlineStr"/>
       <c r="K84" t="inlineStr"/>
       <c r="L84" t="inlineStr"/>
       <c r="M84" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26369</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27537</t>
         </is>
       </c>
     </row>
@@ -4653,11 +4681,11 @@
         </is>
       </c>
       <c r="C85" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>ケロロ軍曹☆</t>
+          <t>薬屋のひとりごと 第3期</t>
         </is>
       </c>
       <c r="E85" t="b">
@@ -4670,7 +4698,7 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>2026年秋</t>
+          <t>第1クール：2026年10月～ 第2クール：2027年4月～ 日本テレビ系にて</t>
         </is>
       </c>
       <c r="H85" t="inlineStr"/>
@@ -4680,7 +4708,7 @@
       <c r="L85" t="inlineStr"/>
       <c r="M85" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27337</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26369</t>
         </is>
       </c>
     </row>
@@ -4694,11 +4722,11 @@
         </is>
       </c>
       <c r="C86" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>幻想水滸伝</t>
+          <t>ケロロ軍曹☆</t>
         </is>
       </c>
       <c r="E86" t="b">
@@ -4711,7 +4739,7 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
+          <t>2026年秋</t>
         </is>
       </c>
       <c r="H86" t="inlineStr"/>
@@ -4721,7 +4749,7 @@
       <c r="L86" t="inlineStr"/>
       <c r="M86" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25616</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27337</t>
         </is>
       </c>
     </row>
@@ -4735,11 +4763,11 @@
         </is>
       </c>
       <c r="C87" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>PSYREN -サイレン-</t>
+          <t>幻想水滸伝</t>
         </is>
       </c>
       <c r="E87" t="b">
@@ -4755,18 +4783,14 @@
           <t>2026年10月～</t>
         </is>
       </c>
-      <c r="H87" t="inlineStr">
-        <is>
-          <t>サテライト</t>
-        </is>
-      </c>
+      <c r="H87" t="inlineStr"/>
       <c r="I87" t="inlineStr"/>
       <c r="J87" t="inlineStr"/>
       <c r="K87" t="inlineStr"/>
       <c r="L87" t="inlineStr"/>
       <c r="M87" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27257</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25616</t>
         </is>
       </c>
     </row>
@@ -4780,11 +4804,11 @@
         </is>
       </c>
       <c r="C88" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>ジャンケットバンク</t>
+          <t>PSYREN -サイレン-</t>
         </is>
       </c>
       <c r="E88" t="b">
@@ -4802,7 +4826,7 @@
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>CUE</t>
+          <t>サテライト</t>
         </is>
       </c>
       <c r="I88" t="inlineStr"/>
@@ -4811,7 +4835,7 @@
       <c r="L88" t="inlineStr"/>
       <c r="M88" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27908</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27257</t>
         </is>
       </c>
     </row>
@@ -4825,11 +4849,11 @@
         </is>
       </c>
       <c r="C89" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>朱色の仮面</t>
+          <t>ジャンケットバンク</t>
         </is>
       </c>
       <c r="E89" t="b">
@@ -4842,17 +4866,21 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>2026年10月～ 読売テレビ・日本テレビ系全国ネットにて</t>
-        </is>
-      </c>
-      <c r="H89" t="inlineStr"/>
+          <t>2026年10月～</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>CUE</t>
+        </is>
+      </c>
       <c r="I89" t="inlineStr"/>
       <c r="J89" t="inlineStr"/>
       <c r="K89" t="inlineStr"/>
       <c r="L89" t="inlineStr"/>
       <c r="M89" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26362</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27908</t>
         </is>
       </c>
     </row>
@@ -4866,11 +4894,11 @@
         </is>
       </c>
       <c r="C90" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>しろたん</t>
+          <t>朱色の仮面</t>
         </is>
       </c>
       <c r="E90" t="b">
@@ -4883,21 +4911,17 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>2026年秋</t>
-        </is>
-      </c>
-      <c r="H90" t="inlineStr">
-        <is>
-          <t>レスプリ</t>
-        </is>
-      </c>
+          <t>2026年10月～ 読売テレビ・日本テレビ系全国ネットにて</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr"/>
       <c r="I90" t="inlineStr"/>
       <c r="J90" t="inlineStr"/>
       <c r="K90" t="inlineStr"/>
       <c r="L90" t="inlineStr"/>
       <c r="M90" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27989</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26362</t>
         </is>
       </c>
     </row>
@@ -4911,11 +4935,11 @@
         </is>
       </c>
       <c r="C91" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>新テニスの王子様 U-17 WORLD CUP 決勝メンバー決定戦</t>
+          <t>獣王武神ダンデヴァイン</t>
         </is>
       </c>
       <c r="E91" t="b">
@@ -4928,17 +4952,29 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>2026年秋</t>
-        </is>
-      </c>
-      <c r="H91" t="inlineStr"/>
-      <c r="I91" t="inlineStr"/>
-      <c r="J91" t="inlineStr"/>
+          <t>2026年10月～</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>ライデンフィルム</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>曲名未発表</t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>西川貴教</t>
+        </is>
+      </c>
       <c r="K91" t="inlineStr"/>
       <c r="L91" t="inlineStr"/>
       <c r="M91" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26829</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28479</t>
         </is>
       </c>
     </row>
@@ -4952,11 +4988,11 @@
         </is>
       </c>
       <c r="C92" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>世界最強の魔女、始めました</t>
+          <t>しろたん</t>
         </is>
       </c>
       <c r="E92" t="b">
@@ -4969,12 +5005,12 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
+          <t>2026年秋</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>ブリッジ</t>
+          <t>レスプリ</t>
         </is>
       </c>
       <c r="I92" t="inlineStr"/>
@@ -4983,7 +5019,7 @@
       <c r="L92" t="inlineStr"/>
       <c r="M92" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28288</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27989</t>
         </is>
       </c>
     </row>
@@ -4997,11 +5033,11 @@
         </is>
       </c>
       <c r="C93" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>#ゾンビさがしてます</t>
+          <t>新テニスの王子様 U-17 WORLD CUP 決勝メンバー決定戦</t>
         </is>
       </c>
       <c r="E93" t="b">
@@ -5014,7 +5050,7 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>2026年10月〜 テレビ朝日系にて</t>
+          <t>2026年秋</t>
         </is>
       </c>
       <c r="H93" t="inlineStr"/>
@@ -5024,7 +5060,7 @@
       <c r="L93" t="inlineStr"/>
       <c r="M93" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26825</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26829</t>
         </is>
       </c>
     </row>
@@ -5038,11 +5074,11 @@
         </is>
       </c>
       <c r="C94" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>タヌキとキツネ</t>
+          <t>世界最強の魔女、始めました</t>
         </is>
       </c>
       <c r="E94" t="b">
@@ -5058,14 +5094,18 @@
           <t>2026年10月～</t>
         </is>
       </c>
-      <c r="H94" t="inlineStr"/>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>ブリッジ</t>
+        </is>
+      </c>
       <c r="I94" t="inlineStr"/>
       <c r="J94" t="inlineStr"/>
       <c r="K94" t="inlineStr"/>
       <c r="L94" t="inlineStr"/>
       <c r="M94" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=6380</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28288</t>
         </is>
       </c>
     </row>
@@ -5079,11 +5119,11 @@
         </is>
       </c>
       <c r="C95" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>TANK CHAIR-戦車椅子-</t>
+          <t>#ゾンビさがしてます</t>
         </is>
       </c>
       <c r="E95" t="b">
@@ -5096,21 +5136,17 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>2026年秋</t>
-        </is>
-      </c>
-      <c r="H95" t="inlineStr">
-        <is>
-          <t>ポリゴン・ピクチュアズ</t>
-        </is>
-      </c>
+          <t>2026年10月〜 テレビ朝日系にて</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr"/>
       <c r="I95" t="inlineStr"/>
       <c r="J95" t="inlineStr"/>
       <c r="K95" t="inlineStr"/>
       <c r="L95" t="inlineStr"/>
       <c r="M95" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27965</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26825</t>
         </is>
       </c>
     </row>
@@ -5124,11 +5160,11 @@
         </is>
       </c>
       <c r="C96" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>探偵はもう、死んでいる。Season2</t>
+          <t>タヌキとキツネ</t>
         </is>
       </c>
       <c r="E96" t="b">
@@ -5141,21 +5177,17 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>2026年10月〜</t>
-        </is>
-      </c>
-      <c r="H96" t="inlineStr">
-        <is>
-          <t>ENGI</t>
-        </is>
-      </c>
+          <t>2026年10月～</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr"/>
       <c r="I96" t="inlineStr"/>
       <c r="J96" t="inlineStr"/>
       <c r="K96" t="inlineStr"/>
       <c r="L96" t="inlineStr"/>
       <c r="M96" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=16348</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=6380</t>
         </is>
       </c>
     </row>
@@ -5169,11 +5201,11 @@
         </is>
       </c>
       <c r="C97" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>超巡！超条先輩</t>
+          <t>TANK CHAIR-戦車椅子-</t>
         </is>
       </c>
       <c r="E97" t="b">
@@ -5186,12 +5218,12 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
+          <t>2026年秋</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>アルボアニメーション</t>
+          <t>ポリゴン・ピクチュアズ</t>
         </is>
       </c>
       <c r="I97" t="inlineStr"/>
@@ -5200,7 +5232,7 @@
       <c r="L97" t="inlineStr"/>
       <c r="M97" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26933</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27965</t>
         </is>
       </c>
     </row>
@@ -5214,11 +5246,11 @@
         </is>
       </c>
       <c r="C98" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>てつりょー！meet with 鉄道むすめ</t>
+          <t>探偵はもう、死んでいる。Season2</t>
         </is>
       </c>
       <c r="E98" t="b">
@@ -5231,12 +5263,12 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>2026年秋</t>
+          <t>2026年10月〜</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>イーストフィッシュスタジオ</t>
+          <t>ENGI</t>
         </is>
       </c>
       <c r="I98" t="inlineStr"/>
@@ -5245,7 +5277,7 @@
       <c r="L98" t="inlineStr"/>
       <c r="M98" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26895</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=16348</t>
         </is>
       </c>
     </row>
@@ -5259,11 +5291,11 @@
         </is>
       </c>
       <c r="C99" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>転生貴族、鑑定スキルで成り上がる 第3期</t>
+          <t>超巡！超条先輩</t>
         </is>
       </c>
       <c r="E99" t="b">
@@ -5276,12 +5308,12 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>2026年秋 CBC/TBS系全国28局ネット「アガルアニメ」にて</t>
+          <t>2026年10月～</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>studio MOTHER</t>
+          <t>アルボアニメーション</t>
         </is>
       </c>
       <c r="I99" t="inlineStr"/>
@@ -5290,7 +5322,7 @@
       <c r="L99" t="inlineStr"/>
       <c r="M99" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25385</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26933</t>
         </is>
       </c>
     </row>
@@ -5304,11 +5336,11 @@
         </is>
       </c>
       <c r="C100" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>転生ゴブリンだけど質問ある？</t>
+          <t>てつりょー！meet with 鉄道むすめ</t>
         </is>
       </c>
       <c r="E100" t="b">
@@ -5321,12 +5353,12 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
+          <t>2026年秋</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>BAKKKA</t>
+          <t>イーストフィッシュスタジオ</t>
         </is>
       </c>
       <c r="I100" t="inlineStr"/>
@@ -5335,7 +5367,7 @@
       <c r="L100" t="inlineStr"/>
       <c r="M100" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27909</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26895</t>
         </is>
       </c>
     </row>
@@ -5349,11 +5381,11 @@
         </is>
       </c>
       <c r="C101" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>転生した大聖女は、聖女であることをひた隠す</t>
+          <t>テムパル～アイテムの力～</t>
         </is>
       </c>
       <c r="E101" t="b">
@@ -5371,32 +5403,16 @@
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>FelixFilm</t>
-        </is>
-      </c>
-      <c r="I101" t="inlineStr">
-        <is>
-          <t>Flare of Soul</t>
-        </is>
-      </c>
-      <c r="J101" t="inlineStr">
-        <is>
-          <t>花耶</t>
-        </is>
-      </c>
-      <c r="K101" t="inlineStr">
-        <is>
-          <t>STELLAR</t>
-        </is>
-      </c>
-      <c r="L101" t="inlineStr">
-        <is>
-          <t>ウタヒメドリーム オールスターズ</t>
-        </is>
-      </c>
+          <t>J.C.STAFF</t>
+        </is>
+      </c>
+      <c r="I101" t="inlineStr"/>
+      <c r="J101" t="inlineStr"/>
+      <c r="K101" t="inlineStr"/>
+      <c r="L101" t="inlineStr"/>
       <c r="M101" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25630</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28478</t>
         </is>
       </c>
     </row>
@@ -5410,11 +5426,11 @@
         </is>
       </c>
       <c r="C102" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>転生したら剣でした 第2期</t>
+          <t>転生貴族、鑑定スキルで成り上がる 第3期</t>
         </is>
       </c>
       <c r="E102" t="b">
@@ -5427,12 +5443,12 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
+          <t>2026年秋 CBC/TBS系全国28局ネット「アガルアニメ」にて</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>C2C</t>
+          <t>studio MOTHER</t>
         </is>
       </c>
       <c r="I102" t="inlineStr"/>
@@ -5441,7 +5457,7 @@
       <c r="L102" t="inlineStr"/>
       <c r="M102" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=19149</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25385</t>
         </is>
       </c>
     </row>
@@ -5455,11 +5471,11 @@
         </is>
       </c>
       <c r="C103" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>とある暗部の少女共棲</t>
+          <t>転生ゴブリンだけど質問ある？</t>
         </is>
       </c>
       <c r="E103" t="b">
@@ -5472,12 +5488,12 @@
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>2026年秋</t>
+          <t>2026年10月～</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>J.C.STAFF</t>
+          <t>BAKKKA</t>
         </is>
       </c>
       <c r="I103" t="inlineStr"/>
@@ -5486,7 +5502,7 @@
       <c r="L103" t="inlineStr"/>
       <c r="M103" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25552</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27909</t>
         </is>
       </c>
     </row>
@@ -5500,11 +5516,11 @@
         </is>
       </c>
       <c r="C104" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>東京リベンジャーズ 三天戦争編</t>
+          <t>転生した大聖女は、聖女であることをひた隠す</t>
         </is>
       </c>
       <c r="E104" t="b">
@@ -5522,16 +5538,32 @@
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>ライデンフィルム</t>
-        </is>
-      </c>
-      <c r="I104" t="inlineStr"/>
-      <c r="J104" t="inlineStr"/>
-      <c r="K104" t="inlineStr"/>
-      <c r="L104" t="inlineStr"/>
+          <t>FelixFilm</t>
+        </is>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>Flare of Soul</t>
+        </is>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>花耶</t>
+        </is>
+      </c>
+      <c r="K104" t="inlineStr">
+        <is>
+          <t>STELLAR</t>
+        </is>
+      </c>
+      <c r="L104" t="inlineStr">
+        <is>
+          <t>ウタヒメドリーム オールスターズ</t>
+        </is>
+      </c>
       <c r="M104" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=24207</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25630</t>
         </is>
       </c>
     </row>
@@ -5545,11 +5577,11 @@
         </is>
       </c>
       <c r="C105" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>桃源暗鬼 ～日光・華厳の滝編～</t>
+          <t>転生したら剣でした 第2期</t>
         </is>
       </c>
       <c r="E105" t="b">
@@ -5562,17 +5594,21 @@
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>2026年10月～ 日本テレビ系「FRIDAY ANIME NIGHT（フラアニ）」枠にて</t>
-        </is>
-      </c>
-      <c r="H105" t="inlineStr"/>
+          <t>2026年10月～</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>C2C</t>
+        </is>
+      </c>
       <c r="I105" t="inlineStr"/>
       <c r="J105" t="inlineStr"/>
       <c r="K105" t="inlineStr"/>
       <c r="L105" t="inlineStr"/>
       <c r="M105" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27376</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=19149</t>
         </is>
       </c>
     </row>
@@ -5586,11 +5622,11 @@
         </is>
       </c>
       <c r="C106" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>ドラゴンボール超 ビルス</t>
+          <t>とある暗部の少女共棲</t>
         </is>
       </c>
       <c r="E106" t="b">
@@ -5603,17 +5639,21 @@
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>2026年秋 フジテレビにて</t>
-        </is>
-      </c>
-      <c r="H106" t="inlineStr"/>
+          <t>2026年秋</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>J.C.STAFF</t>
+        </is>
+      </c>
       <c r="I106" t="inlineStr"/>
       <c r="J106" t="inlineStr"/>
       <c r="K106" t="inlineStr"/>
       <c r="L106" t="inlineStr"/>
       <c r="M106" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27491</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25552</t>
         </is>
       </c>
     </row>
@@ -5627,11 +5667,11 @@
         </is>
       </c>
       <c r="C107" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>鳴海の平日</t>
+          <t>東京リベンジャーズ 三天戦争編</t>
         </is>
       </c>
       <c r="E107" t="b">
@@ -5639,17 +5679,17 @@
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>配信</t>
+          <t>TVアニメ</t>
         </is>
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>2026年秋</t>
+          <t>2026年10月～</t>
         </is>
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>Production I.G</t>
+          <t>ライデンフィルム</t>
         </is>
       </c>
       <c r="I107" t="inlineStr"/>
@@ -5658,7 +5698,7 @@
       <c r="L107" t="inlineStr"/>
       <c r="M107" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28465</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=24207</t>
         </is>
       </c>
     </row>
@@ -5672,11 +5712,11 @@
         </is>
       </c>
       <c r="C108" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>バーテックスフォース</t>
+          <t>桃源暗鬼 ～日光・華厳の滝編～</t>
         </is>
       </c>
       <c r="E108" t="b">
@@ -5689,21 +5729,17 @@
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>2026年10月〜</t>
-        </is>
-      </c>
-      <c r="H108" t="inlineStr">
-        <is>
-          <t>SMDE</t>
-        </is>
-      </c>
+          <t>2026年10月～ 日本テレビ系「FRIDAY ANIME NIGHT（フラアニ）」枠にて</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr"/>
       <c r="I108" t="inlineStr"/>
       <c r="J108" t="inlineStr"/>
       <c r="K108" t="inlineStr"/>
       <c r="L108" t="inlineStr"/>
       <c r="M108" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27988</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27376</t>
         </is>
       </c>
     </row>
@@ -5717,11 +5753,11 @@
         </is>
       </c>
       <c r="C109" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Battle Spirits [Re] 絶界の空</t>
+          <t>ドラゴンボール超 ビルス</t>
         </is>
       </c>
       <c r="E109" t="b">
@@ -5734,7 +5770,7 @@
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>2026年秋</t>
+          <t>2026年秋 フジテレビにて</t>
         </is>
       </c>
       <c r="H109" t="inlineStr"/>
@@ -5744,7 +5780,7 @@
       <c r="L109" t="inlineStr"/>
       <c r="M109" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27954</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27491</t>
         </is>
       </c>
     </row>
@@ -5758,11 +5794,11 @@
         </is>
       </c>
       <c r="C110" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>パンどろぼう</t>
+          <t>鳴海の平日</t>
         </is>
       </c>
       <c r="E110" t="b">
@@ -5770,22 +5806,26 @@
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>TVアニメ</t>
+          <t>配信</t>
         </is>
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>2026年10月〜 NHK Eテレにて</t>
-        </is>
-      </c>
-      <c r="H110" t="inlineStr"/>
+          <t>2026年秋</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>Production I.G</t>
+        </is>
+      </c>
       <c r="I110" t="inlineStr"/>
       <c r="J110" t="inlineStr"/>
       <c r="K110" t="inlineStr"/>
       <c r="L110" t="inlineStr"/>
       <c r="M110" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26163</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28465</t>
         </is>
       </c>
     </row>
@@ -5799,11 +5839,11 @@
         </is>
       </c>
       <c r="C111" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>百妖譜 京師篇</t>
+          <t>バーテックスフォース</t>
         </is>
       </c>
       <c r="E111" t="b">
@@ -5816,17 +5856,21 @@
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>2026年10月〜 フジテレビ「B8station」にて</t>
-        </is>
-      </c>
-      <c r="H111" t="inlineStr"/>
+          <t>2026年10月〜</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>SMDE</t>
+        </is>
+      </c>
       <c r="I111" t="inlineStr"/>
       <c r="J111" t="inlineStr"/>
       <c r="K111" t="inlineStr"/>
       <c r="L111" t="inlineStr"/>
       <c r="M111" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27781</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27988</t>
         </is>
       </c>
     </row>
@@ -5840,11 +5884,11 @@
         </is>
       </c>
       <c r="C112" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>冰剣の魔術師が世界を統べるⅡ</t>
+          <t>Battle Spirits [Re] 絶界の空</t>
         </is>
       </c>
       <c r="E112" t="b">
@@ -5857,21 +5901,17 @@
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>2026年10月〜</t>
-        </is>
-      </c>
-      <c r="H112" t="inlineStr">
-        <is>
-          <t>ゼロジー</t>
-        </is>
-      </c>
+          <t>2026年秋</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr"/>
       <c r="I112" t="inlineStr"/>
       <c r="J112" t="inlineStr"/>
       <c r="K112" t="inlineStr"/>
       <c r="L112" t="inlineStr"/>
       <c r="M112" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28403</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27954</t>
         </is>
       </c>
     </row>
@@ -5885,11 +5925,11 @@
         </is>
       </c>
       <c r="C113" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>ホタルの嫁入り</t>
+          <t>パンどろぼう</t>
         </is>
       </c>
       <c r="E113" t="b">
@@ -5902,21 +5942,17 @@
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>2026年10月～ 全国フジテレビ系“ ノイタミナ ”にて</t>
-        </is>
-      </c>
-      <c r="H113" t="inlineStr">
-        <is>
-          <t>david production</t>
-        </is>
-      </c>
+          <t>2026年10月〜 NHK Eテレにて</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr"/>
       <c r="I113" t="inlineStr"/>
       <c r="J113" t="inlineStr"/>
       <c r="K113" t="inlineStr"/>
       <c r="L113" t="inlineStr"/>
       <c r="M113" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27415</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26163</t>
         </is>
       </c>
     </row>
@@ -5930,11 +5966,11 @@
         </is>
       </c>
       <c r="C114" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>ポップパップポルターズ</t>
+          <t>百妖譜 京師篇</t>
         </is>
       </c>
       <c r="E114" t="b">
@@ -5947,21 +5983,17 @@
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>2026年秋 テレビ朝日にて</t>
-        </is>
-      </c>
-      <c r="H114" t="inlineStr">
-        <is>
-          <t>MOZU STUDIOS</t>
-        </is>
-      </c>
+          <t>2026年10月〜 フジテレビ「B8station」にて</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr"/>
       <c r="I114" t="inlineStr"/>
       <c r="J114" t="inlineStr"/>
       <c r="K114" t="inlineStr"/>
       <c r="L114" t="inlineStr"/>
       <c r="M114" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27823</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27781</t>
         </is>
       </c>
     </row>
@@ -5975,11 +6007,11 @@
         </is>
       </c>
       <c r="C115" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>ホテル・インヒューマンズ 第2期</t>
+          <t>冰剣の魔術師が世界を統べるⅡ</t>
         </is>
       </c>
       <c r="E115" t="b">
@@ -5992,12 +6024,12 @@
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>2026年10月～ テレ東系列ほか</t>
+          <t>2026年10月〜</t>
         </is>
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>ブリッジ</t>
+          <t>ゼロジー</t>
         </is>
       </c>
       <c r="I115" t="inlineStr"/>
@@ -6006,7 +6038,7 @@
       <c r="L115" t="inlineStr"/>
       <c r="M115" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26870</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28403</t>
         </is>
       </c>
     </row>
@@ -6020,11 +6052,11 @@
         </is>
       </c>
       <c r="C116" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>マジカル★エクスプローラー</t>
+          <t>ホタルの嫁入り</t>
         </is>
       </c>
       <c r="E116" t="b">
@@ -6037,12 +6069,12 @@
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>2026年秋</t>
+          <t>2026年10月～ 全国フジテレビ系“ ノイタミナ ”にて</t>
         </is>
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>WHITE FOX</t>
+          <t>david production</t>
         </is>
       </c>
       <c r="I116" t="inlineStr"/>
@@ -6051,7 +6083,7 @@
       <c r="L116" t="inlineStr"/>
       <c r="M116" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=23375</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27415</t>
         </is>
       </c>
     </row>
@@ -6065,11 +6097,11 @@
         </is>
       </c>
       <c r="C117" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>魔法騎士レイアース</t>
+          <t>ポップパップポルターズ</t>
         </is>
       </c>
       <c r="E117" t="b">
@@ -6082,12 +6114,12 @@
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>2026年10月～ テレビ朝日系列にて</t>
+          <t>2026年秋 テレビ朝日にて</t>
         </is>
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>E&amp;H production</t>
+          <t>MOZU STUDIOS</t>
         </is>
       </c>
       <c r="I117" t="inlineStr"/>
@@ -6096,7 +6128,7 @@
       <c r="L117" t="inlineStr"/>
       <c r="M117" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=24301</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27823</t>
         </is>
       </c>
     </row>
@@ -6110,11 +6142,11 @@
         </is>
       </c>
       <c r="C118" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>魔法少女育成計画restart</t>
+          <t>ホテル・インヒューマンズ 第2期</t>
         </is>
       </c>
       <c r="E118" t="b">
@@ -6127,29 +6159,21 @@
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>2026年秋</t>
+          <t>2026年10月～ テレ東系列ほか</t>
         </is>
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>SynergySP</t>
-        </is>
-      </c>
-      <c r="I118" t="inlineStr">
-        <is>
-          <t>No tears here</t>
-        </is>
-      </c>
-      <c r="J118" t="inlineStr">
-        <is>
-          <t>茅原実里</t>
-        </is>
-      </c>
+          <t>ブリッジ</t>
+        </is>
+      </c>
+      <c r="I118" t="inlineStr"/>
+      <c r="J118" t="inlineStr"/>
       <c r="K118" t="inlineStr"/>
       <c r="L118" t="inlineStr"/>
       <c r="M118" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26693</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26870</t>
         </is>
       </c>
     </row>
@@ -6163,11 +6187,11 @@
         </is>
       </c>
       <c r="C119" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>マロニエ王国の七人の騎士</t>
+          <t>マジカル★エクスプローラー</t>
         </is>
       </c>
       <c r="E119" t="b">
@@ -6180,12 +6204,12 @@
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>2026年10月～ NHK Eテレにて</t>
+          <t>2026年秋</t>
         </is>
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>J.C.STAFF</t>
+          <t>WHITE FOX</t>
         </is>
       </c>
       <c r="I119" t="inlineStr"/>
@@ -6194,7 +6218,7 @@
       <c r="L119" t="inlineStr"/>
       <c r="M119" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28456</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=23375</t>
         </is>
       </c>
     </row>
@@ -6208,11 +6232,11 @@
         </is>
       </c>
       <c r="C120" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>目覚めたら最強装備と宇宙船持ちだったので、一戸建て目指して傭兵として自由に生きたい</t>
+          <t>魔法騎士レイアース</t>
         </is>
       </c>
       <c r="E120" t="b">
@@ -6225,12 +6249,12 @@
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>2026年10月〜</t>
+          <t>2026年10月～ テレビ朝日系列にて</t>
         </is>
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>studio A-CAT</t>
+          <t>E&amp;H production</t>
         </is>
       </c>
       <c r="I120" t="inlineStr"/>
@@ -6239,7 +6263,7 @@
       <c r="L120" t="inlineStr"/>
       <c r="M120" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25525</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=24301</t>
         </is>
       </c>
     </row>
@@ -6253,11 +6277,11 @@
         </is>
       </c>
       <c r="C121" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>弱気MAX令嬢なのに、辣腕婚約者様の賭けに乗ってしまった</t>
+          <t>魔法少女育成計画restart</t>
         </is>
       </c>
       <c r="E121" t="b">
@@ -6270,21 +6294,29 @@
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
+          <t>2026年秋</t>
         </is>
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>寿門堂</t>
-        </is>
-      </c>
-      <c r="I121" t="inlineStr"/>
-      <c r="J121" t="inlineStr"/>
+          <t>SynergySP</t>
+        </is>
+      </c>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>No tears here</t>
+        </is>
+      </c>
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>茅原実里</t>
+        </is>
+      </c>
       <c r="K121" t="inlineStr"/>
       <c r="L121" t="inlineStr"/>
       <c r="M121" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26947</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26693</t>
         </is>
       </c>
     </row>
@@ -6298,11 +6330,11 @@
         </is>
       </c>
       <c r="C122" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>らんま1/2 第3期</t>
+          <t>マロニエ王国の七人の騎士</t>
         </is>
       </c>
       <c r="E122" t="b">
@@ -6315,17 +6347,21 @@
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>2026年10月～ 日本テレビ系にて</t>
-        </is>
-      </c>
-      <c r="H122" t="inlineStr"/>
+          <t>2026年10月～ NHK Eテレにて</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>J.C.STAFF</t>
+        </is>
+      </c>
       <c r="I122" t="inlineStr"/>
       <c r="J122" t="inlineStr"/>
       <c r="K122" t="inlineStr"/>
       <c r="L122" t="inlineStr"/>
       <c r="M122" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28013</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28456</t>
         </is>
       </c>
     </row>
@@ -6339,11 +6375,11 @@
         </is>
       </c>
       <c r="C123" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>LEGO® ONE PIECE</t>
+          <t>目覚めたら最強装備と宇宙船持ちだったので、一戸建て目指して傭兵として自由に生きたい</t>
         </is>
       </c>
       <c r="E123" t="b">
@@ -6351,20 +6387,151 @@
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>配信</t>
+          <t>TVアニメ</t>
         </is>
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t>2026年9月29日（火） Netflixにて</t>
-        </is>
-      </c>
-      <c r="H123" t="inlineStr"/>
+          <t>2026年10月〜</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>studio A-CAT</t>
+        </is>
+      </c>
       <c r="I123" t="inlineStr"/>
       <c r="J123" t="inlineStr"/>
       <c r="K123" t="inlineStr"/>
       <c r="L123" t="inlineStr"/>
       <c r="M123" t="inlineStr">
+        <is>
+          <t>https://www.animatetimes.com/tag/details.php?id=25525</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C124" t="n">
+        <v>46</v>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>弱気MAX令嬢なのに、辣腕婚約者様の賭けに乗ってしまった</t>
+        </is>
+      </c>
+      <c r="E124" t="b">
+        <v>0</v>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>TVアニメ</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>2026年10月～</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>寿門堂</t>
+        </is>
+      </c>
+      <c r="I124" t="inlineStr"/>
+      <c r="J124" t="inlineStr"/>
+      <c r="K124" t="inlineStr"/>
+      <c r="L124" t="inlineStr"/>
+      <c r="M124" t="inlineStr">
+        <is>
+          <t>https://www.animatetimes.com/tag/details.php?id=26947</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C125" t="n">
+        <v>47</v>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>らんま1/2 第3期</t>
+        </is>
+      </c>
+      <c r="E125" t="b">
+        <v>0</v>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>TVアニメ</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>2026年10月～ 日本テレビ系にて</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr"/>
+      <c r="I125" t="inlineStr"/>
+      <c r="J125" t="inlineStr"/>
+      <c r="K125" t="inlineStr"/>
+      <c r="L125" t="inlineStr"/>
+      <c r="M125" t="inlineStr">
+        <is>
+          <t>https://www.animatetimes.com/tag/details.php?id=28013</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C126" t="n">
+        <v>48</v>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>LEGO® ONE PIECE</t>
+        </is>
+      </c>
+      <c r="E126" t="b">
+        <v>0</v>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>配信</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>2026年9月29日（火） Netflixにて</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr"/>
+      <c r="I126" t="inlineStr"/>
+      <c r="J126" t="inlineStr"/>
+      <c r="K126" t="inlineStr"/>
+      <c r="L126" t="inlineStr"/>
+      <c r="M126" t="inlineStr">
         <is>
           <t>https://www.animatetimes.com/tag/details.php?id=28168</t>
         </is>
@@ -6381,7 +6548,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L74"/>
+  <dimension ref="A1:L82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7737,7 +7904,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>追放された転生重騎士はゲーム知識で無双する</t>
+          <t>対ありでした。～お嬢さまは格闘ゲームなんてしない～</t>
         </is>
       </c>
       <c r="D34" t="b">
@@ -7745,7 +7912,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F34" t="n">
@@ -7753,12 +7920,12 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Awake</t>
+          <t>NEW GAME</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>SPYAIR</t>
+          <t>halca</t>
         </is>
       </c>
       <c r="I34" t="inlineStr"/>
@@ -7777,7 +7944,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>鉄鍋のジャン！</t>
+          <t>追放された転生重騎士はゲーム知識で無双する</t>
         </is>
       </c>
       <c r="D35" t="b">
@@ -7793,12 +7960,12 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>火宴</t>
+          <t>Awake</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>原因は自分にある。</t>
+          <t>SPYAIR</t>
         </is>
       </c>
       <c r="I35" t="inlineStr"/>
@@ -7817,7 +7984,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>手札が多めのビクトリア</t>
+          <t>鉄鍋のジャン！</t>
         </is>
       </c>
       <c r="D36" t="b">
@@ -7825,7 +7992,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F36" t="n">
@@ -7833,12 +8000,12 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>縁のつき</t>
+          <t>火宴</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>KI_EN</t>
+          <t>原因は自分にある。</t>
         </is>
       </c>
       <c r="I36" t="inlineStr"/>
@@ -7857,7 +8024,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>転校先の清楚可憐な美少女が、昔男子と思って一緒に遊んだ幼馴染だった件</t>
+          <t>手札が多めのビクトリア</t>
         </is>
       </c>
       <c r="D37" t="b">
@@ -7865,7 +8032,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F37" t="n">
@@ -7873,18 +8040,32 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>夏に重ねて</t>
+          <t>縁のつき</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>DIALOGUE+</t>
-        </is>
-      </c>
-      <c r="I37" t="inlineStr"/>
-      <c r="J37" t="inlineStr"/>
-      <c r="K37" t="inlineStr"/>
-      <c r="L37" t="inlineStr"/>
+          <t>KI_EN</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=-HNOXWE2wVU</t>
+        </is>
+      </c>
+      <c r="J37" t="n">
+        <v>107892</v>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>2026-06-04T19:29:01</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -7897,7 +8078,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>天は赤い河のほとり</t>
+          <t>転校先の清楚可憐な美少女が、昔男子と思って一緒に遊んだ幼馴染だった件</t>
         </is>
       </c>
       <c r="D38" t="b">
@@ -7913,12 +8094,12 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>暁の空</t>
+          <t>夏に重ねて</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>七海ひろき</t>
+          <t>DIALOGUE+</t>
         </is>
       </c>
       <c r="I38" t="inlineStr"/>
@@ -7937,7 +8118,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>天幕のジャードゥーガル</t>
+          <t>天は赤い河のほとり</t>
         </is>
       </c>
       <c r="D39" t="b">
@@ -7953,12 +8134,12 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Stella</t>
+          <t>暁の空</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>SEKAI NO OWARI</t>
+          <t>七海ひろき</t>
         </is>
       </c>
       <c r="I39" t="inlineStr"/>
@@ -7977,7 +8158,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>盗掘王</t>
+          <t>天幕のジャードゥーガル</t>
         </is>
       </c>
       <c r="D40" t="b">
@@ -7993,12 +8174,12 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>SHOW DOWN</t>
+          <t>Stella</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>QWER</t>
+          <t>SEKAI NO OWARI</t>
         </is>
       </c>
       <c r="I40" t="inlineStr"/>
@@ -8017,7 +8198,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>透明な夜に駆ける君と、目に見えない恋をした。</t>
+          <t>盗掘王</t>
         </is>
       </c>
       <c r="D41" t="b">
@@ -8025,7 +8206,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F41" t="n">
@@ -8033,12 +8214,12 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>光</t>
+          <t>SHOW DOWN</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>櫻井優衣</t>
+          <t>QWER</t>
         </is>
       </c>
       <c r="I41" t="inlineStr"/>
@@ -8057,7 +8238,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>二十世紀電氣目録-ユーレカ・エヴリカ-</t>
+          <t>透明な夜に駆ける君と、目に見えない恋をした。</t>
         </is>
       </c>
       <c r="D42" t="b">
@@ -8065,7 +8246,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F42" t="n">
@@ -8073,12 +8254,12 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>ユーレカ・エヴリカ</t>
+          <t>光</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>五阿弥ルナ</t>
+          <t>櫻井優衣</t>
         </is>
       </c>
       <c r="I42" t="inlineStr"/>
@@ -8097,7 +8278,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>パイの実 おしの森へようこそ！</t>
+          <t>二十世紀電氣目録-ユーレカ・エヴリカ-</t>
         </is>
       </c>
       <c r="D43" t="b">
@@ -8105,7 +8286,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>主題歌</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F43" t="n">
@@ -8113,12 +8294,12 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>パイしか勝たん！推しの森活</t>
+          <t>ユーレカ・エヴリカ</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>安保心結</t>
+          <t>五阿弥ルナ</t>
         </is>
       </c>
       <c r="I43" t="inlineStr"/>
@@ -8137,7 +8318,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>刃牙道 第2クール</t>
+          <t>パイの実 おしの森へようこそ！</t>
         </is>
       </c>
       <c r="D44" t="b">
@@ -8145,7 +8326,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>主題歌</t>
         </is>
       </c>
       <c r="F44" t="n">
@@ -8153,12 +8334,12 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>フルボコ</t>
+          <t>パイしか勝たん！推しの森活</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>WANIMA</t>
+          <t>安保心結</t>
         </is>
       </c>
       <c r="I44" t="inlineStr"/>
@@ -8177,7 +8358,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>刃牙道 第2クール</t>
+          <t>刃牙道 第1クール（TV放送）</t>
         </is>
       </c>
       <c r="D45" t="b">
@@ -8185,7 +8366,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F45" t="n">
@@ -8193,12 +8374,12 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Mountain Top</t>
+          <t>フルボコ</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>Novel Core</t>
+          <t>WANIMA</t>
         </is>
       </c>
       <c r="I45" t="inlineStr"/>
@@ -8217,7 +8398,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>花ざかりの君たちへ 第2期</t>
+          <t>刃牙道 第1クール（TV放送）</t>
         </is>
       </c>
       <c r="D46" t="b">
@@ -8229,16 +8410,16 @@
         </is>
       </c>
       <c r="F46" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>FLASHBULB</t>
+          <t>六ノ輪</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>Omoinotake</t>
+          <t>Chevon</t>
         </is>
       </c>
       <c r="I46" t="inlineStr"/>
@@ -8257,7 +8438,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>花ざかりの君たちへ 第2期</t>
+          <t>刃牙道 第1クール（TV放送）</t>
         </is>
       </c>
       <c r="D47" t="b">
@@ -8273,12 +8454,12 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>花束</t>
+          <t>Mountain Top</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>Omoinotake</t>
+          <t>Novel Core</t>
         </is>
       </c>
       <c r="I47" t="inlineStr"/>
@@ -8297,7 +8478,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>ヒロイン？聖女？いいえ、オールワークスメイドです（誇）！</t>
+          <t>刃牙道 第1クール（TV放送）</t>
         </is>
       </c>
       <c r="D48" t="b">
@@ -8305,20 +8486,20 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F48" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>マデュアル↔ハート</t>
+          <t>KATANA</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>メロディ・ウェーブ(CV：宮本侑芽) ルシアナ・ルトルバーグ(CV：大久保瑠美)</t>
+          <t>三代目 J SOUL BROTHERS</t>
         </is>
       </c>
       <c r="I48" t="inlineStr"/>
@@ -8337,7 +8518,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>ヒロイン？聖女？いいえ、オールワークスメイドです（誇）！</t>
+          <t>刃牙道 第2クール</t>
         </is>
       </c>
       <c r="D49" t="b">
@@ -8345,7 +8526,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F49" t="n">
@@ -8353,12 +8534,12 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>ハンドメイド</t>
+          <t>フルボコ</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>仲村宗悟</t>
+          <t>WANIMA</t>
         </is>
       </c>
       <c r="I49" t="inlineStr"/>
@@ -8377,7 +8558,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>ブチ切れ令嬢は報復を誓いました。 ～魔導書の力で祖国を叩き潰します～</t>
+          <t>刃牙道 第2クール</t>
         </is>
       </c>
       <c r="D50" t="b">
@@ -8389,16 +8570,16 @@
         </is>
       </c>
       <c r="F50" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Q.E.D.</t>
+          <t>六ノ輪</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>小倉唯</t>
+          <t>Chevon</t>
         </is>
       </c>
       <c r="I50" t="inlineStr"/>
@@ -8417,7 +8598,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>ブチ切れ令嬢は報復を誓いました。 ～魔導書の力で祖国を叩き潰します～</t>
+          <t>刃牙道 第2クール</t>
         </is>
       </c>
       <c r="D51" t="b">
@@ -8433,12 +8614,12 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>グッバイ・ララバイ</t>
+          <t>Mountain Top</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>大西亜玖璃</t>
+          <t>Novel Core</t>
         </is>
       </c>
       <c r="I51" t="inlineStr"/>
@@ -8457,7 +8638,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>プラノサウルス ガチコセイブツ部</t>
+          <t>刃牙道 第2クール</t>
         </is>
       </c>
       <c r="D52" t="b">
@@ -8465,20 +8646,20 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>主題歌</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F52" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>ガチde古生</t>
+          <t>KATANA</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>リンクルプラネット</t>
+          <t>三代目 J SOUL BROTHERS</t>
         </is>
       </c>
       <c r="I52" t="inlineStr"/>
@@ -8497,7 +8678,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>炎の闘球女 ドッジ弾子</t>
+          <t>花ざかりの君たちへ 第2期</t>
         </is>
       </c>
       <c r="D53" t="b">
@@ -8513,12 +8694,12 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>会心の一劇</t>
+          <t>FLASHBULB</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>ももいろクローバーZ</t>
+          <t>Omoinotake</t>
         </is>
       </c>
       <c r="I53" t="inlineStr"/>
@@ -8537,7 +8718,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>炎の闘球女 ドッジ弾子</t>
+          <t>花ざかりの君たちへ 第2期</t>
         </is>
       </c>
       <c r="D54" t="b">
@@ -8553,12 +8734,12 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Welcome to あざとさワールド</t>
+          <t>花束</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>i☆Ris</t>
+          <t>Omoinotake</t>
         </is>
       </c>
       <c r="I54" t="inlineStr"/>
@@ -8577,7 +8758,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>魔法少女リリカルなのは EXCEEDS Gun Blaze Vengeance</t>
+          <t>ヒロイン？聖女？いいえ、オールワークスメイドです（誇）！</t>
         </is>
       </c>
       <c r="D55" t="b">
@@ -8593,12 +8774,12 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>CRIMSON BULLET</t>
+          <t>マデュアル↔ハート</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>水樹奈々</t>
+          <t>メロディ・ウェーブ(CV：宮本侑芽) ルシアナ・ルトルバーグ(CV：大久保瑠美)</t>
         </is>
       </c>
       <c r="I55" t="inlineStr"/>
@@ -8617,7 +8798,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>魔法少女リリカルなのは EXCEEDS Gun Blaze Vengeance</t>
+          <t>ヒロイン？聖女？いいえ、オールワークスメイドです（誇）！</t>
         </is>
       </c>
       <c r="D56" t="b">
@@ -8633,12 +8814,12 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>Ephemeral</t>
+          <t>ハンドメイド</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>青木陽菜</t>
+          <t>仲村宗悟</t>
         </is>
       </c>
       <c r="I56" t="inlineStr"/>
@@ -8657,7 +8838,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>無自覚聖女は今日も無意識に力を垂れ流す</t>
+          <t>ブチ切れ令嬢は報復を誓いました。 ～魔導書の力で祖国を叩き潰します～</t>
         </is>
       </c>
       <c r="D57" t="b">
@@ -8673,12 +8854,12 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>Windmaker</t>
+          <t>Q.E.D.</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>花耶</t>
+          <t>小倉唯</t>
         </is>
       </c>
       <c r="I57" t="inlineStr"/>
@@ -8697,7 +8878,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>無自覚聖女は今日も無意識に力を垂れ流す</t>
+          <t>ブチ切れ令嬢は報復を誓いました。 ～魔導書の力で祖国を叩き潰します～</t>
         </is>
       </c>
       <c r="D58" t="b">
@@ -8713,12 +8894,12 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>アンノウンミー</t>
+          <t>グッバイ・ララバイ</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>ウタヒメドリーム オールスターズ【夢咲いぶき（CV:山﨑玲奈） 桜木舞華（CV:鈴木杏奈） 真白清美（CV:其原有沙） HiREN（CV:花耶） 水月ひかり（CV:礒部花凜） 高木凛（CV:鷲見友美ジェナ） 萩原ひまわり（CV:倉知玲鳳） SAKURAKO（CV:竹内夢）】</t>
+          <t>大西亜玖璃</t>
         </is>
       </c>
       <c r="I58" t="inlineStr"/>
@@ -8737,7 +8918,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>無職転生Ⅲ ～異世界行ったら本気だす～</t>
+          <t>プラノサウルス ガチコセイブツ部</t>
         </is>
       </c>
       <c r="D59" t="b">
@@ -8745,7 +8926,7 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>主題歌</t>
         </is>
       </c>
       <c r="F59" t="n">
@@ -8753,12 +8934,12 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>決意の唄</t>
+          <t>ガチde古生</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>大原ゆい子</t>
+          <t>リンクルプラネット</t>
         </is>
       </c>
       <c r="I59" t="inlineStr"/>
@@ -8777,7 +8958,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>メビウス・ダスト</t>
+          <t>炎の闘球女 ドッジ弾子</t>
         </is>
       </c>
       <c r="D60" t="b">
@@ -8793,12 +8974,12 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>メビウス</t>
+          <t>会心の一劇</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>家入レオ</t>
+          <t>ももいろクローバーZ</t>
         </is>
       </c>
       <c r="I60" t="inlineStr"/>
@@ -8817,7 +8998,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>ヤニねこ</t>
+          <t>炎の闘球女 ドッジ弾子</t>
         </is>
       </c>
       <c r="D61" t="b">
@@ -8825,7 +9006,7 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F61" t="n">
@@ -8833,12 +9014,12 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>なんもねえ</t>
+          <t>Welcome to あざとさワールド</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>忘れらんねえよ</t>
+          <t>i☆Ris</t>
         </is>
       </c>
       <c r="I61" t="inlineStr"/>
@@ -8857,7 +9038,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>鎧真伝サムライトルーパー 第2クール</t>
+          <t>魔法少女リリカルなのは EXCEEDS Gun Blaze Vengeance</t>
         </is>
       </c>
       <c r="D62" t="b">
@@ -8873,12 +9054,12 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>YOAKE</t>
+          <t>CRIMSON BULLET</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>blank paper</t>
+          <t>水樹奈々</t>
         </is>
       </c>
       <c r="I62" t="inlineStr"/>
@@ -8897,7 +9078,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>鎧真伝サムライトルーパー 第2クール</t>
+          <t>魔法少女リリカルなのは EXCEEDS Gun Blaze Vengeance</t>
         </is>
       </c>
       <c r="D63" t="b">
@@ -8905,20 +9086,20 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F63" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>BAD遺伝子</t>
+          <t>Ephemeral</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>Dannie May</t>
+          <t>青木陽菜</t>
         </is>
       </c>
       <c r="I63" t="inlineStr"/>
@@ -8937,7 +9118,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>鎧真伝サムライトルーパー 第2クール</t>
+          <t>無自覚聖女は今日も無意識に力を垂れ流す</t>
         </is>
       </c>
       <c r="D64" t="b">
@@ -8945,7 +9126,7 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F64" t="n">
@@ -8953,12 +9134,12 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>POWER</t>
+          <t>Windmaker</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>ONE OR EIGHT</t>
+          <t>花耶</t>
         </is>
       </c>
       <c r="I64" t="inlineStr"/>
@@ -8977,7 +9158,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>鎧真伝サムライトルーパー 第2クール</t>
+          <t>無自覚聖女は今日も無意識に力を垂れ流す</t>
         </is>
       </c>
       <c r="D65" t="b">
@@ -8989,16 +9170,16 @@
         </is>
       </c>
       <c r="F65" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>ばけもん</t>
+          <t>アンノウンミー</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>カラノア</t>
+          <t>ウタヒメドリーム オールスターズ【夢咲いぶき（CV:山﨑玲奈） 桜木舞華（CV:鈴木杏奈） 真白清美（CV:其原有沙） HiREN（CV:花耶） 水月ひかり（CV:礒部花凜） 高木凛（CV:鷲見友美ジェナ） 萩原ひまわり（CV:倉知玲鳳） SAKURAKO（CV:竹内夢）】</t>
         </is>
       </c>
       <c r="I65" t="inlineStr"/>
@@ -9017,7 +9198,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>落第賢者の学院無双～二度目の転生、Sランクチート魔術師冒険録～</t>
+          <t>無職転生Ⅲ ～異世界行ったら本気だす～</t>
         </is>
       </c>
       <c r="D66" t="b">
@@ -9025,7 +9206,7 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F66" t="n">
@@ -9033,12 +9214,12 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>憧憬</t>
+          <t>決意の唄</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>TrySail</t>
+          <t>大原ゆい子</t>
         </is>
       </c>
       <c r="I66" t="inlineStr"/>
@@ -9057,7 +9238,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>領民0人スタートの辺境領主様</t>
+          <t>メビウス・ダスト</t>
         </is>
       </c>
       <c r="D67" t="b">
@@ -9073,12 +9254,12 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>Wonder</t>
+          <t>メビウス</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>CROWN HEAD</t>
+          <t>家入レオ</t>
         </is>
       </c>
       <c r="I67" t="inlineStr"/>
@@ -9097,7 +9278,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>領民0人スタートの辺境領主様</t>
+          <t>ヤニねこ</t>
         </is>
       </c>
       <c r="D68" t="b">
@@ -9105,7 +9286,7 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F68" t="n">
@@ -9113,12 +9294,12 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>星降る夜の約束</t>
+          <t>なんもねえ</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>花耶</t>
+          <t>忘れらんねえよ</t>
         </is>
       </c>
       <c r="I68" t="inlineStr"/>
@@ -9137,7 +9318,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>令和のダラさん</t>
+          <t>鎧真伝サムライトルーパー 第2クール</t>
         </is>
       </c>
       <c r="D69" t="b">
@@ -9153,12 +9334,12 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>ダラダラ♡ダンシング</t>
+          <t>YOAKE</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>ダラさん（CV：田村睦心） 三⼗⽊⾕⽇向（CV：津田美波） 三⼗⽊⾕薫（CV：寺澤百花） ナレーション（CV：てらそままさき）</t>
+          <t>blank paper</t>
         </is>
       </c>
       <c r="I69" t="inlineStr"/>
@@ -9177,7 +9358,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>LV999の村人</t>
+          <t>鎧真伝サムライトルーパー 第2クール</t>
         </is>
       </c>
       <c r="D70" t="b">
@@ -9189,16 +9370,16 @@
         </is>
       </c>
       <c r="F70" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>Not a Hero</t>
+          <t>BAD遺伝子</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>藍月なくる&amp;棗いつき</t>
+          <t>Dannie May</t>
         </is>
       </c>
       <c r="I70" t="inlineStr"/>
@@ -9217,7 +9398,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>ワールド イズ ダンシング</t>
+          <t>鎧真伝サムライトルーパー 第2クール</t>
         </is>
       </c>
       <c r="D71" t="b">
@@ -9225,7 +9406,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F71" t="n">
@@ -9233,12 +9414,12 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>終宵</t>
+          <t>POWER</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>マカロニえんぴつ</t>
+          <t>ONE OR EIGHT</t>
         </is>
       </c>
       <c r="I71" t="inlineStr"/>
@@ -9248,16 +9429,16 @@
     </row>
     <row r="72">
       <c r="A72" t="n">
-        <v>5947</v>
+        <v>5806</v>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2026秋アニメ</t>
+          <t>2026夏アニメ</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>転生した大聖女は、聖女であることをひた隠す</t>
+          <t>鎧真伝サムライトルーパー 第2クール</t>
         </is>
       </c>
       <c r="D72" t="b">
@@ -9265,20 +9446,20 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F72" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>Flare of Soul</t>
+          <t>ばけもん</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>花耶</t>
+          <t>カラノア</t>
         </is>
       </c>
       <c r="I72" t="inlineStr"/>
@@ -9288,16 +9469,16 @@
     </row>
     <row r="73">
       <c r="A73" t="n">
-        <v>5947</v>
+        <v>5806</v>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2026秋アニメ</t>
+          <t>2026夏アニメ</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>転生した大聖女は、聖女であることをひた隠す</t>
+          <t>落第賢者の学院無双～二度目の転生、Sランクチート魔術師冒険録～</t>
         </is>
       </c>
       <c r="D73" t="b">
@@ -9313,12 +9494,12 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>STELLAR</t>
+          <t>憧憬</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>ウタヒメドリーム オールスターズ</t>
+          <t>TrySail</t>
         </is>
       </c>
       <c r="I73" t="inlineStr"/>
@@ -9328,16 +9509,16 @@
     </row>
     <row r="74">
       <c r="A74" t="n">
-        <v>5947</v>
+        <v>5806</v>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2026秋アニメ</t>
+          <t>2026夏アニメ</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>魔法少女育成計画restart</t>
+          <t>領民0人スタートの辺境領主様</t>
         </is>
       </c>
       <c r="D74" t="b">
@@ -9353,12 +9534,12 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>No tears here</t>
+          <t>Wonder</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>茅原実里</t>
+          <t>CROWN HEAD</t>
         </is>
       </c>
       <c r="I74" t="inlineStr"/>
@@ -9366,6 +9547,326 @@
       <c r="K74" t="inlineStr"/>
       <c r="L74" t="inlineStr"/>
     </row>
+    <row r="75">
+      <c r="A75" t="n">
+        <v>5806</v>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>2026夏アニメ</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>領民0人スタートの辺境領主様</t>
+        </is>
+      </c>
+      <c r="D75" t="b">
+        <v>0</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>ED</t>
+        </is>
+      </c>
+      <c r="F75" t="n">
+        <v>1</v>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>星降る夜の約束</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>花耶</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr"/>
+      <c r="J75" t="inlineStr"/>
+      <c r="K75" t="inlineStr"/>
+      <c r="L75" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" t="n">
+        <v>5806</v>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>2026夏アニメ</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>令和のダラさん</t>
+        </is>
+      </c>
+      <c r="D76" t="b">
+        <v>0</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="F76" t="n">
+        <v>1</v>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>ダラダラ♡ダンシング</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>ダラさん（CV：田村睦心） 三⼗⽊⾕⽇向（CV：津田美波） 三⼗⽊⾕薫（CV：寺澤百花） ナレーション（CV：てらそままさき）</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr"/>
+      <c r="J76" t="inlineStr"/>
+      <c r="K76" t="inlineStr"/>
+      <c r="L76" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" t="n">
+        <v>5806</v>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>2026夏アニメ</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>LV999の村人</t>
+        </is>
+      </c>
+      <c r="D77" t="b">
+        <v>0</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="F77" t="n">
+        <v>1</v>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>Not a Hero</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>藍月なくる&amp;棗いつき</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr"/>
+      <c r="J77" t="inlineStr"/>
+      <c r="K77" t="inlineStr"/>
+      <c r="L77" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" t="n">
+        <v>5806</v>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>2026夏アニメ</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>ワールド イズ ダンシング</t>
+        </is>
+      </c>
+      <c r="D78" t="b">
+        <v>0</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="F78" t="n">
+        <v>1</v>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>終宵</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>マカロニえんぴつ</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr"/>
+      <c r="J78" t="inlineStr"/>
+      <c r="K78" t="inlineStr"/>
+      <c r="L78" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>獣王武神ダンデヴァイン</t>
+        </is>
+      </c>
+      <c r="D79" t="b">
+        <v>0</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="F79" t="n">
+        <v>1</v>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>曲名未発表</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>西川貴教</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr"/>
+      <c r="J79" t="inlineStr"/>
+      <c r="K79" t="inlineStr"/>
+      <c r="L79" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>転生した大聖女は、聖女であることをひた隠す</t>
+        </is>
+      </c>
+      <c r="D80" t="b">
+        <v>0</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="F80" t="n">
+        <v>1</v>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>Flare of Soul</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>花耶</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr"/>
+      <c r="J80" t="inlineStr"/>
+      <c r="K80" t="inlineStr"/>
+      <c r="L80" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>転生した大聖女は、聖女であることをひた隠す</t>
+        </is>
+      </c>
+      <c r="D81" t="b">
+        <v>0</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>ED</t>
+        </is>
+      </c>
+      <c r="F81" t="n">
+        <v>1</v>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>STELLAR</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>ウタヒメドリーム オールスターズ</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr"/>
+      <c r="J81" t="inlineStr"/>
+      <c r="K81" t="inlineStr"/>
+      <c r="L81" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>魔法少女育成計画restart</t>
+        </is>
+      </c>
+      <c r="D82" t="b">
+        <v>0</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="F82" t="n">
+        <v>1</v>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>No tears here</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>茅原実里</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr"/>
+      <c r="J82" t="inlineStr"/>
+      <c r="K82" t="inlineStr"/>
+      <c r="L82" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
auto: anime list update 2026-06-05
</commit_message>
<xml_diff>
--- a/data/anime_list.xlsx
+++ b/data/anime_list.xlsx
@@ -2751,7 +2751,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>2026年7月～ TOKYO MXほか</t>
+          <t>2026年7月4日（土）～ TOKYO MXほか</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -3826,8 +3826,16 @@
           <t>大原ゆい子</t>
         </is>
       </c>
-      <c r="K67" t="inlineStr"/>
-      <c r="L67" t="inlineStr"/>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>祈り、終われば</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>中島美嘉</t>
+        </is>
+      </c>
       <c r="M67" t="inlineStr">
         <is>
           <t>https://www.animatetimes.com/tag/details.php?id=24285</t>
@@ -3861,7 +3869,7 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>2026年7月～</t>
+          <t>2026年7月9日（木）～ TOKYO MXほか</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
@@ -3879,8 +3887,16 @@
           <t>家入レオ</t>
         </is>
       </c>
-      <c r="K68" t="inlineStr"/>
-      <c r="L68" t="inlineStr"/>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>ジレンマ</t>
+        </is>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>冨岡愛</t>
+        </is>
+      </c>
       <c r="M68" t="inlineStr">
         <is>
           <t>https://www.animatetimes.com/tag/details.php?id=28016</t>
@@ -6548,7 +6564,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L82"/>
+  <dimension ref="A1:L84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7368,10 +7384,24 @@
           <t>MIYAVI</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
-      <c r="L20" t="inlineStr"/>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=HSakQbaQifs</t>
+        </is>
+      </c>
+      <c r="J20" t="n">
+        <v>19423</v>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>コードギアスチャンネル CODEGEASS Channel</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>2026-06-05T19:01:45</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -9238,7 +9268,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>メビウス・ダスト</t>
+          <t>無職転生Ⅲ ～異世界行ったら本気だす～</t>
         </is>
       </c>
       <c r="D67" t="b">
@@ -9246,7 +9276,7 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F67" t="n">
@@ -9254,12 +9284,12 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>メビウス</t>
+          <t>祈り、終われば</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>家入レオ</t>
+          <t>中島美嘉</t>
         </is>
       </c>
       <c r="I67" t="inlineStr"/>
@@ -9278,7 +9308,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>ヤニねこ</t>
+          <t>メビウス・ダスト</t>
         </is>
       </c>
       <c r="D68" t="b">
@@ -9294,12 +9324,12 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>なんもねえ</t>
+          <t>メビウス</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>忘れらんねえよ</t>
+          <t>家入レオ</t>
         </is>
       </c>
       <c r="I68" t="inlineStr"/>
@@ -9318,7 +9348,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>鎧真伝サムライトルーパー 第2クール</t>
+          <t>メビウス・ダスト</t>
         </is>
       </c>
       <c r="D69" t="b">
@@ -9326,7 +9356,7 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F69" t="n">
@@ -9334,12 +9364,12 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>YOAKE</t>
+          <t>ジレンマ</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>blank paper</t>
+          <t>冨岡愛</t>
         </is>
       </c>
       <c r="I69" t="inlineStr"/>
@@ -9358,7 +9388,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>鎧真伝サムライトルーパー 第2クール</t>
+          <t>ヤニねこ</t>
         </is>
       </c>
       <c r="D70" t="b">
@@ -9370,16 +9400,16 @@
         </is>
       </c>
       <c r="F70" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>BAD遺伝子</t>
+          <t>なんもねえ</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>Dannie May</t>
+          <t>忘れらんねえよ</t>
         </is>
       </c>
       <c r="I70" t="inlineStr"/>
@@ -9406,7 +9436,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F71" t="n">
@@ -9414,12 +9444,12 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>POWER</t>
+          <t>YOAKE</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>ONE OR EIGHT</t>
+          <t>blank paper</t>
         </is>
       </c>
       <c r="I71" t="inlineStr"/>
@@ -9446,7 +9476,7 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F72" t="n">
@@ -9454,12 +9484,12 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>ばけもん</t>
+          <t>BAD遺伝子</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>カラノア</t>
+          <t>Dannie May</t>
         </is>
       </c>
       <c r="I72" t="inlineStr"/>
@@ -9478,7 +9508,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>落第賢者の学院無双～二度目の転生、Sランクチート魔術師冒険録～</t>
+          <t>鎧真伝サムライトルーパー 第2クール</t>
         </is>
       </c>
       <c r="D73" t="b">
@@ -9494,12 +9524,12 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>憧憬</t>
+          <t>POWER</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>TrySail</t>
+          <t>ONE OR EIGHT</t>
         </is>
       </c>
       <c r="I73" t="inlineStr"/>
@@ -9518,7 +9548,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>領民0人スタートの辺境領主様</t>
+          <t>鎧真伝サムライトルーパー 第2クール</t>
         </is>
       </c>
       <c r="D74" t="b">
@@ -9526,20 +9556,20 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F74" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>Wonder</t>
+          <t>ばけもん</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>CROWN HEAD</t>
+          <t>カラノア</t>
         </is>
       </c>
       <c r="I74" t="inlineStr"/>
@@ -9558,7 +9588,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>領民0人スタートの辺境領主様</t>
+          <t>落第賢者の学院無双～二度目の転生、Sランクチート魔術師冒険録～</t>
         </is>
       </c>
       <c r="D75" t="b">
@@ -9574,12 +9604,12 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>星降る夜の約束</t>
+          <t>憧憬</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>花耶</t>
+          <t>TrySail</t>
         </is>
       </c>
       <c r="I75" t="inlineStr"/>
@@ -9598,7 +9628,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>令和のダラさん</t>
+          <t>領民0人スタートの辺境領主様</t>
         </is>
       </c>
       <c r="D76" t="b">
@@ -9614,12 +9644,12 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>ダラダラ♡ダンシング</t>
+          <t>Wonder</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>ダラさん（CV：田村睦心） 三⼗⽊⾕⽇向（CV：津田美波） 三⼗⽊⾕薫（CV：寺澤百花） ナレーション（CV：てらそままさき）</t>
+          <t>CROWN HEAD</t>
         </is>
       </c>
       <c r="I76" t="inlineStr"/>
@@ -9638,7 +9668,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>LV999の村人</t>
+          <t>領民0人スタートの辺境領主様</t>
         </is>
       </c>
       <c r="D77" t="b">
@@ -9646,7 +9676,7 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F77" t="n">
@@ -9654,12 +9684,12 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>Not a Hero</t>
+          <t>星降る夜の約束</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>藍月なくる&amp;棗いつき</t>
+          <t>花耶</t>
         </is>
       </c>
       <c r="I77" t="inlineStr"/>
@@ -9678,7 +9708,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>ワールド イズ ダンシング</t>
+          <t>令和のダラさん</t>
         </is>
       </c>
       <c r="D78" t="b">
@@ -9694,12 +9724,12 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>終宵</t>
+          <t>ダラダラ♡ダンシング</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>マカロニえんぴつ</t>
+          <t>ダラさん（CV：田村睦心） 三⼗⽊⾕⽇向（CV：津田美波） 三⼗⽊⾕薫（CV：寺澤百花） ナレーション（CV：てらそままさき）</t>
         </is>
       </c>
       <c r="I78" t="inlineStr"/>
@@ -9709,16 +9739,16 @@
     </row>
     <row r="79">
       <c r="A79" t="n">
-        <v>5947</v>
+        <v>5806</v>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2026秋アニメ</t>
+          <t>2026夏アニメ</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>獣王武神ダンデヴァイン</t>
+          <t>LV999の村人</t>
         </is>
       </c>
       <c r="D79" t="b">
@@ -9734,12 +9764,12 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>曲名未発表</t>
+          <t>Not a Hero</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>西川貴教</t>
+          <t>藍月なくる&amp;棗いつき</t>
         </is>
       </c>
       <c r="I79" t="inlineStr"/>
@@ -9749,16 +9779,16 @@
     </row>
     <row r="80">
       <c r="A80" t="n">
-        <v>5947</v>
+        <v>5806</v>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>2026秋アニメ</t>
+          <t>2026夏アニメ</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>転生した大聖女は、聖女であることをひた隠す</t>
+          <t>ワールド イズ ダンシング</t>
         </is>
       </c>
       <c r="D80" t="b">
@@ -9774,12 +9804,12 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>Flare of Soul</t>
+          <t>終宵</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>花耶</t>
+          <t>マカロニえんぴつ</t>
         </is>
       </c>
       <c r="I80" t="inlineStr"/>
@@ -9798,7 +9828,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>転生した大聖女は、聖女であることをひた隠す</t>
+          <t>獣王武神ダンデヴァイン</t>
         </is>
       </c>
       <c r="D81" t="b">
@@ -9806,7 +9836,7 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F81" t="n">
@@ -9814,12 +9844,12 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>STELLAR</t>
+          <t>曲名未発表</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>ウタヒメドリーム オールスターズ</t>
+          <t>西川貴教</t>
         </is>
       </c>
       <c r="I81" t="inlineStr"/>
@@ -9838,7 +9868,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>魔法少女育成計画restart</t>
+          <t>転生した大聖女は、聖女であることをひた隠す</t>
         </is>
       </c>
       <c r="D82" t="b">
@@ -9854,12 +9884,12 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>No tears here</t>
+          <t>Flare of Soul</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>茅原実里</t>
+          <t>花耶</t>
         </is>
       </c>
       <c r="I82" t="inlineStr"/>
@@ -9867,6 +9897,86 @@
       <c r="K82" t="inlineStr"/>
       <c r="L82" t="inlineStr"/>
     </row>
+    <row r="83">
+      <c r="A83" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>転生した大聖女は、聖女であることをひた隠す</t>
+        </is>
+      </c>
+      <c r="D83" t="b">
+        <v>0</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>ED</t>
+        </is>
+      </c>
+      <c r="F83" t="n">
+        <v>1</v>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>STELLAR</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>ウタヒメドリーム オールスターズ</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr"/>
+      <c r="J83" t="inlineStr"/>
+      <c r="K83" t="inlineStr"/>
+      <c r="L83" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>魔法少女育成計画restart</t>
+        </is>
+      </c>
+      <c r="D84" t="b">
+        <v>0</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="F84" t="n">
+        <v>1</v>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>No tears here</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>茅原実里</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr"/>
+      <c r="J84" t="inlineStr"/>
+      <c r="K84" t="inlineStr"/>
+      <c r="L84" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
auto: anime list update 2026-06-10
</commit_message>
<xml_diff>
--- a/data/anime_list.xlsx
+++ b/data/anime_list.xlsx
@@ -1233,7 +1233,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026年7月～</t>
+          <t>2026年7月7日（火）～ TOKYO MX ほか</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1241,10 +1241,26 @@
           <t>ROLL2</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr"/>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Amore</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>ReoNa</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>エテルネル</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>sajou no hana</t>
+        </is>
+      </c>
       <c r="M16" t="inlineStr">
         <is>
           <t>https://www.animatetimes.com/tag/details.php?id=25598</t>
@@ -1441,7 +1457,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>2026年7月～</t>
+          <t>2026年7月8日（水）～ TOKYO MX ほか</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -1449,8 +1465,16 @@
           <t>Lay-duce</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Foreshadow</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>前島麻由</t>
+        </is>
+      </c>
       <c r="K20" t="inlineStr">
         <is>
           <t>Awake Anew</t>
@@ -3195,7 +3219,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>2026年7月～ ABCテレビ・テレビ朝日系・BS日テレにて</t>
+          <t>2026年7月11日（土）～ ABCテレビ・テレビ朝日系・BS日テレにて</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
@@ -3517,8 +3541,16 @@
           <t>動画工房</t>
         </is>
       </c>
-      <c r="I60" t="inlineStr"/>
-      <c r="J60" t="inlineStr"/>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Sunny</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>milet</t>
+        </is>
+      </c>
       <c r="K60" t="inlineStr"/>
       <c r="L60" t="inlineStr"/>
       <c r="M60" t="inlineStr">
@@ -6876,7 +6908,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L103"/>
+  <dimension ref="A1:L107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7672,7 +7704,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>「きみを愛する気はない」と言った次期公爵様がなぜか溺愛してきます</t>
+          <t>きみが死ぬまで恋をしたい</t>
         </is>
       </c>
       <c r="D20" t="b">
@@ -7688,12 +7720,12 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>いつかちゃんと。</t>
+          <t>Amore</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>りりあ。</t>
+          <t>ReoNa</t>
         </is>
       </c>
       <c r="I20" t="inlineStr"/>
@@ -7712,7 +7744,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>「きみを愛する気はない」と言った次期公爵様がなぜか溺愛してきます</t>
+          <t>きみが死ぬまで恋をしたい</t>
         </is>
       </c>
       <c r="D21" t="b">
@@ -7728,12 +7760,12 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>最終回</t>
+          <t>エテルネル</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>sorato</t>
+          <t>sajou no hana</t>
         </is>
       </c>
       <c r="I21" t="inlineStr"/>
@@ -7752,7 +7784,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>ぐらんぶる Season 3</t>
+          <t>「きみを愛する気はない」と言った次期公爵様がなぜか溺愛してきます</t>
         </is>
       </c>
       <c r="D22" t="b">
@@ -7768,12 +7800,12 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>夏子</t>
+          <t>いつかちゃんと。</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>FUNKY MONKEY BΛBY'S</t>
+          <t>りりあ。</t>
         </is>
       </c>
       <c r="I22" t="inlineStr"/>
@@ -7792,7 +7824,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>ぐらんぶる Season 3</t>
+          <t>「きみを愛する気はない」と言った次期公爵様がなぜか溺愛してきます</t>
         </is>
       </c>
       <c r="D23" t="b">
@@ -7808,12 +7840,12 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>裸のマーメード</t>
+          <t>最終回</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>豆柴の大群</t>
+          <t>sorato</t>
         </is>
       </c>
       <c r="I23" t="inlineStr"/>
@@ -7832,7 +7864,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>クレバテスII-魔獣の王と偽りの勇者伝承-</t>
+          <t>ぐらんぶる Season 3</t>
         </is>
       </c>
       <c r="D24" t="b">
@@ -7840,7 +7872,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F24" t="n">
@@ -7848,12 +7880,12 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Awake Anew</t>
+          <t>夏子</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>MYTH &amp; ROID</t>
+          <t>FUNKY MONKEY BΛBY'S</t>
         </is>
       </c>
       <c r="I24" t="inlineStr"/>
@@ -7872,7 +7904,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>コードギアス 奪還のロゼ TV放送</t>
+          <t>ぐらんぶる Season 3</t>
         </is>
       </c>
       <c r="D25" t="b">
@@ -7880,7 +7912,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F25" t="n">
@@ -7888,32 +7920,18 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Running In My Head</t>
+          <t>裸のマーメード</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>MIYAVI</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=HSakQbaQifs</t>
-        </is>
-      </c>
-      <c r="J25" t="n">
-        <v>19423</v>
-      </c>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t>コードギアスチャンネル CODEGEASS Channel</t>
-        </is>
-      </c>
-      <c r="L25" t="inlineStr">
-        <is>
-          <t>2026-06-05T19:01:45</t>
-        </is>
-      </c>
+          <t>豆柴の大群</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -7926,7 +7944,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>コードギアス 奪還のロゼ TV放送</t>
+          <t>クレバテスII-魔獣の王と偽りの勇者伝承-</t>
         </is>
       </c>
       <c r="D26" t="b">
@@ -7934,7 +7952,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F26" t="n">
@@ -7942,12 +7960,12 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>ロゼ (Prod.TeddyLoid)</t>
+          <t>Foreshadow</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>満島ひかり</t>
+          <t>前島麻由</t>
         </is>
       </c>
       <c r="I26" t="inlineStr"/>
@@ -7966,7 +7984,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>これ描いて死ね</t>
+          <t>クレバテスII-魔獣の王と偽りの勇者伝承-</t>
         </is>
       </c>
       <c r="D27" t="b">
@@ -7974,7 +7992,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F27" t="n">
@@ -7982,12 +8000,12 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>遺書</t>
+          <t>Awake Anew</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>キタニタツヤ</t>
+          <t>MYTH &amp; ROID</t>
         </is>
       </c>
       <c r="I27" t="inlineStr"/>
@@ -8006,7 +8024,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>これ描いて死ね</t>
+          <t>コードギアス 奪還のロゼ TV放送</t>
         </is>
       </c>
       <c r="D28" t="b">
@@ -8014,7 +8032,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F28" t="n">
@@ -8022,18 +8040,32 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>コニファー</t>
+          <t>Running In My Head</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>リーガルリリー</t>
-        </is>
-      </c>
-      <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr"/>
-      <c r="L28" t="inlineStr"/>
+          <t>MIYAVI</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=HSakQbaQifs</t>
+        </is>
+      </c>
+      <c r="J28" t="n">
+        <v>19423</v>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>コードギアスチャンネル CODEGEASS Channel</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>2026-06-05T19:01:45</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -8046,7 +8078,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>才女のお世話 高嶺の花だらけな名門校で、学院一のお嬢様(生活能力皆無)を陰ながらお世話することになりました</t>
+          <t>コードギアス 奪還のロゼ TV放送</t>
         </is>
       </c>
       <c r="D29" t="b">
@@ -8054,7 +8086,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F29" t="n">
@@ -8062,12 +8094,12 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>最最最高級のお世話して</t>
+          <t>ロゼ (Prod.TeddyLoid)</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>angela</t>
+          <t>満島ひかり</t>
         </is>
       </c>
       <c r="I29" t="inlineStr"/>
@@ -8086,7 +8118,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>才女のお世話 高嶺の花だらけな名門校で、学院一のお嬢様(生活能力皆無)を陰ながらお世話することになりました</t>
+          <t>これ描いて死ね</t>
         </is>
       </c>
       <c r="D30" t="b">
@@ -8094,7 +8126,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F30" t="n">
@@ -8102,12 +8134,12 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>完璧じゃないわたし</t>
+          <t>遺書</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>前島亜美</t>
+          <t>キタニタツヤ</t>
         </is>
       </c>
       <c r="I30" t="inlineStr"/>
@@ -8126,7 +8158,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>サイボーグ009 ネメシス</t>
+          <t>これ描いて死ね</t>
         </is>
       </c>
       <c r="D31" t="b">
@@ -8134,7 +8166,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F31" t="n">
@@ -8142,12 +8174,12 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>誰がために</t>
+          <t>コニファー</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>杏子</t>
+          <t>リーガルリリー</t>
         </is>
       </c>
       <c r="I31" t="inlineStr"/>
@@ -8166,7 +8198,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>さよならララ</t>
+          <t>才女のお世話 高嶺の花だらけな名門校で、学院一のお嬢様(生活能力皆無)を陰ながらお世話することになりました</t>
         </is>
       </c>
       <c r="D32" t="b">
@@ -8182,12 +8214,12 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>さよならララ</t>
+          <t>最最最高級のお世話して</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>いきものがかり</t>
+          <t>angela</t>
         </is>
       </c>
       <c r="I32" t="inlineStr"/>
@@ -8206,7 +8238,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>スーパーの裏でヤニ吸うふたり</t>
+          <t>才女のお世話 高嶺の花だらけな名門校で、学院一のお嬢様(生活能力皆無)を陰ながらお世話することになりました</t>
         </is>
       </c>
       <c r="D33" t="b">
@@ -8214,7 +8246,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F33" t="n">
@@ -8222,12 +8254,12 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>イチジク煙</t>
+          <t>完璧じゃないわたし</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>ずっと真夜中でいいのに。</t>
+          <t>前島亜美</t>
         </is>
       </c>
       <c r="I33" t="inlineStr"/>
@@ -8246,7 +8278,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>スーパーの裏でヤニ吸うふたり</t>
+          <t>サイボーグ009 ネメシス</t>
         </is>
       </c>
       <c r="D34" t="b">
@@ -8254,7 +8286,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F34" t="n">
@@ -8262,12 +8294,12 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Fiction</t>
+          <t>誰がために</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>imase</t>
+          <t>杏子</t>
         </is>
       </c>
       <c r="I34" t="inlineStr"/>
@@ -8286,7 +8318,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>捨てられ聖女の異世界ごはん旅 隠れスキルでキャンピングカーを召喚しました</t>
+          <t>さよならララ</t>
         </is>
       </c>
       <c r="D35" t="b">
@@ -8302,12 +8334,12 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Butterfly</t>
+          <t>さよならララ</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>INUWASI</t>
+          <t>いきものがかり</t>
         </is>
       </c>
       <c r="I35" t="inlineStr"/>
@@ -8326,7 +8358,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>捨てられ聖女の異世界ごはん旅 隠れスキルでキャンピングカーを召喚しました</t>
+          <t>スーパーの裏でヤニ吸うふたり</t>
         </is>
       </c>
       <c r="D36" t="b">
@@ -8334,7 +8366,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F36" t="n">
@@ -8342,12 +8374,12 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Holy Sweet Home</t>
+          <t>イチジク煙</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>音感れもねゐど</t>
+          <t>ずっと真夜中でいいのに。</t>
         </is>
       </c>
       <c r="I36" t="inlineStr"/>
@@ -8366,15 +8398,15 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>青春ブタ野郎はサンタクロースの夢を見ない</t>
+          <t>スーパーの裏でヤニ吸うふたり</t>
         </is>
       </c>
       <c r="D37" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F37" t="n">
@@ -8382,12 +8414,12 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>スノウドロップ</t>
+          <t>Fiction</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Conton Candy</t>
+          <t>imase</t>
         </is>
       </c>
       <c r="I37" t="inlineStr"/>
@@ -8406,15 +8438,15 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>青春ブタ野郎はサンタクロースの夢を見ない</t>
+          <t>捨てられ聖女の異世界ごはん旅 隠れスキルでキャンピングカーを召喚しました</t>
         </is>
       </c>
       <c r="D38" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F38" t="n">
@@ -8422,12 +8454,12 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>水平線は僕の古傷</t>
+          <t>Butterfly</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>広川卯月、赤城郁実、姫路紗良、霧島透子</t>
+          <t>INUWASI</t>
         </is>
       </c>
       <c r="I38" t="inlineStr"/>
@@ -8446,7 +8478,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>正反対な君と僕 第2期</t>
+          <t>捨てられ聖女の異世界ごはん旅 隠れスキルでキャンピングカーを召喚しました</t>
         </is>
       </c>
       <c r="D39" t="b">
@@ -8454,7 +8486,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F39" t="n">
@@ -8462,12 +8494,12 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>メガネを外して</t>
+          <t>Holy Sweet Home</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>乃紫</t>
+          <t>音感れもねゐど</t>
         </is>
       </c>
       <c r="I39" t="inlineStr"/>
@@ -8486,11 +8518,11 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>正反対な君と僕 第2期</t>
+          <t>青春ブタ野郎はサンタクロースの夢を見ない</t>
         </is>
       </c>
       <c r="D40" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -8498,16 +8530,16 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>猫じゃらし</t>
+          <t>スノウドロップ</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>7co</t>
+          <t>Conton Candy</t>
         </is>
       </c>
       <c r="I40" t="inlineStr"/>
@@ -8526,11 +8558,11 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>正反対な君と僕 第2期</t>
+          <t>青春ブタ野郎はサンタクロースの夢を見ない</t>
         </is>
       </c>
       <c r="D41" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -8542,12 +8574,12 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>ピュア feat. 橋本絵莉子</t>
+          <t>水平線は僕の古傷</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>PAS TASTA</t>
+          <t>広川卯月、赤城郁実、姫路紗良、霧島透子</t>
         </is>
       </c>
       <c r="I41" t="inlineStr"/>
@@ -8566,7 +8598,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>対ありでした。～お嬢さまは格闘ゲームなんてしない～</t>
+          <t>正反対な君と僕 第2期</t>
         </is>
       </c>
       <c r="D42" t="b">
@@ -8582,12 +8614,12 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>命短し対する乙女よ</t>
+          <t>メガネを外して</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>花冷え。</t>
+          <t>乃紫</t>
         </is>
       </c>
       <c r="I42" t="inlineStr"/>
@@ -8606,7 +8638,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>対ありでした。～お嬢さまは格闘ゲームなんてしない～</t>
+          <t>正反対な君と僕 第2期</t>
         </is>
       </c>
       <c r="D43" t="b">
@@ -8614,20 +8646,20 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F43" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>NEW GAME</t>
+          <t>猫じゃらし</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>halca</t>
+          <t>7co</t>
         </is>
       </c>
       <c r="I43" t="inlineStr"/>
@@ -8646,7 +8678,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>追放された転生重騎士はゲーム知識で無双する</t>
+          <t>正反対な君と僕 第2期</t>
         </is>
       </c>
       <c r="D44" t="b">
@@ -8654,7 +8686,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F44" t="n">
@@ -8662,12 +8694,12 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Awake</t>
+          <t>ピュア feat. 橋本絵莉子</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>SPYAIR</t>
+          <t>PAS TASTA</t>
         </is>
       </c>
       <c r="I44" t="inlineStr"/>
@@ -8686,7 +8718,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>鉄鍋のジャン！</t>
+          <t>対ありでした。～お嬢さまは格闘ゲームなんてしない～</t>
         </is>
       </c>
       <c r="D45" t="b">
@@ -8702,12 +8734,12 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>火宴</t>
+          <t>命短し対する乙女よ</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>原因は自分にある。</t>
+          <t>花冷え。</t>
         </is>
       </c>
       <c r="I45" t="inlineStr"/>
@@ -8726,7 +8758,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>手札が多めのビクトリア</t>
+          <t>対ありでした。～お嬢さまは格闘ゲームなんてしない～</t>
         </is>
       </c>
       <c r="D46" t="b">
@@ -8742,32 +8774,18 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>縁のつき</t>
+          <t>NEW GAME</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>KI_EN</t>
-        </is>
-      </c>
-      <c r="I46" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=-HNOXWE2wVU</t>
-        </is>
-      </c>
-      <c r="J46" t="n">
-        <v>107892</v>
-      </c>
-      <c r="K46" t="inlineStr">
-        <is>
-          <t>KADOKAWAanime</t>
-        </is>
-      </c>
-      <c r="L46" t="inlineStr">
-        <is>
-          <t>2026-06-04T19:29:01</t>
-        </is>
-      </c>
+          <t>halca</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr"/>
+      <c r="J46" t="inlineStr"/>
+      <c r="K46" t="inlineStr"/>
+      <c r="L46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -8780,7 +8798,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>転校先の清楚可憐な美少女が、昔男子と思って一緒に遊んだ幼馴染だった件</t>
+          <t>追放された転生重騎士はゲーム知識で無双する</t>
         </is>
       </c>
       <c r="D47" t="b">
@@ -8796,12 +8814,12 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>夏に重ねて</t>
+          <t>Awake</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>DIALOGUE+</t>
+          <t>SPYAIR</t>
         </is>
       </c>
       <c r="I47" t="inlineStr"/>
@@ -8820,7 +8838,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>天は赤い河のほとり</t>
+          <t>鉄鍋のジャン！</t>
         </is>
       </c>
       <c r="D48" t="b">
@@ -8836,12 +8854,12 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>暁の空</t>
+          <t>火宴</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>七海ひろき</t>
+          <t>原因は自分にある。</t>
         </is>
       </c>
       <c r="I48" t="inlineStr"/>
@@ -8860,7 +8878,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>天幕のジャードゥーガル</t>
+          <t>手札が多めのビクトリア</t>
         </is>
       </c>
       <c r="D49" t="b">
@@ -8868,7 +8886,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F49" t="n">
@@ -8876,18 +8894,32 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Stella</t>
+          <t>縁のつき</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>SEKAI NO OWARI</t>
-        </is>
-      </c>
-      <c r="I49" t="inlineStr"/>
-      <c r="J49" t="inlineStr"/>
-      <c r="K49" t="inlineStr"/>
-      <c r="L49" t="inlineStr"/>
+          <t>KI_EN</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=-HNOXWE2wVU</t>
+        </is>
+      </c>
+      <c r="J49" t="n">
+        <v>107892</v>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>2026-06-04T19:29:01</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -8900,7 +8932,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>盗掘王</t>
+          <t>転校先の清楚可憐な美少女が、昔男子と思って一緒に遊んだ幼馴染だった件</t>
         </is>
       </c>
       <c r="D50" t="b">
@@ -8916,12 +8948,12 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>SHOW DOWN</t>
+          <t>夏に重ねて</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>QWER</t>
+          <t>DIALOGUE+</t>
         </is>
       </c>
       <c r="I50" t="inlineStr"/>
@@ -8940,7 +8972,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>透明な夜に駆ける君と、目に見えない恋をした。</t>
+          <t>天は赤い河のほとり</t>
         </is>
       </c>
       <c r="D51" t="b">
@@ -8948,7 +8980,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F51" t="n">
@@ -8956,12 +8988,12 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>光</t>
+          <t>暁の空</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>櫻井優衣</t>
+          <t>七海ひろき</t>
         </is>
       </c>
       <c r="I51" t="inlineStr"/>
@@ -8980,7 +9012,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>トミカとトム</t>
+          <t>天幕のジャードゥーガル</t>
         </is>
       </c>
       <c r="D52" t="b">
@@ -8988,7 +9020,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>主題歌</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F52" t="n">
@@ -8996,12 +9028,12 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>きみのたからもの</t>
+          <t>Stella</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>May J.</t>
+          <t>SEKAI NO OWARI</t>
         </is>
       </c>
       <c r="I52" t="inlineStr"/>
@@ -9020,7 +9052,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>二十世紀電氣目録-ユーレカ・エヴリカ-</t>
+          <t>盗掘王</t>
         </is>
       </c>
       <c r="D53" t="b">
@@ -9036,12 +9068,12 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>ユーレカ・エヴリカ</t>
+          <t>SHOW DOWN</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>五阿弥ルナ</t>
+          <t>QWER</t>
         </is>
       </c>
       <c r="I53" t="inlineStr"/>
@@ -9060,7 +9092,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>パイの実 おしの森へようこそ！</t>
+          <t>透明な夜に駆ける君と、目に見えない恋をした。</t>
         </is>
       </c>
       <c r="D54" t="b">
@@ -9068,7 +9100,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>主題歌</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F54" t="n">
@@ -9076,12 +9108,12 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>パイしか勝たん！推しの森活</t>
+          <t>光</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>安保心結</t>
+          <t>櫻井優衣</t>
         </is>
       </c>
       <c r="I54" t="inlineStr"/>
@@ -9100,7 +9132,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>刃牙道 第1クール（TV放送）</t>
+          <t>トミカとトム</t>
         </is>
       </c>
       <c r="D55" t="b">
@@ -9108,7 +9140,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>主題歌</t>
         </is>
       </c>
       <c r="F55" t="n">
@@ -9116,12 +9148,12 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>フルボコ</t>
+          <t>きみのたからもの</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>WANIMA</t>
+          <t>May J.</t>
         </is>
       </c>
       <c r="I55" t="inlineStr"/>
@@ -9140,7 +9172,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>刃牙道 第1クール（TV放送）</t>
+          <t>二十世紀電氣目録-ユーレカ・エヴリカ-</t>
         </is>
       </c>
       <c r="D56" t="b">
@@ -9152,16 +9184,16 @@
         </is>
       </c>
       <c r="F56" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>六ノ輪</t>
+          <t>ユーレカ・エヴリカ</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>Chevon</t>
+          <t>五阿弥ルナ</t>
         </is>
       </c>
       <c r="I56" t="inlineStr"/>
@@ -9180,7 +9212,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>刃牙道 第1クール（TV放送）</t>
+          <t>パイの実 おしの森へようこそ！</t>
         </is>
       </c>
       <c r="D57" t="b">
@@ -9188,7 +9220,7 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>主題歌</t>
         </is>
       </c>
       <c r="F57" t="n">
@@ -9196,12 +9228,12 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>Mountain Top</t>
+          <t>パイしか勝たん！推しの森活</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>Novel Core</t>
+          <t>安保心結</t>
         </is>
       </c>
       <c r="I57" t="inlineStr"/>
@@ -9228,20 +9260,20 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F58" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>KATANA</t>
+          <t>フルボコ</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>三代目 J SOUL BROTHERS</t>
+          <t>WANIMA</t>
         </is>
       </c>
       <c r="I58" t="inlineStr"/>
@@ -9260,7 +9292,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>刃牙道 第2クール</t>
+          <t>刃牙道 第1クール（TV放送）</t>
         </is>
       </c>
       <c r="D59" t="b">
@@ -9272,16 +9304,16 @@
         </is>
       </c>
       <c r="F59" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>フルボコ</t>
+          <t>六ノ輪</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>WANIMA</t>
+          <t>Chevon</t>
         </is>
       </c>
       <c r="I59" t="inlineStr"/>
@@ -9300,7 +9332,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>刃牙道 第2クール</t>
+          <t>刃牙道 第1クール（TV放送）</t>
         </is>
       </c>
       <c r="D60" t="b">
@@ -9308,20 +9340,20 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F60" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>六ノ輪</t>
+          <t>Mountain Top</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>Chevon</t>
+          <t>Novel Core</t>
         </is>
       </c>
       <c r="I60" t="inlineStr"/>
@@ -9340,7 +9372,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>刃牙道 第2クール</t>
+          <t>刃牙道 第1クール（TV放送）</t>
         </is>
       </c>
       <c r="D61" t="b">
@@ -9352,16 +9384,16 @@
         </is>
       </c>
       <c r="F61" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>Mountain Top</t>
+          <t>KATANA</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>Novel Core</t>
+          <t>三代目 J SOUL BROTHERS</t>
         </is>
       </c>
       <c r="I61" t="inlineStr"/>
@@ -9388,20 +9420,20 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F62" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>KATANA</t>
+          <t>フルボコ</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>三代目 J SOUL BROTHERS</t>
+          <t>WANIMA</t>
         </is>
       </c>
       <c r="I62" t="inlineStr"/>
@@ -9420,7 +9452,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>花ざかりの君たちへ 第2期</t>
+          <t>刃牙道 第2クール</t>
         </is>
       </c>
       <c r="D63" t="b">
@@ -9432,16 +9464,16 @@
         </is>
       </c>
       <c r="F63" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>FLASHBULB</t>
+          <t>六ノ輪</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>Omoinotake</t>
+          <t>Chevon</t>
         </is>
       </c>
       <c r="I63" t="inlineStr"/>
@@ -9460,7 +9492,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>花ざかりの君たちへ 第2期</t>
+          <t>刃牙道 第2クール</t>
         </is>
       </c>
       <c r="D64" t="b">
@@ -9476,12 +9508,12 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>花束</t>
+          <t>Mountain Top</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>Omoinotake</t>
+          <t>Novel Core</t>
         </is>
       </c>
       <c r="I64" t="inlineStr"/>
@@ -9500,7 +9532,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>ヒロイン？聖女？いいえ、オールワークスメイドです（誇）！</t>
+          <t>刃牙道 第2クール</t>
         </is>
       </c>
       <c r="D65" t="b">
@@ -9508,20 +9540,20 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F65" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>マデュアル↔ハート</t>
+          <t>KATANA</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>メロディ・ウェーブ(CV：宮本侑芽) ルシアナ・ルトルバーグ(CV：大久保瑠美)</t>
+          <t>三代目 J SOUL BROTHERS</t>
         </is>
       </c>
       <c r="I65" t="inlineStr"/>
@@ -9540,7 +9572,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>ヒロイン？聖女？いいえ、オールワークスメイドです（誇）！</t>
+          <t>花ざかりの君たちへ 第2期</t>
         </is>
       </c>
       <c r="D66" t="b">
@@ -9548,7 +9580,7 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F66" t="n">
@@ -9556,12 +9588,12 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>ハンドメイド</t>
+          <t>FLASHBULB</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>仲村宗悟</t>
+          <t>Omoinotake</t>
         </is>
       </c>
       <c r="I66" t="inlineStr"/>
@@ -9580,7 +9612,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>ブチ切れ令嬢は報復を誓いました。 ～魔導書の力で祖国を叩き潰します～</t>
+          <t>花ざかりの君たちへ 第2期</t>
         </is>
       </c>
       <c r="D67" t="b">
@@ -9588,7 +9620,7 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F67" t="n">
@@ -9596,12 +9628,12 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>Q.E.D.</t>
+          <t>花束</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>小倉唯</t>
+          <t>Omoinotake</t>
         </is>
       </c>
       <c r="I67" t="inlineStr"/>
@@ -9620,7 +9652,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>ブチ切れ令嬢は報復を誓いました。 ～魔導書の力で祖国を叩き潰します～</t>
+          <t>ヒロイン？聖女？いいえ、オールワークスメイドです（誇）！</t>
         </is>
       </c>
       <c r="D68" t="b">
@@ -9628,7 +9660,7 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F68" t="n">
@@ -9636,12 +9668,12 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>グッバイ・ララバイ</t>
+          <t>マデュアル↔ハート</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>大西亜玖璃</t>
+          <t>メロディ・ウェーブ(CV：宮本侑芽) ルシアナ・ルトルバーグ(CV：大久保瑠美)</t>
         </is>
       </c>
       <c r="I68" t="inlineStr"/>
@@ -9660,7 +9692,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>BLACK TORCH</t>
+          <t>ヒロイン？聖女？いいえ、オールワークスメイドです（誇）！</t>
         </is>
       </c>
       <c r="D69" t="b">
@@ -9668,7 +9700,7 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F69" t="n">
@@ -9676,12 +9708,12 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>FREEZE ME UP</t>
+          <t>ハンドメイド</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>SiM</t>
+          <t>仲村宗悟</t>
         </is>
       </c>
       <c r="I69" t="inlineStr"/>
@@ -9700,7 +9732,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>BLACK TORCH</t>
+          <t>ブチ切れ令嬢は報復を誓いました。 ～魔導書の力で祖国を叩き潰します～</t>
         </is>
       </c>
       <c r="D70" t="b">
@@ -9708,7 +9740,7 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F70" t="n">
@@ -9716,12 +9748,12 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>Groooovy</t>
+          <t>Q.E.D.</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>I Don't Like Mondays.</t>
+          <t>小倉唯</t>
         </is>
       </c>
       <c r="I70" t="inlineStr"/>
@@ -9740,7 +9772,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>プラノサウルス ガチコセイブツ部</t>
+          <t>ブチ切れ令嬢は報復を誓いました。 ～魔導書の力で祖国を叩き潰します～</t>
         </is>
       </c>
       <c r="D71" t="b">
@@ -9748,7 +9780,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>主題歌</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F71" t="n">
@@ -9756,12 +9788,12 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>ガチde古生</t>
+          <t>グッバイ・ララバイ</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>リンクルプラネット</t>
+          <t>大西亜玖璃</t>
         </is>
       </c>
       <c r="I71" t="inlineStr"/>
@@ -9780,7 +9812,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>ヘルモード ～やり込み好きのゲーマーは廃設定の異世界で無双する～ 2nd Season</t>
+          <t>ふつつかな悪女ではございますが～雛宮蝶鼠とりかえ伝～</t>
         </is>
       </c>
       <c r="D72" t="b">
@@ -9796,12 +9828,12 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>○✕△□</t>
+          <t>Sunny</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>浪漫派マシュマロ</t>
+          <t>milet</t>
         </is>
       </c>
       <c r="I72" t="inlineStr"/>
@@ -9820,7 +9852,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>炎の闘球女 ドッジ弾子</t>
+          <t>BLACK TORCH</t>
         </is>
       </c>
       <c r="D73" t="b">
@@ -9836,12 +9868,12 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>会心の一劇</t>
+          <t>FREEZE ME UP</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>ももいろクローバーZ</t>
+          <t>SiM</t>
         </is>
       </c>
       <c r="I73" t="inlineStr"/>
@@ -9860,7 +9892,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>炎の闘球女 ドッジ弾子</t>
+          <t>BLACK TORCH</t>
         </is>
       </c>
       <c r="D74" t="b">
@@ -9876,12 +9908,12 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>Welcome to あざとさワールド</t>
+          <t>Groooovy</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>i☆Ris</t>
+          <t>I Don't Like Mondays.</t>
         </is>
       </c>
       <c r="I74" t="inlineStr"/>
@@ -9900,7 +9932,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>魔法少女リリカルなのは EXCEEDS Gun Blaze Vengeance</t>
+          <t>プラノサウルス ガチコセイブツ部</t>
         </is>
       </c>
       <c r="D75" t="b">
@@ -9908,7 +9940,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>主題歌</t>
         </is>
       </c>
       <c r="F75" t="n">
@@ -9916,12 +9948,12 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>CRIMSON BULLET</t>
+          <t>ガチde古生</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>水樹奈々</t>
+          <t>リンクルプラネット</t>
         </is>
       </c>
       <c r="I75" t="inlineStr"/>
@@ -9940,7 +9972,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>魔法少女リリカルなのは EXCEEDS Gun Blaze Vengeance</t>
+          <t>ヘルモード ～やり込み好きのゲーマーは廃設定の異世界で無双する～ 2nd Season</t>
         </is>
       </c>
       <c r="D76" t="b">
@@ -9948,7 +9980,7 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F76" t="n">
@@ -9956,12 +9988,12 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>Ephemeral</t>
+          <t>○✕△□</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>青木陽菜</t>
+          <t>浪漫派マシュマロ</t>
         </is>
       </c>
       <c r="I76" t="inlineStr"/>
@@ -9980,7 +10012,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>無自覚聖女は今日も無意識に力を垂れ流す</t>
+          <t>炎の闘球女 ドッジ弾子</t>
         </is>
       </c>
       <c r="D77" t="b">
@@ -9996,12 +10028,12 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>Windmaker</t>
+          <t>会心の一劇</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>花耶</t>
+          <t>ももいろクローバーZ</t>
         </is>
       </c>
       <c r="I77" t="inlineStr"/>
@@ -10020,7 +10052,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>無自覚聖女は今日も無意識に力を垂れ流す</t>
+          <t>炎の闘球女 ドッジ弾子</t>
         </is>
       </c>
       <c r="D78" t="b">
@@ -10036,12 +10068,12 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>アンノウンミー</t>
+          <t>Welcome to あざとさワールド</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>ウタヒメドリーム オールスターズ【夢咲いぶき（CV:山﨑玲奈） 桜木舞華（CV:鈴木杏奈） 真白清美（CV:其原有沙） HiREN（CV:花耶） 水月ひかり（CV:礒部花凜） 高木凛（CV:鷲見友美ジェナ） 萩原ひまわり（CV:倉知玲鳳） SAKURAKO（CV:竹内夢）】</t>
+          <t>i☆Ris</t>
         </is>
       </c>
       <c r="I78" t="inlineStr"/>
@@ -10060,7 +10092,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>無職転生Ⅲ ～異世界行ったら本気だす～</t>
+          <t>魔法少女リリカルなのは EXCEEDS Gun Blaze Vengeance</t>
         </is>
       </c>
       <c r="D79" t="b">
@@ -10076,12 +10108,12 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>決意の唄</t>
+          <t>CRIMSON BULLET</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>大原ゆい子</t>
+          <t>水樹奈々</t>
         </is>
       </c>
       <c r="I79" t="inlineStr"/>
@@ -10100,7 +10132,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>無職転生Ⅲ ～異世界行ったら本気だす～</t>
+          <t>魔法少女リリカルなのは EXCEEDS Gun Blaze Vengeance</t>
         </is>
       </c>
       <c r="D80" t="b">
@@ -10116,12 +10148,12 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>祈り、終われば</t>
+          <t>Ephemeral</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>中島美嘉</t>
+          <t>青木陽菜</t>
         </is>
       </c>
       <c r="I80" t="inlineStr"/>
@@ -10140,7 +10172,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>メビウス・ダスト</t>
+          <t>無自覚聖女は今日も無意識に力を垂れ流す</t>
         </is>
       </c>
       <c r="D81" t="b">
@@ -10156,12 +10188,12 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>メビウス</t>
+          <t>Windmaker</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>家入レオ</t>
+          <t>花耶</t>
         </is>
       </c>
       <c r="I81" t="inlineStr"/>
@@ -10180,7 +10212,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>メビウス・ダスト</t>
+          <t>無自覚聖女は今日も無意識に力を垂れ流す</t>
         </is>
       </c>
       <c r="D82" t="b">
@@ -10196,12 +10228,12 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>ジレンマ</t>
+          <t>アンノウンミー</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>冨岡愛</t>
+          <t>ウタヒメドリーム オールスターズ【夢咲いぶき（CV:山﨑玲奈） 桜木舞華（CV:鈴木杏奈） 真白清美（CV:其原有沙） HiREN（CV:花耶） 水月ひかり（CV:礒部花凜） 高木凛（CV:鷲見友美ジェナ） 萩原ひまわり（CV:倉知玲鳳） SAKURAKO（CV:竹内夢）】</t>
         </is>
       </c>
       <c r="I82" t="inlineStr"/>
@@ -10220,7 +10252,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>ヤニねこ</t>
+          <t>無職転生Ⅲ ～異世界行ったら本気だす～</t>
         </is>
       </c>
       <c r="D83" t="b">
@@ -10236,12 +10268,12 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>なんもねえ</t>
+          <t>決意の唄</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>忘れらんねえよ</t>
+          <t>大原ゆい子</t>
         </is>
       </c>
       <c r="I83" t="inlineStr"/>
@@ -10260,7 +10292,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>幼女戦記Ⅱ</t>
+          <t>無職転生Ⅲ ～異世界行ったら本気だす～</t>
         </is>
       </c>
       <c r="D84" t="b">
@@ -10268,7 +10300,7 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F84" t="n">
@@ -10276,12 +10308,12 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>Why? RED induction</t>
+          <t>祈り、終われば</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>MYTH &amp; ROID</t>
+          <t>中島美嘉</t>
         </is>
       </c>
       <c r="I84" t="inlineStr"/>
@@ -10300,7 +10332,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>幼女戦記Ⅱ</t>
+          <t>メビウス・ダスト</t>
         </is>
       </c>
       <c r="D85" t="b">
@@ -10308,7 +10340,7 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F85" t="n">
@@ -10316,12 +10348,12 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>Weiter! Weiter!</t>
+          <t>メビウス</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>ターニャ・デグレチャフ（CV：悠木碧）</t>
+          <t>家入レオ</t>
         </is>
       </c>
       <c r="I85" t="inlineStr"/>
@@ -10340,7 +10372,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>鎧真伝サムライトルーパー 第2クール</t>
+          <t>メビウス・ダスト</t>
         </is>
       </c>
       <c r="D86" t="b">
@@ -10348,7 +10380,7 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F86" t="n">
@@ -10356,12 +10388,12 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>YOAKE</t>
+          <t>ジレンマ</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>blank paper</t>
+          <t>冨岡愛</t>
         </is>
       </c>
       <c r="I86" t="inlineStr"/>
@@ -10380,7 +10412,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>鎧真伝サムライトルーパー 第2クール</t>
+          <t>ヤニねこ</t>
         </is>
       </c>
       <c r="D87" t="b">
@@ -10392,16 +10424,16 @@
         </is>
       </c>
       <c r="F87" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>BAD遺伝子</t>
+          <t>なんもねえ</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>Dannie May</t>
+          <t>忘れらんねえよ</t>
         </is>
       </c>
       <c r="I87" t="inlineStr"/>
@@ -10420,7 +10452,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>鎧真伝サムライトルーパー 第2クール</t>
+          <t>幼女戦記Ⅱ</t>
         </is>
       </c>
       <c r="D88" t="b">
@@ -10428,7 +10460,7 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F88" t="n">
@@ -10436,12 +10468,12 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>POWER</t>
+          <t>Why? RED induction</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>ONE OR EIGHT</t>
+          <t>MYTH &amp; ROID</t>
         </is>
       </c>
       <c r="I88" t="inlineStr"/>
@@ -10460,7 +10492,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>鎧真伝サムライトルーパー 第2クール</t>
+          <t>幼女戦記Ⅱ</t>
         </is>
       </c>
       <c r="D89" t="b">
@@ -10472,16 +10504,16 @@
         </is>
       </c>
       <c r="F89" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>ばけもん</t>
+          <t>Weiter! Weiter!</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>カラノア</t>
+          <t>ターニャ・デグレチャフ（CV：悠木碧）</t>
         </is>
       </c>
       <c r="I89" t="inlineStr"/>
@@ -10500,7 +10532,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>落第賢者の学院無双～二度目の転生、Sランクチート魔術師冒険録～</t>
+          <t>鎧真伝サムライトルーパー 第2クール</t>
         </is>
       </c>
       <c r="D90" t="b">
@@ -10516,12 +10548,12 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>＋ENCOUNT</t>
+          <t>YOAKE</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>FLOW</t>
+          <t>blank paper</t>
         </is>
       </c>
       <c r="I90" t="inlineStr"/>
@@ -10540,7 +10572,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>落第賢者の学院無双～二度目の転生、Sランクチート魔術師冒険録～</t>
+          <t>鎧真伝サムライトルーパー 第2クール</t>
         </is>
       </c>
       <c r="D91" t="b">
@@ -10548,20 +10580,20 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F91" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>憧憬</t>
+          <t>BAD遺伝子</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>TrySail</t>
+          <t>Dannie May</t>
         </is>
       </c>
       <c r="I91" t="inlineStr"/>
@@ -10580,7 +10612,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>領民0人スタートの辺境領主様</t>
+          <t>鎧真伝サムライトルーパー 第2クール</t>
         </is>
       </c>
       <c r="D92" t="b">
@@ -10588,7 +10620,7 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F92" t="n">
@@ -10596,12 +10628,12 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>Wonder</t>
+          <t>POWER</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>CROWN HEAD</t>
+          <t>ONE OR EIGHT</t>
         </is>
       </c>
       <c r="I92" t="inlineStr"/>
@@ -10620,7 +10652,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>領民0人スタートの辺境領主様</t>
+          <t>鎧真伝サムライトルーパー 第2クール</t>
         </is>
       </c>
       <c r="D93" t="b">
@@ -10632,16 +10664,16 @@
         </is>
       </c>
       <c r="F93" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>星降る夜の約束</t>
+          <t>ばけもん</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>花耶</t>
+          <t>カラノア</t>
         </is>
       </c>
       <c r="I93" t="inlineStr"/>
@@ -10660,7 +10692,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>令和のダラさん</t>
+          <t>落第賢者の学院無双～二度目の転生、Sランクチート魔術師冒険録～</t>
         </is>
       </c>
       <c r="D94" t="b">
@@ -10676,12 +10708,12 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>ダラダラ♡ダンシング</t>
+          <t>＋ENCOUNT</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>ダラさん（CV：田村睦心） 三⼗⽊⾕⽇向（CV：津田美波） 三⼗⽊⾕薫（CV：寺澤百花） ナレーション（CV：てらそままさき）</t>
+          <t>FLOW</t>
         </is>
       </c>
       <c r="I94" t="inlineStr"/>
@@ -10700,7 +10732,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>令和のダラさん</t>
+          <t>落第賢者の学院無双～二度目の転生、Sランクチート魔術師冒険録～</t>
         </is>
       </c>
       <c r="D95" t="b">
@@ -10716,12 +10748,12 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>ひなたぼっこ</t>
+          <t>憧憬</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>REIRIE</t>
+          <t>TrySail</t>
         </is>
       </c>
       <c r="I95" t="inlineStr"/>
@@ -10740,7 +10772,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>LV999の村人</t>
+          <t>領民0人スタートの辺境領主様</t>
         </is>
       </c>
       <c r="D96" t="b">
@@ -10756,12 +10788,12 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>Not a Hero</t>
+          <t>Wonder</t>
         </is>
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>藍月なくる&amp;棗いつき</t>
+          <t>CROWN HEAD</t>
         </is>
       </c>
       <c r="I96" t="inlineStr"/>
@@ -10780,7 +10812,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>LV999の村人</t>
+          <t>領民0人スタートの辺境領主様</t>
         </is>
       </c>
       <c r="D97" t="b">
@@ -10796,12 +10828,12 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>星降る夜の約束</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>ゆきむら。</t>
+          <t>花耶</t>
         </is>
       </c>
       <c r="I97" t="inlineStr"/>
@@ -10820,7 +10852,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>ワールド イズ ダンシング</t>
+          <t>令和のダラさん</t>
         </is>
       </c>
       <c r="D98" t="b">
@@ -10836,12 +10868,12 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>終宵</t>
+          <t>ダラダラ♡ダンシング</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>マカロニえんぴつ</t>
+          <t>ダラさん（CV：田村睦心） 三⼗⽊⾕⽇向（CV：津田美波） 三⼗⽊⾕薫（CV：寺澤百花） ナレーション（CV：てらそままさき）</t>
         </is>
       </c>
       <c r="I98" t="inlineStr"/>
@@ -10851,16 +10883,16 @@
     </row>
     <row r="99">
       <c r="A99" t="n">
-        <v>5947</v>
+        <v>5806</v>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>2026秋アニメ</t>
+          <t>2026夏アニメ</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>帰還者の魔法は特別です 第2期</t>
+          <t>令和のダラさん</t>
         </is>
       </c>
       <c r="D99" t="b">
@@ -10868,7 +10900,7 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F99" t="n">
@@ -10876,12 +10908,12 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>Sorrow</t>
+          <t>ひなたぼっこ</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>FLOW</t>
+          <t>REIRIE</t>
         </is>
       </c>
       <c r="I99" t="inlineStr"/>
@@ -10891,16 +10923,16 @@
     </row>
     <row r="100">
       <c r="A100" t="n">
-        <v>5947</v>
+        <v>5806</v>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>2026秋アニメ</t>
+          <t>2026夏アニメ</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>獣王武神ダンデヴァイン</t>
+          <t>LV999の村人</t>
         </is>
       </c>
       <c r="D100" t="b">
@@ -10916,12 +10948,12 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>曲名未発表</t>
+          <t>Not a Hero</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>西川貴教</t>
+          <t>藍月なくる&amp;棗いつき</t>
         </is>
       </c>
       <c r="I100" t="inlineStr"/>
@@ -10931,16 +10963,16 @@
     </row>
     <row r="101">
       <c r="A101" t="n">
-        <v>5947</v>
+        <v>5806</v>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>2026秋アニメ</t>
+          <t>2026夏アニメ</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>転生した大聖女は、聖女であることをひた隠す</t>
+          <t>LV999の村人</t>
         </is>
       </c>
       <c r="D101" t="b">
@@ -10948,7 +10980,7 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F101" t="n">
@@ -10956,12 +10988,12 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>Flare of Soul</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>花耶</t>
+          <t>ゆきむら。</t>
         </is>
       </c>
       <c r="I101" t="inlineStr"/>
@@ -10971,16 +11003,16 @@
     </row>
     <row r="102">
       <c r="A102" t="n">
-        <v>5947</v>
+        <v>5806</v>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>2026秋アニメ</t>
+          <t>2026夏アニメ</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>転生した大聖女は、聖女であることをひた隠す</t>
+          <t>ワールド イズ ダンシング</t>
         </is>
       </c>
       <c r="D102" t="b">
@@ -10988,7 +11020,7 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F102" t="n">
@@ -10996,12 +11028,12 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>STELLAR</t>
+          <t>終宵</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>ウタヒメドリーム オールスターズ</t>
+          <t>マカロニえんぴつ</t>
         </is>
       </c>
       <c r="I102" t="inlineStr"/>
@@ -11020,7 +11052,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>魔法少女育成計画restart</t>
+          <t>帰還者の魔法は特別です 第2期</t>
         </is>
       </c>
       <c r="D103" t="b">
@@ -11036,12 +11068,12 @@
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>No tears here</t>
+          <t>Sorrow</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>茅原実里</t>
+          <t>FLOW</t>
         </is>
       </c>
       <c r="I103" t="inlineStr"/>
@@ -11049,6 +11081,166 @@
       <c r="K103" t="inlineStr"/>
       <c r="L103" t="inlineStr"/>
     </row>
+    <row r="104">
+      <c r="A104" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>獣王武神ダンデヴァイン</t>
+        </is>
+      </c>
+      <c r="D104" t="b">
+        <v>0</v>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="F104" t="n">
+        <v>1</v>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>曲名未発表</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>西川貴教</t>
+        </is>
+      </c>
+      <c r="I104" t="inlineStr"/>
+      <c r="J104" t="inlineStr"/>
+      <c r="K104" t="inlineStr"/>
+      <c r="L104" t="inlineStr"/>
+    </row>
+    <row r="105">
+      <c r="A105" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>転生した大聖女は、聖女であることをひた隠す</t>
+        </is>
+      </c>
+      <c r="D105" t="b">
+        <v>0</v>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="F105" t="n">
+        <v>1</v>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>Flare of Soul</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>花耶</t>
+        </is>
+      </c>
+      <c r="I105" t="inlineStr"/>
+      <c r="J105" t="inlineStr"/>
+      <c r="K105" t="inlineStr"/>
+      <c r="L105" t="inlineStr"/>
+    </row>
+    <row r="106">
+      <c r="A106" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>転生した大聖女は、聖女であることをひた隠す</t>
+        </is>
+      </c>
+      <c r="D106" t="b">
+        <v>0</v>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>ED</t>
+        </is>
+      </c>
+      <c r="F106" t="n">
+        <v>1</v>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>STELLAR</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>ウタヒメドリーム オールスターズ</t>
+        </is>
+      </c>
+      <c r="I106" t="inlineStr"/>
+      <c r="J106" t="inlineStr"/>
+      <c r="K106" t="inlineStr"/>
+      <c r="L106" t="inlineStr"/>
+    </row>
+    <row r="107">
+      <c r="A107" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>魔法少女育成計画restart</t>
+        </is>
+      </c>
+      <c r="D107" t="b">
+        <v>0</v>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="F107" t="n">
+        <v>1</v>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>No tears here</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>茅原実里</t>
+        </is>
+      </c>
+      <c r="I107" t="inlineStr"/>
+      <c r="J107" t="inlineStr"/>
+      <c r="K107" t="inlineStr"/>
+      <c r="L107" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
auto: anime list update 2026-06-11
</commit_message>
<xml_diff>
--- a/data/anime_list.xlsx
+++ b/data/anime_list.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M130"/>
+  <dimension ref="A1:M131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1084,8 +1084,16 @@
           <t>ユニコーン</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>BLUE ENCOUNT</t>
+        </is>
+      </c>
       <c r="M13" t="inlineStr">
         <is>
           <t>https://www.animatetimes.com/tag/details.php?id=26271</t>
@@ -2786,8 +2794,16 @@
           <t>マカリア</t>
         </is>
       </c>
-      <c r="I45" t="inlineStr"/>
-      <c r="J45" t="inlineStr"/>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>ひとひら</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>秦基博</t>
+        </is>
+      </c>
       <c r="K45" t="inlineStr">
         <is>
           <t>光</t>
@@ -3080,11 +3096,11 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>刃牙道 第1クール（TV放送）</t>
+          <t>刃牙道 第2クール</t>
         </is>
       </c>
       <c r="E52" t="b">
@@ -3141,11 +3157,11 @@
         </is>
       </c>
       <c r="C53" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>刃牙道 第2クール</t>
+          <t>花織さんは転生しても喧嘩がしたい</t>
         </is>
       </c>
       <c r="E53" t="b">
@@ -3153,42 +3169,26 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>配信</t>
+          <t>TVアニメ</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>第1クール：2026年2月26日（木）〜 第2クール：2026年6月18日（木）～ Netflixにて 【TV放送】 第1クール：2026年7月5日（日）～ TOKYO MXほか</t>
+          <t>2026年7月11日（土）～ ABCテレビ・テレビ朝日系・BS日テレにて</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>トムス・エンタテインメント</t>
-        </is>
-      </c>
-      <c r="I53" t="inlineStr">
-        <is>
-          <t>フルボコ</t>
-        </is>
-      </c>
-      <c r="J53" t="inlineStr">
-        <is>
-          <t>WANIMA</t>
-        </is>
-      </c>
-      <c r="K53" t="inlineStr">
-        <is>
-          <t>Mountain Top</t>
-        </is>
-      </c>
-      <c r="L53" t="inlineStr">
-        <is>
-          <t>Novel Core</t>
-        </is>
-      </c>
+          <t>ライデンフィルム</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr"/>
+      <c r="J53" t="inlineStr"/>
+      <c r="K53" t="inlineStr"/>
+      <c r="L53" t="inlineStr"/>
       <c r="M53" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=23828</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26828</t>
         </is>
       </c>
     </row>
@@ -3202,11 +3202,11 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>花織さんは転生しても喧嘩がしたい</t>
+          <t>花ざかりの君たちへ 第2期</t>
         </is>
       </c>
       <c r="E54" t="b">
@@ -3219,21 +3219,37 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>2026年7月11日（土）～ ABCテレビ・テレビ朝日系・BS日テレにて</t>
+          <t>2026年7月1日（水）～ TOKYO MX・BS11ほか</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>ライデンフィルム</t>
-        </is>
-      </c>
-      <c r="I54" t="inlineStr"/>
-      <c r="J54" t="inlineStr"/>
-      <c r="K54" t="inlineStr"/>
-      <c r="L54" t="inlineStr"/>
+          <t>シグナル・エムディ（</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>FLASHBULB</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>Omoinotake</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>花束</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>Omoinotake</t>
+        </is>
+      </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26828</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27990</t>
         </is>
       </c>
     </row>
@@ -3247,11 +3263,11 @@
         </is>
       </c>
       <c r="C55" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>花ざかりの君たちへ 第2期</t>
+          <t>バンドリ！ ゆめ∞みた</t>
         </is>
       </c>
       <c r="E55" t="b">
@@ -3264,37 +3280,21 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>2026年7月1日（水）～ TOKYO MX・BS11ほか</t>
+          <t>2026年7月2日（木）～ TOKYO MXほか</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>シグナル・エムディ（</t>
-        </is>
-      </c>
-      <c r="I55" t="inlineStr">
-        <is>
-          <t>FLASHBULB</t>
-        </is>
-      </c>
-      <c r="J55" t="inlineStr">
-        <is>
-          <t>Omoinotake</t>
-        </is>
-      </c>
-      <c r="K55" t="inlineStr">
-        <is>
-          <t>花束</t>
-        </is>
-      </c>
-      <c r="L55" t="inlineStr">
-        <is>
-          <t>Omoinotake</t>
-        </is>
-      </c>
+          <t>ニチカライン（</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr"/>
+      <c r="J55" t="inlineStr"/>
+      <c r="K55" t="inlineStr"/>
+      <c r="L55" t="inlineStr"/>
       <c r="M55" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27990</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26737</t>
         </is>
       </c>
     </row>
@@ -3308,11 +3308,11 @@
         </is>
       </c>
       <c r="C56" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>バンドリ！ ゆめ∞みた</t>
+          <t>パンの赤ちゃん</t>
         </is>
       </c>
       <c r="E56" t="b">
@@ -3325,21 +3325,17 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>2026年7月2日（木）～ TOKYO MXほか</t>
-        </is>
-      </c>
-      <c r="H56" t="inlineStr">
-        <is>
-          <t>ニチカライン（</t>
-        </is>
-      </c>
+          <t>2026年7月4日（土）～ カンテレ・フジテレビ系列「土曜はナニする！？」にて</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr"/>
       <c r="I56" t="inlineStr"/>
       <c r="J56" t="inlineStr"/>
       <c r="K56" t="inlineStr"/>
       <c r="L56" t="inlineStr"/>
       <c r="M56" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26737</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25145</t>
         </is>
       </c>
     </row>
@@ -3353,11 +3349,11 @@
         </is>
       </c>
       <c r="C57" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>パンの赤ちゃん</t>
+          <t>ヒロイン？聖女？いいえ、オールワークスメイドです（誇）！</t>
         </is>
       </c>
       <c r="E57" t="b">
@@ -3370,17 +3366,37 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>2026年7月4日（土）～ カンテレ・フジテレビ系列「土曜はナニする！？」にて</t>
-        </is>
-      </c>
-      <c r="H57" t="inlineStr"/>
-      <c r="I57" t="inlineStr"/>
-      <c r="J57" t="inlineStr"/>
-      <c r="K57" t="inlineStr"/>
-      <c r="L57" t="inlineStr"/>
+          <t>2026年7月1日（水）～ TOKYO MX・BSフジほか</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>EMTスクエアード</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>マデュアル↔ハート</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>メロディ・ウェーブ(CV：宮本侑芽) ルシアナ・ルトルバーグ(CV：大久保瑠美)</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>ハンドメイド</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>仲村宗悟</t>
+        </is>
+      </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25145</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25936</t>
         </is>
       </c>
     </row>
@@ -3394,11 +3410,11 @@
         </is>
       </c>
       <c r="C58" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>ヒロイン？聖女？いいえ、オールワークスメイドです（誇）！</t>
+          <t>ブチ切れ令嬢は報復を誓いました。 ～魔導書の力で祖国を叩き潰します～</t>
         </is>
       </c>
       <c r="E58" t="b">
@@ -3411,37 +3427,37 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>2026年7月1日（水）～ TOKYO MX・BSフジほか</t>
+          <t>2026年7月6日（月）〜 テレ東・BS11ほか</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>EMTスクエアード</t>
+          <t>スタジオコメット</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>マデュアル↔ハート</t>
+          <t>Q.E.D.</t>
         </is>
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>メロディ・ウェーブ(CV：宮本侑芽) ルシアナ・ルトルバーグ(CV：大久保瑠美)</t>
+          <t>小倉唯</t>
         </is>
       </c>
       <c r="K58" t="inlineStr">
         <is>
-          <t>ハンドメイド</t>
+          <t>グッバイ・ララバイ</t>
         </is>
       </c>
       <c r="L58" t="inlineStr">
         <is>
-          <t>仲村宗悟</t>
+          <t>大西亜玖璃</t>
         </is>
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25936</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27366</t>
         </is>
       </c>
     </row>
@@ -3455,11 +3471,11 @@
         </is>
       </c>
       <c r="C59" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>ブチ切れ令嬢は報復を誓いました。 ～魔導書の力で祖国を叩き潰します～</t>
+          <t>ふつつかな悪女ではございますが～雛宮蝶鼠とりかえ伝～</t>
         </is>
       </c>
       <c r="E59" t="b">
@@ -3472,37 +3488,29 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>2026年7月6日（月）〜 テレ東・BS11ほか</t>
+          <t>2026年7月12日（日）〜 テレビ東京系列にて</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>スタジオコメット</t>
+          <t>動画工房</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>Q.E.D.</t>
+          <t>Sunny</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>小倉唯</t>
-        </is>
-      </c>
-      <c r="K59" t="inlineStr">
-        <is>
-          <t>グッバイ・ララバイ</t>
-        </is>
-      </c>
-      <c r="L59" t="inlineStr">
-        <is>
-          <t>大西亜玖璃</t>
-        </is>
-      </c>
+          <t>milet</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr"/>
+      <c r="L59" t="inlineStr"/>
       <c r="M59" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27366</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25702</t>
         </is>
       </c>
     </row>
@@ -3516,11 +3524,11 @@
         </is>
       </c>
       <c r="C60" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>ふつつかな悪女ではございますが～雛宮蝶鼠とりかえ伝～</t>
+          <t>BLACK TORCH</t>
         </is>
       </c>
       <c r="E60" t="b">
@@ -3533,29 +3541,37 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>2026年7月12日（日）〜 テレビ東京系列にて</t>
+          <t>2026年7月4日（土）～ TOKYO MXほか</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>動画工房</t>
+          <t>100studio</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>Sunny</t>
+          <t>FREEZE ME UP</t>
         </is>
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>milet</t>
-        </is>
-      </c>
-      <c r="K60" t="inlineStr"/>
-      <c r="L60" t="inlineStr"/>
+          <t>SiM</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>Groooovy</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>I Don't Like Mondays.</t>
+        </is>
+      </c>
       <c r="M60" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25702</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25641</t>
         </is>
       </c>
     </row>
@@ -3569,11 +3585,11 @@
         </is>
       </c>
       <c r="C61" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>BLACK TORCH</t>
+          <t>プラノサウルス ガチコセイブツ部</t>
         </is>
       </c>
       <c r="E61" t="b">
@@ -3586,37 +3602,21 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>2026年7月4日（土）～ TOKYO MXほか</t>
+          <t>2026年7月～ テレ東系列6局ネット「アニもり！」内にて</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>100studio</t>
-        </is>
-      </c>
-      <c r="I61" t="inlineStr">
-        <is>
-          <t>FREEZE ME UP</t>
-        </is>
-      </c>
-      <c r="J61" t="inlineStr">
-        <is>
-          <t>SiM</t>
-        </is>
-      </c>
-      <c r="K61" t="inlineStr">
-        <is>
-          <t>Groooovy</t>
-        </is>
-      </c>
-      <c r="L61" t="inlineStr">
-        <is>
-          <t>I Don't Like Mondays.</t>
-        </is>
-      </c>
+          <t>SMDE</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr"/>
+      <c r="J61" t="inlineStr"/>
+      <c r="K61" t="inlineStr"/>
+      <c r="L61" t="inlineStr"/>
       <c r="M61" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25641</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27895</t>
         </is>
       </c>
     </row>
@@ -3630,11 +3630,11 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>プラノサウルス ガチコセイブツ部</t>
+          <t>BLEACH 千年血戦篇-禍進譚-</t>
         </is>
       </c>
       <c r="E62" t="b">
@@ -3647,12 +3647,12 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>2026年7月～ テレ東系列6局ネット「アニもり！」内にて</t>
+          <t>2026年7月～ テレ東系列ほか</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>SMDE</t>
+          <t>PIERROT FILMS（</t>
         </is>
       </c>
       <c r="I62" t="inlineStr"/>
@@ -3661,7 +3661,7 @@
       <c r="L62" t="inlineStr"/>
       <c r="M62" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27895</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25417</t>
         </is>
       </c>
     </row>
@@ -3675,11 +3675,11 @@
         </is>
       </c>
       <c r="C63" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>BLEACH 千年血戦篇-禍進譚-</t>
+          <t>文豪ストレイドッグス わん！２</t>
         </is>
       </c>
       <c r="E63" t="b">
@@ -3692,12 +3692,12 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>2026年7月～ テレ東系列ほか</t>
+          <t>2026年7月〜</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>PIERROT FILMS（</t>
+          <t>ボンズ</t>
         </is>
       </c>
       <c r="I63" t="inlineStr"/>
@@ -3706,7 +3706,7 @@
       <c r="L63" t="inlineStr"/>
       <c r="M63" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25417</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27057</t>
         </is>
       </c>
     </row>
@@ -3720,11 +3720,11 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>文豪ストレイドッグス わん！２</t>
+          <t>ヘルモード ～やり込み好きのゲーマーは廃設定の異世界で無双する～ 2nd Season</t>
         </is>
       </c>
       <c r="E64" t="b">
@@ -3737,21 +3737,29 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>2026年7月〜</t>
+          <t>2026年7月3日（金）～ TOKYO MXほか</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>ボンズ</t>
-        </is>
-      </c>
-      <c r="I64" t="inlineStr"/>
-      <c r="J64" t="inlineStr"/>
+          <t>横浜アニメーションラボ</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>○✕△□</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>浪漫派マシュマロ</t>
+        </is>
+      </c>
       <c r="K64" t="inlineStr"/>
       <c r="L64" t="inlineStr"/>
       <c r="M64" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27057</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28020</t>
         </is>
       </c>
     </row>
@@ -3765,11 +3773,11 @@
         </is>
       </c>
       <c r="C65" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>ヘルモード ～やり込み好きのゲーマーは廃設定の異世界で無双する～ 2nd Season</t>
+          <t>北斗の拳 拳王軍ザコたちの挽歌 第2クール</t>
         </is>
       </c>
       <c r="E65" t="b">
@@ -3782,29 +3790,37 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>2026年7月3日（金）～ TOKYO MXほか</t>
+          <t>第1クール：2026年1月5日（月）～2026年3月23日（月） 第2クール：2026年7月6日（月）～ AT-X・TOKYO MXにて</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>横浜アニメーションラボ</t>
+          <t>動楽</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>○✕△□</t>
+          <t>Blacker Co., Ltd.</t>
         </is>
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>浪漫派マシュマロ</t>
-        </is>
-      </c>
-      <c r="K65" t="inlineStr"/>
-      <c r="L65" t="inlineStr"/>
+          <t>イツカ▶</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>Elegy of the Enemies</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>The Canbellz</t>
+        </is>
+      </c>
       <c r="M65" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28020</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26775</t>
         </is>
       </c>
     </row>
@@ -3818,7 +3834,7 @@
         </is>
       </c>
       <c r="C66" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
@@ -3879,7 +3895,7 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
@@ -3940,7 +3956,7 @@
         </is>
       </c>
       <c r="C68" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
@@ -3985,7 +4001,7 @@
         </is>
       </c>
       <c r="C69" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D69" t="inlineStr">
         <is>
@@ -4046,7 +4062,7 @@
         </is>
       </c>
       <c r="C70" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
@@ -4103,7 +4119,7 @@
         </is>
       </c>
       <c r="C71" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
@@ -4164,7 +4180,7 @@
         </is>
       </c>
       <c r="C72" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
@@ -4217,7 +4233,7 @@
         </is>
       </c>
       <c r="C73" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
@@ -4278,7 +4294,7 @@
         </is>
       </c>
       <c r="C74" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
@@ -4339,7 +4355,7 @@
         </is>
       </c>
       <c r="C75" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
@@ -4400,7 +4416,7 @@
         </is>
       </c>
       <c r="C76" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
@@ -4461,7 +4477,7 @@
         </is>
       </c>
       <c r="C77" t="n">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
@@ -4522,7 +4538,7 @@
         </is>
       </c>
       <c r="C78" t="n">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
@@ -4567,7 +4583,7 @@
         </is>
       </c>
       <c r="C79" t="n">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
@@ -4628,7 +4644,7 @@
         </is>
       </c>
       <c r="C80" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
@@ -4681,7 +4697,7 @@
         </is>
       </c>
       <c r="C81" t="n">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D81" t="inlineStr">
         <is>
@@ -5700,7 +5716,7 @@
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>てつりょー！meet with 鉄道むすめ</t>
+          <t>追放されたチート付与魔術師は気ままなセカンドライフを謳歌する。</t>
         </is>
       </c>
       <c r="E104" t="b">
@@ -5713,12 +5729,12 @@
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>2026年秋</t>
+          <t>2026年10月～ テレ東系列にて</t>
         </is>
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>イーストフィッシュスタジオ</t>
+          <t>P.A.WORKS</t>
         </is>
       </c>
       <c r="I104" t="inlineStr"/>
@@ -5727,7 +5743,7 @@
       <c r="L104" t="inlineStr"/>
       <c r="M104" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26895</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27631</t>
         </is>
       </c>
     </row>
@@ -5745,7 +5761,7 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>テムパル～アイテムの力～</t>
+          <t>てつりょー！meet with 鉄道むすめ</t>
         </is>
       </c>
       <c r="E105" t="b">
@@ -5758,12 +5774,12 @@
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
+          <t>2026年秋</t>
         </is>
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>J.C.STAFF</t>
+          <t>イーストフィッシュスタジオ</t>
         </is>
       </c>
       <c r="I105" t="inlineStr"/>
@@ -5772,7 +5788,7 @@
       <c r="L105" t="inlineStr"/>
       <c r="M105" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28478</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26895</t>
         </is>
       </c>
     </row>
@@ -5790,7 +5806,7 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>転生貴族、鑑定スキルで成り上がる 第3期</t>
+          <t>テムパル～アイテムの力～</t>
         </is>
       </c>
       <c r="E106" t="b">
@@ -5803,12 +5819,12 @@
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>2026年秋 CBC/TBS系全国28局ネット「アガルアニメ」にて</t>
+          <t>2026年10月～</t>
         </is>
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>studio MOTHER</t>
+          <t>J.C.STAFF</t>
         </is>
       </c>
       <c r="I106" t="inlineStr"/>
@@ -5817,7 +5833,7 @@
       <c r="L106" t="inlineStr"/>
       <c r="M106" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25385</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28478</t>
         </is>
       </c>
     </row>
@@ -5835,7 +5851,7 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>転生ゴブリンだけど質問ある？</t>
+          <t>転生貴族、鑑定スキルで成り上がる 第3期</t>
         </is>
       </c>
       <c r="E107" t="b">
@@ -5848,12 +5864,12 @@
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
+          <t>2026年秋 CBC/TBS系全国28局ネット「アガルアニメ」にて</t>
         </is>
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>BAKKKA</t>
+          <t>studio MOTHER</t>
         </is>
       </c>
       <c r="I107" t="inlineStr"/>
@@ -5862,7 +5878,7 @@
       <c r="L107" t="inlineStr"/>
       <c r="M107" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27909</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25385</t>
         </is>
       </c>
     </row>
@@ -5880,7 +5896,7 @@
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>転生した大聖女は、聖女であることをひた隠す</t>
+          <t>転生ゴブリンだけど質問ある？</t>
         </is>
       </c>
       <c r="E108" t="b">
@@ -5898,32 +5914,16 @@
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>FelixFilm</t>
-        </is>
-      </c>
-      <c r="I108" t="inlineStr">
-        <is>
-          <t>Flare of Soul</t>
-        </is>
-      </c>
-      <c r="J108" t="inlineStr">
-        <is>
-          <t>花耶</t>
-        </is>
-      </c>
-      <c r="K108" t="inlineStr">
-        <is>
-          <t>STELLAR</t>
-        </is>
-      </c>
-      <c r="L108" t="inlineStr">
-        <is>
-          <t>ウタヒメドリーム オールスターズ</t>
-        </is>
-      </c>
+          <t>BAKKKA</t>
+        </is>
+      </c>
+      <c r="I108" t="inlineStr"/>
+      <c r="J108" t="inlineStr"/>
+      <c r="K108" t="inlineStr"/>
+      <c r="L108" t="inlineStr"/>
       <c r="M108" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25630</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27909</t>
         </is>
       </c>
     </row>
@@ -5941,7 +5941,7 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>転生したら剣でした 第2期</t>
+          <t>転生した大聖女は、聖女であることをひた隠す</t>
         </is>
       </c>
       <c r="E109" t="b">
@@ -5959,16 +5959,32 @@
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>C2C</t>
-        </is>
-      </c>
-      <c r="I109" t="inlineStr"/>
-      <c r="J109" t="inlineStr"/>
-      <c r="K109" t="inlineStr"/>
-      <c r="L109" t="inlineStr"/>
+          <t>FelixFilm</t>
+        </is>
+      </c>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>Flare of Soul</t>
+        </is>
+      </c>
+      <c r="J109" t="inlineStr">
+        <is>
+          <t>花耶</t>
+        </is>
+      </c>
+      <c r="K109" t="inlineStr">
+        <is>
+          <t>STELLAR</t>
+        </is>
+      </c>
+      <c r="L109" t="inlineStr">
+        <is>
+          <t>ウタヒメドリーム オールスターズ</t>
+        </is>
+      </c>
       <c r="M109" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=19149</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25630</t>
         </is>
       </c>
     </row>
@@ -5986,7 +6002,7 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>とある暗部の少女共棲</t>
+          <t>転生したら剣でした 第2期</t>
         </is>
       </c>
       <c r="E110" t="b">
@@ -5999,12 +6015,12 @@
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>2026年秋</t>
+          <t>2026年10月～</t>
         </is>
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>J.C.STAFF</t>
+          <t>C2C</t>
         </is>
       </c>
       <c r="I110" t="inlineStr"/>
@@ -6013,7 +6029,7 @@
       <c r="L110" t="inlineStr"/>
       <c r="M110" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25552</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=19149</t>
         </is>
       </c>
     </row>
@@ -6031,7 +6047,7 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>東京リベンジャーズ 三天戦争編</t>
+          <t>とある暗部の少女共棲</t>
         </is>
       </c>
       <c r="E111" t="b">
@@ -6044,12 +6060,12 @@
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
+          <t>2026年秋</t>
         </is>
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>ライデンフィルム</t>
+          <t>J.C.STAFF</t>
         </is>
       </c>
       <c r="I111" t="inlineStr"/>
@@ -6058,7 +6074,7 @@
       <c r="L111" t="inlineStr"/>
       <c r="M111" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=24207</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25552</t>
         </is>
       </c>
     </row>
@@ -6076,7 +6092,7 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>桃源暗鬼 ～日光・華厳の滝編～</t>
+          <t>東京リベンジャーズ 三天戦争編</t>
         </is>
       </c>
       <c r="E112" t="b">
@@ -6089,17 +6105,21 @@
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>2026年10月～ 日本テレビ系「FRIDAY ANIME NIGHT（フラアニ）」枠にて</t>
-        </is>
-      </c>
-      <c r="H112" t="inlineStr"/>
+          <t>2026年10月～</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>ライデンフィルム</t>
+        </is>
+      </c>
       <c r="I112" t="inlineStr"/>
       <c r="J112" t="inlineStr"/>
       <c r="K112" t="inlineStr"/>
       <c r="L112" t="inlineStr"/>
       <c r="M112" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27376</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=24207</t>
         </is>
       </c>
     </row>
@@ -6117,7 +6137,7 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>ドラゴンボール超 ビルス</t>
+          <t>桃源暗鬼 ～日光・華厳の滝編～</t>
         </is>
       </c>
       <c r="E113" t="b">
@@ -6130,7 +6150,7 @@
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>2026年秋 フジテレビにて</t>
+          <t>2026年10月～ 日本テレビ系「FRIDAY ANIME NIGHT（フラアニ）」枠にて</t>
         </is>
       </c>
       <c r="H113" t="inlineStr"/>
@@ -6140,7 +6160,7 @@
       <c r="L113" t="inlineStr"/>
       <c r="M113" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27491</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27376</t>
         </is>
       </c>
     </row>
@@ -6158,7 +6178,7 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>鳴海の平日</t>
+          <t>ドラゴンボール超 ビルス</t>
         </is>
       </c>
       <c r="E114" t="b">
@@ -6166,26 +6186,22 @@
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>配信</t>
+          <t>TVアニメ</t>
         </is>
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>2026年秋</t>
-        </is>
-      </c>
-      <c r="H114" t="inlineStr">
-        <is>
-          <t>Production I.G</t>
-        </is>
-      </c>
+          <t>2026年秋 フジテレビにて</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr"/>
       <c r="I114" t="inlineStr"/>
       <c r="J114" t="inlineStr"/>
       <c r="K114" t="inlineStr"/>
       <c r="L114" t="inlineStr"/>
       <c r="M114" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28465</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27491</t>
         </is>
       </c>
     </row>
@@ -6203,7 +6219,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>バーテックスフォース</t>
+          <t>鳴海の平日</t>
         </is>
       </c>
       <c r="E115" t="b">
@@ -6211,17 +6227,17 @@
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>TVアニメ</t>
+          <t>配信</t>
         </is>
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>2026年10月〜</t>
+          <t>2026年秋</t>
         </is>
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>SMDE</t>
+          <t>Production I.G</t>
         </is>
       </c>
       <c r="I115" t="inlineStr"/>
@@ -6230,7 +6246,7 @@
       <c r="L115" t="inlineStr"/>
       <c r="M115" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27988</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28465</t>
         </is>
       </c>
     </row>
@@ -6248,7 +6264,7 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Battle Spirits [Re] 絶界の空</t>
+          <t>バーテックスフォース</t>
         </is>
       </c>
       <c r="E116" t="b">
@@ -6261,17 +6277,21 @@
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>2026年秋</t>
-        </is>
-      </c>
-      <c r="H116" t="inlineStr"/>
+          <t>2026年10月〜</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>SMDE</t>
+        </is>
+      </c>
       <c r="I116" t="inlineStr"/>
       <c r="J116" t="inlineStr"/>
       <c r="K116" t="inlineStr"/>
       <c r="L116" t="inlineStr"/>
       <c r="M116" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27954</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27988</t>
         </is>
       </c>
     </row>
@@ -6289,7 +6309,7 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>パンどろぼう</t>
+          <t>Battle Spirits [Re] 絶界の空</t>
         </is>
       </c>
       <c r="E117" t="b">
@@ -6302,7 +6322,7 @@
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>2026年10月〜 NHK Eテレにて</t>
+          <t>2026年秋</t>
         </is>
       </c>
       <c r="H117" t="inlineStr"/>
@@ -6312,7 +6332,7 @@
       <c r="L117" t="inlineStr"/>
       <c r="M117" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26163</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27954</t>
         </is>
       </c>
     </row>
@@ -6330,7 +6350,7 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>百妖譜 京師篇</t>
+          <t>パンどろぼう</t>
         </is>
       </c>
       <c r="E118" t="b">
@@ -6343,7 +6363,7 @@
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>2026年10月〜 フジテレビ「B8station」にて</t>
+          <t>2026年10月〜 NHK Eテレにて</t>
         </is>
       </c>
       <c r="H118" t="inlineStr"/>
@@ -6353,7 +6373,7 @@
       <c r="L118" t="inlineStr"/>
       <c r="M118" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27781</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26163</t>
         </is>
       </c>
     </row>
@@ -6371,7 +6391,7 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>冰剣の魔術師が世界を統べるⅡ</t>
+          <t>百妖譜 京師篇</t>
         </is>
       </c>
       <c r="E119" t="b">
@@ -6384,21 +6404,17 @@
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>2026年10月〜</t>
-        </is>
-      </c>
-      <c r="H119" t="inlineStr">
-        <is>
-          <t>ゼロジー</t>
-        </is>
-      </c>
+          <t>2026年10月〜 フジテレビ「B8station」にて</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr"/>
       <c r="I119" t="inlineStr"/>
       <c r="J119" t="inlineStr"/>
       <c r="K119" t="inlineStr"/>
       <c r="L119" t="inlineStr"/>
       <c r="M119" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28403</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27781</t>
         </is>
       </c>
     </row>
@@ -6416,7 +6432,7 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>ホタルの嫁入り</t>
+          <t>冰剣の魔術師が世界を統べるⅡ</t>
         </is>
       </c>
       <c r="E120" t="b">
@@ -6429,12 +6445,12 @@
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>2026年10月～ 全国フジテレビ系“ ノイタミナ ”にて</t>
+          <t>2026年10月〜</t>
         </is>
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>david production</t>
+          <t>ゼロジー</t>
         </is>
       </c>
       <c r="I120" t="inlineStr"/>
@@ -6443,7 +6459,7 @@
       <c r="L120" t="inlineStr"/>
       <c r="M120" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27415</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28403</t>
         </is>
       </c>
     </row>
@@ -6461,7 +6477,7 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>ポップパップポルターズ</t>
+          <t>ホタルの嫁入り</t>
         </is>
       </c>
       <c r="E121" t="b">
@@ -6474,12 +6490,12 @@
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>2026年秋 テレビ朝日にて</t>
+          <t>2026年10月～ 全国フジテレビ系“ ノイタミナ ”にて</t>
         </is>
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>MOZU STUDIOS</t>
+          <t>david production</t>
         </is>
       </c>
       <c r="I121" t="inlineStr"/>
@@ -6488,7 +6504,7 @@
       <c r="L121" t="inlineStr"/>
       <c r="M121" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27823</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27415</t>
         </is>
       </c>
     </row>
@@ -6506,7 +6522,7 @@
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>ホテル・インヒューマンズ 第2期</t>
+          <t>ポップパップポルターズ</t>
         </is>
       </c>
       <c r="E122" t="b">
@@ -6519,12 +6535,12 @@
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>2026年10月～ テレ東系列ほか</t>
+          <t>2026年秋 テレビ朝日にて</t>
         </is>
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>ブリッジ</t>
+          <t>MOZU STUDIOS</t>
         </is>
       </c>
       <c r="I122" t="inlineStr"/>
@@ -6533,7 +6549,7 @@
       <c r="L122" t="inlineStr"/>
       <c r="M122" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26870</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27823</t>
         </is>
       </c>
     </row>
@@ -6551,7 +6567,7 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>マジカル★エクスプローラー</t>
+          <t>ホテル・インヒューマンズ 第2期</t>
         </is>
       </c>
       <c r="E123" t="b">
@@ -6564,12 +6580,12 @@
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t>2026年秋</t>
+          <t>2026年10月～ テレ東系列ほか</t>
         </is>
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>WHITE FOX</t>
+          <t>ブリッジ</t>
         </is>
       </c>
       <c r="I123" t="inlineStr"/>
@@ -6578,7 +6594,7 @@
       <c r="L123" t="inlineStr"/>
       <c r="M123" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=23375</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26870</t>
         </is>
       </c>
     </row>
@@ -6596,7 +6612,7 @@
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>魔法騎士レイアース</t>
+          <t>マジカル★エクスプローラー</t>
         </is>
       </c>
       <c r="E124" t="b">
@@ -6609,12 +6625,12 @@
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>2026年10月～ テレビ朝日系列にて</t>
+          <t>2026年秋</t>
         </is>
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>E&amp;H production</t>
+          <t>WHITE FOX</t>
         </is>
       </c>
       <c r="I124" t="inlineStr"/>
@@ -6623,7 +6639,7 @@
       <c r="L124" t="inlineStr"/>
       <c r="M124" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=24301</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=23375</t>
         </is>
       </c>
     </row>
@@ -6641,7 +6657,7 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>魔法少女育成計画restart</t>
+          <t>魔法騎士レイアース</t>
         </is>
       </c>
       <c r="E125" t="b">
@@ -6654,29 +6670,21 @@
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>2026年秋</t>
+          <t>2026年10月～ テレビ朝日系列にて</t>
         </is>
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>SynergySP</t>
-        </is>
-      </c>
-      <c r="I125" t="inlineStr">
-        <is>
-          <t>No tears here</t>
-        </is>
-      </c>
-      <c r="J125" t="inlineStr">
-        <is>
-          <t>茅原実里</t>
-        </is>
-      </c>
+          <t>E&amp;H production</t>
+        </is>
+      </c>
+      <c r="I125" t="inlineStr"/>
+      <c r="J125" t="inlineStr"/>
       <c r="K125" t="inlineStr"/>
       <c r="L125" t="inlineStr"/>
       <c r="M125" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26693</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=24301</t>
         </is>
       </c>
     </row>
@@ -6694,7 +6702,7 @@
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>マロニエ王国の七人の騎士</t>
+          <t>魔法少女育成計画restart</t>
         </is>
       </c>
       <c r="E126" t="b">
@@ -6707,21 +6715,29 @@
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t>2026年10月～ NHK Eテレにて</t>
+          <t>2026年秋</t>
         </is>
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>J.C.STAFF</t>
-        </is>
-      </c>
-      <c r="I126" t="inlineStr"/>
-      <c r="J126" t="inlineStr"/>
+          <t>SynergySP</t>
+        </is>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>No tears here</t>
+        </is>
+      </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>茅原実里</t>
+        </is>
+      </c>
       <c r="K126" t="inlineStr"/>
       <c r="L126" t="inlineStr"/>
       <c r="M126" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28456</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26693</t>
         </is>
       </c>
     </row>
@@ -6739,7 +6755,7 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>目覚めたら最強装備と宇宙船持ちだったので、一戸建て目指して傭兵として自由に生きたい</t>
+          <t>マロニエ王国の七人の騎士</t>
         </is>
       </c>
       <c r="E127" t="b">
@@ -6752,12 +6768,12 @@
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t>2026年10月〜</t>
+          <t>2026年10月～ NHK Eテレにて</t>
         </is>
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>studio A-CAT</t>
+          <t>J.C.STAFF</t>
         </is>
       </c>
       <c r="I127" t="inlineStr"/>
@@ -6766,7 +6782,7 @@
       <c r="L127" t="inlineStr"/>
       <c r="M127" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25525</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28456</t>
         </is>
       </c>
     </row>
@@ -6784,7 +6800,7 @@
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>弱気MAX令嬢なのに、辣腕婚約者様の賭けに乗ってしまった</t>
+          <t>目覚めたら最強装備と宇宙船持ちだったので、一戸建て目指して傭兵として自由に生きたい</t>
         </is>
       </c>
       <c r="E128" t="b">
@@ -6797,12 +6813,12 @@
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
+          <t>2026年10月〜</t>
         </is>
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>寿門堂</t>
+          <t>studio A-CAT</t>
         </is>
       </c>
       <c r="I128" t="inlineStr"/>
@@ -6811,7 +6827,7 @@
       <c r="L128" t="inlineStr"/>
       <c r="M128" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26947</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25525</t>
         </is>
       </c>
     </row>
@@ -6829,7 +6845,7 @@
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>らんま1/2 第3期</t>
+          <t>弱気MAX令嬢なのに、辣腕婚約者様の賭けに乗ってしまった</t>
         </is>
       </c>
       <c r="E129" t="b">
@@ -6842,17 +6858,21 @@
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>2026年10月～ 日本テレビ系にて</t>
-        </is>
-      </c>
-      <c r="H129" t="inlineStr"/>
+          <t>2026年10月～</t>
+        </is>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>寿門堂</t>
+        </is>
+      </c>
       <c r="I129" t="inlineStr"/>
       <c r="J129" t="inlineStr"/>
       <c r="K129" t="inlineStr"/>
       <c r="L129" t="inlineStr"/>
       <c r="M129" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28013</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26947</t>
         </is>
       </c>
     </row>
@@ -6870,7 +6890,7 @@
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>LEGO® ONE PIECE</t>
+          <t>らんま1/2 第3期</t>
         </is>
       </c>
       <c r="E130" t="b">
@@ -6878,12 +6898,12 @@
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>配信</t>
+          <t>TVアニメ</t>
         </is>
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>2026年9月29日（火） Netflixにて</t>
+          <t>2026年10月～ 日本テレビ系にて</t>
         </is>
       </c>
       <c r="H130" t="inlineStr"/>
@@ -6892,6 +6912,47 @@
       <c r="K130" t="inlineStr"/>
       <c r="L130" t="inlineStr"/>
       <c r="M130" t="inlineStr">
+        <is>
+          <t>https://www.animatetimes.com/tag/details.php?id=28013</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C131" t="n">
+        <v>50</v>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>LEGO® ONE PIECE</t>
+        </is>
+      </c>
+      <c r="E131" t="b">
+        <v>0</v>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>配信</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>2026年9月29日（火） Netflixにて</t>
+        </is>
+      </c>
+      <c r="H131" t="inlineStr"/>
+      <c r="I131" t="inlineStr"/>
+      <c r="J131" t="inlineStr"/>
+      <c r="K131" t="inlineStr"/>
+      <c r="L131" t="inlineStr"/>
+      <c r="M131" t="inlineStr">
         <is>
           <t>https://www.animatetimes.com/tag/details.php?id=28168</t>
         </is>
@@ -6908,7 +6969,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L107"/>
+  <dimension ref="A1:L108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7584,7 +7645,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>株式会社マジルミエ 第2期</t>
+          <t>片田舎のおっさん、剣聖になるII</t>
         </is>
       </c>
       <c r="D17" t="b">
@@ -7600,12 +7661,12 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>BooooM!!!</t>
+          <t>未完成</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>宝鐘マリン</t>
+          <t>BLUE ENCOUNT</t>
         </is>
       </c>
       <c r="I17" t="inlineStr"/>
@@ -7624,15 +7685,15 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>帰還者の魔法は特別です</t>
+          <t>株式会社マジルミエ 第2期</t>
         </is>
       </c>
       <c r="D18" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F18" t="n">
@@ -7640,12 +7701,12 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>GET BACK</t>
+          <t>BooooM!!!</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>FLOW</t>
+          <t>宝鐘マリン</t>
         </is>
       </c>
       <c r="I18" t="inlineStr"/>
@@ -7672,7 +7733,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F19" t="n">
@@ -7680,12 +7741,12 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>6を撫でる</t>
+          <t>GET BACK</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>ももすももす</t>
+          <t>FLOW</t>
         </is>
       </c>
       <c r="I19" t="inlineStr"/>
@@ -7704,15 +7765,15 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>きみが死ぬまで恋をしたい</t>
+          <t>帰還者の魔法は特別です</t>
         </is>
       </c>
       <c r="D20" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F20" t="n">
@@ -7720,12 +7781,12 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Amore</t>
+          <t>6を撫でる</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>ReoNa</t>
+          <t>ももすももす</t>
         </is>
       </c>
       <c r="I20" t="inlineStr"/>
@@ -7752,7 +7813,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F21" t="n">
@@ -7760,12 +7821,12 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>エテルネル</t>
+          <t>Amore</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>sajou no hana</t>
+          <t>ReoNa</t>
         </is>
       </c>
       <c r="I21" t="inlineStr"/>
@@ -7784,7 +7845,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>「きみを愛する気はない」と言った次期公爵様がなぜか溺愛してきます</t>
+          <t>きみが死ぬまで恋をしたい</t>
         </is>
       </c>
       <c r="D22" t="b">
@@ -7792,7 +7853,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F22" t="n">
@@ -7800,12 +7861,12 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>いつかちゃんと。</t>
+          <t>エテルネル</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>りりあ。</t>
+          <t>sajou no hana</t>
         </is>
       </c>
       <c r="I22" t="inlineStr"/>
@@ -7832,7 +7893,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F23" t="n">
@@ -7840,12 +7901,12 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>最終回</t>
+          <t>いつかちゃんと。</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>sorato</t>
+          <t>りりあ。</t>
         </is>
       </c>
       <c r="I23" t="inlineStr"/>
@@ -7864,7 +7925,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>ぐらんぶる Season 3</t>
+          <t>「きみを愛する気はない」と言った次期公爵様がなぜか溺愛してきます</t>
         </is>
       </c>
       <c r="D24" t="b">
@@ -7872,7 +7933,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F24" t="n">
@@ -7880,12 +7941,12 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>夏子</t>
+          <t>最終回</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>FUNKY MONKEY BΛBY'S</t>
+          <t>sorato</t>
         </is>
       </c>
       <c r="I24" t="inlineStr"/>
@@ -7912,7 +7973,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F25" t="n">
@@ -7920,12 +7981,12 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>裸のマーメード</t>
+          <t>夏子</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>豆柴の大群</t>
+          <t>FUNKY MONKEY BΛBY'S</t>
         </is>
       </c>
       <c r="I25" t="inlineStr"/>
@@ -7944,7 +8005,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>クレバテスII-魔獣の王と偽りの勇者伝承-</t>
+          <t>ぐらんぶる Season 3</t>
         </is>
       </c>
       <c r="D26" t="b">
@@ -7952,7 +8013,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F26" t="n">
@@ -7960,12 +8021,12 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Foreshadow</t>
+          <t>裸のマーメード</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>前島麻由</t>
+          <t>豆柴の大群</t>
         </is>
       </c>
       <c r="I26" t="inlineStr"/>
@@ -7992,7 +8053,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F27" t="n">
@@ -8000,12 +8061,12 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Awake Anew</t>
+          <t>Foreshadow</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>MYTH &amp; ROID</t>
+          <t>前島麻由</t>
         </is>
       </c>
       <c r="I27" t="inlineStr"/>
@@ -8024,7 +8085,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>コードギアス 奪還のロゼ TV放送</t>
+          <t>クレバテスII-魔獣の王と偽りの勇者伝承-</t>
         </is>
       </c>
       <c r="D28" t="b">
@@ -8032,7 +8093,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F28" t="n">
@@ -8040,32 +8101,18 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Running In My Head</t>
+          <t>Awake Anew</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>MIYAVI</t>
-        </is>
-      </c>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=HSakQbaQifs</t>
-        </is>
-      </c>
-      <c r="J28" t="n">
-        <v>19423</v>
-      </c>
-      <c r="K28" t="inlineStr">
-        <is>
-          <t>コードギアスチャンネル CODEGEASS Channel</t>
-        </is>
-      </c>
-      <c r="L28" t="inlineStr">
-        <is>
-          <t>2026-06-05T19:01:45</t>
-        </is>
-      </c>
+          <t>MYTH &amp; ROID</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -8086,7 +8133,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F29" t="n">
@@ -8094,18 +8141,32 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>ロゼ (Prod.TeddyLoid)</t>
+          <t>Running In My Head</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>満島ひかり</t>
-        </is>
-      </c>
-      <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr"/>
-      <c r="K29" t="inlineStr"/>
-      <c r="L29" t="inlineStr"/>
+          <t>MIYAVI</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=HSakQbaQifs</t>
+        </is>
+      </c>
+      <c r="J29" t="n">
+        <v>19423</v>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>コードギアスチャンネル CODEGEASS Channel</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>2026-06-05T19:01:45</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -8118,7 +8179,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>これ描いて死ね</t>
+          <t>コードギアス 奪還のロゼ TV放送</t>
         </is>
       </c>
       <c r="D30" t="b">
@@ -8126,7 +8187,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F30" t="n">
@@ -8134,12 +8195,12 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>遺書</t>
+          <t>ロゼ (Prod.TeddyLoid)</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>キタニタツヤ</t>
+          <t>満島ひかり</t>
         </is>
       </c>
       <c r="I30" t="inlineStr"/>
@@ -8166,7 +8227,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F31" t="n">
@@ -8174,12 +8235,12 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>コニファー</t>
+          <t>遺書</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>リーガルリリー</t>
+          <t>キタニタツヤ</t>
         </is>
       </c>
       <c r="I31" t="inlineStr"/>
@@ -8198,7 +8259,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>才女のお世話 高嶺の花だらけな名門校で、学院一のお嬢様(生活能力皆無)を陰ながらお世話することになりました</t>
+          <t>これ描いて死ね</t>
         </is>
       </c>
       <c r="D32" t="b">
@@ -8206,7 +8267,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F32" t="n">
@@ -8214,12 +8275,12 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>最最最高級のお世話して</t>
+          <t>コニファー</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>angela</t>
+          <t>リーガルリリー</t>
         </is>
       </c>
       <c r="I32" t="inlineStr"/>
@@ -8246,7 +8307,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F33" t="n">
@@ -8254,12 +8315,12 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>完璧じゃないわたし</t>
+          <t>最最最高級のお世話して</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>前島亜美</t>
+          <t>angela</t>
         </is>
       </c>
       <c r="I33" t="inlineStr"/>
@@ -8278,7 +8339,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>サイボーグ009 ネメシス</t>
+          <t>才女のお世話 高嶺の花だらけな名門校で、学院一のお嬢様(生活能力皆無)を陰ながらお世話することになりました</t>
         </is>
       </c>
       <c r="D34" t="b">
@@ -8286,7 +8347,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F34" t="n">
@@ -8294,12 +8355,12 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>誰がために</t>
+          <t>完璧じゃないわたし</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>杏子</t>
+          <t>前島亜美</t>
         </is>
       </c>
       <c r="I34" t="inlineStr"/>
@@ -8318,7 +8379,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>さよならララ</t>
+          <t>サイボーグ009 ネメシス</t>
         </is>
       </c>
       <c r="D35" t="b">
@@ -8334,12 +8395,12 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>さよならララ</t>
+          <t>誰がために</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>いきものがかり</t>
+          <t>杏子</t>
         </is>
       </c>
       <c r="I35" t="inlineStr"/>
@@ -8358,7 +8419,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>スーパーの裏でヤニ吸うふたり</t>
+          <t>さよならララ</t>
         </is>
       </c>
       <c r="D36" t="b">
@@ -8374,12 +8435,12 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>イチジク煙</t>
+          <t>さよならララ</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>ずっと真夜中でいいのに。</t>
+          <t>いきものがかり</t>
         </is>
       </c>
       <c r="I36" t="inlineStr"/>
@@ -8406,7 +8467,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F37" t="n">
@@ -8414,12 +8475,12 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Fiction</t>
+          <t>イチジク煙</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>imase</t>
+          <t>ずっと真夜中でいいのに。</t>
         </is>
       </c>
       <c r="I37" t="inlineStr"/>
@@ -8438,7 +8499,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>捨てられ聖女の異世界ごはん旅 隠れスキルでキャンピングカーを召喚しました</t>
+          <t>スーパーの裏でヤニ吸うふたり</t>
         </is>
       </c>
       <c r="D38" t="b">
@@ -8446,7 +8507,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F38" t="n">
@@ -8454,12 +8515,12 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Butterfly</t>
+          <t>Fiction</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>INUWASI</t>
+          <t>imase</t>
         </is>
       </c>
       <c r="I38" t="inlineStr"/>
@@ -8486,7 +8547,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F39" t="n">
@@ -8494,12 +8555,12 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Holy Sweet Home</t>
+          <t>Butterfly</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>音感れもねゐど</t>
+          <t>INUWASI</t>
         </is>
       </c>
       <c r="I39" t="inlineStr"/>
@@ -8518,15 +8579,15 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>青春ブタ野郎はサンタクロースの夢を見ない</t>
+          <t>捨てられ聖女の異世界ごはん旅 隠れスキルでキャンピングカーを召喚しました</t>
         </is>
       </c>
       <c r="D40" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F40" t="n">
@@ -8534,12 +8595,12 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>スノウドロップ</t>
+          <t>Holy Sweet Home</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>Conton Candy</t>
+          <t>音感れもねゐど</t>
         </is>
       </c>
       <c r="I40" t="inlineStr"/>
@@ -8566,7 +8627,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F41" t="n">
@@ -8574,12 +8635,12 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>水平線は僕の古傷</t>
+          <t>スノウドロップ</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>広川卯月、赤城郁実、姫路紗良、霧島透子</t>
+          <t>Conton Candy</t>
         </is>
       </c>
       <c r="I41" t="inlineStr"/>
@@ -8598,15 +8659,15 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>正反対な君と僕 第2期</t>
+          <t>青春ブタ野郎はサンタクロースの夢を見ない</t>
         </is>
       </c>
       <c r="D42" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F42" t="n">
@@ -8614,12 +8675,12 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>メガネを外して</t>
+          <t>水平線は僕の古傷</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>乃紫</t>
+          <t>広川卯月、赤城郁実、姫路紗良、霧島透子</t>
         </is>
       </c>
       <c r="I42" t="inlineStr"/>
@@ -8650,16 +8711,16 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>猫じゃらし</t>
+          <t>メガネを外して</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>7co</t>
+          <t>乃紫</t>
         </is>
       </c>
       <c r="I43" t="inlineStr"/>
@@ -8686,20 +8747,20 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F44" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>ピュア feat. 橋本絵莉子</t>
+          <t>猫じゃらし</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>PAS TASTA</t>
+          <t>7co</t>
         </is>
       </c>
       <c r="I44" t="inlineStr"/>
@@ -8718,7 +8779,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>対ありでした。～お嬢さまは格闘ゲームなんてしない～</t>
+          <t>正反対な君と僕 第2期</t>
         </is>
       </c>
       <c r="D45" t="b">
@@ -8726,7 +8787,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F45" t="n">
@@ -8734,12 +8795,12 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>命短し対する乙女よ</t>
+          <t>ピュア feat. 橋本絵莉子</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>花冷え。</t>
+          <t>PAS TASTA</t>
         </is>
       </c>
       <c r="I45" t="inlineStr"/>
@@ -8766,7 +8827,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F46" t="n">
@@ -8774,12 +8835,12 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>NEW GAME</t>
+          <t>命短し対する乙女よ</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>halca</t>
+          <t>花冷え。</t>
         </is>
       </c>
       <c r="I46" t="inlineStr"/>
@@ -8798,7 +8859,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>追放された転生重騎士はゲーム知識で無双する</t>
+          <t>対ありでした。～お嬢さまは格闘ゲームなんてしない～</t>
         </is>
       </c>
       <c r="D47" t="b">
@@ -8806,7 +8867,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F47" t="n">
@@ -8814,12 +8875,12 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Awake</t>
+          <t>NEW GAME</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>SPYAIR</t>
+          <t>halca</t>
         </is>
       </c>
       <c r="I47" t="inlineStr"/>
@@ -8838,7 +8899,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>鉄鍋のジャン！</t>
+          <t>追放された転生重騎士はゲーム知識で無双する</t>
         </is>
       </c>
       <c r="D48" t="b">
@@ -8854,12 +8915,12 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>火宴</t>
+          <t>Awake</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>原因は自分にある。</t>
+          <t>SPYAIR</t>
         </is>
       </c>
       <c r="I48" t="inlineStr"/>
@@ -8878,7 +8939,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>手札が多めのビクトリア</t>
+          <t>鉄鍋のジャン！</t>
         </is>
       </c>
       <c r="D49" t="b">
@@ -8886,7 +8947,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F49" t="n">
@@ -8894,32 +8955,18 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>縁のつき</t>
+          <t>火宴</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>KI_EN</t>
-        </is>
-      </c>
-      <c r="I49" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=-HNOXWE2wVU</t>
-        </is>
-      </c>
-      <c r="J49" t="n">
-        <v>107892</v>
-      </c>
-      <c r="K49" t="inlineStr">
-        <is>
-          <t>KADOKAWAanime</t>
-        </is>
-      </c>
-      <c r="L49" t="inlineStr">
-        <is>
-          <t>2026-06-04T19:29:01</t>
-        </is>
-      </c>
+          <t>原因は自分にある。</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr"/>
+      <c r="J49" t="inlineStr"/>
+      <c r="K49" t="inlineStr"/>
+      <c r="L49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -8932,7 +8979,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>転校先の清楚可憐な美少女が、昔男子と思って一緒に遊んだ幼馴染だった件</t>
+          <t>手札が多めのビクトリア</t>
         </is>
       </c>
       <c r="D50" t="b">
@@ -8940,7 +8987,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F50" t="n">
@@ -8948,12 +8995,12 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>夏に重ねて</t>
+          <t>縁のつき</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>DIALOGUE+</t>
+          <t>KI_EN</t>
         </is>
       </c>
       <c r="I50" t="inlineStr"/>
@@ -8972,7 +9019,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>天は赤い河のほとり</t>
+          <t>転校先の清楚可憐な美少女が、昔男子と思って一緒に遊んだ幼馴染だった件</t>
         </is>
       </c>
       <c r="D51" t="b">
@@ -8988,12 +9035,12 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>暁の空</t>
+          <t>夏に重ねて</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>七海ひろき</t>
+          <t>DIALOGUE+</t>
         </is>
       </c>
       <c r="I51" t="inlineStr"/>
@@ -9012,7 +9059,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>天幕のジャードゥーガル</t>
+          <t>天は赤い河のほとり</t>
         </is>
       </c>
       <c r="D52" t="b">
@@ -9028,12 +9075,12 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Stella</t>
+          <t>暁の空</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>SEKAI NO OWARI</t>
+          <t>七海ひろき</t>
         </is>
       </c>
       <c r="I52" t="inlineStr"/>
@@ -9052,7 +9099,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>盗掘王</t>
+          <t>天幕のジャードゥーガル</t>
         </is>
       </c>
       <c r="D53" t="b">
@@ -9068,12 +9115,12 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>SHOW DOWN</t>
+          <t>Stella</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>QWER</t>
+          <t>SEKAI NO OWARI</t>
         </is>
       </c>
       <c r="I53" t="inlineStr"/>
@@ -9092,7 +9139,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>透明な夜に駆ける君と、目に見えない恋をした。</t>
+          <t>盗掘王</t>
         </is>
       </c>
       <c r="D54" t="b">
@@ -9100,7 +9147,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F54" t="n">
@@ -9108,12 +9155,12 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>光</t>
+          <t>SHOW DOWN</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>櫻井優衣</t>
+          <t>QWER</t>
         </is>
       </c>
       <c r="I54" t="inlineStr"/>
@@ -9132,7 +9179,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>トミカとトム</t>
+          <t>透明な夜に駆ける君と、目に見えない恋をした。</t>
         </is>
       </c>
       <c r="D55" t="b">
@@ -9140,7 +9187,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>主題歌</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F55" t="n">
@@ -9148,12 +9195,12 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>きみのたからもの</t>
+          <t>ひとひら</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>May J.</t>
+          <t>秦基博</t>
         </is>
       </c>
       <c r="I55" t="inlineStr"/>
@@ -9172,7 +9219,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>二十世紀電氣目録-ユーレカ・エヴリカ-</t>
+          <t>透明な夜に駆ける君と、目に見えない恋をした。</t>
         </is>
       </c>
       <c r="D56" t="b">
@@ -9180,7 +9227,7 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F56" t="n">
@@ -9188,12 +9235,12 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>ユーレカ・エヴリカ</t>
+          <t>光</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>五阿弥ルナ</t>
+          <t>櫻井優衣</t>
         </is>
       </c>
       <c r="I56" t="inlineStr"/>
@@ -9212,7 +9259,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>パイの実 おしの森へようこそ！</t>
+          <t>トミカとトム</t>
         </is>
       </c>
       <c r="D57" t="b">
@@ -9228,12 +9275,12 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>パイしか勝たん！推しの森活</t>
+          <t>きみのたからもの</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>安保心結</t>
+          <t>May J.</t>
         </is>
       </c>
       <c r="I57" t="inlineStr"/>
@@ -9252,7 +9299,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>刃牙道 第1クール（TV放送）</t>
+          <t>二十世紀電氣目録-ユーレカ・エヴリカ-</t>
         </is>
       </c>
       <c r="D58" t="b">
@@ -9268,12 +9315,12 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>フルボコ</t>
+          <t>ユーレカ・エヴリカ</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>WANIMA</t>
+          <t>五阿弥ルナ</t>
         </is>
       </c>
       <c r="I58" t="inlineStr"/>
@@ -9292,7 +9339,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>刃牙道 第1クール（TV放送）</t>
+          <t>パイの実 おしの森へようこそ！</t>
         </is>
       </c>
       <c r="D59" t="b">
@@ -9300,20 +9347,20 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>主題歌</t>
         </is>
       </c>
       <c r="F59" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>六ノ輪</t>
+          <t>パイしか勝たん！推しの森活</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>Chevon</t>
+          <t>安保心結</t>
         </is>
       </c>
       <c r="I59" t="inlineStr"/>
@@ -9332,7 +9379,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>刃牙道 第1クール（TV放送）</t>
+          <t>刃牙道 第2クール</t>
         </is>
       </c>
       <c r="D60" t="b">
@@ -9340,7 +9387,7 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F60" t="n">
@@ -9348,12 +9395,12 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>Mountain Top</t>
+          <t>フルボコ</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>Novel Core</t>
+          <t>WANIMA</t>
         </is>
       </c>
       <c r="I60" t="inlineStr"/>
@@ -9372,7 +9419,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>刃牙道 第1クール（TV放送）</t>
+          <t>刃牙道 第2クール</t>
         </is>
       </c>
       <c r="D61" t="b">
@@ -9380,7 +9427,7 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F61" t="n">
@@ -9388,12 +9435,12 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>KATANA</t>
+          <t>六ノ輪</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>三代目 J SOUL BROTHERS</t>
+          <t>Chevon</t>
         </is>
       </c>
       <c r="I61" t="inlineStr"/>
@@ -9420,7 +9467,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F62" t="n">
@@ -9428,12 +9475,12 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>フルボコ</t>
+          <t>Mountain Top</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>WANIMA</t>
+          <t>Novel Core</t>
         </is>
       </c>
       <c r="I62" t="inlineStr"/>
@@ -9460,7 +9507,7 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F63" t="n">
@@ -9468,12 +9515,12 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>六ノ輪</t>
+          <t>KATANA</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>Chevon</t>
+          <t>三代目 J SOUL BROTHERS</t>
         </is>
       </c>
       <c r="I63" t="inlineStr"/>
@@ -9492,7 +9539,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>刃牙道 第2クール</t>
+          <t>花ざかりの君たちへ 第2期</t>
         </is>
       </c>
       <c r="D64" t="b">
@@ -9500,7 +9547,7 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F64" t="n">
@@ -9508,12 +9555,12 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>Mountain Top</t>
+          <t>FLASHBULB</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>Novel Core</t>
+          <t>Omoinotake</t>
         </is>
       </c>
       <c r="I64" t="inlineStr"/>
@@ -9532,7 +9579,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>刃牙道 第2クール</t>
+          <t>花ざかりの君たちへ 第2期</t>
         </is>
       </c>
       <c r="D65" t="b">
@@ -9544,16 +9591,16 @@
         </is>
       </c>
       <c r="F65" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>KATANA</t>
+          <t>花束</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>三代目 J SOUL BROTHERS</t>
+          <t>Omoinotake</t>
         </is>
       </c>
       <c r="I65" t="inlineStr"/>
@@ -9572,7 +9619,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>花ざかりの君たちへ 第2期</t>
+          <t>ヒロイン？聖女？いいえ、オールワークスメイドです（誇）！</t>
         </is>
       </c>
       <c r="D66" t="b">
@@ -9588,12 +9635,12 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>FLASHBULB</t>
+          <t>マデュアル↔ハート</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>Omoinotake</t>
+          <t>メロディ・ウェーブ(CV：宮本侑芽) ルシアナ・ルトルバーグ(CV：大久保瑠美)</t>
         </is>
       </c>
       <c r="I66" t="inlineStr"/>
@@ -9612,7 +9659,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>花ざかりの君たちへ 第2期</t>
+          <t>ヒロイン？聖女？いいえ、オールワークスメイドです（誇）！</t>
         </is>
       </c>
       <c r="D67" t="b">
@@ -9628,12 +9675,12 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>花束</t>
+          <t>ハンドメイド</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>Omoinotake</t>
+          <t>仲村宗悟</t>
         </is>
       </c>
       <c r="I67" t="inlineStr"/>
@@ -9652,7 +9699,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>ヒロイン？聖女？いいえ、オールワークスメイドです（誇）！</t>
+          <t>ブチ切れ令嬢は報復を誓いました。 ～魔導書の力で祖国を叩き潰します～</t>
         </is>
       </c>
       <c r="D68" t="b">
@@ -9668,12 +9715,12 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>マデュアル↔ハート</t>
+          <t>Q.E.D.</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>メロディ・ウェーブ(CV：宮本侑芽) ルシアナ・ルトルバーグ(CV：大久保瑠美)</t>
+          <t>小倉唯</t>
         </is>
       </c>
       <c r="I68" t="inlineStr"/>
@@ -9692,7 +9739,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>ヒロイン？聖女？いいえ、オールワークスメイドです（誇）！</t>
+          <t>ブチ切れ令嬢は報復を誓いました。 ～魔導書の力で祖国を叩き潰します～</t>
         </is>
       </c>
       <c r="D69" t="b">
@@ -9708,12 +9755,12 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>ハンドメイド</t>
+          <t>グッバイ・ララバイ</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>仲村宗悟</t>
+          <t>大西亜玖璃</t>
         </is>
       </c>
       <c r="I69" t="inlineStr"/>
@@ -9732,7 +9779,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>ブチ切れ令嬢は報復を誓いました。 ～魔導書の力で祖国を叩き潰します～</t>
+          <t>ふつつかな悪女ではございますが～雛宮蝶鼠とりかえ伝～</t>
         </is>
       </c>
       <c r="D70" t="b">
@@ -9748,12 +9795,12 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>Q.E.D.</t>
+          <t>Sunny</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>小倉唯</t>
+          <t>milet</t>
         </is>
       </c>
       <c r="I70" t="inlineStr"/>
@@ -9772,7 +9819,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>ブチ切れ令嬢は報復を誓いました。 ～魔導書の力で祖国を叩き潰します～</t>
+          <t>BLACK TORCH</t>
         </is>
       </c>
       <c r="D71" t="b">
@@ -9780,7 +9827,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F71" t="n">
@@ -9788,12 +9835,12 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>グッバイ・ララバイ</t>
+          <t>FREEZE ME UP</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>大西亜玖璃</t>
+          <t>SiM</t>
         </is>
       </c>
       <c r="I71" t="inlineStr"/>
@@ -9812,7 +9859,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>ふつつかな悪女ではございますが～雛宮蝶鼠とりかえ伝～</t>
+          <t>BLACK TORCH</t>
         </is>
       </c>
       <c r="D72" t="b">
@@ -9820,7 +9867,7 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F72" t="n">
@@ -9828,12 +9875,12 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>Sunny</t>
+          <t>Groooovy</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>milet</t>
+          <t>I Don't Like Mondays.</t>
         </is>
       </c>
       <c r="I72" t="inlineStr"/>
@@ -9852,7 +9899,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>BLACK TORCH</t>
+          <t>プラノサウルス ガチコセイブツ部</t>
         </is>
       </c>
       <c r="D73" t="b">
@@ -9860,7 +9907,7 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>主題歌</t>
         </is>
       </c>
       <c r="F73" t="n">
@@ -9868,12 +9915,12 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>FREEZE ME UP</t>
+          <t>ガチde古生</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>SiM</t>
+          <t>リンクルプラネット</t>
         </is>
       </c>
       <c r="I73" t="inlineStr"/>
@@ -9892,7 +9939,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>BLACK TORCH</t>
+          <t>ヘルモード ～やり込み好きのゲーマーは廃設定の異世界で無双する～ 2nd Season</t>
         </is>
       </c>
       <c r="D74" t="b">
@@ -9900,7 +9947,7 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F74" t="n">
@@ -9908,12 +9955,12 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>Groooovy</t>
+          <t>○✕△□</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>I Don't Like Mondays.</t>
+          <t>浪漫派マシュマロ</t>
         </is>
       </c>
       <c r="I74" t="inlineStr"/>
@@ -9932,7 +9979,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>プラノサウルス ガチコセイブツ部</t>
+          <t>北斗の拳 拳王軍ザコたちの挽歌 第2クール</t>
         </is>
       </c>
       <c r="D75" t="b">
@@ -9940,7 +9987,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>主題歌</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F75" t="n">
@@ -9948,12 +9995,12 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>ガチde古生</t>
+          <t>Blacker Co., Ltd.</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>リンクルプラネット</t>
+          <t>イツカ▶</t>
         </is>
       </c>
       <c r="I75" t="inlineStr"/>
@@ -9972,7 +10019,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>ヘルモード ～やり込み好きのゲーマーは廃設定の異世界で無双する～ 2nd Season</t>
+          <t>北斗の拳 拳王軍ザコたちの挽歌 第2クール</t>
         </is>
       </c>
       <c r="D76" t="b">
@@ -9980,7 +10027,7 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F76" t="n">
@@ -9988,12 +10035,12 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>○✕△□</t>
+          <t>Elegy of the Enemies</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>浪漫派マシュマロ</t>
+          <t>The Canbellz</t>
         </is>
       </c>
       <c r="I76" t="inlineStr"/>
@@ -10012,7 +10059,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>炎の闘球女 ドッジ弾子</t>
+          <t>北斗の拳 拳王軍ザコたちの挽歌 第2クール</t>
         </is>
       </c>
       <c r="D77" t="b">
@@ -10020,20 +10067,20 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F77" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>会心の一劇</t>
+          <t>白い蝶が飛んだら</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>ももいろクローバーZ</t>
+          <t>イツカ▶ feat. Dr. Washington | Special Guest Guitar:Tsuyoshi Ujiki</t>
         </is>
       </c>
       <c r="I77" t="inlineStr"/>
@@ -10060,7 +10107,7 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F78" t="n">
@@ -10068,12 +10115,12 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>Welcome to あざとさワールド</t>
+          <t>会心の一劇</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>i☆Ris</t>
+          <t>ももいろクローバーZ</t>
         </is>
       </c>
       <c r="I78" t="inlineStr"/>
@@ -10092,7 +10139,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>魔法少女リリカルなのは EXCEEDS Gun Blaze Vengeance</t>
+          <t>炎の闘球女 ドッジ弾子</t>
         </is>
       </c>
       <c r="D79" t="b">
@@ -10100,7 +10147,7 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F79" t="n">
@@ -10108,12 +10155,12 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>CRIMSON BULLET</t>
+          <t>Welcome to あざとさワールド</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>水樹奈々</t>
+          <t>i☆Ris</t>
         </is>
       </c>
       <c r="I79" t="inlineStr"/>
@@ -10140,7 +10187,7 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F80" t="n">
@@ -10148,12 +10195,12 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>Ephemeral</t>
+          <t>CRIMSON BULLET</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>青木陽菜</t>
+          <t>水樹奈々</t>
         </is>
       </c>
       <c r="I80" t="inlineStr"/>
@@ -10172,7 +10219,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>無自覚聖女は今日も無意識に力を垂れ流す</t>
+          <t>魔法少女リリカルなのは EXCEEDS Gun Blaze Vengeance</t>
         </is>
       </c>
       <c r="D81" t="b">
@@ -10180,7 +10227,7 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F81" t="n">
@@ -10188,12 +10235,12 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>Windmaker</t>
+          <t>Ephemeral</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>花耶</t>
+          <t>青木陽菜</t>
         </is>
       </c>
       <c r="I81" t="inlineStr"/>
@@ -10220,7 +10267,7 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F82" t="n">
@@ -10228,12 +10275,12 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>アンノウンミー</t>
+          <t>Windmaker</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>ウタヒメドリーム オールスターズ【夢咲いぶき（CV:山﨑玲奈） 桜木舞華（CV:鈴木杏奈） 真白清美（CV:其原有沙） HiREN（CV:花耶） 水月ひかり（CV:礒部花凜） 高木凛（CV:鷲見友美ジェナ） 萩原ひまわり（CV:倉知玲鳳） SAKURAKO（CV:竹内夢）】</t>
+          <t>花耶</t>
         </is>
       </c>
       <c r="I82" t="inlineStr"/>
@@ -10252,7 +10299,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>無職転生Ⅲ ～異世界行ったら本気だす～</t>
+          <t>無自覚聖女は今日も無意識に力を垂れ流す</t>
         </is>
       </c>
       <c r="D83" t="b">
@@ -10260,7 +10307,7 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F83" t="n">
@@ -10268,12 +10315,12 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>決意の唄</t>
+          <t>アンノウンミー</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>大原ゆい子</t>
+          <t>ウタヒメドリーム オールスターズ【夢咲いぶき（CV:山﨑玲奈） 桜木舞華（CV:鈴木杏奈） 真白清美（CV:其原有沙） HiREN（CV:花耶） 水月ひかり（CV:礒部花凜） 高木凛（CV:鷲見友美ジェナ） 萩原ひまわり（CV:倉知玲鳳） SAKURAKO（CV:竹内夢）】</t>
         </is>
       </c>
       <c r="I83" t="inlineStr"/>
@@ -10300,7 +10347,7 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F84" t="n">
@@ -10308,12 +10355,12 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>祈り、終われば</t>
+          <t>決意の唄</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>中島美嘉</t>
+          <t>大原ゆい子</t>
         </is>
       </c>
       <c r="I84" t="inlineStr"/>
@@ -10332,7 +10379,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>メビウス・ダスト</t>
+          <t>無職転生Ⅲ ～異世界行ったら本気だす～</t>
         </is>
       </c>
       <c r="D85" t="b">
@@ -10340,7 +10387,7 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F85" t="n">
@@ -10348,12 +10395,12 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>メビウス</t>
+          <t>祈り、終われば</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>家入レオ</t>
+          <t>中島美嘉</t>
         </is>
       </c>
       <c r="I85" t="inlineStr"/>
@@ -10380,7 +10427,7 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F86" t="n">
@@ -10388,12 +10435,12 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>ジレンマ</t>
+          <t>メビウス</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>冨岡愛</t>
+          <t>家入レオ</t>
         </is>
       </c>
       <c r="I86" t="inlineStr"/>
@@ -10412,7 +10459,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>ヤニねこ</t>
+          <t>メビウス・ダスト</t>
         </is>
       </c>
       <c r="D87" t="b">
@@ -10420,7 +10467,7 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F87" t="n">
@@ -10428,12 +10475,12 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>なんもねえ</t>
+          <t>ジレンマ</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>忘れらんねえよ</t>
+          <t>冨岡愛</t>
         </is>
       </c>
       <c r="I87" t="inlineStr"/>
@@ -10452,7 +10499,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>幼女戦記Ⅱ</t>
+          <t>ヤニねこ</t>
         </is>
       </c>
       <c r="D88" t="b">
@@ -10468,12 +10515,12 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>Why? RED induction</t>
+          <t>なんもねえ</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>MYTH &amp; ROID</t>
+          <t>忘れらんねえよ</t>
         </is>
       </c>
       <c r="I88" t="inlineStr"/>
@@ -10500,7 +10547,7 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F89" t="n">
@@ -10508,12 +10555,12 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>Weiter! Weiter!</t>
+          <t>Why? RED induction</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>ターニャ・デグレチャフ（CV：悠木碧）</t>
+          <t>MYTH &amp; ROID</t>
         </is>
       </c>
       <c r="I89" t="inlineStr"/>
@@ -10532,7 +10579,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>鎧真伝サムライトルーパー 第2クール</t>
+          <t>幼女戦記Ⅱ</t>
         </is>
       </c>
       <c r="D90" t="b">
@@ -10540,7 +10587,7 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F90" t="n">
@@ -10548,12 +10595,12 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>YOAKE</t>
+          <t>Weiter! Weiter!</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>blank paper</t>
+          <t>ターニャ・デグレチャフ（CV：悠木碧）</t>
         </is>
       </c>
       <c r="I90" t="inlineStr"/>
@@ -10584,16 +10631,16 @@
         </is>
       </c>
       <c r="F91" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>BAD遺伝子</t>
+          <t>YOAKE</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>Dannie May</t>
+          <t>blank paper</t>
         </is>
       </c>
       <c r="I91" t="inlineStr"/>
@@ -10620,20 +10667,20 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F92" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>POWER</t>
+          <t>BAD遺伝子</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>ONE OR EIGHT</t>
+          <t>Dannie May</t>
         </is>
       </c>
       <c r="I92" t="inlineStr"/>
@@ -10664,16 +10711,16 @@
         </is>
       </c>
       <c r="F93" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>ばけもん</t>
+          <t>POWER</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>カラノア</t>
+          <t>ONE OR EIGHT</t>
         </is>
       </c>
       <c r="I93" t="inlineStr"/>
@@ -10692,7 +10739,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>落第賢者の学院無双～二度目の転生、Sランクチート魔術師冒険録～</t>
+          <t>鎧真伝サムライトルーパー 第2クール</t>
         </is>
       </c>
       <c r="D94" t="b">
@@ -10700,20 +10747,20 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F94" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>＋ENCOUNT</t>
+          <t>ばけもん</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>FLOW</t>
+          <t>カラノア</t>
         </is>
       </c>
       <c r="I94" t="inlineStr"/>
@@ -10740,7 +10787,7 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F95" t="n">
@@ -10748,12 +10795,12 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>憧憬</t>
+          <t>＋ENCOUNT</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>TrySail</t>
+          <t>FLOW</t>
         </is>
       </c>
       <c r="I95" t="inlineStr"/>
@@ -10772,7 +10819,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>領民0人スタートの辺境領主様</t>
+          <t>落第賢者の学院無双～二度目の転生、Sランクチート魔術師冒険録～</t>
         </is>
       </c>
       <c r="D96" t="b">
@@ -10780,7 +10827,7 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F96" t="n">
@@ -10788,12 +10835,12 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>Wonder</t>
+          <t>憧憬</t>
         </is>
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>CROWN HEAD</t>
+          <t>TrySail</t>
         </is>
       </c>
       <c r="I96" t="inlineStr"/>
@@ -10820,7 +10867,7 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F97" t="n">
@@ -10828,12 +10875,12 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>星降る夜の約束</t>
+          <t>Wonder</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>花耶</t>
+          <t>CROWN HEAD</t>
         </is>
       </c>
       <c r="I97" t="inlineStr"/>
@@ -10852,7 +10899,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>令和のダラさん</t>
+          <t>領民0人スタートの辺境領主様</t>
         </is>
       </c>
       <c r="D98" t="b">
@@ -10860,7 +10907,7 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F98" t="n">
@@ -10868,12 +10915,12 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>ダラダラ♡ダンシング</t>
+          <t>星降る夜の約束</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>ダラさん（CV：田村睦心） 三⼗⽊⾕⽇向（CV：津田美波） 三⼗⽊⾕薫（CV：寺澤百花） ナレーション（CV：てらそままさき）</t>
+          <t>花耶</t>
         </is>
       </c>
       <c r="I98" t="inlineStr"/>
@@ -10900,7 +10947,7 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F99" t="n">
@@ -10908,12 +10955,12 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>ひなたぼっこ</t>
+          <t>ダラダラ♡ダンシング</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>REIRIE</t>
+          <t>ダラさん（CV：田村睦心） 三⼗⽊⾕⽇向（CV：津田美波） 三⼗⽊⾕薫（CV：寺澤百花） ナレーション（CV：てらそままさき）</t>
         </is>
       </c>
       <c r="I99" t="inlineStr"/>
@@ -10932,7 +10979,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>LV999の村人</t>
+          <t>令和のダラさん</t>
         </is>
       </c>
       <c r="D100" t="b">
@@ -10940,7 +10987,7 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F100" t="n">
@@ -10948,12 +10995,12 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>Not a Hero</t>
+          <t>ひなたぼっこ</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>藍月なくる&amp;棗いつき</t>
+          <t>REIRIE</t>
         </is>
       </c>
       <c r="I100" t="inlineStr"/>
@@ -10980,7 +11027,7 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F101" t="n">
@@ -10988,12 +11035,12 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>Not a Hero</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>ゆきむら。</t>
+          <t>藍月なくる&amp;棗いつき</t>
         </is>
       </c>
       <c r="I101" t="inlineStr"/>
@@ -11012,7 +11059,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>ワールド イズ ダンシング</t>
+          <t>LV999の村人</t>
         </is>
       </c>
       <c r="D102" t="b">
@@ -11020,7 +11067,7 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F102" t="n">
@@ -11028,12 +11075,12 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>終宵</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>マカロニえんぴつ</t>
+          <t>ゆきむら。</t>
         </is>
       </c>
       <c r="I102" t="inlineStr"/>
@@ -11043,16 +11090,16 @@
     </row>
     <row r="103">
       <c r="A103" t="n">
-        <v>5947</v>
+        <v>5806</v>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>2026秋アニメ</t>
+          <t>2026夏アニメ</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>帰還者の魔法は特別です 第2期</t>
+          <t>ワールド イズ ダンシング</t>
         </is>
       </c>
       <c r="D103" t="b">
@@ -11068,12 +11115,12 @@
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>Sorrow</t>
+          <t>終宵</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>FLOW</t>
+          <t>マカロニえんぴつ</t>
         </is>
       </c>
       <c r="I103" t="inlineStr"/>
@@ -11092,7 +11139,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>獣王武神ダンデヴァイン</t>
+          <t>帰還者の魔法は特別です 第2期</t>
         </is>
       </c>
       <c r="D104" t="b">
@@ -11108,12 +11155,12 @@
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>曲名未発表</t>
+          <t>Sorrow</t>
         </is>
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>西川貴教</t>
+          <t>FLOW</t>
         </is>
       </c>
       <c r="I104" t="inlineStr"/>
@@ -11132,7 +11179,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>転生した大聖女は、聖女であることをひた隠す</t>
+          <t>獣王武神ダンデヴァイン</t>
         </is>
       </c>
       <c r="D105" t="b">
@@ -11148,12 +11195,12 @@
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>Flare of Soul</t>
+          <t>曲名未発表</t>
         </is>
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>花耶</t>
+          <t>西川貴教</t>
         </is>
       </c>
       <c r="I105" t="inlineStr"/>
@@ -11180,7 +11227,7 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F106" t="n">
@@ -11188,12 +11235,12 @@
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>STELLAR</t>
+          <t>Flare of Soul</t>
         </is>
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>ウタヒメドリーム オールスターズ</t>
+          <t>花耶</t>
         </is>
       </c>
       <c r="I106" t="inlineStr"/>
@@ -11212,7 +11259,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>魔法少女育成計画restart</t>
+          <t>転生した大聖女は、聖女であることをひた隠す</t>
         </is>
       </c>
       <c r="D107" t="b">
@@ -11220,7 +11267,7 @@
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F107" t="n">
@@ -11228,12 +11275,12 @@
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>No tears here</t>
+          <t>STELLAR</t>
         </is>
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>茅原実里</t>
+          <t>ウタヒメドリーム オールスターズ</t>
         </is>
       </c>
       <c r="I107" t="inlineStr"/>
@@ -11241,6 +11288,46 @@
       <c r="K107" t="inlineStr"/>
       <c r="L107" t="inlineStr"/>
     </row>
+    <row r="108">
+      <c r="A108" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>魔法少女育成計画restart</t>
+        </is>
+      </c>
+      <c r="D108" t="b">
+        <v>0</v>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="F108" t="n">
+        <v>1</v>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>No tears here</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>茅原実里</t>
+        </is>
+      </c>
+      <c r="I108" t="inlineStr"/>
+      <c r="J108" t="inlineStr"/>
+      <c r="K108" t="inlineStr"/>
+      <c r="L108" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
auto: anime list update 2026-06-12
</commit_message>
<xml_diff>
--- a/data/anime_list.xlsx
+++ b/data/anime_list.xlsx
@@ -1404,7 +1404,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2026年7月～ TOKYO MX・BS11・MBSにて</t>
+          <t>2026年7月6日（月）～ TOKYO MX・BS11・MBSにて</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1577,8 +1577,16 @@
       </c>
       <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
-      <c r="L22" t="inlineStr"/>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>Blue</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>MILLENNIUM PARADE feat. Saya Gray, Daniel Caesar</t>
+        </is>
+      </c>
       <c r="M22" t="inlineStr">
         <is>
           <t>https://www.animatetimes.com/tag/details.php?id=24096</t>
@@ -1987,14 +1995,22 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>2026年7月～ フジテレビ「+Ultra」にて</t>
+          <t>2026年7月8日（水）～ フジテレビ「+Ultra」にて</t>
         </is>
       </c>
       <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr"/>
       <c r="J30" t="inlineStr"/>
-      <c r="K30" t="inlineStr"/>
-      <c r="L30" t="inlineStr"/>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>しゅるれりら</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>音羽-otoha-</t>
+        </is>
+      </c>
       <c r="M30" t="inlineStr">
         <is>
           <t>https://www.animatetimes.com/tag/details.php?id=27611</t>
@@ -2028,7 +2044,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>2026年7月～ TBS系にて</t>
+          <t>2026年7月9日（木）～ TBS系にて</t>
         </is>
       </c>
       <c r="H31" t="inlineStr"/>
@@ -2085,7 +2101,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>2026年7月～ TOKYO MX・ＢＳ日テレほか</t>
+          <t>2026年7月6日（月）～ TOKYO MX・ＢＳ日テレほか</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -6969,7 +6985,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L108"/>
+  <dimension ref="A1:L110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8125,7 +8141,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>コードギアス 奪還のロゼ TV放送</t>
+          <t>攻殻機動隊 THE GHOST IN THE SHELL</t>
         </is>
       </c>
       <c r="D29" t="b">
@@ -8133,7 +8149,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F29" t="n">
@@ -8141,32 +8157,18 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Running In My Head</t>
+          <t>Blue</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>MIYAVI</t>
-        </is>
-      </c>
-      <c r="I29" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=HSakQbaQifs</t>
-        </is>
-      </c>
-      <c r="J29" t="n">
-        <v>19423</v>
-      </c>
-      <c r="K29" t="inlineStr">
-        <is>
-          <t>コードギアスチャンネル CODEGEASS Channel</t>
-        </is>
-      </c>
-      <c r="L29" t="inlineStr">
-        <is>
-          <t>2026-06-05T19:01:45</t>
-        </is>
-      </c>
+          <t>MILLENNIUM PARADE feat. Saya Gray, Daniel Caesar</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr"/>
+      <c r="L29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -8187,7 +8189,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F30" t="n">
@@ -8195,12 +8197,12 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>ロゼ (Prod.TeddyLoid)</t>
+          <t>Running In My Head</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>満島ひかり</t>
+          <t>MIYAVI</t>
         </is>
       </c>
       <c r="I30" t="inlineStr"/>
@@ -8219,7 +8221,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>これ描いて死ね</t>
+          <t>コードギアス 奪還のロゼ TV放送</t>
         </is>
       </c>
       <c r="D31" t="b">
@@ -8227,7 +8229,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F31" t="n">
@@ -8235,12 +8237,12 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>遺書</t>
+          <t>ロゼ (Prod.TeddyLoid)</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>キタニタツヤ</t>
+          <t>満島ひかり</t>
         </is>
       </c>
       <c r="I31" t="inlineStr"/>
@@ -8267,7 +8269,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F32" t="n">
@@ -8275,12 +8277,12 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>コニファー</t>
+          <t>遺書</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>リーガルリリー</t>
+          <t>キタニタツヤ</t>
         </is>
       </c>
       <c r="I32" t="inlineStr"/>
@@ -8299,7 +8301,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>才女のお世話 高嶺の花だらけな名門校で、学院一のお嬢様(生活能力皆無)を陰ながらお世話することになりました</t>
+          <t>これ描いて死ね</t>
         </is>
       </c>
       <c r="D33" t="b">
@@ -8307,7 +8309,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F33" t="n">
@@ -8315,12 +8317,12 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>最最最高級のお世話して</t>
+          <t>コニファー</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>angela</t>
+          <t>リーガルリリー</t>
         </is>
       </c>
       <c r="I33" t="inlineStr"/>
@@ -8347,7 +8349,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F34" t="n">
@@ -8355,12 +8357,12 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>完璧じゃないわたし</t>
+          <t>最最最高級のお世話して</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>前島亜美</t>
+          <t>angela</t>
         </is>
       </c>
       <c r="I34" t="inlineStr"/>
@@ -8379,7 +8381,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>サイボーグ009 ネメシス</t>
+          <t>才女のお世話 高嶺の花だらけな名門校で、学院一のお嬢様(生活能力皆無)を陰ながらお世話することになりました</t>
         </is>
       </c>
       <c r="D35" t="b">
@@ -8387,7 +8389,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F35" t="n">
@@ -8395,12 +8397,12 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>誰がために</t>
+          <t>完璧じゃないわたし</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>杏子</t>
+          <t>前島亜美</t>
         </is>
       </c>
       <c r="I35" t="inlineStr"/>
@@ -8419,7 +8421,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>さよならララ</t>
+          <t>サイボーグ009 ネメシス</t>
         </is>
       </c>
       <c r="D36" t="b">
@@ -8435,12 +8437,12 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>さよならララ</t>
+          <t>誰がために</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>いきものがかり</t>
+          <t>杏子</t>
         </is>
       </c>
       <c r="I36" t="inlineStr"/>
@@ -8459,7 +8461,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>スーパーの裏でヤニ吸うふたり</t>
+          <t>さよならララ</t>
         </is>
       </c>
       <c r="D37" t="b">
@@ -8475,12 +8477,12 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>イチジク煙</t>
+          <t>さよならララ</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>ずっと真夜中でいいのに。</t>
+          <t>いきものがかり</t>
         </is>
       </c>
       <c r="I37" t="inlineStr"/>
@@ -8499,7 +8501,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>スーパーの裏でヤニ吸うふたり</t>
+          <t>サンダー３</t>
         </is>
       </c>
       <c r="D38" t="b">
@@ -8515,12 +8517,12 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Fiction</t>
+          <t>しゅるれりら</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>imase</t>
+          <t>音羽-otoha-</t>
         </is>
       </c>
       <c r="I38" t="inlineStr"/>
@@ -8539,7 +8541,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>捨てられ聖女の異世界ごはん旅 隠れスキルでキャンピングカーを召喚しました</t>
+          <t>スーパーの裏でヤニ吸うふたり</t>
         </is>
       </c>
       <c r="D39" t="b">
@@ -8555,12 +8557,12 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Butterfly</t>
+          <t>イチジク煙</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>INUWASI</t>
+          <t>ずっと真夜中でいいのに。</t>
         </is>
       </c>
       <c r="I39" t="inlineStr"/>
@@ -8579,7 +8581,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>捨てられ聖女の異世界ごはん旅 隠れスキルでキャンピングカーを召喚しました</t>
+          <t>スーパーの裏でヤニ吸うふたり</t>
         </is>
       </c>
       <c r="D40" t="b">
@@ -8595,12 +8597,12 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Holy Sweet Home</t>
+          <t>Fiction</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>音感れもねゐど</t>
+          <t>imase</t>
         </is>
       </c>
       <c r="I40" t="inlineStr"/>
@@ -8619,11 +8621,11 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>青春ブタ野郎はサンタクロースの夢を見ない</t>
+          <t>捨てられ聖女の異世界ごはん旅 隠れスキルでキャンピングカーを召喚しました</t>
         </is>
       </c>
       <c r="D41" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -8635,12 +8637,12 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>スノウドロップ</t>
+          <t>Butterfly</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>Conton Candy</t>
+          <t>INUWASI</t>
         </is>
       </c>
       <c r="I41" t="inlineStr"/>
@@ -8659,11 +8661,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>青春ブタ野郎はサンタクロースの夢を見ない</t>
+          <t>捨てられ聖女の異世界ごはん旅 隠れスキルでキャンピングカーを召喚しました</t>
         </is>
       </c>
       <c r="D42" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -8675,12 +8677,12 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>水平線は僕の古傷</t>
+          <t>Holy Sweet Home</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>広川卯月、赤城郁実、姫路紗良、霧島透子</t>
+          <t>音感れもねゐど</t>
         </is>
       </c>
       <c r="I42" t="inlineStr"/>
@@ -8699,11 +8701,11 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>正反対な君と僕 第2期</t>
+          <t>青春ブタ野郎はサンタクロースの夢を見ない</t>
         </is>
       </c>
       <c r="D43" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -8715,12 +8717,12 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>メガネを外して</t>
+          <t>スノウドロップ</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>乃紫</t>
+          <t>Conton Candy</t>
         </is>
       </c>
       <c r="I43" t="inlineStr"/>
@@ -8739,28 +8741,28 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>正反対な君と僕 第2期</t>
+          <t>青春ブタ野郎はサンタクロースの夢を見ない</t>
         </is>
       </c>
       <c r="D44" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F44" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>猫じゃらし</t>
+          <t>水平線は僕の古傷</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>7co</t>
+          <t>広川卯月、赤城郁実、姫路紗良、霧島透子</t>
         </is>
       </c>
       <c r="I44" t="inlineStr"/>
@@ -8787,7 +8789,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F45" t="n">
@@ -8795,12 +8797,12 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>ピュア feat. 橋本絵莉子</t>
+          <t>メガネを外して</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>PAS TASTA</t>
+          <t>乃紫</t>
         </is>
       </c>
       <c r="I45" t="inlineStr"/>
@@ -8819,7 +8821,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>対ありでした。～お嬢さまは格闘ゲームなんてしない～</t>
+          <t>正反対な君と僕 第2期</t>
         </is>
       </c>
       <c r="D46" t="b">
@@ -8831,16 +8833,16 @@
         </is>
       </c>
       <c r="F46" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>命短し対する乙女よ</t>
+          <t>猫じゃらし</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>花冷え。</t>
+          <t>7co</t>
         </is>
       </c>
       <c r="I46" t="inlineStr"/>
@@ -8859,7 +8861,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>対ありでした。～お嬢さまは格闘ゲームなんてしない～</t>
+          <t>正反対な君と僕 第2期</t>
         </is>
       </c>
       <c r="D47" t="b">
@@ -8875,12 +8877,12 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>NEW GAME</t>
+          <t>ピュア feat. 橋本絵莉子</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>halca</t>
+          <t>PAS TASTA</t>
         </is>
       </c>
       <c r="I47" t="inlineStr"/>
@@ -8899,7 +8901,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>追放された転生重騎士はゲーム知識で無双する</t>
+          <t>対ありでした。～お嬢さまは格闘ゲームなんてしない～</t>
         </is>
       </c>
       <c r="D48" t="b">
@@ -8915,12 +8917,12 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Awake</t>
+          <t>命短し対する乙女よ</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>SPYAIR</t>
+          <t>花冷え。</t>
         </is>
       </c>
       <c r="I48" t="inlineStr"/>
@@ -8939,7 +8941,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>鉄鍋のジャン！</t>
+          <t>対ありでした。～お嬢さまは格闘ゲームなんてしない～</t>
         </is>
       </c>
       <c r="D49" t="b">
@@ -8947,7 +8949,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F49" t="n">
@@ -8955,12 +8957,12 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>火宴</t>
+          <t>NEW GAME</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>原因は自分にある。</t>
+          <t>halca</t>
         </is>
       </c>
       <c r="I49" t="inlineStr"/>
@@ -8979,7 +8981,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>手札が多めのビクトリア</t>
+          <t>追放された転生重騎士はゲーム知識で無双する</t>
         </is>
       </c>
       <c r="D50" t="b">
@@ -8987,7 +8989,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F50" t="n">
@@ -8995,12 +8997,12 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>縁のつき</t>
+          <t>Awake</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>KI_EN</t>
+          <t>SPYAIR</t>
         </is>
       </c>
       <c r="I50" t="inlineStr"/>
@@ -9019,7 +9021,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>転校先の清楚可憐な美少女が、昔男子と思って一緒に遊んだ幼馴染だった件</t>
+          <t>鉄鍋のジャン！</t>
         </is>
       </c>
       <c r="D51" t="b">
@@ -9035,12 +9037,12 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>夏に重ねて</t>
+          <t>火宴</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>DIALOGUE+</t>
+          <t>原因は自分にある。</t>
         </is>
       </c>
       <c r="I51" t="inlineStr"/>
@@ -9059,7 +9061,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>天は赤い河のほとり</t>
+          <t>手札が多めのビクトリア</t>
         </is>
       </c>
       <c r="D52" t="b">
@@ -9067,7 +9069,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F52" t="n">
@@ -9075,12 +9077,12 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>暁の空</t>
+          <t>縁のつき</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>七海ひろき</t>
+          <t>KI_EN</t>
         </is>
       </c>
       <c r="I52" t="inlineStr"/>
@@ -9099,7 +9101,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>天幕のジャードゥーガル</t>
+          <t>転校先の清楚可憐な美少女が、昔男子と思って一緒に遊んだ幼馴染だった件</t>
         </is>
       </c>
       <c r="D53" t="b">
@@ -9115,12 +9117,12 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>Stella</t>
+          <t>夏に重ねて</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>SEKAI NO OWARI</t>
+          <t>DIALOGUE+</t>
         </is>
       </c>
       <c r="I53" t="inlineStr"/>
@@ -9139,7 +9141,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>盗掘王</t>
+          <t>天は赤い河のほとり</t>
         </is>
       </c>
       <c r="D54" t="b">
@@ -9155,12 +9157,12 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>SHOW DOWN</t>
+          <t>暁の空</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>QWER</t>
+          <t>七海ひろき</t>
         </is>
       </c>
       <c r="I54" t="inlineStr"/>
@@ -9179,7 +9181,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>透明な夜に駆ける君と、目に見えない恋をした。</t>
+          <t>天幕のジャードゥーガル</t>
         </is>
       </c>
       <c r="D55" t="b">
@@ -9195,12 +9197,12 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>ひとひら</t>
+          <t>Stella</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>秦基博</t>
+          <t>SEKAI NO OWARI</t>
         </is>
       </c>
       <c r="I55" t="inlineStr"/>
@@ -9219,7 +9221,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>透明な夜に駆ける君と、目に見えない恋をした。</t>
+          <t>盗掘王</t>
         </is>
       </c>
       <c r="D56" t="b">
@@ -9227,7 +9229,7 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F56" t="n">
@@ -9235,12 +9237,12 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>光</t>
+          <t>SHOW DOWN</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>櫻井優衣</t>
+          <t>QWER</t>
         </is>
       </c>
       <c r="I56" t="inlineStr"/>
@@ -9259,7 +9261,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>トミカとトム</t>
+          <t>透明な夜に駆ける君と、目に見えない恋をした。</t>
         </is>
       </c>
       <c r="D57" t="b">
@@ -9267,7 +9269,7 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>主題歌</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F57" t="n">
@@ -9275,12 +9277,12 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>きみのたからもの</t>
+          <t>ひとひら</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>May J.</t>
+          <t>秦基博</t>
         </is>
       </c>
       <c r="I57" t="inlineStr"/>
@@ -9299,7 +9301,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>二十世紀電氣目録-ユーレカ・エヴリカ-</t>
+          <t>透明な夜に駆ける君と、目に見えない恋をした。</t>
         </is>
       </c>
       <c r="D58" t="b">
@@ -9307,7 +9309,7 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F58" t="n">
@@ -9315,12 +9317,12 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>ユーレカ・エヴリカ</t>
+          <t>光</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>五阿弥ルナ</t>
+          <t>櫻井優衣</t>
         </is>
       </c>
       <c r="I58" t="inlineStr"/>
@@ -9339,7 +9341,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>パイの実 おしの森へようこそ！</t>
+          <t>トミカとトム</t>
         </is>
       </c>
       <c r="D59" t="b">
@@ -9355,12 +9357,12 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>パイしか勝たん！推しの森活</t>
+          <t>きみのたからもの</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>安保心結</t>
+          <t>May J.</t>
         </is>
       </c>
       <c r="I59" t="inlineStr"/>
@@ -9379,7 +9381,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>刃牙道 第2クール</t>
+          <t>二十世紀電氣目録-ユーレカ・エヴリカ-</t>
         </is>
       </c>
       <c r="D60" t="b">
@@ -9395,12 +9397,12 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>フルボコ</t>
+          <t>ユーレカ・エヴリカ</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>WANIMA</t>
+          <t>五阿弥ルナ</t>
         </is>
       </c>
       <c r="I60" t="inlineStr"/>
@@ -9419,7 +9421,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>刃牙道 第2クール</t>
+          <t>パイの実 おしの森へようこそ！</t>
         </is>
       </c>
       <c r="D61" t="b">
@@ -9427,20 +9429,20 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>主題歌</t>
         </is>
       </c>
       <c r="F61" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>六ノ輪</t>
+          <t>パイしか勝たん！推しの森活</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>Chevon</t>
+          <t>安保心結</t>
         </is>
       </c>
       <c r="I61" t="inlineStr"/>
@@ -9467,7 +9469,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F62" t="n">
@@ -9475,12 +9477,12 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>Mountain Top</t>
+          <t>フルボコ</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>Novel Core</t>
+          <t>WANIMA</t>
         </is>
       </c>
       <c r="I62" t="inlineStr"/>
@@ -9507,7 +9509,7 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F63" t="n">
@@ -9515,12 +9517,12 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>KATANA</t>
+          <t>六ノ輪</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>三代目 J SOUL BROTHERS</t>
+          <t>Chevon</t>
         </is>
       </c>
       <c r="I63" t="inlineStr"/>
@@ -9539,7 +9541,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>花ざかりの君たちへ 第2期</t>
+          <t>刃牙道 第2クール</t>
         </is>
       </c>
       <c r="D64" t="b">
@@ -9547,7 +9549,7 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F64" t="n">
@@ -9555,12 +9557,12 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>FLASHBULB</t>
+          <t>Mountain Top</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>Omoinotake</t>
+          <t>Novel Core</t>
         </is>
       </c>
       <c r="I64" t="inlineStr"/>
@@ -9579,7 +9581,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>花ざかりの君たちへ 第2期</t>
+          <t>刃牙道 第2クール</t>
         </is>
       </c>
       <c r="D65" t="b">
@@ -9591,16 +9593,16 @@
         </is>
       </c>
       <c r="F65" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>花束</t>
+          <t>KATANA</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>Omoinotake</t>
+          <t>三代目 J SOUL BROTHERS</t>
         </is>
       </c>
       <c r="I65" t="inlineStr"/>
@@ -9619,7 +9621,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>ヒロイン？聖女？いいえ、オールワークスメイドです（誇）！</t>
+          <t>花ざかりの君たちへ 第2期</t>
         </is>
       </c>
       <c r="D66" t="b">
@@ -9635,12 +9637,12 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>マデュアル↔ハート</t>
+          <t>FLASHBULB</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>メロディ・ウェーブ(CV：宮本侑芽) ルシアナ・ルトルバーグ(CV：大久保瑠美)</t>
+          <t>Omoinotake</t>
         </is>
       </c>
       <c r="I66" t="inlineStr"/>
@@ -9659,7 +9661,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>ヒロイン？聖女？いいえ、オールワークスメイドです（誇）！</t>
+          <t>花ざかりの君たちへ 第2期</t>
         </is>
       </c>
       <c r="D67" t="b">
@@ -9675,12 +9677,12 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>ハンドメイド</t>
+          <t>花束</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>仲村宗悟</t>
+          <t>Omoinotake</t>
         </is>
       </c>
       <c r="I67" t="inlineStr"/>
@@ -9699,7 +9701,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>ブチ切れ令嬢は報復を誓いました。 ～魔導書の力で祖国を叩き潰します～</t>
+          <t>ヒロイン？聖女？いいえ、オールワークスメイドです（誇）！</t>
         </is>
       </c>
       <c r="D68" t="b">
@@ -9715,12 +9717,12 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>Q.E.D.</t>
+          <t>マデュアル↔ハート</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>小倉唯</t>
+          <t>メロディ・ウェーブ(CV：宮本侑芽) ルシアナ・ルトルバーグ(CV：大久保瑠美)</t>
         </is>
       </c>
       <c r="I68" t="inlineStr"/>
@@ -9739,7 +9741,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>ブチ切れ令嬢は報復を誓いました。 ～魔導書の力で祖国を叩き潰します～</t>
+          <t>ヒロイン？聖女？いいえ、オールワークスメイドです（誇）！</t>
         </is>
       </c>
       <c r="D69" t="b">
@@ -9755,12 +9757,12 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>グッバイ・ララバイ</t>
+          <t>ハンドメイド</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>大西亜玖璃</t>
+          <t>仲村宗悟</t>
         </is>
       </c>
       <c r="I69" t="inlineStr"/>
@@ -9779,7 +9781,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>ふつつかな悪女ではございますが～雛宮蝶鼠とりかえ伝～</t>
+          <t>ブチ切れ令嬢は報復を誓いました。 ～魔導書の力で祖国を叩き潰します～</t>
         </is>
       </c>
       <c r="D70" t="b">
@@ -9795,12 +9797,12 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>Sunny</t>
+          <t>Q.E.D.</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>milet</t>
+          <t>小倉唯</t>
         </is>
       </c>
       <c r="I70" t="inlineStr"/>
@@ -9819,7 +9821,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>BLACK TORCH</t>
+          <t>ブチ切れ令嬢は報復を誓いました。 ～魔導書の力で祖国を叩き潰します～</t>
         </is>
       </c>
       <c r="D71" t="b">
@@ -9827,7 +9829,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F71" t="n">
@@ -9835,12 +9837,12 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>FREEZE ME UP</t>
+          <t>グッバイ・ララバイ</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>SiM</t>
+          <t>大西亜玖璃</t>
         </is>
       </c>
       <c r="I71" t="inlineStr"/>
@@ -9859,7 +9861,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>BLACK TORCH</t>
+          <t>ふつつかな悪女ではございますが～雛宮蝶鼠とりかえ伝～</t>
         </is>
       </c>
       <c r="D72" t="b">
@@ -9867,7 +9869,7 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F72" t="n">
@@ -9875,12 +9877,12 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>Groooovy</t>
+          <t>Sunny</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>I Don't Like Mondays.</t>
+          <t>milet</t>
         </is>
       </c>
       <c r="I72" t="inlineStr"/>
@@ -9899,7 +9901,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>プラノサウルス ガチコセイブツ部</t>
+          <t>BLACK TORCH</t>
         </is>
       </c>
       <c r="D73" t="b">
@@ -9907,7 +9909,7 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>主題歌</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F73" t="n">
@@ -9915,12 +9917,12 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>ガチde古生</t>
+          <t>FREEZE ME UP</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>リンクルプラネット</t>
+          <t>SiM</t>
         </is>
       </c>
       <c r="I73" t="inlineStr"/>
@@ -9939,7 +9941,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>ヘルモード ～やり込み好きのゲーマーは廃設定の異世界で無双する～ 2nd Season</t>
+          <t>BLACK TORCH</t>
         </is>
       </c>
       <c r="D74" t="b">
@@ -9947,7 +9949,7 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F74" t="n">
@@ -9955,12 +9957,12 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>○✕△□</t>
+          <t>Groooovy</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>浪漫派マシュマロ</t>
+          <t>I Don't Like Mondays.</t>
         </is>
       </c>
       <c r="I74" t="inlineStr"/>
@@ -9979,7 +9981,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>北斗の拳 拳王軍ザコたちの挽歌 第2クール</t>
+          <t>プラノサウルス ガチコセイブツ部</t>
         </is>
       </c>
       <c r="D75" t="b">
@@ -9987,7 +9989,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>主題歌</t>
         </is>
       </c>
       <c r="F75" t="n">
@@ -9995,12 +9997,12 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>Blacker Co., Ltd.</t>
+          <t>ガチde古生</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>イツカ▶</t>
+          <t>リンクルプラネット</t>
         </is>
       </c>
       <c r="I75" t="inlineStr"/>
@@ -10019,7 +10021,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>北斗の拳 拳王軍ザコたちの挽歌 第2クール</t>
+          <t>ヘルモード ～やり込み好きのゲーマーは廃設定の異世界で無双する～ 2nd Season</t>
         </is>
       </c>
       <c r="D76" t="b">
@@ -10027,7 +10029,7 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F76" t="n">
@@ -10035,12 +10037,12 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>Elegy of the Enemies</t>
+          <t>○✕△□</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>The Canbellz</t>
+          <t>浪漫派マシュマロ</t>
         </is>
       </c>
       <c r="I76" t="inlineStr"/>
@@ -10067,20 +10069,20 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F77" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>白い蝶が飛んだら</t>
+          <t>Blacker Co., Ltd.</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>イツカ▶ feat. Dr. Washington | Special Guest Guitar:Tsuyoshi Ujiki</t>
+          <t>イツカ▶</t>
         </is>
       </c>
       <c r="I77" t="inlineStr"/>
@@ -10099,7 +10101,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>炎の闘球女 ドッジ弾子</t>
+          <t>北斗の拳 拳王軍ザコたちの挽歌 第2クール</t>
         </is>
       </c>
       <c r="D78" t="b">
@@ -10107,7 +10109,7 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F78" t="n">
@@ -10115,12 +10117,12 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>会心の一劇</t>
+          <t>Elegy of the Enemies</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>ももいろクローバーZ</t>
+          <t>The Canbellz</t>
         </is>
       </c>
       <c r="I78" t="inlineStr"/>
@@ -10139,7 +10141,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>炎の闘球女 ドッジ弾子</t>
+          <t>北斗の拳 拳王軍ザコたちの挽歌 第2クール</t>
         </is>
       </c>
       <c r="D79" t="b">
@@ -10151,16 +10153,16 @@
         </is>
       </c>
       <c r="F79" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>Welcome to あざとさワールド</t>
+          <t>白い蝶が飛んだら</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>i☆Ris</t>
+          <t>イツカ▶ feat. Dr. Washington | Special Guest Guitar:Tsuyoshi Ujiki</t>
         </is>
       </c>
       <c r="I79" t="inlineStr"/>
@@ -10179,7 +10181,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>魔法少女リリカルなのは EXCEEDS Gun Blaze Vengeance</t>
+          <t>炎の闘球女 ドッジ弾子</t>
         </is>
       </c>
       <c r="D80" t="b">
@@ -10195,12 +10197,12 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>CRIMSON BULLET</t>
+          <t>会心の一劇</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>水樹奈々</t>
+          <t>ももいろクローバーZ</t>
         </is>
       </c>
       <c r="I80" t="inlineStr"/>
@@ -10219,7 +10221,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>魔法少女リリカルなのは EXCEEDS Gun Blaze Vengeance</t>
+          <t>炎の闘球女 ドッジ弾子</t>
         </is>
       </c>
       <c r="D81" t="b">
@@ -10235,12 +10237,12 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>Ephemeral</t>
+          <t>Welcome to あざとさワールド</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>青木陽菜</t>
+          <t>i☆Ris</t>
         </is>
       </c>
       <c r="I81" t="inlineStr"/>
@@ -10259,7 +10261,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>無自覚聖女は今日も無意識に力を垂れ流す</t>
+          <t>魔法少女リリカルなのは EXCEEDS Gun Blaze Vengeance</t>
         </is>
       </c>
       <c r="D82" t="b">
@@ -10275,12 +10277,12 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>Windmaker</t>
+          <t>CRIMSON BULLET</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>花耶</t>
+          <t>水樹奈々</t>
         </is>
       </c>
       <c r="I82" t="inlineStr"/>
@@ -10299,7 +10301,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>無自覚聖女は今日も無意識に力を垂れ流す</t>
+          <t>魔法少女リリカルなのは EXCEEDS Gun Blaze Vengeance</t>
         </is>
       </c>
       <c r="D83" t="b">
@@ -10315,12 +10317,12 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>アンノウンミー</t>
+          <t>Ephemeral</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>ウタヒメドリーム オールスターズ【夢咲いぶき（CV:山﨑玲奈） 桜木舞華（CV:鈴木杏奈） 真白清美（CV:其原有沙） HiREN（CV:花耶） 水月ひかり（CV:礒部花凜） 高木凛（CV:鷲見友美ジェナ） 萩原ひまわり（CV:倉知玲鳳） SAKURAKO（CV:竹内夢）】</t>
+          <t>青木陽菜</t>
         </is>
       </c>
       <c r="I83" t="inlineStr"/>
@@ -10339,7 +10341,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>無職転生Ⅲ ～異世界行ったら本気だす～</t>
+          <t>無自覚聖女は今日も無意識に力を垂れ流す</t>
         </is>
       </c>
       <c r="D84" t="b">
@@ -10355,12 +10357,12 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>決意の唄</t>
+          <t>Windmaker</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>大原ゆい子</t>
+          <t>花耶</t>
         </is>
       </c>
       <c r="I84" t="inlineStr"/>
@@ -10379,7 +10381,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>無職転生Ⅲ ～異世界行ったら本気だす～</t>
+          <t>無自覚聖女は今日も無意識に力を垂れ流す</t>
         </is>
       </c>
       <c r="D85" t="b">
@@ -10395,12 +10397,12 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>祈り、終われば</t>
+          <t>アンノウンミー</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>中島美嘉</t>
+          <t>ウタヒメドリーム オールスターズ【夢咲いぶき（CV:山﨑玲奈） 桜木舞華（CV:鈴木杏奈） 真白清美（CV:其原有沙） HiREN（CV:花耶） 水月ひかり（CV:礒部花凜） 高木凛（CV:鷲見友美ジェナ） 萩原ひまわり（CV:倉知玲鳳） SAKURAKO（CV:竹内夢）】</t>
         </is>
       </c>
       <c r="I85" t="inlineStr"/>
@@ -10419,7 +10421,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>メビウス・ダスト</t>
+          <t>無職転生Ⅲ ～異世界行ったら本気だす～</t>
         </is>
       </c>
       <c r="D86" t="b">
@@ -10435,12 +10437,12 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>メビウス</t>
+          <t>決意の唄</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>家入レオ</t>
+          <t>大原ゆい子</t>
         </is>
       </c>
       <c r="I86" t="inlineStr"/>
@@ -10459,7 +10461,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>メビウス・ダスト</t>
+          <t>無職転生Ⅲ ～異世界行ったら本気だす～</t>
         </is>
       </c>
       <c r="D87" t="b">
@@ -10475,12 +10477,12 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>ジレンマ</t>
+          <t>祈り、終われば</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>冨岡愛</t>
+          <t>中島美嘉</t>
         </is>
       </c>
       <c r="I87" t="inlineStr"/>
@@ -10499,7 +10501,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>ヤニねこ</t>
+          <t>メビウス・ダスト</t>
         </is>
       </c>
       <c r="D88" t="b">
@@ -10515,12 +10517,12 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>なんもねえ</t>
+          <t>メビウス</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>忘れらんねえよ</t>
+          <t>家入レオ</t>
         </is>
       </c>
       <c r="I88" t="inlineStr"/>
@@ -10539,7 +10541,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>幼女戦記Ⅱ</t>
+          <t>メビウス・ダスト</t>
         </is>
       </c>
       <c r="D89" t="b">
@@ -10547,7 +10549,7 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F89" t="n">
@@ -10555,12 +10557,12 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>Why? RED induction</t>
+          <t>ジレンマ</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>MYTH &amp; ROID</t>
+          <t>冨岡愛</t>
         </is>
       </c>
       <c r="I89" t="inlineStr"/>
@@ -10579,7 +10581,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>幼女戦記Ⅱ</t>
+          <t>ヤニねこ</t>
         </is>
       </c>
       <c r="D90" t="b">
@@ -10587,7 +10589,7 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F90" t="n">
@@ -10595,12 +10597,12 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>Weiter! Weiter!</t>
+          <t>なんもねえ</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>ターニャ・デグレチャフ（CV：悠木碧）</t>
+          <t>忘れらんねえよ</t>
         </is>
       </c>
       <c r="I90" t="inlineStr"/>
@@ -10619,7 +10621,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>鎧真伝サムライトルーパー 第2クール</t>
+          <t>幼女戦記Ⅱ</t>
         </is>
       </c>
       <c r="D91" t="b">
@@ -10635,12 +10637,12 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>YOAKE</t>
+          <t>Why? RED induction</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>blank paper</t>
+          <t>MYTH &amp; ROID</t>
         </is>
       </c>
       <c r="I91" t="inlineStr"/>
@@ -10659,7 +10661,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>鎧真伝サムライトルーパー 第2クール</t>
+          <t>幼女戦記Ⅱ</t>
         </is>
       </c>
       <c r="D92" t="b">
@@ -10667,20 +10669,20 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F92" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>BAD遺伝子</t>
+          <t>Weiter! Weiter!</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>Dannie May</t>
+          <t>ターニャ・デグレチャフ（CV：悠木碧）</t>
         </is>
       </c>
       <c r="I92" t="inlineStr"/>
@@ -10707,7 +10709,7 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F93" t="n">
@@ -10715,12 +10717,12 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>POWER</t>
+          <t>YOAKE</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>ONE OR EIGHT</t>
+          <t>blank paper</t>
         </is>
       </c>
       <c r="I93" t="inlineStr"/>
@@ -10747,7 +10749,7 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F94" t="n">
@@ -10755,12 +10757,12 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>ばけもん</t>
+          <t>BAD遺伝子</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>カラノア</t>
+          <t>Dannie May</t>
         </is>
       </c>
       <c r="I94" t="inlineStr"/>
@@ -10779,7 +10781,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>落第賢者の学院無双～二度目の転生、Sランクチート魔術師冒険録～</t>
+          <t>鎧真伝サムライトルーパー 第2クール</t>
         </is>
       </c>
       <c r="D95" t="b">
@@ -10787,7 +10789,7 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F95" t="n">
@@ -10795,12 +10797,12 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>＋ENCOUNT</t>
+          <t>POWER</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>FLOW</t>
+          <t>ONE OR EIGHT</t>
         </is>
       </c>
       <c r="I95" t="inlineStr"/>
@@ -10819,7 +10821,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>落第賢者の学院無双～二度目の転生、Sランクチート魔術師冒険録～</t>
+          <t>鎧真伝サムライトルーパー 第2クール</t>
         </is>
       </c>
       <c r="D96" t="b">
@@ -10831,16 +10833,16 @@
         </is>
       </c>
       <c r="F96" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>憧憬</t>
+          <t>ばけもん</t>
         </is>
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>TrySail</t>
+          <t>カラノア</t>
         </is>
       </c>
       <c r="I96" t="inlineStr"/>
@@ -10859,7 +10861,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>領民0人スタートの辺境領主様</t>
+          <t>落第賢者の学院無双～二度目の転生、Sランクチート魔術師冒険録～</t>
         </is>
       </c>
       <c r="D97" t="b">
@@ -10875,12 +10877,12 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>Wonder</t>
+          <t>＋ENCOUNT</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>CROWN HEAD</t>
+          <t>FLOW</t>
         </is>
       </c>
       <c r="I97" t="inlineStr"/>
@@ -10899,7 +10901,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>領民0人スタートの辺境領主様</t>
+          <t>落第賢者の学院無双～二度目の転生、Sランクチート魔術師冒険録～</t>
         </is>
       </c>
       <c r="D98" t="b">
@@ -10915,12 +10917,12 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>星降る夜の約束</t>
+          <t>憧憬</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>花耶</t>
+          <t>TrySail</t>
         </is>
       </c>
       <c r="I98" t="inlineStr"/>
@@ -10939,7 +10941,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>令和のダラさん</t>
+          <t>領民0人スタートの辺境領主様</t>
         </is>
       </c>
       <c r="D99" t="b">
@@ -10955,12 +10957,12 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>ダラダラ♡ダンシング</t>
+          <t>Wonder</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>ダラさん（CV：田村睦心） 三⼗⽊⾕⽇向（CV：津田美波） 三⼗⽊⾕薫（CV：寺澤百花） ナレーション（CV：てらそままさき）</t>
+          <t>CROWN HEAD</t>
         </is>
       </c>
       <c r="I99" t="inlineStr"/>
@@ -10979,7 +10981,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>令和のダラさん</t>
+          <t>領民0人スタートの辺境領主様</t>
         </is>
       </c>
       <c r="D100" t="b">
@@ -10995,12 +10997,12 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>ひなたぼっこ</t>
+          <t>星降る夜の約束</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>REIRIE</t>
+          <t>花耶</t>
         </is>
       </c>
       <c r="I100" t="inlineStr"/>
@@ -11019,7 +11021,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>LV999の村人</t>
+          <t>令和のダラさん</t>
         </is>
       </c>
       <c r="D101" t="b">
@@ -11035,12 +11037,12 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>Not a Hero</t>
+          <t>ダラダラ♡ダンシング</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>藍月なくる&amp;棗いつき</t>
+          <t>ダラさん（CV：田村睦心） 三⼗⽊⾕⽇向（CV：津田美波） 三⼗⽊⾕薫（CV：寺澤百花） ナレーション（CV：てらそままさき）</t>
         </is>
       </c>
       <c r="I101" t="inlineStr"/>
@@ -11059,7 +11061,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>LV999の村人</t>
+          <t>令和のダラさん</t>
         </is>
       </c>
       <c r="D102" t="b">
@@ -11075,12 +11077,12 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>ひなたぼっこ</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>ゆきむら。</t>
+          <t>REIRIE</t>
         </is>
       </c>
       <c r="I102" t="inlineStr"/>
@@ -11099,7 +11101,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>ワールド イズ ダンシング</t>
+          <t>LV999の村人</t>
         </is>
       </c>
       <c r="D103" t="b">
@@ -11115,12 +11117,12 @@
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>終宵</t>
+          <t>Not a Hero</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>マカロニえんぴつ</t>
+          <t>藍月なくる&amp;棗いつき</t>
         </is>
       </c>
       <c r="I103" t="inlineStr"/>
@@ -11130,16 +11132,16 @@
     </row>
     <row r="104">
       <c r="A104" t="n">
-        <v>5947</v>
+        <v>5806</v>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>2026秋アニメ</t>
+          <t>2026夏アニメ</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>帰還者の魔法は特別です 第2期</t>
+          <t>LV999の村人</t>
         </is>
       </c>
       <c r="D104" t="b">
@@ -11147,7 +11149,7 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F104" t="n">
@@ -11155,12 +11157,12 @@
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>Sorrow</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>FLOW</t>
+          <t>ゆきむら。</t>
         </is>
       </c>
       <c r="I104" t="inlineStr"/>
@@ -11170,16 +11172,16 @@
     </row>
     <row r="105">
       <c r="A105" t="n">
-        <v>5947</v>
+        <v>5806</v>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>2026秋アニメ</t>
+          <t>2026夏アニメ</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>獣王武神ダンデヴァイン</t>
+          <t>ワールド イズ ダンシング</t>
         </is>
       </c>
       <c r="D105" t="b">
@@ -11195,12 +11197,12 @@
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>曲名未発表</t>
+          <t>終宵</t>
         </is>
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>西川貴教</t>
+          <t>マカロニえんぴつ</t>
         </is>
       </c>
       <c r="I105" t="inlineStr"/>
@@ -11219,7 +11221,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>転生した大聖女は、聖女であることをひた隠す</t>
+          <t>帰還者の魔法は特別です 第2期</t>
         </is>
       </c>
       <c r="D106" t="b">
@@ -11235,12 +11237,12 @@
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>Flare of Soul</t>
+          <t>Sorrow</t>
         </is>
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>花耶</t>
+          <t>FLOW</t>
         </is>
       </c>
       <c r="I106" t="inlineStr"/>
@@ -11259,7 +11261,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>転生した大聖女は、聖女であることをひた隠す</t>
+          <t>獣王武神ダンデヴァイン</t>
         </is>
       </c>
       <c r="D107" t="b">
@@ -11267,7 +11269,7 @@
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F107" t="n">
@@ -11275,12 +11277,12 @@
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>STELLAR</t>
+          <t>曲名未発表</t>
         </is>
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>ウタヒメドリーム オールスターズ</t>
+          <t>西川貴教</t>
         </is>
       </c>
       <c r="I107" t="inlineStr"/>
@@ -11299,7 +11301,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>魔法少女育成計画restart</t>
+          <t>転生した大聖女は、聖女であることをひた隠す</t>
         </is>
       </c>
       <c r="D108" t="b">
@@ -11315,12 +11317,12 @@
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>No tears here</t>
+          <t>Flare of Soul</t>
         </is>
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>茅原実里</t>
+          <t>花耶</t>
         </is>
       </c>
       <c r="I108" t="inlineStr"/>
@@ -11328,6 +11330,86 @@
       <c r="K108" t="inlineStr"/>
       <c r="L108" t="inlineStr"/>
     </row>
+    <row r="109">
+      <c r="A109" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>転生した大聖女は、聖女であることをひた隠す</t>
+        </is>
+      </c>
+      <c r="D109" t="b">
+        <v>0</v>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>ED</t>
+        </is>
+      </c>
+      <c r="F109" t="n">
+        <v>1</v>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>STELLAR</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>ウタヒメドリーム オールスターズ</t>
+        </is>
+      </c>
+      <c r="I109" t="inlineStr"/>
+      <c r="J109" t="inlineStr"/>
+      <c r="K109" t="inlineStr"/>
+      <c r="L109" t="inlineStr"/>
+    </row>
+    <row r="110">
+      <c r="A110" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>魔法少女育成計画restart</t>
+        </is>
+      </c>
+      <c r="D110" t="b">
+        <v>0</v>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="F110" t="n">
+        <v>1</v>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>No tears here</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>茅原実里</t>
+        </is>
+      </c>
+      <c r="I110" t="inlineStr"/>
+      <c r="J110" t="inlineStr"/>
+      <c r="K110" t="inlineStr"/>
+      <c r="L110" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
auto: anime list update 2026-06-13
</commit_message>
<xml_diff>
--- a/data/anime_list.xlsx
+++ b/data/anime_list.xlsx
@@ -6985,7 +6985,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L110"/>
+  <dimension ref="A1:O110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7046,6 +7046,21 @@
       </c>
       <c r="L1" t="inlineStr">
         <is>
+          <t>anime_youtube_url</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>anime_youtube_views</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>anime_youtube_channel</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
           <t>last_searched_at</t>
         </is>
       </c>
@@ -7089,6 +7104,9 @@
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -7129,6 +7147,9 @@
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -7169,6 +7190,9 @@
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -7209,6 +7233,9 @@
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -7249,6 +7276,9 @@
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -7289,6 +7319,9 @@
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -7329,6 +7362,9 @@
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -7369,6 +7405,9 @@
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -7409,6 +7448,9 @@
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -7449,6 +7491,9 @@
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -7489,6 +7534,9 @@
       <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -7529,6 +7577,9 @@
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -7569,6 +7620,9 @@
       <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="inlineStr"/>
+      <c r="O14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -7609,6 +7663,9 @@
       <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="inlineStr"/>
+      <c r="O15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -7649,6 +7706,9 @@
       <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" t="inlineStr"/>
+      <c r="O16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -7689,6 +7749,9 @@
       <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="inlineStr"/>
+      <c r="O17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -7729,6 +7792,9 @@
       <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="inlineStr"/>
+      <c r="O18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -7769,6 +7835,9 @@
       <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" t="inlineStr"/>
+      <c r="O19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -7809,6 +7878,9 @@
       <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr"/>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="inlineStr"/>
+      <c r="O20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -7849,6 +7921,9 @@
       <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" t="inlineStr"/>
+      <c r="O21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -7889,6 +7964,9 @@
       <c r="J22" t="inlineStr"/>
       <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr"/>
+      <c r="M22" t="inlineStr"/>
+      <c r="N22" t="inlineStr"/>
+      <c r="O22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -7929,6 +8007,9 @@
       <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr"/>
+      <c r="M23" t="inlineStr"/>
+      <c r="N23" t="inlineStr"/>
+      <c r="O23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -7969,6 +8050,9 @@
       <c r="J24" t="inlineStr"/>
       <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr"/>
+      <c r="M24" t="inlineStr"/>
+      <c r="N24" t="inlineStr"/>
+      <c r="O24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -8009,6 +8093,9 @@
       <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr"/>
+      <c r="M25" t="inlineStr"/>
+      <c r="N25" t="inlineStr"/>
+      <c r="O25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -8049,6 +8136,9 @@
       <c r="J26" t="inlineStr"/>
       <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr"/>
+      <c r="M26" t="inlineStr"/>
+      <c r="N26" t="inlineStr"/>
+      <c r="O26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -8089,6 +8179,9 @@
       <c r="J27" t="inlineStr"/>
       <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr"/>
+      <c r="M27" t="inlineStr"/>
+      <c r="N27" t="inlineStr"/>
+      <c r="O27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -8129,6 +8222,9 @@
       <c r="J28" t="inlineStr"/>
       <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr"/>
+      <c r="M28" t="inlineStr"/>
+      <c r="N28" t="inlineStr"/>
+      <c r="O28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -8169,6 +8265,9 @@
       <c r="J29" t="inlineStr"/>
       <c r="K29" t="inlineStr"/>
       <c r="L29" t="inlineStr"/>
+      <c r="M29" t="inlineStr"/>
+      <c r="N29" t="inlineStr"/>
+      <c r="O29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -8209,6 +8308,9 @@
       <c r="J30" t="inlineStr"/>
       <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr"/>
+      <c r="M30" t="inlineStr"/>
+      <c r="N30" t="inlineStr"/>
+      <c r="O30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -8249,6 +8351,9 @@
       <c r="J31" t="inlineStr"/>
       <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr"/>
+      <c r="M31" t="inlineStr"/>
+      <c r="N31" t="inlineStr"/>
+      <c r="O31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -8289,6 +8394,9 @@
       <c r="J32" t="inlineStr"/>
       <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr"/>
+      <c r="M32" t="inlineStr"/>
+      <c r="N32" t="inlineStr"/>
+      <c r="O32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -8329,6 +8437,9 @@
       <c r="J33" t="inlineStr"/>
       <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr"/>
+      <c r="M33" t="inlineStr"/>
+      <c r="N33" t="inlineStr"/>
+      <c r="O33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -8369,6 +8480,9 @@
       <c r="J34" t="inlineStr"/>
       <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr"/>
+      <c r="M34" t="inlineStr"/>
+      <c r="N34" t="inlineStr"/>
+      <c r="O34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -8409,6 +8523,9 @@
       <c r="J35" t="inlineStr"/>
       <c r="K35" t="inlineStr"/>
       <c r="L35" t="inlineStr"/>
+      <c r="M35" t="inlineStr"/>
+      <c r="N35" t="inlineStr"/>
+      <c r="O35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -8449,6 +8566,9 @@
       <c r="J36" t="inlineStr"/>
       <c r="K36" t="inlineStr"/>
       <c r="L36" t="inlineStr"/>
+      <c r="M36" t="inlineStr"/>
+      <c r="N36" t="inlineStr"/>
+      <c r="O36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -8489,6 +8609,9 @@
       <c r="J37" t="inlineStr"/>
       <c r="K37" t="inlineStr"/>
       <c r="L37" t="inlineStr"/>
+      <c r="M37" t="inlineStr"/>
+      <c r="N37" t="inlineStr"/>
+      <c r="O37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -8529,6 +8652,9 @@
       <c r="J38" t="inlineStr"/>
       <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr"/>
+      <c r="M38" t="inlineStr"/>
+      <c r="N38" t="inlineStr"/>
+      <c r="O38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -8569,6 +8695,9 @@
       <c r="J39" t="inlineStr"/>
       <c r="K39" t="inlineStr"/>
       <c r="L39" t="inlineStr"/>
+      <c r="M39" t="inlineStr"/>
+      <c r="N39" t="inlineStr"/>
+      <c r="O39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -8609,6 +8738,9 @@
       <c r="J40" t="inlineStr"/>
       <c r="K40" t="inlineStr"/>
       <c r="L40" t="inlineStr"/>
+      <c r="M40" t="inlineStr"/>
+      <c r="N40" t="inlineStr"/>
+      <c r="O40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -8649,6 +8781,9 @@
       <c r="J41" t="inlineStr"/>
       <c r="K41" t="inlineStr"/>
       <c r="L41" t="inlineStr"/>
+      <c r="M41" t="inlineStr"/>
+      <c r="N41" t="inlineStr"/>
+      <c r="O41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -8689,6 +8824,9 @@
       <c r="J42" t="inlineStr"/>
       <c r="K42" t="inlineStr"/>
       <c r="L42" t="inlineStr"/>
+      <c r="M42" t="inlineStr"/>
+      <c r="N42" t="inlineStr"/>
+      <c r="O42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -8729,6 +8867,9 @@
       <c r="J43" t="inlineStr"/>
       <c r="K43" t="inlineStr"/>
       <c r="L43" t="inlineStr"/>
+      <c r="M43" t="inlineStr"/>
+      <c r="N43" t="inlineStr"/>
+      <c r="O43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -8769,6 +8910,9 @@
       <c r="J44" t="inlineStr"/>
       <c r="K44" t="inlineStr"/>
       <c r="L44" t="inlineStr"/>
+      <c r="M44" t="inlineStr"/>
+      <c r="N44" t="inlineStr"/>
+      <c r="O44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -8809,6 +8953,9 @@
       <c r="J45" t="inlineStr"/>
       <c r="K45" t="inlineStr"/>
       <c r="L45" t="inlineStr"/>
+      <c r="M45" t="inlineStr"/>
+      <c r="N45" t="inlineStr"/>
+      <c r="O45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -8849,6 +8996,9 @@
       <c r="J46" t="inlineStr"/>
       <c r="K46" t="inlineStr"/>
       <c r="L46" t="inlineStr"/>
+      <c r="M46" t="inlineStr"/>
+      <c r="N46" t="inlineStr"/>
+      <c r="O46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -8889,6 +9039,9 @@
       <c r="J47" t="inlineStr"/>
       <c r="K47" t="inlineStr"/>
       <c r="L47" t="inlineStr"/>
+      <c r="M47" t="inlineStr"/>
+      <c r="N47" t="inlineStr"/>
+      <c r="O47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -8929,6 +9082,9 @@
       <c r="J48" t="inlineStr"/>
       <c r="K48" t="inlineStr"/>
       <c r="L48" t="inlineStr"/>
+      <c r="M48" t="inlineStr"/>
+      <c r="N48" t="inlineStr"/>
+      <c r="O48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -8969,6 +9125,9 @@
       <c r="J49" t="inlineStr"/>
       <c r="K49" t="inlineStr"/>
       <c r="L49" t="inlineStr"/>
+      <c r="M49" t="inlineStr"/>
+      <c r="N49" t="inlineStr"/>
+      <c r="O49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -9009,6 +9168,9 @@
       <c r="J50" t="inlineStr"/>
       <c r="K50" t="inlineStr"/>
       <c r="L50" t="inlineStr"/>
+      <c r="M50" t="inlineStr"/>
+      <c r="N50" t="inlineStr"/>
+      <c r="O50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -9049,6 +9211,9 @@
       <c r="J51" t="inlineStr"/>
       <c r="K51" t="inlineStr"/>
       <c r="L51" t="inlineStr"/>
+      <c r="M51" t="inlineStr"/>
+      <c r="N51" t="inlineStr"/>
+      <c r="O51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -9089,6 +9254,9 @@
       <c r="J52" t="inlineStr"/>
       <c r="K52" t="inlineStr"/>
       <c r="L52" t="inlineStr"/>
+      <c r="M52" t="inlineStr"/>
+      <c r="N52" t="inlineStr"/>
+      <c r="O52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -9129,6 +9297,9 @@
       <c r="J53" t="inlineStr"/>
       <c r="K53" t="inlineStr"/>
       <c r="L53" t="inlineStr"/>
+      <c r="M53" t="inlineStr"/>
+      <c r="N53" t="inlineStr"/>
+      <c r="O53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -9169,6 +9340,9 @@
       <c r="J54" t="inlineStr"/>
       <c r="K54" t="inlineStr"/>
       <c r="L54" t="inlineStr"/>
+      <c r="M54" t="inlineStr"/>
+      <c r="N54" t="inlineStr"/>
+      <c r="O54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -9209,6 +9383,9 @@
       <c r="J55" t="inlineStr"/>
       <c r="K55" t="inlineStr"/>
       <c r="L55" t="inlineStr"/>
+      <c r="M55" t="inlineStr"/>
+      <c r="N55" t="inlineStr"/>
+      <c r="O55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -9249,6 +9426,9 @@
       <c r="J56" t="inlineStr"/>
       <c r="K56" t="inlineStr"/>
       <c r="L56" t="inlineStr"/>
+      <c r="M56" t="inlineStr"/>
+      <c r="N56" t="inlineStr"/>
+      <c r="O56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -9289,6 +9469,9 @@
       <c r="J57" t="inlineStr"/>
       <c r="K57" t="inlineStr"/>
       <c r="L57" t="inlineStr"/>
+      <c r="M57" t="inlineStr"/>
+      <c r="N57" t="inlineStr"/>
+      <c r="O57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -9329,6 +9512,9 @@
       <c r="J58" t="inlineStr"/>
       <c r="K58" t="inlineStr"/>
       <c r="L58" t="inlineStr"/>
+      <c r="M58" t="inlineStr"/>
+      <c r="N58" t="inlineStr"/>
+      <c r="O58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -9369,6 +9555,9 @@
       <c r="J59" t="inlineStr"/>
       <c r="K59" t="inlineStr"/>
       <c r="L59" t="inlineStr"/>
+      <c r="M59" t="inlineStr"/>
+      <c r="N59" t="inlineStr"/>
+      <c r="O59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -9409,6 +9598,9 @@
       <c r="J60" t="inlineStr"/>
       <c r="K60" t="inlineStr"/>
       <c r="L60" t="inlineStr"/>
+      <c r="M60" t="inlineStr"/>
+      <c r="N60" t="inlineStr"/>
+      <c r="O60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -9449,6 +9641,9 @@
       <c r="J61" t="inlineStr"/>
       <c r="K61" t="inlineStr"/>
       <c r="L61" t="inlineStr"/>
+      <c r="M61" t="inlineStr"/>
+      <c r="N61" t="inlineStr"/>
+      <c r="O61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -9489,6 +9684,9 @@
       <c r="J62" t="inlineStr"/>
       <c r="K62" t="inlineStr"/>
       <c r="L62" t="inlineStr"/>
+      <c r="M62" t="inlineStr"/>
+      <c r="N62" t="inlineStr"/>
+      <c r="O62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -9529,6 +9727,9 @@
       <c r="J63" t="inlineStr"/>
       <c r="K63" t="inlineStr"/>
       <c r="L63" t="inlineStr"/>
+      <c r="M63" t="inlineStr"/>
+      <c r="N63" t="inlineStr"/>
+      <c r="O63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -9569,6 +9770,9 @@
       <c r="J64" t="inlineStr"/>
       <c r="K64" t="inlineStr"/>
       <c r="L64" t="inlineStr"/>
+      <c r="M64" t="inlineStr"/>
+      <c r="N64" t="inlineStr"/>
+      <c r="O64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -9609,6 +9813,9 @@
       <c r="J65" t="inlineStr"/>
       <c r="K65" t="inlineStr"/>
       <c r="L65" t="inlineStr"/>
+      <c r="M65" t="inlineStr"/>
+      <c r="N65" t="inlineStr"/>
+      <c r="O65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -9649,6 +9856,9 @@
       <c r="J66" t="inlineStr"/>
       <c r="K66" t="inlineStr"/>
       <c r="L66" t="inlineStr"/>
+      <c r="M66" t="inlineStr"/>
+      <c r="N66" t="inlineStr"/>
+      <c r="O66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -9689,6 +9899,9 @@
       <c r="J67" t="inlineStr"/>
       <c r="K67" t="inlineStr"/>
       <c r="L67" t="inlineStr"/>
+      <c r="M67" t="inlineStr"/>
+      <c r="N67" t="inlineStr"/>
+      <c r="O67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -9729,6 +9942,9 @@
       <c r="J68" t="inlineStr"/>
       <c r="K68" t="inlineStr"/>
       <c r="L68" t="inlineStr"/>
+      <c r="M68" t="inlineStr"/>
+      <c r="N68" t="inlineStr"/>
+      <c r="O68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -9769,6 +9985,9 @@
       <c r="J69" t="inlineStr"/>
       <c r="K69" t="inlineStr"/>
       <c r="L69" t="inlineStr"/>
+      <c r="M69" t="inlineStr"/>
+      <c r="N69" t="inlineStr"/>
+      <c r="O69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -9809,6 +10028,9 @@
       <c r="J70" t="inlineStr"/>
       <c r="K70" t="inlineStr"/>
       <c r="L70" t="inlineStr"/>
+      <c r="M70" t="inlineStr"/>
+      <c r="N70" t="inlineStr"/>
+      <c r="O70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -9849,6 +10071,9 @@
       <c r="J71" t="inlineStr"/>
       <c r="K71" t="inlineStr"/>
       <c r="L71" t="inlineStr"/>
+      <c r="M71" t="inlineStr"/>
+      <c r="N71" t="inlineStr"/>
+      <c r="O71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -9889,6 +10114,9 @@
       <c r="J72" t="inlineStr"/>
       <c r="K72" t="inlineStr"/>
       <c r="L72" t="inlineStr"/>
+      <c r="M72" t="inlineStr"/>
+      <c r="N72" t="inlineStr"/>
+      <c r="O72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -9929,6 +10157,9 @@
       <c r="J73" t="inlineStr"/>
       <c r="K73" t="inlineStr"/>
       <c r="L73" t="inlineStr"/>
+      <c r="M73" t="inlineStr"/>
+      <c r="N73" t="inlineStr"/>
+      <c r="O73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -9969,6 +10200,9 @@
       <c r="J74" t="inlineStr"/>
       <c r="K74" t="inlineStr"/>
       <c r="L74" t="inlineStr"/>
+      <c r="M74" t="inlineStr"/>
+      <c r="N74" t="inlineStr"/>
+      <c r="O74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -10009,6 +10243,9 @@
       <c r="J75" t="inlineStr"/>
       <c r="K75" t="inlineStr"/>
       <c r="L75" t="inlineStr"/>
+      <c r="M75" t="inlineStr"/>
+      <c r="N75" t="inlineStr"/>
+      <c r="O75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -10049,6 +10286,9 @@
       <c r="J76" t="inlineStr"/>
       <c r="K76" t="inlineStr"/>
       <c r="L76" t="inlineStr"/>
+      <c r="M76" t="inlineStr"/>
+      <c r="N76" t="inlineStr"/>
+      <c r="O76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -10089,6 +10329,9 @@
       <c r="J77" t="inlineStr"/>
       <c r="K77" t="inlineStr"/>
       <c r="L77" t="inlineStr"/>
+      <c r="M77" t="inlineStr"/>
+      <c r="N77" t="inlineStr"/>
+      <c r="O77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -10129,6 +10372,9 @@
       <c r="J78" t="inlineStr"/>
       <c r="K78" t="inlineStr"/>
       <c r="L78" t="inlineStr"/>
+      <c r="M78" t="inlineStr"/>
+      <c r="N78" t="inlineStr"/>
+      <c r="O78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -10169,6 +10415,9 @@
       <c r="J79" t="inlineStr"/>
       <c r="K79" t="inlineStr"/>
       <c r="L79" t="inlineStr"/>
+      <c r="M79" t="inlineStr"/>
+      <c r="N79" t="inlineStr"/>
+      <c r="O79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -10209,6 +10458,9 @@
       <c r="J80" t="inlineStr"/>
       <c r="K80" t="inlineStr"/>
       <c r="L80" t="inlineStr"/>
+      <c r="M80" t="inlineStr"/>
+      <c r="N80" t="inlineStr"/>
+      <c r="O80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -10249,6 +10501,9 @@
       <c r="J81" t="inlineStr"/>
       <c r="K81" t="inlineStr"/>
       <c r="L81" t="inlineStr"/>
+      <c r="M81" t="inlineStr"/>
+      <c r="N81" t="inlineStr"/>
+      <c r="O81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -10289,6 +10544,9 @@
       <c r="J82" t="inlineStr"/>
       <c r="K82" t="inlineStr"/>
       <c r="L82" t="inlineStr"/>
+      <c r="M82" t="inlineStr"/>
+      <c r="N82" t="inlineStr"/>
+      <c r="O82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -10329,6 +10587,9 @@
       <c r="J83" t="inlineStr"/>
       <c r="K83" t="inlineStr"/>
       <c r="L83" t="inlineStr"/>
+      <c r="M83" t="inlineStr"/>
+      <c r="N83" t="inlineStr"/>
+      <c r="O83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -10369,6 +10630,9 @@
       <c r="J84" t="inlineStr"/>
       <c r="K84" t="inlineStr"/>
       <c r="L84" t="inlineStr"/>
+      <c r="M84" t="inlineStr"/>
+      <c r="N84" t="inlineStr"/>
+      <c r="O84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="n">
@@ -10409,6 +10673,9 @@
       <c r="J85" t="inlineStr"/>
       <c r="K85" t="inlineStr"/>
       <c r="L85" t="inlineStr"/>
+      <c r="M85" t="inlineStr"/>
+      <c r="N85" t="inlineStr"/>
+      <c r="O85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -10449,6 +10716,9 @@
       <c r="J86" t="inlineStr"/>
       <c r="K86" t="inlineStr"/>
       <c r="L86" t="inlineStr"/>
+      <c r="M86" t="inlineStr"/>
+      <c r="N86" t="inlineStr"/>
+      <c r="O86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="n">
@@ -10489,6 +10759,9 @@
       <c r="J87" t="inlineStr"/>
       <c r="K87" t="inlineStr"/>
       <c r="L87" t="inlineStr"/>
+      <c r="M87" t="inlineStr"/>
+      <c r="N87" t="inlineStr"/>
+      <c r="O87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -10529,6 +10802,9 @@
       <c r="J88" t="inlineStr"/>
       <c r="K88" t="inlineStr"/>
       <c r="L88" t="inlineStr"/>
+      <c r="M88" t="inlineStr"/>
+      <c r="N88" t="inlineStr"/>
+      <c r="O88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -10569,6 +10845,9 @@
       <c r="J89" t="inlineStr"/>
       <c r="K89" t="inlineStr"/>
       <c r="L89" t="inlineStr"/>
+      <c r="M89" t="inlineStr"/>
+      <c r="N89" t="inlineStr"/>
+      <c r="O89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -10609,6 +10888,9 @@
       <c r="J90" t="inlineStr"/>
       <c r="K90" t="inlineStr"/>
       <c r="L90" t="inlineStr"/>
+      <c r="M90" t="inlineStr"/>
+      <c r="N90" t="inlineStr"/>
+      <c r="O90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -10649,6 +10931,9 @@
       <c r="J91" t="inlineStr"/>
       <c r="K91" t="inlineStr"/>
       <c r="L91" t="inlineStr"/>
+      <c r="M91" t="inlineStr"/>
+      <c r="N91" t="inlineStr"/>
+      <c r="O91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -10689,6 +10974,9 @@
       <c r="J92" t="inlineStr"/>
       <c r="K92" t="inlineStr"/>
       <c r="L92" t="inlineStr"/>
+      <c r="M92" t="inlineStr"/>
+      <c r="N92" t="inlineStr"/>
+      <c r="O92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -10729,6 +11017,9 @@
       <c r="J93" t="inlineStr"/>
       <c r="K93" t="inlineStr"/>
       <c r="L93" t="inlineStr"/>
+      <c r="M93" t="inlineStr"/>
+      <c r="N93" t="inlineStr"/>
+      <c r="O93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -10769,6 +11060,9 @@
       <c r="J94" t="inlineStr"/>
       <c r="K94" t="inlineStr"/>
       <c r="L94" t="inlineStr"/>
+      <c r="M94" t="inlineStr"/>
+      <c r="N94" t="inlineStr"/>
+      <c r="O94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -10809,6 +11103,9 @@
       <c r="J95" t="inlineStr"/>
       <c r="K95" t="inlineStr"/>
       <c r="L95" t="inlineStr"/>
+      <c r="M95" t="inlineStr"/>
+      <c r="N95" t="inlineStr"/>
+      <c r="O95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -10849,6 +11146,9 @@
       <c r="J96" t="inlineStr"/>
       <c r="K96" t="inlineStr"/>
       <c r="L96" t="inlineStr"/>
+      <c r="M96" t="inlineStr"/>
+      <c r="N96" t="inlineStr"/>
+      <c r="O96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="n">
@@ -10889,6 +11189,9 @@
       <c r="J97" t="inlineStr"/>
       <c r="K97" t="inlineStr"/>
       <c r="L97" t="inlineStr"/>
+      <c r="M97" t="inlineStr"/>
+      <c r="N97" t="inlineStr"/>
+      <c r="O97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -10929,6 +11232,9 @@
       <c r="J98" t="inlineStr"/>
       <c r="K98" t="inlineStr"/>
       <c r="L98" t="inlineStr"/>
+      <c r="M98" t="inlineStr"/>
+      <c r="N98" t="inlineStr"/>
+      <c r="O98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="n">
@@ -10969,6 +11275,9 @@
       <c r="J99" t="inlineStr"/>
       <c r="K99" t="inlineStr"/>
       <c r="L99" t="inlineStr"/>
+      <c r="M99" t="inlineStr"/>
+      <c r="N99" t="inlineStr"/>
+      <c r="O99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="n">
@@ -11009,6 +11318,9 @@
       <c r="J100" t="inlineStr"/>
       <c r="K100" t="inlineStr"/>
       <c r="L100" t="inlineStr"/>
+      <c r="M100" t="inlineStr"/>
+      <c r="N100" t="inlineStr"/>
+      <c r="O100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -11049,6 +11361,9 @@
       <c r="J101" t="inlineStr"/>
       <c r="K101" t="inlineStr"/>
       <c r="L101" t="inlineStr"/>
+      <c r="M101" t="inlineStr"/>
+      <c r="N101" t="inlineStr"/>
+      <c r="O101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="n">
@@ -11089,6 +11404,9 @@
       <c r="J102" t="inlineStr"/>
       <c r="K102" t="inlineStr"/>
       <c r="L102" t="inlineStr"/>
+      <c r="M102" t="inlineStr"/>
+      <c r="N102" t="inlineStr"/>
+      <c r="O102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="n">
@@ -11129,6 +11447,9 @@
       <c r="J103" t="inlineStr"/>
       <c r="K103" t="inlineStr"/>
       <c r="L103" t="inlineStr"/>
+      <c r="M103" t="inlineStr"/>
+      <c r="N103" t="inlineStr"/>
+      <c r="O103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="n">
@@ -11169,6 +11490,9 @@
       <c r="J104" t="inlineStr"/>
       <c r="K104" t="inlineStr"/>
       <c r="L104" t="inlineStr"/>
+      <c r="M104" t="inlineStr"/>
+      <c r="N104" t="inlineStr"/>
+      <c r="O104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="n">
@@ -11209,6 +11533,9 @@
       <c r="J105" t="inlineStr"/>
       <c r="K105" t="inlineStr"/>
       <c r="L105" t="inlineStr"/>
+      <c r="M105" t="inlineStr"/>
+      <c r="N105" t="inlineStr"/>
+      <c r="O105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="n">
@@ -11249,6 +11576,9 @@
       <c r="J106" t="inlineStr"/>
       <c r="K106" t="inlineStr"/>
       <c r="L106" t="inlineStr"/>
+      <c r="M106" t="inlineStr"/>
+      <c r="N106" t="inlineStr"/>
+      <c r="O106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="n">
@@ -11289,6 +11619,9 @@
       <c r="J107" t="inlineStr"/>
       <c r="K107" t="inlineStr"/>
       <c r="L107" t="inlineStr"/>
+      <c r="M107" t="inlineStr"/>
+      <c r="N107" t="inlineStr"/>
+      <c r="O107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="n">
@@ -11329,6 +11662,9 @@
       <c r="J108" t="inlineStr"/>
       <c r="K108" t="inlineStr"/>
       <c r="L108" t="inlineStr"/>
+      <c r="M108" t="inlineStr"/>
+      <c r="N108" t="inlineStr"/>
+      <c r="O108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="n">
@@ -11369,6 +11705,9 @@
       <c r="J109" t="inlineStr"/>
       <c r="K109" t="inlineStr"/>
       <c r="L109" t="inlineStr"/>
+      <c r="M109" t="inlineStr"/>
+      <c r="N109" t="inlineStr"/>
+      <c r="O109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="n">
@@ -11409,6 +11748,9 @@
       <c r="J110" t="inlineStr"/>
       <c r="K110" t="inlineStr"/>
       <c r="L110" t="inlineStr"/>
+      <c r="M110" t="inlineStr"/>
+      <c r="N110" t="inlineStr"/>
+      <c r="O110" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
auto: anime list update 2026-06-14
</commit_message>
<xml_diff>
--- a/data/anime_list.xlsx
+++ b/data/anime_list.xlsx
@@ -7960,13 +7960,27 @@
           <t>sajou no hana</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=1qcDcvE9lWc</t>
+        </is>
+      </c>
+      <c r="J22" t="n">
+        <v>1654</v>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>sajou no hana Official Channel</t>
+        </is>
+      </c>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="inlineStr"/>
       <c r="N22" t="inlineStr"/>
-      <c r="O22" t="inlineStr"/>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>2026-06-14T18:14:57</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">

</xml_diff>

<commit_message>
auto: anime list update 2026-06-15
</commit_message>
<xml_diff>
--- a/data/anime_list.xlsx
+++ b/data/anime_list.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M131"/>
+  <dimension ref="A1:M132"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -556,14 +556,30 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026年7月～</t>
+          <t>2026年7月8日（水）～ tvkテレビ神奈川・テレ玉ほか</t>
         </is>
       </c>
       <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>雨宿りの憧憬</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Lia</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>クレール</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>AVAM</t>
+        </is>
+      </c>
       <c r="M3" t="inlineStr">
         <is>
           <t>https://www.animatetimes.com/tag/details.php?id=26511</t>
@@ -597,7 +613,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026年7月4日（土）～ TOKYO MX・サンテレビにて</t>
+          <t>2026年7月4日（土）～ TOKYO MX・サンテレビほか</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -964,14 +980,30 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026年7月～</t>
+          <t>2026年7月4日（土）～ TOKYO MX・BS11ほか</t>
         </is>
       </c>
       <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>ヒトコト</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>ClariS</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>心星</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>山崎育三郎</t>
+        </is>
+      </c>
       <c r="M11" t="inlineStr">
         <is>
           <t>https://www.animatetimes.com/tag/details.php?id=26164</t>
@@ -1526,14 +1558,30 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>2026年7月～</t>
+          <t>2026年7月4日（土）～ TOKYO MX・BS11ほか</t>
         </is>
       </c>
       <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
-      <c r="L21" t="inlineStr"/>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>ユラリユレル</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>NOMELON NOLEMON</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>DAYS!</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>Aooo</t>
+        </is>
+      </c>
       <c r="M21" t="inlineStr">
         <is>
           <t>https://www.animatetimes.com/tag/details.php?id=26410</t>
@@ -2749,7 +2797,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>2026年7月8日（水）～ フジテレビ・関西テレビほか</t>
+          <t>2026年7月8日（水）～ フジテレビほか</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -2767,8 +2815,16 @@
           <t>QWER</t>
         </is>
       </c>
-      <c r="K44" t="inlineStr"/>
-      <c r="L44" t="inlineStr"/>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>To Be Continued</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>QWER</t>
+        </is>
+      </c>
       <c r="M44" t="inlineStr">
         <is>
           <t>https://www.animatetimes.com/tag/details.php?id=27435</t>
@@ -2963,8 +3019,16 @@
           <t>五阿弥ルナ</t>
         </is>
       </c>
-      <c r="K48" t="inlineStr"/>
-      <c r="L48" t="inlineStr"/>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>Soarin’</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>Ginger Root</t>
+        </is>
+      </c>
       <c r="M48" t="inlineStr">
         <is>
           <t>https://www.animatetimes.com/tag/details.php?id=27014</t>
@@ -3708,7 +3772,7 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>2026年7月〜</t>
+          <t>2026年7月2日（木）～ TOKYO MX1・サンテレビほか</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
@@ -3718,8 +3782,16 @@
       </c>
       <c r="I63" t="inlineStr"/>
       <c r="J63" t="inlineStr"/>
-      <c r="K63" t="inlineStr"/>
-      <c r="L63" t="inlineStr"/>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>僕ら～芥川龍之介Ver.～</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>芥川龍之介（CV.小野賢章）</t>
+        </is>
+      </c>
       <c r="M63" t="inlineStr">
         <is>
           <t>https://www.animatetimes.com/tag/details.php?id=27057</t>
@@ -6121,7 +6193,7 @@
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
+          <t>2026年10月2日（金）～ MBS・TBS・CBC”アニメイズム”枠ほか</t>
         </is>
       </c>
       <c r="H112" t="inlineStr">
@@ -6906,11 +6978,11 @@
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>らんま1/2 第3期</t>
+          <t>ラブライブ！虹ヶ咲学園スクールアイドル同好会 第2期</t>
         </is>
       </c>
       <c r="E130" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F130" t="inlineStr">
         <is>
@@ -6919,17 +6991,21 @@
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>2026年10月～ 日本テレビ系にて</t>
-        </is>
-      </c>
-      <c r="H130" t="inlineStr"/>
+          <t>2022年4月2日（土）～2022年6月25日（土） TOKYO MXほか 【再放送】 2026年9月30日（水）〜 BS日テレにて</t>
+        </is>
+      </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>サンライズ</t>
+        </is>
+      </c>
       <c r="I130" t="inlineStr"/>
       <c r="J130" t="inlineStr"/>
       <c r="K130" t="inlineStr"/>
       <c r="L130" t="inlineStr"/>
       <c r="M130" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28013</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=14120</t>
         </is>
       </c>
     </row>
@@ -6947,7 +7023,7 @@
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>LEGO® ONE PIECE</t>
+          <t>らんま1/2 第3期</t>
         </is>
       </c>
       <c r="E131" t="b">
@@ -6955,12 +7031,12 @@
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>配信</t>
+          <t>TVアニメ</t>
         </is>
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>2026年9月29日（火） Netflixにて</t>
+          <t>2026年10月～ 日本テレビ系にて</t>
         </is>
       </c>
       <c r="H131" t="inlineStr"/>
@@ -6969,6 +7045,47 @@
       <c r="K131" t="inlineStr"/>
       <c r="L131" t="inlineStr"/>
       <c r="M131" t="inlineStr">
+        <is>
+          <t>https://www.animatetimes.com/tag/details.php?id=28013</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C132" t="n">
+        <v>51</v>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>LEGO® ONE PIECE</t>
+        </is>
+      </c>
+      <c r="E132" t="b">
+        <v>0</v>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>配信</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>2026年9月29日（火） Netflixにて</t>
+        </is>
+      </c>
+      <c r="H132" t="inlineStr"/>
+      <c r="I132" t="inlineStr"/>
+      <c r="J132" t="inlineStr"/>
+      <c r="K132" t="inlineStr"/>
+      <c r="L132" t="inlineStr"/>
+      <c r="M132" t="inlineStr">
         <is>
           <t>https://www.animatetimes.com/tag/details.php?id=28168</t>
         </is>
@@ -6985,7 +7102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O110"/>
+  <dimension ref="A1:O120"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7162,7 +7279,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>岩元先輩ノ推薦</t>
+          <t>いびってこない義母と義姉</t>
         </is>
       </c>
       <c r="D4" t="b">
@@ -7178,12 +7295,12 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>BUDDING</t>
+          <t>雨宿りの憧憬</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>THE JET BOY BANGERZ</t>
+          <t>Lia</t>
         </is>
       </c>
       <c r="I4" t="inlineStr"/>
@@ -7205,7 +7322,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>岩元先輩ノ推薦</t>
+          <t>いびってこない義母と義姉</t>
         </is>
       </c>
       <c r="D5" t="b">
@@ -7221,12 +7338,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>ココニイル</t>
+          <t>クレール</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>WOLF HOWL HARMONY</t>
+          <t>AVAM</t>
         </is>
       </c>
       <c r="I5" t="inlineStr"/>
@@ -7248,7 +7365,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>うしろの正面カムイさん</t>
+          <t>岩元先輩ノ推薦</t>
         </is>
       </c>
       <c r="D6" t="b">
@@ -7264,12 +7381,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>成仏Come true</t>
+          <t>BUDDING</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>ORCALAND</t>
+          <t>THE JET BOY BANGERZ</t>
         </is>
       </c>
       <c r="I6" t="inlineStr"/>
@@ -7291,7 +7408,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>うしろの正面カムイさん</t>
+          <t>岩元先輩ノ推薦</t>
         </is>
       </c>
       <c r="D7" t="b">
@@ -7307,12 +7424,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>SAY-BYE!!</t>
+          <t>ココニイル</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>KOTOKO</t>
+          <t>WOLF HOWL HARMONY</t>
         </is>
       </c>
       <c r="I7" t="inlineStr"/>
@@ -7334,7 +7451,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>うちの弟どもがすみません</t>
+          <t>うしろの正面カムイさん</t>
         </is>
       </c>
       <c r="D8" t="b">
@@ -7350,12 +7467,12 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>アイコトバ</t>
+          <t>成仏Come true</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>DISH//</t>
+          <t>ORCALAND</t>
         </is>
       </c>
       <c r="I8" t="inlineStr"/>
@@ -7377,7 +7494,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>うちの弟どもがすみません</t>
+          <t>うしろの正面カムイさん</t>
         </is>
       </c>
       <c r="D9" t="b">
@@ -7393,12 +7510,12 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Clover</t>
+          <t>SAY-BYE!!</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>汐れいら</t>
+          <t>KOTOKO</t>
         </is>
       </c>
       <c r="I9" t="inlineStr"/>
@@ -7420,7 +7537,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>ウルトラマンテオ</t>
+          <t>うちの弟どもがすみません</t>
         </is>
       </c>
       <c r="D10" t="b">
@@ -7428,7 +7545,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>主題歌</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F10" t="n">
@@ -7436,12 +7553,12 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>LINK HEARTS</t>
+          <t>アイコトバ</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>ASTRO DONUTS</t>
+          <t>DISH//</t>
         </is>
       </c>
       <c r="I10" t="inlineStr"/>
@@ -7463,7 +7580,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>乙女怪獣キャラメリゼ</t>
+          <t>うちの弟どもがすみません</t>
         </is>
       </c>
       <c r="D11" t="b">
@@ -7471,7 +7588,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F11" t="n">
@@ -7479,12 +7596,12 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>乙女怪獣</t>
+          <t>Clover</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>METANICK</t>
+          <t>汐れいら</t>
         </is>
       </c>
       <c r="I11" t="inlineStr"/>
@@ -7506,7 +7623,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>乙女怪獣キャラメリゼ</t>
+          <t>ウルトラマンテオ</t>
         </is>
       </c>
       <c r="D12" t="b">
@@ -7514,7 +7631,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>主題歌</t>
         </is>
       </c>
       <c r="F12" t="n">
@@ -7522,12 +7639,12 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>オトメノホンキ</t>
+          <t>LINK HEARTS</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>HoneyWorks feat.ハコニワリリィ</t>
+          <t>ASTRO DONUTS</t>
         </is>
       </c>
       <c r="I12" t="inlineStr"/>
@@ -7549,7 +7666,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>同じゼミの染谷さんがセクシー女優だった話。</t>
+          <t>乙女怪獣キャラメリゼ</t>
         </is>
       </c>
       <c r="D13" t="b">
@@ -7557,7 +7674,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>主題歌</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F13" t="n">
@@ -7565,12 +7682,12 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>未来コントレール</t>
+          <t>乙女怪獣</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>桜空もも</t>
+          <t>METANICK</t>
         </is>
       </c>
       <c r="I13" t="inlineStr"/>
@@ -7592,7 +7709,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>骸骨騎士様、只今異世界へお出掛け中Ⅱ</t>
+          <t>乙女怪獣キャラメリゼ</t>
         </is>
       </c>
       <c r="D14" t="b">
@@ -7600,7 +7717,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F14" t="n">
@@ -7608,12 +7725,12 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>浪漫街道、お散歩中</t>
+          <t>オトメノホンキ</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>PelleK</t>
+          <t>HoneyWorks feat.ハコニワリリィ</t>
         </is>
       </c>
       <c r="I14" t="inlineStr"/>
@@ -7635,7 +7752,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>骸骨騎士様、只今異世界へお出掛け中Ⅱ</t>
+          <t>同じゼミの染谷さんがセクシー女優だった話。</t>
         </is>
       </c>
       <c r="D15" t="b">
@@ -7643,7 +7760,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>主題歌</t>
         </is>
       </c>
       <c r="F15" t="n">
@@ -7651,12 +7768,12 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>奇跡は起きない</t>
+          <t>未来コントレール</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>DIALOGUE+</t>
+          <t>桜空もも</t>
         </is>
       </c>
       <c r="I15" t="inlineStr"/>
@@ -7678,7 +7795,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>片田舎のおっさん、剣聖になるII</t>
+          <t>鬼の花嫁</t>
         </is>
       </c>
       <c r="D16" t="b">
@@ -7694,12 +7811,12 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>クレナイノハ</t>
+          <t>ヒトコト</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>ユニコーン</t>
+          <t>ClariS</t>
         </is>
       </c>
       <c r="I16" t="inlineStr"/>
@@ -7721,7 +7838,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>片田舎のおっさん、剣聖になるII</t>
+          <t>鬼の花嫁</t>
         </is>
       </c>
       <c r="D17" t="b">
@@ -7737,12 +7854,12 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>未完成</t>
+          <t>心星</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>BLUE ENCOUNT</t>
+          <t>山崎育三郎</t>
         </is>
       </c>
       <c r="I17" t="inlineStr"/>
@@ -7764,7 +7881,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>株式会社マジルミエ 第2期</t>
+          <t>骸骨騎士様、只今異世界へお出掛け中Ⅱ</t>
         </is>
       </c>
       <c r="D18" t="b">
@@ -7772,7 +7889,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F18" t="n">
@@ -7780,12 +7897,12 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>BooooM!!!</t>
+          <t>浪漫街道、お散歩中</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>宝鐘マリン</t>
+          <t>PelleK</t>
         </is>
       </c>
       <c r="I18" t="inlineStr"/>
@@ -7807,15 +7924,15 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>帰還者の魔法は特別です</t>
+          <t>骸骨騎士様、只今異世界へお出掛け中Ⅱ</t>
         </is>
       </c>
       <c r="D19" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F19" t="n">
@@ -7823,12 +7940,12 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>GET BACK</t>
+          <t>奇跡は起きない</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>FLOW</t>
+          <t>DIALOGUE+</t>
         </is>
       </c>
       <c r="I19" t="inlineStr"/>
@@ -7850,15 +7967,15 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>帰還者の魔法は特別です</t>
+          <t>片田舎のおっさん、剣聖になるII</t>
         </is>
       </c>
       <c r="D20" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F20" t="n">
@@ -7866,12 +7983,12 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>6を撫でる</t>
+          <t>クレナイノハ</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>ももすももす</t>
+          <t>ユニコーン</t>
         </is>
       </c>
       <c r="I20" t="inlineStr"/>
@@ -7893,7 +8010,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>きみが死ぬまで恋をしたい</t>
+          <t>片田舎のおっさん、剣聖になるII</t>
         </is>
       </c>
       <c r="D21" t="b">
@@ -7901,7 +8018,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F21" t="n">
@@ -7909,12 +8026,12 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Amore</t>
+          <t>未完成</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>ReoNa</t>
+          <t>BLUE ENCOUNT</t>
         </is>
       </c>
       <c r="I21" t="inlineStr"/>
@@ -7936,7 +8053,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>きみが死ぬまで恋をしたい</t>
+          <t>株式会社マジルミエ 第2期</t>
         </is>
       </c>
       <c r="D22" t="b">
@@ -7952,35 +8069,21 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>エテルネル</t>
+          <t>BooooM!!!</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>sajou no hana</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=1qcDcvE9lWc</t>
-        </is>
-      </c>
-      <c r="J22" t="n">
-        <v>1654</v>
-      </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>sajou no hana Official Channel</t>
-        </is>
-      </c>
+          <t>宝鐘マリン</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="inlineStr"/>
       <c r="N22" t="inlineStr"/>
-      <c r="O22" t="inlineStr">
-        <is>
-          <t>2026-06-14T18:14:57</t>
-        </is>
-      </c>
+      <c r="O22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -7993,11 +8096,11 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>「きみを愛する気はない」と言った次期公爵様がなぜか溺愛してきます</t>
+          <t>帰還者の魔法は特別です</t>
         </is>
       </c>
       <c r="D23" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -8009,12 +8112,12 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>いつかちゃんと。</t>
+          <t>GET BACK</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>りりあ。</t>
+          <t>FLOW</t>
         </is>
       </c>
       <c r="I23" t="inlineStr"/>
@@ -8036,11 +8139,11 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>「きみを愛する気はない」と言った次期公爵様がなぜか溺愛してきます</t>
+          <t>帰還者の魔法は特別です</t>
         </is>
       </c>
       <c r="D24" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -8052,12 +8155,12 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>最終回</t>
+          <t>6を撫でる</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>sorato</t>
+          <t>ももすももす</t>
         </is>
       </c>
       <c r="I24" t="inlineStr"/>
@@ -8079,7 +8182,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>ぐらんぶる Season 3</t>
+          <t>きみが死ぬまで恋をしたい</t>
         </is>
       </c>
       <c r="D25" t="b">
@@ -8095,12 +8198,12 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>夏子</t>
+          <t>Amore</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>FUNKY MONKEY BΛBY'S</t>
+          <t>ReoNa</t>
         </is>
       </c>
       <c r="I25" t="inlineStr"/>
@@ -8122,7 +8225,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>ぐらんぶる Season 3</t>
+          <t>きみが死ぬまで恋をしたい</t>
         </is>
       </c>
       <c r="D26" t="b">
@@ -8138,21 +8241,35 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>裸のマーメード</t>
+          <t>エテルネル</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>豆柴の大群</t>
-        </is>
-      </c>
-      <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr"/>
+          <t>sajou no hana</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=1qcDcvE9lWc</t>
+        </is>
+      </c>
+      <c r="J26" t="n">
+        <v>1654</v>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>sajou no hana Official Channel</t>
+        </is>
+      </c>
       <c r="L26" t="inlineStr"/>
       <c r="M26" t="inlineStr"/>
       <c r="N26" t="inlineStr"/>
-      <c r="O26" t="inlineStr"/>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>2026-06-14T18:14:57</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -8165,7 +8282,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>クレバテスII-魔獣の王と偽りの勇者伝承-</t>
+          <t>「きみを愛する気はない」と言った次期公爵様がなぜか溺愛してきます</t>
         </is>
       </c>
       <c r="D27" t="b">
@@ -8181,12 +8298,12 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Foreshadow</t>
+          <t>いつかちゃんと。</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>前島麻由</t>
+          <t>りりあ。</t>
         </is>
       </c>
       <c r="I27" t="inlineStr"/>
@@ -8208,7 +8325,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>クレバテスII-魔獣の王と偽りの勇者伝承-</t>
+          <t>「きみを愛する気はない」と言った次期公爵様がなぜか溺愛してきます</t>
         </is>
       </c>
       <c r="D28" t="b">
@@ -8224,12 +8341,12 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Awake Anew</t>
+          <t>最終回</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>MYTH &amp; ROID</t>
+          <t>sorato</t>
         </is>
       </c>
       <c r="I28" t="inlineStr"/>
@@ -8251,7 +8368,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>攻殻機動隊 THE GHOST IN THE SHELL</t>
+          <t>ぐらんぶる Season 3</t>
         </is>
       </c>
       <c r="D29" t="b">
@@ -8259,7 +8376,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F29" t="n">
@@ -8267,12 +8384,12 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Blue</t>
+          <t>夏子</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>MILLENNIUM PARADE feat. Saya Gray, Daniel Caesar</t>
+          <t>FUNKY MONKEY BΛBY'S</t>
         </is>
       </c>
       <c r="I29" t="inlineStr"/>
@@ -8294,7 +8411,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>コードギアス 奪還のロゼ TV放送</t>
+          <t>ぐらんぶる Season 3</t>
         </is>
       </c>
       <c r="D30" t="b">
@@ -8302,7 +8419,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F30" t="n">
@@ -8310,12 +8427,12 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Running In My Head</t>
+          <t>裸のマーメード</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>MIYAVI</t>
+          <t>豆柴の大群</t>
         </is>
       </c>
       <c r="I30" t="inlineStr"/>
@@ -8337,7 +8454,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>コードギアス 奪還のロゼ TV放送</t>
+          <t>クレバテスII-魔獣の王と偽りの勇者伝承-</t>
         </is>
       </c>
       <c r="D31" t="b">
@@ -8345,7 +8462,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F31" t="n">
@@ -8353,12 +8470,12 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>ロゼ (Prod.TeddyLoid)</t>
+          <t>Foreshadow</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>満島ひかり</t>
+          <t>前島麻由</t>
         </is>
       </c>
       <c r="I31" t="inlineStr"/>
@@ -8380,7 +8497,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>これ描いて死ね</t>
+          <t>クレバテスII-魔獣の王と偽りの勇者伝承-</t>
         </is>
       </c>
       <c r="D32" t="b">
@@ -8388,7 +8505,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F32" t="n">
@@ -8396,12 +8513,12 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>遺書</t>
+          <t>Awake Anew</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>キタニタツヤ</t>
+          <t>MYTH &amp; ROID</t>
         </is>
       </c>
       <c r="I32" t="inlineStr"/>
@@ -8423,7 +8540,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>これ描いて死ね</t>
+          <t>グロウアップショウ ～ひまわりのサーカス団～</t>
         </is>
       </c>
       <c r="D33" t="b">
@@ -8431,7 +8548,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F33" t="n">
@@ -8439,12 +8556,12 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>コニファー</t>
+          <t>ユラリユレル</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>リーガルリリー</t>
+          <t>NOMELON NOLEMON</t>
         </is>
       </c>
       <c r="I33" t="inlineStr"/>
@@ -8466,7 +8583,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>才女のお世話 高嶺の花だらけな名門校で、学院一のお嬢様(生活能力皆無)を陰ながらお世話することになりました</t>
+          <t>グロウアップショウ ～ひまわりのサーカス団～</t>
         </is>
       </c>
       <c r="D34" t="b">
@@ -8474,7 +8591,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F34" t="n">
@@ -8482,12 +8599,12 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>最最最高級のお世話して</t>
+          <t>DAYS!</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>angela</t>
+          <t>Aooo</t>
         </is>
       </c>
       <c r="I34" t="inlineStr"/>
@@ -8509,7 +8626,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>才女のお世話 高嶺の花だらけな名門校で、学院一のお嬢様(生活能力皆無)を陰ながらお世話することになりました</t>
+          <t>攻殻機動隊 THE GHOST IN THE SHELL</t>
         </is>
       </c>
       <c r="D35" t="b">
@@ -8525,12 +8642,12 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>完璧じゃないわたし</t>
+          <t>Blue</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>前島亜美</t>
+          <t>MILLENNIUM PARADE feat. Saya Gray, Daniel Caesar</t>
         </is>
       </c>
       <c r="I35" t="inlineStr"/>
@@ -8552,7 +8669,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>サイボーグ009 ネメシス</t>
+          <t>コードギアス 奪還のロゼ TV放送</t>
         </is>
       </c>
       <c r="D36" t="b">
@@ -8568,12 +8685,12 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>誰がために</t>
+          <t>Running In My Head</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>杏子</t>
+          <t>MIYAVI</t>
         </is>
       </c>
       <c r="I36" t="inlineStr"/>
@@ -8595,7 +8712,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>さよならララ</t>
+          <t>コードギアス 奪還のロゼ TV放送</t>
         </is>
       </c>
       <c r="D37" t="b">
@@ -8603,7 +8720,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F37" t="n">
@@ -8611,12 +8728,12 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>さよならララ</t>
+          <t>ロゼ (Prod.TeddyLoid)</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>いきものがかり</t>
+          <t>満島ひかり</t>
         </is>
       </c>
       <c r="I37" t="inlineStr"/>
@@ -8638,7 +8755,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>サンダー３</t>
+          <t>これ描いて死ね</t>
         </is>
       </c>
       <c r="D38" t="b">
@@ -8646,7 +8763,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F38" t="n">
@@ -8654,12 +8771,12 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>しゅるれりら</t>
+          <t>遺書</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>音羽-otoha-</t>
+          <t>キタニタツヤ</t>
         </is>
       </c>
       <c r="I38" t="inlineStr"/>
@@ -8681,7 +8798,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>スーパーの裏でヤニ吸うふたり</t>
+          <t>これ描いて死ね</t>
         </is>
       </c>
       <c r="D39" t="b">
@@ -8689,7 +8806,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F39" t="n">
@@ -8697,12 +8814,12 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>イチジク煙</t>
+          <t>コニファー</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>ずっと真夜中でいいのに。</t>
+          <t>リーガルリリー</t>
         </is>
       </c>
       <c r="I39" t="inlineStr"/>
@@ -8724,7 +8841,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>スーパーの裏でヤニ吸うふたり</t>
+          <t>才女のお世話 高嶺の花だらけな名門校で、学院一のお嬢様(生活能力皆無)を陰ながらお世話することになりました</t>
         </is>
       </c>
       <c r="D40" t="b">
@@ -8732,7 +8849,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F40" t="n">
@@ -8740,12 +8857,12 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Fiction</t>
+          <t>最最最高級のお世話して</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>imase</t>
+          <t>angela</t>
         </is>
       </c>
       <c r="I40" t="inlineStr"/>
@@ -8767,7 +8884,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>捨てられ聖女の異世界ごはん旅 隠れスキルでキャンピングカーを召喚しました</t>
+          <t>才女のお世話 高嶺の花だらけな名門校で、学院一のお嬢様(生活能力皆無)を陰ながらお世話することになりました</t>
         </is>
       </c>
       <c r="D41" t="b">
@@ -8775,7 +8892,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F41" t="n">
@@ -8783,12 +8900,12 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Butterfly</t>
+          <t>完璧じゃないわたし</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>INUWASI</t>
+          <t>前島亜美</t>
         </is>
       </c>
       <c r="I41" t="inlineStr"/>
@@ -8810,7 +8927,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>捨てられ聖女の異世界ごはん旅 隠れスキルでキャンピングカーを召喚しました</t>
+          <t>サイボーグ009 ネメシス</t>
         </is>
       </c>
       <c r="D42" t="b">
@@ -8818,7 +8935,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F42" t="n">
@@ -8826,12 +8943,12 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Holy Sweet Home</t>
+          <t>誰がために</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>音感れもねゐど</t>
+          <t>杏子</t>
         </is>
       </c>
       <c r="I42" t="inlineStr"/>
@@ -8853,11 +8970,11 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>青春ブタ野郎はサンタクロースの夢を見ない</t>
+          <t>さよならララ</t>
         </is>
       </c>
       <c r="D43" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -8869,12 +8986,12 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>スノウドロップ</t>
+          <t>さよならララ</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>Conton Candy</t>
+          <t>いきものがかり</t>
         </is>
       </c>
       <c r="I43" t="inlineStr"/>
@@ -8896,11 +9013,11 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>青春ブタ野郎はサンタクロースの夢を見ない</t>
+          <t>サンダー３</t>
         </is>
       </c>
       <c r="D44" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -8912,12 +9029,12 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>水平線は僕の古傷</t>
+          <t>しゅるれりら</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>広川卯月、赤城郁実、姫路紗良、霧島透子</t>
+          <t>音羽-otoha-</t>
         </is>
       </c>
       <c r="I44" t="inlineStr"/>
@@ -8939,7 +9056,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>正反対な君と僕 第2期</t>
+          <t>スーパーの裏でヤニ吸うふたり</t>
         </is>
       </c>
       <c r="D45" t="b">
@@ -8955,12 +9072,12 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>メガネを外して</t>
+          <t>イチジク煙</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>乃紫</t>
+          <t>ずっと真夜中でいいのに。</t>
         </is>
       </c>
       <c r="I45" t="inlineStr"/>
@@ -8982,7 +9099,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>正反対な君と僕 第2期</t>
+          <t>スーパーの裏でヤニ吸うふたり</t>
         </is>
       </c>
       <c r="D46" t="b">
@@ -8990,20 +9107,20 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F46" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>猫じゃらし</t>
+          <t>Fiction</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>7co</t>
+          <t>imase</t>
         </is>
       </c>
       <c r="I46" t="inlineStr"/>
@@ -9025,7 +9142,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>正反対な君と僕 第2期</t>
+          <t>捨てられ聖女の異世界ごはん旅 隠れスキルでキャンピングカーを召喚しました</t>
         </is>
       </c>
       <c r="D47" t="b">
@@ -9033,7 +9150,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F47" t="n">
@@ -9041,12 +9158,12 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>ピュア feat. 橋本絵莉子</t>
+          <t>Butterfly</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>PAS TASTA</t>
+          <t>INUWASI</t>
         </is>
       </c>
       <c r="I47" t="inlineStr"/>
@@ -9068,7 +9185,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>対ありでした。～お嬢さまは格闘ゲームなんてしない～</t>
+          <t>捨てられ聖女の異世界ごはん旅 隠れスキルでキャンピングカーを召喚しました</t>
         </is>
       </c>
       <c r="D48" t="b">
@@ -9076,7 +9193,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F48" t="n">
@@ -9084,12 +9201,12 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>命短し対する乙女よ</t>
+          <t>Holy Sweet Home</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>花冷え。</t>
+          <t>音感れもねゐど</t>
         </is>
       </c>
       <c r="I48" t="inlineStr"/>
@@ -9111,15 +9228,15 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>対ありでした。～お嬢さまは格闘ゲームなんてしない～</t>
+          <t>青春ブタ野郎はサンタクロースの夢を見ない</t>
         </is>
       </c>
       <c r="D49" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F49" t="n">
@@ -9127,12 +9244,12 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>NEW GAME</t>
+          <t>スノウドロップ</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>halca</t>
+          <t>Conton Candy</t>
         </is>
       </c>
       <c r="I49" t="inlineStr"/>
@@ -9154,15 +9271,15 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>追放された転生重騎士はゲーム知識で無双する</t>
+          <t>青春ブタ野郎はサンタクロースの夢を見ない</t>
         </is>
       </c>
       <c r="D50" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F50" t="n">
@@ -9170,12 +9287,12 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Awake</t>
+          <t>水平線は僕の古傷</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>SPYAIR</t>
+          <t>広川卯月、赤城郁実、姫路紗良、霧島透子</t>
         </is>
       </c>
       <c r="I50" t="inlineStr"/>
@@ -9197,7 +9314,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>鉄鍋のジャン！</t>
+          <t>正反対な君と僕 第2期</t>
         </is>
       </c>
       <c r="D51" t="b">
@@ -9213,12 +9330,12 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>火宴</t>
+          <t>メガネを外して</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>原因は自分にある。</t>
+          <t>乃紫</t>
         </is>
       </c>
       <c r="I51" t="inlineStr"/>
@@ -9240,7 +9357,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>手札が多めのビクトリア</t>
+          <t>正反対な君と僕 第2期</t>
         </is>
       </c>
       <c r="D52" t="b">
@@ -9248,20 +9365,20 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F52" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>縁のつき</t>
+          <t>猫じゃらし</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>KI_EN</t>
+          <t>7co</t>
         </is>
       </c>
       <c r="I52" t="inlineStr"/>
@@ -9283,7 +9400,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>転校先の清楚可憐な美少女が、昔男子と思って一緒に遊んだ幼馴染だった件</t>
+          <t>正反対な君と僕 第2期</t>
         </is>
       </c>
       <c r="D53" t="b">
@@ -9291,7 +9408,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F53" t="n">
@@ -9299,12 +9416,12 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>夏に重ねて</t>
+          <t>ピュア feat. 橋本絵莉子</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>DIALOGUE+</t>
+          <t>PAS TASTA</t>
         </is>
       </c>
       <c r="I53" t="inlineStr"/>
@@ -9326,7 +9443,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>天は赤い河のほとり</t>
+          <t>対ありでした。～お嬢さまは格闘ゲームなんてしない～</t>
         </is>
       </c>
       <c r="D54" t="b">
@@ -9342,12 +9459,12 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>暁の空</t>
+          <t>命短し対する乙女よ</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>七海ひろき</t>
+          <t>花冷え。</t>
         </is>
       </c>
       <c r="I54" t="inlineStr"/>
@@ -9369,7 +9486,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>天幕のジャードゥーガル</t>
+          <t>対ありでした。～お嬢さまは格闘ゲームなんてしない～</t>
         </is>
       </c>
       <c r="D55" t="b">
@@ -9377,7 +9494,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F55" t="n">
@@ -9385,12 +9502,12 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>Stella</t>
+          <t>NEW GAME</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>SEKAI NO OWARI</t>
+          <t>halca</t>
         </is>
       </c>
       <c r="I55" t="inlineStr"/>
@@ -9412,7 +9529,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>盗掘王</t>
+          <t>追放された転生重騎士はゲーム知識で無双する</t>
         </is>
       </c>
       <c r="D56" t="b">
@@ -9428,12 +9545,12 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>SHOW DOWN</t>
+          <t>Awake</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>QWER</t>
+          <t>SPYAIR</t>
         </is>
       </c>
       <c r="I56" t="inlineStr"/>
@@ -9455,7 +9572,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>透明な夜に駆ける君と、目に見えない恋をした。</t>
+          <t>鉄鍋のジャン！</t>
         </is>
       </c>
       <c r="D57" t="b">
@@ -9471,12 +9588,12 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>ひとひら</t>
+          <t>火宴</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>秦基博</t>
+          <t>原因は自分にある。</t>
         </is>
       </c>
       <c r="I57" t="inlineStr"/>
@@ -9498,7 +9615,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>透明な夜に駆ける君と、目に見えない恋をした。</t>
+          <t>手札が多めのビクトリア</t>
         </is>
       </c>
       <c r="D58" t="b">
@@ -9514,12 +9631,12 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>光</t>
+          <t>縁のつき</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>櫻井優衣</t>
+          <t>KI_EN</t>
         </is>
       </c>
       <c r="I58" t="inlineStr"/>
@@ -9541,7 +9658,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>トミカとトム</t>
+          <t>転校先の清楚可憐な美少女が、昔男子と思って一緒に遊んだ幼馴染だった件</t>
         </is>
       </c>
       <c r="D59" t="b">
@@ -9549,7 +9666,7 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>主題歌</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F59" t="n">
@@ -9557,12 +9674,12 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>きみのたからもの</t>
+          <t>夏に重ねて</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>May J.</t>
+          <t>DIALOGUE+</t>
         </is>
       </c>
       <c r="I59" t="inlineStr"/>
@@ -9584,7 +9701,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>二十世紀電氣目録-ユーレカ・エヴリカ-</t>
+          <t>天は赤い河のほとり</t>
         </is>
       </c>
       <c r="D60" t="b">
@@ -9600,12 +9717,12 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>ユーレカ・エヴリカ</t>
+          <t>暁の空</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>五阿弥ルナ</t>
+          <t>七海ひろき</t>
         </is>
       </c>
       <c r="I60" t="inlineStr"/>
@@ -9627,7 +9744,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>パイの実 おしの森へようこそ！</t>
+          <t>天幕のジャードゥーガル</t>
         </is>
       </c>
       <c r="D61" t="b">
@@ -9635,7 +9752,7 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>主題歌</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F61" t="n">
@@ -9643,12 +9760,12 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>パイしか勝たん！推しの森活</t>
+          <t>Stella</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>安保心結</t>
+          <t>SEKAI NO OWARI</t>
         </is>
       </c>
       <c r="I61" t="inlineStr"/>
@@ -9670,7 +9787,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>刃牙道 第2クール</t>
+          <t>盗掘王</t>
         </is>
       </c>
       <c r="D62" t="b">
@@ -9686,12 +9803,12 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>フルボコ</t>
+          <t>SHOW DOWN</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>WANIMA</t>
+          <t>QWER</t>
         </is>
       </c>
       <c r="I62" t="inlineStr"/>
@@ -9713,7 +9830,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>刃牙道 第2クール</t>
+          <t>盗掘王</t>
         </is>
       </c>
       <c r="D63" t="b">
@@ -9721,20 +9838,20 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F63" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>六ノ輪</t>
+          <t>To Be Continued</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>Chevon</t>
+          <t>QWER</t>
         </is>
       </c>
       <c r="I63" t="inlineStr"/>
@@ -9756,7 +9873,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>刃牙道 第2クール</t>
+          <t>透明な夜に駆ける君と、目に見えない恋をした。</t>
         </is>
       </c>
       <c r="D64" t="b">
@@ -9764,7 +9881,7 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F64" t="n">
@@ -9772,12 +9889,12 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>Mountain Top</t>
+          <t>ひとひら</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>Novel Core</t>
+          <t>秦基博</t>
         </is>
       </c>
       <c r="I64" t="inlineStr"/>
@@ -9799,7 +9916,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>刃牙道 第2クール</t>
+          <t>透明な夜に駆ける君と、目に見えない恋をした。</t>
         </is>
       </c>
       <c r="D65" t="b">
@@ -9811,16 +9928,16 @@
         </is>
       </c>
       <c r="F65" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>KATANA</t>
+          <t>光</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>三代目 J SOUL BROTHERS</t>
+          <t>櫻井優衣</t>
         </is>
       </c>
       <c r="I65" t="inlineStr"/>
@@ -9842,7 +9959,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>花ざかりの君たちへ 第2期</t>
+          <t>トミカとトム</t>
         </is>
       </c>
       <c r="D66" t="b">
@@ -9850,7 +9967,7 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>主題歌</t>
         </is>
       </c>
       <c r="F66" t="n">
@@ -9858,12 +9975,12 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>FLASHBULB</t>
+          <t>きみのたからもの</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>Omoinotake</t>
+          <t>May J.</t>
         </is>
       </c>
       <c r="I66" t="inlineStr"/>
@@ -9885,7 +10002,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>花ざかりの君たちへ 第2期</t>
+          <t>二十世紀電氣目録-ユーレカ・エヴリカ-</t>
         </is>
       </c>
       <c r="D67" t="b">
@@ -9893,7 +10010,7 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F67" t="n">
@@ -9901,12 +10018,12 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>花束</t>
+          <t>ユーレカ・エヴリカ</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>Omoinotake</t>
+          <t>五阿弥ルナ</t>
         </is>
       </c>
       <c r="I67" t="inlineStr"/>
@@ -9928,7 +10045,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>ヒロイン？聖女？いいえ、オールワークスメイドです（誇）！</t>
+          <t>二十世紀電氣目録-ユーレカ・エヴリカ-</t>
         </is>
       </c>
       <c r="D68" t="b">
@@ -9936,7 +10053,7 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F68" t="n">
@@ -9944,12 +10061,12 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>マデュアル↔ハート</t>
+          <t>Soarin’</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>メロディ・ウェーブ(CV：宮本侑芽) ルシアナ・ルトルバーグ(CV：大久保瑠美)</t>
+          <t>Ginger Root</t>
         </is>
       </c>
       <c r="I68" t="inlineStr"/>
@@ -9971,7 +10088,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>ヒロイン？聖女？いいえ、オールワークスメイドです（誇）！</t>
+          <t>パイの実 おしの森へようこそ！</t>
         </is>
       </c>
       <c r="D69" t="b">
@@ -9979,7 +10096,7 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>主題歌</t>
         </is>
       </c>
       <c r="F69" t="n">
@@ -9987,12 +10104,12 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>ハンドメイド</t>
+          <t>パイしか勝たん！推しの森活</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>仲村宗悟</t>
+          <t>安保心結</t>
         </is>
       </c>
       <c r="I69" t="inlineStr"/>
@@ -10014,7 +10131,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>ブチ切れ令嬢は報復を誓いました。 ～魔導書の力で祖国を叩き潰します～</t>
+          <t>刃牙道 第2クール</t>
         </is>
       </c>
       <c r="D70" t="b">
@@ -10030,12 +10147,12 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>Q.E.D.</t>
+          <t>フルボコ</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>小倉唯</t>
+          <t>WANIMA</t>
         </is>
       </c>
       <c r="I70" t="inlineStr"/>
@@ -10057,7 +10174,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>ブチ切れ令嬢は報復を誓いました。 ～魔導書の力で祖国を叩き潰します～</t>
+          <t>刃牙道 第2クール</t>
         </is>
       </c>
       <c r="D71" t="b">
@@ -10065,20 +10182,20 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F71" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>グッバイ・ララバイ</t>
+          <t>六ノ輪</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>大西亜玖璃</t>
+          <t>Chevon</t>
         </is>
       </c>
       <c r="I71" t="inlineStr"/>
@@ -10100,7 +10217,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>ふつつかな悪女ではございますが～雛宮蝶鼠とりかえ伝～</t>
+          <t>刃牙道 第2クール</t>
         </is>
       </c>
       <c r="D72" t="b">
@@ -10108,7 +10225,7 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F72" t="n">
@@ -10116,12 +10233,12 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>Sunny</t>
+          <t>Mountain Top</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>milet</t>
+          <t>Novel Core</t>
         </is>
       </c>
       <c r="I72" t="inlineStr"/>
@@ -10143,7 +10260,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>BLACK TORCH</t>
+          <t>刃牙道 第2クール</t>
         </is>
       </c>
       <c r="D73" t="b">
@@ -10151,20 +10268,20 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F73" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>FREEZE ME UP</t>
+          <t>KATANA</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>SiM</t>
+          <t>三代目 J SOUL BROTHERS</t>
         </is>
       </c>
       <c r="I73" t="inlineStr"/>
@@ -10186,7 +10303,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>BLACK TORCH</t>
+          <t>花ざかりの君たちへ 第2期</t>
         </is>
       </c>
       <c r="D74" t="b">
@@ -10194,7 +10311,7 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F74" t="n">
@@ -10202,12 +10319,12 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>Groooovy</t>
+          <t>FLASHBULB</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>I Don't Like Mondays.</t>
+          <t>Omoinotake</t>
         </is>
       </c>
       <c r="I74" t="inlineStr"/>
@@ -10229,7 +10346,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>プラノサウルス ガチコセイブツ部</t>
+          <t>花ざかりの君たちへ 第2期</t>
         </is>
       </c>
       <c r="D75" t="b">
@@ -10237,7 +10354,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>主題歌</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F75" t="n">
@@ -10245,12 +10362,12 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>ガチde古生</t>
+          <t>花束</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>リンクルプラネット</t>
+          <t>Omoinotake</t>
         </is>
       </c>
       <c r="I75" t="inlineStr"/>
@@ -10272,7 +10389,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>ヘルモード ～やり込み好きのゲーマーは廃設定の異世界で無双する～ 2nd Season</t>
+          <t>ヒロイン？聖女？いいえ、オールワークスメイドです（誇）！</t>
         </is>
       </c>
       <c r="D76" t="b">
@@ -10288,12 +10405,12 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>○✕△□</t>
+          <t>マデュアル↔ハート</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>浪漫派マシュマロ</t>
+          <t>メロディ・ウェーブ(CV：宮本侑芽) ルシアナ・ルトルバーグ(CV：大久保瑠美)</t>
         </is>
       </c>
       <c r="I76" t="inlineStr"/>
@@ -10315,7 +10432,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>北斗の拳 拳王軍ザコたちの挽歌 第2クール</t>
+          <t>ヒロイン？聖女？いいえ、オールワークスメイドです（誇）！</t>
         </is>
       </c>
       <c r="D77" t="b">
@@ -10323,7 +10440,7 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F77" t="n">
@@ -10331,12 +10448,12 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>Blacker Co., Ltd.</t>
+          <t>ハンドメイド</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>イツカ▶</t>
+          <t>仲村宗悟</t>
         </is>
       </c>
       <c r="I77" t="inlineStr"/>
@@ -10358,7 +10475,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>北斗の拳 拳王軍ザコたちの挽歌 第2クール</t>
+          <t>ブチ切れ令嬢は報復を誓いました。 ～魔導書の力で祖国を叩き潰します～</t>
         </is>
       </c>
       <c r="D78" t="b">
@@ -10366,7 +10483,7 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F78" t="n">
@@ -10374,12 +10491,12 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>Elegy of the Enemies</t>
+          <t>Q.E.D.</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>The Canbellz</t>
+          <t>小倉唯</t>
         </is>
       </c>
       <c r="I78" t="inlineStr"/>
@@ -10401,7 +10518,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>北斗の拳 拳王軍ザコたちの挽歌 第2クール</t>
+          <t>ブチ切れ令嬢は報復を誓いました。 ～魔導書の力で祖国を叩き潰します～</t>
         </is>
       </c>
       <c r="D79" t="b">
@@ -10413,16 +10530,16 @@
         </is>
       </c>
       <c r="F79" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>白い蝶が飛んだら</t>
+          <t>グッバイ・ララバイ</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>イツカ▶ feat. Dr. Washington | Special Guest Guitar:Tsuyoshi Ujiki</t>
+          <t>大西亜玖璃</t>
         </is>
       </c>
       <c r="I79" t="inlineStr"/>
@@ -10444,7 +10561,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>炎の闘球女 ドッジ弾子</t>
+          <t>ふつつかな悪女ではございますが～雛宮蝶鼠とりかえ伝～</t>
         </is>
       </c>
       <c r="D80" t="b">
@@ -10460,12 +10577,12 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>会心の一劇</t>
+          <t>Sunny</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>ももいろクローバーZ</t>
+          <t>milet</t>
         </is>
       </c>
       <c r="I80" t="inlineStr"/>
@@ -10487,7 +10604,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>炎の闘球女 ドッジ弾子</t>
+          <t>BLACK TORCH</t>
         </is>
       </c>
       <c r="D81" t="b">
@@ -10495,7 +10612,7 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F81" t="n">
@@ -10503,12 +10620,12 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>Welcome to あざとさワールド</t>
+          <t>FREEZE ME UP</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>i☆Ris</t>
+          <t>SiM</t>
         </is>
       </c>
       <c r="I81" t="inlineStr"/>
@@ -10530,7 +10647,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>魔法少女リリカルなのは EXCEEDS Gun Blaze Vengeance</t>
+          <t>BLACK TORCH</t>
         </is>
       </c>
       <c r="D82" t="b">
@@ -10538,7 +10655,7 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F82" t="n">
@@ -10546,12 +10663,12 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>CRIMSON BULLET</t>
+          <t>Groooovy</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>水樹奈々</t>
+          <t>I Don't Like Mondays.</t>
         </is>
       </c>
       <c r="I82" t="inlineStr"/>
@@ -10573,7 +10690,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>魔法少女リリカルなのは EXCEEDS Gun Blaze Vengeance</t>
+          <t>プラノサウルス ガチコセイブツ部</t>
         </is>
       </c>
       <c r="D83" t="b">
@@ -10581,7 +10698,7 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>主題歌</t>
         </is>
       </c>
       <c r="F83" t="n">
@@ -10589,12 +10706,12 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>Ephemeral</t>
+          <t>ガチde古生</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>青木陽菜</t>
+          <t>リンクルプラネット</t>
         </is>
       </c>
       <c r="I83" t="inlineStr"/>
@@ -10616,7 +10733,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>無自覚聖女は今日も無意識に力を垂れ流す</t>
+          <t>文豪ストレイドッグス わん！２</t>
         </is>
       </c>
       <c r="D84" t="b">
@@ -10624,7 +10741,7 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F84" t="n">
@@ -10632,12 +10749,12 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>Windmaker</t>
+          <t>僕ら～芥川龍之介Ver.～</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>花耶</t>
+          <t>芥川龍之介（CV.小野賢章）</t>
         </is>
       </c>
       <c r="I84" t="inlineStr"/>
@@ -10659,7 +10776,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>無自覚聖女は今日も無意識に力を垂れ流す</t>
+          <t>ヘルモード ～やり込み好きのゲーマーは廃設定の異世界で無双する～ 2nd Season</t>
         </is>
       </c>
       <c r="D85" t="b">
@@ -10667,7 +10784,7 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F85" t="n">
@@ -10675,12 +10792,12 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>アンノウンミー</t>
+          <t>○✕△□</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>ウタヒメドリーム オールスターズ【夢咲いぶき（CV:山﨑玲奈） 桜木舞華（CV:鈴木杏奈） 真白清美（CV:其原有沙） HiREN（CV:花耶） 水月ひかり（CV:礒部花凜） 高木凛（CV:鷲見友美ジェナ） 萩原ひまわり（CV:倉知玲鳳） SAKURAKO（CV:竹内夢）】</t>
+          <t>浪漫派マシュマロ</t>
         </is>
       </c>
       <c r="I85" t="inlineStr"/>
@@ -10702,7 +10819,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>無職転生Ⅲ ～異世界行ったら本気だす～</t>
+          <t>北斗の拳 拳王軍ザコたちの挽歌 第2クール</t>
         </is>
       </c>
       <c r="D86" t="b">
@@ -10718,12 +10835,12 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>決意の唄</t>
+          <t>Blacker Co., Ltd.</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>大原ゆい子</t>
+          <t>イツカ▶</t>
         </is>
       </c>
       <c r="I86" t="inlineStr"/>
@@ -10745,7 +10862,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>無職転生Ⅲ ～異世界行ったら本気だす～</t>
+          <t>北斗の拳 拳王軍ザコたちの挽歌 第2クール</t>
         </is>
       </c>
       <c r="D87" t="b">
@@ -10761,12 +10878,12 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>祈り、終われば</t>
+          <t>Elegy of the Enemies</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>中島美嘉</t>
+          <t>The Canbellz</t>
         </is>
       </c>
       <c r="I87" t="inlineStr"/>
@@ -10788,7 +10905,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>メビウス・ダスト</t>
+          <t>北斗の拳 拳王軍ザコたちの挽歌 第2クール</t>
         </is>
       </c>
       <c r="D88" t="b">
@@ -10796,20 +10913,20 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F88" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>メビウス</t>
+          <t>白い蝶が飛んだら</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>家入レオ</t>
+          <t>イツカ▶ feat. Dr. Washington | Special Guest Guitar:Tsuyoshi Ujiki</t>
         </is>
       </c>
       <c r="I88" t="inlineStr"/>
@@ -10831,7 +10948,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>メビウス・ダスト</t>
+          <t>炎の闘球女 ドッジ弾子</t>
         </is>
       </c>
       <c r="D89" t="b">
@@ -10839,7 +10956,7 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F89" t="n">
@@ -10847,12 +10964,12 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>ジレンマ</t>
+          <t>会心の一劇</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>冨岡愛</t>
+          <t>ももいろクローバーZ</t>
         </is>
       </c>
       <c r="I89" t="inlineStr"/>
@@ -10874,7 +10991,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>ヤニねこ</t>
+          <t>炎の闘球女 ドッジ弾子</t>
         </is>
       </c>
       <c r="D90" t="b">
@@ -10882,7 +10999,7 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F90" t="n">
@@ -10890,12 +11007,12 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>なんもねえ</t>
+          <t>Welcome to あざとさワールド</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>忘れらんねえよ</t>
+          <t>i☆Ris</t>
         </is>
       </c>
       <c r="I90" t="inlineStr"/>
@@ -10917,7 +11034,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>幼女戦記Ⅱ</t>
+          <t>魔法少女リリカルなのは EXCEEDS Gun Blaze Vengeance</t>
         </is>
       </c>
       <c r="D91" t="b">
@@ -10933,12 +11050,12 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>Why? RED induction</t>
+          <t>CRIMSON BULLET</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>MYTH &amp; ROID</t>
+          <t>水樹奈々</t>
         </is>
       </c>
       <c r="I91" t="inlineStr"/>
@@ -10960,7 +11077,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>幼女戦記Ⅱ</t>
+          <t>魔法少女リリカルなのは EXCEEDS Gun Blaze Vengeance</t>
         </is>
       </c>
       <c r="D92" t="b">
@@ -10976,12 +11093,12 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>Weiter! Weiter!</t>
+          <t>Ephemeral</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>ターニャ・デグレチャフ（CV：悠木碧）</t>
+          <t>青木陽菜</t>
         </is>
       </c>
       <c r="I92" t="inlineStr"/>
@@ -11003,7 +11120,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>鎧真伝サムライトルーパー 第2クール</t>
+          <t>無自覚聖女は今日も無意識に力を垂れ流す</t>
         </is>
       </c>
       <c r="D93" t="b">
@@ -11019,12 +11136,12 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>YOAKE</t>
+          <t>Windmaker</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>blank paper</t>
+          <t>花耶</t>
         </is>
       </c>
       <c r="I93" t="inlineStr"/>
@@ -11046,7 +11163,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>鎧真伝サムライトルーパー 第2クール</t>
+          <t>無自覚聖女は今日も無意識に力を垂れ流す</t>
         </is>
       </c>
       <c r="D94" t="b">
@@ -11054,20 +11171,20 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F94" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>BAD遺伝子</t>
+          <t>アンノウンミー</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>Dannie May</t>
+          <t>ウタヒメドリーム オールスターズ【夢咲いぶき（CV:山﨑玲奈） 桜木舞華（CV:鈴木杏奈） 真白清美（CV:其原有沙） HiREN（CV:花耶） 水月ひかり（CV:礒部花凜） 高木凛（CV:鷲見友美ジェナ） 萩原ひまわり（CV:倉知玲鳳） SAKURAKO（CV:竹内夢）】</t>
         </is>
       </c>
       <c r="I94" t="inlineStr"/>
@@ -11089,7 +11206,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>鎧真伝サムライトルーパー 第2クール</t>
+          <t>無職転生Ⅲ ～異世界行ったら本気だす～</t>
         </is>
       </c>
       <c r="D95" t="b">
@@ -11097,7 +11214,7 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F95" t="n">
@@ -11105,12 +11222,12 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>POWER</t>
+          <t>決意の唄</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>ONE OR EIGHT</t>
+          <t>大原ゆい子</t>
         </is>
       </c>
       <c r="I95" t="inlineStr"/>
@@ -11132,7 +11249,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>鎧真伝サムライトルーパー 第2クール</t>
+          <t>無職転生Ⅲ ～異世界行ったら本気だす～</t>
         </is>
       </c>
       <c r="D96" t="b">
@@ -11144,16 +11261,16 @@
         </is>
       </c>
       <c r="F96" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>ばけもん</t>
+          <t>祈り、終われば</t>
         </is>
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>カラノア</t>
+          <t>中島美嘉</t>
         </is>
       </c>
       <c r="I96" t="inlineStr"/>
@@ -11175,7 +11292,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>落第賢者の学院無双～二度目の転生、Sランクチート魔術師冒険録～</t>
+          <t>メビウス・ダスト</t>
         </is>
       </c>
       <c r="D97" t="b">
@@ -11191,12 +11308,12 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>＋ENCOUNT</t>
+          <t>メビウス</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>FLOW</t>
+          <t>家入レオ</t>
         </is>
       </c>
       <c r="I97" t="inlineStr"/>
@@ -11218,7 +11335,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>落第賢者の学院無双～二度目の転生、Sランクチート魔術師冒険録～</t>
+          <t>メビウス・ダスト</t>
         </is>
       </c>
       <c r="D98" t="b">
@@ -11234,12 +11351,12 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>憧憬</t>
+          <t>ジレンマ</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>TrySail</t>
+          <t>冨岡愛</t>
         </is>
       </c>
       <c r="I98" t="inlineStr"/>
@@ -11261,7 +11378,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>領民0人スタートの辺境領主様</t>
+          <t>ヤニねこ</t>
         </is>
       </c>
       <c r="D99" t="b">
@@ -11277,12 +11394,12 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>Wonder</t>
+          <t>なんもねえ</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>CROWN HEAD</t>
+          <t>忘れらんねえよ</t>
         </is>
       </c>
       <c r="I99" t="inlineStr"/>
@@ -11304,7 +11421,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>領民0人スタートの辺境領主様</t>
+          <t>幼女戦記Ⅱ</t>
         </is>
       </c>
       <c r="D100" t="b">
@@ -11312,7 +11429,7 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F100" t="n">
@@ -11320,12 +11437,12 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>星降る夜の約束</t>
+          <t>Why? RED induction</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>花耶</t>
+          <t>MYTH &amp; ROID</t>
         </is>
       </c>
       <c r="I100" t="inlineStr"/>
@@ -11347,7 +11464,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>令和のダラさん</t>
+          <t>幼女戦記Ⅱ</t>
         </is>
       </c>
       <c r="D101" t="b">
@@ -11355,7 +11472,7 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F101" t="n">
@@ -11363,12 +11480,12 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>ダラダラ♡ダンシング</t>
+          <t>Weiter! Weiter!</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>ダラさん（CV：田村睦心） 三⼗⽊⾕⽇向（CV：津田美波） 三⼗⽊⾕薫（CV：寺澤百花） ナレーション（CV：てらそままさき）</t>
+          <t>ターニャ・デグレチャフ（CV：悠木碧）</t>
         </is>
       </c>
       <c r="I101" t="inlineStr"/>
@@ -11390,7 +11507,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>令和のダラさん</t>
+          <t>鎧真伝サムライトルーパー 第2クール</t>
         </is>
       </c>
       <c r="D102" t="b">
@@ -11398,7 +11515,7 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F102" t="n">
@@ -11406,12 +11523,12 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>ひなたぼっこ</t>
+          <t>YOAKE</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>REIRIE</t>
+          <t>blank paper</t>
         </is>
       </c>
       <c r="I102" t="inlineStr"/>
@@ -11433,7 +11550,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>LV999の村人</t>
+          <t>鎧真伝サムライトルーパー 第2クール</t>
         </is>
       </c>
       <c r="D103" t="b">
@@ -11445,16 +11562,16 @@
         </is>
       </c>
       <c r="F103" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>Not a Hero</t>
+          <t>BAD遺伝子</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>藍月なくる&amp;棗いつき</t>
+          <t>Dannie May</t>
         </is>
       </c>
       <c r="I103" t="inlineStr"/>
@@ -11476,7 +11593,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>LV999の村人</t>
+          <t>鎧真伝サムライトルーパー 第2クール</t>
         </is>
       </c>
       <c r="D104" t="b">
@@ -11492,12 +11609,12 @@
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>POWER</t>
         </is>
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>ゆきむら。</t>
+          <t>ONE OR EIGHT</t>
         </is>
       </c>
       <c r="I104" t="inlineStr"/>
@@ -11519,7 +11636,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>ワールド イズ ダンシング</t>
+          <t>鎧真伝サムライトルーパー 第2クール</t>
         </is>
       </c>
       <c r="D105" t="b">
@@ -11527,20 +11644,20 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F105" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>終宵</t>
+          <t>ばけもん</t>
         </is>
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>マカロニえんぴつ</t>
+          <t>カラノア</t>
         </is>
       </c>
       <c r="I105" t="inlineStr"/>
@@ -11553,16 +11670,16 @@
     </row>
     <row r="106">
       <c r="A106" t="n">
-        <v>5947</v>
+        <v>5806</v>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>2026秋アニメ</t>
+          <t>2026夏アニメ</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>帰還者の魔法は特別です 第2期</t>
+          <t>落第賢者の学院無双～二度目の転生、Sランクチート魔術師冒険録～</t>
         </is>
       </c>
       <c r="D106" t="b">
@@ -11578,7 +11695,7 @@
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>Sorrow</t>
+          <t>＋ENCOUNT</t>
         </is>
       </c>
       <c r="H106" t="inlineStr">
@@ -11596,16 +11713,16 @@
     </row>
     <row r="107">
       <c r="A107" t="n">
-        <v>5947</v>
+        <v>5806</v>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>2026秋アニメ</t>
+          <t>2026夏アニメ</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>獣王武神ダンデヴァイン</t>
+          <t>落第賢者の学院無双～二度目の転生、Sランクチート魔術師冒険録～</t>
         </is>
       </c>
       <c r="D107" t="b">
@@ -11613,7 +11730,7 @@
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F107" t="n">
@@ -11621,12 +11738,12 @@
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>曲名未発表</t>
+          <t>憧憬</t>
         </is>
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>西川貴教</t>
+          <t>TrySail</t>
         </is>
       </c>
       <c r="I107" t="inlineStr"/>
@@ -11639,16 +11756,16 @@
     </row>
     <row r="108">
       <c r="A108" t="n">
-        <v>5947</v>
+        <v>5806</v>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>2026秋アニメ</t>
+          <t>2026夏アニメ</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>転生した大聖女は、聖女であることをひた隠す</t>
+          <t>領民0人スタートの辺境領主様</t>
         </is>
       </c>
       <c r="D108" t="b">
@@ -11664,12 +11781,12 @@
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>Flare of Soul</t>
+          <t>Wonder</t>
         </is>
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>花耶</t>
+          <t>CROWN HEAD</t>
         </is>
       </c>
       <c r="I108" t="inlineStr"/>
@@ -11682,16 +11799,16 @@
     </row>
     <row r="109">
       <c r="A109" t="n">
-        <v>5947</v>
+        <v>5806</v>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>2026秋アニメ</t>
+          <t>2026夏アニメ</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>転生した大聖女は、聖女であることをひた隠す</t>
+          <t>領民0人スタートの辺境領主様</t>
         </is>
       </c>
       <c r="D109" t="b">
@@ -11707,12 +11824,12 @@
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>STELLAR</t>
+          <t>星降る夜の約束</t>
         </is>
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>ウタヒメドリーム オールスターズ</t>
+          <t>花耶</t>
         </is>
       </c>
       <c r="I109" t="inlineStr"/>
@@ -11725,16 +11842,16 @@
     </row>
     <row r="110">
       <c r="A110" t="n">
-        <v>5947</v>
+        <v>5806</v>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>2026秋アニメ</t>
+          <t>2026夏アニメ</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>魔法少女育成計画restart</t>
+          <t>令和のダラさん</t>
         </is>
       </c>
       <c r="D110" t="b">
@@ -11750,12 +11867,12 @@
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>No tears here</t>
+          <t>ダラダラ♡ダンシング</t>
         </is>
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>茅原実里</t>
+          <t>ダラさん（CV：田村睦心） 三⼗⽊⾕⽇向（CV：津田美波） 三⼗⽊⾕薫（CV：寺澤百花） ナレーション（CV：てらそままさき）</t>
         </is>
       </c>
       <c r="I110" t="inlineStr"/>
@@ -11766,6 +11883,436 @@
       <c r="N110" t="inlineStr"/>
       <c r="O110" t="inlineStr"/>
     </row>
+    <row r="111">
+      <c r="A111" t="n">
+        <v>5806</v>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>2026夏アニメ</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>令和のダラさん</t>
+        </is>
+      </c>
+      <c r="D111" t="b">
+        <v>0</v>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>ED</t>
+        </is>
+      </c>
+      <c r="F111" t="n">
+        <v>1</v>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>ひなたぼっこ</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>REIRIE</t>
+        </is>
+      </c>
+      <c r="I111" t="inlineStr"/>
+      <c r="J111" t="inlineStr"/>
+      <c r="K111" t="inlineStr"/>
+      <c r="L111" t="inlineStr"/>
+      <c r="M111" t="inlineStr"/>
+      <c r="N111" t="inlineStr"/>
+      <c r="O111" t="inlineStr"/>
+    </row>
+    <row r="112">
+      <c r="A112" t="n">
+        <v>5806</v>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>2026夏アニメ</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>LV999の村人</t>
+        </is>
+      </c>
+      <c r="D112" t="b">
+        <v>0</v>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="F112" t="n">
+        <v>1</v>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>Not a Hero</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>藍月なくる&amp;棗いつき</t>
+        </is>
+      </c>
+      <c r="I112" t="inlineStr"/>
+      <c r="J112" t="inlineStr"/>
+      <c r="K112" t="inlineStr"/>
+      <c r="L112" t="inlineStr"/>
+      <c r="M112" t="inlineStr"/>
+      <c r="N112" t="inlineStr"/>
+      <c r="O112" t="inlineStr"/>
+    </row>
+    <row r="113">
+      <c r="A113" t="n">
+        <v>5806</v>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>2026夏アニメ</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>LV999の村人</t>
+        </is>
+      </c>
+      <c r="D113" t="b">
+        <v>0</v>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>ED</t>
+        </is>
+      </c>
+      <c r="F113" t="n">
+        <v>1</v>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>HP</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>ゆきむら。</t>
+        </is>
+      </c>
+      <c r="I113" t="inlineStr"/>
+      <c r="J113" t="inlineStr"/>
+      <c r="K113" t="inlineStr"/>
+      <c r="L113" t="inlineStr"/>
+      <c r="M113" t="inlineStr"/>
+      <c r="N113" t="inlineStr"/>
+      <c r="O113" t="inlineStr"/>
+    </row>
+    <row r="114">
+      <c r="A114" t="n">
+        <v>5806</v>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>2026夏アニメ</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>ワールド イズ ダンシング</t>
+        </is>
+      </c>
+      <c r="D114" t="b">
+        <v>0</v>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="F114" t="n">
+        <v>1</v>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>終宵</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>マカロニえんぴつ</t>
+        </is>
+      </c>
+      <c r="I114" t="inlineStr"/>
+      <c r="J114" t="inlineStr"/>
+      <c r="K114" t="inlineStr"/>
+      <c r="L114" t="inlineStr"/>
+      <c r="M114" t="inlineStr"/>
+      <c r="N114" t="inlineStr"/>
+      <c r="O114" t="inlineStr"/>
+    </row>
+    <row r="115">
+      <c r="A115" t="n">
+        <v>5806</v>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>2026夏アニメ</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>ONE PIECE HEROINES</t>
+        </is>
+      </c>
+      <c r="D115" t="b">
+        <v>0</v>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>主題歌</t>
+        </is>
+      </c>
+      <c r="F115" t="n">
+        <v>1</v>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>ONE PIECE（モノクロ版）</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>電子書籍（コミック）</t>
+        </is>
+      </c>
+      <c r="I115" t="inlineStr"/>
+      <c r="J115" t="inlineStr"/>
+      <c r="K115" t="inlineStr"/>
+      <c r="L115" t="inlineStr"/>
+      <c r="M115" t="inlineStr"/>
+      <c r="N115" t="inlineStr"/>
+      <c r="O115" t="inlineStr"/>
+    </row>
+    <row r="116">
+      <c r="A116" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>帰還者の魔法は特別です 第2期</t>
+        </is>
+      </c>
+      <c r="D116" t="b">
+        <v>0</v>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="F116" t="n">
+        <v>1</v>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>Sorrow</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>FLOW</t>
+        </is>
+      </c>
+      <c r="I116" t="inlineStr"/>
+      <c r="J116" t="inlineStr"/>
+      <c r="K116" t="inlineStr"/>
+      <c r="L116" t="inlineStr"/>
+      <c r="M116" t="inlineStr"/>
+      <c r="N116" t="inlineStr"/>
+      <c r="O116" t="inlineStr"/>
+    </row>
+    <row r="117">
+      <c r="A117" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>獣王武神ダンデヴァイン</t>
+        </is>
+      </c>
+      <c r="D117" t="b">
+        <v>0</v>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="F117" t="n">
+        <v>1</v>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>曲名未発表</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>西川貴教</t>
+        </is>
+      </c>
+      <c r="I117" t="inlineStr"/>
+      <c r="J117" t="inlineStr"/>
+      <c r="K117" t="inlineStr"/>
+      <c r="L117" t="inlineStr"/>
+      <c r="M117" t="inlineStr"/>
+      <c r="N117" t="inlineStr"/>
+      <c r="O117" t="inlineStr"/>
+    </row>
+    <row r="118">
+      <c r="A118" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>転生した大聖女は、聖女であることをひた隠す</t>
+        </is>
+      </c>
+      <c r="D118" t="b">
+        <v>0</v>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="F118" t="n">
+        <v>1</v>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>Flare of Soul</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>花耶</t>
+        </is>
+      </c>
+      <c r="I118" t="inlineStr"/>
+      <c r="J118" t="inlineStr"/>
+      <c r="K118" t="inlineStr"/>
+      <c r="L118" t="inlineStr"/>
+      <c r="M118" t="inlineStr"/>
+      <c r="N118" t="inlineStr"/>
+      <c r="O118" t="inlineStr"/>
+    </row>
+    <row r="119">
+      <c r="A119" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>転生した大聖女は、聖女であることをひた隠す</t>
+        </is>
+      </c>
+      <c r="D119" t="b">
+        <v>0</v>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>ED</t>
+        </is>
+      </c>
+      <c r="F119" t="n">
+        <v>1</v>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>STELLAR</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>ウタヒメドリーム オールスターズ</t>
+        </is>
+      </c>
+      <c r="I119" t="inlineStr"/>
+      <c r="J119" t="inlineStr"/>
+      <c r="K119" t="inlineStr"/>
+      <c r="L119" t="inlineStr"/>
+      <c r="M119" t="inlineStr"/>
+      <c r="N119" t="inlineStr"/>
+      <c r="O119" t="inlineStr"/>
+    </row>
+    <row r="120">
+      <c r="A120" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>魔法少女育成計画restart</t>
+        </is>
+      </c>
+      <c r="D120" t="b">
+        <v>0</v>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="F120" t="n">
+        <v>1</v>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>No tears here</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>茅原実里</t>
+        </is>
+      </c>
+      <c r="I120" t="inlineStr"/>
+      <c r="J120" t="inlineStr"/>
+      <c r="K120" t="inlineStr"/>
+      <c r="L120" t="inlineStr"/>
+      <c r="M120" t="inlineStr"/>
+      <c r="N120" t="inlineStr"/>
+      <c r="O120" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
auto: anime list update (PC) 2026-06-21
</commit_message>
<xml_diff>
--- a/data/anime_list.xlsx
+++ b/data/anime_list.xlsx
@@ -18,13 +18,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -35,7 +38,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -43,12 +46,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -418,67 +430,67 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>season_id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>season_label</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>order</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>title</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>is_rerun</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>broadcast_format</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>broadcast_start</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>animation_studio</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>op_title</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>op_artist</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>ed_title</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>ed_artist</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>detail_url</t>
         </is>
@@ -7476,77 +7488,77 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>season_id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>season_label</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>anime_title</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>is_rerun</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>kind</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>index</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>song_title</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>artist</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>youtube_url</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>youtube_views</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>youtube_channel</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>anime_youtube_url</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>anime_youtube_views</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>anime_youtube_channel</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>last_searched_at</t>
         </is>
@@ -7587,13 +7599,37 @@
           <t>榊原ゆい</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=KJkoRG38MXo</t>
+        </is>
+      </c>
+      <c r="J2" t="n">
+        <v>52344</v>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>アズールレーン</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=bFCBwBCTCBU</t>
+        </is>
+      </c>
+      <c r="M2" t="n">
+        <v>26101</v>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>SHOCHIKU anime Channel</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>2026-06-21T18:13:31</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -7845,13 +7881,37 @@
           <t>ORCALAND</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
-      <c r="O8" t="inlineStr"/>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=fI6BUhMXqKQ</t>
+        </is>
+      </c>
+      <c r="J8" t="n">
+        <v>22060</v>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>デレギュラ【新アニメレーベル】</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=fI6BUhMXqKQ</t>
+        </is>
+      </c>
+      <c r="M8" t="n">
+        <v>22060</v>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>デレギュラ【新アニメレーベル】</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>2026-06-21T18:14:06</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -7888,13 +7948,37 @@
           <t>KOTOKO</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" t="inlineStr"/>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=mcFFaGYC9JU</t>
+        </is>
+      </c>
+      <c r="J9" t="n">
+        <v>20903</v>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>デレギュラ【新アニメレーベル】</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=mcFFaGYC9JU</t>
+        </is>
+      </c>
+      <c r="M9" t="n">
+        <v>20903</v>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>デレギュラ【新アニメレーベル】</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>2026-06-21T18:14:12</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -7931,13 +8015,37 @@
           <t>DISH//</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
-      <c r="O10" t="inlineStr"/>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=8So8zgJAYMI</t>
+        </is>
+      </c>
+      <c r="J10" t="n">
+        <v>6811</v>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>アニプレックス チャンネル</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=8So8zgJAYMI</t>
+        </is>
+      </c>
+      <c r="M10" t="n">
+        <v>6811</v>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>アニプレックス チャンネル</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>2026-06-21T18:14:24</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -7974,13 +8082,37 @@
           <t>汐れいら</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr"/>
-      <c r="O11" t="inlineStr"/>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=6fUdDUk-FZQ</t>
+        </is>
+      </c>
+      <c r="J11" t="n">
+        <v>3487</v>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>アニプレックス チャンネル</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=6fUdDUk-FZQ</t>
+        </is>
+      </c>
+      <c r="M11" t="n">
+        <v>3487</v>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>アニプレックス チャンネル</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>2026-06-21T18:14:33</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -8404,13 +8536,27 @@
           <t>DIALOGUE+</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=YCCI6qrDhow</t>
+        </is>
+      </c>
+      <c r="J21" t="n">
+        <v>362547</v>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>DIALOGUE＋Official Channel</t>
+        </is>
+      </c>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="inlineStr"/>
       <c r="N21" t="inlineStr"/>
-      <c r="O21" t="inlineStr"/>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>2026-06-21T18:16:17</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -8533,13 +8679,27 @@
           <t>syudou×八木勇征(FANTASTICS)</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr"/>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=46w2OsPayB4</t>
+        </is>
+      </c>
+      <c r="J24" t="n">
+        <v>13154</v>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>TVアニメ『株式会社マジルミエ』公式チャンネル</t>
+        </is>
+      </c>
       <c r="L24" t="inlineStr"/>
       <c r="M24" t="inlineStr"/>
       <c r="N24" t="inlineStr"/>
-      <c r="O24" t="inlineStr"/>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>2026-06-21T18:16:54</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -8576,13 +8736,37 @@
           <t>宝鐘マリン</t>
         </is>
       </c>
-      <c r="I25" t="inlineStr"/>
-      <c r="J25" t="inlineStr"/>
-      <c r="K25" t="inlineStr"/>
-      <c r="L25" t="inlineStr"/>
-      <c r="M25" t="inlineStr"/>
-      <c r="N25" t="inlineStr"/>
-      <c r="O25" t="inlineStr"/>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=2_opjVlYhi4</t>
+        </is>
+      </c>
+      <c r="J25" t="n">
+        <v>16610711</v>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>Marine Ch. 宝鐘マリン</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=R6oIaWuN0lk</t>
+        </is>
+      </c>
+      <c r="M25" t="n">
+        <v>223037</v>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>TVアニメ『株式会社マジルミエ』公式チャンネル</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>2026-06-21T18:17:17</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -8754,7 +8938,7 @@
         </is>
       </c>
       <c r="J29" t="n">
-        <v>1654</v>
+        <v>1851</v>
       </c>
       <c r="K29" t="inlineStr">
         <is>
@@ -8766,7 +8950,7 @@
       <c r="N29" t="inlineStr"/>
       <c r="O29" t="inlineStr">
         <is>
-          <t>2026-06-14T18:14:57</t>
+          <t>2026-06-21T18:17:42</t>
         </is>
       </c>
     </row>
@@ -8934,13 +9118,37 @@
           <t>豆柴の大群</t>
         </is>
       </c>
-      <c r="I33" t="inlineStr"/>
-      <c r="J33" t="inlineStr"/>
-      <c r="K33" t="inlineStr"/>
-      <c r="L33" t="inlineStr"/>
-      <c r="M33" t="inlineStr"/>
-      <c r="N33" t="inlineStr"/>
-      <c r="O33" t="inlineStr"/>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=_gLM5qjn5Hk</t>
+        </is>
+      </c>
+      <c r="J33" t="n">
+        <v>466412</v>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>NBCUniversal Anime/Music</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=_gLM5qjn5Hk</t>
+        </is>
+      </c>
+      <c r="M33" t="n">
+        <v>466412</v>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>NBCUniversal Anime/Music</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>2026-06-21T18:18:12</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -9063,13 +9271,37 @@
           <t>NOMELON NOLEMON</t>
         </is>
       </c>
-      <c r="I36" t="inlineStr"/>
-      <c r="J36" t="inlineStr"/>
-      <c r="K36" t="inlineStr"/>
-      <c r="L36" t="inlineStr"/>
-      <c r="M36" t="inlineStr"/>
-      <c r="N36" t="inlineStr"/>
-      <c r="O36" t="inlineStr"/>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=IYW8Mfdzwfo</t>
+        </is>
+      </c>
+      <c r="J36" t="n">
+        <v>11744</v>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>アニプレックス チャンネル</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=IYW8Mfdzwfo</t>
+        </is>
+      </c>
+      <c r="M36" t="n">
+        <v>11744</v>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>アニプレックス チャンネル</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>2026-06-21T18:18:28</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -9106,13 +9338,37 @@
           <t>Aooo</t>
         </is>
       </c>
-      <c r="I37" t="inlineStr"/>
-      <c r="J37" t="inlineStr"/>
-      <c r="K37" t="inlineStr"/>
-      <c r="L37" t="inlineStr"/>
-      <c r="M37" t="inlineStr"/>
-      <c r="N37" t="inlineStr"/>
-      <c r="O37" t="inlineStr"/>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=_HJ9d-6oNt4</t>
+        </is>
+      </c>
+      <c r="J37" t="n">
+        <v>13489</v>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>アニプレックス チャンネル</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=_HJ9d-6oNt4</t>
+        </is>
+      </c>
+      <c r="M37" t="n">
+        <v>13489</v>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>アニプレックス チャンネル</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>2026-06-21T18:18:33</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -9149,13 +9405,27 @@
           <t>MILLENNIUM PARADE feat. Saya Gray, Daniel Caesar</t>
         </is>
       </c>
-      <c r="I38" t="inlineStr"/>
-      <c r="J38" t="inlineStr"/>
-      <c r="K38" t="inlineStr"/>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=fuXZMQAD9vU</t>
+        </is>
+      </c>
+      <c r="J38" t="n">
+        <v>12852008</v>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>MILLENNIUM PARADE Official YouTube Channel</t>
+        </is>
+      </c>
       <c r="L38" t="inlineStr"/>
       <c r="M38" t="inlineStr"/>
       <c r="N38" t="inlineStr"/>
-      <c r="O38" t="inlineStr"/>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>2026-06-21T18:19:08</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -9192,13 +9462,27 @@
           <t>MIYAVI</t>
         </is>
       </c>
-      <c r="I39" t="inlineStr"/>
-      <c r="J39" t="inlineStr"/>
-      <c r="K39" t="inlineStr"/>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=0ym3Zj4kJyo</t>
+        </is>
+      </c>
+      <c r="J39" t="n">
+        <v>295392</v>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>コードギアスチャンネル CODEGEASS Channel</t>
+        </is>
+      </c>
       <c r="L39" t="inlineStr"/>
       <c r="M39" t="inlineStr"/>
       <c r="N39" t="inlineStr"/>
-      <c r="O39" t="inlineStr"/>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>2026-06-21T18:19:26</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -9235,13 +9519,27 @@
           <t>満島ひかり</t>
         </is>
       </c>
-      <c r="I40" t="inlineStr"/>
-      <c r="J40" t="inlineStr"/>
-      <c r="K40" t="inlineStr"/>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=0ym3Zj4kJyo</t>
+        </is>
+      </c>
+      <c r="J40" t="n">
+        <v>295392</v>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>コードギアスチャンネル CODEGEASS Channel</t>
+        </is>
+      </c>
       <c r="L40" t="inlineStr"/>
       <c r="M40" t="inlineStr"/>
       <c r="N40" t="inlineStr"/>
-      <c r="O40" t="inlineStr"/>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>2026-06-21T18:19:43</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -9364,13 +9662,27 @@
           <t>キタニタツヤ</t>
         </is>
       </c>
-      <c r="I43" t="inlineStr"/>
-      <c r="J43" t="inlineStr"/>
-      <c r="K43" t="inlineStr"/>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=MQhd0ne_uYo</t>
+        </is>
+      </c>
+      <c r="J43" t="n">
+        <v>6682341</v>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>キタニタツヤ / Tatsuya Kitani</t>
+        </is>
+      </c>
       <c r="L43" t="inlineStr"/>
       <c r="M43" t="inlineStr"/>
       <c r="N43" t="inlineStr"/>
-      <c r="O43" t="inlineStr"/>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>2026-06-21T18:20:22</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -9407,13 +9719,37 @@
           <t>リーガルリリー</t>
         </is>
       </c>
-      <c r="I44" t="inlineStr"/>
-      <c r="J44" t="inlineStr"/>
-      <c r="K44" t="inlineStr"/>
-      <c r="L44" t="inlineStr"/>
-      <c r="M44" t="inlineStr"/>
-      <c r="N44" t="inlineStr"/>
-      <c r="O44" t="inlineStr"/>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=jI61NtGuxV4</t>
+        </is>
+      </c>
+      <c r="J44" t="n">
+        <v>42562</v>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>VAP Official</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=GVgOmS-7xBg</t>
+        </is>
+      </c>
+      <c r="M44" t="n">
+        <v>145</v>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>Anime Pulse Japan ⚡</t>
+        </is>
+      </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>2026-06-21T18:20:33</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -9579,13 +9915,27 @@
           <t>前島亜美</t>
         </is>
       </c>
-      <c r="I48" t="inlineStr"/>
-      <c r="J48" t="inlineStr"/>
-      <c r="K48" t="inlineStr"/>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=BnQf97HkufE</t>
+        </is>
+      </c>
+      <c r="J48" t="n">
+        <v>4032</v>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>前島亜美</t>
+        </is>
+      </c>
       <c r="L48" t="inlineStr"/>
       <c r="M48" t="inlineStr"/>
       <c r="N48" t="inlineStr"/>
-      <c r="O48" t="inlineStr"/>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>2026-06-21T18:21:04</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -9622,13 +9972,27 @@
           <t>杏子</t>
         </is>
       </c>
-      <c r="I49" t="inlineStr"/>
-      <c r="J49" t="inlineStr"/>
-      <c r="K49" t="inlineStr"/>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=wc1Npu2_IFs</t>
+        </is>
+      </c>
+      <c r="J49" t="n">
+        <v>13236</v>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>杏子</t>
+        </is>
+      </c>
       <c r="L49" t="inlineStr"/>
       <c r="M49" t="inlineStr"/>
       <c r="N49" t="inlineStr"/>
-      <c r="O49" t="inlineStr"/>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>2026-06-21T18:21:26</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -9665,13 +10029,37 @@
           <t>いきものがかり</t>
         </is>
       </c>
-      <c r="I50" t="inlineStr"/>
-      <c r="J50" t="inlineStr"/>
-      <c r="K50" t="inlineStr"/>
-      <c r="L50" t="inlineStr"/>
-      <c r="M50" t="inlineStr"/>
-      <c r="N50" t="inlineStr"/>
-      <c r="O50" t="inlineStr"/>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=c4-6PwVRRj8</t>
+        </is>
+      </c>
+      <c r="J50" t="n">
+        <v>305568</v>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=c4-6PwVRRj8</t>
+        </is>
+      </c>
+      <c r="M50" t="n">
+        <v>305568</v>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>2026-06-21T18:21:38</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -9751,13 +10139,37 @@
           <t>ずっと真夜中でいいのに。</t>
         </is>
       </c>
-      <c r="I52" t="inlineStr"/>
-      <c r="J52" t="inlineStr"/>
-      <c r="K52" t="inlineStr"/>
-      <c r="L52" t="inlineStr"/>
-      <c r="M52" t="inlineStr"/>
-      <c r="N52" t="inlineStr"/>
-      <c r="O52" t="inlineStr"/>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=ut889MZ9yNo</t>
+        </is>
+      </c>
+      <c r="J52" t="n">
+        <v>6309471</v>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>ずっと真夜中でいいのに。 ZUTOMAYO</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=OUmtsSroxns</t>
+        </is>
+      </c>
+      <c r="M52" t="n">
+        <v>594902</v>
+      </c>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>Asmik Ace</t>
+        </is>
+      </c>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>2026-06-21T18:21:56</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -9794,13 +10206,37 @@
           <t>imase</t>
         </is>
       </c>
-      <c r="I53" t="inlineStr"/>
-      <c r="J53" t="inlineStr"/>
-      <c r="K53" t="inlineStr"/>
-      <c r="L53" t="inlineStr"/>
-      <c r="M53" t="inlineStr"/>
-      <c r="N53" t="inlineStr"/>
-      <c r="O53" t="inlineStr"/>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=9eo3M7-wAtU</t>
+        </is>
+      </c>
+      <c r="J53" t="n">
+        <v>867945</v>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>Asmik Ace</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=9eo3M7-wAtU</t>
+        </is>
+      </c>
+      <c r="M53" t="n">
+        <v>867945</v>
+      </c>
+      <c r="N53" t="inlineStr">
+        <is>
+          <t>Asmik Ace</t>
+        </is>
+      </c>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>2026-06-21T18:22:09</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -10009,13 +10445,37 @@
           <t>乃紫</t>
         </is>
       </c>
-      <c r="I58" t="inlineStr"/>
-      <c r="J58" t="inlineStr"/>
-      <c r="K58" t="inlineStr"/>
-      <c r="L58" t="inlineStr"/>
-      <c r="M58" t="inlineStr"/>
-      <c r="N58" t="inlineStr"/>
-      <c r="O58" t="inlineStr"/>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=XOKQluw_YLU</t>
+        </is>
+      </c>
+      <c r="J58" t="n">
+        <v>3803168</v>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>乃紫</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=JIn6WqZ_Fs4</t>
+        </is>
+      </c>
+      <c r="M58" t="n">
+        <v>1711081</v>
+      </c>
+      <c r="N58" t="inlineStr">
+        <is>
+          <t>SHOCHIKU anime Channel</t>
+        </is>
+      </c>
+      <c r="O58" t="inlineStr">
+        <is>
+          <t>2026-06-21T18:22:34</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -10052,13 +10512,37 @@
           <t>7co</t>
         </is>
       </c>
-      <c r="I59" t="inlineStr"/>
-      <c r="J59" t="inlineStr"/>
-      <c r="K59" t="inlineStr"/>
-      <c r="L59" t="inlineStr"/>
-      <c r="M59" t="inlineStr"/>
-      <c r="N59" t="inlineStr"/>
-      <c r="O59" t="inlineStr"/>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=JIn6WqZ_Fs4</t>
+        </is>
+      </c>
+      <c r="J59" t="n">
+        <v>1711081</v>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>SHOCHIKU anime Channel</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=JIn6WqZ_Fs4</t>
+        </is>
+      </c>
+      <c r="M59" t="n">
+        <v>1711081</v>
+      </c>
+      <c r="N59" t="inlineStr">
+        <is>
+          <t>SHOCHIKU anime Channel</t>
+        </is>
+      </c>
+      <c r="O59" t="inlineStr">
+        <is>
+          <t>2026-06-21T18:22:43</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -10095,13 +10579,37 @@
           <t>PAS TASTA</t>
         </is>
       </c>
-      <c r="I60" t="inlineStr"/>
-      <c r="J60" t="inlineStr"/>
-      <c r="K60" t="inlineStr"/>
-      <c r="L60" t="inlineStr"/>
-      <c r="M60" t="inlineStr"/>
-      <c r="N60" t="inlineStr"/>
-      <c r="O60" t="inlineStr"/>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=A6aH9jPW8ZY</t>
+        </is>
+      </c>
+      <c r="J60" t="n">
+        <v>273328</v>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>SHOCHIKU anime Channel</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=A6aH9jPW8ZY</t>
+        </is>
+      </c>
+      <c r="M60" t="n">
+        <v>273328</v>
+      </c>
+      <c r="N60" t="inlineStr">
+        <is>
+          <t>SHOCHIKU anime Channel</t>
+        </is>
+      </c>
+      <c r="O60" t="inlineStr">
+        <is>
+          <t>2026-06-21T18:22:55</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -10439,13 +10947,37 @@
           <t>KI_EN</t>
         </is>
       </c>
-      <c r="I68" t="inlineStr"/>
-      <c r="J68" t="inlineStr"/>
-      <c r="K68" t="inlineStr"/>
-      <c r="L68" t="inlineStr"/>
-      <c r="M68" t="inlineStr"/>
-      <c r="N68" t="inlineStr"/>
-      <c r="O68" t="inlineStr"/>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=-HNOXWE2wVU</t>
+        </is>
+      </c>
+      <c r="J68" t="n">
+        <v>140125</v>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=-HNOXWE2wVU</t>
+        </is>
+      </c>
+      <c r="M68" t="n">
+        <v>140125</v>
+      </c>
+      <c r="N68" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="O68" t="inlineStr">
+        <is>
+          <t>2026-06-21T18:23:55</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -10525,13 +11057,27 @@
           <t>七海ひろき</t>
         </is>
       </c>
-      <c r="I70" t="inlineStr"/>
-      <c r="J70" t="inlineStr"/>
-      <c r="K70" t="inlineStr"/>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=qpFcQ1Bek08</t>
+        </is>
+      </c>
+      <c r="J70" t="n">
+        <v>69452</v>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>VAP Official</t>
+        </is>
+      </c>
       <c r="L70" t="inlineStr"/>
       <c r="M70" t="inlineStr"/>
       <c r="N70" t="inlineStr"/>
-      <c r="O70" t="inlineStr"/>
+      <c r="O70" t="inlineStr">
+        <is>
+          <t>2026-06-21T18:24:32</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -10869,13 +11415,37 @@
           <t>Ginger Root</t>
         </is>
       </c>
-      <c r="I78" t="inlineStr"/>
-      <c r="J78" t="inlineStr"/>
-      <c r="K78" t="inlineStr"/>
-      <c r="L78" t="inlineStr"/>
-      <c r="M78" t="inlineStr"/>
-      <c r="N78" t="inlineStr"/>
-      <c r="O78" t="inlineStr"/>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=5rQWh9aIflw</t>
+        </is>
+      </c>
+      <c r="J78" t="n">
+        <v>3207</v>
+      </c>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>Lantis Channel</t>
+        </is>
+      </c>
+      <c r="L78" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=5rQWh9aIflw</t>
+        </is>
+      </c>
+      <c r="M78" t="n">
+        <v>3207</v>
+      </c>
+      <c r="N78" t="inlineStr">
+        <is>
+          <t>Lantis Channel</t>
+        </is>
+      </c>
+      <c r="O78" t="inlineStr">
+        <is>
+          <t>2026-06-21T18:26:16</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -10955,13 +11525,37 @@
           <t>WANIMA</t>
         </is>
       </c>
-      <c r="I80" t="inlineStr"/>
-      <c r="J80" t="inlineStr"/>
-      <c r="K80" t="inlineStr"/>
-      <c r="L80" t="inlineStr"/>
-      <c r="M80" t="inlineStr"/>
-      <c r="N80" t="inlineStr"/>
-      <c r="O80" t="inlineStr"/>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=3KIPGQJh4vI</t>
+        </is>
+      </c>
+      <c r="J80" t="n">
+        <v>402991</v>
+      </c>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>TMSアニメ公式チャンネル</t>
+        </is>
+      </c>
+      <c r="L80" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=3KIPGQJh4vI</t>
+        </is>
+      </c>
+      <c r="M80" t="n">
+        <v>402991</v>
+      </c>
+      <c r="N80" t="inlineStr">
+        <is>
+          <t>TMSアニメ公式チャンネル</t>
+        </is>
+      </c>
+      <c r="O80" t="inlineStr">
+        <is>
+          <t>2026-06-21T18:26:31</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -10998,13 +11592,37 @@
           <t>Chevon</t>
         </is>
       </c>
-      <c r="I81" t="inlineStr"/>
-      <c r="J81" t="inlineStr"/>
-      <c r="K81" t="inlineStr"/>
-      <c r="L81" t="inlineStr"/>
-      <c r="M81" t="inlineStr"/>
-      <c r="N81" t="inlineStr"/>
-      <c r="O81" t="inlineStr"/>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=x0ygvWo5e3k</t>
+        </is>
+      </c>
+      <c r="J81" t="n">
+        <v>174316</v>
+      </c>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>TMSアニメ公式チャンネル</t>
+        </is>
+      </c>
+      <c r="L81" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=x0ygvWo5e3k</t>
+        </is>
+      </c>
+      <c r="M81" t="n">
+        <v>174316</v>
+      </c>
+      <c r="N81" t="inlineStr">
+        <is>
+          <t>TMSアニメ公式チャンネル</t>
+        </is>
+      </c>
+      <c r="O81" t="inlineStr">
+        <is>
+          <t>2026-06-21T18:26:42</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -11041,13 +11659,37 @@
           <t>Novel Core</t>
         </is>
       </c>
-      <c r="I82" t="inlineStr"/>
-      <c r="J82" t="inlineStr"/>
-      <c r="K82" t="inlineStr"/>
-      <c r="L82" t="inlineStr"/>
-      <c r="M82" t="inlineStr"/>
-      <c r="N82" t="inlineStr"/>
-      <c r="O82" t="inlineStr"/>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=KKOr3xF2iOM</t>
+        </is>
+      </c>
+      <c r="J82" t="n">
+        <v>294329</v>
+      </c>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t>TMSアニメ公式チャンネル</t>
+        </is>
+      </c>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=KKOr3xF2iOM</t>
+        </is>
+      </c>
+      <c r="M82" t="n">
+        <v>294329</v>
+      </c>
+      <c r="N82" t="inlineStr">
+        <is>
+          <t>TMSアニメ公式チャンネル</t>
+        </is>
+      </c>
+      <c r="O82" t="inlineStr">
+        <is>
+          <t>2026-06-21T18:26:53</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -11084,13 +11726,37 @@
           <t>三代目 J SOUL BROTHERS</t>
         </is>
       </c>
-      <c r="I83" t="inlineStr"/>
-      <c r="J83" t="inlineStr"/>
-      <c r="K83" t="inlineStr"/>
-      <c r="L83" t="inlineStr"/>
-      <c r="M83" t="inlineStr"/>
-      <c r="N83" t="inlineStr"/>
-      <c r="O83" t="inlineStr"/>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=1LBv6-z-0ok</t>
+        </is>
+      </c>
+      <c r="J83" t="n">
+        <v>25824</v>
+      </c>
+      <c r="K83" t="inlineStr">
+        <is>
+          <t>TMSアニメ公式チャンネル</t>
+        </is>
+      </c>
+      <c r="L83" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=1LBv6-z-0ok</t>
+        </is>
+      </c>
+      <c r="M83" t="n">
+        <v>25824</v>
+      </c>
+      <c r="N83" t="inlineStr">
+        <is>
+          <t>TMSアニメ公式チャンネル</t>
+        </is>
+      </c>
+      <c r="O83" t="inlineStr">
+        <is>
+          <t>2026-06-21T18:27:05</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -11299,13 +11965,27 @@
           <t>小倉唯</t>
         </is>
       </c>
-      <c r="I88" t="inlineStr"/>
-      <c r="J88" t="inlineStr"/>
-      <c r="K88" t="inlineStr"/>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=LFS_qg2JrPI</t>
+        </is>
+      </c>
+      <c r="J88" t="n">
+        <v>11323</v>
+      </c>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>Yui Ogura YouTube OFFICIAL CHANNEL</t>
+        </is>
+      </c>
       <c r="L88" t="inlineStr"/>
       <c r="M88" t="inlineStr"/>
       <c r="N88" t="inlineStr"/>
-      <c r="O88" t="inlineStr"/>
+      <c r="O88" t="inlineStr">
+        <is>
+          <t>2026-06-21T18:27:45</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -11342,13 +12022,27 @@
           <t>大西亜玖璃</t>
         </is>
       </c>
-      <c r="I89" t="inlineStr"/>
-      <c r="J89" t="inlineStr"/>
-      <c r="K89" t="inlineStr"/>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=MzjYjMBpQ6g</t>
+        </is>
+      </c>
+      <c r="J89" t="n">
+        <v>4603</v>
+      </c>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>大西亜玖璃 - Aguri Onishi</t>
+        </is>
+      </c>
       <c r="L89" t="inlineStr"/>
       <c r="M89" t="inlineStr"/>
       <c r="N89" t="inlineStr"/>
-      <c r="O89" t="inlineStr"/>
+      <c r="O89" t="inlineStr">
+        <is>
+          <t>2026-06-21T18:27:58</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -11385,13 +12079,27 @@
           <t>milet</t>
         </is>
       </c>
-      <c r="I90" t="inlineStr"/>
-      <c r="J90" t="inlineStr"/>
-      <c r="K90" t="inlineStr"/>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=nR_vqhD2rGM</t>
+        </is>
+      </c>
+      <c r="J90" t="n">
+        <v>451401</v>
+      </c>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>TOHO animation</t>
+        </is>
+      </c>
       <c r="L90" t="inlineStr"/>
       <c r="M90" t="inlineStr"/>
       <c r="N90" t="inlineStr"/>
-      <c r="O90" t="inlineStr"/>
+      <c r="O90" t="inlineStr">
+        <is>
+          <t>2026-06-21T18:28:12</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -11858,13 +12566,27 @@
           <t>水樹奈々</t>
         </is>
       </c>
-      <c r="I101" t="inlineStr"/>
-      <c r="J101" t="inlineStr"/>
-      <c r="K101" t="inlineStr"/>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=TzvGIjaMbYE</t>
+        </is>
+      </c>
+      <c r="J101" t="n">
+        <v>590624</v>
+      </c>
+      <c r="K101" t="inlineStr">
+        <is>
+          <t>魔法少女リリカルなのは YouTube OFFICIAL CHANNEL</t>
+        </is>
+      </c>
       <c r="L101" t="inlineStr"/>
       <c r="M101" t="inlineStr"/>
       <c r="N101" t="inlineStr"/>
-      <c r="O101" t="inlineStr"/>
+      <c r="O101" t="inlineStr">
+        <is>
+          <t>2026-06-21T18:29:37</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="n">
@@ -11901,13 +12623,27 @@
           <t>青木陽菜</t>
         </is>
       </c>
-      <c r="I102" t="inlineStr"/>
-      <c r="J102" t="inlineStr"/>
-      <c r="K102" t="inlineStr"/>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=TzvGIjaMbYE</t>
+        </is>
+      </c>
+      <c r="J102" t="n">
+        <v>590624</v>
+      </c>
+      <c r="K102" t="inlineStr">
+        <is>
+          <t>魔法少女リリカルなのは YouTube OFFICIAL CHANNEL</t>
+        </is>
+      </c>
       <c r="L102" t="inlineStr"/>
       <c r="M102" t="inlineStr"/>
       <c r="N102" t="inlineStr"/>
-      <c r="O102" t="inlineStr"/>
+      <c r="O102" t="inlineStr">
+        <is>
+          <t>2026-06-21T18:29:56</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="n">
@@ -12030,13 +12766,37 @@
           <t>大原ゆい子</t>
         </is>
       </c>
-      <c r="I105" t="inlineStr"/>
-      <c r="J105" t="inlineStr"/>
-      <c r="K105" t="inlineStr"/>
-      <c r="L105" t="inlineStr"/>
-      <c r="M105" t="inlineStr"/>
-      <c r="N105" t="inlineStr"/>
-      <c r="O105" t="inlineStr"/>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=hZ6TnKvB2rc</t>
+        </is>
+      </c>
+      <c r="J105" t="n">
+        <v>12105753</v>
+      </c>
+      <c r="K105" t="inlineStr">
+        <is>
+          <t>大原ゆい子Official YouTube</t>
+        </is>
+      </c>
+      <c r="L105" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=PINgF6rCuME</t>
+        </is>
+      </c>
+      <c r="M105" t="n">
+        <v>2457533</v>
+      </c>
+      <c r="N105" t="inlineStr">
+        <is>
+          <t>TOHO animation</t>
+        </is>
+      </c>
+      <c r="O105" t="inlineStr">
+        <is>
+          <t>2026-06-21T18:30:35</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="n">
@@ -12073,13 +12833,27 @@
           <t>中島美嘉</t>
         </is>
       </c>
-      <c r="I106" t="inlineStr"/>
-      <c r="J106" t="inlineStr"/>
-      <c r="K106" t="inlineStr"/>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=ODxfIvSgWuo</t>
+        </is>
+      </c>
+      <c r="J106" t="n">
+        <v>1140774</v>
+      </c>
+      <c r="K106" t="inlineStr">
+        <is>
+          <t>TOHO animation</t>
+        </is>
+      </c>
       <c r="L106" t="inlineStr"/>
       <c r="M106" t="inlineStr"/>
       <c r="N106" t="inlineStr"/>
-      <c r="O106" t="inlineStr"/>
+      <c r="O106" t="inlineStr">
+        <is>
+          <t>2026-06-21T18:31:08</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="n">
@@ -12116,13 +12890,37 @@
           <t>家入レオ</t>
         </is>
       </c>
-      <c r="I107" t="inlineStr"/>
-      <c r="J107" t="inlineStr"/>
-      <c r="K107" t="inlineStr"/>
-      <c r="L107" t="inlineStr"/>
-      <c r="M107" t="inlineStr"/>
-      <c r="N107" t="inlineStr"/>
-      <c r="O107" t="inlineStr"/>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=vJzWWkigrU8</t>
+        </is>
+      </c>
+      <c r="J107" t="n">
+        <v>32222</v>
+      </c>
+      <c r="K107" t="inlineStr">
+        <is>
+          <t>家入レオ</t>
+        </is>
+      </c>
+      <c r="L107" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=5QGZX_Kky4I</t>
+        </is>
+      </c>
+      <c r="M107" t="n">
+        <v>27576</v>
+      </c>
+      <c r="N107" t="inlineStr">
+        <is>
+          <t>leafstamp</t>
+        </is>
+      </c>
+      <c r="O107" t="inlineStr">
+        <is>
+          <t>2026-06-21T18:31:32</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="n">
@@ -12202,13 +13000,27 @@
           <t>忘れらんねえよ</t>
         </is>
       </c>
-      <c r="I109" t="inlineStr"/>
-      <c r="J109" t="inlineStr"/>
-      <c r="K109" t="inlineStr"/>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=ydK2WdTAOgU</t>
+        </is>
+      </c>
+      <c r="J109" t="n">
+        <v>480871</v>
+      </c>
+      <c r="K109" t="inlineStr">
+        <is>
+          <t>TVアニメ『ヤニねこ』公式【ハメちゃんねる】</t>
+        </is>
+      </c>
       <c r="L109" t="inlineStr"/>
       <c r="M109" t="inlineStr"/>
       <c r="N109" t="inlineStr"/>
-      <c r="O109" t="inlineStr"/>
+      <c r="O109" t="inlineStr">
+        <is>
+          <t>2026-06-21T18:32:14</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="n">
@@ -12245,13 +13057,27 @@
           <t>ネクライトーキー</t>
         </is>
       </c>
-      <c r="I110" t="inlineStr"/>
-      <c r="J110" t="inlineStr"/>
-      <c r="K110" t="inlineStr"/>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=ydK2WdTAOgU</t>
+        </is>
+      </c>
+      <c r="J110" t="n">
+        <v>480871</v>
+      </c>
+      <c r="K110" t="inlineStr">
+        <is>
+          <t>TVアニメ『ヤニねこ』公式【ハメちゃんねる】</t>
+        </is>
+      </c>
       <c r="L110" t="inlineStr"/>
       <c r="M110" t="inlineStr"/>
       <c r="N110" t="inlineStr"/>
-      <c r="O110" t="inlineStr"/>
+      <c r="O110" t="inlineStr">
+        <is>
+          <t>2026-06-21T18:32:32</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="n">
@@ -12288,13 +13114,27 @@
           <t>MYTH &amp; ROID</t>
         </is>
       </c>
-      <c r="I111" t="inlineStr"/>
-      <c r="J111" t="inlineStr"/>
-      <c r="K111" t="inlineStr"/>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=RMaOR0Pyfts</t>
+        </is>
+      </c>
+      <c r="J111" t="n">
+        <v>50838</v>
+      </c>
+      <c r="K111" t="inlineStr">
+        <is>
+          <t>MYTH &amp; ROID Official Channel</t>
+        </is>
+      </c>
       <c r="L111" t="inlineStr"/>
       <c r="M111" t="inlineStr"/>
       <c r="N111" t="inlineStr"/>
-      <c r="O111" t="inlineStr"/>
+      <c r="O111" t="inlineStr">
+        <is>
+          <t>2026-06-21T18:33:01</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="n">
@@ -12374,13 +13214,37 @@
           <t>blank paper</t>
         </is>
       </c>
-      <c r="I113" t="inlineStr"/>
-      <c r="J113" t="inlineStr"/>
-      <c r="K113" t="inlineStr"/>
-      <c r="L113" t="inlineStr"/>
-      <c r="M113" t="inlineStr"/>
-      <c r="N113" t="inlineStr"/>
-      <c r="O113" t="inlineStr"/>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=kHUPdA8H6qk</t>
+        </is>
+      </c>
+      <c r="J113" t="n">
+        <v>603666</v>
+      </c>
+      <c r="K113" t="inlineStr">
+        <is>
+          <t>TVアニメ『鎧真伝サムライトルーパー』公式</t>
+        </is>
+      </c>
+      <c r="L113" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=kHUPdA8H6qk</t>
+        </is>
+      </c>
+      <c r="M113" t="n">
+        <v>603666</v>
+      </c>
+      <c r="N113" t="inlineStr">
+        <is>
+          <t>TVアニメ『鎧真伝サムライトルーパー』公式</t>
+        </is>
+      </c>
+      <c r="O113" t="inlineStr">
+        <is>
+          <t>2026-06-21T18:33:22</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="n">
@@ -12417,13 +13281,27 @@
           <t>Dannie May</t>
         </is>
       </c>
-      <c r="I114" t="inlineStr"/>
-      <c r="J114" t="inlineStr"/>
-      <c r="K114" t="inlineStr"/>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=OKEoQo3cGVg</t>
+        </is>
+      </c>
+      <c r="J114" t="n">
+        <v>66350</v>
+      </c>
+      <c r="K114" t="inlineStr">
+        <is>
+          <t>TVアニメ『鎧真伝サムライトルーパー』公式</t>
+        </is>
+      </c>
       <c r="L114" t="inlineStr"/>
       <c r="M114" t="inlineStr"/>
       <c r="N114" t="inlineStr"/>
-      <c r="O114" t="inlineStr"/>
+      <c r="O114" t="inlineStr">
+        <is>
+          <t>2026-06-21T18:33:34</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="n">
@@ -12460,13 +13338,37 @@
           <t>ONE OR EIGHT</t>
         </is>
       </c>
-      <c r="I115" t="inlineStr"/>
-      <c r="J115" t="inlineStr"/>
-      <c r="K115" t="inlineStr"/>
-      <c r="L115" t="inlineStr"/>
-      <c r="M115" t="inlineStr"/>
-      <c r="N115" t="inlineStr"/>
-      <c r="O115" t="inlineStr"/>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=aw45Q_mr0_M</t>
+        </is>
+      </c>
+      <c r="J115" t="n">
+        <v>9441868</v>
+      </c>
+      <c r="K115" t="inlineStr">
+        <is>
+          <t>ONE OR EIGHT</t>
+        </is>
+      </c>
+      <c r="L115" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=VJflo-z7e7A</t>
+        </is>
+      </c>
+      <c r="M115" t="n">
+        <v>151043</v>
+      </c>
+      <c r="N115" t="inlineStr">
+        <is>
+          <t>TVアニメ『鎧真伝サムライトルーパー』公式</t>
+        </is>
+      </c>
+      <c r="O115" t="inlineStr">
+        <is>
+          <t>2026-06-21T18:33:47</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="n">
@@ -12503,13 +13405,27 @@
           <t>カラノア</t>
         </is>
       </c>
-      <c r="I116" t="inlineStr"/>
-      <c r="J116" t="inlineStr"/>
-      <c r="K116" t="inlineStr"/>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=OKEoQo3cGVg</t>
+        </is>
+      </c>
+      <c r="J116" t="n">
+        <v>66350</v>
+      </c>
+      <c r="K116" t="inlineStr">
+        <is>
+          <t>TVアニメ『鎧真伝サムライトルーパー』公式</t>
+        </is>
+      </c>
       <c r="L116" t="inlineStr"/>
       <c r="M116" t="inlineStr"/>
       <c r="N116" t="inlineStr"/>
-      <c r="O116" t="inlineStr"/>
+      <c r="O116" t="inlineStr">
+        <is>
+          <t>2026-06-21T18:34:00</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="n">
@@ -12804,13 +13720,27 @@
           <t>藍月なくる&amp;棗いつき</t>
         </is>
       </c>
-      <c r="I123" t="inlineStr"/>
-      <c r="J123" t="inlineStr"/>
-      <c r="K123" t="inlineStr"/>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=9-RVzXLF53U</t>
+        </is>
+      </c>
+      <c r="J123" t="n">
+        <v>78910</v>
+      </c>
+      <c r="K123" t="inlineStr">
+        <is>
+          <t>Itsuki Natsume / 棗いつき</t>
+        </is>
+      </c>
       <c r="L123" t="inlineStr"/>
       <c r="M123" t="inlineStr"/>
       <c r="N123" t="inlineStr"/>
-      <c r="O123" t="inlineStr"/>
+      <c r="O123" t="inlineStr">
+        <is>
+          <t>2026-06-21T18:35:08</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="n">
@@ -12890,13 +13820,37 @@
           <t>マカロニえんぴつ</t>
         </is>
       </c>
-      <c r="I125" t="inlineStr"/>
-      <c r="J125" t="inlineStr"/>
-      <c r="K125" t="inlineStr"/>
-      <c r="L125" t="inlineStr"/>
-      <c r="M125" t="inlineStr"/>
-      <c r="N125" t="inlineStr"/>
-      <c r="O125" t="inlineStr"/>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=Zu45LJG7Chs</t>
+        </is>
+      </c>
+      <c r="J125" t="n">
+        <v>262519</v>
+      </c>
+      <c r="K125" t="inlineStr">
+        <is>
+          <t>SHOCHIKU anime Channel</t>
+        </is>
+      </c>
+      <c r="L125" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=Zu45LJG7Chs</t>
+        </is>
+      </c>
+      <c r="M125" t="n">
+        <v>262519</v>
+      </c>
+      <c r="N125" t="inlineStr">
+        <is>
+          <t>SHOCHIKU anime Channel</t>
+        </is>
+      </c>
+      <c r="O125" t="inlineStr">
+        <is>
+          <t>2026-06-21T18:35:26</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="n">
@@ -12933,13 +13887,37 @@
           <t>電子書籍（コミック）</t>
         </is>
       </c>
-      <c r="I126" t="inlineStr"/>
-      <c r="J126" t="inlineStr"/>
-      <c r="K126" t="inlineStr"/>
-      <c r="L126" t="inlineStr"/>
-      <c r="M126" t="inlineStr"/>
-      <c r="N126" t="inlineStr"/>
-      <c r="O126" t="inlineStr"/>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=6hRjsvdINgg</t>
+        </is>
+      </c>
+      <c r="J126" t="n">
+        <v>17920416</v>
+      </c>
+      <c r="K126" t="inlineStr">
+        <is>
+          <t>ONE PIECE Official YouTube Channel</t>
+        </is>
+      </c>
+      <c r="L126" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=YFbno_aPm0w</t>
+        </is>
+      </c>
+      <c r="M126" t="n">
+        <v>27924515</v>
+      </c>
+      <c r="N126" t="inlineStr">
+        <is>
+          <t>ONE PIECE Official YouTube Channel</t>
+        </is>
+      </c>
+      <c r="O126" t="inlineStr">
+        <is>
+          <t>2026-06-21T18:35:55</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="n">
@@ -13234,13 +14212,27 @@
           <t>茅原実里</t>
         </is>
       </c>
-      <c r="I133" t="inlineStr"/>
-      <c r="J133" t="inlineStr"/>
-      <c r="K133" t="inlineStr"/>
+      <c r="I133" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=-PX7FqZ55tE</t>
+        </is>
+      </c>
+      <c r="J133" t="n">
+        <v>105042</v>
+      </c>
+      <c r="K133" t="inlineStr">
+        <is>
+          <t>TVアニメ「魔法少女育成計画restart」公式チャンネル</t>
+        </is>
+      </c>
       <c r="L133" t="inlineStr"/>
       <c r="M133" t="inlineStr"/>
       <c r="N133" t="inlineStr"/>
-      <c r="O133" t="inlineStr"/>
+      <c r="O133" t="inlineStr">
+        <is>
+          <t>2026-06-21T18:36:51</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
auto: anime list update (PC) 2026-06-25
</commit_message>
<xml_diff>
--- a/data/anime_list.xlsx
+++ b/data/anime_list.xlsx
@@ -4238,7 +4238,7 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>2026年7月4日（土）～ TOKYO MX・BS11にて</t>
+          <t>2026年7月4日（土）～ TOKYO MX・BS11ほか</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
@@ -5485,7 +5485,7 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>2026年10月〜</t>
+          <t>2026年10月1日（木）〜 テレビ神奈川・CBCテレビにて</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
@@ -11652,13 +11652,37 @@
           <t>QWER</t>
         </is>
       </c>
-      <c r="I76" t="inlineStr"/>
-      <c r="J76" t="inlineStr"/>
-      <c r="K76" t="inlineStr"/>
-      <c r="L76" t="inlineStr"/>
-      <c r="M76" t="inlineStr"/>
-      <c r="N76" t="inlineStr"/>
-      <c r="O76" t="inlineStr"/>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=PVN8Pj_Ykyo</t>
+        </is>
+      </c>
+      <c r="J76" t="n">
+        <v>16839</v>
+      </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=PVN8Pj_Ykyo</t>
+        </is>
+      </c>
+      <c r="M76" t="n">
+        <v>16839</v>
+      </c>
+      <c r="N76" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="O76" t="inlineStr">
+        <is>
+          <t>2026-06-25T09:05:01</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -11695,13 +11719,37 @@
           <t>QWER</t>
         </is>
       </c>
-      <c r="I77" t="inlineStr"/>
-      <c r="J77" t="inlineStr"/>
-      <c r="K77" t="inlineStr"/>
-      <c r="L77" t="inlineStr"/>
-      <c r="M77" t="inlineStr"/>
-      <c r="N77" t="inlineStr"/>
-      <c r="O77" t="inlineStr"/>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=PVN8Pj_Ykyo</t>
+        </is>
+      </c>
+      <c r="J77" t="n">
+        <v>16839</v>
+      </c>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="L77" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=PVN8Pj_Ykyo</t>
+        </is>
+      </c>
+      <c r="M77" t="n">
+        <v>16839</v>
+      </c>
+      <c r="N77" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="O77" t="inlineStr">
+        <is>
+          <t>2026-06-25T09:05:10</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -12374,13 +12422,27 @@
           <t>Omoinotake</t>
         </is>
       </c>
-      <c r="I90" t="inlineStr"/>
-      <c r="J90" t="inlineStr"/>
-      <c r="K90" t="inlineStr"/>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=s1bZEnGAX8I</t>
+        </is>
+      </c>
+      <c r="J90" t="n">
+        <v>3841595</v>
+      </c>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>Omoinotake</t>
+        </is>
+      </c>
       <c r="L90" t="inlineStr"/>
       <c r="M90" t="inlineStr"/>
       <c r="N90" t="inlineStr"/>
-      <c r="O90" t="inlineStr"/>
+      <c r="O90" t="inlineStr">
+        <is>
+          <t>2026-06-25T09:06:54</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -12417,13 +12479,27 @@
           <t>Omoinotake</t>
         </is>
       </c>
-      <c r="I91" t="inlineStr"/>
-      <c r="J91" t="inlineStr"/>
-      <c r="K91" t="inlineStr"/>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=s1bZEnGAX8I</t>
+        </is>
+      </c>
+      <c r="J91" t="n">
+        <v>3841595</v>
+      </c>
+      <c r="K91" t="inlineStr">
+        <is>
+          <t>Omoinotake</t>
+        </is>
+      </c>
       <c r="L91" t="inlineStr"/>
       <c r="M91" t="inlineStr"/>
       <c r="N91" t="inlineStr"/>
-      <c r="O91" t="inlineStr"/>
+      <c r="O91" t="inlineStr">
+        <is>
+          <t>2026-06-25T09:07:22</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="n">

</xml_diff>

<commit_message>
auto: anime list update (PC) 2026-06-26
</commit_message>
<xml_diff>
--- a/data/anime_list.xlsx
+++ b/data/anime_list.xlsx
@@ -2732,8 +2732,16 @@
           <t>原因は自分にある。</t>
         </is>
       </c>
-      <c r="K41" t="inlineStr"/>
-      <c r="L41" t="inlineStr"/>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>泣いた悪魔</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>えむにみに</t>
+        </is>
+      </c>
       <c r="M41" t="inlineStr">
         <is>
           <t>https://www.animatetimes.com/tag/details.php?id=27260</t>
@@ -3468,10 +3476,26 @@
           <t>ライデンフィルム</t>
         </is>
       </c>
-      <c r="I55" t="inlineStr"/>
-      <c r="J55" t="inlineStr"/>
-      <c r="K55" t="inlineStr"/>
-      <c r="L55" t="inlineStr"/>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>ハイメンテナンスガール</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>オーイシマサヨシ</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>ベリーグッド・エンカウント</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>内田真礼</t>
+        </is>
+      </c>
       <c r="M55" t="inlineStr">
         <is>
           <t>https://www.animatetimes.com/tag/details.php?id=26828</t>
@@ -7793,7 +7817,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O147"/>
+  <dimension ref="A1:O150"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11375,7 +11399,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>手札が多めのビクトリア</t>
+          <t>鉄鍋のジャン！</t>
         </is>
       </c>
       <c r="D71" t="b">
@@ -11391,45 +11415,21 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>縁のつき</t>
+          <t>泣いた悪魔</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>KI_EN</t>
-        </is>
-      </c>
-      <c r="I71" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=-HNOXWE2wVU</t>
-        </is>
-      </c>
-      <c r="J71" t="n">
-        <v>140125</v>
-      </c>
-      <c r="K71" t="inlineStr">
-        <is>
-          <t>KADOKAWAanime</t>
-        </is>
-      </c>
-      <c r="L71" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=-HNOXWE2wVU</t>
-        </is>
-      </c>
-      <c r="M71" t="n">
-        <v>140125</v>
-      </c>
-      <c r="N71" t="inlineStr">
-        <is>
-          <t>KADOKAWAanime</t>
-        </is>
-      </c>
-      <c r="O71" t="inlineStr">
-        <is>
-          <t>2026-06-21T18:23:55</t>
-        </is>
-      </c>
+          <t>えむにみに</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr"/>
+      <c r="J71" t="inlineStr"/>
+      <c r="K71" t="inlineStr"/>
+      <c r="L71" t="inlineStr"/>
+      <c r="M71" t="inlineStr"/>
+      <c r="N71" t="inlineStr"/>
+      <c r="O71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -11442,7 +11442,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>転校先の清楚可憐な美少女が、昔男子と思って一緒に遊んだ幼馴染だった件</t>
+          <t>手札が多めのビクトリア</t>
         </is>
       </c>
       <c r="D72" t="b">
@@ -11450,7 +11450,7 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F72" t="n">
@@ -11458,21 +11458,45 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>夏に重ねて</t>
+          <t>縁のつき</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>DIALOGUE+</t>
-        </is>
-      </c>
-      <c r="I72" t="inlineStr"/>
-      <c r="J72" t="inlineStr"/>
-      <c r="K72" t="inlineStr"/>
-      <c r="L72" t="inlineStr"/>
-      <c r="M72" t="inlineStr"/>
-      <c r="N72" t="inlineStr"/>
-      <c r="O72" t="inlineStr"/>
+          <t>KI_EN</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=-HNOXWE2wVU</t>
+        </is>
+      </c>
+      <c r="J72" t="n">
+        <v>140125</v>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=-HNOXWE2wVU</t>
+        </is>
+      </c>
+      <c r="M72" t="n">
+        <v>140125</v>
+      </c>
+      <c r="N72" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="O72" t="inlineStr">
+        <is>
+          <t>2026-06-21T18:23:55</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -11493,7 +11517,7 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F73" t="n">
@@ -11501,12 +11525,12 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>Tilt</t>
+          <t>夏に重ねて</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>harmoe</t>
+          <t>DIALOGUE+</t>
         </is>
       </c>
       <c r="I73" t="inlineStr"/>
@@ -11528,7 +11552,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>天は赤い河のほとり</t>
+          <t>転校先の清楚可憐な美少女が、昔男子と思って一緒に遊んだ幼馴染だった件</t>
         </is>
       </c>
       <c r="D74" t="b">
@@ -11536,7 +11560,7 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F74" t="n">
@@ -11544,35 +11568,21 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>暁の空</t>
+          <t>Tilt</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>七海ひろき</t>
-        </is>
-      </c>
-      <c r="I74" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=qpFcQ1Bek08</t>
-        </is>
-      </c>
-      <c r="J74" t="n">
-        <v>69452</v>
-      </c>
-      <c r="K74" t="inlineStr">
-        <is>
-          <t>VAP Official</t>
-        </is>
-      </c>
+          <t>harmoe</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr"/>
+      <c r="J74" t="inlineStr"/>
+      <c r="K74" t="inlineStr"/>
       <c r="L74" t="inlineStr"/>
       <c r="M74" t="inlineStr"/>
       <c r="N74" t="inlineStr"/>
-      <c r="O74" t="inlineStr">
-        <is>
-          <t>2026-06-21T18:24:32</t>
-        </is>
-      </c>
+      <c r="O74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -11585,7 +11595,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>天幕のジャードゥーガル</t>
+          <t>天は赤い河のほとり</t>
         </is>
       </c>
       <c r="D75" t="b">
@@ -11601,21 +11611,35 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>Stella</t>
+          <t>暁の空</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>SEKAI NO OWARI</t>
-        </is>
-      </c>
-      <c r="I75" t="inlineStr"/>
-      <c r="J75" t="inlineStr"/>
-      <c r="K75" t="inlineStr"/>
+          <t>七海ひろき</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=qpFcQ1Bek08</t>
+        </is>
+      </c>
+      <c r="J75" t="n">
+        <v>69452</v>
+      </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>VAP Official</t>
+        </is>
+      </c>
       <c r="L75" t="inlineStr"/>
       <c r="M75" t="inlineStr"/>
       <c r="N75" t="inlineStr"/>
-      <c r="O75" t="inlineStr"/>
+      <c r="O75" t="inlineStr">
+        <is>
+          <t>2026-06-21T18:24:32</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -11628,7 +11652,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>盗掘王</t>
+          <t>天幕のジャードゥーガル</t>
         </is>
       </c>
       <c r="D76" t="b">
@@ -11644,45 +11668,21 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>SHOW DOWN</t>
+          <t>Stella</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>QWER</t>
-        </is>
-      </c>
-      <c r="I76" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=PVN8Pj_Ykyo</t>
-        </is>
-      </c>
-      <c r="J76" t="n">
-        <v>16839</v>
-      </c>
-      <c r="K76" t="inlineStr">
-        <is>
-          <t>KADOKAWAanime</t>
-        </is>
-      </c>
-      <c r="L76" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=PVN8Pj_Ykyo</t>
-        </is>
-      </c>
-      <c r="M76" t="n">
-        <v>16839</v>
-      </c>
-      <c r="N76" t="inlineStr">
-        <is>
-          <t>KADOKAWAanime</t>
-        </is>
-      </c>
-      <c r="O76" t="inlineStr">
-        <is>
-          <t>2026-06-25T09:05:01</t>
-        </is>
-      </c>
+          <t>SEKAI NO OWARI</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr"/>
+      <c r="J76" t="inlineStr"/>
+      <c r="K76" t="inlineStr"/>
+      <c r="L76" t="inlineStr"/>
+      <c r="M76" t="inlineStr"/>
+      <c r="N76" t="inlineStr"/>
+      <c r="O76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -11703,7 +11703,7 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F77" t="n">
@@ -11711,7 +11711,7 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>To Be Continued</t>
+          <t>SHOW DOWN</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
@@ -11747,7 +11747,7 @@
       </c>
       <c r="O77" t="inlineStr">
         <is>
-          <t>2026-06-25T09:05:10</t>
+          <t>2026-06-25T09:05:01</t>
         </is>
       </c>
     </row>
@@ -11762,7 +11762,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>透明な夜に駆ける君と、目に見えない恋をした。</t>
+          <t>盗掘王</t>
         </is>
       </c>
       <c r="D78" t="b">
@@ -11770,7 +11770,7 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F78" t="n">
@@ -11778,21 +11778,45 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>ひとひら</t>
+          <t>To Be Continued</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>秦基博</t>
-        </is>
-      </c>
-      <c r="I78" t="inlineStr"/>
-      <c r="J78" t="inlineStr"/>
-      <c r="K78" t="inlineStr"/>
-      <c r="L78" t="inlineStr"/>
-      <c r="M78" t="inlineStr"/>
-      <c r="N78" t="inlineStr"/>
-      <c r="O78" t="inlineStr"/>
+          <t>QWER</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=PVN8Pj_Ykyo</t>
+        </is>
+      </c>
+      <c r="J78" t="n">
+        <v>16839</v>
+      </c>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="L78" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=PVN8Pj_Ykyo</t>
+        </is>
+      </c>
+      <c r="M78" t="n">
+        <v>16839</v>
+      </c>
+      <c r="N78" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="O78" t="inlineStr">
+        <is>
+          <t>2026-06-25T09:05:10</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -11813,7 +11837,7 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F79" t="n">
@@ -11821,12 +11845,12 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>光</t>
+          <t>ひとひら</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>櫻井優衣</t>
+          <t>秦基博</t>
         </is>
       </c>
       <c r="I79" t="inlineStr"/>
@@ -11848,7 +11872,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>トミカとトム</t>
+          <t>透明な夜に駆ける君と、目に見えない恋をした。</t>
         </is>
       </c>
       <c r="D80" t="b">
@@ -11856,7 +11880,7 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>主題歌</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F80" t="n">
@@ -11864,12 +11888,12 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>きみのたからもの</t>
+          <t>光</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>May J.</t>
+          <t>櫻井優衣</t>
         </is>
       </c>
       <c r="I80" t="inlineStr"/>
@@ -11891,7 +11915,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>二十世紀電氣目録-ユーレカ・エヴリカ-</t>
+          <t>トミカとトム</t>
         </is>
       </c>
       <c r="D81" t="b">
@@ -11899,7 +11923,7 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>主題歌</t>
         </is>
       </c>
       <c r="F81" t="n">
@@ -11907,12 +11931,12 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>ユーレカ・エヴリカ</t>
+          <t>きみのたからもの</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>五阿弥ルナ</t>
+          <t>May J.</t>
         </is>
       </c>
       <c r="I81" t="inlineStr"/>
@@ -11942,7 +11966,7 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F82" t="n">
@@ -11950,45 +11974,21 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>Soarin’</t>
+          <t>ユーレカ・エヴリカ</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>Ginger Root</t>
-        </is>
-      </c>
-      <c r="I82" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=5rQWh9aIflw</t>
-        </is>
-      </c>
-      <c r="J82" t="n">
-        <v>3207</v>
-      </c>
-      <c r="K82" t="inlineStr">
-        <is>
-          <t>Lantis Channel</t>
-        </is>
-      </c>
-      <c r="L82" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=5rQWh9aIflw</t>
-        </is>
-      </c>
-      <c r="M82" t="n">
-        <v>3207</v>
-      </c>
-      <c r="N82" t="inlineStr">
-        <is>
-          <t>Lantis Channel</t>
-        </is>
-      </c>
-      <c r="O82" t="inlineStr">
-        <is>
-          <t>2026-06-21T18:26:16</t>
-        </is>
-      </c>
+          <t>五阿弥ルナ</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr"/>
+      <c r="J82" t="inlineStr"/>
+      <c r="K82" t="inlineStr"/>
+      <c r="L82" t="inlineStr"/>
+      <c r="M82" t="inlineStr"/>
+      <c r="N82" t="inlineStr"/>
+      <c r="O82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -12001,7 +12001,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>猫と竜</t>
+          <t>二十世紀電氣目録-ユーレカ・エヴリカ-</t>
         </is>
       </c>
       <c r="D83" t="b">
@@ -12009,7 +12009,7 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F83" t="n">
@@ -12017,21 +12017,45 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>猫日</t>
+          <t>Soarin’</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>suis from ヨルシカ</t>
-        </is>
-      </c>
-      <c r="I83" t="inlineStr"/>
-      <c r="J83" t="inlineStr"/>
-      <c r="K83" t="inlineStr"/>
-      <c r="L83" t="inlineStr"/>
-      <c r="M83" t="inlineStr"/>
-      <c r="N83" t="inlineStr"/>
-      <c r="O83" t="inlineStr"/>
+          <t>Ginger Root</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=5rQWh9aIflw</t>
+        </is>
+      </c>
+      <c r="J83" t="n">
+        <v>3207</v>
+      </c>
+      <c r="K83" t="inlineStr">
+        <is>
+          <t>Lantis Channel</t>
+        </is>
+      </c>
+      <c r="L83" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=5rQWh9aIflw</t>
+        </is>
+      </c>
+      <c r="M83" t="n">
+        <v>3207</v>
+      </c>
+      <c r="N83" t="inlineStr">
+        <is>
+          <t>Lantis Channel</t>
+        </is>
+      </c>
+      <c r="O83" t="inlineStr">
+        <is>
+          <t>2026-06-21T18:26:16</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -12052,7 +12076,7 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F84" t="n">
@@ -12060,21 +12084,35 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>ただいまの場所</t>
+          <t>猫日</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>shallm</t>
-        </is>
-      </c>
-      <c r="I84" t="inlineStr"/>
-      <c r="J84" t="inlineStr"/>
-      <c r="K84" t="inlineStr"/>
+          <t>suis from ヨルシカ</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=5Of2HNJa_gs</t>
+        </is>
+      </c>
+      <c r="J84" t="n">
+        <v>5618588</v>
+      </c>
+      <c r="K84" t="inlineStr">
+        <is>
+          <t>ヨルシカ / n-buna Official</t>
+        </is>
+      </c>
       <c r="L84" t="inlineStr"/>
       <c r="M84" t="inlineStr"/>
       <c r="N84" t="inlineStr"/>
-      <c r="O84" t="inlineStr"/>
+      <c r="O84" t="inlineStr">
+        <is>
+          <t>2026-06-26T09:06:03</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="n">
@@ -12087,7 +12125,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>パイの実 おしの森へようこそ！</t>
+          <t>猫と竜</t>
         </is>
       </c>
       <c r="D85" t="b">
@@ -12095,7 +12133,7 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>主題歌</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F85" t="n">
@@ -12103,12 +12141,12 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>パイしか勝たん！推しの森活</t>
+          <t>ただいまの場所</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>安保心結</t>
+          <t>shallm</t>
         </is>
       </c>
       <c r="I85" t="inlineStr"/>
@@ -12130,7 +12168,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>刃牙道 第2クール</t>
+          <t>パイの実 おしの森へようこそ！</t>
         </is>
       </c>
       <c r="D86" t="b">
@@ -12138,7 +12176,7 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>主題歌</t>
         </is>
       </c>
       <c r="F86" t="n">
@@ -12146,45 +12184,21 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>フルボコ</t>
+          <t>パイしか勝たん！推しの森活</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>WANIMA</t>
-        </is>
-      </c>
-      <c r="I86" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=3KIPGQJh4vI</t>
-        </is>
-      </c>
-      <c r="J86" t="n">
-        <v>402991</v>
-      </c>
-      <c r="K86" t="inlineStr">
-        <is>
-          <t>TMSアニメ公式チャンネル</t>
-        </is>
-      </c>
-      <c r="L86" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=3KIPGQJh4vI</t>
-        </is>
-      </c>
-      <c r="M86" t="n">
-        <v>402991</v>
-      </c>
-      <c r="N86" t="inlineStr">
-        <is>
-          <t>TMSアニメ公式チャンネル</t>
-        </is>
-      </c>
-      <c r="O86" t="inlineStr">
-        <is>
-          <t>2026-06-21T18:26:31</t>
-        </is>
-      </c>
+          <t>安保心結</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr"/>
+      <c r="J86" t="inlineStr"/>
+      <c r="K86" t="inlineStr"/>
+      <c r="L86" t="inlineStr"/>
+      <c r="M86" t="inlineStr"/>
+      <c r="N86" t="inlineStr"/>
+      <c r="O86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="n">
@@ -12209,25 +12223,25 @@
         </is>
       </c>
       <c r="F87" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>六ノ輪</t>
+          <t>フルボコ</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>Chevon</t>
+          <t>WANIMA</t>
         </is>
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=x0ygvWo5e3k</t>
+          <t>https://www.youtube.com/watch?v=3KIPGQJh4vI</t>
         </is>
       </c>
       <c r="J87" t="n">
-        <v>174316</v>
+        <v>402991</v>
       </c>
       <c r="K87" t="inlineStr">
         <is>
@@ -12236,11 +12250,11 @@
       </c>
       <c r="L87" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=x0ygvWo5e3k</t>
+          <t>https://www.youtube.com/watch?v=3KIPGQJh4vI</t>
         </is>
       </c>
       <c r="M87" t="n">
-        <v>174316</v>
+        <v>402991</v>
       </c>
       <c r="N87" t="inlineStr">
         <is>
@@ -12249,7 +12263,7 @@
       </c>
       <c r="O87" t="inlineStr">
         <is>
-          <t>2026-06-21T18:26:42</t>
+          <t>2026-06-21T18:26:31</t>
         </is>
       </c>
     </row>
@@ -12272,29 +12286,29 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F88" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>Mountain Top</t>
+          <t>六ノ輪</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>Novel Core</t>
+          <t>Chevon</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=KKOr3xF2iOM</t>
+          <t>https://www.youtube.com/watch?v=x0ygvWo5e3k</t>
         </is>
       </c>
       <c r="J88" t="n">
-        <v>294329</v>
+        <v>174316</v>
       </c>
       <c r="K88" t="inlineStr">
         <is>
@@ -12303,11 +12317,11 @@
       </c>
       <c r="L88" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=KKOr3xF2iOM</t>
+          <t>https://www.youtube.com/watch?v=x0ygvWo5e3k</t>
         </is>
       </c>
       <c r="M88" t="n">
-        <v>294329</v>
+        <v>174316</v>
       </c>
       <c r="N88" t="inlineStr">
         <is>
@@ -12316,7 +12330,7 @@
       </c>
       <c r="O88" t="inlineStr">
         <is>
-          <t>2026-06-21T18:26:53</t>
+          <t>2026-06-21T18:26:42</t>
         </is>
       </c>
     </row>
@@ -12343,25 +12357,25 @@
         </is>
       </c>
       <c r="F89" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>KATANA</t>
+          <t>Mountain Top</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>三代目 J SOUL BROTHERS</t>
+          <t>Novel Core</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=1LBv6-z-0ok</t>
+          <t>https://www.youtube.com/watch?v=KKOr3xF2iOM</t>
         </is>
       </c>
       <c r="J89" t="n">
-        <v>25824</v>
+        <v>294329</v>
       </c>
       <c r="K89" t="inlineStr">
         <is>
@@ -12370,11 +12384,11 @@
       </c>
       <c r="L89" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=1LBv6-z-0ok</t>
+          <t>https://www.youtube.com/watch?v=KKOr3xF2iOM</t>
         </is>
       </c>
       <c r="M89" t="n">
-        <v>25824</v>
+        <v>294329</v>
       </c>
       <c r="N89" t="inlineStr">
         <is>
@@ -12383,7 +12397,7 @@
       </c>
       <c r="O89" t="inlineStr">
         <is>
-          <t>2026-06-21T18:27:05</t>
+          <t>2026-06-21T18:26:53</t>
         </is>
       </c>
     </row>
@@ -12398,7 +12412,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>花ざかりの君たちへ 第2期</t>
+          <t>刃牙道 第2クール</t>
         </is>
       </c>
       <c r="D90" t="b">
@@ -12406,41 +12420,51 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F90" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>FLASHBULB</t>
+          <t>KATANA</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>Omoinotake</t>
+          <t>三代目 J SOUL BROTHERS</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=s1bZEnGAX8I</t>
+          <t>https://www.youtube.com/watch?v=1LBv6-z-0ok</t>
         </is>
       </c>
       <c r="J90" t="n">
-        <v>3841595</v>
+        <v>25824</v>
       </c>
       <c r="K90" t="inlineStr">
         <is>
-          <t>Omoinotake</t>
-        </is>
-      </c>
-      <c r="L90" t="inlineStr"/>
-      <c r="M90" t="inlineStr"/>
-      <c r="N90" t="inlineStr"/>
+          <t>TMSアニメ公式チャンネル</t>
+        </is>
+      </c>
+      <c r="L90" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=1LBv6-z-0ok</t>
+        </is>
+      </c>
+      <c r="M90" t="n">
+        <v>25824</v>
+      </c>
+      <c r="N90" t="inlineStr">
+        <is>
+          <t>TMSアニメ公式チャンネル</t>
+        </is>
+      </c>
       <c r="O90" t="inlineStr">
         <is>
-          <t>2026-06-25T09:06:54</t>
+          <t>2026-06-21T18:27:05</t>
         </is>
       </c>
     </row>
@@ -12455,7 +12479,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>花ざかりの君たちへ 第2期</t>
+          <t>花織さんは転生しても喧嘩がしたい</t>
         </is>
       </c>
       <c r="D91" t="b">
@@ -12463,7 +12487,7 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F91" t="n">
@@ -12471,35 +12495,21 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>花束</t>
+          <t>ハイメンテナンスガール</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>Omoinotake</t>
-        </is>
-      </c>
-      <c r="I91" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=s1bZEnGAX8I</t>
-        </is>
-      </c>
-      <c r="J91" t="n">
-        <v>3841595</v>
-      </c>
-      <c r="K91" t="inlineStr">
-        <is>
-          <t>Omoinotake</t>
-        </is>
-      </c>
+          <t>オーイシマサヨシ</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr"/>
+      <c r="J91" t="inlineStr"/>
+      <c r="K91" t="inlineStr"/>
       <c r="L91" t="inlineStr"/>
       <c r="M91" t="inlineStr"/>
       <c r="N91" t="inlineStr"/>
-      <c r="O91" t="inlineStr">
-        <is>
-          <t>2026-06-25T09:07:22</t>
-        </is>
-      </c>
+      <c r="O91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -12512,7 +12522,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>バンドリ！ ゆめ∞みた</t>
+          <t>花織さんは転生しても喧嘩がしたい</t>
         </is>
       </c>
       <c r="D92" t="b">
@@ -12520,7 +12530,7 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F92" t="n">
@@ -12528,45 +12538,21 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>これはぼくたちの生存のあらすじ</t>
+          <t>ベリーグッド・エンカウント</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>夢限大みゅーたいぷ</t>
-        </is>
-      </c>
-      <c r="I92" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=Ech7Tj8ga0Y</t>
-        </is>
-      </c>
-      <c r="J92" t="n">
-        <v>124089</v>
-      </c>
-      <c r="K92" t="inlineStr">
-        <is>
-          <t>BanG Dream Channel☆</t>
-        </is>
-      </c>
-      <c r="L92" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=Ech7Tj8ga0Y</t>
-        </is>
-      </c>
-      <c r="M92" t="n">
-        <v>124089</v>
-      </c>
-      <c r="N92" t="inlineStr">
-        <is>
-          <t>BanG Dream Channel☆</t>
-        </is>
-      </c>
-      <c r="O92" t="inlineStr">
-        <is>
-          <t>2026-06-24T09:06:31</t>
-        </is>
-      </c>
+          <t>内田真礼</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr"/>
+      <c r="J92" t="inlineStr"/>
+      <c r="K92" t="inlineStr"/>
+      <c r="L92" t="inlineStr"/>
+      <c r="M92" t="inlineStr"/>
+      <c r="N92" t="inlineStr"/>
+      <c r="O92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -12579,7 +12565,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>ヒロイン？聖女？いいえ、オールワークスメイドです（誇）！</t>
+          <t>花ざかりの君たちへ 第2期</t>
         </is>
       </c>
       <c r="D93" t="b">
@@ -12595,21 +12581,35 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>マデュアル↔ハート</t>
+          <t>FLASHBULB</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>メロディ・ウェーブ(CV：宮本侑芽) ルシアナ・ルトルバーグ(CV：大久保瑠美)</t>
-        </is>
-      </c>
-      <c r="I93" t="inlineStr"/>
-      <c r="J93" t="inlineStr"/>
-      <c r="K93" t="inlineStr"/>
+          <t>Omoinotake</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=s1bZEnGAX8I</t>
+        </is>
+      </c>
+      <c r="J93" t="n">
+        <v>3841595</v>
+      </c>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>Omoinotake</t>
+        </is>
+      </c>
       <c r="L93" t="inlineStr"/>
       <c r="M93" t="inlineStr"/>
       <c r="N93" t="inlineStr"/>
-      <c r="O93" t="inlineStr"/>
+      <c r="O93" t="inlineStr">
+        <is>
+          <t>2026-06-25T09:06:54</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -12622,7 +12622,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>ヒロイン？聖女？いいえ、オールワークスメイドです（誇）！</t>
+          <t>花ざかりの君たちへ 第2期</t>
         </is>
       </c>
       <c r="D94" t="b">
@@ -12638,21 +12638,35 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>ハンドメイド</t>
+          <t>花束</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>仲村宗悟</t>
-        </is>
-      </c>
-      <c r="I94" t="inlineStr"/>
-      <c r="J94" t="inlineStr"/>
-      <c r="K94" t="inlineStr"/>
+          <t>Omoinotake</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=s1bZEnGAX8I</t>
+        </is>
+      </c>
+      <c r="J94" t="n">
+        <v>3841595</v>
+      </c>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>Omoinotake</t>
+        </is>
+      </c>
       <c r="L94" t="inlineStr"/>
       <c r="M94" t="inlineStr"/>
       <c r="N94" t="inlineStr"/>
-      <c r="O94" t="inlineStr"/>
+      <c r="O94" t="inlineStr">
+        <is>
+          <t>2026-06-25T09:07:22</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -12665,7 +12679,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>ブチ切れ令嬢は報復を誓いました。 ～魔導書の力で祖国を叩き潰します～</t>
+          <t>バンドリ！ ゆめ∞みた</t>
         </is>
       </c>
       <c r="D95" t="b">
@@ -12681,33 +12695,43 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>Q.E.D.</t>
+          <t>これはぼくたちの生存のあらすじ</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>小倉唯</t>
+          <t>夢限大みゅーたいぷ</t>
         </is>
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=LFS_qg2JrPI</t>
+          <t>https://www.youtube.com/watch?v=Ech7Tj8ga0Y</t>
         </is>
       </c>
       <c r="J95" t="n">
-        <v>11323</v>
+        <v>124089</v>
       </c>
       <c r="K95" t="inlineStr">
         <is>
-          <t>Yui Ogura YouTube OFFICIAL CHANNEL</t>
-        </is>
-      </c>
-      <c r="L95" t="inlineStr"/>
-      <c r="M95" t="inlineStr"/>
-      <c r="N95" t="inlineStr"/>
+          <t>BanG Dream Channel☆</t>
+        </is>
+      </c>
+      <c r="L95" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=Ech7Tj8ga0Y</t>
+        </is>
+      </c>
+      <c r="M95" t="n">
+        <v>124089</v>
+      </c>
+      <c r="N95" t="inlineStr">
+        <is>
+          <t>BanG Dream Channel☆</t>
+        </is>
+      </c>
       <c r="O95" t="inlineStr">
         <is>
-          <t>2026-06-21T18:27:45</t>
+          <t>2026-06-24T09:06:31</t>
         </is>
       </c>
     </row>
@@ -12722,7 +12746,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>ブチ切れ令嬢は報復を誓いました。 ～魔導書の力で祖国を叩き潰します～</t>
+          <t>ヒロイン？聖女？いいえ、オールワークスメイドです（誇）！</t>
         </is>
       </c>
       <c r="D96" t="b">
@@ -12730,7 +12754,7 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F96" t="n">
@@ -12738,35 +12762,21 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>グッバイ・ララバイ</t>
+          <t>マデュアル↔ハート</t>
         </is>
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>大西亜玖璃</t>
-        </is>
-      </c>
-      <c r="I96" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=MzjYjMBpQ6g</t>
-        </is>
-      </c>
-      <c r="J96" t="n">
-        <v>4603</v>
-      </c>
-      <c r="K96" t="inlineStr">
-        <is>
-          <t>大西亜玖璃 - Aguri Onishi</t>
-        </is>
-      </c>
+          <t>メロディ・ウェーブ(CV：宮本侑芽) ルシアナ・ルトルバーグ(CV：大久保瑠美)</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr"/>
+      <c r="J96" t="inlineStr"/>
+      <c r="K96" t="inlineStr"/>
       <c r="L96" t="inlineStr"/>
       <c r="M96" t="inlineStr"/>
       <c r="N96" t="inlineStr"/>
-      <c r="O96" t="inlineStr">
-        <is>
-          <t>2026-06-21T18:27:58</t>
-        </is>
-      </c>
+      <c r="O96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="n">
@@ -12779,7 +12789,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>ふつつかな悪女ではございますが～雛宮蝶鼠とりかえ伝～</t>
+          <t>ヒロイン？聖女？いいえ、オールワークスメイドです（誇）！</t>
         </is>
       </c>
       <c r="D97" t="b">
@@ -12787,7 +12797,7 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F97" t="n">
@@ -12795,35 +12805,21 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>Sunny</t>
+          <t>ハンドメイド</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>milet</t>
-        </is>
-      </c>
-      <c r="I97" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=nR_vqhD2rGM</t>
-        </is>
-      </c>
-      <c r="J97" t="n">
-        <v>451401</v>
-      </c>
-      <c r="K97" t="inlineStr">
-        <is>
-          <t>TOHO animation</t>
-        </is>
-      </c>
+          <t>仲村宗悟</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr"/>
+      <c r="J97" t="inlineStr"/>
+      <c r="K97" t="inlineStr"/>
       <c r="L97" t="inlineStr"/>
       <c r="M97" t="inlineStr"/>
       <c r="N97" t="inlineStr"/>
-      <c r="O97" t="inlineStr">
-        <is>
-          <t>2026-06-21T18:28:12</t>
-        </is>
-      </c>
+      <c r="O97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -12836,7 +12832,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>BLACK TORCH</t>
+          <t>ブチ切れ令嬢は報復を誓いました。 ～魔導書の力で祖国を叩き潰します～</t>
         </is>
       </c>
       <c r="D98" t="b">
@@ -12852,21 +12848,35 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>FREEZE ME UP</t>
+          <t>Q.E.D.</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>SiM</t>
-        </is>
-      </c>
-      <c r="I98" t="inlineStr"/>
-      <c r="J98" t="inlineStr"/>
-      <c r="K98" t="inlineStr"/>
+          <t>小倉唯</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=LFS_qg2JrPI</t>
+        </is>
+      </c>
+      <c r="J98" t="n">
+        <v>11323</v>
+      </c>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>Yui Ogura YouTube OFFICIAL CHANNEL</t>
+        </is>
+      </c>
       <c r="L98" t="inlineStr"/>
       <c r="M98" t="inlineStr"/>
       <c r="N98" t="inlineStr"/>
-      <c r="O98" t="inlineStr"/>
+      <c r="O98" t="inlineStr">
+        <is>
+          <t>2026-06-21T18:27:45</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="n">
@@ -12879,7 +12889,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>BLACK TORCH</t>
+          <t>ブチ切れ令嬢は報復を誓いました。 ～魔導書の力で祖国を叩き潰します～</t>
         </is>
       </c>
       <c r="D99" t="b">
@@ -12895,21 +12905,35 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>Groooovy</t>
+          <t>グッバイ・ララバイ</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>I Don't Like Mondays.</t>
-        </is>
-      </c>
-      <c r="I99" t="inlineStr"/>
-      <c r="J99" t="inlineStr"/>
-      <c r="K99" t="inlineStr"/>
+          <t>大西亜玖璃</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=MzjYjMBpQ6g</t>
+        </is>
+      </c>
+      <c r="J99" t="n">
+        <v>4603</v>
+      </c>
+      <c r="K99" t="inlineStr">
+        <is>
+          <t>大西亜玖璃 - Aguri Onishi</t>
+        </is>
+      </c>
       <c r="L99" t="inlineStr"/>
       <c r="M99" t="inlineStr"/>
       <c r="N99" t="inlineStr"/>
-      <c r="O99" t="inlineStr"/>
+      <c r="O99" t="inlineStr">
+        <is>
+          <t>2026-06-21T18:27:58</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="n">
@@ -12922,7 +12946,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>プラノサウルス ガチコセイブツ部</t>
+          <t>ふつつかな悪女ではございますが～雛宮蝶鼠とりかえ伝～</t>
         </is>
       </c>
       <c r="D100" t="b">
@@ -12930,7 +12954,7 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>主題歌</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F100" t="n">
@@ -12938,21 +12962,35 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>ガチde古生</t>
+          <t>Sunny</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>リンクルプラネット</t>
-        </is>
-      </c>
-      <c r="I100" t="inlineStr"/>
-      <c r="J100" t="inlineStr"/>
-      <c r="K100" t="inlineStr"/>
+          <t>milet</t>
+        </is>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=nR_vqhD2rGM</t>
+        </is>
+      </c>
+      <c r="J100" t="n">
+        <v>451401</v>
+      </c>
+      <c r="K100" t="inlineStr">
+        <is>
+          <t>TOHO animation</t>
+        </is>
+      </c>
       <c r="L100" t="inlineStr"/>
       <c r="M100" t="inlineStr"/>
       <c r="N100" t="inlineStr"/>
-      <c r="O100" t="inlineStr"/>
+      <c r="O100" t="inlineStr">
+        <is>
+          <t>2026-06-21T18:28:12</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -12965,7 +13003,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>BLEACH 千年血戦篇-禍進譚-</t>
+          <t>BLACK TORCH</t>
         </is>
       </c>
       <c r="D101" t="b">
@@ -12981,12 +13019,12 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>I-BULL</t>
+          <t>FREEZE ME UP</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>jo0ji</t>
+          <t>SiM</t>
         </is>
       </c>
       <c r="I101" t="inlineStr"/>
@@ -13008,7 +13046,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>BLEACH 千年血戦篇-禍進譚-</t>
+          <t>BLACK TORCH</t>
         </is>
       </c>
       <c r="D102" t="b">
@@ -13024,12 +13062,12 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>螺旋</t>
+          <t>Groooovy</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>9Lana</t>
+          <t>I Don't Like Mondays.</t>
         </is>
       </c>
       <c r="I102" t="inlineStr"/>
@@ -13051,7 +13089,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>文豪ストレイドッグス わん！２</t>
+          <t>プラノサウルス ガチコセイブツ部</t>
         </is>
       </c>
       <c r="D103" t="b">
@@ -13059,7 +13097,7 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>主題歌</t>
         </is>
       </c>
       <c r="F103" t="n">
@@ -13067,12 +13105,12 @@
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>僕ら～芥川龍之介Ver.～</t>
+          <t>ガチde古生</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>芥川龍之介（CV.小野賢章）</t>
+          <t>リンクルプラネット</t>
         </is>
       </c>
       <c r="I103" t="inlineStr"/>
@@ -13094,7 +13132,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>ヘルモード ～やり込み好きのゲーマーは廃設定の異世界で無双する～ 2nd Season</t>
+          <t>BLEACH 千年血戦篇-禍進譚-</t>
         </is>
       </c>
       <c r="D104" t="b">
@@ -13110,12 +13148,12 @@
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>○✕△□</t>
+          <t>I-BULL</t>
         </is>
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>浪漫派マシュマロ</t>
+          <t>jo0ji</t>
         </is>
       </c>
       <c r="I104" t="inlineStr"/>
@@ -13137,7 +13175,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>ヘルモード ～やり込み好きのゲーマーは廃設定の異世界で無双する～ 2nd Season</t>
+          <t>BLEACH 千年血戦篇-禍進譚-</t>
         </is>
       </c>
       <c r="D105" t="b">
@@ -13153,12 +13191,12 @@
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>Firetail</t>
+          <t>螺旋</t>
         </is>
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>チョーキューメイ</t>
+          <t>9Lana</t>
         </is>
       </c>
       <c r="I105" t="inlineStr"/>
@@ -13180,7 +13218,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>北斗の拳 拳王軍ザコたちの挽歌 第2クール</t>
+          <t>文豪ストレイドッグス わん！２</t>
         </is>
       </c>
       <c r="D106" t="b">
@@ -13188,7 +13226,7 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F106" t="n">
@@ -13196,12 +13234,12 @@
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>Blacker Co., Ltd.</t>
+          <t>僕ら～芥川龍之介Ver.～</t>
         </is>
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>イツカ▶</t>
+          <t>芥川龍之介（CV.小野賢章）</t>
         </is>
       </c>
       <c r="I106" t="inlineStr"/>
@@ -13223,7 +13261,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>北斗の拳 拳王軍ザコたちの挽歌 第2クール</t>
+          <t>ヘルモード ～やり込み好きのゲーマーは廃設定の異世界で無双する～ 2nd Season</t>
         </is>
       </c>
       <c r="D107" t="b">
@@ -13231,7 +13269,7 @@
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F107" t="n">
@@ -13239,12 +13277,12 @@
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>Elegy of the Enemies</t>
+          <t>○✕△□</t>
         </is>
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>The Canbellz</t>
+          <t>浪漫派マシュマロ</t>
         </is>
       </c>
       <c r="I107" t="inlineStr"/>
@@ -13266,7 +13304,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>北斗の拳 拳王軍ザコたちの挽歌 第2クール</t>
+          <t>ヘルモード ～やり込み好きのゲーマーは廃設定の異世界で無双する～ 2nd Season</t>
         </is>
       </c>
       <c r="D108" t="b">
@@ -13278,16 +13316,16 @@
         </is>
       </c>
       <c r="F108" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>白い蝶が飛んだら</t>
+          <t>Firetail</t>
         </is>
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>イツカ▶ feat. Dr. Washington | Special Guest Guitar:Tsuyoshi Ujiki</t>
+          <t>チョーキューメイ</t>
         </is>
       </c>
       <c r="I108" t="inlineStr"/>
@@ -13309,7 +13347,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>炎の闘球女 ドッジ弾子</t>
+          <t>北斗の拳 拳王軍ザコたちの挽歌 第2クール</t>
         </is>
       </c>
       <c r="D109" t="b">
@@ -13325,12 +13363,12 @@
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>会心の一劇</t>
+          <t>Blacker Co., Ltd.</t>
         </is>
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>ももいろクローバーZ</t>
+          <t>イツカ▶</t>
         </is>
       </c>
       <c r="I109" t="inlineStr"/>
@@ -13352,7 +13390,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>炎の闘球女 ドッジ弾子</t>
+          <t>北斗の拳 拳王軍ザコたちの挽歌 第2クール</t>
         </is>
       </c>
       <c r="D110" t="b">
@@ -13368,12 +13406,12 @@
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>Welcome to あざとさワールド</t>
+          <t>Elegy of the Enemies</t>
         </is>
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>i☆Ris</t>
+          <t>The Canbellz</t>
         </is>
       </c>
       <c r="I110" t="inlineStr"/>
@@ -13395,7 +13433,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>魔法少女リリカルなのは EXCEEDS Gun Blaze Vengeance</t>
+          <t>北斗の拳 拳王軍ザコたちの挽歌 第2クール</t>
         </is>
       </c>
       <c r="D111" t="b">
@@ -13403,43 +13441,29 @@
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F111" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>CRIMSON BULLET</t>
+          <t>白い蝶が飛んだら</t>
         </is>
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>水樹奈々</t>
-        </is>
-      </c>
-      <c r="I111" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=TzvGIjaMbYE</t>
-        </is>
-      </c>
-      <c r="J111" t="n">
-        <v>590624</v>
-      </c>
-      <c r="K111" t="inlineStr">
-        <is>
-          <t>魔法少女リリカルなのは YouTube OFFICIAL CHANNEL</t>
-        </is>
-      </c>
+          <t>イツカ▶ feat. Dr. Washington | Special Guest Guitar:Tsuyoshi Ujiki</t>
+        </is>
+      </c>
+      <c r="I111" t="inlineStr"/>
+      <c r="J111" t="inlineStr"/>
+      <c r="K111" t="inlineStr"/>
       <c r="L111" t="inlineStr"/>
       <c r="M111" t="inlineStr"/>
       <c r="N111" t="inlineStr"/>
-      <c r="O111" t="inlineStr">
-        <is>
-          <t>2026-06-21T18:29:37</t>
-        </is>
-      </c>
+      <c r="O111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="n">
@@ -13452,7 +13476,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>魔法少女リリカルなのは EXCEEDS Gun Blaze Vengeance</t>
+          <t>炎の闘球女 ドッジ弾子</t>
         </is>
       </c>
       <c r="D112" t="b">
@@ -13460,7 +13484,7 @@
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F112" t="n">
@@ -13468,35 +13492,21 @@
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>Ephemeral</t>
+          <t>会心の一劇</t>
         </is>
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>青木陽菜</t>
-        </is>
-      </c>
-      <c r="I112" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=TzvGIjaMbYE</t>
-        </is>
-      </c>
-      <c r="J112" t="n">
-        <v>590624</v>
-      </c>
-      <c r="K112" t="inlineStr">
-        <is>
-          <t>魔法少女リリカルなのは YouTube OFFICIAL CHANNEL</t>
-        </is>
-      </c>
+          <t>ももいろクローバーZ</t>
+        </is>
+      </c>
+      <c r="I112" t="inlineStr"/>
+      <c r="J112" t="inlineStr"/>
+      <c r="K112" t="inlineStr"/>
       <c r="L112" t="inlineStr"/>
       <c r="M112" t="inlineStr"/>
       <c r="N112" t="inlineStr"/>
-      <c r="O112" t="inlineStr">
-        <is>
-          <t>2026-06-21T18:29:56</t>
-        </is>
-      </c>
+      <c r="O112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="n">
@@ -13509,7 +13519,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>身代わり令嬢を救ったのは冷酷無慈悲な氷の王子の愛でした</t>
+          <t>炎の闘球女 ドッジ弾子</t>
         </is>
       </c>
       <c r="D113" t="b">
@@ -13525,12 +13535,12 @@
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>とけて煌る</t>
+          <t>Welcome to あざとさワールド</t>
         </is>
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>neNna</t>
+          <t>i☆Ris</t>
         </is>
       </c>
       <c r="I113" t="inlineStr"/>
@@ -13552,7 +13562,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>無自覚聖女は今日も無意識に力を垂れ流す</t>
+          <t>魔法少女リリカルなのは EXCEEDS Gun Blaze Vengeance</t>
         </is>
       </c>
       <c r="D114" t="b">
@@ -13568,21 +13578,35 @@
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>Windmaker</t>
+          <t>CRIMSON BULLET</t>
         </is>
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>花耶</t>
-        </is>
-      </c>
-      <c r="I114" t="inlineStr"/>
-      <c r="J114" t="inlineStr"/>
-      <c r="K114" t="inlineStr"/>
+          <t>水樹奈々</t>
+        </is>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=TzvGIjaMbYE</t>
+        </is>
+      </c>
+      <c r="J114" t="n">
+        <v>590624</v>
+      </c>
+      <c r="K114" t="inlineStr">
+        <is>
+          <t>魔法少女リリカルなのは YouTube OFFICIAL CHANNEL</t>
+        </is>
+      </c>
       <c r="L114" t="inlineStr"/>
       <c r="M114" t="inlineStr"/>
       <c r="N114" t="inlineStr"/>
-      <c r="O114" t="inlineStr"/>
+      <c r="O114" t="inlineStr">
+        <is>
+          <t>2026-06-21T18:29:37</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="n">
@@ -13595,7 +13619,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>無自覚聖女は今日も無意識に力を垂れ流す</t>
+          <t>魔法少女リリカルなのは EXCEEDS Gun Blaze Vengeance</t>
         </is>
       </c>
       <c r="D115" t="b">
@@ -13611,21 +13635,35 @@
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>アンノウンミー</t>
+          <t>Ephemeral</t>
         </is>
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>ウタヒメドリーム オールスターズ【夢咲いぶき（CV:山﨑玲奈） 桜木舞華（CV:鈴木杏奈） 真白清美（CV:其原有沙） HiREN（CV:花耶） 水月ひかり（CV:礒部花凜） 高木凛（CV:鷲見友美ジェナ） 萩原ひまわり（CV:倉知玲鳳） SAKURAKO（CV:竹内夢）】</t>
-        </is>
-      </c>
-      <c r="I115" t="inlineStr"/>
-      <c r="J115" t="inlineStr"/>
-      <c r="K115" t="inlineStr"/>
+          <t>青木陽菜</t>
+        </is>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=TzvGIjaMbYE</t>
+        </is>
+      </c>
+      <c r="J115" t="n">
+        <v>590624</v>
+      </c>
+      <c r="K115" t="inlineStr">
+        <is>
+          <t>魔法少女リリカルなのは YouTube OFFICIAL CHANNEL</t>
+        </is>
+      </c>
       <c r="L115" t="inlineStr"/>
       <c r="M115" t="inlineStr"/>
       <c r="N115" t="inlineStr"/>
-      <c r="O115" t="inlineStr"/>
+      <c r="O115" t="inlineStr">
+        <is>
+          <t>2026-06-21T18:29:56</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="n">
@@ -13638,7 +13676,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>無職転生Ⅲ ～異世界行ったら本気だす～</t>
+          <t>身代わり令嬢を救ったのは冷酷無慈悲な氷の王子の愛でした</t>
         </is>
       </c>
       <c r="D116" t="b">
@@ -13646,7 +13684,7 @@
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F116" t="n">
@@ -13654,45 +13692,21 @@
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>決意の唄</t>
+          <t>とけて煌る</t>
         </is>
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>大原ゆい子</t>
-        </is>
-      </c>
-      <c r="I116" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=hZ6TnKvB2rc</t>
-        </is>
-      </c>
-      <c r="J116" t="n">
-        <v>12105753</v>
-      </c>
-      <c r="K116" t="inlineStr">
-        <is>
-          <t>大原ゆい子Official YouTube</t>
-        </is>
-      </c>
-      <c r="L116" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=PINgF6rCuME</t>
-        </is>
-      </c>
-      <c r="M116" t="n">
-        <v>2457533</v>
-      </c>
-      <c r="N116" t="inlineStr">
-        <is>
-          <t>TOHO animation</t>
-        </is>
-      </c>
-      <c r="O116" t="inlineStr">
-        <is>
-          <t>2026-06-21T18:30:35</t>
-        </is>
-      </c>
+          <t>neNna</t>
+        </is>
+      </c>
+      <c r="I116" t="inlineStr"/>
+      <c r="J116" t="inlineStr"/>
+      <c r="K116" t="inlineStr"/>
+      <c r="L116" t="inlineStr"/>
+      <c r="M116" t="inlineStr"/>
+      <c r="N116" t="inlineStr"/>
+      <c r="O116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="n">
@@ -13705,7 +13719,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>無職転生Ⅲ ～異世界行ったら本気だす～</t>
+          <t>無自覚聖女は今日も無意識に力を垂れ流す</t>
         </is>
       </c>
       <c r="D117" t="b">
@@ -13713,7 +13727,7 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F117" t="n">
@@ -13721,35 +13735,21 @@
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>祈り、終われば</t>
+          <t>Windmaker</t>
         </is>
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>中島美嘉</t>
-        </is>
-      </c>
-      <c r="I117" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=ODxfIvSgWuo</t>
-        </is>
-      </c>
-      <c r="J117" t="n">
-        <v>1140774</v>
-      </c>
-      <c r="K117" t="inlineStr">
-        <is>
-          <t>TOHO animation</t>
-        </is>
-      </c>
+          <t>花耶</t>
+        </is>
+      </c>
+      <c r="I117" t="inlineStr"/>
+      <c r="J117" t="inlineStr"/>
+      <c r="K117" t="inlineStr"/>
       <c r="L117" t="inlineStr"/>
       <c r="M117" t="inlineStr"/>
       <c r="N117" t="inlineStr"/>
-      <c r="O117" t="inlineStr">
-        <is>
-          <t>2026-06-21T18:31:08</t>
-        </is>
-      </c>
+      <c r="O117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="n">
@@ -13762,7 +13762,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>メビウス・ダスト</t>
+          <t>無自覚聖女は今日も無意識に力を垂れ流す</t>
         </is>
       </c>
       <c r="D118" t="b">
@@ -13770,7 +13770,7 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F118" t="n">
@@ -13778,45 +13778,21 @@
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>メビウス</t>
+          <t>アンノウンミー</t>
         </is>
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>家入レオ</t>
-        </is>
-      </c>
-      <c r="I118" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=vJzWWkigrU8</t>
-        </is>
-      </c>
-      <c r="J118" t="n">
-        <v>32222</v>
-      </c>
-      <c r="K118" t="inlineStr">
-        <is>
-          <t>家入レオ</t>
-        </is>
-      </c>
-      <c r="L118" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=5QGZX_Kky4I</t>
-        </is>
-      </c>
-      <c r="M118" t="n">
-        <v>27576</v>
-      </c>
-      <c r="N118" t="inlineStr">
-        <is>
-          <t>leafstamp</t>
-        </is>
-      </c>
-      <c r="O118" t="inlineStr">
-        <is>
-          <t>2026-06-21T18:31:32</t>
-        </is>
-      </c>
+          <t>ウタヒメドリーム オールスターズ【夢咲いぶき（CV:山﨑玲奈） 桜木舞華（CV:鈴木杏奈） 真白清美（CV:其原有沙） HiREN（CV:花耶） 水月ひかり（CV:礒部花凜） 高木凛（CV:鷲見友美ジェナ） 萩原ひまわり（CV:倉知玲鳳） SAKURAKO（CV:竹内夢）】</t>
+        </is>
+      </c>
+      <c r="I118" t="inlineStr"/>
+      <c r="J118" t="inlineStr"/>
+      <c r="K118" t="inlineStr"/>
+      <c r="L118" t="inlineStr"/>
+      <c r="M118" t="inlineStr"/>
+      <c r="N118" t="inlineStr"/>
+      <c r="O118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="n">
@@ -13829,7 +13805,7 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>メビウス・ダスト</t>
+          <t>無職転生Ⅲ ～異世界行ったら本気だす～</t>
         </is>
       </c>
       <c r="D119" t="b">
@@ -13837,7 +13813,7 @@
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F119" t="n">
@@ -13845,21 +13821,45 @@
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>ジレンマ</t>
+          <t>決意の唄</t>
         </is>
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>冨岡愛</t>
-        </is>
-      </c>
-      <c r="I119" t="inlineStr"/>
-      <c r="J119" t="inlineStr"/>
-      <c r="K119" t="inlineStr"/>
-      <c r="L119" t="inlineStr"/>
-      <c r="M119" t="inlineStr"/>
-      <c r="N119" t="inlineStr"/>
-      <c r="O119" t="inlineStr"/>
+          <t>大原ゆい子</t>
+        </is>
+      </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=hZ6TnKvB2rc</t>
+        </is>
+      </c>
+      <c r="J119" t="n">
+        <v>12105753</v>
+      </c>
+      <c r="K119" t="inlineStr">
+        <is>
+          <t>大原ゆい子Official YouTube</t>
+        </is>
+      </c>
+      <c r="L119" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=PINgF6rCuME</t>
+        </is>
+      </c>
+      <c r="M119" t="n">
+        <v>2457533</v>
+      </c>
+      <c r="N119" t="inlineStr">
+        <is>
+          <t>TOHO animation</t>
+        </is>
+      </c>
+      <c r="O119" t="inlineStr">
+        <is>
+          <t>2026-06-21T18:30:35</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="n">
@@ -13872,7 +13872,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>ヤニねこ</t>
+          <t>無職転生Ⅲ ～異世界行ったら本気だす～</t>
         </is>
       </c>
       <c r="D120" t="b">
@@ -13880,7 +13880,7 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F120" t="n">
@@ -13888,25 +13888,25 @@
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>なんもねえ</t>
+          <t>祈り、終われば</t>
         </is>
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>忘れらんねえよ</t>
+          <t>中島美嘉</t>
         </is>
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=ydK2WdTAOgU</t>
+          <t>https://www.youtube.com/watch?v=ODxfIvSgWuo</t>
         </is>
       </c>
       <c r="J120" t="n">
-        <v>480871</v>
+        <v>1140774</v>
       </c>
       <c r="K120" t="inlineStr">
         <is>
-          <t>TVアニメ『ヤニねこ』公式【ハメちゃんねる】</t>
+          <t>TOHO animation</t>
         </is>
       </c>
       <c r="L120" t="inlineStr"/>
@@ -13914,7 +13914,7 @@
       <c r="N120" t="inlineStr"/>
       <c r="O120" t="inlineStr">
         <is>
-          <t>2026-06-21T18:32:14</t>
+          <t>2026-06-21T18:31:08</t>
         </is>
       </c>
     </row>
@@ -13929,7 +13929,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>ヤニねこ</t>
+          <t>メビウス・ダスト</t>
         </is>
       </c>
       <c r="D121" t="b">
@@ -13937,7 +13937,7 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F121" t="n">
@@ -13945,33 +13945,43 @@
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>煙とブルー</t>
+          <t>メビウス</t>
         </is>
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>ネクライトーキー</t>
+          <t>家入レオ</t>
         </is>
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=ydK2WdTAOgU</t>
+          <t>https://www.youtube.com/watch?v=vJzWWkigrU8</t>
         </is>
       </c>
       <c r="J121" t="n">
-        <v>480871</v>
+        <v>32222</v>
       </c>
       <c r="K121" t="inlineStr">
         <is>
-          <t>TVアニメ『ヤニねこ』公式【ハメちゃんねる】</t>
-        </is>
-      </c>
-      <c r="L121" t="inlineStr"/>
-      <c r="M121" t="inlineStr"/>
-      <c r="N121" t="inlineStr"/>
+          <t>家入レオ</t>
+        </is>
+      </c>
+      <c r="L121" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=5QGZX_Kky4I</t>
+        </is>
+      </c>
+      <c r="M121" t="n">
+        <v>27576</v>
+      </c>
+      <c r="N121" t="inlineStr">
+        <is>
+          <t>leafstamp</t>
+        </is>
+      </c>
       <c r="O121" t="inlineStr">
         <is>
-          <t>2026-06-21T18:32:32</t>
+          <t>2026-06-21T18:31:32</t>
         </is>
       </c>
     </row>
@@ -13986,7 +13996,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>闇芝居 十七期</t>
+          <t>メビウス・ダスト</t>
         </is>
       </c>
       <c r="D122" t="b">
@@ -14002,12 +14012,12 @@
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>闇芝居のブルース</t>
+          <t>ジレンマ</t>
         </is>
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>風輪（徳間ジャパンコミュニケーションズ）</t>
+          <t>冨岡愛</t>
         </is>
       </c>
       <c r="I122" t="inlineStr"/>
@@ -14029,7 +14039,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>幼女戦記Ⅱ</t>
+          <t>ヤニねこ</t>
         </is>
       </c>
       <c r="D123" t="b">
@@ -14045,25 +14055,25 @@
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t>Why? RED induction</t>
+          <t>なんもねえ</t>
         </is>
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>MYTH &amp; ROID</t>
+          <t>忘れらんねえよ</t>
         </is>
       </c>
       <c r="I123" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=RMaOR0Pyfts</t>
+          <t>https://www.youtube.com/watch?v=ydK2WdTAOgU</t>
         </is>
       </c>
       <c r="J123" t="n">
-        <v>50838</v>
+        <v>480871</v>
       </c>
       <c r="K123" t="inlineStr">
         <is>
-          <t>MYTH &amp; ROID Official Channel</t>
+          <t>TVアニメ『ヤニねこ』公式【ハメちゃんねる】</t>
         </is>
       </c>
       <c r="L123" t="inlineStr"/>
@@ -14071,7 +14081,7 @@
       <c r="N123" t="inlineStr"/>
       <c r="O123" t="inlineStr">
         <is>
-          <t>2026-06-21T18:33:01</t>
+          <t>2026-06-21T18:32:14</t>
         </is>
       </c>
     </row>
@@ -14086,7 +14096,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>幼女戦記Ⅱ</t>
+          <t>ヤニねこ</t>
         </is>
       </c>
       <c r="D124" t="b">
@@ -14102,21 +14112,35 @@
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>Weiter! Weiter!</t>
+          <t>煙とブルー</t>
         </is>
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>ターニャ・デグレチャフ（CV：悠木碧）</t>
-        </is>
-      </c>
-      <c r="I124" t="inlineStr"/>
-      <c r="J124" t="inlineStr"/>
-      <c r="K124" t="inlineStr"/>
+          <t>ネクライトーキー</t>
+        </is>
+      </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=ydK2WdTAOgU</t>
+        </is>
+      </c>
+      <c r="J124" t="n">
+        <v>480871</v>
+      </c>
+      <c r="K124" t="inlineStr">
+        <is>
+          <t>TVアニメ『ヤニねこ』公式【ハメちゃんねる】</t>
+        </is>
+      </c>
       <c r="L124" t="inlineStr"/>
       <c r="M124" t="inlineStr"/>
       <c r="N124" t="inlineStr"/>
-      <c r="O124" t="inlineStr"/>
+      <c r="O124" t="inlineStr">
+        <is>
+          <t>2026-06-21T18:32:32</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="n">
@@ -14129,7 +14153,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>鎧真伝サムライトルーパー 第2クール</t>
+          <t>闇芝居 十七期</t>
         </is>
       </c>
       <c r="D125" t="b">
@@ -14137,7 +14161,7 @@
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F125" t="n">
@@ -14145,45 +14169,21 @@
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>YOAKE</t>
+          <t>闇芝居のブルース</t>
         </is>
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>blank paper</t>
-        </is>
-      </c>
-      <c r="I125" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=kHUPdA8H6qk</t>
-        </is>
-      </c>
-      <c r="J125" t="n">
-        <v>603666</v>
-      </c>
-      <c r="K125" t="inlineStr">
-        <is>
-          <t>TVアニメ『鎧真伝サムライトルーパー』公式</t>
-        </is>
-      </c>
-      <c r="L125" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=kHUPdA8H6qk</t>
-        </is>
-      </c>
-      <c r="M125" t="n">
-        <v>603666</v>
-      </c>
-      <c r="N125" t="inlineStr">
-        <is>
-          <t>TVアニメ『鎧真伝サムライトルーパー』公式</t>
-        </is>
-      </c>
-      <c r="O125" t="inlineStr">
-        <is>
-          <t>2026-06-21T18:33:22</t>
-        </is>
-      </c>
+          <t>風輪（徳間ジャパンコミュニケーションズ）</t>
+        </is>
+      </c>
+      <c r="I125" t="inlineStr"/>
+      <c r="J125" t="inlineStr"/>
+      <c r="K125" t="inlineStr"/>
+      <c r="L125" t="inlineStr"/>
+      <c r="M125" t="inlineStr"/>
+      <c r="N125" t="inlineStr"/>
+      <c r="O125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="n">
@@ -14196,7 +14196,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>鎧真伝サムライトルーパー 第2クール</t>
+          <t>幼女戦記Ⅱ</t>
         </is>
       </c>
       <c r="D126" t="b">
@@ -14208,29 +14208,29 @@
         </is>
       </c>
       <c r="F126" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t>BAD遺伝子</t>
+          <t>Why? RED induction</t>
         </is>
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>Dannie May</t>
+          <t>MYTH &amp; ROID</t>
         </is>
       </c>
       <c r="I126" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=OKEoQo3cGVg</t>
+          <t>https://www.youtube.com/watch?v=RMaOR0Pyfts</t>
         </is>
       </c>
       <c r="J126" t="n">
-        <v>66350</v>
+        <v>50838</v>
       </c>
       <c r="K126" t="inlineStr">
         <is>
-          <t>TVアニメ『鎧真伝サムライトルーパー』公式</t>
+          <t>MYTH &amp; ROID Official Channel</t>
         </is>
       </c>
       <c r="L126" t="inlineStr"/>
@@ -14238,7 +14238,7 @@
       <c r="N126" t="inlineStr"/>
       <c r="O126" t="inlineStr">
         <is>
-          <t>2026-06-21T18:33:34</t>
+          <t>2026-06-21T18:33:01</t>
         </is>
       </c>
     </row>
@@ -14253,7 +14253,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>鎧真伝サムライトルーパー 第2クール</t>
+          <t>幼女戦記Ⅱ</t>
         </is>
       </c>
       <c r="D127" t="b">
@@ -14269,45 +14269,21 @@
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t>POWER</t>
+          <t>Weiter! Weiter!</t>
         </is>
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>ONE OR EIGHT</t>
-        </is>
-      </c>
-      <c r="I127" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=aw45Q_mr0_M</t>
-        </is>
-      </c>
-      <c r="J127" t="n">
-        <v>9441868</v>
-      </c>
-      <c r="K127" t="inlineStr">
-        <is>
-          <t>ONE OR EIGHT</t>
-        </is>
-      </c>
-      <c r="L127" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=VJflo-z7e7A</t>
-        </is>
-      </c>
-      <c r="M127" t="n">
-        <v>151043</v>
-      </c>
-      <c r="N127" t="inlineStr">
-        <is>
-          <t>TVアニメ『鎧真伝サムライトルーパー』公式</t>
-        </is>
-      </c>
-      <c r="O127" t="inlineStr">
-        <is>
-          <t>2026-06-21T18:33:47</t>
-        </is>
-      </c>
+          <t>ターニャ・デグレチャフ（CV：悠木碧）</t>
+        </is>
+      </c>
+      <c r="I127" t="inlineStr"/>
+      <c r="J127" t="inlineStr"/>
+      <c r="K127" t="inlineStr"/>
+      <c r="L127" t="inlineStr"/>
+      <c r="M127" t="inlineStr"/>
+      <c r="N127" t="inlineStr"/>
+      <c r="O127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="n">
@@ -14328,41 +14304,51 @@
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F128" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t>ばけもん</t>
+          <t>YOAKE</t>
         </is>
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>カラノア</t>
+          <t>blank paper</t>
         </is>
       </c>
       <c r="I128" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=OKEoQo3cGVg</t>
+          <t>https://www.youtube.com/watch?v=kHUPdA8H6qk</t>
         </is>
       </c>
       <c r="J128" t="n">
-        <v>66350</v>
+        <v>603666</v>
       </c>
       <c r="K128" t="inlineStr">
         <is>
           <t>TVアニメ『鎧真伝サムライトルーパー』公式</t>
         </is>
       </c>
-      <c r="L128" t="inlineStr"/>
-      <c r="M128" t="inlineStr"/>
-      <c r="N128" t="inlineStr"/>
+      <c r="L128" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=kHUPdA8H6qk</t>
+        </is>
+      </c>
+      <c r="M128" t="n">
+        <v>603666</v>
+      </c>
+      <c r="N128" t="inlineStr">
+        <is>
+          <t>TVアニメ『鎧真伝サムライトルーパー』公式</t>
+        </is>
+      </c>
       <c r="O128" t="inlineStr">
         <is>
-          <t>2026-06-21T18:34:00</t>
+          <t>2026-06-21T18:33:22</t>
         </is>
       </c>
     </row>
@@ -14377,7 +14363,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>落第賢者の学院無双～二度目の転生、Sランクチート魔術師冒険録～</t>
+          <t>鎧真伝サムライトルーパー 第2クール</t>
         </is>
       </c>
       <c r="D129" t="b">
@@ -14389,25 +14375,39 @@
         </is>
       </c>
       <c r="F129" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>＋ENCOUNT</t>
+          <t>BAD遺伝子</t>
         </is>
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>FLOW</t>
-        </is>
-      </c>
-      <c r="I129" t="inlineStr"/>
-      <c r="J129" t="inlineStr"/>
-      <c r="K129" t="inlineStr"/>
+          <t>Dannie May</t>
+        </is>
+      </c>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=OKEoQo3cGVg</t>
+        </is>
+      </c>
+      <c r="J129" t="n">
+        <v>66350</v>
+      </c>
+      <c r="K129" t="inlineStr">
+        <is>
+          <t>TVアニメ『鎧真伝サムライトルーパー』公式</t>
+        </is>
+      </c>
       <c r="L129" t="inlineStr"/>
       <c r="M129" t="inlineStr"/>
       <c r="N129" t="inlineStr"/>
-      <c r="O129" t="inlineStr"/>
+      <c r="O129" t="inlineStr">
+        <is>
+          <t>2026-06-21T18:33:34</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="n">
@@ -14420,7 +14420,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>落第賢者の学院無双～二度目の転生、Sランクチート魔術師冒険録～</t>
+          <t>鎧真伝サムライトルーパー 第2クール</t>
         </is>
       </c>
       <c r="D130" t="b">
@@ -14436,21 +14436,45 @@
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>憧憬</t>
+          <t>POWER</t>
         </is>
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>TrySail</t>
-        </is>
-      </c>
-      <c r="I130" t="inlineStr"/>
-      <c r="J130" t="inlineStr"/>
-      <c r="K130" t="inlineStr"/>
-      <c r="L130" t="inlineStr"/>
-      <c r="M130" t="inlineStr"/>
-      <c r="N130" t="inlineStr"/>
-      <c r="O130" t="inlineStr"/>
+          <t>ONE OR EIGHT</t>
+        </is>
+      </c>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=aw45Q_mr0_M</t>
+        </is>
+      </c>
+      <c r="J130" t="n">
+        <v>9441868</v>
+      </c>
+      <c r="K130" t="inlineStr">
+        <is>
+          <t>ONE OR EIGHT</t>
+        </is>
+      </c>
+      <c r="L130" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=VJflo-z7e7A</t>
+        </is>
+      </c>
+      <c r="M130" t="n">
+        <v>151043</v>
+      </c>
+      <c r="N130" t="inlineStr">
+        <is>
+          <t>TVアニメ『鎧真伝サムライトルーパー』公式</t>
+        </is>
+      </c>
+      <c r="O130" t="inlineStr">
+        <is>
+          <t>2026-06-21T18:33:47</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="n">
@@ -14463,37 +14487,51 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>ラブライブ！虹ヶ咲学園スクールアイドル同好会</t>
+          <t>鎧真伝サムライトルーパー 第2クール</t>
         </is>
       </c>
       <c r="D131" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F131" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>虹色Passions！</t>
+          <t>ばけもん</t>
         </is>
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>虹ヶ咲学園スクールアイドル同好会</t>
-        </is>
-      </c>
-      <c r="I131" t="inlineStr"/>
-      <c r="J131" t="inlineStr"/>
-      <c r="K131" t="inlineStr"/>
+          <t>カラノア</t>
+        </is>
+      </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=OKEoQo3cGVg</t>
+        </is>
+      </c>
+      <c r="J131" t="n">
+        <v>66350</v>
+      </c>
+      <c r="K131" t="inlineStr">
+        <is>
+          <t>TVアニメ『鎧真伝サムライトルーパー』公式</t>
+        </is>
+      </c>
       <c r="L131" t="inlineStr"/>
       <c r="M131" t="inlineStr"/>
       <c r="N131" t="inlineStr"/>
-      <c r="O131" t="inlineStr"/>
+      <c r="O131" t="inlineStr">
+        <is>
+          <t>2026-06-21T18:34:00</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="n">
@@ -14506,15 +14544,15 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>ラブライブ！虹ヶ咲学園スクールアイドル同好会</t>
+          <t>落第賢者の学院無双～二度目の転生、Sランクチート魔術師冒険録～</t>
         </is>
       </c>
       <c r="D132" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F132" t="n">
@@ -14522,12 +14560,12 @@
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>NEO SKY, NEO MAP!</t>
+          <t>＋ENCOUNT</t>
         </is>
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>虹ヶ咲学園スクールアイドル同好会</t>
+          <t>FLOW</t>
         </is>
       </c>
       <c r="I132" t="inlineStr"/>
@@ -14549,7 +14587,7 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>領民0人スタートの辺境領主様</t>
+          <t>落第賢者の学院無双～二度目の転生、Sランクチート魔術師冒険録～</t>
         </is>
       </c>
       <c r="D133" t="b">
@@ -14557,7 +14595,7 @@
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F133" t="n">
@@ -14565,12 +14603,12 @@
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>Wonder</t>
+          <t>憧憬</t>
         </is>
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>CROWN HEAD</t>
+          <t>TrySail</t>
         </is>
       </c>
       <c r="I133" t="inlineStr"/>
@@ -14592,15 +14630,15 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>領民0人スタートの辺境領主様</t>
+          <t>ラブライブ！虹ヶ咲学園スクールアイドル同好会</t>
         </is>
       </c>
       <c r="D134" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F134" t="n">
@@ -14608,12 +14646,12 @@
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>星降る夜の約束</t>
+          <t>虹色Passions！</t>
         </is>
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>花耶</t>
+          <t>虹ヶ咲学園スクールアイドル同好会</t>
         </is>
       </c>
       <c r="I134" t="inlineStr"/>
@@ -14635,15 +14673,15 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>令和のダラさん</t>
+          <t>ラブライブ！虹ヶ咲学園スクールアイドル同好会</t>
         </is>
       </c>
       <c r="D135" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F135" t="n">
@@ -14651,12 +14689,12 @@
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>ダラダラ♡ダンシング</t>
+          <t>NEO SKY, NEO MAP!</t>
         </is>
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>ダラさん（CV：田村睦心） 三⼗⽊⾕⽇向（CV：津田美波） 三⼗⽊⾕薫（CV：寺澤百花） ナレーション（CV：てらそままさき）</t>
+          <t>虹ヶ咲学園スクールアイドル同好会</t>
         </is>
       </c>
       <c r="I135" t="inlineStr"/>
@@ -14678,7 +14716,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>令和のダラさん</t>
+          <t>領民0人スタートの辺境領主様</t>
         </is>
       </c>
       <c r="D136" t="b">
@@ -14686,7 +14724,7 @@
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F136" t="n">
@@ -14694,12 +14732,12 @@
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>ひなたぼっこ</t>
+          <t>Wonder</t>
         </is>
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>REIRIE</t>
+          <t>CROWN HEAD</t>
         </is>
       </c>
       <c r="I136" t="inlineStr"/>
@@ -14721,7 +14759,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>LV999の村人</t>
+          <t>領民0人スタートの辺境領主様</t>
         </is>
       </c>
       <c r="D137" t="b">
@@ -14729,7 +14767,7 @@
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F137" t="n">
@@ -14737,35 +14775,21 @@
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>Not a Hero</t>
+          <t>星降る夜の約束</t>
         </is>
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>藍月なくる&amp;棗いつき</t>
-        </is>
-      </c>
-      <c r="I137" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=9-RVzXLF53U</t>
-        </is>
-      </c>
-      <c r="J137" t="n">
-        <v>78910</v>
-      </c>
-      <c r="K137" t="inlineStr">
-        <is>
-          <t>Itsuki Natsume / 棗いつき</t>
-        </is>
-      </c>
+          <t>花耶</t>
+        </is>
+      </c>
+      <c r="I137" t="inlineStr"/>
+      <c r="J137" t="inlineStr"/>
+      <c r="K137" t="inlineStr"/>
       <c r="L137" t="inlineStr"/>
       <c r="M137" t="inlineStr"/>
       <c r="N137" t="inlineStr"/>
-      <c r="O137" t="inlineStr">
-        <is>
-          <t>2026-06-21T18:35:08</t>
-        </is>
-      </c>
+      <c r="O137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="n">
@@ -14778,7 +14802,7 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>LV999の村人</t>
+          <t>令和のダラさん</t>
         </is>
       </c>
       <c r="D138" t="b">
@@ -14786,7 +14810,7 @@
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F138" t="n">
@@ -14794,12 +14818,12 @@
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>ダラダラ♡ダンシング</t>
         </is>
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>ゆきむら。</t>
+          <t>ダラさん（CV：田村睦心） 三⼗⽊⾕⽇向（CV：津田美波） 三⼗⽊⾕薫（CV：寺澤百花） ナレーション（CV：てらそままさき）</t>
         </is>
       </c>
       <c r="I138" t="inlineStr"/>
@@ -14821,7 +14845,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>ワールド イズ ダンシング</t>
+          <t>令和のダラさん</t>
         </is>
       </c>
       <c r="D139" t="b">
@@ -14829,7 +14853,7 @@
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F139" t="n">
@@ -14837,45 +14861,21 @@
       </c>
       <c r="G139" t="inlineStr">
         <is>
-          <t>終宵</t>
+          <t>ひなたぼっこ</t>
         </is>
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>マカロニえんぴつ</t>
-        </is>
-      </c>
-      <c r="I139" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=Zu45LJG7Chs</t>
-        </is>
-      </c>
-      <c r="J139" t="n">
-        <v>262519</v>
-      </c>
-      <c r="K139" t="inlineStr">
-        <is>
-          <t>SHOCHIKU anime Channel</t>
-        </is>
-      </c>
-      <c r="L139" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=Zu45LJG7Chs</t>
-        </is>
-      </c>
-      <c r="M139" t="n">
-        <v>262519</v>
-      </c>
-      <c r="N139" t="inlineStr">
-        <is>
-          <t>SHOCHIKU anime Channel</t>
-        </is>
-      </c>
-      <c r="O139" t="inlineStr">
-        <is>
-          <t>2026-06-21T18:35:26</t>
-        </is>
-      </c>
+          <t>REIRIE</t>
+        </is>
+      </c>
+      <c r="I139" t="inlineStr"/>
+      <c r="J139" t="inlineStr"/>
+      <c r="K139" t="inlineStr"/>
+      <c r="L139" t="inlineStr"/>
+      <c r="M139" t="inlineStr"/>
+      <c r="N139" t="inlineStr"/>
+      <c r="O139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="n">
@@ -14888,7 +14888,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>ONE PIECE HEROINES</t>
+          <t>LV999の村人</t>
         </is>
       </c>
       <c r="D140" t="b">
@@ -14896,7 +14896,7 @@
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>主題歌</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F140" t="n">
@@ -14904,58 +14904,48 @@
       </c>
       <c r="G140" t="inlineStr">
         <is>
-          <t>ONE PIECE（モノクロ版）</t>
+          <t>Not a Hero</t>
         </is>
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>電子書籍（コミック）</t>
+          <t>藍月なくる&amp;棗いつき</t>
         </is>
       </c>
       <c r="I140" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=6hRjsvdINgg</t>
+          <t>https://www.youtube.com/watch?v=9-RVzXLF53U</t>
         </is>
       </c>
       <c r="J140" t="n">
-        <v>17920416</v>
+        <v>78910</v>
       </c>
       <c r="K140" t="inlineStr">
         <is>
-          <t>ONE PIECE Official YouTube Channel</t>
-        </is>
-      </c>
-      <c r="L140" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=YFbno_aPm0w</t>
-        </is>
-      </c>
-      <c r="M140" t="n">
-        <v>27924515</v>
-      </c>
-      <c r="N140" t="inlineStr">
-        <is>
-          <t>ONE PIECE Official YouTube Channel</t>
-        </is>
-      </c>
+          <t>Itsuki Natsume / 棗いつき</t>
+        </is>
+      </c>
+      <c r="L140" t="inlineStr"/>
+      <c r="M140" t="inlineStr"/>
+      <c r="N140" t="inlineStr"/>
       <c r="O140" t="inlineStr">
         <is>
-          <t>2026-06-21T18:35:55</t>
+          <t>2026-06-21T18:35:08</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="n">
-        <v>5947</v>
+        <v>5806</v>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>2026秋アニメ</t>
+          <t>2026夏アニメ</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>帰還者の魔法は特別です 第2期</t>
+          <t>LV999の村人</t>
         </is>
       </c>
       <c r="D141" t="b">
@@ -14963,7 +14953,7 @@
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F141" t="n">
@@ -14971,12 +14961,12 @@
       </c>
       <c r="G141" t="inlineStr">
         <is>
-          <t>Sorrow</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>FLOW</t>
+          <t>ゆきむら。</t>
         </is>
       </c>
       <c r="I141" t="inlineStr"/>
@@ -14989,16 +14979,16 @@
     </row>
     <row r="142">
       <c r="A142" t="n">
-        <v>5947</v>
+        <v>5806</v>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>2026秋アニメ</t>
+          <t>2026夏アニメ</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>獣王武神ダンデヴァイン</t>
+          <t>ワールド イズ ダンシング</t>
         </is>
       </c>
       <c r="D142" t="b">
@@ -15014,34 +15004,58 @@
       </c>
       <c r="G142" t="inlineStr">
         <is>
-          <t>曲名未発表</t>
+          <t>終宵</t>
         </is>
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>西川貴教</t>
-        </is>
-      </c>
-      <c r="I142" t="inlineStr"/>
-      <c r="J142" t="inlineStr"/>
-      <c r="K142" t="inlineStr"/>
-      <c r="L142" t="inlineStr"/>
-      <c r="M142" t="inlineStr"/>
-      <c r="N142" t="inlineStr"/>
-      <c r="O142" t="inlineStr"/>
+          <t>マカロニえんぴつ</t>
+        </is>
+      </c>
+      <c r="I142" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=Zu45LJG7Chs</t>
+        </is>
+      </c>
+      <c r="J142" t="n">
+        <v>262519</v>
+      </c>
+      <c r="K142" t="inlineStr">
+        <is>
+          <t>SHOCHIKU anime Channel</t>
+        </is>
+      </c>
+      <c r="L142" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=Zu45LJG7Chs</t>
+        </is>
+      </c>
+      <c r="M142" t="n">
+        <v>262519</v>
+      </c>
+      <c r="N142" t="inlineStr">
+        <is>
+          <t>SHOCHIKU anime Channel</t>
+        </is>
+      </c>
+      <c r="O142" t="inlineStr">
+        <is>
+          <t>2026-06-21T18:35:26</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="n">
-        <v>5947</v>
+        <v>5806</v>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>2026秋アニメ</t>
+          <t>2026夏アニメ</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>転生した大聖女は、聖女であることをひた隠す</t>
+          <t>ONE PIECE HEROINES</t>
         </is>
       </c>
       <c r="D143" t="b">
@@ -15049,7 +15063,7 @@
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>主題歌</t>
         </is>
       </c>
       <c r="F143" t="n">
@@ -15057,21 +15071,45 @@
       </c>
       <c r="G143" t="inlineStr">
         <is>
-          <t>Flare of Soul</t>
+          <t>ONE PIECE（モノクロ版）</t>
         </is>
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>花耶</t>
-        </is>
-      </c>
-      <c r="I143" t="inlineStr"/>
-      <c r="J143" t="inlineStr"/>
-      <c r="K143" t="inlineStr"/>
-      <c r="L143" t="inlineStr"/>
-      <c r="M143" t="inlineStr"/>
-      <c r="N143" t="inlineStr"/>
-      <c r="O143" t="inlineStr"/>
+          <t>電子書籍（コミック）</t>
+        </is>
+      </c>
+      <c r="I143" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=6hRjsvdINgg</t>
+        </is>
+      </c>
+      <c r="J143" t="n">
+        <v>17920416</v>
+      </c>
+      <c r="K143" t="inlineStr">
+        <is>
+          <t>ONE PIECE Official YouTube Channel</t>
+        </is>
+      </c>
+      <c r="L143" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=YFbno_aPm0w</t>
+        </is>
+      </c>
+      <c r="M143" t="n">
+        <v>27924515</v>
+      </c>
+      <c r="N143" t="inlineStr">
+        <is>
+          <t>ONE PIECE Official YouTube Channel</t>
+        </is>
+      </c>
+      <c r="O143" t="inlineStr">
+        <is>
+          <t>2026-06-21T18:35:55</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="n">
@@ -15084,7 +15122,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>転生した大聖女は、聖女であることをひた隠す</t>
+          <t>帰還者の魔法は特別です 第2期</t>
         </is>
       </c>
       <c r="D144" t="b">
@@ -15092,7 +15130,7 @@
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F144" t="n">
@@ -15100,12 +15138,12 @@
       </c>
       <c r="G144" t="inlineStr">
         <is>
-          <t>STELLAR</t>
+          <t>Sorrow</t>
         </is>
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>ウタヒメドリーム オールスターズ</t>
+          <t>FLOW</t>
         </is>
       </c>
       <c r="I144" t="inlineStr"/>
@@ -15127,7 +15165,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>魔法少女育成計画restart</t>
+          <t>獣王武神ダンデヴァイン</t>
         </is>
       </c>
       <c r="D145" t="b">
@@ -15143,35 +15181,21 @@
       </c>
       <c r="G145" t="inlineStr">
         <is>
-          <t>No tears here</t>
+          <t>曲名未発表</t>
         </is>
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>茅原実里</t>
-        </is>
-      </c>
-      <c r="I145" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=-PX7FqZ55tE</t>
-        </is>
-      </c>
-      <c r="J145" t="n">
-        <v>105042</v>
-      </c>
-      <c r="K145" t="inlineStr">
-        <is>
-          <t>TVアニメ「魔法少女育成計画restart」公式チャンネル</t>
-        </is>
-      </c>
+          <t>西川貴教</t>
+        </is>
+      </c>
+      <c r="I145" t="inlineStr"/>
+      <c r="J145" t="inlineStr"/>
+      <c r="K145" t="inlineStr"/>
       <c r="L145" t="inlineStr"/>
       <c r="M145" t="inlineStr"/>
       <c r="N145" t="inlineStr"/>
-      <c r="O145" t="inlineStr">
-        <is>
-          <t>2026-06-21T18:36:51</t>
-        </is>
-      </c>
+      <c r="O145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="n">
@@ -15184,7 +15208,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>魔法の姉妹ルルットリリィ 第2クール</t>
+          <t>転生した大聖女は、聖女であることをひた隠す</t>
         </is>
       </c>
       <c r="D146" t="b">
@@ -15200,45 +15224,21 @@
       </c>
       <c r="G146" t="inlineStr">
         <is>
-          <t>Bubee</t>
+          <t>Flare of Soul</t>
         </is>
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>ILLIT</t>
-        </is>
-      </c>
-      <c r="I146" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=sNIntrw0m-g</t>
-        </is>
-      </c>
-      <c r="J146" t="n">
-        <v>66633</v>
-      </c>
-      <c r="K146" t="inlineStr">
-        <is>
-          <t>Bandai Namco Filmworks Channel</t>
-        </is>
-      </c>
-      <c r="L146" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=sNIntrw0m-g</t>
-        </is>
-      </c>
-      <c r="M146" t="n">
-        <v>66633</v>
-      </c>
-      <c r="N146" t="inlineStr">
-        <is>
-          <t>Bandai Namco Filmworks Channel</t>
-        </is>
-      </c>
-      <c r="O146" t="inlineStr">
-        <is>
-          <t>2026-06-24T09:09:26</t>
-        </is>
-      </c>
+          <t>花耶</t>
+        </is>
+      </c>
+      <c r="I146" t="inlineStr"/>
+      <c r="J146" t="inlineStr"/>
+      <c r="K146" t="inlineStr"/>
+      <c r="L146" t="inlineStr"/>
+      <c r="M146" t="inlineStr"/>
+      <c r="N146" t="inlineStr"/>
+      <c r="O146" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" t="n">
@@ -15251,7 +15251,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>魔法の姉妹ルルットリリィ 第2クール</t>
+          <t>転生した大聖女は、聖女であることをひた隠す</t>
         </is>
       </c>
       <c r="D147" t="b">
@@ -15267,41 +15267,208 @@
       </c>
       <c r="G147" t="inlineStr">
         <is>
+          <t>STELLAR</t>
+        </is>
+      </c>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>ウタヒメドリーム オールスターズ</t>
+        </is>
+      </c>
+      <c r="I147" t="inlineStr"/>
+      <c r="J147" t="inlineStr"/>
+      <c r="K147" t="inlineStr"/>
+      <c r="L147" t="inlineStr"/>
+      <c r="M147" t="inlineStr"/>
+      <c r="N147" t="inlineStr"/>
+      <c r="O147" t="inlineStr"/>
+    </row>
+    <row r="148">
+      <c r="A148" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>魔法少女育成計画restart</t>
+        </is>
+      </c>
+      <c r="D148" t="b">
+        <v>0</v>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="F148" t="n">
+        <v>1</v>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>No tears here</t>
+        </is>
+      </c>
+      <c r="H148" t="inlineStr">
+        <is>
+          <t>茅原実里</t>
+        </is>
+      </c>
+      <c r="I148" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=-PX7FqZ55tE</t>
+        </is>
+      </c>
+      <c r="J148" t="n">
+        <v>105042</v>
+      </c>
+      <c r="K148" t="inlineStr">
+        <is>
+          <t>TVアニメ「魔法少女育成計画restart」公式チャンネル</t>
+        </is>
+      </c>
+      <c r="L148" t="inlineStr"/>
+      <c r="M148" t="inlineStr"/>
+      <c r="N148" t="inlineStr"/>
+      <c r="O148" t="inlineStr">
+        <is>
+          <t>2026-06-21T18:36:51</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>魔法の姉妹ルルットリリィ 第2クール</t>
+        </is>
+      </c>
+      <c r="D149" t="b">
+        <v>0</v>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="F149" t="n">
+        <v>1</v>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>Bubee</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>ILLIT</t>
+        </is>
+      </c>
+      <c r="I149" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=sNIntrw0m-g</t>
+        </is>
+      </c>
+      <c r="J149" t="n">
+        <v>66633</v>
+      </c>
+      <c r="K149" t="inlineStr">
+        <is>
+          <t>Bandai Namco Filmworks Channel</t>
+        </is>
+      </c>
+      <c r="L149" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=sNIntrw0m-g</t>
+        </is>
+      </c>
+      <c r="M149" t="n">
+        <v>66633</v>
+      </c>
+      <c r="N149" t="inlineStr">
+        <is>
+          <t>Bandai Namco Filmworks Channel</t>
+        </is>
+      </c>
+      <c r="O149" t="inlineStr">
+        <is>
+          <t>2026-06-24T09:09:26</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>魔法の姉妹ルルットリリィ 第2クール</t>
+        </is>
+      </c>
+      <c r="D150" t="b">
+        <v>0</v>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>ED</t>
+        </is>
+      </c>
+      <c r="F150" t="n">
+        <v>1</v>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
           <t>Calling</t>
         </is>
       </c>
-      <c r="H147" t="inlineStr">
+      <c r="H150" t="inlineStr">
         <is>
           <t>ルルットリリィ（こんぺとリリィ（CV.橘めい）、ましゅールル（CV.小鹿なお））</t>
         </is>
       </c>
-      <c r="I147" t="inlineStr">
+      <c r="I150" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=7oNuxIfJqiI</t>
         </is>
       </c>
-      <c r="J147" t="n">
+      <c r="J150" t="n">
         <v>195116</v>
       </c>
-      <c r="K147" t="inlineStr">
+      <c r="K150" t="inlineStr">
         <is>
           <t>Bandai Namco Filmworks Channel</t>
         </is>
       </c>
-      <c r="L147" t="inlineStr">
+      <c r="L150" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=7oNuxIfJqiI</t>
         </is>
       </c>
-      <c r="M147" t="n">
+      <c r="M150" t="n">
         <v>195116</v>
       </c>
-      <c r="N147" t="inlineStr">
+      <c r="N150" t="inlineStr">
         <is>
           <t>Bandai Namco Filmworks Channel</t>
         </is>
       </c>
-      <c r="O147" t="inlineStr">
+      <c r="O150" t="inlineStr">
         <is>
           <t>2026-06-24T09:09:35</t>
         </is>

</xml_diff>

<commit_message>
auto: anime list update (PC) 2026-06-29
</commit_message>
<xml_diff>
--- a/data/anime_list.xlsx
+++ b/data/anime_list.xlsx
@@ -7946,29 +7946,19 @@
         </is>
       </c>
       <c r="J2" t="n">
-        <v>52344</v>
+        <v>53914</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
           <t>アズールレーン</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=bFCBwBCTCBU</t>
-        </is>
-      </c>
-      <c r="M2" t="n">
-        <v>26101</v>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>SHOCHIKU anime Channel</t>
-        </is>
-      </c>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
       <c r="O2" t="inlineStr">
         <is>
-          <t>2026-06-21T18:13:31</t>
+          <t>2026-06-29T09:00:17</t>
         </is>
       </c>
     </row>
@@ -8285,7 +8275,7 @@
         </is>
       </c>
       <c r="J9" t="n">
-        <v>22060</v>
+        <v>24042</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
@@ -8298,7 +8288,7 @@
         </is>
       </c>
       <c r="M9" t="n">
-        <v>22060</v>
+        <v>24042</v>
       </c>
       <c r="N9" t="inlineStr">
         <is>
@@ -8307,7 +8297,7 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>2026-06-21T18:14:06</t>
+          <t>2026-06-29T09:00:48</t>
         </is>
       </c>
     </row>
@@ -8352,7 +8342,7 @@
         </is>
       </c>
       <c r="J10" t="n">
-        <v>20903</v>
+        <v>22520</v>
       </c>
       <c r="K10" t="inlineStr">
         <is>
@@ -8365,7 +8355,7 @@
         </is>
       </c>
       <c r="M10" t="n">
-        <v>20903</v>
+        <v>22520</v>
       </c>
       <c r="N10" t="inlineStr">
         <is>
@@ -8374,7 +8364,7 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>2026-06-21T18:14:12</t>
+          <t>2026-06-29T09:00:53</t>
         </is>
       </c>
     </row>
@@ -8415,11 +8405,11 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=8So8zgJAYMI</t>
+          <t>https://www.youtube.com/watch?v=X_knFby9AJc</t>
         </is>
       </c>
       <c r="J11" t="n">
-        <v>6811</v>
+        <v>35315</v>
       </c>
       <c r="K11" t="inlineStr">
         <is>
@@ -8428,11 +8418,11 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=8So8zgJAYMI</t>
+          <t>https://www.youtube.com/watch?v=X_knFby9AJc</t>
         </is>
       </c>
       <c r="M11" t="n">
-        <v>6811</v>
+        <v>35315</v>
       </c>
       <c r="N11" t="inlineStr">
         <is>
@@ -8441,7 +8431,7 @@
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>2026-06-21T18:14:24</t>
+          <t>2026-06-29T09:01:02</t>
         </is>
       </c>
     </row>
@@ -8480,37 +8470,13 @@
           <t>汐れいら</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=6fUdDUk-FZQ</t>
-        </is>
-      </c>
-      <c r="J12" t="n">
-        <v>3487</v>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>アニプレックス チャンネル</t>
-        </is>
-      </c>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=6fUdDUk-FZQ</t>
-        </is>
-      </c>
-      <c r="M12" t="n">
-        <v>3487</v>
-      </c>
-      <c r="N12" t="inlineStr">
-        <is>
-          <t>アニプレックス チャンネル</t>
-        </is>
-      </c>
-      <c r="O12" t="inlineStr">
-        <is>
-          <t>2026-06-21T18:14:33</t>
-        </is>
-      </c>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -8940,7 +8906,7 @@
         </is>
       </c>
       <c r="J22" t="n">
-        <v>362547</v>
+        <v>365426</v>
       </c>
       <c r="K22" t="inlineStr">
         <is>
@@ -8952,7 +8918,7 @@
       <c r="N22" t="inlineStr"/>
       <c r="O22" t="inlineStr">
         <is>
-          <t>2026-06-21T18:16:17</t>
+          <t>2026-06-29T09:02:33</t>
         </is>
       </c>
     </row>
@@ -8991,13 +8957,37 @@
           <t>ユニコーン</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
-      <c r="L23" t="inlineStr"/>
-      <c r="M23" t="inlineStr"/>
-      <c r="N23" t="inlineStr"/>
-      <c r="O23" t="inlineStr"/>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=7BDs9fUOFu8</t>
+        </is>
+      </c>
+      <c r="J23" t="n">
+        <v>9248</v>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>NBCUniversal Anime/Music</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=7BDs9fUOFu8</t>
+        </is>
+      </c>
+      <c r="M23" t="n">
+        <v>9248</v>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>NBCUniversal Anime/Music</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>2026-06-29T09:02:42</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -9034,13 +9024,37 @@
           <t>BLUE ENCOUNT</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr"/>
-      <c r="L24" t="inlineStr"/>
-      <c r="M24" t="inlineStr"/>
-      <c r="N24" t="inlineStr"/>
-      <c r="O24" t="inlineStr"/>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=1Q1Kgixu70g</t>
+        </is>
+      </c>
+      <c r="J24" t="n">
+        <v>899</v>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>NBCUniversal Anime/Music</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=1Q1Kgixu70g</t>
+        </is>
+      </c>
+      <c r="M24" t="n">
+        <v>899</v>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>NBCUniversal Anime/Music</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>2026-06-29T09:02:51</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -9083,7 +9097,7 @@
         </is>
       </c>
       <c r="J25" t="n">
-        <v>13154</v>
+        <v>19123</v>
       </c>
       <c r="K25" t="inlineStr">
         <is>
@@ -9095,7 +9109,7 @@
       <c r="N25" t="inlineStr"/>
       <c r="O25" t="inlineStr">
         <is>
-          <t>2026-06-21T18:16:54</t>
+          <t>2026-06-29T09:03:02</t>
         </is>
       </c>
     </row>
@@ -9140,7 +9154,7 @@
         </is>
       </c>
       <c r="J26" t="n">
-        <v>16610711</v>
+        <v>16727541</v>
       </c>
       <c r="K26" t="inlineStr">
         <is>
@@ -9153,7 +9167,7 @@
         </is>
       </c>
       <c r="M26" t="n">
-        <v>223037</v>
+        <v>224181</v>
       </c>
       <c r="N26" t="inlineStr">
         <is>
@@ -9162,7 +9176,7 @@
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>2026-06-21T18:17:17</t>
+          <t>2026-06-29T09:03:21</t>
         </is>
       </c>
     </row>
@@ -9336,7 +9350,7 @@
         </is>
       </c>
       <c r="J30" t="n">
-        <v>1851</v>
+        <v>2093</v>
       </c>
       <c r="K30" t="inlineStr">
         <is>
@@ -9348,7 +9362,7 @@
       <c r="N30" t="inlineStr"/>
       <c r="O30" t="inlineStr">
         <is>
-          <t>2026-06-21T18:17:42</t>
+          <t>2026-06-29T09:03:43</t>
         </is>
       </c>
     </row>
@@ -9522,7 +9536,7 @@
         </is>
       </c>
       <c r="J34" t="n">
-        <v>466412</v>
+        <v>470198</v>
       </c>
       <c r="K34" t="inlineStr">
         <is>
@@ -9535,7 +9549,7 @@
         </is>
       </c>
       <c r="M34" t="n">
-        <v>466412</v>
+        <v>470198</v>
       </c>
       <c r="N34" t="inlineStr">
         <is>
@@ -9544,7 +9558,7 @@
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>2026-06-21T18:18:12</t>
+          <t>2026-06-29T09:04:09</t>
         </is>
       </c>
     </row>
@@ -9675,7 +9689,7 @@
         </is>
       </c>
       <c r="J37" t="n">
-        <v>11744</v>
+        <v>13244</v>
       </c>
       <c r="K37" t="inlineStr">
         <is>
@@ -9688,7 +9702,7 @@
         </is>
       </c>
       <c r="M37" t="n">
-        <v>11744</v>
+        <v>13244</v>
       </c>
       <c r="N37" t="inlineStr">
         <is>
@@ -9697,7 +9711,7 @@
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>2026-06-21T18:18:28</t>
+          <t>2026-06-29T09:04:26</t>
         </is>
       </c>
     </row>
@@ -9742,7 +9756,7 @@
         </is>
       </c>
       <c r="J38" t="n">
-        <v>13489</v>
+        <v>14672</v>
       </c>
       <c r="K38" t="inlineStr">
         <is>
@@ -9755,7 +9769,7 @@
         </is>
       </c>
       <c r="M38" t="n">
-        <v>13489</v>
+        <v>14672</v>
       </c>
       <c r="N38" t="inlineStr">
         <is>
@@ -9764,7 +9778,7 @@
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>2026-06-21T18:18:33</t>
+          <t>2026-06-29T09:04:30</t>
         </is>
       </c>
     </row>
@@ -9805,11 +9819,11 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=fuXZMQAD9vU</t>
+          <t>https://www.youtube.com/watch?v=R3V4sAXUJ-g</t>
         </is>
       </c>
       <c r="J39" t="n">
-        <v>12852008</v>
+        <v>66192472</v>
       </c>
       <c r="K39" t="inlineStr">
         <is>
@@ -9821,7 +9835,7 @@
       <c r="N39" t="inlineStr"/>
       <c r="O39" t="inlineStr">
         <is>
-          <t>2026-06-21T18:19:08</t>
+          <t>2026-06-29T09:04:58</t>
         </is>
       </c>
     </row>
@@ -9866,7 +9880,7 @@
         </is>
       </c>
       <c r="J40" t="n">
-        <v>295392</v>
+        <v>296633</v>
       </c>
       <c r="K40" t="inlineStr">
         <is>
@@ -9878,7 +9892,7 @@
       <c r="N40" t="inlineStr"/>
       <c r="O40" t="inlineStr">
         <is>
-          <t>2026-06-21T18:19:26</t>
+          <t>2026-06-29T09:05:13</t>
         </is>
       </c>
     </row>
@@ -9923,7 +9937,7 @@
         </is>
       </c>
       <c r="J41" t="n">
-        <v>295392</v>
+        <v>296633</v>
       </c>
       <c r="K41" t="inlineStr">
         <is>
@@ -9935,7 +9949,7 @@
       <c r="N41" t="inlineStr"/>
       <c r="O41" t="inlineStr">
         <is>
-          <t>2026-06-21T18:19:43</t>
+          <t>2026-06-29T09:05:27</t>
         </is>
       </c>
     </row>
@@ -10066,7 +10080,7 @@
         </is>
       </c>
       <c r="J44" t="n">
-        <v>6682341</v>
+        <v>6747037</v>
       </c>
       <c r="K44" t="inlineStr">
         <is>
@@ -10078,7 +10092,7 @@
       <c r="N44" t="inlineStr"/>
       <c r="O44" t="inlineStr">
         <is>
-          <t>2026-06-21T18:20:22</t>
+          <t>2026-06-29T09:06:00</t>
         </is>
       </c>
     </row>
@@ -10123,7 +10137,7 @@
         </is>
       </c>
       <c r="J45" t="n">
-        <v>42562</v>
+        <v>53817</v>
       </c>
       <c r="K45" t="inlineStr">
         <is>
@@ -10136,7 +10150,7 @@
         </is>
       </c>
       <c r="M45" t="n">
-        <v>145</v>
+        <v>162</v>
       </c>
       <c r="N45" t="inlineStr">
         <is>
@@ -10145,7 +10159,7 @@
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>2026-06-21T18:20:33</t>
+          <t>2026-06-29T09:06:09</t>
         </is>
       </c>
     </row>
@@ -10319,7 +10333,7 @@
         </is>
       </c>
       <c r="J49" t="n">
-        <v>4032</v>
+        <v>4309</v>
       </c>
       <c r="K49" t="inlineStr">
         <is>
@@ -10331,7 +10345,7 @@
       <c r="N49" t="inlineStr"/>
       <c r="O49" t="inlineStr">
         <is>
-          <t>2026-06-21T18:21:04</t>
+          <t>2026-06-29T09:06:39</t>
         </is>
       </c>
     </row>
@@ -10376,7 +10390,7 @@
         </is>
       </c>
       <c r="J50" t="n">
-        <v>13236</v>
+        <v>19444</v>
       </c>
       <c r="K50" t="inlineStr">
         <is>
@@ -10388,7 +10402,7 @@
       <c r="N50" t="inlineStr"/>
       <c r="O50" t="inlineStr">
         <is>
-          <t>2026-06-21T18:21:26</t>
+          <t>2026-06-29T09:06:57</t>
         </is>
       </c>
     </row>
@@ -10476,7 +10490,7 @@
         </is>
       </c>
       <c r="J52" t="n">
-        <v>305568</v>
+        <v>310640</v>
       </c>
       <c r="K52" t="inlineStr">
         <is>
@@ -10489,7 +10503,7 @@
         </is>
       </c>
       <c r="M52" t="n">
-        <v>305568</v>
+        <v>310640</v>
       </c>
       <c r="N52" t="inlineStr">
         <is>
@@ -10498,7 +10512,7 @@
       </c>
       <c r="O52" t="inlineStr">
         <is>
-          <t>2026-06-21T18:21:38</t>
+          <t>2026-06-29T09:07:13</t>
         </is>
       </c>
     </row>
@@ -10629,7 +10643,7 @@
         </is>
       </c>
       <c r="J55" t="n">
-        <v>6309471</v>
+        <v>6358421</v>
       </c>
       <c r="K55" t="inlineStr">
         <is>
@@ -10642,7 +10656,7 @@
         </is>
       </c>
       <c r="M55" t="n">
-        <v>594902</v>
+        <v>631848</v>
       </c>
       <c r="N55" t="inlineStr">
         <is>
@@ -10651,7 +10665,7 @@
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>2026-06-21T18:21:56</t>
+          <t>2026-06-29T09:07:37</t>
         </is>
       </c>
     </row>
@@ -10696,7 +10710,7 @@
         </is>
       </c>
       <c r="J56" t="n">
-        <v>867945</v>
+        <v>993597</v>
       </c>
       <c r="K56" t="inlineStr">
         <is>
@@ -10709,7 +10723,7 @@
         </is>
       </c>
       <c r="M56" t="n">
-        <v>867945</v>
+        <v>993597</v>
       </c>
       <c r="N56" t="inlineStr">
         <is>
@@ -10718,7 +10732,7 @@
       </c>
       <c r="O56" t="inlineStr">
         <is>
-          <t>2026-06-21T18:22:09</t>
+          <t>2026-06-29T09:07:46</t>
         </is>
       </c>
     </row>
@@ -10935,7 +10949,7 @@
         </is>
       </c>
       <c r="J61" t="n">
-        <v>3803168</v>
+        <v>3923215</v>
       </c>
       <c r="K61" t="inlineStr">
         <is>
@@ -10948,7 +10962,7 @@
         </is>
       </c>
       <c r="M61" t="n">
-        <v>1711081</v>
+        <v>1763982</v>
       </c>
       <c r="N61" t="inlineStr">
         <is>
@@ -10957,7 +10971,7 @@
       </c>
       <c r="O61" t="inlineStr">
         <is>
-          <t>2026-06-21T18:22:34</t>
+          <t>2026-06-29T09:08:11</t>
         </is>
       </c>
     </row>
@@ -11002,7 +11016,7 @@
         </is>
       </c>
       <c r="J62" t="n">
-        <v>1711081</v>
+        <v>1763982</v>
       </c>
       <c r="K62" t="inlineStr">
         <is>
@@ -11015,7 +11029,7 @@
         </is>
       </c>
       <c r="M62" t="n">
-        <v>1711081</v>
+        <v>1763982</v>
       </c>
       <c r="N62" t="inlineStr">
         <is>
@@ -11024,7 +11038,7 @@
       </c>
       <c r="O62" t="inlineStr">
         <is>
-          <t>2026-06-21T18:22:43</t>
+          <t>2026-06-29T09:08:20</t>
         </is>
       </c>
     </row>
@@ -11069,7 +11083,7 @@
         </is>
       </c>
       <c r="J63" t="n">
-        <v>273328</v>
+        <v>278831</v>
       </c>
       <c r="K63" t="inlineStr">
         <is>
@@ -11082,7 +11096,7 @@
         </is>
       </c>
       <c r="M63" t="n">
-        <v>273328</v>
+        <v>278831</v>
       </c>
       <c r="N63" t="inlineStr">
         <is>
@@ -11091,7 +11105,7 @@
       </c>
       <c r="O63" t="inlineStr">
         <is>
-          <t>2026-06-21T18:22:55</t>
+          <t>2026-06-29T09:08:30</t>
         </is>
       </c>
     </row>
@@ -11566,7 +11580,7 @@
         </is>
       </c>
       <c r="J74" t="n">
-        <v>140125</v>
+        <v>154655</v>
       </c>
       <c r="K74" t="inlineStr">
         <is>
@@ -11579,7 +11593,7 @@
         </is>
       </c>
       <c r="M74" t="n">
-        <v>140125</v>
+        <v>154655</v>
       </c>
       <c r="N74" t="inlineStr">
         <is>
@@ -11588,7 +11602,7 @@
       </c>
       <c r="O74" t="inlineStr">
         <is>
-          <t>2026-06-21T18:23:55</t>
+          <t>2026-06-29T09:09:43</t>
         </is>
       </c>
     </row>
@@ -11733,7 +11747,7 @@
         </is>
       </c>
       <c r="J77" t="n">
-        <v>69452</v>
+        <v>152288</v>
       </c>
       <c r="K77" t="inlineStr">
         <is>
@@ -11745,7 +11759,7 @@
       <c r="N77" t="inlineStr"/>
       <c r="O77" t="inlineStr">
         <is>
-          <t>2026-06-21T18:24:32</t>
+          <t>2026-06-29T09:10:19</t>
         </is>
       </c>
     </row>
@@ -12139,7 +12153,7 @@
         </is>
       </c>
       <c r="J85" t="n">
-        <v>3207</v>
+        <v>3926</v>
       </c>
       <c r="K85" t="inlineStr">
         <is>
@@ -12152,7 +12166,7 @@
         </is>
       </c>
       <c r="M85" t="n">
-        <v>3207</v>
+        <v>3926</v>
       </c>
       <c r="N85" t="inlineStr">
         <is>
@@ -12161,7 +12175,7 @@
       </c>
       <c r="O85" t="inlineStr">
         <is>
-          <t>2026-06-21T18:26:16</t>
+          <t>2026-06-29T09:11:03</t>
         </is>
       </c>
     </row>
@@ -12349,7 +12363,7 @@
         </is>
       </c>
       <c r="J89" t="n">
-        <v>402991</v>
+        <v>415759</v>
       </c>
       <c r="K89" t="inlineStr">
         <is>
@@ -12362,7 +12376,7 @@
         </is>
       </c>
       <c r="M89" t="n">
-        <v>402991</v>
+        <v>415759</v>
       </c>
       <c r="N89" t="inlineStr">
         <is>
@@ -12371,7 +12385,7 @@
       </c>
       <c r="O89" t="inlineStr">
         <is>
-          <t>2026-06-21T18:26:31</t>
+          <t>2026-06-29T09:11:24</t>
         </is>
       </c>
     </row>
@@ -12416,7 +12430,7 @@
         </is>
       </c>
       <c r="J90" t="n">
-        <v>174316</v>
+        <v>256550</v>
       </c>
       <c r="K90" t="inlineStr">
         <is>
@@ -12429,7 +12443,7 @@
         </is>
       </c>
       <c r="M90" t="n">
-        <v>174316</v>
+        <v>256550</v>
       </c>
       <c r="N90" t="inlineStr">
         <is>
@@ -12438,7 +12452,7 @@
       </c>
       <c r="O90" t="inlineStr">
         <is>
-          <t>2026-06-21T18:26:42</t>
+          <t>2026-06-29T09:11:33</t>
         </is>
       </c>
     </row>
@@ -12479,33 +12493,33 @@
       </c>
       <c r="I91" t="inlineStr">
         <is>
+          <t>https://www.youtube.com/watch?v=FhZYDK_IPYg</t>
+        </is>
+      </c>
+      <c r="J91" t="n">
+        <v>323173</v>
+      </c>
+      <c r="K91" t="inlineStr">
+        <is>
+          <t>Novel Core Official</t>
+        </is>
+      </c>
+      <c r="L91" t="inlineStr">
+        <is>
           <t>https://www.youtube.com/watch?v=KKOr3xF2iOM</t>
         </is>
       </c>
-      <c r="J91" t="n">
-        <v>294329</v>
-      </c>
-      <c r="K91" t="inlineStr">
+      <c r="M91" t="n">
+        <v>305984</v>
+      </c>
+      <c r="N91" t="inlineStr">
         <is>
           <t>TMSアニメ公式チャンネル</t>
         </is>
       </c>
-      <c r="L91" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=KKOr3xF2iOM</t>
-        </is>
-      </c>
-      <c r="M91" t="n">
-        <v>294329</v>
-      </c>
-      <c r="N91" t="inlineStr">
-        <is>
-          <t>TMSアニメ公式チャンネル</t>
-        </is>
-      </c>
       <c r="O91" t="inlineStr">
         <is>
-          <t>2026-06-21T18:26:53</t>
+          <t>2026-06-29T09:11:42</t>
         </is>
       </c>
     </row>
@@ -12550,7 +12564,7 @@
         </is>
       </c>
       <c r="J92" t="n">
-        <v>25824</v>
+        <v>42531</v>
       </c>
       <c r="K92" t="inlineStr">
         <is>
@@ -12563,7 +12577,7 @@
         </is>
       </c>
       <c r="M92" t="n">
-        <v>25824</v>
+        <v>42531</v>
       </c>
       <c r="N92" t="inlineStr">
         <is>
@@ -12572,7 +12586,7 @@
       </c>
       <c r="O92" t="inlineStr">
         <is>
-          <t>2026-06-21T18:27:05</t>
+          <t>2026-06-29T09:11:52</t>
         </is>
       </c>
     </row>
@@ -12970,7 +12984,7 @@
         </is>
       </c>
       <c r="J100" t="n">
-        <v>11323</v>
+        <v>17064</v>
       </c>
       <c r="K100" t="inlineStr">
         <is>
@@ -12982,7 +12996,7 @@
       <c r="N100" t="inlineStr"/>
       <c r="O100" t="inlineStr">
         <is>
-          <t>2026-06-21T18:27:45</t>
+          <t>2026-06-29T09:12:27</t>
         </is>
       </c>
     </row>
@@ -13027,7 +13041,7 @@
         </is>
       </c>
       <c r="J101" t="n">
-        <v>4603</v>
+        <v>5332</v>
       </c>
       <c r="K101" t="inlineStr">
         <is>
@@ -13039,7 +13053,7 @@
       <c r="N101" t="inlineStr"/>
       <c r="O101" t="inlineStr">
         <is>
-          <t>2026-06-21T18:27:58</t>
+          <t>2026-06-29T09:12:38</t>
         </is>
       </c>
     </row>
@@ -13084,7 +13098,7 @@
         </is>
       </c>
       <c r="J102" t="n">
-        <v>451401</v>
+        <v>561951</v>
       </c>
       <c r="K102" t="inlineStr">
         <is>
@@ -13096,7 +13110,7 @@
       <c r="N102" t="inlineStr"/>
       <c r="O102" t="inlineStr">
         <is>
-          <t>2026-06-21T18:28:12</t>
+          <t>2026-06-29T09:12:50</t>
         </is>
       </c>
     </row>
@@ -13724,7 +13738,7 @@
         </is>
       </c>
       <c r="J116" t="n">
-        <v>590624</v>
+        <v>604011</v>
       </c>
       <c r="K116" t="inlineStr">
         <is>
@@ -13736,7 +13750,7 @@
       <c r="N116" t="inlineStr"/>
       <c r="O116" t="inlineStr">
         <is>
-          <t>2026-06-21T18:29:37</t>
+          <t>2026-06-29T09:14:07</t>
         </is>
       </c>
     </row>
@@ -13781,7 +13795,7 @@
         </is>
       </c>
       <c r="J117" t="n">
-        <v>590624</v>
+        <v>604011</v>
       </c>
       <c r="K117" t="inlineStr">
         <is>
@@ -13793,7 +13807,7 @@
       <c r="N117" t="inlineStr"/>
       <c r="O117" t="inlineStr">
         <is>
-          <t>2026-06-21T18:29:56</t>
+          <t>2026-06-29T09:14:25</t>
         </is>
       </c>
     </row>
@@ -13967,7 +13981,7 @@
         </is>
       </c>
       <c r="J121" t="n">
-        <v>12105753</v>
+        <v>12139251</v>
       </c>
       <c r="K121" t="inlineStr">
         <is>
@@ -13976,11 +13990,11 @@
       </c>
       <c r="L121" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=PINgF6rCuME</t>
+          <t>https://www.youtube.com/watch?v=3mLWoJF17U4</t>
         </is>
       </c>
       <c r="M121" t="n">
-        <v>2457533</v>
+        <v>2141307</v>
       </c>
       <c r="N121" t="inlineStr">
         <is>
@@ -13989,7 +14003,7 @@
       </c>
       <c r="O121" t="inlineStr">
         <is>
-          <t>2026-06-21T18:30:35</t>
+          <t>2026-06-29T09:14:54</t>
         </is>
       </c>
     </row>
@@ -14034,7 +14048,7 @@
         </is>
       </c>
       <c r="J122" t="n">
-        <v>1140774</v>
+        <v>1221650</v>
       </c>
       <c r="K122" t="inlineStr">
         <is>
@@ -14046,7 +14060,7 @@
       <c r="N122" t="inlineStr"/>
       <c r="O122" t="inlineStr">
         <is>
-          <t>2026-06-21T18:31:08</t>
+          <t>2026-06-29T09:15:22</t>
         </is>
       </c>
     </row>
@@ -14091,7 +14105,7 @@
         </is>
       </c>
       <c r="J123" t="n">
-        <v>32222</v>
+        <v>35365</v>
       </c>
       <c r="K123" t="inlineStr">
         <is>
@@ -14100,20 +14114,20 @@
       </c>
       <c r="L123" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=5QGZX_Kky4I</t>
+          <t>https://www.youtube.com/watch?v=Q1UXK9Pwbtk</t>
         </is>
       </c>
       <c r="M123" t="n">
-        <v>27576</v>
+        <v>32188</v>
       </c>
       <c r="N123" t="inlineStr">
         <is>
-          <t>leafstamp</t>
+          <t>アニメ映画予告編アーカイブ</t>
         </is>
       </c>
       <c r="O123" t="inlineStr">
         <is>
-          <t>2026-06-21T18:31:32</t>
+          <t>2026-06-29T09:15:41</t>
         </is>
       </c>
     </row>
@@ -14201,7 +14215,7 @@
         </is>
       </c>
       <c r="J125" t="n">
-        <v>480871</v>
+        <v>553776</v>
       </c>
       <c r="K125" t="inlineStr">
         <is>
@@ -14213,7 +14227,7 @@
       <c r="N125" t="inlineStr"/>
       <c r="O125" t="inlineStr">
         <is>
-          <t>2026-06-21T18:32:14</t>
+          <t>2026-06-29T09:16:16</t>
         </is>
       </c>
     </row>
@@ -14258,7 +14272,7 @@
         </is>
       </c>
       <c r="J126" t="n">
-        <v>480871</v>
+        <v>553776</v>
       </c>
       <c r="K126" t="inlineStr">
         <is>
@@ -14270,7 +14284,7 @@
       <c r="N126" t="inlineStr"/>
       <c r="O126" t="inlineStr">
         <is>
-          <t>2026-06-21T18:32:32</t>
+          <t>2026-06-29T09:16:34</t>
         </is>
       </c>
     </row>
@@ -14358,7 +14372,7 @@
         </is>
       </c>
       <c r="J128" t="n">
-        <v>50838</v>
+        <v>54413</v>
       </c>
       <c r="K128" t="inlineStr">
         <is>
@@ -14370,7 +14384,7 @@
       <c r="N128" t="inlineStr"/>
       <c r="O128" t="inlineStr">
         <is>
-          <t>2026-06-21T18:33:01</t>
+          <t>2026-06-29T09:16:59</t>
         </is>
       </c>
     </row>
@@ -14458,7 +14472,7 @@
         </is>
       </c>
       <c r="J130" t="n">
-        <v>603666</v>
+        <v>605707</v>
       </c>
       <c r="K130" t="inlineStr">
         <is>
@@ -14471,7 +14485,7 @@
         </is>
       </c>
       <c r="M130" t="n">
-        <v>603666</v>
+        <v>605707</v>
       </c>
       <c r="N130" t="inlineStr">
         <is>
@@ -14480,7 +14494,7 @@
       </c>
       <c r="O130" t="inlineStr">
         <is>
-          <t>2026-06-21T18:33:22</t>
+          <t>2026-06-29T09:17:16</t>
         </is>
       </c>
     </row>
@@ -14521,11 +14535,11 @@
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=OKEoQo3cGVg</t>
+          <t>https://www.youtube.com/watch?v=QbQyWTgxy-c</t>
         </is>
       </c>
       <c r="J131" t="n">
-        <v>66350</v>
+        <v>72668</v>
       </c>
       <c r="K131" t="inlineStr">
         <is>
@@ -14537,7 +14551,7 @@
       <c r="N131" t="inlineStr"/>
       <c r="O131" t="inlineStr">
         <is>
-          <t>2026-06-21T18:33:34</t>
+          <t>2026-06-29T09:17:26</t>
         </is>
       </c>
     </row>
@@ -14578,15 +14592,15 @@
       </c>
       <c r="I132" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=aw45Q_mr0_M</t>
+          <t>https://www.youtube.com/watch?v=eP-bP5dET_k</t>
         </is>
       </c>
       <c r="J132" t="n">
-        <v>9441868</v>
+        <v>241550</v>
       </c>
       <c r="K132" t="inlineStr">
         <is>
-          <t>ONE OR EIGHT</t>
+          <t>TVアニメ『鎧真伝サムライトルーパー』公式</t>
         </is>
       </c>
       <c r="L132" t="inlineStr">
@@ -14595,7 +14609,7 @@
         </is>
       </c>
       <c r="M132" t="n">
-        <v>151043</v>
+        <v>152090</v>
       </c>
       <c r="N132" t="inlineStr">
         <is>
@@ -14604,7 +14618,7 @@
       </c>
       <c r="O132" t="inlineStr">
         <is>
-          <t>2026-06-21T18:33:47</t>
+          <t>2026-06-29T09:17:36</t>
         </is>
       </c>
     </row>
@@ -14645,11 +14659,11 @@
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=OKEoQo3cGVg</t>
+          <t>https://www.youtube.com/watch?v=QbQyWTgxy-c</t>
         </is>
       </c>
       <c r="J133" t="n">
-        <v>66350</v>
+        <v>72668</v>
       </c>
       <c r="K133" t="inlineStr">
         <is>
@@ -14661,7 +14675,7 @@
       <c r="N133" t="inlineStr"/>
       <c r="O133" t="inlineStr">
         <is>
-          <t>2026-06-21T18:34:00</t>
+          <t>2026-06-29T09:17:47</t>
         </is>
       </c>
     </row>
@@ -15074,7 +15088,7 @@
         </is>
       </c>
       <c r="J142" t="n">
-        <v>78910</v>
+        <v>98450</v>
       </c>
       <c r="K142" t="inlineStr">
         <is>
@@ -15086,7 +15100,7 @@
       <c r="N142" t="inlineStr"/>
       <c r="O142" t="inlineStr">
         <is>
-          <t>2026-06-21T18:35:08</t>
+          <t>2026-06-29T09:18:37</t>
         </is>
       </c>
     </row>
@@ -15174,7 +15188,7 @@
         </is>
       </c>
       <c r="J144" t="n">
-        <v>262519</v>
+        <v>276043</v>
       </c>
       <c r="K144" t="inlineStr">
         <is>
@@ -15187,7 +15201,7 @@
         </is>
       </c>
       <c r="M144" t="n">
-        <v>262519</v>
+        <v>276043</v>
       </c>
       <c r="N144" t="inlineStr">
         <is>
@@ -15196,7 +15210,7 @@
       </c>
       <c r="O144" t="inlineStr">
         <is>
-          <t>2026-06-21T18:35:26</t>
+          <t>2026-06-29T09:18:56</t>
         </is>
       </c>
     </row>
@@ -15237,11 +15251,11 @@
       </c>
       <c r="I145" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=6hRjsvdINgg</t>
+          <t>https://www.youtube.com/watch?v=z_qWsQNWSVI</t>
         </is>
       </c>
       <c r="J145" t="n">
-        <v>17920416</v>
+        <v>6035898</v>
       </c>
       <c r="K145" t="inlineStr">
         <is>
@@ -15254,7 +15268,7 @@
         </is>
       </c>
       <c r="M145" t="n">
-        <v>27924515</v>
+        <v>28000133</v>
       </c>
       <c r="N145" t="inlineStr">
         <is>
@@ -15263,7 +15277,7 @@
       </c>
       <c r="O145" t="inlineStr">
         <is>
-          <t>2026-06-21T18:35:55</t>
+          <t>2026-06-29T09:19:20</t>
         </is>
       </c>
     </row>
@@ -15480,7 +15494,7 @@
         </is>
       </c>
       <c r="J150" t="n">
-        <v>105042</v>
+        <v>105506</v>
       </c>
       <c r="K150" t="inlineStr">
         <is>
@@ -15492,7 +15506,7 @@
       <c r="N150" t="inlineStr"/>
       <c r="O150" t="inlineStr">
         <is>
-          <t>2026-06-21T18:36:51</t>
+          <t>2026-06-29T09:20:07</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: anime list update (PC) 2026-07-03
</commit_message>
<xml_diff>
--- a/data/anime_list.xlsx
+++ b/data/anime_list.xlsx
@@ -11936,13 +11936,37 @@
           <t>SPYAIR</t>
         </is>
       </c>
-      <c r="I71" t="inlineStr"/>
-      <c r="J71" t="inlineStr"/>
-      <c r="K71" t="inlineStr"/>
-      <c r="L71" t="inlineStr"/>
-      <c r="M71" t="inlineStr"/>
-      <c r="N71" t="inlineStr"/>
-      <c r="O71" t="inlineStr"/>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=_j3Bm3tr7dA</t>
+        </is>
+      </c>
+      <c r="J71" t="n">
+        <v>4513</v>
+      </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>SHOCHIKU anime Channel</t>
+        </is>
+      </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=_j3Bm3tr7dA</t>
+        </is>
+      </c>
+      <c r="M71" t="n">
+        <v>4513</v>
+      </c>
+      <c r="N71" t="inlineStr">
+        <is>
+          <t>SHOCHIKU anime Channel</t>
+        </is>
+      </c>
+      <c r="O71" t="inlineStr">
+        <is>
+          <t>2026-07-03T09:03:44</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -12022,13 +12046,27 @@
           <t>原因は自分にある。</t>
         </is>
       </c>
-      <c r="I73" t="inlineStr"/>
-      <c r="J73" t="inlineStr"/>
-      <c r="K73" t="inlineStr"/>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=Nqel4e1h8YQ</t>
+        </is>
+      </c>
+      <c r="J73" t="n">
+        <v>15417</v>
+      </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>原因は自分にある。Official</t>
+        </is>
+      </c>
       <c r="L73" t="inlineStr"/>
       <c r="M73" t="inlineStr"/>
       <c r="N73" t="inlineStr"/>
-      <c r="O73" t="inlineStr"/>
+      <c r="O73" t="inlineStr">
+        <is>
+          <t>2026-07-03T09:04:04</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -14090,13 +14128,27 @@
           <t>I Don't Like Mondays.</t>
         </is>
       </c>
-      <c r="I111" t="inlineStr"/>
-      <c r="J111" t="inlineStr"/>
-      <c r="K111" t="inlineStr"/>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=r-4zKDCNjwM</t>
+        </is>
+      </c>
+      <c r="J111" t="n">
+        <v>980</v>
+      </c>
+      <c r="K111" t="inlineStr">
+        <is>
+          <t>I Don't Like Mondays.</t>
+        </is>
+      </c>
       <c r="L111" t="inlineStr"/>
       <c r="M111" t="inlineStr"/>
       <c r="N111" t="inlineStr"/>
-      <c r="O111" t="inlineStr"/>
+      <c r="O111" t="inlineStr">
+        <is>
+          <t>2026-07-03T09:05:57</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="n">

</xml_diff>

<commit_message>
auto: anime list update (PC) 2026-07-04
</commit_message>
<xml_diff>
--- a/data/anime_list.xlsx
+++ b/data/anime_list.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M150"/>
+  <dimension ref="A1:M151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5965,7 +5965,7 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>サイバーパンク：エッジランナーズ2</t>
+          <t>氷の城壁 第2期</t>
         </is>
       </c>
       <c r="E101" t="b">
@@ -5973,17 +5973,17 @@
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>配信</t>
+          <t>TVアニメ</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>2026年秋 Netflixにて</t>
+          <t>2026年10月1日（木）～ TBS系28局にて</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>TRIGGER</t>
+          <t>スタジオKAI</t>
         </is>
       </c>
       <c r="I101" t="inlineStr"/>
@@ -5992,7 +5992,7 @@
       <c r="L101" t="inlineStr"/>
       <c r="M101" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28680</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25508</t>
         </is>
       </c>
     </row>
@@ -6010,7 +6010,7 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>PSYREN -サイレン-</t>
+          <t>サイバーパンク：エッジランナーズ2</t>
         </is>
       </c>
       <c r="E102" t="b">
@@ -6018,17 +6018,17 @@
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>TVアニメ</t>
+          <t>配信</t>
         </is>
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>2026年10月～ TOKYO MX・BS11ほか</t>
+          <t>2026年秋 Netflixにて</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>サテライト</t>
+          <t>TRIGGER</t>
         </is>
       </c>
       <c r="I102" t="inlineStr"/>
@@ -6037,7 +6037,7 @@
       <c r="L102" t="inlineStr"/>
       <c r="M102" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27257</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28680</t>
         </is>
       </c>
     </row>
@@ -6055,7 +6055,7 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>佐々木とピーちゃん シーズン２</t>
+          <t>PSYREN -サイレン-</t>
         </is>
       </c>
       <c r="E103" t="b">
@@ -6068,12 +6068,12 @@
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
+          <t>2026年10月～ TOKYO MX・BS11ほか</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>SILVER LINK.</t>
+          <t>サテライト</t>
         </is>
       </c>
       <c r="I103" t="inlineStr"/>
@@ -6082,7 +6082,7 @@
       <c r="L103" t="inlineStr"/>
       <c r="M103" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=23804</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27257</t>
         </is>
       </c>
     </row>
@@ -6100,7 +6100,7 @@
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>塩対応の佐藤さんが俺にだけ甘い</t>
+          <t>佐々木とピーちゃん シーズン２</t>
         </is>
       </c>
       <c r="E104" t="b">
@@ -6116,14 +6116,18 @@
           <t>2026年10月～</t>
         </is>
       </c>
-      <c r="H104" t="inlineStr"/>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>SILVER LINK.</t>
+        </is>
+      </c>
       <c r="I104" t="inlineStr"/>
       <c r="J104" t="inlineStr"/>
       <c r="K104" t="inlineStr"/>
       <c r="L104" t="inlineStr"/>
       <c r="M104" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27964</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=23804</t>
         </is>
       </c>
     </row>
@@ -6141,7 +6145,7 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>ジャンケットバンク</t>
+          <t>塩対応の佐藤さんが俺にだけ甘い</t>
         </is>
       </c>
       <c r="E105" t="b">
@@ -6157,18 +6161,14 @@
           <t>2026年10月～</t>
         </is>
       </c>
-      <c r="H105" t="inlineStr">
-        <is>
-          <t>CUE</t>
-        </is>
-      </c>
+      <c r="H105" t="inlineStr"/>
       <c r="I105" t="inlineStr"/>
       <c r="J105" t="inlineStr"/>
       <c r="K105" t="inlineStr"/>
       <c r="L105" t="inlineStr"/>
       <c r="M105" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27908</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27964</t>
         </is>
       </c>
     </row>
@@ -6186,7 +6186,7 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>朱色の仮面</t>
+          <t>ジャンケットバンク</t>
         </is>
       </c>
       <c r="E106" t="b">
@@ -6199,17 +6199,21 @@
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>2026年10月～ 読売テレビ・日本テレビ系全国ネットにて</t>
-        </is>
-      </c>
-      <c r="H106" t="inlineStr"/>
+          <t>2026年10月～</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>CUE</t>
+        </is>
+      </c>
       <c r="I106" t="inlineStr"/>
       <c r="J106" t="inlineStr"/>
       <c r="K106" t="inlineStr"/>
       <c r="L106" t="inlineStr"/>
       <c r="M106" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26362</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27908</t>
         </is>
       </c>
     </row>
@@ -6227,7 +6231,7 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>獣王武神ダンデヴァイン</t>
+          <t>朱色の仮面</t>
         </is>
       </c>
       <c r="E107" t="b">
@@ -6240,29 +6244,17 @@
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
-        </is>
-      </c>
-      <c r="H107" t="inlineStr">
-        <is>
-          <t>ライデンフィルム</t>
-        </is>
-      </c>
-      <c r="I107" t="inlineStr">
-        <is>
-          <t>曲名未発表</t>
-        </is>
-      </c>
-      <c r="J107" t="inlineStr">
-        <is>
-          <t>西川貴教</t>
-        </is>
-      </c>
+          <t>2026年10月～ 読売テレビ・日本テレビ系全国ネットにて</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr"/>
+      <c r="I107" t="inlineStr"/>
+      <c r="J107" t="inlineStr"/>
       <c r="K107" t="inlineStr"/>
       <c r="L107" t="inlineStr"/>
       <c r="M107" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28479</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26362</t>
         </is>
       </c>
     </row>
@@ -6280,7 +6272,7 @@
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>しろたん</t>
+          <t>獣王武神ダンデヴァイン</t>
         </is>
       </c>
       <c r="E108" t="b">
@@ -6293,21 +6285,29 @@
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>2026年10月～ テレビ朝日にて</t>
+          <t>2026年10月～</t>
         </is>
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>レスプリ</t>
-        </is>
-      </c>
-      <c r="I108" t="inlineStr"/>
-      <c r="J108" t="inlineStr"/>
+          <t>ライデンフィルム</t>
+        </is>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>曲名未発表</t>
+        </is>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>西川貴教</t>
+        </is>
+      </c>
       <c r="K108" t="inlineStr"/>
       <c r="L108" t="inlineStr"/>
       <c r="M108" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27989</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28479</t>
         </is>
       </c>
     </row>
@@ -6325,7 +6325,7 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>新テニスの王子様 U-17 WORLD CUP 決勝メンバー決定戦</t>
+          <t>しろたん</t>
         </is>
       </c>
       <c r="E109" t="b">
@@ -6338,17 +6338,21 @@
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>2026年秋</t>
-        </is>
-      </c>
-      <c r="H109" t="inlineStr"/>
+          <t>2026年10月～ テレビ朝日にて</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>レスプリ</t>
+        </is>
+      </c>
       <c r="I109" t="inlineStr"/>
       <c r="J109" t="inlineStr"/>
       <c r="K109" t="inlineStr"/>
       <c r="L109" t="inlineStr"/>
       <c r="M109" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26829</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27989</t>
         </is>
       </c>
     </row>
@@ -6366,7 +6370,7 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>世界最強の魔女、始めました</t>
+          <t>新テニスの王子様 U-17 WORLD CUP 決勝メンバー決定戦</t>
         </is>
       </c>
       <c r="E110" t="b">
@@ -6379,21 +6383,17 @@
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
-        </is>
-      </c>
-      <c r="H110" t="inlineStr">
-        <is>
-          <t>ブリッジ</t>
-        </is>
-      </c>
+          <t>2026年秋</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr"/>
       <c r="I110" t="inlineStr"/>
       <c r="J110" t="inlineStr"/>
       <c r="K110" t="inlineStr"/>
       <c r="L110" t="inlineStr"/>
       <c r="M110" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28288</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26829</t>
         </is>
       </c>
     </row>
@@ -6411,7 +6411,7 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>#ゾンビさがしてます</t>
+          <t>世界最強の魔女、始めました</t>
         </is>
       </c>
       <c r="E111" t="b">
@@ -6424,17 +6424,21 @@
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>2026年10月〜 テレビ朝日系にて</t>
-        </is>
-      </c>
-      <c r="H111" t="inlineStr"/>
+          <t>2026年10月～</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>ブリッジ</t>
+        </is>
+      </c>
       <c r="I111" t="inlineStr"/>
       <c r="J111" t="inlineStr"/>
       <c r="K111" t="inlineStr"/>
       <c r="L111" t="inlineStr"/>
       <c r="M111" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26825</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28288</t>
         </is>
       </c>
     </row>
@@ -6452,7 +6456,7 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>ダイヤのA actⅡ -Second Season- 第2クール</t>
+          <t>#ゾンビさがしてます</t>
         </is>
       </c>
       <c r="E112" t="b">
@@ -6465,37 +6469,17 @@
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>第1クール：2026年4月5日（日）～2026年6月28日（日） 第2クール：2026年10月～ テレビ東京ほか</t>
-        </is>
-      </c>
-      <c r="H112" t="inlineStr">
-        <is>
-          <t>OLM</t>
-        </is>
-      </c>
-      <c r="I112" t="inlineStr">
-        <is>
-          <t>Let's Go Crazy</t>
-        </is>
-      </c>
-      <c r="J112" t="inlineStr">
-        <is>
-          <t>Baby Canta</t>
-        </is>
-      </c>
-      <c r="K112" t="inlineStr">
-        <is>
-          <t>NUMBER</t>
-        </is>
-      </c>
-      <c r="L112" t="inlineStr">
-        <is>
-          <t>SUPER★DRAGON</t>
-        </is>
-      </c>
+          <t>2026年10月〜 テレビ朝日系にて</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr"/>
+      <c r="I112" t="inlineStr"/>
+      <c r="J112" t="inlineStr"/>
+      <c r="K112" t="inlineStr"/>
+      <c r="L112" t="inlineStr"/>
       <c r="M112" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=24072</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26825</t>
         </is>
       </c>
     </row>
@@ -6513,7 +6497,7 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>タヌキとキツネ</t>
+          <t>ダイヤのA actⅡ -Second Season- 第2クール</t>
         </is>
       </c>
       <c r="E113" t="b">
@@ -6526,17 +6510,37 @@
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
-        </is>
-      </c>
-      <c r="H113" t="inlineStr"/>
-      <c r="I113" t="inlineStr"/>
-      <c r="J113" t="inlineStr"/>
-      <c r="K113" t="inlineStr"/>
-      <c r="L113" t="inlineStr"/>
+          <t>第1クール：2026年4月5日（日）～2026年6月28日（日） 第2クール：2026年10月～ テレビ東京ほか</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>OLM</t>
+        </is>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>Let's Go Crazy</t>
+        </is>
+      </c>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t>Baby Canta</t>
+        </is>
+      </c>
+      <c r="K113" t="inlineStr">
+        <is>
+          <t>NUMBER</t>
+        </is>
+      </c>
+      <c r="L113" t="inlineStr">
+        <is>
+          <t>SUPER★DRAGON</t>
+        </is>
+      </c>
       <c r="M113" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=6380</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=24072</t>
         </is>
       </c>
     </row>
@@ -6554,7 +6558,7 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>TANK CHAIR-戦車椅子-</t>
+          <t>タヌキとキツネ</t>
         </is>
       </c>
       <c r="E114" t="b">
@@ -6567,21 +6571,17 @@
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>2026年秋</t>
-        </is>
-      </c>
-      <c r="H114" t="inlineStr">
-        <is>
-          <t>ポリゴン・ピクチュアズ</t>
-        </is>
-      </c>
+          <t>2026年10月～</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr"/>
       <c r="I114" t="inlineStr"/>
       <c r="J114" t="inlineStr"/>
       <c r="K114" t="inlineStr"/>
       <c r="L114" t="inlineStr"/>
       <c r="M114" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27965</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=6380</t>
         </is>
       </c>
     </row>
@@ -6599,7 +6599,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>探偵はもう、死んでいる。Season2</t>
+          <t>TANK CHAIR-戦車椅子-</t>
         </is>
       </c>
       <c r="E115" t="b">
@@ -6612,12 +6612,12 @@
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>2026年10月〜</t>
+          <t>2026年秋</t>
         </is>
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>ENGI</t>
+          <t>ポリゴン・ピクチュアズ</t>
         </is>
       </c>
       <c r="I115" t="inlineStr"/>
@@ -6626,7 +6626,7 @@
       <c r="L115" t="inlineStr"/>
       <c r="M115" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=16348</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27965</t>
         </is>
       </c>
     </row>
@@ -6644,7 +6644,7 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>超巡！超条先輩</t>
+          <t>探偵はもう、死んでいる。Season2</t>
         </is>
       </c>
       <c r="E116" t="b">
@@ -6657,12 +6657,12 @@
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>2026年10月～ カンテレ・フジテレビ系全国ネットにて</t>
+          <t>2026年10月〜</t>
         </is>
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>アルボアニメーション</t>
+          <t>ENGI</t>
         </is>
       </c>
       <c r="I116" t="inlineStr"/>
@@ -6671,7 +6671,7 @@
       <c r="L116" t="inlineStr"/>
       <c r="M116" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26933</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=16348</t>
         </is>
       </c>
     </row>
@@ -6689,7 +6689,7 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>追放されたチート付与魔術師は気ままなセカンドライフを謳歌する。</t>
+          <t>超巡！超条先輩</t>
         </is>
       </c>
       <c r="E117" t="b">
@@ -6702,12 +6702,12 @@
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>2026年10月～ テレ東系列にて</t>
+          <t>2026年10月～ カンテレ・フジテレビ系全国ネットにて</t>
         </is>
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>P.A.WORKS</t>
+          <t>アルボアニメーション</t>
         </is>
       </c>
       <c r="I117" t="inlineStr"/>
@@ -6716,7 +6716,7 @@
       <c r="L117" t="inlineStr"/>
       <c r="M117" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27631</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26933</t>
         </is>
       </c>
     </row>
@@ -6734,7 +6734,7 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>てつりょー！meet with 鉄道むすめ</t>
+          <t>追放されたチート付与魔術師は気ままなセカンドライフを謳歌する。</t>
         </is>
       </c>
       <c r="E118" t="b">
@@ -6747,12 +6747,12 @@
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>2026年秋</t>
+          <t>2026年10月～ テレ東系列にて</t>
         </is>
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>イーストフィッシュスタジオ</t>
+          <t>P.A.WORKS</t>
         </is>
       </c>
       <c r="I118" t="inlineStr"/>
@@ -6761,7 +6761,7 @@
       <c r="L118" t="inlineStr"/>
       <c r="M118" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26895</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27631</t>
         </is>
       </c>
     </row>
@@ -6779,7 +6779,7 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>テムパル～アイテムの力～</t>
+          <t>てつりょー！meet with 鉄道むすめ</t>
         </is>
       </c>
       <c r="E119" t="b">
@@ -6792,12 +6792,12 @@
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
+          <t>2026年秋</t>
         </is>
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>J.C.STAFF</t>
+          <t>イーストフィッシュスタジオ</t>
         </is>
       </c>
       <c r="I119" t="inlineStr"/>
@@ -6806,7 +6806,7 @@
       <c r="L119" t="inlineStr"/>
       <c r="M119" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28478</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26895</t>
         </is>
       </c>
     </row>
@@ -6824,7 +6824,7 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>転生貴族、鑑定スキルで成り上がる 第3期</t>
+          <t>テムパル～アイテムの力～</t>
         </is>
       </c>
       <c r="E120" t="b">
@@ -6837,12 +6837,12 @@
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>2026年秋 CBC/TBS系全国28局ネット「アガルアニメ」にて</t>
+          <t>2026年10月～</t>
         </is>
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>studio MOTHER</t>
+          <t>J.C.STAFF</t>
         </is>
       </c>
       <c r="I120" t="inlineStr"/>
@@ -6851,7 +6851,7 @@
       <c r="L120" t="inlineStr"/>
       <c r="M120" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25385</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28478</t>
         </is>
       </c>
     </row>
@@ -6869,7 +6869,7 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>転生ゴブリンだけど質問ある？</t>
+          <t>転生貴族、鑑定スキルで成り上がる 第3期</t>
         </is>
       </c>
       <c r="E121" t="b">
@@ -6882,12 +6882,12 @@
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
+          <t>2026年秋 CBC/TBS系全国28局ネット「アガルアニメ」にて</t>
         </is>
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>BAKKKA</t>
+          <t>studio MOTHER</t>
         </is>
       </c>
       <c r="I121" t="inlineStr"/>
@@ -6896,7 +6896,7 @@
       <c r="L121" t="inlineStr"/>
       <c r="M121" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27909</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25385</t>
         </is>
       </c>
     </row>
@@ -6914,7 +6914,7 @@
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>転生した大聖女は、聖女であることをひた隠す</t>
+          <t>転生ゴブリンだけど質問ある？</t>
         </is>
       </c>
       <c r="E122" t="b">
@@ -6932,32 +6932,16 @@
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>FelixFilm</t>
-        </is>
-      </c>
-      <c r="I122" t="inlineStr">
-        <is>
-          <t>Flare of Soul</t>
-        </is>
-      </c>
-      <c r="J122" t="inlineStr">
-        <is>
-          <t>花耶</t>
-        </is>
-      </c>
-      <c r="K122" t="inlineStr">
-        <is>
-          <t>STELLAR</t>
-        </is>
-      </c>
-      <c r="L122" t="inlineStr">
-        <is>
-          <t>ウタヒメドリーム オールスターズ</t>
-        </is>
-      </c>
+          <t>BAKKKA</t>
+        </is>
+      </c>
+      <c r="I122" t="inlineStr"/>
+      <c r="J122" t="inlineStr"/>
+      <c r="K122" t="inlineStr"/>
+      <c r="L122" t="inlineStr"/>
       <c r="M122" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25630</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27909</t>
         </is>
       </c>
     </row>
@@ -6975,7 +6959,7 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>転生したら剣でした 第2期</t>
+          <t>転生した大聖女は、聖女であることをひた隠す</t>
         </is>
       </c>
       <c r="E123" t="b">
@@ -6993,16 +6977,32 @@
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>C2C</t>
-        </is>
-      </c>
-      <c r="I123" t="inlineStr"/>
-      <c r="J123" t="inlineStr"/>
-      <c r="K123" t="inlineStr"/>
-      <c r="L123" t="inlineStr"/>
+          <t>FelixFilm</t>
+        </is>
+      </c>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>Flare of Soul</t>
+        </is>
+      </c>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t>花耶</t>
+        </is>
+      </c>
+      <c r="K123" t="inlineStr">
+        <is>
+          <t>STELLAR</t>
+        </is>
+      </c>
+      <c r="L123" t="inlineStr">
+        <is>
+          <t>ウタヒメドリーム オールスターズ</t>
+        </is>
+      </c>
       <c r="M123" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=19149</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25630</t>
         </is>
       </c>
     </row>
@@ -7020,7 +7020,7 @@
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>とある暗部の少女共棲</t>
+          <t>転生したら剣でした 第2期</t>
         </is>
       </c>
       <c r="E124" t="b">
@@ -7033,12 +7033,12 @@
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>2026年秋</t>
+          <t>2026年10月～</t>
         </is>
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>J.C.STAFF</t>
+          <t>C2C</t>
         </is>
       </c>
       <c r="I124" t="inlineStr"/>
@@ -7047,7 +7047,7 @@
       <c r="L124" t="inlineStr"/>
       <c r="M124" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25552</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=19149</t>
         </is>
       </c>
     </row>
@@ -7065,7 +7065,7 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>東京リベンジャーズ 三天戦争編</t>
+          <t>とある暗部の少女共棲</t>
         </is>
       </c>
       <c r="E125" t="b">
@@ -7078,12 +7078,12 @@
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>2026年10月2日（金）～ MBS・TBS・CBC”アニメイズム”枠ほか</t>
+          <t>2026年秋</t>
         </is>
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>ライデンフィルム</t>
+          <t>J.C.STAFF</t>
         </is>
       </c>
       <c r="I125" t="inlineStr"/>
@@ -7092,7 +7092,7 @@
       <c r="L125" t="inlineStr"/>
       <c r="M125" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=24207</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25552</t>
         </is>
       </c>
     </row>
@@ -7110,7 +7110,7 @@
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>桃源暗鬼 ～日光・華厳の滝編～</t>
+          <t>東京リベンジャーズ 三天戦争編</t>
         </is>
       </c>
       <c r="E126" t="b">
@@ -7123,17 +7123,21 @@
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t>2026年10月～ 日本テレビ系「FRIDAY ANIME NIGHT（フラアニ）」枠にて</t>
-        </is>
-      </c>
-      <c r="H126" t="inlineStr"/>
+          <t>2026年10月2日（金）～ MBS・TBS・CBC”アニメイズム”枠ほか</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>ライデンフィルム</t>
+        </is>
+      </c>
       <c r="I126" t="inlineStr"/>
       <c r="J126" t="inlineStr"/>
       <c r="K126" t="inlineStr"/>
       <c r="L126" t="inlineStr"/>
       <c r="M126" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27376</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=24207</t>
         </is>
       </c>
     </row>
@@ -7151,7 +7155,7 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>どうも、好きな人に惚れ薬を依頼された魔女です。</t>
+          <t>桃源暗鬼 ～日光・華厳の滝編～</t>
         </is>
       </c>
       <c r="E127" t="b">
@@ -7164,21 +7168,17 @@
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
-        </is>
-      </c>
-      <c r="H127" t="inlineStr">
-        <is>
-          <t>ディオメディア</t>
-        </is>
-      </c>
+          <t>2026年10月～ 日本テレビ系「FRIDAY ANIME NIGHT（フラアニ）」枠にて</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr"/>
       <c r="I127" t="inlineStr"/>
       <c r="J127" t="inlineStr"/>
       <c r="K127" t="inlineStr"/>
       <c r="L127" t="inlineStr"/>
       <c r="M127" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27581</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27376</t>
         </is>
       </c>
     </row>
@@ -7196,7 +7196,7 @@
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>ドラゴンボール超 ビルス</t>
+          <t>どうも、好きな人に惚れ薬を依頼された魔女です。</t>
         </is>
       </c>
       <c r="E128" t="b">
@@ -7209,17 +7209,21 @@
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t>2026年秋 フジテレビにて</t>
-        </is>
-      </c>
-      <c r="H128" t="inlineStr"/>
+          <t>2026年10月～</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>ディオメディア</t>
+        </is>
+      </c>
       <c r="I128" t="inlineStr"/>
       <c r="J128" t="inlineStr"/>
       <c r="K128" t="inlineStr"/>
       <c r="L128" t="inlineStr"/>
       <c r="M128" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27491</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27581</t>
         </is>
       </c>
     </row>
@@ -7237,7 +7241,7 @@
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>鳴海の平日</t>
+          <t>ドラゴンボール超 ビルス</t>
         </is>
       </c>
       <c r="E129" t="b">
@@ -7245,26 +7249,22 @@
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>配信</t>
+          <t>TVアニメ</t>
         </is>
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>2026年秋</t>
-        </is>
-      </c>
-      <c r="H129" t="inlineStr">
-        <is>
-          <t>Production I.G</t>
-        </is>
-      </c>
+          <t>2026年秋 フジテレビにて</t>
+        </is>
+      </c>
+      <c r="H129" t="inlineStr"/>
       <c r="I129" t="inlineStr"/>
       <c r="J129" t="inlineStr"/>
       <c r="K129" t="inlineStr"/>
       <c r="L129" t="inlineStr"/>
       <c r="M129" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28465</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27491</t>
         </is>
       </c>
     </row>
@@ -7282,7 +7282,7 @@
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>バーテックスフォース</t>
+          <t>鳴海の平日</t>
         </is>
       </c>
       <c r="E130" t="b">
@@ -7290,17 +7290,17 @@
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>TVアニメ</t>
+          <t>配信</t>
         </is>
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>2026年10月〜</t>
+          <t>2026年秋</t>
         </is>
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>SMDE</t>
+          <t>Production I.G</t>
         </is>
       </c>
       <c r="I130" t="inlineStr"/>
@@ -7309,7 +7309,7 @@
       <c r="L130" t="inlineStr"/>
       <c r="M130" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27988</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28465</t>
         </is>
       </c>
     </row>
@@ -7327,7 +7327,7 @@
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>Battle Spirits [Re] 絶界の空</t>
+          <t>バーテックスフォース</t>
         </is>
       </c>
       <c r="E131" t="b">
@@ -7340,17 +7340,21 @@
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>2026年秋</t>
-        </is>
-      </c>
-      <c r="H131" t="inlineStr"/>
+          <t>2026年10月〜</t>
+        </is>
+      </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>SMDE</t>
+        </is>
+      </c>
       <c r="I131" t="inlineStr"/>
       <c r="J131" t="inlineStr"/>
       <c r="K131" t="inlineStr"/>
       <c r="L131" t="inlineStr"/>
       <c r="M131" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27954</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27988</t>
         </is>
       </c>
     </row>
@@ -7368,7 +7372,7 @@
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>パンどろぼう</t>
+          <t>Battle Spirits [Re] 絶界の空</t>
         </is>
       </c>
       <c r="E132" t="b">
@@ -7381,7 +7385,7 @@
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>2026年10月〜 NHK Eテレにて</t>
+          <t>2026年秋</t>
         </is>
       </c>
       <c r="H132" t="inlineStr"/>
@@ -7391,7 +7395,7 @@
       <c r="L132" t="inlineStr"/>
       <c r="M132" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26163</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27954</t>
         </is>
       </c>
     </row>
@@ -7409,7 +7413,7 @@
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>百妖譜 京師篇</t>
+          <t>パンどろぼう</t>
         </is>
       </c>
       <c r="E133" t="b">
@@ -7422,7 +7426,7 @@
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>2026年10月〜 フジテレビ「B8station」にて</t>
+          <t>2026年10月〜 NHK Eテレにて</t>
         </is>
       </c>
       <c r="H133" t="inlineStr"/>
@@ -7432,7 +7436,7 @@
       <c r="L133" t="inlineStr"/>
       <c r="M133" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27781</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26163</t>
         </is>
       </c>
     </row>
@@ -7450,7 +7454,7 @@
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>冰剣の魔術師が世界を統べるⅡ</t>
+          <t>百妖譜 京師篇</t>
         </is>
       </c>
       <c r="E134" t="b">
@@ -7463,21 +7467,17 @@
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>2026年10月〜</t>
-        </is>
-      </c>
-      <c r="H134" t="inlineStr">
-        <is>
-          <t>ゼロジー</t>
-        </is>
-      </c>
+          <t>2026年10月〜 フジテレビ「B8station」にて</t>
+        </is>
+      </c>
+      <c r="H134" t="inlineStr"/>
       <c r="I134" t="inlineStr"/>
       <c r="J134" t="inlineStr"/>
       <c r="K134" t="inlineStr"/>
       <c r="L134" t="inlineStr"/>
       <c r="M134" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28403</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27781</t>
         </is>
       </c>
     </row>
@@ -7495,7 +7495,7 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>ブラッククローバー 2nd Season</t>
+          <t>冰剣の魔術師が世界を統べるⅡ</t>
         </is>
       </c>
       <c r="E135" t="b">
@@ -7508,12 +7508,12 @@
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>2026年10月～ テレ東系列ほか</t>
+          <t>2026年10月〜</t>
         </is>
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>スタジオぴえろ</t>
+          <t>ゼロジー</t>
         </is>
       </c>
       <c r="I135" t="inlineStr"/>
@@ -7522,7 +7522,7 @@
       <c r="L135" t="inlineStr"/>
       <c r="M135" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26361</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28403</t>
         </is>
       </c>
     </row>
@@ -7540,7 +7540,7 @@
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>ホタルの嫁入り</t>
+          <t>ブラッククローバー 2nd Season</t>
         </is>
       </c>
       <c r="E136" t="b">
@@ -7553,12 +7553,12 @@
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>2026年10月～ 全国フジテレビ系“ ノイタミナ ”にて</t>
+          <t>2026年10月～ テレ東系列ほか</t>
         </is>
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>david production</t>
+          <t>スタジオぴえろ</t>
         </is>
       </c>
       <c r="I136" t="inlineStr"/>
@@ -7567,7 +7567,7 @@
       <c r="L136" t="inlineStr"/>
       <c r="M136" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27415</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26361</t>
         </is>
       </c>
     </row>
@@ -7585,7 +7585,7 @@
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>ポップパップポルターズ</t>
+          <t>ホタルの嫁入り</t>
         </is>
       </c>
       <c r="E137" t="b">
@@ -7598,12 +7598,12 @@
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>2026年10月～ テレビ朝日「PicoAniTime」にて</t>
+          <t>2026年10月～ 全国フジテレビ系“ ノイタミナ ”にて</t>
         </is>
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>MOZU STUDIOS</t>
+          <t>david production</t>
         </is>
       </c>
       <c r="I137" t="inlineStr"/>
@@ -7612,7 +7612,7 @@
       <c r="L137" t="inlineStr"/>
       <c r="M137" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27823</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27415</t>
         </is>
       </c>
     </row>
@@ -7630,7 +7630,7 @@
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>ホテル・インヒューマンズ 第2期</t>
+          <t>ポップパップポルターズ</t>
         </is>
       </c>
       <c r="E138" t="b">
@@ -7643,12 +7643,12 @@
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t>2026年10月～ テレ東系列ほか</t>
+          <t>2026年10月～ テレビ朝日「PicoAniTime」にて</t>
         </is>
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>ブリッジ</t>
+          <t>MOZU STUDIOS</t>
         </is>
       </c>
       <c r="I138" t="inlineStr"/>
@@ -7657,7 +7657,7 @@
       <c r="L138" t="inlineStr"/>
       <c r="M138" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26870</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27823</t>
         </is>
       </c>
     </row>
@@ -7675,7 +7675,7 @@
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>マジカル★エクスプローラー</t>
+          <t>ホテル・インヒューマンズ 第2期</t>
         </is>
       </c>
       <c r="E139" t="b">
@@ -7688,12 +7688,12 @@
       </c>
       <c r="G139" t="inlineStr">
         <is>
-          <t>2026年秋</t>
+          <t>2026年10月～ テレ東系列ほか</t>
         </is>
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>WHITE FOX</t>
+          <t>ブリッジ</t>
         </is>
       </c>
       <c r="I139" t="inlineStr"/>
@@ -7702,7 +7702,7 @@
       <c r="L139" t="inlineStr"/>
       <c r="M139" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=23375</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26870</t>
         </is>
       </c>
     </row>
@@ -7720,7 +7720,7 @@
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>魔法騎士レイアース</t>
+          <t>マジカル★エクスプローラー</t>
         </is>
       </c>
       <c r="E140" t="b">
@@ -7733,12 +7733,12 @@
       </c>
       <c r="G140" t="inlineStr">
         <is>
-          <t>2026年10月～ テレビ朝日系列にて</t>
+          <t>2026年秋</t>
         </is>
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>E&amp;H production</t>
+          <t>WHITE FOX</t>
         </is>
       </c>
       <c r="I140" t="inlineStr"/>
@@ -7747,7 +7747,7 @@
       <c r="L140" t="inlineStr"/>
       <c r="M140" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=24301</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=23375</t>
         </is>
       </c>
     </row>
@@ -7765,7 +7765,7 @@
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>魔法少女育成計画restart</t>
+          <t>魔法騎士レイアース</t>
         </is>
       </c>
       <c r="E141" t="b">
@@ -7778,29 +7778,21 @@
       </c>
       <c r="G141" t="inlineStr">
         <is>
-          <t>2026年秋</t>
+          <t>2026年10月～ テレビ朝日系列にて</t>
         </is>
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>SynergySP</t>
-        </is>
-      </c>
-      <c r="I141" t="inlineStr">
-        <is>
-          <t>No tears here</t>
-        </is>
-      </c>
-      <c r="J141" t="inlineStr">
-        <is>
-          <t>茅原実里</t>
-        </is>
-      </c>
+          <t>E&amp;H production</t>
+        </is>
+      </c>
+      <c r="I141" t="inlineStr"/>
+      <c r="J141" t="inlineStr"/>
       <c r="K141" t="inlineStr"/>
       <c r="L141" t="inlineStr"/>
       <c r="M141" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26693</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=24301</t>
         </is>
       </c>
     </row>
@@ -7818,7 +7810,7 @@
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>魔法の姉妹ルルットリリィ 第2クール</t>
+          <t>魔法少女育成計画restart</t>
         </is>
       </c>
       <c r="E142" t="b">
@@ -7831,37 +7823,29 @@
       </c>
       <c r="G142" t="inlineStr">
         <is>
-          <t>第1クール：2026年4月5日（日）～2026年6月21日（日） 第2クール：2026年10月～ TOKYO MX・ABCテレビほか</t>
+          <t>2026年秋</t>
         </is>
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>スタジオぴえろ</t>
+          <t>SynergySP</t>
         </is>
       </c>
       <c r="I142" t="inlineStr">
         <is>
-          <t>Bubee</t>
+          <t>No tears here</t>
         </is>
       </c>
       <c r="J142" t="inlineStr">
         <is>
-          <t>ILLIT</t>
-        </is>
-      </c>
-      <c r="K142" t="inlineStr">
-        <is>
-          <t>Calling</t>
-        </is>
-      </c>
-      <c r="L142" t="inlineStr">
-        <is>
-          <t>ルルットリリィ（こんぺとリリィ（CV.橘めい）、ましゅールル（CV.小鹿なお））</t>
-        </is>
-      </c>
+          <t>茅原実里</t>
+        </is>
+      </c>
+      <c r="K142" t="inlineStr"/>
+      <c r="L142" t="inlineStr"/>
       <c r="M142" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=24293</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26693</t>
         </is>
       </c>
     </row>
@@ -7879,7 +7863,7 @@
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>マロニエ王国の七人の騎士</t>
+          <t>魔法の姉妹ルルットリリィ 第2クール</t>
         </is>
       </c>
       <c r="E143" t="b">
@@ -7892,21 +7876,37 @@
       </c>
       <c r="G143" t="inlineStr">
         <is>
-          <t>2026年10月～ NHK Eテレにて</t>
+          <t>第1クール：2026年4月5日（日）～2026年6月21日（日） 第2クール：2026年10月～ TOKYO MX・ABCテレビほか</t>
         </is>
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>J.C.STAFF</t>
-        </is>
-      </c>
-      <c r="I143" t="inlineStr"/>
-      <c r="J143" t="inlineStr"/>
-      <c r="K143" t="inlineStr"/>
-      <c r="L143" t="inlineStr"/>
+          <t>スタジオぴえろ</t>
+        </is>
+      </c>
+      <c r="I143" t="inlineStr">
+        <is>
+          <t>Bubee</t>
+        </is>
+      </c>
+      <c r="J143" t="inlineStr">
+        <is>
+          <t>ILLIT</t>
+        </is>
+      </c>
+      <c r="K143" t="inlineStr">
+        <is>
+          <t>Calling</t>
+        </is>
+      </c>
+      <c r="L143" t="inlineStr">
+        <is>
+          <t>ルルットリリィ（こんぺとリリィ（CV.橘めい）、ましゅールル（CV.小鹿なお））</t>
+        </is>
+      </c>
       <c r="M143" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28456</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=24293</t>
         </is>
       </c>
     </row>
@@ -7924,7 +7924,7 @@
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>目覚めたら最強装備と宇宙船持ちだったので、一戸建て目指して傭兵として自由に生きたい</t>
+          <t>マロニエ王国の七人の騎士</t>
         </is>
       </c>
       <c r="E144" t="b">
@@ -7937,12 +7937,12 @@
       </c>
       <c r="G144" t="inlineStr">
         <is>
-          <t>2026年10月〜</t>
+          <t>2026年10月～ NHK Eテレにて</t>
         </is>
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>studio A-CAT</t>
+          <t>J.C.STAFF</t>
         </is>
       </c>
       <c r="I144" t="inlineStr"/>
@@ -7951,7 +7951,7 @@
       <c r="L144" t="inlineStr"/>
       <c r="M144" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25525</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28456</t>
         </is>
       </c>
     </row>
@@ -7969,7 +7969,7 @@
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>ゆるゆる図鑑</t>
+          <t>目覚めたら最強装備と宇宙船持ちだったので、一戸建て目指して傭兵として自由に生きたい</t>
         </is>
       </c>
       <c r="E145" t="b">
@@ -7982,17 +7982,21 @@
       </c>
       <c r="G145" t="inlineStr">
         <is>
-          <t>2026年10月～ テレ東系列6局ネット「アニもり！」内にて</t>
-        </is>
-      </c>
-      <c r="H145" t="inlineStr"/>
+          <t>2026年10月〜</t>
+        </is>
+      </c>
+      <c r="H145" t="inlineStr">
+        <is>
+          <t>studio A-CAT</t>
+        </is>
+      </c>
       <c r="I145" t="inlineStr"/>
       <c r="J145" t="inlineStr"/>
       <c r="K145" t="inlineStr"/>
       <c r="L145" t="inlineStr"/>
       <c r="M145" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28579</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25525</t>
         </is>
       </c>
     </row>
@@ -8010,7 +8014,7 @@
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>夜桜さんちの大作戦 第2期 第2クール</t>
+          <t>ゆるゆる図鑑</t>
         </is>
       </c>
       <c r="E146" t="b">
@@ -8023,37 +8027,17 @@
       </c>
       <c r="G146" t="inlineStr">
         <is>
-          <t>第1クール：2026年4月12日（日）～2026年6月28日（日） 第2クール：2026年10月〜 MBS／TBS系全国28局ネットにて</t>
-        </is>
-      </c>
-      <c r="H146" t="inlineStr">
-        <is>
-          <t>SILVER LINK.</t>
-        </is>
-      </c>
-      <c r="I146" t="inlineStr">
-        <is>
-          <t>What's "KAZOKU"</t>
-        </is>
-      </c>
-      <c r="J146" t="inlineStr">
-        <is>
-          <t>櫻坂46</t>
-        </is>
-      </c>
-      <c r="K146" t="inlineStr">
-        <is>
-          <t>Shalala</t>
-        </is>
-      </c>
-      <c r="L146" t="inlineStr">
-        <is>
-          <t>ピラフ星人</t>
-        </is>
-      </c>
+          <t>2026年10月～ テレ東系列6局ネット「アニもり！」内にて</t>
+        </is>
+      </c>
+      <c r="H146" t="inlineStr"/>
+      <c r="I146" t="inlineStr"/>
+      <c r="J146" t="inlineStr"/>
+      <c r="K146" t="inlineStr"/>
+      <c r="L146" t="inlineStr"/>
       <c r="M146" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25032</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28579</t>
         </is>
       </c>
     </row>
@@ -8071,7 +8055,7 @@
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>弱気MAX令嬢なのに、辣腕婚約者様の賭けに乗ってしまった</t>
+          <t>夜桜さんちの大作戦 第2期 第2クール</t>
         </is>
       </c>
       <c r="E147" t="b">
@@ -8084,21 +8068,37 @@
       </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
+          <t>第1クール：2026年4月12日（日）～2026年6月28日（日） 第2クール：2026年10月〜 MBS／TBS系全国28局ネットにて</t>
         </is>
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>寿門堂</t>
-        </is>
-      </c>
-      <c r="I147" t="inlineStr"/>
-      <c r="J147" t="inlineStr"/>
-      <c r="K147" t="inlineStr"/>
-      <c r="L147" t="inlineStr"/>
+          <t>SILVER LINK.</t>
+        </is>
+      </c>
+      <c r="I147" t="inlineStr">
+        <is>
+          <t>What's "KAZOKU"</t>
+        </is>
+      </c>
+      <c r="J147" t="inlineStr">
+        <is>
+          <t>櫻坂46</t>
+        </is>
+      </c>
+      <c r="K147" t="inlineStr">
+        <is>
+          <t>Shalala</t>
+        </is>
+      </c>
+      <c r="L147" t="inlineStr">
+        <is>
+          <t>ピラフ星人</t>
+        </is>
+      </c>
       <c r="M147" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26947</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25032</t>
         </is>
       </c>
     </row>
@@ -8116,11 +8116,11 @@
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>ラブライブ！虹ヶ咲学園スクールアイドル同好会 第2期</t>
+          <t>弱気MAX令嬢なのに、辣腕婚約者様の賭けに乗ってしまった</t>
         </is>
       </c>
       <c r="E148" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F148" t="inlineStr">
         <is>
@@ -8129,12 +8129,12 @@
       </c>
       <c r="G148" t="inlineStr">
         <is>
-          <t>2022年4月2日（土）～2022年6月25日（土） TOKYO MXほか 【再放送】 2026年9月30日（水）〜 BS日テレにて</t>
+          <t>2026年10月～</t>
         </is>
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>サンライズ</t>
+          <t>寿門堂</t>
         </is>
       </c>
       <c r="I148" t="inlineStr"/>
@@ -8143,7 +8143,7 @@
       <c r="L148" t="inlineStr"/>
       <c r="M148" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=14120</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26947</t>
         </is>
       </c>
     </row>
@@ -8161,11 +8161,11 @@
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>らんま1/2 第3期</t>
+          <t>ラブライブ！虹ヶ咲学園スクールアイドル同好会 第2期</t>
         </is>
       </c>
       <c r="E149" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F149" t="inlineStr">
         <is>
@@ -8174,17 +8174,21 @@
       </c>
       <c r="G149" t="inlineStr">
         <is>
-          <t>2026年10月～ 日本テレビ系にて</t>
-        </is>
-      </c>
-      <c r="H149" t="inlineStr"/>
+          <t>2022年4月2日（土）～2022年6月25日（土） TOKYO MXほか 【再放送】 2026年9月30日（水）〜 BS日テレにて</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>サンライズ</t>
+        </is>
+      </c>
       <c r="I149" t="inlineStr"/>
       <c r="J149" t="inlineStr"/>
       <c r="K149" t="inlineStr"/>
       <c r="L149" t="inlineStr"/>
       <c r="M149" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28013</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=14120</t>
         </is>
       </c>
     </row>
@@ -8202,7 +8206,7 @@
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>LEGO® ONE PIECE</t>
+          <t>らんま1/2 第3期</t>
         </is>
       </c>
       <c r="E150" t="b">
@@ -8210,12 +8214,12 @@
       </c>
       <c r="F150" t="inlineStr">
         <is>
-          <t>配信</t>
+          <t>TVアニメ</t>
         </is>
       </c>
       <c r="G150" t="inlineStr">
         <is>
-          <t>2026年9月29日（火） Netflixにて</t>
+          <t>2026年10月～ 日本テレビ系にて</t>
         </is>
       </c>
       <c r="H150" t="inlineStr"/>
@@ -8224,6 +8228,47 @@
       <c r="K150" t="inlineStr"/>
       <c r="L150" t="inlineStr"/>
       <c r="M150" t="inlineStr">
+        <is>
+          <t>https://www.animatetimes.com/tag/details.php?id=28013</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C151" t="n">
+        <v>64</v>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>LEGO® ONE PIECE</t>
+        </is>
+      </c>
+      <c r="E151" t="b">
+        <v>0</v>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>配信</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>2026年9月29日（火） Netflixにて</t>
+        </is>
+      </c>
+      <c r="H151" t="inlineStr"/>
+      <c r="I151" t="inlineStr"/>
+      <c r="J151" t="inlineStr"/>
+      <c r="K151" t="inlineStr"/>
+      <c r="L151" t="inlineStr"/>
+      <c r="M151" t="inlineStr">
         <is>
           <t>https://www.animatetimes.com/tag/details.php?id=28168</t>
         </is>
@@ -9921,13 +9966,27 @@
           <t>りりあ。</t>
         </is>
       </c>
-      <c r="I32" t="inlineStr"/>
-      <c r="J32" t="inlineStr"/>
-      <c r="K32" t="inlineStr"/>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=mgW0k9I0n-8</t>
+        </is>
+      </c>
+      <c r="J32" t="n">
+        <v>5468</v>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>りりあ。</t>
+        </is>
+      </c>
       <c r="L32" t="inlineStr"/>
       <c r="M32" t="inlineStr"/>
       <c r="N32" t="inlineStr"/>
-      <c r="O32" t="inlineStr"/>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>2026-07-04T09:02:48</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -12329,7 +12388,7 @@
         </is>
       </c>
       <c r="J78" t="n">
-        <v>2770</v>
+        <v>3309</v>
       </c>
       <c r="K78" t="inlineStr">
         <is>
@@ -12341,7 +12400,7 @@
       <c r="N78" t="inlineStr"/>
       <c r="O78" t="inlineStr">
         <is>
-          <t>2026-06-27T09:04:53</t>
+          <t>2026-07-04T09:05:20</t>
         </is>
       </c>
     </row>
@@ -12941,11 +13000,11 @@
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=5Of2HNJa_gs</t>
+          <t>https://www.youtube.com/watch?v=JJaCwW4HyVs</t>
         </is>
       </c>
       <c r="J90" t="n">
-        <v>5618588</v>
+        <v>51132323</v>
       </c>
       <c r="K90" t="inlineStr">
         <is>
@@ -12957,7 +13016,7 @@
       <c r="N90" t="inlineStr"/>
       <c r="O90" t="inlineStr">
         <is>
-          <t>2026-06-26T09:06:03</t>
+          <t>2026-07-04T09:06:55</t>
         </is>
       </c>
     </row>
@@ -14067,7 +14126,7 @@
         </is>
       </c>
       <c r="J110" t="n">
-        <v>25222</v>
+        <v>410448</v>
       </c>
       <c r="K110" t="inlineStr">
         <is>
@@ -14080,7 +14139,7 @@
         </is>
       </c>
       <c r="M110" t="n">
-        <v>25222</v>
+        <v>410448</v>
       </c>
       <c r="N110" t="inlineStr">
         <is>
@@ -14089,7 +14148,7 @@
       </c>
       <c r="O110" t="inlineStr">
         <is>
-          <t>2026-06-27T09:06:42</t>
+          <t>2026-07-04T09:07:38</t>
         </is>
       </c>
     </row>
@@ -14414,13 +14473,37 @@
           <t>チョーキューメイ</t>
         </is>
       </c>
-      <c r="I117" t="inlineStr"/>
-      <c r="J117" t="inlineStr"/>
-      <c r="K117" t="inlineStr"/>
-      <c r="L117" t="inlineStr"/>
-      <c r="M117" t="inlineStr"/>
-      <c r="N117" t="inlineStr"/>
-      <c r="O117" t="inlineStr"/>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=SYpHpUiGcQU</t>
+        </is>
+      </c>
+      <c r="J117" t="n">
+        <v>1041</v>
+      </c>
+      <c r="K117" t="inlineStr">
+        <is>
+          <t>MBS animation 公式チャンネル</t>
+        </is>
+      </c>
+      <c r="L117" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=SYpHpUiGcQU</t>
+        </is>
+      </c>
+      <c r="M117" t="n">
+        <v>1041</v>
+      </c>
+      <c r="N117" t="inlineStr">
+        <is>
+          <t>MBS animation 公式チャンネル</t>
+        </is>
+      </c>
+      <c r="O117" t="inlineStr">
+        <is>
+          <t>2026-07-04T09:08:03</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="n">
@@ -15897,13 +15980,27 @@
           <t>花耶</t>
         </is>
       </c>
-      <c r="I146" t="inlineStr"/>
-      <c r="J146" t="inlineStr"/>
-      <c r="K146" t="inlineStr"/>
+      <c r="I146" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=Wx9lV4C2ShU</t>
+        </is>
+      </c>
+      <c r="J146" t="n">
+        <v>1391</v>
+      </c>
+      <c r="K146" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kaya Official YouTube Channel </t>
+        </is>
+      </c>
       <c r="L146" t="inlineStr"/>
       <c r="M146" t="inlineStr"/>
       <c r="N146" t="inlineStr"/>
-      <c r="O146" t="inlineStr"/>
+      <c r="O146" t="inlineStr">
+        <is>
+          <t>2026-07-04T09:09:16</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="n">
@@ -15989,7 +16086,7 @@
         </is>
       </c>
       <c r="J148" t="n">
-        <v>15548</v>
+        <v>145139</v>
       </c>
       <c r="K148" t="inlineStr">
         <is>
@@ -16002,7 +16099,7 @@
         </is>
       </c>
       <c r="M148" t="n">
-        <v>15548</v>
+        <v>145139</v>
       </c>
       <c r="N148" t="inlineStr">
         <is>
@@ -16011,7 +16108,7 @@
       </c>
       <c r="O148" t="inlineStr">
         <is>
-          <t>2026-06-27T09:08:38</t>
+          <t>2026-07-04T09:09:27</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: anime list update (PC) 2026-07-06
</commit_message>
<xml_diff>
--- a/data/anime_list.xlsx
+++ b/data/anime_list.xlsx
@@ -8643,13 +8643,37 @@
           <t>THE JET BOY BANGERZ</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=ms6fXO3Ngk4</t>
+        </is>
+      </c>
+      <c r="J7" t="n">
+        <v>9401</v>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>ヤンジャン漫画TV【集英社ヤングジャンプ公式】</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=ms6fXO3Ngk4</t>
+        </is>
+      </c>
+      <c r="M7" t="n">
+        <v>9401</v>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>ヤンジャン漫画TV【集英社ヤングジャンプ公式】</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>2026-07-06T09:00:34</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -8686,13 +8710,37 @@
           <t>WOLF HOWL HARMONY</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
-      <c r="O8" t="inlineStr"/>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=WM9BicFEhKs</t>
+        </is>
+      </c>
+      <c r="J8" t="n">
+        <v>4198</v>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>ヤンジャン漫画TV【集英社ヤングジャンプ公式】</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=WM9BicFEhKs</t>
+        </is>
+      </c>
+      <c r="M8" t="n">
+        <v>4198</v>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>ヤンジャン漫画TV【集英社ヤングジャンプ公式】</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>2026-07-06T09:00:43</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -9279,13 +9327,37 @@
           <t>ClariS</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr"/>
-      <c r="M19" t="inlineStr"/>
-      <c r="N19" t="inlineStr"/>
-      <c r="O19" t="inlineStr"/>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=MnFWBiWIfPg</t>
+        </is>
+      </c>
+      <c r="J19" t="n">
+        <v>47490</v>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>アニプレックス チャンネル</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=MnFWBiWIfPg</t>
+        </is>
+      </c>
+      <c r="M19" t="n">
+        <v>47490</v>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>アニプレックス チャンネル</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>2026-07-06T09:01:28</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -9322,13 +9394,37 @@
           <t>山崎育三郎</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
-      <c r="L20" t="inlineStr"/>
-      <c r="M20" t="inlineStr"/>
-      <c r="N20" t="inlineStr"/>
-      <c r="O20" t="inlineStr"/>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=ercJJBclL9k</t>
+        </is>
+      </c>
+      <c r="J20" t="n">
+        <v>20400</v>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>アニプレックス チャンネル</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=ercJJBclL9k</t>
+        </is>
+      </c>
+      <c r="M20" t="n">
+        <v>20400</v>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>アニプレックス チャンネル</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>2026-07-06T09:01:37</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -9923,13 +10019,37 @@
           <t>恋太郎ファミリー</t>
         </is>
       </c>
-      <c r="I31" t="inlineStr"/>
-      <c r="J31" t="inlineStr"/>
-      <c r="K31" t="inlineStr"/>
-      <c r="L31" t="inlineStr"/>
-      <c r="M31" t="inlineStr"/>
-      <c r="N31" t="inlineStr"/>
-      <c r="O31" t="inlineStr"/>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=cBhaKIqvUrQ</t>
+        </is>
+      </c>
+      <c r="J31" t="n">
+        <v>6356365</v>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>Bandai Namco Filmworks Channel</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=cBhaKIqvUrQ</t>
+        </is>
+      </c>
+      <c r="M31" t="n">
+        <v>6356365</v>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>Bandai Namco Filmworks Channel</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>2026-07-06T09:01:56</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -10863,13 +10983,37 @@
           <t>angela</t>
         </is>
       </c>
-      <c r="I49" t="inlineStr"/>
-      <c r="J49" t="inlineStr"/>
-      <c r="K49" t="inlineStr"/>
-      <c r="L49" t="inlineStr"/>
-      <c r="M49" t="inlineStr"/>
-      <c r="N49" t="inlineStr"/>
-      <c r="O49" t="inlineStr"/>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=nWwsthEoUnQ</t>
+        </is>
+      </c>
+      <c r="J49" t="n">
+        <v>14061</v>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>MBS animation 公式チャンネル</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=nWwsthEoUnQ</t>
+        </is>
+      </c>
+      <c r="M49" t="n">
+        <v>14061</v>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>MBS animation 公式チャンネル</t>
+        </is>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>2026-07-06T09:02:54</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -11780,13 +11924,37 @@
           <t>Redhair Rosy</t>
         </is>
       </c>
-      <c r="I66" t="inlineStr"/>
-      <c r="J66" t="inlineStr"/>
-      <c r="K66" t="inlineStr"/>
-      <c r="L66" t="inlineStr"/>
-      <c r="M66" t="inlineStr"/>
-      <c r="N66" t="inlineStr"/>
-      <c r="O66" t="inlineStr"/>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=RSfkFGTuPyo</t>
+        </is>
+      </c>
+      <c r="J66" t="n">
+        <v>2364</v>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>KING AMUSEMENT CREATIVE official channel</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=RSfkFGTuPyo</t>
+        </is>
+      </c>
+      <c r="M66" t="n">
+        <v>2364</v>
+      </c>
+      <c r="N66" t="inlineStr">
+        <is>
+          <t>KING AMUSEMENT CREATIVE official channel</t>
+        </is>
+      </c>
+      <c r="O66" t="inlineStr">
+        <is>
+          <t>2026-07-06T09:03:37</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -11823,13 +11991,37 @@
           <t>インナージャーニー</t>
         </is>
       </c>
-      <c r="I67" t="inlineStr"/>
-      <c r="J67" t="inlineStr"/>
-      <c r="K67" t="inlineStr"/>
-      <c r="L67" t="inlineStr"/>
-      <c r="M67" t="inlineStr"/>
-      <c r="N67" t="inlineStr"/>
-      <c r="O67" t="inlineStr"/>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=lrB8anaL9X4</t>
+        </is>
+      </c>
+      <c r="J67" t="n">
+        <v>1321</v>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>KING AMUSEMENT CREATIVE official channel</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=lrB8anaL9X4</t>
+        </is>
+      </c>
+      <c r="M67" t="n">
+        <v>1321</v>
+      </c>
+      <c r="N67" t="inlineStr">
+        <is>
+          <t>KING AMUSEMENT CREATIVE official channel</t>
+        </is>
+      </c>
+      <c r="O67" t="inlineStr">
+        <is>
+          <t>2026-07-06T09:03:46</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -12539,13 +12731,37 @@
           <t>SEKAI NO OWARI</t>
         </is>
       </c>
-      <c r="I81" t="inlineStr"/>
-      <c r="J81" t="inlineStr"/>
-      <c r="K81" t="inlineStr"/>
-      <c r="L81" t="inlineStr"/>
-      <c r="M81" t="inlineStr"/>
-      <c r="N81" t="inlineStr"/>
-      <c r="O81" t="inlineStr"/>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=_GlLp6hyM2E</t>
+        </is>
+      </c>
+      <c r="J81" t="n">
+        <v>124925</v>
+      </c>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>tv asahi  animation YouTubeチャンネル</t>
+        </is>
+      </c>
+      <c r="L81" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=_GlLp6hyM2E</t>
+        </is>
+      </c>
+      <c r="M81" t="n">
+        <v>124925</v>
+      </c>
+      <c r="N81" t="inlineStr">
+        <is>
+          <t>tv asahi  animation YouTubeチャンネル</t>
+        </is>
+      </c>
+      <c r="O81" t="inlineStr">
+        <is>
+          <t>2026-07-06T09:04:33</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -12582,13 +12798,37 @@
           <t>女王蜂</t>
         </is>
       </c>
-      <c r="I82" t="inlineStr"/>
-      <c r="J82" t="inlineStr"/>
-      <c r="K82" t="inlineStr"/>
-      <c r="L82" t="inlineStr"/>
-      <c r="M82" t="inlineStr"/>
-      <c r="N82" t="inlineStr"/>
-      <c r="O82" t="inlineStr"/>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=bLQV43WeRvk</t>
+        </is>
+      </c>
+      <c r="J82" t="n">
+        <v>42587</v>
+      </c>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t>tv asahi  animation YouTubeチャンネル</t>
+        </is>
+      </c>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=bLQV43WeRvk</t>
+        </is>
+      </c>
+      <c r="M82" t="n">
+        <v>42587</v>
+      </c>
+      <c r="N82" t="inlineStr">
+        <is>
+          <t>tv asahi  animation YouTubeチャンネル</t>
+        </is>
+      </c>
+      <c r="O82" t="inlineStr">
+        <is>
+          <t>2026-07-06T09:04:42</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -12888,13 +13128,37 @@
           <t>五阿弥ルナ</t>
         </is>
       </c>
-      <c r="I88" t="inlineStr"/>
-      <c r="J88" t="inlineStr"/>
-      <c r="K88" t="inlineStr"/>
-      <c r="L88" t="inlineStr"/>
-      <c r="M88" t="inlineStr"/>
-      <c r="N88" t="inlineStr"/>
-      <c r="O88" t="inlineStr"/>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=PX-b7KO3HOw</t>
+        </is>
+      </c>
+      <c r="J88" t="n">
+        <v>8471</v>
+      </c>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>KyoaniChannel</t>
+        </is>
+      </c>
+      <c r="L88" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=PX-b7KO3HOw</t>
+        </is>
+      </c>
+      <c r="M88" t="n">
+        <v>8471</v>
+      </c>
+      <c r="N88" t="inlineStr">
+        <is>
+          <t>KyoaniChannel</t>
+        </is>
+      </c>
+      <c r="O88" t="inlineStr">
+        <is>
+          <t>2026-07-06T09:05:07</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -13495,13 +13759,27 @@
           <t>内田真礼</t>
         </is>
       </c>
-      <c r="I99" t="inlineStr"/>
-      <c r="J99" t="inlineStr"/>
-      <c r="K99" t="inlineStr"/>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=SN2CGcKOZuY</t>
+        </is>
+      </c>
+      <c r="J99" t="n">
+        <v>3525</v>
+      </c>
+      <c r="K99" t="inlineStr">
+        <is>
+          <t>内田真礼（UCHIDA MAAYA）Official Channel</t>
+        </is>
+      </c>
       <c r="L99" t="inlineStr"/>
       <c r="M99" t="inlineStr"/>
       <c r="N99" t="inlineStr"/>
-      <c r="O99" t="inlineStr"/>
+      <c r="O99" t="inlineStr">
+        <is>
+          <t>2026-07-06T09:05:39</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="n">
@@ -14287,13 +14565,37 @@
           <t>jo0ji</t>
         </is>
       </c>
-      <c r="I113" t="inlineStr"/>
-      <c r="J113" t="inlineStr"/>
-      <c r="K113" t="inlineStr"/>
-      <c r="L113" t="inlineStr"/>
-      <c r="M113" t="inlineStr"/>
-      <c r="N113" t="inlineStr"/>
-      <c r="O113" t="inlineStr"/>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=IJONbpfIlUg</t>
+        </is>
+      </c>
+      <c r="J113" t="n">
+        <v>740213</v>
+      </c>
+      <c r="K113" t="inlineStr">
+        <is>
+          <t>『BLEACH』アニメ公式チャンネル</t>
+        </is>
+      </c>
+      <c r="L113" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=Ngy3tyOc0Rs</t>
+        </is>
+      </c>
+      <c r="M113" t="n">
+        <v>253343</v>
+      </c>
+      <c r="N113" t="inlineStr">
+        <is>
+          <t>『BLEACH』アニメ公式チャンネル</t>
+        </is>
+      </c>
+      <c r="O113" t="inlineStr">
+        <is>
+          <t>2026-07-06T09:06:00</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="n">
@@ -14669,13 +14971,27 @@
           <t>ももいろクローバーZ</t>
         </is>
       </c>
-      <c r="I121" t="inlineStr"/>
-      <c r="J121" t="inlineStr"/>
-      <c r="K121" t="inlineStr"/>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=udTJAApluV4</t>
+        </is>
+      </c>
+      <c r="J121" t="n">
+        <v>60</v>
+      </c>
+      <c r="K121" t="inlineStr">
+        <is>
+          <t>mogepuff rhythm channel</t>
+        </is>
+      </c>
       <c r="L121" t="inlineStr"/>
       <c r="M121" t="inlineStr"/>
       <c r="N121" t="inlineStr"/>
-      <c r="O121" t="inlineStr"/>
+      <c r="O121" t="inlineStr">
+        <is>
+          <t>2026-07-06T09:06:36</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="n">
@@ -16214,13 +16530,37 @@
           <t>雨穴</t>
         </is>
       </c>
-      <c r="I150" t="inlineStr"/>
-      <c r="J150" t="inlineStr"/>
-      <c r="K150" t="inlineStr"/>
-      <c r="L150" t="inlineStr"/>
-      <c r="M150" t="inlineStr"/>
-      <c r="N150" t="inlineStr"/>
-      <c r="O150" t="inlineStr"/>
+      <c r="I150" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=MnDO2Vv4ZkA</t>
+        </is>
+      </c>
+      <c r="J150" t="n">
+        <v>25023</v>
+      </c>
+      <c r="K150" t="inlineStr">
+        <is>
+          <t>TBSアニメ</t>
+        </is>
+      </c>
+      <c r="L150" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=MnDO2Vv4ZkA</t>
+        </is>
+      </c>
+      <c r="M150" t="n">
+        <v>25023</v>
+      </c>
+      <c r="N150" t="inlineStr">
+        <is>
+          <t>TBSアニメ</t>
+        </is>
+      </c>
+      <c r="O150" t="inlineStr">
+        <is>
+          <t>2026-07-06T09:07:31</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="n">

</xml_diff>

<commit_message>
auto: anime list update (PC) 2026-07-08
</commit_message>
<xml_diff>
--- a/data/anime_list.xlsx
+++ b/data/anime_list.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M155"/>
+  <dimension ref="A1:M156"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6443,7 +6443,7 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>新テニスの王子様 U-17 WORLD CUP 決勝メンバー決定戦</t>
+          <t>信者ゼロの女神サマと始める異世界攻略</t>
         </is>
       </c>
       <c r="E111" t="b">
@@ -6456,17 +6456,21 @@
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>2026年秋</t>
-        </is>
-      </c>
-      <c r="H111" t="inlineStr"/>
+          <t>2026年10月～</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>HORNETS</t>
+        </is>
+      </c>
       <c r="I111" t="inlineStr"/>
       <c r="J111" t="inlineStr"/>
       <c r="K111" t="inlineStr"/>
       <c r="L111" t="inlineStr"/>
       <c r="M111" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26829</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27418</t>
         </is>
       </c>
     </row>
@@ -6484,7 +6488,7 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>スティール・ボール・ラン ジョジョの奇妙な冒険 2nd &amp; 3rd STAGE</t>
+          <t>新テニスの王子様 U-17 WORLD CUP 決勝メンバー決定戦</t>
         </is>
       </c>
       <c r="E112" t="b">
@@ -6492,26 +6496,22 @@
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>配信</t>
+          <t>TVアニメ</t>
         </is>
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>1st STAGE：2026年3月19日（木）～ 2nd&amp;3rd STAGE：2026年9月25日（金）～ Netflixにて</t>
-        </is>
-      </c>
-      <c r="H112" t="inlineStr">
-        <is>
-          <t>david production</t>
-        </is>
-      </c>
+          <t>2026年秋</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr"/>
       <c r="I112" t="inlineStr"/>
       <c r="J112" t="inlineStr"/>
       <c r="K112" t="inlineStr"/>
       <c r="L112" t="inlineStr"/>
       <c r="M112" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25812</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26829</t>
         </is>
       </c>
     </row>
@@ -6529,7 +6529,7 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>生徒会にも穴はある！</t>
+          <t>スティール・ボール・ラン ジョジョの奇妙な冒険 2nd &amp; 3rd STAGE</t>
         </is>
       </c>
       <c r="E113" t="b">
@@ -6537,22 +6537,26 @@
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>TVアニメ</t>
+          <t>配信</t>
         </is>
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
-        </is>
-      </c>
-      <c r="H113" t="inlineStr"/>
+          <t>1st STAGE：2026年3月19日（木）～ 2nd&amp;3rd STAGE：2026年9月25日（金）～ Netflixにて</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>david production</t>
+        </is>
+      </c>
       <c r="I113" t="inlineStr"/>
       <c r="J113" t="inlineStr"/>
       <c r="K113" t="inlineStr"/>
       <c r="L113" t="inlineStr"/>
       <c r="M113" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25874</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25812</t>
         </is>
       </c>
     </row>
@@ -6570,7 +6574,7 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>世界最強の魔女、始めました</t>
+          <t>生徒会にも穴はある！</t>
         </is>
       </c>
       <c r="E114" t="b">
@@ -6586,18 +6590,14 @@
           <t>2026年10月～</t>
         </is>
       </c>
-      <c r="H114" t="inlineStr">
-        <is>
-          <t>ブリッジ</t>
-        </is>
-      </c>
+      <c r="H114" t="inlineStr"/>
       <c r="I114" t="inlineStr"/>
       <c r="J114" t="inlineStr"/>
       <c r="K114" t="inlineStr"/>
       <c r="L114" t="inlineStr"/>
       <c r="M114" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28288</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25874</t>
         </is>
       </c>
     </row>
@@ -6615,7 +6615,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>#ゾンビさがしてます</t>
+          <t>世界最強の魔女、始めました</t>
         </is>
       </c>
       <c r="E115" t="b">
@@ -6628,17 +6628,21 @@
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>2026年10月〜 テレビ朝日系にて</t>
-        </is>
-      </c>
-      <c r="H115" t="inlineStr"/>
+          <t>2026年10月～</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>ブリッジ</t>
+        </is>
+      </c>
       <c r="I115" t="inlineStr"/>
       <c r="J115" t="inlineStr"/>
       <c r="K115" t="inlineStr"/>
       <c r="L115" t="inlineStr"/>
       <c r="M115" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26825</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28288</t>
         </is>
       </c>
     </row>
@@ -6656,7 +6660,7 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>ダイヤのA actⅡ -Second Season- 第2クール</t>
+          <t>#ゾンビさがしてます</t>
         </is>
       </c>
       <c r="E116" t="b">
@@ -6669,37 +6673,17 @@
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>第1クール：2026年4月5日（日）～2026年6月28日（日） 第2クール：2026年10月～ テレビ東京ほか</t>
-        </is>
-      </c>
-      <c r="H116" t="inlineStr">
-        <is>
-          <t>OLM</t>
-        </is>
-      </c>
-      <c r="I116" t="inlineStr">
-        <is>
-          <t>Let's Go Crazy</t>
-        </is>
-      </c>
-      <c r="J116" t="inlineStr">
-        <is>
-          <t>Baby Canta</t>
-        </is>
-      </c>
-      <c r="K116" t="inlineStr">
-        <is>
-          <t>NUMBER</t>
-        </is>
-      </c>
-      <c r="L116" t="inlineStr">
-        <is>
-          <t>SUPER★DRAGON</t>
-        </is>
-      </c>
+          <t>2026年10月〜 テレビ朝日系にて</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr"/>
+      <c r="I116" t="inlineStr"/>
+      <c r="J116" t="inlineStr"/>
+      <c r="K116" t="inlineStr"/>
+      <c r="L116" t="inlineStr"/>
       <c r="M116" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=24072</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26825</t>
         </is>
       </c>
     </row>
@@ -6717,7 +6701,7 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>タヌキとキツネ</t>
+          <t>ダイヤのA actⅡ -Second Season- 第2クール</t>
         </is>
       </c>
       <c r="E117" t="b">
@@ -6730,17 +6714,37 @@
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
-        </is>
-      </c>
-      <c r="H117" t="inlineStr"/>
-      <c r="I117" t="inlineStr"/>
-      <c r="J117" t="inlineStr"/>
-      <c r="K117" t="inlineStr"/>
-      <c r="L117" t="inlineStr"/>
+          <t>第1クール：2026年4月5日（日）～2026年6月28日（日） 第2クール：2026年10月～ テレビ東京ほか</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>OLM</t>
+        </is>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>Let's Go Crazy</t>
+        </is>
+      </c>
+      <c r="J117" t="inlineStr">
+        <is>
+          <t>Baby Canta</t>
+        </is>
+      </c>
+      <c r="K117" t="inlineStr">
+        <is>
+          <t>NUMBER</t>
+        </is>
+      </c>
+      <c r="L117" t="inlineStr">
+        <is>
+          <t>SUPER★DRAGON</t>
+        </is>
+      </c>
       <c r="M117" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=6380</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=24072</t>
         </is>
       </c>
     </row>
@@ -6758,7 +6762,7 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>TANK CHAIR-戦車椅子-</t>
+          <t>タヌキとキツネ</t>
         </is>
       </c>
       <c r="E118" t="b">
@@ -6771,21 +6775,17 @@
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>2026年秋</t>
-        </is>
-      </c>
-      <c r="H118" t="inlineStr">
-        <is>
-          <t>ポリゴン・ピクチュアズ</t>
-        </is>
-      </c>
+          <t>2026年10月～</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr"/>
       <c r="I118" t="inlineStr"/>
       <c r="J118" t="inlineStr"/>
       <c r="K118" t="inlineStr"/>
       <c r="L118" t="inlineStr"/>
       <c r="M118" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27965</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=6380</t>
         </is>
       </c>
     </row>
@@ -6803,7 +6803,7 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>探偵はもう、死んでいる。Season2</t>
+          <t>TANK CHAIR-戦車椅子-</t>
         </is>
       </c>
       <c r="E119" t="b">
@@ -6816,12 +6816,12 @@
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>2026年10月〜</t>
+          <t>2026年秋</t>
         </is>
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>ENGI</t>
+          <t>ポリゴン・ピクチュアズ</t>
         </is>
       </c>
       <c r="I119" t="inlineStr"/>
@@ -6830,7 +6830,7 @@
       <c r="L119" t="inlineStr"/>
       <c r="M119" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=16348</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27965</t>
         </is>
       </c>
     </row>
@@ -6848,7 +6848,7 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>超巡！超条先輩</t>
+          <t>探偵はもう、死んでいる。Season2</t>
         </is>
       </c>
       <c r="E120" t="b">
@@ -6861,12 +6861,12 @@
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>2026年10月～ カンテレ・フジテレビ系全国ネットにて</t>
+          <t>2026年10月〜</t>
         </is>
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>アルボアニメーション</t>
+          <t>ENGI</t>
         </is>
       </c>
       <c r="I120" t="inlineStr"/>
@@ -6875,7 +6875,7 @@
       <c r="L120" t="inlineStr"/>
       <c r="M120" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26933</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=16348</t>
         </is>
       </c>
     </row>
@@ -6893,7 +6893,7 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>追放されたチート付与魔術師は気ままなセカンドライフを謳歌する。</t>
+          <t>超巡！超条先輩</t>
         </is>
       </c>
       <c r="E121" t="b">
@@ -6906,12 +6906,12 @@
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>2026年10月～ テレ東系列にて</t>
+          <t>2026年10月～ カンテレ・フジテレビ系全国ネットにて</t>
         </is>
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>P.A.WORKS</t>
+          <t>アルボアニメーション</t>
         </is>
       </c>
       <c r="I121" t="inlineStr"/>
@@ -6920,7 +6920,7 @@
       <c r="L121" t="inlineStr"/>
       <c r="M121" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27631</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26933</t>
         </is>
       </c>
     </row>
@@ -6938,7 +6938,7 @@
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>てつりょー！meet with 鉄道むすめ</t>
+          <t>追放されたチート付与魔術師は気ままなセカンドライフを謳歌する。</t>
         </is>
       </c>
       <c r="E122" t="b">
@@ -6951,12 +6951,12 @@
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>2026年秋</t>
+          <t>2026年10月～ テレ東系列にて</t>
         </is>
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>イーストフィッシュスタジオ</t>
+          <t>P.A.WORKS</t>
         </is>
       </c>
       <c r="I122" t="inlineStr"/>
@@ -6965,7 +6965,7 @@
       <c r="L122" t="inlineStr"/>
       <c r="M122" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26895</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27631</t>
         </is>
       </c>
     </row>
@@ -6983,7 +6983,7 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>テムパル～アイテムの力～</t>
+          <t>てつりょー！meet with 鉄道むすめ</t>
         </is>
       </c>
       <c r="E123" t="b">
@@ -6996,12 +6996,12 @@
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
+          <t>2026年秋</t>
         </is>
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>J.C.STAFF</t>
+          <t>イーストフィッシュスタジオ</t>
         </is>
       </c>
       <c r="I123" t="inlineStr"/>
@@ -7010,7 +7010,7 @@
       <c r="L123" t="inlineStr"/>
       <c r="M123" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28478</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26895</t>
         </is>
       </c>
     </row>
@@ -7028,7 +7028,7 @@
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>デモンズ・クレスト</t>
+          <t>テムパル～アイテムの力～</t>
         </is>
       </c>
       <c r="E124" t="b">
@@ -7036,34 +7036,26 @@
       </c>
       <c r="F124" t="inlineStr">
         <is>
-          <t>配信</t>
+          <t>TVアニメ</t>
         </is>
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>2026年11月6日（金） Prime Videoにて</t>
+          <t>2026年10月～</t>
         </is>
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>Production I.G</t>
-        </is>
-      </c>
-      <c r="I124" t="inlineStr">
-        <is>
-          <t>シンカ</t>
-        </is>
-      </c>
-      <c r="J124" t="inlineStr">
-        <is>
-          <t>Ado</t>
-        </is>
-      </c>
+          <t>J.C.STAFF</t>
+        </is>
+      </c>
+      <c r="I124" t="inlineStr"/>
+      <c r="J124" t="inlineStr"/>
       <c r="K124" t="inlineStr"/>
       <c r="L124" t="inlineStr"/>
       <c r="M124" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27189</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28478</t>
         </is>
       </c>
     </row>
@@ -7081,7 +7073,7 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>転生貴族、鑑定スキルで成り上がる 第3期</t>
+          <t>デモンズ・クレスト</t>
         </is>
       </c>
       <c r="E125" t="b">
@@ -7089,26 +7081,34 @@
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>TVアニメ</t>
+          <t>配信</t>
         </is>
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>2026年秋 CBC/TBS系全国28局ネット「アガルアニメ」にて</t>
+          <t>2026年11月6日（金） Prime Videoにて</t>
         </is>
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>studio MOTHER</t>
-        </is>
-      </c>
-      <c r="I125" t="inlineStr"/>
-      <c r="J125" t="inlineStr"/>
+          <t>Production I.G</t>
+        </is>
+      </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>シンカ</t>
+        </is>
+      </c>
+      <c r="J125" t="inlineStr">
+        <is>
+          <t>Ado</t>
+        </is>
+      </c>
       <c r="K125" t="inlineStr"/>
       <c r="L125" t="inlineStr"/>
       <c r="M125" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25385</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27189</t>
         </is>
       </c>
     </row>
@@ -7126,7 +7126,7 @@
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>転生ゴブリンだけど質問ある？</t>
+          <t>転生貴族、鑑定スキルで成り上がる 第3期</t>
         </is>
       </c>
       <c r="E126" t="b">
@@ -7139,12 +7139,12 @@
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
+          <t>2026年秋 CBC/TBS系全国28局ネット「アガルアニメ」にて</t>
         </is>
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>BAKKKA</t>
+          <t>studio MOTHER</t>
         </is>
       </c>
       <c r="I126" t="inlineStr"/>
@@ -7153,7 +7153,7 @@
       <c r="L126" t="inlineStr"/>
       <c r="M126" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27909</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25385</t>
         </is>
       </c>
     </row>
@@ -7171,7 +7171,7 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>転生した大聖女は、聖女であることをひた隠す</t>
+          <t>転生ゴブリンだけど質問ある？</t>
         </is>
       </c>
       <c r="E127" t="b">
@@ -7189,32 +7189,16 @@
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>FelixFilm</t>
-        </is>
-      </c>
-      <c r="I127" t="inlineStr">
-        <is>
-          <t>Flare of Soul</t>
-        </is>
-      </c>
-      <c r="J127" t="inlineStr">
-        <is>
-          <t>花耶</t>
-        </is>
-      </c>
-      <c r="K127" t="inlineStr">
-        <is>
-          <t>STELLAR</t>
-        </is>
-      </c>
-      <c r="L127" t="inlineStr">
-        <is>
-          <t>ウタヒメドリーム オールスターズ</t>
-        </is>
-      </c>
+          <t>BAKKKA</t>
+        </is>
+      </c>
+      <c r="I127" t="inlineStr"/>
+      <c r="J127" t="inlineStr"/>
+      <c r="K127" t="inlineStr"/>
+      <c r="L127" t="inlineStr"/>
       <c r="M127" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25630</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27909</t>
         </is>
       </c>
     </row>
@@ -7232,7 +7216,7 @@
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>転生したら剣でした 第2期</t>
+          <t>転生した大聖女は、聖女であることをひた隠す</t>
         </is>
       </c>
       <c r="E128" t="b">
@@ -7250,16 +7234,32 @@
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>C2C</t>
-        </is>
-      </c>
-      <c r="I128" t="inlineStr"/>
-      <c r="J128" t="inlineStr"/>
-      <c r="K128" t="inlineStr"/>
-      <c r="L128" t="inlineStr"/>
+          <t>FelixFilm</t>
+        </is>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>Flare of Soul</t>
+        </is>
+      </c>
+      <c r="J128" t="inlineStr">
+        <is>
+          <t>花耶</t>
+        </is>
+      </c>
+      <c r="K128" t="inlineStr">
+        <is>
+          <t>STELLAR</t>
+        </is>
+      </c>
+      <c r="L128" t="inlineStr">
+        <is>
+          <t>ウタヒメドリーム オールスターズ</t>
+        </is>
+      </c>
       <c r="M128" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=19149</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25630</t>
         </is>
       </c>
     </row>
@@ -7277,7 +7277,7 @@
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>とある暗部の少女共棲</t>
+          <t>転生したら剣でした 第2期</t>
         </is>
       </c>
       <c r="E129" t="b">
@@ -7290,37 +7290,21 @@
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>2026年10月9日（金）～ TOKYO MXほか</t>
+          <t>2026年10月～</t>
         </is>
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>J.C.STAFF</t>
-        </is>
-      </c>
-      <c r="I129" t="inlineStr">
-        <is>
-          <t>Ghost Sequence</t>
-        </is>
-      </c>
-      <c r="J129" t="inlineStr">
-        <is>
-          <t>East Of Eden</t>
-        </is>
-      </c>
-      <c r="K129" t="inlineStr">
-        <is>
-          <t>原子崩し(メルトダウナー)</t>
-        </is>
-      </c>
-      <c r="L129" t="inlineStr">
-        <is>
-          <t>岸田教団&amp;THE明星ロケッツ</t>
-        </is>
-      </c>
+          <t>C2C</t>
+        </is>
+      </c>
+      <c r="I129" t="inlineStr"/>
+      <c r="J129" t="inlineStr"/>
+      <c r="K129" t="inlineStr"/>
+      <c r="L129" t="inlineStr"/>
       <c r="M129" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25552</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=19149</t>
         </is>
       </c>
     </row>
@@ -7338,7 +7322,7 @@
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>東京リベンジャーズ 三天戦争編</t>
+          <t>とある暗部の少女共棲</t>
         </is>
       </c>
       <c r="E130" t="b">
@@ -7351,21 +7335,37 @@
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>2026年10月2日（金）～ MBS・TBS・CBC”アニメイズム”枠ほか</t>
+          <t>2026年10月9日（金）～ TOKYO MXほか</t>
         </is>
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>ライデンフィルム</t>
-        </is>
-      </c>
-      <c r="I130" t="inlineStr"/>
-      <c r="J130" t="inlineStr"/>
-      <c r="K130" t="inlineStr"/>
-      <c r="L130" t="inlineStr"/>
+          <t>J.C.STAFF</t>
+        </is>
+      </c>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>Ghost Sequence</t>
+        </is>
+      </c>
+      <c r="J130" t="inlineStr">
+        <is>
+          <t>East Of Eden</t>
+        </is>
+      </c>
+      <c r="K130" t="inlineStr">
+        <is>
+          <t>原子崩し(メルトダウナー)</t>
+        </is>
+      </c>
+      <c r="L130" t="inlineStr">
+        <is>
+          <t>岸田教団&amp;THE明星ロケッツ</t>
+        </is>
+      </c>
       <c r="M130" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=24207</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25552</t>
         </is>
       </c>
     </row>
@@ -7383,7 +7383,7 @@
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>桃源暗鬼 ～日光・華厳の滝編～</t>
+          <t>東京リベンジャーズ 三天戦争編</t>
         </is>
       </c>
       <c r="E131" t="b">
@@ -7396,17 +7396,21 @@
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>2026年10月～ 日本テレビ系「FRIDAY ANIME NIGHT（フラアニ）」枠にて</t>
-        </is>
-      </c>
-      <c r="H131" t="inlineStr"/>
+          <t>2026年10月2日（金）～ MBS・TBS・CBC”アニメイズム”枠ほか</t>
+        </is>
+      </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>ライデンフィルム</t>
+        </is>
+      </c>
       <c r="I131" t="inlineStr"/>
       <c r="J131" t="inlineStr"/>
       <c r="K131" t="inlineStr"/>
       <c r="L131" t="inlineStr"/>
       <c r="M131" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27376</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=24207</t>
         </is>
       </c>
     </row>
@@ -7424,7 +7428,7 @@
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>どうも、好きな人に惚れ薬を依頼された魔女です。</t>
+          <t>桃源暗鬼 ～日光・華厳の滝編～</t>
         </is>
       </c>
       <c r="E132" t="b">
@@ -7437,21 +7441,17 @@
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
-        </is>
-      </c>
-      <c r="H132" t="inlineStr">
-        <is>
-          <t>ディオメディア</t>
-        </is>
-      </c>
+          <t>2026年10月～ 日本テレビ系「FRIDAY ANIME NIGHT（フラアニ）」枠にて</t>
+        </is>
+      </c>
+      <c r="H132" t="inlineStr"/>
       <c r="I132" t="inlineStr"/>
       <c r="J132" t="inlineStr"/>
       <c r="K132" t="inlineStr"/>
       <c r="L132" t="inlineStr"/>
       <c r="M132" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27581</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27376</t>
         </is>
       </c>
     </row>
@@ -7469,7 +7469,7 @@
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>ドラゴンボール超 ビルス</t>
+          <t>どうも、好きな人に惚れ薬を依頼された魔女です。</t>
         </is>
       </c>
       <c r="E133" t="b">
@@ -7482,17 +7482,21 @@
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>2026年秋 フジテレビにて</t>
-        </is>
-      </c>
-      <c r="H133" t="inlineStr"/>
+          <t>2026年10月～</t>
+        </is>
+      </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>ディオメディア</t>
+        </is>
+      </c>
       <c r="I133" t="inlineStr"/>
       <c r="J133" t="inlineStr"/>
       <c r="K133" t="inlineStr"/>
       <c r="L133" t="inlineStr"/>
       <c r="M133" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27491</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27581</t>
         </is>
       </c>
     </row>
@@ -7510,7 +7514,7 @@
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>鳴海の平日</t>
+          <t>ドラゴンボール超 ビルス</t>
         </is>
       </c>
       <c r="E134" t="b">
@@ -7518,26 +7522,22 @@
       </c>
       <c r="F134" t="inlineStr">
         <is>
-          <t>配信</t>
+          <t>TVアニメ</t>
         </is>
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>2026年秋</t>
-        </is>
-      </c>
-      <c r="H134" t="inlineStr">
-        <is>
-          <t>Production I.G</t>
-        </is>
-      </c>
+          <t>2026年秋 フジテレビにて</t>
+        </is>
+      </c>
+      <c r="H134" t="inlineStr"/>
       <c r="I134" t="inlineStr"/>
       <c r="J134" t="inlineStr"/>
       <c r="K134" t="inlineStr"/>
       <c r="L134" t="inlineStr"/>
       <c r="M134" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28465</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27491</t>
         </is>
       </c>
     </row>
@@ -7555,7 +7555,7 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>バーテックスフォース</t>
+          <t>鳴海の平日</t>
         </is>
       </c>
       <c r="E135" t="b">
@@ -7563,17 +7563,17 @@
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>TVアニメ</t>
+          <t>配信</t>
         </is>
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>2026年10月〜</t>
+          <t>2026年秋</t>
         </is>
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>SMDE</t>
+          <t>Production I.G</t>
         </is>
       </c>
       <c r="I135" t="inlineStr"/>
@@ -7582,7 +7582,7 @@
       <c r="L135" t="inlineStr"/>
       <c r="M135" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27988</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28465</t>
         </is>
       </c>
     </row>
@@ -7600,7 +7600,7 @@
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>Battle Spirits [Re] 絶界の空</t>
+          <t>バーテックスフォース</t>
         </is>
       </c>
       <c r="E136" t="b">
@@ -7613,17 +7613,21 @@
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>2026年秋</t>
-        </is>
-      </c>
-      <c r="H136" t="inlineStr"/>
+          <t>2026年10月〜</t>
+        </is>
+      </c>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>SMDE</t>
+        </is>
+      </c>
       <c r="I136" t="inlineStr"/>
       <c r="J136" t="inlineStr"/>
       <c r="K136" t="inlineStr"/>
       <c r="L136" t="inlineStr"/>
       <c r="M136" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27954</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27988</t>
         </is>
       </c>
     </row>
@@ -7641,7 +7645,7 @@
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>パンどろぼう</t>
+          <t>Battle Spirits [Re] 絶界の空</t>
         </is>
       </c>
       <c r="E137" t="b">
@@ -7654,7 +7658,7 @@
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>2026年10月〜 NHK Eテレにて</t>
+          <t>2026年秋</t>
         </is>
       </c>
       <c r="H137" t="inlineStr"/>
@@ -7664,7 +7668,7 @@
       <c r="L137" t="inlineStr"/>
       <c r="M137" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26163</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27954</t>
         </is>
       </c>
     </row>
@@ -7682,7 +7686,7 @@
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>百妖譜 京師篇</t>
+          <t>パンどろぼう</t>
         </is>
       </c>
       <c r="E138" t="b">
@@ -7695,7 +7699,7 @@
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t>2026年10月〜 フジテレビ「B8station」にて</t>
+          <t>2026年10月〜 NHK Eテレにて</t>
         </is>
       </c>
       <c r="H138" t="inlineStr"/>
@@ -7705,7 +7709,7 @@
       <c r="L138" t="inlineStr"/>
       <c r="M138" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27781</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26163</t>
         </is>
       </c>
     </row>
@@ -7723,7 +7727,7 @@
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>冰剣の魔術師が世界を統べるⅡ</t>
+          <t>百妖譜 京師篇</t>
         </is>
       </c>
       <c r="E139" t="b">
@@ -7736,21 +7740,17 @@
       </c>
       <c r="G139" t="inlineStr">
         <is>
-          <t>2026年10月〜</t>
-        </is>
-      </c>
-      <c r="H139" t="inlineStr">
-        <is>
-          <t>ゼロジー</t>
-        </is>
-      </c>
+          <t>2026年10月〜 フジテレビ「B8station」にて</t>
+        </is>
+      </c>
+      <c r="H139" t="inlineStr"/>
       <c r="I139" t="inlineStr"/>
       <c r="J139" t="inlineStr"/>
       <c r="K139" t="inlineStr"/>
       <c r="L139" t="inlineStr"/>
       <c r="M139" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28403</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27781</t>
         </is>
       </c>
     </row>
@@ -7768,7 +7768,7 @@
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>ブラッククローバー 2nd Season</t>
+          <t>冰剣の魔術師が世界を統べるⅡ</t>
         </is>
       </c>
       <c r="E140" t="b">
@@ -7781,29 +7781,21 @@
       </c>
       <c r="G140" t="inlineStr">
         <is>
-          <t>2026年10月～ テレ東系列ほか</t>
+          <t>2026年10月〜</t>
         </is>
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>スタジオぴえろ</t>
-        </is>
-      </c>
-      <c r="I140" t="inlineStr">
-        <is>
-          <t>消えない理由</t>
-        </is>
-      </c>
-      <c r="J140" t="inlineStr">
-        <is>
-          <t>WANIMA</t>
-        </is>
-      </c>
+          <t>ゼロジー</t>
+        </is>
+      </c>
+      <c r="I140" t="inlineStr"/>
+      <c r="J140" t="inlineStr"/>
       <c r="K140" t="inlineStr"/>
       <c r="L140" t="inlineStr"/>
       <c r="M140" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26361</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28403</t>
         </is>
       </c>
     </row>
@@ -7821,7 +7813,7 @@
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>ホタルの嫁入り</t>
+          <t>ブラッククローバー 2nd Season</t>
         </is>
       </c>
       <c r="E141" t="b">
@@ -7834,21 +7826,29 @@
       </c>
       <c r="G141" t="inlineStr">
         <is>
-          <t>2026年10月～ 全国フジテレビ系“ ノイタミナ ”にて</t>
+          <t>2026年10月～ テレ東系列ほか</t>
         </is>
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>david production</t>
-        </is>
-      </c>
-      <c r="I141" t="inlineStr"/>
-      <c r="J141" t="inlineStr"/>
+          <t>スタジオぴえろ</t>
+        </is>
+      </c>
+      <c r="I141" t="inlineStr">
+        <is>
+          <t>消えない理由</t>
+        </is>
+      </c>
+      <c r="J141" t="inlineStr">
+        <is>
+          <t>WANIMA</t>
+        </is>
+      </c>
       <c r="K141" t="inlineStr"/>
       <c r="L141" t="inlineStr"/>
       <c r="M141" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27415</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26361</t>
         </is>
       </c>
     </row>
@@ -7866,7 +7866,7 @@
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>ポップパップポルターズ</t>
+          <t>ホタルの嫁入り</t>
         </is>
       </c>
       <c r="E142" t="b">
@@ -7879,12 +7879,12 @@
       </c>
       <c r="G142" t="inlineStr">
         <is>
-          <t>2026年10月～ テレビ朝日「PicoAniTime」にて</t>
+          <t>2026年10月～ 全国フジテレビ系“ ノイタミナ ”にて</t>
         </is>
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>MOZU STUDIOS</t>
+          <t>david production</t>
         </is>
       </c>
       <c r="I142" t="inlineStr"/>
@@ -7893,7 +7893,7 @@
       <c r="L142" t="inlineStr"/>
       <c r="M142" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27823</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27415</t>
         </is>
       </c>
     </row>
@@ -7911,7 +7911,7 @@
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>ホテル・インヒューマンズ 第2期</t>
+          <t>ポップパップポルターズ</t>
         </is>
       </c>
       <c r="E143" t="b">
@@ -7924,12 +7924,12 @@
       </c>
       <c r="G143" t="inlineStr">
         <is>
-          <t>2026年10月～ テレ東系列ほか</t>
+          <t>2026年10月～ テレビ朝日「PicoAniTime」にて</t>
         </is>
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>ブリッジ</t>
+          <t>MOZU STUDIOS</t>
         </is>
       </c>
       <c r="I143" t="inlineStr"/>
@@ -7938,7 +7938,7 @@
       <c r="L143" t="inlineStr"/>
       <c r="M143" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26870</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27823</t>
         </is>
       </c>
     </row>
@@ -7956,7 +7956,7 @@
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>マジカル★エクスプローラー</t>
+          <t>ホテル・インヒューマンズ 第2期</t>
         </is>
       </c>
       <c r="E144" t="b">
@@ -7969,12 +7969,12 @@
       </c>
       <c r="G144" t="inlineStr">
         <is>
-          <t>2026年秋</t>
+          <t>2026年10月～ テレ東系列ほか</t>
         </is>
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>WHITE FOX</t>
+          <t>ブリッジ</t>
         </is>
       </c>
       <c r="I144" t="inlineStr"/>
@@ -7983,7 +7983,7 @@
       <c r="L144" t="inlineStr"/>
       <c r="M144" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=23375</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26870</t>
         </is>
       </c>
     </row>
@@ -8001,7 +8001,7 @@
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>魔法騎士レイアース</t>
+          <t>マジカル★エクスプローラー</t>
         </is>
       </c>
       <c r="E145" t="b">
@@ -8014,12 +8014,12 @@
       </c>
       <c r="G145" t="inlineStr">
         <is>
-          <t>2026年10月7日（水）～ テレビ朝日系列にて</t>
+          <t>2026年秋</t>
         </is>
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>E&amp;H production</t>
+          <t>WHITE FOX</t>
         </is>
       </c>
       <c r="I145" t="inlineStr"/>
@@ -8028,7 +8028,7 @@
       <c r="L145" t="inlineStr"/>
       <c r="M145" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=24301</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=23375</t>
         </is>
       </c>
     </row>
@@ -8046,7 +8046,7 @@
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>魔法少女育成計画restart</t>
+          <t>魔法騎士レイアース</t>
         </is>
       </c>
       <c r="E146" t="b">
@@ -8059,29 +8059,21 @@
       </c>
       <c r="G146" t="inlineStr">
         <is>
-          <t>2026年秋</t>
+          <t>2026年10月7日（水）～ テレビ朝日系列にて</t>
         </is>
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>SynergySP</t>
-        </is>
-      </c>
-      <c r="I146" t="inlineStr">
-        <is>
-          <t>No tears here</t>
-        </is>
-      </c>
-      <c r="J146" t="inlineStr">
-        <is>
-          <t>茅原実里</t>
-        </is>
-      </c>
+          <t>E&amp;H production</t>
+        </is>
+      </c>
+      <c r="I146" t="inlineStr"/>
+      <c r="J146" t="inlineStr"/>
       <c r="K146" t="inlineStr"/>
       <c r="L146" t="inlineStr"/>
       <c r="M146" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26693</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=24301</t>
         </is>
       </c>
     </row>
@@ -8099,7 +8091,7 @@
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>魔法の姉妹ルルットリリィ 第2クール</t>
+          <t>魔法少女育成計画restart</t>
         </is>
       </c>
       <c r="E147" t="b">
@@ -8112,37 +8104,29 @@
       </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t>第1クール：2026年4月5日（日）～2026年6月21日（日） 第2クール：2026年10月～ TOKYO MX・ABCテレビほか</t>
+          <t>2026年秋</t>
         </is>
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>スタジオぴえろ</t>
+          <t>SynergySP</t>
         </is>
       </c>
       <c r="I147" t="inlineStr">
         <is>
-          <t>Bubee</t>
+          <t>No tears here</t>
         </is>
       </c>
       <c r="J147" t="inlineStr">
         <is>
-          <t>ILLIT</t>
-        </is>
-      </c>
-      <c r="K147" t="inlineStr">
-        <is>
-          <t>Calling</t>
-        </is>
-      </c>
-      <c r="L147" t="inlineStr">
-        <is>
-          <t>ルルットリリィ（こんぺとリリィ（CV.橘めい）、ましゅールル（CV.小鹿なお））</t>
-        </is>
-      </c>
+          <t>茅原実里</t>
+        </is>
+      </c>
+      <c r="K147" t="inlineStr"/>
+      <c r="L147" t="inlineStr"/>
       <c r="M147" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=24293</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26693</t>
         </is>
       </c>
     </row>
@@ -8160,7 +8144,7 @@
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>マロニエ王国の七人の騎士</t>
+          <t>魔法の姉妹ルルットリリィ 第2クール</t>
         </is>
       </c>
       <c r="E148" t="b">
@@ -8173,21 +8157,37 @@
       </c>
       <c r="G148" t="inlineStr">
         <is>
-          <t>2026年10月～ NHK Eテレにて</t>
+          <t>第1クール：2026年4月5日（日）～2026年6月21日（日） 第2クール：2026年10月～ TOKYO MX・ABCテレビほか</t>
         </is>
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>J.C.STAFF</t>
-        </is>
-      </c>
-      <c r="I148" t="inlineStr"/>
-      <c r="J148" t="inlineStr"/>
-      <c r="K148" t="inlineStr"/>
-      <c r="L148" t="inlineStr"/>
+          <t>スタジオぴえろ</t>
+        </is>
+      </c>
+      <c r="I148" t="inlineStr">
+        <is>
+          <t>Bubee</t>
+        </is>
+      </c>
+      <c r="J148" t="inlineStr">
+        <is>
+          <t>ILLIT</t>
+        </is>
+      </c>
+      <c r="K148" t="inlineStr">
+        <is>
+          <t>Calling</t>
+        </is>
+      </c>
+      <c r="L148" t="inlineStr">
+        <is>
+          <t>ルルットリリィ（こんぺとリリィ（CV.橘めい）、ましゅールル（CV.小鹿なお））</t>
+        </is>
+      </c>
       <c r="M148" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28456</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=24293</t>
         </is>
       </c>
     </row>
@@ -8205,7 +8205,7 @@
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>目覚めたら最強装備と宇宙船持ちだったので、一戸建て目指して傭兵として自由に生きたい</t>
+          <t>マロニエ王国の七人の騎士</t>
         </is>
       </c>
       <c r="E149" t="b">
@@ -8218,12 +8218,12 @@
       </c>
       <c r="G149" t="inlineStr">
         <is>
-          <t>2026年10月〜</t>
+          <t>2026年10月～ NHK Eテレにて</t>
         </is>
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>studio A-CAT</t>
+          <t>J.C.STAFF</t>
         </is>
       </c>
       <c r="I149" t="inlineStr"/>
@@ -8232,7 +8232,7 @@
       <c r="L149" t="inlineStr"/>
       <c r="M149" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25525</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28456</t>
         </is>
       </c>
     </row>
@@ -8250,7 +8250,7 @@
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>ゆるゆる図鑑</t>
+          <t>目覚めたら最強装備と宇宙船持ちだったので、一戸建て目指して傭兵として自由に生きたい</t>
         </is>
       </c>
       <c r="E150" t="b">
@@ -8263,17 +8263,37 @@
       </c>
       <c r="G150" t="inlineStr">
         <is>
-          <t>2026年10月～ テレ東系列6局ネット「アニもり！」内にて</t>
-        </is>
-      </c>
-      <c r="H150" t="inlineStr"/>
-      <c r="I150" t="inlineStr"/>
-      <c r="J150" t="inlineStr"/>
-      <c r="K150" t="inlineStr"/>
-      <c r="L150" t="inlineStr"/>
+          <t>2026年10月〜 TOKYO MX・読売テレビ・中京テレビほか</t>
+        </is>
+      </c>
+      <c r="H150" t="inlineStr">
+        <is>
+          <t>studio A-CAT</t>
+        </is>
+      </c>
+      <c r="I150" t="inlineStr">
+        <is>
+          <t>UNSTOPPABLE</t>
+        </is>
+      </c>
+      <c r="J150" t="inlineStr">
+        <is>
+          <t>FLOW</t>
+        </is>
+      </c>
+      <c r="K150" t="inlineStr">
+        <is>
+          <t>MY WAY</t>
+        </is>
+      </c>
+      <c r="L150" t="inlineStr">
+        <is>
+          <t>ASTERISM</t>
+        </is>
+      </c>
       <c r="M150" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28579</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25525</t>
         </is>
       </c>
     </row>
@@ -8291,7 +8311,7 @@
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>夜桜さんちの大作戦 第2期 第2クール</t>
+          <t>ゆるゆる図鑑</t>
         </is>
       </c>
       <c r="E151" t="b">
@@ -8304,37 +8324,17 @@
       </c>
       <c r="G151" t="inlineStr">
         <is>
-          <t>第1クール：2026年4月12日（日）～2026年6月28日（日） 第2クール：2026年10月〜 MBS／TBS系全国28局ネットにて</t>
-        </is>
-      </c>
-      <c r="H151" t="inlineStr">
-        <is>
-          <t>SILVER LINK.</t>
-        </is>
-      </c>
-      <c r="I151" t="inlineStr">
-        <is>
-          <t>What's "KAZOKU"</t>
-        </is>
-      </c>
-      <c r="J151" t="inlineStr">
-        <is>
-          <t>櫻坂46</t>
-        </is>
-      </c>
-      <c r="K151" t="inlineStr">
-        <is>
-          <t>Shalala</t>
-        </is>
-      </c>
-      <c r="L151" t="inlineStr">
-        <is>
-          <t>ピラフ星人</t>
-        </is>
-      </c>
+          <t>2026年10月～ テレ東系列6局ネット「アニもり！」内にて</t>
+        </is>
+      </c>
+      <c r="H151" t="inlineStr"/>
+      <c r="I151" t="inlineStr"/>
+      <c r="J151" t="inlineStr"/>
+      <c r="K151" t="inlineStr"/>
+      <c r="L151" t="inlineStr"/>
       <c r="M151" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25032</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28579</t>
         </is>
       </c>
     </row>
@@ -8352,7 +8352,7 @@
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>弱気MAX令嬢なのに、辣腕婚約者様の賭けに乗ってしまった</t>
+          <t>夜桜さんちの大作戦 第2期 第2クール</t>
         </is>
       </c>
       <c r="E152" t="b">
@@ -8365,21 +8365,37 @@
       </c>
       <c r="G152" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
+          <t>第1クール：2026年4月12日（日）～2026年6月28日（日） 第2クール：2026年10月〜 MBS／TBS系全国28局ネットにて</t>
         </is>
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>寿門堂</t>
-        </is>
-      </c>
-      <c r="I152" t="inlineStr"/>
-      <c r="J152" t="inlineStr"/>
-      <c r="K152" t="inlineStr"/>
-      <c r="L152" t="inlineStr"/>
+          <t>SILVER LINK.</t>
+        </is>
+      </c>
+      <c r="I152" t="inlineStr">
+        <is>
+          <t>What's "KAZOKU"</t>
+        </is>
+      </c>
+      <c r="J152" t="inlineStr">
+        <is>
+          <t>櫻坂46</t>
+        </is>
+      </c>
+      <c r="K152" t="inlineStr">
+        <is>
+          <t>Shalala</t>
+        </is>
+      </c>
+      <c r="L152" t="inlineStr">
+        <is>
+          <t>ピラフ星人</t>
+        </is>
+      </c>
       <c r="M152" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26947</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25032</t>
         </is>
       </c>
     </row>
@@ -8397,11 +8413,11 @@
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>ラブライブ！虹ヶ咲学園スクールアイドル同好会 第2期</t>
+          <t>弱気MAX令嬢なのに、辣腕婚約者様の賭けに乗ってしまった</t>
         </is>
       </c>
       <c r="E153" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F153" t="inlineStr">
         <is>
@@ -8410,12 +8426,12 @@
       </c>
       <c r="G153" t="inlineStr">
         <is>
-          <t>2022年4月2日（土）～2022年6月25日（土） TOKYO MXほか 【再放送】 2026年9月30日（水）〜 BS日テレにて</t>
+          <t>2026年10月～</t>
         </is>
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>サンライズ</t>
+          <t>寿門堂</t>
         </is>
       </c>
       <c r="I153" t="inlineStr"/>
@@ -8424,7 +8440,7 @@
       <c r="L153" t="inlineStr"/>
       <c r="M153" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=14120</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26947</t>
         </is>
       </c>
     </row>
@@ -8442,11 +8458,11 @@
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>らんま1/2 第3期</t>
+          <t>ラブライブ！虹ヶ咲学園スクールアイドル同好会 第2期</t>
         </is>
       </c>
       <c r="E154" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F154" t="inlineStr">
         <is>
@@ -8455,17 +8471,21 @@
       </c>
       <c r="G154" t="inlineStr">
         <is>
-          <t>2026年10月～ 日本テレビ系にて</t>
-        </is>
-      </c>
-      <c r="H154" t="inlineStr"/>
+          <t>2022年4月2日（土）～2022年6月25日（土） TOKYO MXほか 【再放送】 2026年9月30日（水）〜 BS日テレにて</t>
+        </is>
+      </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>サンライズ</t>
+        </is>
+      </c>
       <c r="I154" t="inlineStr"/>
       <c r="J154" t="inlineStr"/>
       <c r="K154" t="inlineStr"/>
       <c r="L154" t="inlineStr"/>
       <c r="M154" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28013</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=14120</t>
         </is>
       </c>
     </row>
@@ -8483,7 +8503,7 @@
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>LEGO® ONE PIECE</t>
+          <t>らんま1/2 第3期</t>
         </is>
       </c>
       <c r="E155" t="b">
@@ -8491,12 +8511,12 @@
       </c>
       <c r="F155" t="inlineStr">
         <is>
-          <t>配信</t>
+          <t>TVアニメ</t>
         </is>
       </c>
       <c r="G155" t="inlineStr">
         <is>
-          <t>2026年9月29日（火） Netflixにて</t>
+          <t>2026年10月～ 日本テレビ系にて</t>
         </is>
       </c>
       <c r="H155" t="inlineStr"/>
@@ -8505,6 +8525,47 @@
       <c r="K155" t="inlineStr"/>
       <c r="L155" t="inlineStr"/>
       <c r="M155" t="inlineStr">
+        <is>
+          <t>https://www.animatetimes.com/tag/details.php?id=28013</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C156" t="n">
+        <v>69</v>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>LEGO® ONE PIECE</t>
+        </is>
+      </c>
+      <c r="E156" t="b">
+        <v>0</v>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>配信</t>
+        </is>
+      </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>2026年9月29日（火） Netflixにて</t>
+        </is>
+      </c>
+      <c r="H156" t="inlineStr"/>
+      <c r="I156" t="inlineStr"/>
+      <c r="J156" t="inlineStr"/>
+      <c r="K156" t="inlineStr"/>
+      <c r="L156" t="inlineStr"/>
+      <c r="M156" t="inlineStr">
         <is>
           <t>https://www.animatetimes.com/tag/details.php?id=28168</t>
         </is>
@@ -8521,7 +8582,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O174"/>
+  <dimension ref="A1:O176"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11869,13 +11930,37 @@
           <t>INUWASI</t>
         </is>
       </c>
-      <c r="I59" t="inlineStr"/>
-      <c r="J59" t="inlineStr"/>
-      <c r="K59" t="inlineStr"/>
-      <c r="L59" t="inlineStr"/>
-      <c r="M59" t="inlineStr"/>
-      <c r="N59" t="inlineStr"/>
-      <c r="O59" t="inlineStr"/>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=sdOQK3KW2vI</t>
+        </is>
+      </c>
+      <c r="J59" t="n">
+        <v>5579</v>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>ハピネット【アニメ公式】</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=sdOQK3KW2vI</t>
+        </is>
+      </c>
+      <c r="M59" t="n">
+        <v>5579</v>
+      </c>
+      <c r="N59" t="inlineStr">
+        <is>
+          <t>ハピネット【アニメ公式】</t>
+        </is>
+      </c>
+      <c r="O59" t="inlineStr">
+        <is>
+          <t>2026-07-08T09:02:08</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -11912,13 +11997,37 @@
           <t>音感れもねゐど</t>
         </is>
       </c>
-      <c r="I60" t="inlineStr"/>
-      <c r="J60" t="inlineStr"/>
-      <c r="K60" t="inlineStr"/>
-      <c r="L60" t="inlineStr"/>
-      <c r="M60" t="inlineStr"/>
-      <c r="N60" t="inlineStr"/>
-      <c r="O60" t="inlineStr"/>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=5EcanUJkPOY</t>
+        </is>
+      </c>
+      <c r="J60" t="n">
+        <v>1207</v>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>ハピネット【アニメ公式】</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=5EcanUJkPOY</t>
+        </is>
+      </c>
+      <c r="M60" t="n">
+        <v>1207</v>
+      </c>
+      <c r="N60" t="inlineStr">
+        <is>
+          <t>ハピネット【アニメ公式】</t>
+        </is>
+      </c>
+      <c r="O60" t="inlineStr">
+        <is>
+          <t>2026-07-08T09:02:17</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -12433,13 +12542,37 @@
           <t>花冷え。</t>
         </is>
       </c>
-      <c r="I69" t="inlineStr"/>
-      <c r="J69" t="inlineStr"/>
-      <c r="K69" t="inlineStr"/>
-      <c r="L69" t="inlineStr"/>
-      <c r="M69" t="inlineStr"/>
-      <c r="N69" t="inlineStr"/>
-      <c r="O69" t="inlineStr"/>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=0T9ekzDoW1k</t>
+        </is>
+      </c>
+      <c r="J69" t="n">
+        <v>13887</v>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=0T9ekzDoW1k</t>
+        </is>
+      </c>
+      <c r="M69" t="n">
+        <v>13887</v>
+      </c>
+      <c r="N69" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="O69" t="inlineStr">
+        <is>
+          <t>2026-07-08T09:02:26</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -12906,13 +13039,27 @@
           <t>DIALOGUE+</t>
         </is>
       </c>
-      <c r="I78" t="inlineStr"/>
-      <c r="J78" t="inlineStr"/>
-      <c r="K78" t="inlineStr"/>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=kP1sP50Tzn4</t>
+        </is>
+      </c>
+      <c r="J78" t="n">
+        <v>6632</v>
+      </c>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>DIALOGUE＋Official Channel</t>
+        </is>
+      </c>
       <c r="L78" t="inlineStr"/>
       <c r="M78" t="inlineStr"/>
       <c r="N78" t="inlineStr"/>
-      <c r="O78" t="inlineStr"/>
+      <c r="O78" t="inlineStr">
+        <is>
+          <t>2026-07-08T09:03:06</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -13063,13 +13210,27 @@
           <t>清水美依紗</t>
         </is>
       </c>
-      <c r="I81" t="inlineStr"/>
-      <c r="J81" t="inlineStr"/>
-      <c r="K81" t="inlineStr"/>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=7UEZMkMqjVY</t>
+        </is>
+      </c>
+      <c r="J81" t="n">
+        <v>4059</v>
+      </c>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>清水美依紗 Miisha Shimizu</t>
+        </is>
+      </c>
       <c r="L81" t="inlineStr"/>
       <c r="M81" t="inlineStr"/>
       <c r="N81" t="inlineStr"/>
-      <c r="O81" t="inlineStr"/>
+      <c r="O81" t="inlineStr">
+        <is>
+          <t>2026-07-08T09:03:18</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -17329,21 +17490,21 @@
       </c>
       <c r="G157" t="inlineStr">
         <is>
-          <t>ONE PIECE（モノクロ版）</t>
+          <t>Blue Shining Star</t>
         </is>
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>電子書籍（コミック）</t>
+          <t>アイナ・ジ・エンド</t>
         </is>
       </c>
       <c r="I157" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=8dfGSzacxzc</t>
+          <t>https://www.youtube.com/watch?v=X48ZNGHBa8A</t>
         </is>
       </c>
       <c r="J157" t="n">
-        <v>11426324</v>
+        <v>2766827</v>
       </c>
       <c r="K157" t="inlineStr">
         <is>
@@ -17352,11 +17513,11 @@
       </c>
       <c r="L157" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=YFbno_aPm0w</t>
+          <t>https://www.youtube.com/watch?v=X48ZNGHBa8A</t>
         </is>
       </c>
       <c r="M157" t="n">
-        <v>28079784</v>
+        <v>2766827</v>
       </c>
       <c r="N157" t="inlineStr">
         <is>
@@ -17365,7 +17526,7 @@
       </c>
       <c r="O157" t="inlineStr">
         <is>
-          <t>2026-07-07T09:18:34</t>
+          <t>2026-07-08T09:05:44</t>
         </is>
       </c>
     </row>
@@ -18101,7 +18262,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>夜桜さんちの大作戦 第2期 第2クール</t>
+          <t>目覚めたら最強装備と宇宙船持ちだったので、一戸建て目指して傭兵として自由に生きたい</t>
         </is>
       </c>
       <c r="D173" t="b">
@@ -18117,45 +18278,21 @@
       </c>
       <c r="G173" t="inlineStr">
         <is>
-          <t>What's "KAZOKU"</t>
+          <t>UNSTOPPABLE</t>
         </is>
       </c>
       <c r="H173" t="inlineStr">
         <is>
-          <t>櫻坂46</t>
-        </is>
-      </c>
-      <c r="I173" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=4SdeuouXcWI</t>
-        </is>
-      </c>
-      <c r="J173" t="n">
-        <v>669793</v>
-      </c>
-      <c r="K173" t="inlineStr">
-        <is>
-          <t>櫻坂46 OFFICIAL YouTube CHANNEL</t>
-        </is>
-      </c>
-      <c r="L173" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=AIspds2UVts</t>
-        </is>
-      </c>
-      <c r="M173" t="n">
-        <v>347279</v>
-      </c>
-      <c r="N173" t="inlineStr">
-        <is>
-          <t>NBCUniversal Anime/Music</t>
-        </is>
-      </c>
-      <c r="O173" t="inlineStr">
-        <is>
-          <t>2026-07-07T09:20:03</t>
-        </is>
-      </c>
+          <t>FLOW</t>
+        </is>
+      </c>
+      <c r="I173" t="inlineStr"/>
+      <c r="J173" t="inlineStr"/>
+      <c r="K173" t="inlineStr"/>
+      <c r="L173" t="inlineStr"/>
+      <c r="M173" t="inlineStr"/>
+      <c r="N173" t="inlineStr"/>
+      <c r="O173" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" t="n">
@@ -18168,7 +18305,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>夜桜さんちの大作戦 第2期 第2クール</t>
+          <t>目覚めたら最強装備と宇宙船持ちだったので、一戸建て目指して傭兵として自由に生きたい</t>
         </is>
       </c>
       <c r="D174" t="b">
@@ -18184,41 +18321,151 @@
       </c>
       <c r="G174" t="inlineStr">
         <is>
+          <t>MY WAY</t>
+        </is>
+      </c>
+      <c r="H174" t="inlineStr">
+        <is>
+          <t>ASTERISM</t>
+        </is>
+      </c>
+      <c r="I174" t="inlineStr"/>
+      <c r="J174" t="inlineStr"/>
+      <c r="K174" t="inlineStr"/>
+      <c r="L174" t="inlineStr"/>
+      <c r="M174" t="inlineStr"/>
+      <c r="N174" t="inlineStr"/>
+      <c r="O174" t="inlineStr"/>
+    </row>
+    <row r="175">
+      <c r="A175" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>夜桜さんちの大作戦 第2期 第2クール</t>
+        </is>
+      </c>
+      <c r="D175" t="b">
+        <v>0</v>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="F175" t="n">
+        <v>1</v>
+      </c>
+      <c r="G175" t="inlineStr">
+        <is>
+          <t>What's "KAZOKU"</t>
+        </is>
+      </c>
+      <c r="H175" t="inlineStr">
+        <is>
+          <t>櫻坂46</t>
+        </is>
+      </c>
+      <c r="I175" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=4SdeuouXcWI</t>
+        </is>
+      </c>
+      <c r="J175" t="n">
+        <v>669793</v>
+      </c>
+      <c r="K175" t="inlineStr">
+        <is>
+          <t>櫻坂46 OFFICIAL YouTube CHANNEL</t>
+        </is>
+      </c>
+      <c r="L175" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=AIspds2UVts</t>
+        </is>
+      </c>
+      <c r="M175" t="n">
+        <v>347279</v>
+      </c>
+      <c r="N175" t="inlineStr">
+        <is>
+          <t>NBCUniversal Anime/Music</t>
+        </is>
+      </c>
+      <c r="O175" t="inlineStr">
+        <is>
+          <t>2026-07-07T09:20:03</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>夜桜さんちの大作戦 第2期 第2クール</t>
+        </is>
+      </c>
+      <c r="D176" t="b">
+        <v>0</v>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>ED</t>
+        </is>
+      </c>
+      <c r="F176" t="n">
+        <v>1</v>
+      </c>
+      <c r="G176" t="inlineStr">
+        <is>
           <t>Shalala</t>
         </is>
       </c>
-      <c r="H174" t="inlineStr">
+      <c r="H176" t="inlineStr">
         <is>
           <t>ピラフ星人</t>
         </is>
       </c>
-      <c r="I174" t="inlineStr">
+      <c r="I176" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=X6fNe1uPs9E</t>
         </is>
       </c>
-      <c r="J174" t="n">
+      <c r="J176" t="n">
         <v>369976</v>
       </c>
-      <c r="K174" t="inlineStr">
+      <c r="K176" t="inlineStr">
         <is>
           <t>NBCUniversal Anime/Music</t>
         </is>
       </c>
-      <c r="L174" t="inlineStr">
+      <c r="L176" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=X6fNe1uPs9E</t>
         </is>
       </c>
-      <c r="M174" t="n">
+      <c r="M176" t="n">
         <v>369976</v>
       </c>
-      <c r="N174" t="inlineStr">
+      <c r="N176" t="inlineStr">
         <is>
           <t>NBCUniversal Anime/Music</t>
         </is>
       </c>
-      <c r="O174" t="inlineStr">
+      <c r="O176" t="inlineStr">
         <is>
           <t>2026-07-07T09:20:12</t>
         </is>

</xml_diff>

<commit_message>
auto: anime list update (PC) 2026-07-10
</commit_message>
<xml_diff>
--- a/data/anime_list.xlsx
+++ b/data/anime_list.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M156"/>
+  <dimension ref="A1:M157"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2228,7 +2228,11 @@
           <t>2026年7月8日（水）～ フジテレビ「+Ultra」にて</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr"/>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>UNEND</t>
+        </is>
+      </c>
       <c r="I32" t="inlineStr">
         <is>
           <t>サンダーボルト</t>
@@ -4045,7 +4049,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>2026年7月～ テレ東系列6局ネット「アニもり！」内にて</t>
+          <t>2026年7月12日（日）～ テレ東系列6局ネット「アニもり！」内にて</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
@@ -5066,7 +5070,7 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>領民0人スタートの辺境領主様</t>
+          <t>ラブル＆クルー</t>
         </is>
       </c>
       <c r="E82" t="b">
@@ -5079,37 +5083,17 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>2026年7月10日（金）～ TOKYO MXほか</t>
-        </is>
-      </c>
-      <c r="H82" t="inlineStr">
-        <is>
-          <t>animation studio42</t>
-        </is>
-      </c>
-      <c r="I82" t="inlineStr">
-        <is>
-          <t>Wonder</t>
-        </is>
-      </c>
-      <c r="J82" t="inlineStr">
-        <is>
-          <t>CROWN HEAD</t>
-        </is>
-      </c>
-      <c r="K82" t="inlineStr">
-        <is>
-          <t>星降る夜の約束</t>
-        </is>
-      </c>
-      <c r="L82" t="inlineStr">
-        <is>
-          <t>花耶</t>
-        </is>
-      </c>
+          <t>2026年7月12日（日）～ テレ東系6局ネット「アニもり！」内にて</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr"/>
+      <c r="I82" t="inlineStr"/>
+      <c r="J82" t="inlineStr"/>
+      <c r="K82" t="inlineStr"/>
+      <c r="L82" t="inlineStr"/>
       <c r="M82" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26472</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26683</t>
         </is>
       </c>
     </row>
@@ -5127,7 +5111,7 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>令和のダラさん</t>
+          <t>領民0人スタートの辺境領主様</t>
         </is>
       </c>
       <c r="E83" t="b">
@@ -5140,37 +5124,37 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>2026年7月2日（木）～ AT-X・TOKYO MXほか</t>
+          <t>2026年7月10日（金）～ TOKYO MXほか</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>旭プロダクション</t>
+          <t>animation studio42</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>ダラダラ♡ダンシング</t>
+          <t>Wonder</t>
         </is>
       </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t>ダラさん（CV：田村睦心） 三⼗⽊⾕⽇向（CV：津田美波） 三⼗⽊⾕薫（CV：寺澤百花） ナレーション（CV：てらそままさき）</t>
+          <t>CROWN HEAD</t>
         </is>
       </c>
       <c r="K83" t="inlineStr">
         <is>
-          <t>ひなたぼっこ</t>
+          <t>星降る夜の約束</t>
         </is>
       </c>
       <c r="L83" t="inlineStr">
         <is>
-          <t>REIRIE</t>
+          <t>花耶</t>
         </is>
       </c>
       <c r="M83" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27242</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26472</t>
         </is>
       </c>
     </row>
@@ -5188,7 +5172,7 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>レッツゴー怪奇組</t>
+          <t>令和のダラさん</t>
         </is>
       </c>
       <c r="E84" t="b">
@@ -5201,37 +5185,37 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>2026年7月5日（日）〜 TBS系全国28局ネットにて</t>
+          <t>2026年7月2日（木）～ AT-X・TOKYO MXほか</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>C-Station</t>
+          <t>旭プロダクション</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>気味が悪いんだからねっ</t>
+          <t>ダラダラ♡ダンシング</t>
         </is>
       </c>
       <c r="J84" t="inlineStr">
         <is>
-          <t>SWEET STEADY</t>
+          <t>ダラさん（CV：田村睦心） 三⼗⽊⾕⽇向（CV：津田美波） 三⼗⽊⾕薫（CV：寺澤百花） ナレーション（CV：てらそままさき）</t>
         </is>
       </c>
       <c r="K84" t="inlineStr">
         <is>
-          <t>呪わしてね？</t>
+          <t>ひなたぼっこ</t>
         </is>
       </c>
       <c r="L84" t="inlineStr">
         <is>
-          <t>雨穴</t>
+          <t>REIRIE</t>
         </is>
       </c>
       <c r="M84" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28373</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27242</t>
         </is>
       </c>
     </row>
@@ -5249,7 +5233,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>LV999の村人</t>
+          <t>レッツゴー怪奇組</t>
         </is>
       </c>
       <c r="E85" t="b">
@@ -5262,37 +5246,37 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>2026年7月1日（水）～ テレ東ほか</t>
+          <t>2026年7月5日（日）〜 TBS系全国28局ネットにて</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>ブレインズ・ベース</t>
+          <t>C-Station</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>Not a Hero</t>
+          <t>気味が悪いんだからねっ</t>
         </is>
       </c>
       <c r="J85" t="inlineStr">
         <is>
-          <t>藍月なくる&amp;棗いつき</t>
+          <t>SWEET STEADY</t>
         </is>
       </c>
       <c r="K85" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>呪わしてね？</t>
         </is>
       </c>
       <c r="L85" t="inlineStr">
         <is>
-          <t>ゆきむら。</t>
+          <t>雨穴</t>
         </is>
       </c>
       <c r="M85" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26648</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28373</t>
         </is>
       </c>
     </row>
@@ -5310,7 +5294,7 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>ワールド イズ ダンシング</t>
+          <t>LV999の村人</t>
         </is>
       </c>
       <c r="E86" t="b">
@@ -5323,37 +5307,37 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>2026年7月2日（木）～ TOKYO MX・BS朝日ほか</t>
+          <t>2026年7月1日（水）～ テレ東ほか</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>サイピク</t>
+          <t>ブレインズ・ベース</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>終宵</t>
+          <t>Not a Hero</t>
         </is>
       </c>
       <c r="J86" t="inlineStr">
         <is>
-          <t>マカロニえんぴつ</t>
+          <t>藍月なくる&amp;棗いつき</t>
         </is>
       </c>
       <c r="K86" t="inlineStr">
         <is>
-          <t>名もない花</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="L86" t="inlineStr">
         <is>
-          <t>hockrockb</t>
+          <t>ゆきむら。</t>
         </is>
       </c>
       <c r="M86" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27472</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26648</t>
         </is>
       </c>
     </row>
@@ -5371,7 +5355,7 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>ONE PIECE HEROINES</t>
+          <t>ワールド イズ ダンシング</t>
         </is>
       </c>
       <c r="E87" t="b">
@@ -5384,35 +5368,55 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>2026年7月5日（日） 全国フジテレビ系にて</t>
-        </is>
-      </c>
-      <c r="H87" t="inlineStr"/>
-      <c r="I87" t="inlineStr"/>
-      <c r="J87" t="inlineStr"/>
-      <c r="K87" t="inlineStr"/>
-      <c r="L87" t="inlineStr"/>
+          <t>2026年7月2日（木）～ TOKYO MX・BS朝日ほか</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>サイピク</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>終宵</t>
+        </is>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>マカロニえんぴつ</t>
+        </is>
+      </c>
+      <c r="K87" t="inlineStr">
+        <is>
+          <t>名もない花</t>
+        </is>
+      </c>
+      <c r="L87" t="inlineStr">
+        <is>
+          <t>hockrockb</t>
+        </is>
+      </c>
       <c r="M87" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26606</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27472</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="n">
-        <v>5947</v>
+        <v>5806</v>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>2026秋アニメ</t>
+          <t>2026夏アニメ</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>1</v>
+        <v>87</v>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>アオアシ Season2</t>
+          <t>ONE PIECE HEROINES</t>
         </is>
       </c>
       <c r="E88" t="b">
@@ -5425,21 +5429,17 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>2026年10月4日（日）～ NHK Eテレにて</t>
-        </is>
-      </c>
-      <c r="H88" t="inlineStr">
-        <is>
-          <t>トムス・エンタテインメント</t>
-        </is>
-      </c>
+          <t>2026年7月5日（日） 全国フジテレビ系にて</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr"/>
       <c r="I88" t="inlineStr"/>
       <c r="J88" t="inlineStr"/>
       <c r="K88" t="inlineStr"/>
       <c r="L88" t="inlineStr"/>
       <c r="M88" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25889</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26606</t>
         </is>
       </c>
     </row>
@@ -5453,11 +5453,11 @@
         </is>
       </c>
       <c r="C89" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>アオのハコ 第2期</t>
+          <t>アオアシ Season2</t>
         </is>
       </c>
       <c r="E89" t="b">
@@ -5470,12 +5470,12 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>2026年10月4日（日）～ TBS系にて</t>
+          <t>2026年10月4日（日）～ NHK Eテレにて</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>エレクトリックサーカス</t>
+          <t>トムス・エンタテインメント</t>
         </is>
       </c>
       <c r="I89" t="inlineStr"/>
@@ -5484,7 +5484,7 @@
       <c r="L89" t="inlineStr"/>
       <c r="M89" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25746</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25889</t>
         </is>
       </c>
     </row>
@@ -5498,11 +5498,11 @@
         </is>
       </c>
       <c r="C90" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>おじさんはカワイイものがお好き。</t>
+          <t>アオのハコ 第2期</t>
         </is>
       </c>
       <c r="E90" t="b">
@@ -5515,12 +5515,12 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
+          <t>2026年10月4日（日）～ TBS系にて</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>ライデンフィルム</t>
+          <t>エレクトリックサーカス</t>
         </is>
       </c>
       <c r="I90" t="inlineStr"/>
@@ -5529,7 +5529,7 @@
       <c r="L90" t="inlineStr"/>
       <c r="M90" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27078</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25746</t>
         </is>
       </c>
     </row>
@@ -5543,11 +5543,11 @@
         </is>
       </c>
       <c r="C91" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>カードファイト!! ヴァンガード Divinez 運命星戦編</t>
+          <t>おじさんはカワイイものがお好き。</t>
         </is>
       </c>
       <c r="E91" t="b">
@@ -5560,12 +5560,12 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>2026年11月7日（土）～2026年11月21日（土） テレビ愛知・テレ東系列6局ネットほか 【劇場先行】 2026年10月2日（金）</t>
+          <t>2026年10月～</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>キネマシトラス</t>
+          <t>ライデンフィルム</t>
         </is>
       </c>
       <c r="I91" t="inlineStr"/>
@@ -5574,7 +5574,7 @@
       <c r="L91" t="inlineStr"/>
       <c r="M91" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28214</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27078</t>
         </is>
       </c>
     </row>
@@ -5588,11 +5588,11 @@
         </is>
       </c>
       <c r="C92" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>ガールズ＆パンツァー もっとらぶらぶ作戦です！</t>
+          <t>カードファイト!! ヴァンガード Divinez 運命星戦編</t>
         </is>
       </c>
       <c r="E92" t="b">
@@ -5605,12 +5605,12 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>2026年10月～ TOKYO MX・BS日テレほか</t>
+          <t>2026年11月7日（土）～2026年11月21日（土） テレビ愛知・テレ東系列6局ネットほか 【劇場先行】 2026年10月2日（金）</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>P.A.WORKS</t>
+          <t>キネマシトラス</t>
         </is>
       </c>
       <c r="I92" t="inlineStr"/>
@@ -5619,7 +5619,7 @@
       <c r="L92" t="inlineStr"/>
       <c r="M92" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25683</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28214</t>
         </is>
       </c>
     </row>
@@ -5633,11 +5633,11 @@
         </is>
       </c>
       <c r="C93" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>貸した魔力は【リボ払い】で強制徴収</t>
+          <t>ガールズ＆パンツァー もっとらぶらぶ作戦です！</t>
         </is>
       </c>
       <c r="E93" t="b">
@@ -5650,12 +5650,12 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>2026年10月～ テレビ朝日系ほか</t>
+          <t>2026年10月～ TOKYO MX・BS日テレほか</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>SynergySP</t>
+          <t>P.A.WORKS</t>
         </is>
       </c>
       <c r="I93" t="inlineStr"/>
@@ -5664,7 +5664,7 @@
       <c r="L93" t="inlineStr"/>
       <c r="M93" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27102</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25683</t>
         </is>
       </c>
     </row>
@@ -5678,11 +5678,11 @@
         </is>
       </c>
       <c r="C94" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>仮面ライダーマイス</t>
+          <t>貸した魔力は【リボ払い】で強制徴収</t>
         </is>
       </c>
       <c r="E94" t="b">
@@ -5690,22 +5690,26 @@
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>特撮</t>
+          <t>TVアニメ</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>2026年9月〜 テレビ朝日系列にて</t>
-        </is>
-      </c>
-      <c r="H94" t="inlineStr"/>
+          <t>2026年10月～ テレビ朝日系ほか</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>SynergySP</t>
+        </is>
+      </c>
       <c r="I94" t="inlineStr"/>
       <c r="J94" t="inlineStr"/>
       <c r="K94" t="inlineStr"/>
       <c r="L94" t="inlineStr"/>
       <c r="M94" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28713</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27102</t>
         </is>
       </c>
     </row>
@@ -5719,11 +5723,11 @@
         </is>
       </c>
       <c r="C95" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>帰還者の魔法は特別です 第2期</t>
+          <t>仮面ライダーマイス</t>
         </is>
       </c>
       <c r="E95" t="b">
@@ -5731,42 +5735,22 @@
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>TVアニメ</t>
+          <t>特撮</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>2026年10月〜 フジテレビ「＋Ultra」ほか</t>
-        </is>
-      </c>
-      <c r="H95" t="inlineStr">
-        <is>
-          <t>アルボアニメーション</t>
-        </is>
-      </c>
-      <c r="I95" t="inlineStr">
-        <is>
-          <t>Sorrow</t>
-        </is>
-      </c>
-      <c r="J95" t="inlineStr">
-        <is>
-          <t>FLOW</t>
-        </is>
-      </c>
-      <c r="K95" t="inlineStr">
-        <is>
-          <t>Everlasting</t>
-        </is>
-      </c>
-      <c r="L95" t="inlineStr">
-        <is>
-          <t>krage</t>
-        </is>
-      </c>
+          <t>2026年9月〜 テレビ朝日系列にて</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr"/>
+      <c r="I95" t="inlineStr"/>
+      <c r="J95" t="inlineStr"/>
+      <c r="K95" t="inlineStr"/>
+      <c r="L95" t="inlineStr"/>
       <c r="M95" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=23327</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28713</t>
         </is>
       </c>
     </row>
@@ -5780,11 +5764,11 @@
         </is>
       </c>
       <c r="C96" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>傷だらけ聖女より報復をこめて Season2</t>
+          <t>帰還者の魔法は特別です 第2期</t>
         </is>
       </c>
       <c r="E96" t="b">
@@ -5797,21 +5781,37 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>2026年10月1日（木）〜 テレビ神奈川・CBCテレビにて</t>
+          <t>2026年10月〜 フジテレビ「＋Ultra」ほか</t>
         </is>
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>Imagica Infos</t>
-        </is>
-      </c>
-      <c r="I96" t="inlineStr"/>
-      <c r="J96" t="inlineStr"/>
-      <c r="K96" t="inlineStr"/>
-      <c r="L96" t="inlineStr"/>
+          <t>アルボアニメーション</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>Sorrow</t>
+        </is>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>FLOW</t>
+        </is>
+      </c>
+      <c r="K96" t="inlineStr">
+        <is>
+          <t>Everlasting</t>
+        </is>
+      </c>
+      <c r="L96" t="inlineStr">
+        <is>
+          <t>krage</t>
+        </is>
+      </c>
       <c r="M96" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25118</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=23327</t>
         </is>
       </c>
     </row>
@@ -5825,11 +5825,11 @@
         </is>
       </c>
       <c r="C97" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>恐怖コレクター</t>
+          <t>傷だらけ聖女より報復をこめて Season2</t>
         </is>
       </c>
       <c r="E97" t="b">
@@ -5842,17 +5842,21 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>2026年10月～ NHK総合にて</t>
-        </is>
-      </c>
-      <c r="H97" t="inlineStr"/>
+          <t>2026年10月1日（木）〜 テレビ神奈川・CBCテレビにて</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>Imagica Infos</t>
+        </is>
+      </c>
       <c r="I97" t="inlineStr"/>
       <c r="J97" t="inlineStr"/>
       <c r="K97" t="inlineStr"/>
       <c r="L97" t="inlineStr"/>
       <c r="M97" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27214</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25118</t>
         </is>
       </c>
     </row>
@@ -5866,11 +5870,11 @@
         </is>
       </c>
       <c r="C98" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>凶乱令嬢ニア・リストン 病弱令嬢に転生した神殺しの武人の華麗なる無双録</t>
+          <t>恐怖コレクター</t>
         </is>
       </c>
       <c r="E98" t="b">
@@ -5883,21 +5887,17 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
-        </is>
-      </c>
-      <c r="H98" t="inlineStr">
-        <is>
-          <t>KONAMI animation</t>
-        </is>
-      </c>
+          <t>2026年10月～ NHK総合にて</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr"/>
       <c r="I98" t="inlineStr"/>
       <c r="J98" t="inlineStr"/>
       <c r="K98" t="inlineStr"/>
       <c r="L98" t="inlineStr"/>
       <c r="M98" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27537</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27214</t>
         </is>
       </c>
     </row>
@@ -5911,11 +5911,11 @@
         </is>
       </c>
       <c r="C99" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>薬屋のひとりごと 第3期</t>
+          <t>凶乱令嬢ニア・リストン 病弱令嬢に転生した神殺しの武人の華麗なる無双録</t>
         </is>
       </c>
       <c r="E99" t="b">
@@ -5928,17 +5928,21 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>第1クール：2026年10月～ 第2クール：2027年4月～ 日本テレビ系にて</t>
-        </is>
-      </c>
-      <c r="H99" t="inlineStr"/>
+          <t>2026年10月～</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>KONAMI animation</t>
+        </is>
+      </c>
       <c r="I99" t="inlineStr"/>
       <c r="J99" t="inlineStr"/>
       <c r="K99" t="inlineStr"/>
       <c r="L99" t="inlineStr"/>
       <c r="M99" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26369</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27537</t>
         </is>
       </c>
     </row>
@@ -5952,11 +5956,11 @@
         </is>
       </c>
       <c r="C100" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>ケロロ軍曹☆</t>
+          <t>薬屋のひとりごと 第3期</t>
         </is>
       </c>
       <c r="E100" t="b">
@@ -5969,7 +5973,7 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>2026年秋</t>
+          <t>第1クール：2026年10月～ 第2クール：2027年4月～ 日本テレビ系にて</t>
         </is>
       </c>
       <c r="H100" t="inlineStr"/>
@@ -5979,7 +5983,7 @@
       <c r="L100" t="inlineStr"/>
       <c r="M100" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27337</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26369</t>
         </is>
       </c>
     </row>
@@ -5993,11 +5997,11 @@
         </is>
       </c>
       <c r="C101" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>幻想水滸伝</t>
+          <t>ケロロ軍曹☆</t>
         </is>
       </c>
       <c r="E101" t="b">
@@ -6010,25 +6014,17 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>2026年10月～ TOKYO MX ほか</t>
+          <t>2026年秋</t>
         </is>
       </c>
       <c r="H101" t="inlineStr"/>
-      <c r="I101" t="inlineStr">
-        <is>
-          <t>悲しみさえ大人びて</t>
-        </is>
-      </c>
-      <c r="J101" t="inlineStr">
-        <is>
-          <t>amazarashi</t>
-        </is>
-      </c>
+      <c r="I101" t="inlineStr"/>
+      <c r="J101" t="inlineStr"/>
       <c r="K101" t="inlineStr"/>
       <c r="L101" t="inlineStr"/>
       <c r="M101" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25616</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27337</t>
         </is>
       </c>
     </row>
@@ -6042,11 +6038,11 @@
         </is>
       </c>
       <c r="C102" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>氷の城壁 第2期</t>
+          <t>幻想水滸伝</t>
         </is>
       </c>
       <c r="E102" t="b">
@@ -6059,21 +6055,25 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>2026年10月1日（木）～ TBS系28局にて</t>
-        </is>
-      </c>
-      <c r="H102" t="inlineStr">
-        <is>
-          <t>スタジオKAI</t>
-        </is>
-      </c>
-      <c r="I102" t="inlineStr"/>
-      <c r="J102" t="inlineStr"/>
+          <t>2026年10月～ TOKYO MX ほか</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr"/>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>悲しみさえ大人びて</t>
+        </is>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>amazarashi</t>
+        </is>
+      </c>
       <c r="K102" t="inlineStr"/>
       <c r="L102" t="inlineStr"/>
       <c r="M102" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25508</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25616</t>
         </is>
       </c>
     </row>
@@ -6087,11 +6087,11 @@
         </is>
       </c>
       <c r="C103" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>サイバーパンク：エッジランナーズ2</t>
+          <t>氷の城壁 第2期</t>
         </is>
       </c>
       <c r="E103" t="b">
@@ -6099,17 +6099,17 @@
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>配信</t>
+          <t>TVアニメ</t>
         </is>
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>2026年秋 Netflixにて</t>
+          <t>2026年10月1日（木）～ TBS系28局にて</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>TRIGGER</t>
+          <t>スタジオKAI</t>
         </is>
       </c>
       <c r="I103" t="inlineStr"/>
@@ -6118,7 +6118,7 @@
       <c r="L103" t="inlineStr"/>
       <c r="M103" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28680</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25508</t>
         </is>
       </c>
     </row>
@@ -6132,11 +6132,11 @@
         </is>
       </c>
       <c r="C104" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>PSYREN -サイレン-</t>
+          <t>サイバーパンク：エッジランナーズ2</t>
         </is>
       </c>
       <c r="E104" t="b">
@@ -6144,17 +6144,17 @@
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>TVアニメ</t>
+          <t>配信</t>
         </is>
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>2026年10月～ TOKYO MX・BS11ほか</t>
+          <t>2026年秋 Netflixにて</t>
         </is>
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>サテライト</t>
+          <t>TRIGGER</t>
         </is>
       </c>
       <c r="I104" t="inlineStr"/>
@@ -6163,7 +6163,7 @@
       <c r="L104" t="inlineStr"/>
       <c r="M104" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27257</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28680</t>
         </is>
       </c>
     </row>
@@ -6177,11 +6177,11 @@
         </is>
       </c>
       <c r="C105" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>佐々木とピーちゃん シーズン２</t>
+          <t>PSYREN -サイレン-</t>
         </is>
       </c>
       <c r="E105" t="b">
@@ -6194,12 +6194,12 @@
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
+          <t>2026年10月～ TOKYO MX・BS11ほか</t>
         </is>
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>SILVER LINK.</t>
+          <t>サテライト</t>
         </is>
       </c>
       <c r="I105" t="inlineStr"/>
@@ -6208,7 +6208,7 @@
       <c r="L105" t="inlineStr"/>
       <c r="M105" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=23804</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27257</t>
         </is>
       </c>
     </row>
@@ -6222,11 +6222,11 @@
         </is>
       </c>
       <c r="C106" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>塩対応の佐藤さんが俺にだけ甘い</t>
+          <t>佐々木とピーちゃん シーズン２</t>
         </is>
       </c>
       <c r="E106" t="b">
@@ -6242,14 +6242,18 @@
           <t>2026年10月～</t>
         </is>
       </c>
-      <c r="H106" t="inlineStr"/>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>SILVER LINK.</t>
+        </is>
+      </c>
       <c r="I106" t="inlineStr"/>
       <c r="J106" t="inlineStr"/>
       <c r="K106" t="inlineStr"/>
       <c r="L106" t="inlineStr"/>
       <c r="M106" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27964</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=23804</t>
         </is>
       </c>
     </row>
@@ -6263,11 +6267,11 @@
         </is>
       </c>
       <c r="C107" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>ジャンケットバンク</t>
+          <t>塩対応の佐藤さんが俺にだけ甘い</t>
         </is>
       </c>
       <c r="E107" t="b">
@@ -6283,18 +6287,14 @@
           <t>2026年10月～</t>
         </is>
       </c>
-      <c r="H107" t="inlineStr">
-        <is>
-          <t>CUE</t>
-        </is>
-      </c>
+      <c r="H107" t="inlineStr"/>
       <c r="I107" t="inlineStr"/>
       <c r="J107" t="inlineStr"/>
       <c r="K107" t="inlineStr"/>
       <c r="L107" t="inlineStr"/>
       <c r="M107" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27908</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27964</t>
         </is>
       </c>
     </row>
@@ -6308,11 +6308,11 @@
         </is>
       </c>
       <c r="C108" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>朱色の仮面</t>
+          <t>ジャンケットバンク</t>
         </is>
       </c>
       <c r="E108" t="b">
@@ -6325,17 +6325,21 @@
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>2026年10月～ 読売テレビ・日本テレビ系全国ネットにて</t>
-        </is>
-      </c>
-      <c r="H108" t="inlineStr"/>
+          <t>2026年10月～</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>CUE</t>
+        </is>
+      </c>
       <c r="I108" t="inlineStr"/>
       <c r="J108" t="inlineStr"/>
       <c r="K108" t="inlineStr"/>
       <c r="L108" t="inlineStr"/>
       <c r="M108" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26362</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27908</t>
         </is>
       </c>
     </row>
@@ -6349,11 +6353,11 @@
         </is>
       </c>
       <c r="C109" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>獣王武神ダンデヴァイン</t>
+          <t>朱色の仮面</t>
         </is>
       </c>
       <c r="E109" t="b">
@@ -6366,29 +6370,17 @@
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
-        </is>
-      </c>
-      <c r="H109" t="inlineStr">
-        <is>
-          <t>ライデンフィルム</t>
-        </is>
-      </c>
-      <c r="I109" t="inlineStr">
-        <is>
-          <t>曲名未発表</t>
-        </is>
-      </c>
-      <c r="J109" t="inlineStr">
-        <is>
-          <t>西川貴教</t>
-        </is>
-      </c>
+          <t>2026年10月～ 読売テレビ・日本テレビ系全国ネットにて</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr"/>
+      <c r="I109" t="inlineStr"/>
+      <c r="J109" t="inlineStr"/>
       <c r="K109" t="inlineStr"/>
       <c r="L109" t="inlineStr"/>
       <c r="M109" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28479</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26362</t>
         </is>
       </c>
     </row>
@@ -6402,11 +6394,11 @@
         </is>
       </c>
       <c r="C110" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>しろたん</t>
+          <t>獣王武神ダンデヴァイン</t>
         </is>
       </c>
       <c r="E110" t="b">
@@ -6419,21 +6411,29 @@
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>2026年10月～ テレビ朝日にて</t>
+          <t>2026年10月～</t>
         </is>
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>レスプリ</t>
-        </is>
-      </c>
-      <c r="I110" t="inlineStr"/>
-      <c r="J110" t="inlineStr"/>
+          <t>ライデンフィルム</t>
+        </is>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>曲名未発表</t>
+        </is>
+      </c>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>西川貴教</t>
+        </is>
+      </c>
       <c r="K110" t="inlineStr"/>
       <c r="L110" t="inlineStr"/>
       <c r="M110" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27989</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28479</t>
         </is>
       </c>
     </row>
@@ -6447,11 +6447,11 @@
         </is>
       </c>
       <c r="C111" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>信者ゼロの女神サマと始める異世界攻略</t>
+          <t>しろたん</t>
         </is>
       </c>
       <c r="E111" t="b">
@@ -6464,12 +6464,12 @@
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
+          <t>2026年10月～ テレビ朝日にて</t>
         </is>
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>HORNETS</t>
+          <t>レスプリ</t>
         </is>
       </c>
       <c r="I111" t="inlineStr"/>
@@ -6478,7 +6478,7 @@
       <c r="L111" t="inlineStr"/>
       <c r="M111" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27418</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27989</t>
         </is>
       </c>
     </row>
@@ -6492,11 +6492,11 @@
         </is>
       </c>
       <c r="C112" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>新テニスの王子様 U-17 WORLD CUP 決勝メンバー決定戦</t>
+          <t>信者ゼロの女神サマと始める異世界攻略</t>
         </is>
       </c>
       <c r="E112" t="b">
@@ -6509,17 +6509,21 @@
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>2026年秋</t>
-        </is>
-      </c>
-      <c r="H112" t="inlineStr"/>
+          <t>2026年10月～</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>HORNETS</t>
+        </is>
+      </c>
       <c r="I112" t="inlineStr"/>
       <c r="J112" t="inlineStr"/>
       <c r="K112" t="inlineStr"/>
       <c r="L112" t="inlineStr"/>
       <c r="M112" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26829</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27418</t>
         </is>
       </c>
     </row>
@@ -6533,11 +6537,11 @@
         </is>
       </c>
       <c r="C113" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>スティール・ボール・ラン ジョジョの奇妙な冒険 2nd &amp; 3rd STAGE</t>
+          <t>新テニスの王子様 U-17 WORLD CUP 決勝メンバー決定戦</t>
         </is>
       </c>
       <c r="E113" t="b">
@@ -6545,26 +6549,22 @@
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>配信</t>
+          <t>TVアニメ</t>
         </is>
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>1st STAGE：2026年3月19日（木）～ 2nd&amp;3rd STAGE：2026年9月25日（金）～ Netflixにて</t>
-        </is>
-      </c>
-      <c r="H113" t="inlineStr">
-        <is>
-          <t>david production</t>
-        </is>
-      </c>
+          <t>2026年秋</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr"/>
       <c r="I113" t="inlineStr"/>
       <c r="J113" t="inlineStr"/>
       <c r="K113" t="inlineStr"/>
       <c r="L113" t="inlineStr"/>
       <c r="M113" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25812</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26829</t>
         </is>
       </c>
     </row>
@@ -6578,11 +6578,11 @@
         </is>
       </c>
       <c r="C114" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>生徒会にも穴はある！</t>
+          <t>スティール・ボール・ラン ジョジョの奇妙な冒険 2nd &amp; 3rd STAGE</t>
         </is>
       </c>
       <c r="E114" t="b">
@@ -6590,22 +6590,26 @@
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>TVアニメ</t>
+          <t>配信</t>
         </is>
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
-        </is>
-      </c>
-      <c r="H114" t="inlineStr"/>
+          <t>1st STAGE：2026年3月19日（木）～ 2nd&amp;3rd STAGE：2026年9月25日（金）～ Netflixにて</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>david production</t>
+        </is>
+      </c>
       <c r="I114" t="inlineStr"/>
       <c r="J114" t="inlineStr"/>
       <c r="K114" t="inlineStr"/>
       <c r="L114" t="inlineStr"/>
       <c r="M114" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25874</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25812</t>
         </is>
       </c>
     </row>
@@ -6619,11 +6623,11 @@
         </is>
       </c>
       <c r="C115" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>世界最強の魔女、始めました</t>
+          <t>生徒会にも穴はある！</t>
         </is>
       </c>
       <c r="E115" t="b">
@@ -6639,18 +6643,14 @@
           <t>2026年10月～</t>
         </is>
       </c>
-      <c r="H115" t="inlineStr">
-        <is>
-          <t>ブリッジ</t>
-        </is>
-      </c>
+      <c r="H115" t="inlineStr"/>
       <c r="I115" t="inlineStr"/>
       <c r="J115" t="inlineStr"/>
       <c r="K115" t="inlineStr"/>
       <c r="L115" t="inlineStr"/>
       <c r="M115" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28288</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25874</t>
         </is>
       </c>
     </row>
@@ -6664,11 +6664,11 @@
         </is>
       </c>
       <c r="C116" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>#ゾンビさがしてます</t>
+          <t>世界最強の魔女、始めました</t>
         </is>
       </c>
       <c r="E116" t="b">
@@ -6681,17 +6681,21 @@
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>2026年10月〜 テレビ朝日系にて</t>
-        </is>
-      </c>
-      <c r="H116" t="inlineStr"/>
+          <t>2026年10月～</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>ブリッジ</t>
+        </is>
+      </c>
       <c r="I116" t="inlineStr"/>
       <c r="J116" t="inlineStr"/>
       <c r="K116" t="inlineStr"/>
       <c r="L116" t="inlineStr"/>
       <c r="M116" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26825</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28288</t>
         </is>
       </c>
     </row>
@@ -6705,11 +6709,11 @@
         </is>
       </c>
       <c r="C117" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>ダイヤのA actⅡ -Second Season- 第2クール</t>
+          <t>#ゾンビさがしてます</t>
         </is>
       </c>
       <c r="E117" t="b">
@@ -6722,37 +6726,17 @@
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>第1クール：2026年4月5日（日）～2026年6月28日（日） 第2クール：2026年10月～ テレビ東京ほか</t>
-        </is>
-      </c>
-      <c r="H117" t="inlineStr">
-        <is>
-          <t>OLM</t>
-        </is>
-      </c>
-      <c r="I117" t="inlineStr">
-        <is>
-          <t>Let's Go Crazy</t>
-        </is>
-      </c>
-      <c r="J117" t="inlineStr">
-        <is>
-          <t>Baby Canta</t>
-        </is>
-      </c>
-      <c r="K117" t="inlineStr">
-        <is>
-          <t>NUMBER</t>
-        </is>
-      </c>
-      <c r="L117" t="inlineStr">
-        <is>
-          <t>SUPER★DRAGON</t>
-        </is>
-      </c>
+          <t>2026年10月〜 テレビ朝日系にて</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr"/>
+      <c r="I117" t="inlineStr"/>
+      <c r="J117" t="inlineStr"/>
+      <c r="K117" t="inlineStr"/>
+      <c r="L117" t="inlineStr"/>
       <c r="M117" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=24072</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26825</t>
         </is>
       </c>
     </row>
@@ -6766,11 +6750,11 @@
         </is>
       </c>
       <c r="C118" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>タヌキとキツネ</t>
+          <t>ダイヤのA actⅡ -Second Season- 第2クール</t>
         </is>
       </c>
       <c r="E118" t="b">
@@ -6783,17 +6767,37 @@
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
-        </is>
-      </c>
-      <c r="H118" t="inlineStr"/>
-      <c r="I118" t="inlineStr"/>
-      <c r="J118" t="inlineStr"/>
-      <c r="K118" t="inlineStr"/>
-      <c r="L118" t="inlineStr"/>
+          <t>第1クール：2026年4月5日（日）～2026年6月28日（日） 第2クール：2026年10月～ テレビ東京ほか</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>OLM</t>
+        </is>
+      </c>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>Let's Go Crazy</t>
+        </is>
+      </c>
+      <c r="J118" t="inlineStr">
+        <is>
+          <t>Baby Canta</t>
+        </is>
+      </c>
+      <c r="K118" t="inlineStr">
+        <is>
+          <t>NUMBER</t>
+        </is>
+      </c>
+      <c r="L118" t="inlineStr">
+        <is>
+          <t>SUPER★DRAGON</t>
+        </is>
+      </c>
       <c r="M118" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=6380</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=24072</t>
         </is>
       </c>
     </row>
@@ -6807,11 +6811,11 @@
         </is>
       </c>
       <c r="C119" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>TANK CHAIR-戦車椅子-</t>
+          <t>タヌキとキツネ</t>
         </is>
       </c>
       <c r="E119" t="b">
@@ -6824,21 +6828,17 @@
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>2026年秋</t>
-        </is>
-      </c>
-      <c r="H119" t="inlineStr">
-        <is>
-          <t>ポリゴン・ピクチュアズ</t>
-        </is>
-      </c>
+          <t>2026年10月～</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr"/>
       <c r="I119" t="inlineStr"/>
       <c r="J119" t="inlineStr"/>
       <c r="K119" t="inlineStr"/>
       <c r="L119" t="inlineStr"/>
       <c r="M119" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27965</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=6380</t>
         </is>
       </c>
     </row>
@@ -6852,11 +6852,11 @@
         </is>
       </c>
       <c r="C120" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>探偵はもう、死んでいる。Season2</t>
+          <t>TANK CHAIR-戦車椅子-</t>
         </is>
       </c>
       <c r="E120" t="b">
@@ -6869,12 +6869,12 @@
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>2026年10月〜</t>
+          <t>2026年秋</t>
         </is>
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>ENGI</t>
+          <t>ポリゴン・ピクチュアズ</t>
         </is>
       </c>
       <c r="I120" t="inlineStr"/>
@@ -6883,7 +6883,7 @@
       <c r="L120" t="inlineStr"/>
       <c r="M120" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=16348</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27965</t>
         </is>
       </c>
     </row>
@@ -6897,11 +6897,11 @@
         </is>
       </c>
       <c r="C121" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>超巡！超条先輩</t>
+          <t>探偵はもう、死んでいる。Season2</t>
         </is>
       </c>
       <c r="E121" t="b">
@@ -6914,12 +6914,12 @@
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>2026年10月～ カンテレ・フジテレビ系全国ネットにて</t>
+          <t>2026年10月〜</t>
         </is>
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>アルボアニメーション</t>
+          <t>ENGI</t>
         </is>
       </c>
       <c r="I121" t="inlineStr"/>
@@ -6928,7 +6928,7 @@
       <c r="L121" t="inlineStr"/>
       <c r="M121" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26933</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=16348</t>
         </is>
       </c>
     </row>
@@ -6942,11 +6942,11 @@
         </is>
       </c>
       <c r="C122" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>追放されたチート付与魔術師は気ままなセカンドライフを謳歌する。</t>
+          <t>超巡！超条先輩</t>
         </is>
       </c>
       <c r="E122" t="b">
@@ -6959,12 +6959,12 @@
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>2026年10月～ テレ東系列にて</t>
+          <t>2026年10月～ カンテレ・フジテレビ系全国ネットにて</t>
         </is>
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>P.A.WORKS</t>
+          <t>アルボアニメーション</t>
         </is>
       </c>
       <c r="I122" t="inlineStr"/>
@@ -6973,7 +6973,7 @@
       <c r="L122" t="inlineStr"/>
       <c r="M122" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27631</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26933</t>
         </is>
       </c>
     </row>
@@ -6987,11 +6987,11 @@
         </is>
       </c>
       <c r="C123" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>てつりょー！meet with 鉄道むすめ</t>
+          <t>追放されたチート付与魔術師は気ままなセカンドライフを謳歌する。</t>
         </is>
       </c>
       <c r="E123" t="b">
@@ -7004,12 +7004,12 @@
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t>2026年秋</t>
+          <t>2026年10月～ テレ東系列にて</t>
         </is>
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>イーストフィッシュスタジオ</t>
+          <t>P.A.WORKS</t>
         </is>
       </c>
       <c r="I123" t="inlineStr"/>
@@ -7018,7 +7018,7 @@
       <c r="L123" t="inlineStr"/>
       <c r="M123" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26895</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27631</t>
         </is>
       </c>
     </row>
@@ -7032,11 +7032,11 @@
         </is>
       </c>
       <c r="C124" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>テムパル～アイテムの力～</t>
+          <t>てつりょー！meet with 鉄道むすめ</t>
         </is>
       </c>
       <c r="E124" t="b">
@@ -7049,12 +7049,12 @@
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
+          <t>2026年秋</t>
         </is>
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>J.C.STAFF</t>
+          <t>イーストフィッシュスタジオ</t>
         </is>
       </c>
       <c r="I124" t="inlineStr"/>
@@ -7063,7 +7063,7 @@
       <c r="L124" t="inlineStr"/>
       <c r="M124" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28478</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26895</t>
         </is>
       </c>
     </row>
@@ -7077,11 +7077,11 @@
         </is>
       </c>
       <c r="C125" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>デモンズ・クレスト</t>
+          <t>テムパル～アイテムの力～</t>
         </is>
       </c>
       <c r="E125" t="b">
@@ -7089,34 +7089,26 @@
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>配信</t>
+          <t>TVアニメ</t>
         </is>
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>2026年11月6日（金） Prime Videoにて</t>
+          <t>2026年10月～</t>
         </is>
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>Production I.G</t>
-        </is>
-      </c>
-      <c r="I125" t="inlineStr">
-        <is>
-          <t>シンカ</t>
-        </is>
-      </c>
-      <c r="J125" t="inlineStr">
-        <is>
-          <t>Ado</t>
-        </is>
-      </c>
+          <t>J.C.STAFF</t>
+        </is>
+      </c>
+      <c r="I125" t="inlineStr"/>
+      <c r="J125" t="inlineStr"/>
       <c r="K125" t="inlineStr"/>
       <c r="L125" t="inlineStr"/>
       <c r="M125" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27189</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28478</t>
         </is>
       </c>
     </row>
@@ -7130,11 +7122,11 @@
         </is>
       </c>
       <c r="C126" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>転生貴族、鑑定スキルで成り上がる 第3期</t>
+          <t>デモンズ・クレスト</t>
         </is>
       </c>
       <c r="E126" t="b">
@@ -7142,26 +7134,34 @@
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>TVアニメ</t>
+          <t>配信</t>
         </is>
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t>2026年秋 CBC/TBS系全国28局ネット「アガルアニメ」にて</t>
+          <t>2026年11月6日（金） Prime Videoにて</t>
         </is>
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>studio MOTHER</t>
-        </is>
-      </c>
-      <c r="I126" t="inlineStr"/>
-      <c r="J126" t="inlineStr"/>
+          <t>Production I.G</t>
+        </is>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>シンカ</t>
+        </is>
+      </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>Ado</t>
+        </is>
+      </c>
       <c r="K126" t="inlineStr"/>
       <c r="L126" t="inlineStr"/>
       <c r="M126" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25385</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27189</t>
         </is>
       </c>
     </row>
@@ -7175,11 +7175,11 @@
         </is>
       </c>
       <c r="C127" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>転生ゴブリンだけど質問ある？</t>
+          <t>転生貴族、鑑定スキルで成り上がる 第3期</t>
         </is>
       </c>
       <c r="E127" t="b">
@@ -7192,12 +7192,12 @@
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
+          <t>2026年秋 CBC/TBS系全国28局ネット「アガルアニメ」にて</t>
         </is>
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>BAKKKA</t>
+          <t>studio MOTHER</t>
         </is>
       </c>
       <c r="I127" t="inlineStr"/>
@@ -7206,7 +7206,7 @@
       <c r="L127" t="inlineStr"/>
       <c r="M127" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27909</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25385</t>
         </is>
       </c>
     </row>
@@ -7220,11 +7220,11 @@
         </is>
       </c>
       <c r="C128" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>転生した大聖女は、聖女であることをひた隠す</t>
+          <t>転生ゴブリンだけど質問ある？</t>
         </is>
       </c>
       <c r="E128" t="b">
@@ -7242,32 +7242,16 @@
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>FelixFilm</t>
-        </is>
-      </c>
-      <c r="I128" t="inlineStr">
-        <is>
-          <t>Flare of Soul</t>
-        </is>
-      </c>
-      <c r="J128" t="inlineStr">
-        <is>
-          <t>花耶</t>
-        </is>
-      </c>
-      <c r="K128" t="inlineStr">
-        <is>
-          <t>STELLAR</t>
-        </is>
-      </c>
-      <c r="L128" t="inlineStr">
-        <is>
-          <t>ウタヒメドリーム オールスターズ</t>
-        </is>
-      </c>
+          <t>BAKKKA</t>
+        </is>
+      </c>
+      <c r="I128" t="inlineStr"/>
+      <c r="J128" t="inlineStr"/>
+      <c r="K128" t="inlineStr"/>
+      <c r="L128" t="inlineStr"/>
       <c r="M128" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25630</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27909</t>
         </is>
       </c>
     </row>
@@ -7281,11 +7265,11 @@
         </is>
       </c>
       <c r="C129" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>転生したら剣でした 第2期</t>
+          <t>転生した大聖女は、聖女であることをひた隠す</t>
         </is>
       </c>
       <c r="E129" t="b">
@@ -7303,16 +7287,32 @@
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>C2C</t>
-        </is>
-      </c>
-      <c r="I129" t="inlineStr"/>
-      <c r="J129" t="inlineStr"/>
-      <c r="K129" t="inlineStr"/>
-      <c r="L129" t="inlineStr"/>
+          <t>FelixFilm</t>
+        </is>
+      </c>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>Flare of Soul</t>
+        </is>
+      </c>
+      <c r="J129" t="inlineStr">
+        <is>
+          <t>花耶</t>
+        </is>
+      </c>
+      <c r="K129" t="inlineStr">
+        <is>
+          <t>STELLAR</t>
+        </is>
+      </c>
+      <c r="L129" t="inlineStr">
+        <is>
+          <t>ウタヒメドリーム オールスターズ</t>
+        </is>
+      </c>
       <c r="M129" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=19149</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25630</t>
         </is>
       </c>
     </row>
@@ -7326,11 +7326,11 @@
         </is>
       </c>
       <c r="C130" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>とある暗部の少女共棲</t>
+          <t>転生したら剣でした 第2期</t>
         </is>
       </c>
       <c r="E130" t="b">
@@ -7343,37 +7343,21 @@
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>2026年10月9日（金）～ TOKYO MXほか</t>
+          <t>2026年10月～</t>
         </is>
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>J.C.STAFF</t>
-        </is>
-      </c>
-      <c r="I130" t="inlineStr">
-        <is>
-          <t>Ghost Sequence</t>
-        </is>
-      </c>
-      <c r="J130" t="inlineStr">
-        <is>
-          <t>East Of Eden</t>
-        </is>
-      </c>
-      <c r="K130" t="inlineStr">
-        <is>
-          <t>原子崩し(メルトダウナー)</t>
-        </is>
-      </c>
-      <c r="L130" t="inlineStr">
-        <is>
-          <t>岸田教団&amp;THE明星ロケッツ</t>
-        </is>
-      </c>
+          <t>C2C</t>
+        </is>
+      </c>
+      <c r="I130" t="inlineStr"/>
+      <c r="J130" t="inlineStr"/>
+      <c r="K130" t="inlineStr"/>
+      <c r="L130" t="inlineStr"/>
       <c r="M130" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25552</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=19149</t>
         </is>
       </c>
     </row>
@@ -7387,11 +7371,11 @@
         </is>
       </c>
       <c r="C131" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>東京リベンジャーズ 三天戦争編</t>
+          <t>とある暗部の少女共棲</t>
         </is>
       </c>
       <c r="E131" t="b">
@@ -7404,21 +7388,37 @@
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>2026年10月2日（金）～ MBS・TBS・CBC”アニメイズム”枠ほか</t>
+          <t>2026年10月9日（金）～ TOKYO MXほか</t>
         </is>
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>ライデンフィルム</t>
-        </is>
-      </c>
-      <c r="I131" t="inlineStr"/>
-      <c r="J131" t="inlineStr"/>
-      <c r="K131" t="inlineStr"/>
-      <c r="L131" t="inlineStr"/>
+          <t>J.C.STAFF</t>
+        </is>
+      </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>Ghost Sequence</t>
+        </is>
+      </c>
+      <c r="J131" t="inlineStr">
+        <is>
+          <t>East Of Eden</t>
+        </is>
+      </c>
+      <c r="K131" t="inlineStr">
+        <is>
+          <t>原子崩し(メルトダウナー)</t>
+        </is>
+      </c>
+      <c r="L131" t="inlineStr">
+        <is>
+          <t>岸田教団&amp;THE明星ロケッツ</t>
+        </is>
+      </c>
       <c r="M131" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=24207</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25552</t>
         </is>
       </c>
     </row>
@@ -7432,11 +7432,11 @@
         </is>
       </c>
       <c r="C132" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>桃源暗鬼 ～日光・華厳の滝編～</t>
+          <t>東京リベンジャーズ 三天戦争編</t>
         </is>
       </c>
       <c r="E132" t="b">
@@ -7449,17 +7449,21 @@
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>2026年10月～ 日本テレビ系「FRIDAY ANIME NIGHT（フラアニ）」枠にて</t>
-        </is>
-      </c>
-      <c r="H132" t="inlineStr"/>
+          <t>2026年10月2日（金）～ MBS・TBS・CBC”アニメイズム”枠ほか</t>
+        </is>
+      </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>ライデンフィルム</t>
+        </is>
+      </c>
       <c r="I132" t="inlineStr"/>
       <c r="J132" t="inlineStr"/>
       <c r="K132" t="inlineStr"/>
       <c r="L132" t="inlineStr"/>
       <c r="M132" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27376</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=24207</t>
         </is>
       </c>
     </row>
@@ -7473,11 +7477,11 @@
         </is>
       </c>
       <c r="C133" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>どうも、好きな人に惚れ薬を依頼された魔女です。</t>
+          <t>桃源暗鬼 ～日光・華厳の滝編～</t>
         </is>
       </c>
       <c r="E133" t="b">
@@ -7490,21 +7494,17 @@
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
-        </is>
-      </c>
-      <c r="H133" t="inlineStr">
-        <is>
-          <t>ディオメディア</t>
-        </is>
-      </c>
+          <t>2026年10月～ 日本テレビ系「FRIDAY ANIME NIGHT（フラアニ）」枠にて</t>
+        </is>
+      </c>
+      <c r="H133" t="inlineStr"/>
       <c r="I133" t="inlineStr"/>
       <c r="J133" t="inlineStr"/>
       <c r="K133" t="inlineStr"/>
       <c r="L133" t="inlineStr"/>
       <c r="M133" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27581</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27376</t>
         </is>
       </c>
     </row>
@@ -7518,11 +7518,11 @@
         </is>
       </c>
       <c r="C134" t="n">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>ドラゴンボール超 ビルス</t>
+          <t>どうも、好きな人に惚れ薬を依頼された魔女です。</t>
         </is>
       </c>
       <c r="E134" t="b">
@@ -7535,17 +7535,21 @@
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>2026年秋 フジテレビにて</t>
-        </is>
-      </c>
-      <c r="H134" t="inlineStr"/>
+          <t>2026年10月～</t>
+        </is>
+      </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>ディオメディア</t>
+        </is>
+      </c>
       <c r="I134" t="inlineStr"/>
       <c r="J134" t="inlineStr"/>
       <c r="K134" t="inlineStr"/>
       <c r="L134" t="inlineStr"/>
       <c r="M134" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27491</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27581</t>
         </is>
       </c>
     </row>
@@ -7559,11 +7563,11 @@
         </is>
       </c>
       <c r="C135" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>鳴海の平日</t>
+          <t>ドラゴンボール超 ビルス</t>
         </is>
       </c>
       <c r="E135" t="b">
@@ -7571,26 +7575,22 @@
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>配信</t>
+          <t>TVアニメ</t>
         </is>
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>2026年秋</t>
-        </is>
-      </c>
-      <c r="H135" t="inlineStr">
-        <is>
-          <t>Production I.G</t>
-        </is>
-      </c>
+          <t>2026年秋 フジテレビにて</t>
+        </is>
+      </c>
+      <c r="H135" t="inlineStr"/>
       <c r="I135" t="inlineStr"/>
       <c r="J135" t="inlineStr"/>
       <c r="K135" t="inlineStr"/>
       <c r="L135" t="inlineStr"/>
       <c r="M135" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28465</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27491</t>
         </is>
       </c>
     </row>
@@ -7604,11 +7604,11 @@
         </is>
       </c>
       <c r="C136" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>バーテックスフォース</t>
+          <t>鳴海の平日</t>
         </is>
       </c>
       <c r="E136" t="b">
@@ -7616,17 +7616,17 @@
       </c>
       <c r="F136" t="inlineStr">
         <is>
-          <t>TVアニメ</t>
+          <t>配信</t>
         </is>
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>2026年10月〜</t>
+          <t>2026年秋</t>
         </is>
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>SMDE</t>
+          <t>Production I.G</t>
         </is>
       </c>
       <c r="I136" t="inlineStr"/>
@@ -7635,7 +7635,7 @@
       <c r="L136" t="inlineStr"/>
       <c r="M136" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27988</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28465</t>
         </is>
       </c>
     </row>
@@ -7649,11 +7649,11 @@
         </is>
       </c>
       <c r="C137" t="n">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>Battle Spirits [Re] 絶界の空</t>
+          <t>バーテックスフォース</t>
         </is>
       </c>
       <c r="E137" t="b">
@@ -7666,17 +7666,21 @@
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>2026年秋</t>
-        </is>
-      </c>
-      <c r="H137" t="inlineStr"/>
+          <t>2026年10月〜</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>SMDE</t>
+        </is>
+      </c>
       <c r="I137" t="inlineStr"/>
       <c r="J137" t="inlineStr"/>
       <c r="K137" t="inlineStr"/>
       <c r="L137" t="inlineStr"/>
       <c r="M137" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27954</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27988</t>
         </is>
       </c>
     </row>
@@ -7690,11 +7694,11 @@
         </is>
       </c>
       <c r="C138" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>パンどろぼう</t>
+          <t>Battle Spirits [Re] 絶界の空</t>
         </is>
       </c>
       <c r="E138" t="b">
@@ -7707,7 +7711,7 @@
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t>2026年10月〜 NHK Eテレにて</t>
+          <t>2026年秋</t>
         </is>
       </c>
       <c r="H138" t="inlineStr"/>
@@ -7717,7 +7721,7 @@
       <c r="L138" t="inlineStr"/>
       <c r="M138" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26163</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27954</t>
         </is>
       </c>
     </row>
@@ -7731,11 +7735,11 @@
         </is>
       </c>
       <c r="C139" t="n">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>百妖譜 京師篇</t>
+          <t>パンどろぼう</t>
         </is>
       </c>
       <c r="E139" t="b">
@@ -7748,7 +7752,7 @@
       </c>
       <c r="G139" t="inlineStr">
         <is>
-          <t>2026年10月〜 フジテレビ「B8station」にて</t>
+          <t>2026年10月〜 NHK Eテレにて</t>
         </is>
       </c>
       <c r="H139" t="inlineStr"/>
@@ -7758,7 +7762,7 @@
       <c r="L139" t="inlineStr"/>
       <c r="M139" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27781</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26163</t>
         </is>
       </c>
     </row>
@@ -7772,11 +7776,11 @@
         </is>
       </c>
       <c r="C140" t="n">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>冰剣の魔術師が世界を統べるⅡ</t>
+          <t>百妖譜 京師篇</t>
         </is>
       </c>
       <c r="E140" t="b">
@@ -7789,21 +7793,17 @@
       </c>
       <c r="G140" t="inlineStr">
         <is>
-          <t>2026年10月〜</t>
-        </is>
-      </c>
-      <c r="H140" t="inlineStr">
-        <is>
-          <t>ゼロジー</t>
-        </is>
-      </c>
+          <t>2026年10月〜 フジテレビ「B8station」にて</t>
+        </is>
+      </c>
+      <c r="H140" t="inlineStr"/>
       <c r="I140" t="inlineStr"/>
       <c r="J140" t="inlineStr"/>
       <c r="K140" t="inlineStr"/>
       <c r="L140" t="inlineStr"/>
       <c r="M140" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28403</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27781</t>
         </is>
       </c>
     </row>
@@ -7817,11 +7817,11 @@
         </is>
       </c>
       <c r="C141" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>ブラッククローバー 2nd Season</t>
+          <t>冰剣の魔術師が世界を統べるⅡ</t>
         </is>
       </c>
       <c r="E141" t="b">
@@ -7834,29 +7834,21 @@
       </c>
       <c r="G141" t="inlineStr">
         <is>
-          <t>2026年10月～ テレ東系列ほか</t>
+          <t>2026年10月〜</t>
         </is>
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>スタジオぴえろ</t>
-        </is>
-      </c>
-      <c r="I141" t="inlineStr">
-        <is>
-          <t>消えない理由</t>
-        </is>
-      </c>
-      <c r="J141" t="inlineStr">
-        <is>
-          <t>WANIMA</t>
-        </is>
-      </c>
+          <t>ゼロジー</t>
+        </is>
+      </c>
+      <c r="I141" t="inlineStr"/>
+      <c r="J141" t="inlineStr"/>
       <c r="K141" t="inlineStr"/>
       <c r="L141" t="inlineStr"/>
       <c r="M141" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26361</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28403</t>
         </is>
       </c>
     </row>
@@ -7870,11 +7862,11 @@
         </is>
       </c>
       <c r="C142" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>ホタルの嫁入り</t>
+          <t>ブラッククローバー 2nd Season</t>
         </is>
       </c>
       <c r="E142" t="b">
@@ -7887,21 +7879,29 @@
       </c>
       <c r="G142" t="inlineStr">
         <is>
-          <t>2026年10月～ 全国フジテレビ系“ ノイタミナ ”にて</t>
+          <t>2026年10月～ テレ東系列ほか</t>
         </is>
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>david production</t>
-        </is>
-      </c>
-      <c r="I142" t="inlineStr"/>
-      <c r="J142" t="inlineStr"/>
+          <t>スタジオぴえろ</t>
+        </is>
+      </c>
+      <c r="I142" t="inlineStr">
+        <is>
+          <t>消えない理由</t>
+        </is>
+      </c>
+      <c r="J142" t="inlineStr">
+        <is>
+          <t>WANIMA</t>
+        </is>
+      </c>
       <c r="K142" t="inlineStr"/>
       <c r="L142" t="inlineStr"/>
       <c r="M142" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27415</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26361</t>
         </is>
       </c>
     </row>
@@ -7915,11 +7915,11 @@
         </is>
       </c>
       <c r="C143" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>ポップパップポルターズ</t>
+          <t>ホタルの嫁入り</t>
         </is>
       </c>
       <c r="E143" t="b">
@@ -7932,12 +7932,12 @@
       </c>
       <c r="G143" t="inlineStr">
         <is>
-          <t>2026年10月～ テレビ朝日「PicoAniTime」にて</t>
+          <t>2026年10月～ 全国フジテレビ系“ ノイタミナ ”にて</t>
         </is>
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>MOZU STUDIOS</t>
+          <t>david production</t>
         </is>
       </c>
       <c r="I143" t="inlineStr"/>
@@ -7946,7 +7946,7 @@
       <c r="L143" t="inlineStr"/>
       <c r="M143" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27823</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27415</t>
         </is>
       </c>
     </row>
@@ -7960,11 +7960,11 @@
         </is>
       </c>
       <c r="C144" t="n">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>ホテル・インヒューマンズ 第2期</t>
+          <t>ポップパップポルターズ</t>
         </is>
       </c>
       <c r="E144" t="b">
@@ -7977,12 +7977,12 @@
       </c>
       <c r="G144" t="inlineStr">
         <is>
-          <t>2026年10月～ テレ東系列ほか</t>
+          <t>2026年10月～ テレビ朝日「PicoAniTime」にて</t>
         </is>
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>ブリッジ</t>
+          <t>MOZU STUDIOS</t>
         </is>
       </c>
       <c r="I144" t="inlineStr"/>
@@ -7991,7 +7991,7 @@
       <c r="L144" t="inlineStr"/>
       <c r="M144" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26870</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27823</t>
         </is>
       </c>
     </row>
@@ -8005,11 +8005,11 @@
         </is>
       </c>
       <c r="C145" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>マジカル★エクスプローラー</t>
+          <t>ホテル・インヒューマンズ 第2期</t>
         </is>
       </c>
       <c r="E145" t="b">
@@ -8022,12 +8022,12 @@
       </c>
       <c r="G145" t="inlineStr">
         <is>
-          <t>2026年秋</t>
+          <t>2026年10月～ テレ東系列ほか</t>
         </is>
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>WHITE FOX</t>
+          <t>ブリッジ</t>
         </is>
       </c>
       <c r="I145" t="inlineStr"/>
@@ -8036,7 +8036,7 @@
       <c r="L145" t="inlineStr"/>
       <c r="M145" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=23375</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26870</t>
         </is>
       </c>
     </row>
@@ -8050,11 +8050,11 @@
         </is>
       </c>
       <c r="C146" t="n">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>魔法騎士レイアース</t>
+          <t>マジカル★エクスプローラー</t>
         </is>
       </c>
       <c r="E146" t="b">
@@ -8067,12 +8067,12 @@
       </c>
       <c r="G146" t="inlineStr">
         <is>
-          <t>2026年10月7日（水）～ テレビ朝日系列にて</t>
+          <t>2026年秋</t>
         </is>
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>E&amp;H production</t>
+          <t>WHITE FOX</t>
         </is>
       </c>
       <c r="I146" t="inlineStr"/>
@@ -8081,7 +8081,7 @@
       <c r="L146" t="inlineStr"/>
       <c r="M146" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=24301</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=23375</t>
         </is>
       </c>
     </row>
@@ -8095,11 +8095,11 @@
         </is>
       </c>
       <c r="C147" t="n">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>魔法少女育成計画restart</t>
+          <t>魔法騎士レイアース</t>
         </is>
       </c>
       <c r="E147" t="b">
@@ -8112,29 +8112,21 @@
       </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t>2026年秋</t>
+          <t>2026年10月7日（水）～ テレビ朝日系列にて</t>
         </is>
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>SynergySP</t>
-        </is>
-      </c>
-      <c r="I147" t="inlineStr">
-        <is>
-          <t>No tears here</t>
-        </is>
-      </c>
-      <c r="J147" t="inlineStr">
-        <is>
-          <t>茅原実里</t>
-        </is>
-      </c>
+          <t>E&amp;H production</t>
+        </is>
+      </c>
+      <c r="I147" t="inlineStr"/>
+      <c r="J147" t="inlineStr"/>
       <c r="K147" t="inlineStr"/>
       <c r="L147" t="inlineStr"/>
       <c r="M147" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26693</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=24301</t>
         </is>
       </c>
     </row>
@@ -8148,11 +8140,11 @@
         </is>
       </c>
       <c r="C148" t="n">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>魔法の姉妹ルルットリリィ 第2クール</t>
+          <t>魔法少女育成計画restart</t>
         </is>
       </c>
       <c r="E148" t="b">
@@ -8165,37 +8157,29 @@
       </c>
       <c r="G148" t="inlineStr">
         <is>
-          <t>第1クール：2026年4月5日（日）～2026年6月21日（日） 第2クール：2026年10月～ TOKYO MX・ABCテレビほか</t>
+          <t>2026年秋</t>
         </is>
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>スタジオぴえろ</t>
+          <t>SynergySP</t>
         </is>
       </c>
       <c r="I148" t="inlineStr">
         <is>
-          <t>Bubee</t>
+          <t>No tears here</t>
         </is>
       </c>
       <c r="J148" t="inlineStr">
         <is>
-          <t>ILLIT</t>
-        </is>
-      </c>
-      <c r="K148" t="inlineStr">
-        <is>
-          <t>Calling</t>
-        </is>
-      </c>
-      <c r="L148" t="inlineStr">
-        <is>
-          <t>ルルットリリィ（こんぺとリリィ（CV.橘めい）、ましゅールル（CV.小鹿なお））</t>
-        </is>
-      </c>
+          <t>茅原実里</t>
+        </is>
+      </c>
+      <c r="K148" t="inlineStr"/>
+      <c r="L148" t="inlineStr"/>
       <c r="M148" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=24293</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26693</t>
         </is>
       </c>
     </row>
@@ -8209,11 +8193,11 @@
         </is>
       </c>
       <c r="C149" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>マロニエ王国の七人の騎士</t>
+          <t>魔法の姉妹ルルットリリィ 第2クール</t>
         </is>
       </c>
       <c r="E149" t="b">
@@ -8226,21 +8210,37 @@
       </c>
       <c r="G149" t="inlineStr">
         <is>
-          <t>2026年10月～ NHK Eテレにて</t>
+          <t>第1クール：2026年4月5日（日）～2026年6月21日（日） 第2クール：2026年10月～ TOKYO MX・ABCテレビほか</t>
         </is>
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>J.C.STAFF</t>
-        </is>
-      </c>
-      <c r="I149" t="inlineStr"/>
-      <c r="J149" t="inlineStr"/>
-      <c r="K149" t="inlineStr"/>
-      <c r="L149" t="inlineStr"/>
+          <t>スタジオぴえろ</t>
+        </is>
+      </c>
+      <c r="I149" t="inlineStr">
+        <is>
+          <t>Bubee</t>
+        </is>
+      </c>
+      <c r="J149" t="inlineStr">
+        <is>
+          <t>ILLIT</t>
+        </is>
+      </c>
+      <c r="K149" t="inlineStr">
+        <is>
+          <t>Calling</t>
+        </is>
+      </c>
+      <c r="L149" t="inlineStr">
+        <is>
+          <t>ルルットリリィ（こんぺとリリィ（CV.橘めい）、ましゅールル（CV.小鹿なお））</t>
+        </is>
+      </c>
       <c r="M149" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28456</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=24293</t>
         </is>
       </c>
     </row>
@@ -8254,11 +8254,11 @@
         </is>
       </c>
       <c r="C150" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>目覚めたら最強装備と宇宙船持ちだったので、一戸建て目指して傭兵として自由に生きたい</t>
+          <t>マロニエ王国の七人の騎士</t>
         </is>
       </c>
       <c r="E150" t="b">
@@ -8271,37 +8271,21 @@
       </c>
       <c r="G150" t="inlineStr">
         <is>
-          <t>2026年10月〜 TOKYO MX・読売テレビ・中京テレビほか</t>
+          <t>2026年10月～ NHK Eテレにて</t>
         </is>
       </c>
       <c r="H150" t="inlineStr">
         <is>
-          <t>studio A-CAT</t>
-        </is>
-      </c>
-      <c r="I150" t="inlineStr">
-        <is>
-          <t>UNSTOPPABLE</t>
-        </is>
-      </c>
-      <c r="J150" t="inlineStr">
-        <is>
-          <t>FLOW</t>
-        </is>
-      </c>
-      <c r="K150" t="inlineStr">
-        <is>
-          <t>MY WAY</t>
-        </is>
-      </c>
-      <c r="L150" t="inlineStr">
-        <is>
-          <t>ASTERISM</t>
-        </is>
-      </c>
+          <t>J.C.STAFF</t>
+        </is>
+      </c>
+      <c r="I150" t="inlineStr"/>
+      <c r="J150" t="inlineStr"/>
+      <c r="K150" t="inlineStr"/>
+      <c r="L150" t="inlineStr"/>
       <c r="M150" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25525</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28456</t>
         </is>
       </c>
     </row>
@@ -8315,11 +8299,11 @@
         </is>
       </c>
       <c r="C151" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>ゆるゆる図鑑</t>
+          <t>目覚めたら最強装備と宇宙船持ちだったので、一戸建て目指して傭兵として自由に生きたい</t>
         </is>
       </c>
       <c r="E151" t="b">
@@ -8332,17 +8316,37 @@
       </c>
       <c r="G151" t="inlineStr">
         <is>
-          <t>2026年10月～ テレ東系列6局ネット「アニもり！」内にて</t>
-        </is>
-      </c>
-      <c r="H151" t="inlineStr"/>
-      <c r="I151" t="inlineStr"/>
-      <c r="J151" t="inlineStr"/>
-      <c r="K151" t="inlineStr"/>
-      <c r="L151" t="inlineStr"/>
+          <t>2026年10月〜 TOKYO MX・読売テレビ・中京テレビほか</t>
+        </is>
+      </c>
+      <c r="H151" t="inlineStr">
+        <is>
+          <t>studio A-CAT</t>
+        </is>
+      </c>
+      <c r="I151" t="inlineStr">
+        <is>
+          <t>UNSTOPPABLE</t>
+        </is>
+      </c>
+      <c r="J151" t="inlineStr">
+        <is>
+          <t>FLOW</t>
+        </is>
+      </c>
+      <c r="K151" t="inlineStr">
+        <is>
+          <t>MY WAY</t>
+        </is>
+      </c>
+      <c r="L151" t="inlineStr">
+        <is>
+          <t>ASTERISM</t>
+        </is>
+      </c>
       <c r="M151" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28579</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25525</t>
         </is>
       </c>
     </row>
@@ -8356,11 +8360,11 @@
         </is>
       </c>
       <c r="C152" t="n">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>夜桜さんちの大作戦 第2期 第2クール</t>
+          <t>ゆるゆる図鑑</t>
         </is>
       </c>
       <c r="E152" t="b">
@@ -8373,37 +8377,17 @@
       </c>
       <c r="G152" t="inlineStr">
         <is>
-          <t>第1クール：2026年4月12日（日）～2026年6月28日（日） 第2クール：2026年10月〜 MBS／TBS系全国28局ネットにて</t>
-        </is>
-      </c>
-      <c r="H152" t="inlineStr">
-        <is>
-          <t>SILVER LINK.</t>
-        </is>
-      </c>
-      <c r="I152" t="inlineStr">
-        <is>
-          <t>What's "KAZOKU"</t>
-        </is>
-      </c>
-      <c r="J152" t="inlineStr">
-        <is>
-          <t>櫻坂46</t>
-        </is>
-      </c>
-      <c r="K152" t="inlineStr">
-        <is>
-          <t>Shalala</t>
-        </is>
-      </c>
-      <c r="L152" t="inlineStr">
-        <is>
-          <t>ピラフ星人</t>
-        </is>
-      </c>
+          <t>2026年10月～ テレ東系列6局ネット「アニもり！」内にて</t>
+        </is>
+      </c>
+      <c r="H152" t="inlineStr"/>
+      <c r="I152" t="inlineStr"/>
+      <c r="J152" t="inlineStr"/>
+      <c r="K152" t="inlineStr"/>
+      <c r="L152" t="inlineStr"/>
       <c r="M152" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25032</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28579</t>
         </is>
       </c>
     </row>
@@ -8417,11 +8401,11 @@
         </is>
       </c>
       <c r="C153" t="n">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>弱気MAX令嬢なのに、辣腕婚約者様の賭けに乗ってしまった</t>
+          <t>夜桜さんちの大作戦 第2期 第2クール</t>
         </is>
       </c>
       <c r="E153" t="b">
@@ -8434,21 +8418,37 @@
       </c>
       <c r="G153" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
+          <t>第1クール：2026年4月12日（日）～2026年6月28日（日） 第2クール：2026年10月〜 MBS／TBS系全国28局ネットにて</t>
         </is>
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>寿門堂</t>
-        </is>
-      </c>
-      <c r="I153" t="inlineStr"/>
-      <c r="J153" t="inlineStr"/>
-      <c r="K153" t="inlineStr"/>
-      <c r="L153" t="inlineStr"/>
+          <t>SILVER LINK.</t>
+        </is>
+      </c>
+      <c r="I153" t="inlineStr">
+        <is>
+          <t>What's "KAZOKU"</t>
+        </is>
+      </c>
+      <c r="J153" t="inlineStr">
+        <is>
+          <t>櫻坂46</t>
+        </is>
+      </c>
+      <c r="K153" t="inlineStr">
+        <is>
+          <t>Shalala</t>
+        </is>
+      </c>
+      <c r="L153" t="inlineStr">
+        <is>
+          <t>ピラフ星人</t>
+        </is>
+      </c>
       <c r="M153" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26947</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25032</t>
         </is>
       </c>
     </row>
@@ -8462,15 +8462,15 @@
         </is>
       </c>
       <c r="C154" t="n">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>ラブライブ！虹ヶ咲学園スクールアイドル同好会 第2期</t>
+          <t>弱気MAX令嬢なのに、辣腕婚約者様の賭けに乗ってしまった</t>
         </is>
       </c>
       <c r="E154" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F154" t="inlineStr">
         <is>
@@ -8479,12 +8479,12 @@
       </c>
       <c r="G154" t="inlineStr">
         <is>
-          <t>2022年4月2日（土）～2022年6月25日（土） TOKYO MXほか 【再放送】 2026年9月30日（水）〜 BS日テレにて</t>
+          <t>2026年10月～</t>
         </is>
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>サンライズ</t>
+          <t>寿門堂</t>
         </is>
       </c>
       <c r="I154" t="inlineStr"/>
@@ -8493,7 +8493,7 @@
       <c r="L154" t="inlineStr"/>
       <c r="M154" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=14120</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26947</t>
         </is>
       </c>
     </row>
@@ -8507,15 +8507,15 @@
         </is>
       </c>
       <c r="C155" t="n">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>らんま1/2 第3期</t>
+          <t>ラブライブ！虹ヶ咲学園スクールアイドル同好会 第2期</t>
         </is>
       </c>
       <c r="E155" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F155" t="inlineStr">
         <is>
@@ -8524,17 +8524,21 @@
       </c>
       <c r="G155" t="inlineStr">
         <is>
-          <t>2026年10月～ 日本テレビ系にて</t>
-        </is>
-      </c>
-      <c r="H155" t="inlineStr"/>
+          <t>2022年4月2日（土）～2022年6月25日（土） TOKYO MXほか 【再放送】 2026年9月30日（水）〜 BS日テレにて</t>
+        </is>
+      </c>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>サンライズ</t>
+        </is>
+      </c>
       <c r="I155" t="inlineStr"/>
       <c r="J155" t="inlineStr"/>
       <c r="K155" t="inlineStr"/>
       <c r="L155" t="inlineStr"/>
       <c r="M155" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28013</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=14120</t>
         </is>
       </c>
     </row>
@@ -8548,11 +8552,11 @@
         </is>
       </c>
       <c r="C156" t="n">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>LEGO® ONE PIECE</t>
+          <t>らんま1/2 第3期</t>
         </is>
       </c>
       <c r="E156" t="b">
@@ -8560,12 +8564,12 @@
       </c>
       <c r="F156" t="inlineStr">
         <is>
-          <t>配信</t>
+          <t>TVアニメ</t>
         </is>
       </c>
       <c r="G156" t="inlineStr">
         <is>
-          <t>2026年9月29日（火） Netflixにて</t>
+          <t>2026年10月～ 日本テレビ系にて</t>
         </is>
       </c>
       <c r="H156" t="inlineStr"/>
@@ -8574,6 +8578,47 @@
       <c r="K156" t="inlineStr"/>
       <c r="L156" t="inlineStr"/>
       <c r="M156" t="inlineStr">
+        <is>
+          <t>https://www.animatetimes.com/tag/details.php?id=28013</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C157" t="n">
+        <v>69</v>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>LEGO® ONE PIECE</t>
+        </is>
+      </c>
+      <c r="E157" t="b">
+        <v>0</v>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>配信</t>
+        </is>
+      </c>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>2026年9月29日（火） Netflixにて</t>
+        </is>
+      </c>
+      <c r="H157" t="inlineStr"/>
+      <c r="I157" t="inlineStr"/>
+      <c r="J157" t="inlineStr"/>
+      <c r="K157" t="inlineStr"/>
+      <c r="L157" t="inlineStr"/>
+      <c r="M157" t="inlineStr">
         <is>
           <t>https://www.animatetimes.com/tag/details.php?id=28168</t>
         </is>
@@ -8821,7 +8866,7 @@
         </is>
       </c>
       <c r="J4" t="n">
-        <v>3941540</v>
+        <v>3969358</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -8833,7 +8878,7 @@
       <c r="N4" t="inlineStr"/>
       <c r="O4" t="inlineStr">
         <is>
-          <t>2026-07-02T09:00:27</t>
+          <t>2026-07-10T09:00:44</t>
         </is>
       </c>
     </row>
@@ -9423,29 +9468,29 @@
         </is>
       </c>
       <c r="J14" t="n">
-        <v>701</v>
+        <v>22799</v>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>METANICK - Topic</t>
+          <t>METANICK</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=wh36fOeXxqg</t>
+          <t>https://www.youtube.com/watch?v=waOUdRPozDY</t>
         </is>
       </c>
       <c r="M14" t="n">
-        <v>253305</v>
+        <v>1332</v>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>KADOKAWA Official Channel</t>
+          <t>GOOD SMILE CHANNEL</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>2026-07-02T09:01:13</t>
+          <t>2026-07-10T09:01:05</t>
         </is>
       </c>
     </row>
@@ -9854,23 +9899,33 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=vxtUG2AWn80</t>
+          <t>https://www.youtube.com/watch?v=MeZ6ECW4tWk</t>
         </is>
       </c>
       <c r="J21" t="n">
-        <v>1313434</v>
+        <v>6810695</v>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>pellekofficial</t>
-        </is>
-      </c>
-      <c r="L21" t="inlineStr"/>
-      <c r="M21" t="inlineStr"/>
-      <c r="N21" t="inlineStr"/>
+          <t>PelleK - Topic</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=9Qr1nkwhqvM</t>
+        </is>
+      </c>
+      <c r="M21" t="n">
+        <v>73451</v>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>オーバーラップチャンネル</t>
+        </is>
+      </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>2026-07-02T09:02:14</t>
+          <t>2026-07-10T09:01:17</t>
         </is>
       </c>
     </row>
@@ -11904,13 +11959,37 @@
           <t>音羽-otoha-</t>
         </is>
       </c>
-      <c r="I57" t="inlineStr"/>
-      <c r="J57" t="inlineStr"/>
-      <c r="K57" t="inlineStr"/>
-      <c r="L57" t="inlineStr"/>
-      <c r="M57" t="inlineStr"/>
-      <c r="N57" t="inlineStr"/>
-      <c r="O57" t="inlineStr"/>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=2SXzmgP26bk</t>
+        </is>
+      </c>
+      <c r="J57" t="n">
+        <v>2681</v>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>【フジテレビ】アニメ公式チャンネル</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=2SXzmgP26bk</t>
+        </is>
+      </c>
+      <c r="M57" t="n">
+        <v>2681</v>
+      </c>
+      <c r="N57" t="inlineStr">
+        <is>
+          <t>【フジテレビ】アニメ公式チャンネル</t>
+        </is>
+      </c>
+      <c r="O57" t="inlineStr">
+        <is>
+          <t>2026-07-10T09:02:29</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -12504,23 +12583,33 @@
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=aRB6zduYtKg</t>
+          <t>https://www.youtube.com/watch?v=yeVq367DvIg</t>
         </is>
       </c>
       <c r="J67" t="n">
-        <v>881</v>
+        <v>96982</v>
       </c>
       <c r="K67" t="inlineStr">
         <is>
           <t>Mega Shinnosuke</t>
         </is>
       </c>
-      <c r="L67" t="inlineStr"/>
-      <c r="M67" t="inlineStr"/>
-      <c r="N67" t="inlineStr"/>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=A6aH9jPW8ZY</t>
+        </is>
+      </c>
+      <c r="M67" t="n">
+        <v>289860</v>
+      </c>
+      <c r="N67" t="inlineStr">
+        <is>
+          <t>SHOCHIKU anime Channel</t>
+        </is>
+      </c>
       <c r="O67" t="inlineStr">
         <is>
-          <t>2026-07-02T09:04:25</t>
+          <t>2026-07-10T09:02:49</t>
         </is>
       </c>
     </row>
@@ -12913,13 +13002,27 @@
           <t>ReoNa</t>
         </is>
       </c>
-      <c r="I74" t="inlineStr"/>
-      <c r="J74" t="inlineStr"/>
-      <c r="K74" t="inlineStr"/>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=ylYL2rDyIHc</t>
+        </is>
+      </c>
+      <c r="J74" t="n">
+        <v>131604</v>
+      </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>ReoNa official YouTube channel</t>
+        </is>
+      </c>
       <c r="L74" t="inlineStr"/>
       <c r="M74" t="inlineStr"/>
       <c r="N74" t="inlineStr"/>
-      <c r="O74" t="inlineStr"/>
+      <c r="O74" t="inlineStr">
+        <is>
+          <t>2026-07-10T09:03:11</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -13558,7 +13661,7 @@
         </is>
       </c>
       <c r="J85" t="n">
-        <v>106573</v>
+        <v>160213</v>
       </c>
       <c r="K85" t="inlineStr">
         <is>
@@ -13571,7 +13674,7 @@
         </is>
       </c>
       <c r="M85" t="n">
-        <v>106573</v>
+        <v>160213</v>
       </c>
       <c r="N85" t="inlineStr">
         <is>
@@ -13580,7 +13683,7 @@
       </c>
       <c r="O85" t="inlineStr">
         <is>
-          <t>2026-07-02T09:05:53</t>
+          <t>2026-07-10T09:03:24</t>
         </is>
       </c>
     </row>
@@ -13625,7 +13728,7 @@
         </is>
       </c>
       <c r="J86" t="n">
-        <v>106573</v>
+        <v>160213</v>
       </c>
       <c r="K86" t="inlineStr">
         <is>
@@ -13638,7 +13741,7 @@
         </is>
       </c>
       <c r="M86" t="n">
-        <v>106573</v>
+        <v>160213</v>
       </c>
       <c r="N86" t="inlineStr">
         <is>
@@ -13647,7 +13750,7 @@
       </c>
       <c r="O86" t="inlineStr">
         <is>
-          <t>2026-07-02T09:06:02</t>
+          <t>2026-07-10T09:03:33</t>
         </is>
       </c>
     </row>
@@ -14548,33 +14651,33 @@
       </c>
       <c r="I103" t="inlineStr">
         <is>
+          <t>https://www.youtube.com/watch?v=XkMdJycOZcQ</t>
+        </is>
+      </c>
+      <c r="J103" t="n">
+        <v>916149</v>
+      </c>
+      <c r="K103" t="inlineStr">
+        <is>
+          <t>Omoinotake</t>
+        </is>
+      </c>
+      <c r="L103" t="inlineStr">
+        <is>
           <t>https://www.youtube.com/watch?v=SccI7wPhm5s</t>
         </is>
       </c>
-      <c r="J103" t="n">
-        <v>4459</v>
-      </c>
-      <c r="K103" t="inlineStr">
+      <c r="M103" t="n">
+        <v>89187</v>
+      </c>
+      <c r="N103" t="inlineStr">
         <is>
           <t>アニプレックス チャンネル</t>
         </is>
       </c>
-      <c r="L103" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=SccI7wPhm5s</t>
-        </is>
-      </c>
-      <c r="M103" t="n">
-        <v>4459</v>
-      </c>
-      <c r="N103" t="inlineStr">
-        <is>
-          <t>アニプレックス チャンネル</t>
-        </is>
-      </c>
       <c r="O103" t="inlineStr">
         <is>
-          <t>2026-07-02T09:07:29</t>
+          <t>2026-07-10T09:04:36</t>
         </is>
       </c>
     </row>
@@ -14615,11 +14718,11 @@
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=s1bZEnGAX8I</t>
+          <t>https://www.youtube.com/watch?v=XkMdJycOZcQ</t>
         </is>
       </c>
       <c r="J104" t="n">
-        <v>3855744</v>
+        <v>916149</v>
       </c>
       <c r="K104" t="inlineStr">
         <is>
@@ -14632,7 +14735,7 @@
         </is>
       </c>
       <c r="M104" t="n">
-        <v>4459</v>
+        <v>89187</v>
       </c>
       <c r="N104" t="inlineStr">
         <is>
@@ -14641,7 +14744,7 @@
       </c>
       <c r="O104" t="inlineStr">
         <is>
-          <t>2026-07-02T09:07:38</t>
+          <t>2026-07-10T09:04:45</t>
         </is>
       </c>
     </row>
@@ -14729,7 +14832,7 @@
         </is>
       </c>
       <c r="J106" t="n">
-        <v>368101</v>
+        <v>495982</v>
       </c>
       <c r="K106" t="inlineStr">
         <is>
@@ -14742,7 +14845,7 @@
         </is>
       </c>
       <c r="M106" t="n">
-        <v>368101</v>
+        <v>495982</v>
       </c>
       <c r="N106" t="inlineStr">
         <is>
@@ -14751,7 +14854,7 @@
       </c>
       <c r="O106" t="inlineStr">
         <is>
-          <t>2026-07-02T09:07:49</t>
+          <t>2026-07-10T09:04:55</t>
         </is>
       </c>
     </row>
@@ -14863,7 +14966,7 @@
         </is>
       </c>
       <c r="J108" t="n">
-        <v>4786</v>
+        <v>17402</v>
       </c>
       <c r="K108" t="inlineStr">
         <is>
@@ -14876,7 +14979,7 @@
         </is>
       </c>
       <c r="M108" t="n">
-        <v>1316</v>
+        <v>10957</v>
       </c>
       <c r="N108" t="inlineStr">
         <is>
@@ -14885,7 +14988,7 @@
       </c>
       <c r="O108" t="inlineStr">
         <is>
-          <t>2026-07-02T09:08:02</t>
+          <t>2026-07-10T09:05:04</t>
         </is>
       </c>
     </row>
@@ -16932,13 +17035,27 @@
           <t>TrySail</t>
         </is>
       </c>
-      <c r="I145" t="inlineStr"/>
-      <c r="J145" t="inlineStr"/>
-      <c r="K145" t="inlineStr"/>
+      <c r="I145" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=7hWVEf4JTrI</t>
+        </is>
+      </c>
+      <c r="J145" t="n">
+        <v>13368</v>
+      </c>
+      <c r="K145" t="inlineStr">
+        <is>
+          <t>TrySail（麻倉もも・雨宮天・夏川椎菜）official YouTube channel</t>
+        </is>
+      </c>
       <c r="L145" t="inlineStr"/>
       <c r="M145" t="inlineStr"/>
       <c r="N145" t="inlineStr"/>
-      <c r="O145" t="inlineStr"/>
+      <c r="O145" t="inlineStr">
+        <is>
+          <t>2026-07-10T09:06:17</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="n">
@@ -17273,11 +17390,11 @@
       </c>
       <c r="I152" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=xtGGu2ShVSI</t>
+          <t>https://www.youtube.com/watch?v=GEZWCWyX-is</t>
         </is>
       </c>
       <c r="J152" t="n">
-        <v>7800</v>
+        <v>60984</v>
       </c>
       <c r="K152" t="inlineStr">
         <is>
@@ -17286,11 +17403,11 @@
       </c>
       <c r="L152" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=xtGGu2ShVSI</t>
+          <t>https://www.youtube.com/watch?v=GEZWCWyX-is</t>
         </is>
       </c>
       <c r="M152" t="n">
-        <v>7800</v>
+        <v>60984</v>
       </c>
       <c r="N152" t="inlineStr">
         <is>
@@ -17299,7 +17416,7 @@
       </c>
       <c r="O152" t="inlineStr">
         <is>
-          <t>2026-07-02T09:09:44</t>
+          <t>2026-07-10T09:06:36</t>
         </is>
       </c>
     </row>
@@ -17612,7 +17729,7 @@
         </is>
       </c>
       <c r="J157" t="n">
-        <v>133601</v>
+        <v>261225</v>
       </c>
       <c r="K157" t="inlineStr">
         <is>
@@ -17625,7 +17742,7 @@
         </is>
       </c>
       <c r="M157" t="n">
-        <v>133601</v>
+        <v>261225</v>
       </c>
       <c r="N157" t="inlineStr">
         <is>
@@ -17634,7 +17751,7 @@
       </c>
       <c r="O157" t="inlineStr">
         <is>
-          <t>2026-07-02T09:10:02</t>
+          <t>2026-07-10T09:06:43</t>
         </is>
       </c>
     </row>
@@ -18333,7 +18450,7 @@
         </is>
       </c>
       <c r="J172" t="n">
-        <v>284433</v>
+        <v>290217</v>
       </c>
       <c r="K172" t="inlineStr">
         <is>
@@ -18346,7 +18463,7 @@
         </is>
       </c>
       <c r="M172" t="n">
-        <v>284433</v>
+        <v>290217</v>
       </c>
       <c r="N172" t="inlineStr">
         <is>
@@ -18355,7 +18472,7 @@
       </c>
       <c r="O172" t="inlineStr">
         <is>
-          <t>2026-07-02T09:10:45</t>
+          <t>2026-07-10T09:07:47</t>
         </is>
       </c>
     </row>
@@ -18400,7 +18517,7 @@
         </is>
       </c>
       <c r="J173" t="n">
-        <v>284434</v>
+        <v>290217</v>
       </c>
       <c r="K173" t="inlineStr">
         <is>
@@ -18413,7 +18530,7 @@
         </is>
       </c>
       <c r="M173" t="n">
-        <v>284434</v>
+        <v>290217</v>
       </c>
       <c r="N173" t="inlineStr">
         <is>
@@ -18422,7 +18539,7 @@
       </c>
       <c r="O173" t="inlineStr">
         <is>
-          <t>2026-07-02T09:10:54</t>
+          <t>2026-07-10T09:07:56</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: anime list update (PC) 2026-07-11
</commit_message>
<xml_diff>
--- a/data/anime_list.xlsx
+++ b/data/anime_list.xlsx
@@ -10613,13 +10613,27 @@
           <t>sorato</t>
         </is>
       </c>
-      <c r="I33" t="inlineStr"/>
-      <c r="J33" t="inlineStr"/>
-      <c r="K33" t="inlineStr"/>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=D2yjyOW6tjc</t>
+        </is>
+      </c>
+      <c r="J33" t="n">
+        <v>1056</v>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>sorato</t>
+        </is>
+      </c>
       <c r="L33" t="inlineStr"/>
       <c r="M33" t="inlineStr"/>
       <c r="N33" t="inlineStr"/>
-      <c r="O33" t="inlineStr"/>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>2026-07-11T09:00:59</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -11234,13 +11248,37 @@
           <t>sajou no hana</t>
         </is>
       </c>
-      <c r="I44" t="inlineStr"/>
-      <c r="J44" t="inlineStr"/>
-      <c r="K44" t="inlineStr"/>
-      <c r="L44" t="inlineStr"/>
-      <c r="M44" t="inlineStr"/>
-      <c r="N44" t="inlineStr"/>
-      <c r="O44" t="inlineStr"/>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=lMq8obidFDI</t>
+        </is>
+      </c>
+      <c r="J44" t="n">
+        <v>7262</v>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>GREE Entertainment ANIME &amp; GAME【公式】</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=lMq8obidFDI</t>
+        </is>
+      </c>
+      <c r="M44" t="n">
+        <v>7262</v>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>GREE Entertainment ANIME &amp; GAME【公式】</t>
+        </is>
+      </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>2026-07-11T09:01:36</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -12941,7 +12979,7 @@
         </is>
       </c>
       <c r="J73" t="n">
-        <v>4513</v>
+        <v>100304</v>
       </c>
       <c r="K73" t="inlineStr">
         <is>
@@ -12954,7 +12992,7 @@
         </is>
       </c>
       <c r="M73" t="n">
-        <v>4513</v>
+        <v>100304</v>
       </c>
       <c r="N73" t="inlineStr">
         <is>
@@ -12963,7 +13001,7 @@
       </c>
       <c r="O73" t="inlineStr">
         <is>
-          <t>2026-07-03T09:03:44</t>
+          <t>2026-07-11T09:02:25</t>
         </is>
       </c>
     </row>
@@ -13061,11 +13099,11 @@
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=Nqel4e1h8YQ</t>
+          <t>https://www.youtube.com/watch?v=j44OcUcmKCU</t>
         </is>
       </c>
       <c r="J75" t="n">
-        <v>15417</v>
+        <v>47223</v>
       </c>
       <c r="K75" t="inlineStr">
         <is>
@@ -13077,7 +13115,7 @@
       <c r="N75" t="inlineStr"/>
       <c r="O75" t="inlineStr">
         <is>
-          <t>2026-07-03T09:04:04</t>
+          <t>2026-07-11T09:02:43</t>
         </is>
       </c>
     </row>
@@ -14152,13 +14190,27 @@
           <t>shallm</t>
         </is>
       </c>
-      <c r="I94" t="inlineStr"/>
-      <c r="J94" t="inlineStr"/>
-      <c r="K94" t="inlineStr"/>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=CuPyVWq5Bes</t>
+        </is>
+      </c>
+      <c r="J94" t="n">
+        <v>2547</v>
+      </c>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>shallm</t>
+        </is>
+      </c>
       <c r="L94" t="inlineStr"/>
       <c r="M94" t="inlineStr"/>
       <c r="N94" t="inlineStr"/>
-      <c r="O94" t="inlineStr"/>
+      <c r="O94" t="inlineStr">
+        <is>
+          <t>2026-07-11T09:03:50</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -15344,23 +15396,33 @@
       </c>
       <c r="I114" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=r-4zKDCNjwM</t>
+          <t>https://www.youtube.com/watch?v=PWN4MO0ILIM</t>
         </is>
       </c>
       <c r="J114" t="n">
-        <v>980</v>
+        <v>266478</v>
       </c>
       <c r="K114" t="inlineStr">
         <is>
           <t>I Don't Like Mondays.</t>
         </is>
       </c>
-      <c r="L114" t="inlineStr"/>
-      <c r="M114" t="inlineStr"/>
-      <c r="N114" t="inlineStr"/>
+      <c r="L114" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=yaX2p36llik</t>
+        </is>
+      </c>
+      <c r="M114" t="n">
+        <v>16260</v>
+      </c>
+      <c r="N114" t="inlineStr">
+        <is>
+          <t>ShoProアニメチャンネル</t>
+        </is>
+      </c>
       <c r="O114" t="inlineStr">
         <is>
-          <t>2026-07-03T09:05:57</t>
+          <t>2026-07-11T09:04:15</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: anime list update (PC) 2026-07-12
</commit_message>
<xml_diff>
--- a/data/anime_list.xlsx
+++ b/data/anime_list.xlsx
@@ -10562,7 +10562,7 @@
         </is>
       </c>
       <c r="J32" t="n">
-        <v>5468</v>
+        <v>62831</v>
       </c>
       <c r="K32" t="inlineStr">
         <is>
@@ -10574,7 +10574,7 @@
       <c r="N32" t="inlineStr"/>
       <c r="O32" t="inlineStr">
         <is>
-          <t>2026-07-04T09:02:48</t>
+          <t>2026-07-12T09:00:45</t>
         </is>
       </c>
     </row>
@@ -13390,11 +13390,11 @@
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=d4TzLZZaeac</t>
+          <t>https://www.youtube.com/watch?v=UTEjVKRw1Gs</t>
         </is>
       </c>
       <c r="J80" t="n">
-        <v>3309</v>
+        <v>4523</v>
       </c>
       <c r="K80" t="inlineStr">
         <is>
@@ -13406,7 +13406,7 @@
       <c r="N80" t="inlineStr"/>
       <c r="O80" t="inlineStr">
         <is>
-          <t>2026-07-04T09:05:20</t>
+          <t>2026-07-12T09:02:10</t>
         </is>
       </c>
     </row>
@@ -14135,23 +14135,33 @@
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=JJaCwW4HyVs</t>
+          <t>https://www.youtube.com/watch?v=ZH8xYK5vac0</t>
         </is>
       </c>
       <c r="J93" t="n">
-        <v>51132323</v>
+        <v>72237</v>
       </c>
       <c r="K93" t="inlineStr">
         <is>
-          <t>ヨルシカ / n-buna Official</t>
-        </is>
-      </c>
-      <c r="L93" t="inlineStr"/>
-      <c r="M93" t="inlineStr"/>
-      <c r="N93" t="inlineStr"/>
+          <t>宝島社公式</t>
+        </is>
+      </c>
+      <c r="L93" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=ZH8xYK5vac0</t>
+        </is>
+      </c>
+      <c r="M93" t="n">
+        <v>72237</v>
+      </c>
+      <c r="N93" t="inlineStr">
+        <is>
+          <t>宝島社公式</t>
+        </is>
+      </c>
       <c r="O93" t="inlineStr">
         <is>
-          <t>2026-07-04T09:06:55</t>
+          <t>2026-07-12T09:02:53</t>
         </is>
       </c>
     </row>
@@ -15333,7 +15343,7 @@
         </is>
       </c>
       <c r="J113" t="n">
-        <v>410448</v>
+        <v>472908</v>
       </c>
       <c r="K113" t="inlineStr">
         <is>
@@ -15346,7 +15356,7 @@
         </is>
       </c>
       <c r="M113" t="n">
-        <v>410448</v>
+        <v>472908</v>
       </c>
       <c r="N113" t="inlineStr">
         <is>
@@ -15355,7 +15365,7 @@
       </c>
       <c r="O113" t="inlineStr">
         <is>
-          <t>2026-07-04T09:07:38</t>
+          <t>2026-07-12T09:03:19</t>
         </is>
       </c>
     </row>
@@ -15720,7 +15730,7 @@
         </is>
       </c>
       <c r="J120" t="n">
-        <v>1041</v>
+        <v>13869</v>
       </c>
       <c r="K120" t="inlineStr">
         <is>
@@ -15733,7 +15743,7 @@
         </is>
       </c>
       <c r="M120" t="n">
-        <v>1041</v>
+        <v>13869</v>
       </c>
       <c r="N120" t="inlineStr">
         <is>
@@ -15742,7 +15752,7 @@
       </c>
       <c r="O120" t="inlineStr">
         <is>
-          <t>2026-07-04T09:08:03</t>
+          <t>2026-07-12T09:03:41</t>
         </is>
       </c>
     </row>
@@ -17289,19 +17299,29 @@
         </is>
       </c>
       <c r="J149" t="n">
-        <v>1391</v>
+        <v>8320</v>
       </c>
       <c r="K149" t="inlineStr">
         <is>
           <t xml:space="preserve">Kaya Official YouTube Channel </t>
         </is>
       </c>
-      <c r="L149" t="inlineStr"/>
-      <c r="M149" t="inlineStr"/>
-      <c r="N149" t="inlineStr"/>
+      <c r="L149" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=dhAKFhT6pno</t>
+        </is>
+      </c>
+      <c r="M149" t="n">
+        <v>5403</v>
+      </c>
+      <c r="N149" t="inlineStr">
+        <is>
+          <t>NBCUniversal Anime/Music</t>
+        </is>
+      </c>
       <c r="O149" t="inlineStr">
         <is>
-          <t>2026-07-04T09:09:16</t>
+          <t>2026-07-12T09:04:43</t>
         </is>
       </c>
     </row>
@@ -17389,7 +17409,7 @@
         </is>
       </c>
       <c r="J151" t="n">
-        <v>145139</v>
+        <v>173757</v>
       </c>
       <c r="K151" t="inlineStr">
         <is>
@@ -17402,7 +17422,7 @@
         </is>
       </c>
       <c r="M151" t="n">
-        <v>145139</v>
+        <v>173757</v>
       </c>
       <c r="N151" t="inlineStr">
         <is>
@@ -17411,7 +17431,7 @@
       </c>
       <c r="O151" t="inlineStr">
         <is>
-          <t>2026-07-04T09:09:27</t>
+          <t>2026-07-12T09:04:54</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: anime list update (PC) 2026-07-13
</commit_message>
<xml_diff>
--- a/data/anime_list.xlsx
+++ b/data/anime_list.xlsx
@@ -11897,13 +11897,27 @@
           <t>Hana Hope</t>
         </is>
       </c>
-      <c r="I55" t="inlineStr"/>
-      <c r="J55" t="inlineStr"/>
-      <c r="K55" t="inlineStr"/>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=H8BSBY59Dh0</t>
+        </is>
+      </c>
+      <c r="J55" t="n">
+        <v>1198</v>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>Hana Hope</t>
+        </is>
+      </c>
       <c r="L55" t="inlineStr"/>
       <c r="M55" t="inlineStr"/>
       <c r="N55" t="inlineStr"/>
-      <c r="O55" t="inlineStr"/>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t>2026-07-13T09:01:34</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -14611,13 +14625,37 @@
           <t>オーイシマサヨシ</t>
         </is>
       </c>
-      <c r="I101" t="inlineStr"/>
-      <c r="J101" t="inlineStr"/>
-      <c r="K101" t="inlineStr"/>
-      <c r="L101" t="inlineStr"/>
-      <c r="M101" t="inlineStr"/>
-      <c r="N101" t="inlineStr"/>
-      <c r="O101" t="inlineStr"/>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=dv1TGoV_aS8</t>
+        </is>
+      </c>
+      <c r="J101" t="n">
+        <v>10238</v>
+      </c>
+      <c r="K101" t="inlineStr">
+        <is>
+          <t>ぽにきゃん-Anime PONY CANYON</t>
+        </is>
+      </c>
+      <c r="L101" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=dv1TGoV_aS8</t>
+        </is>
+      </c>
+      <c r="M101" t="n">
+        <v>10238</v>
+      </c>
+      <c r="N101" t="inlineStr">
+        <is>
+          <t>ぽにきゃん-Anime PONY CANYON</t>
+        </is>
+      </c>
+      <c r="O101" t="inlineStr">
+        <is>
+          <t>2026-07-13T09:02:41</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="n">
@@ -17250,13 +17288,27 @@
           <t>CROWN HEAD</t>
         </is>
       </c>
-      <c r="I148" t="inlineStr"/>
-      <c r="J148" t="inlineStr"/>
-      <c r="K148" t="inlineStr"/>
+      <c r="I148" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=ivJRaXk3GUw</t>
+        </is>
+      </c>
+      <c r="J148" t="n">
+        <v>634</v>
+      </c>
+      <c r="K148" t="inlineStr">
+        <is>
+          <t>CROWN HEAD</t>
+        </is>
+      </c>
       <c r="L148" t="inlineStr"/>
       <c r="M148" t="inlineStr"/>
       <c r="N148" t="inlineStr"/>
-      <c r="O148" t="inlineStr"/>
+      <c r="O148" t="inlineStr">
+        <is>
+          <t>2026-07-13T09:04:01</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="n">

</xml_diff>

<commit_message>
auto: anime list update (PC) 2026-07-14
</commit_message>
<xml_diff>
--- a/data/anime_list.xlsx
+++ b/data/anime_list.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M157"/>
+  <dimension ref="A1:M158"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6946,7 +6946,7 @@
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>超巡！超条先輩</t>
+          <t>千歳くんはラムネ瓶のなか 第2クール</t>
         </is>
       </c>
       <c r="E122" t="b">
@@ -6959,21 +6959,37 @@
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>2026年10月～ カンテレ・フジテレビ系全国ネットにて</t>
+          <t>第1クール：2025年10月7日（火）～ 2025年12月30日（火） AT-X・TOKYO MXほか 第2クール：2026年10月〜</t>
         </is>
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>アルボアニメーション</t>
-        </is>
-      </c>
-      <c r="I122" t="inlineStr"/>
-      <c r="J122" t="inlineStr"/>
-      <c r="K122" t="inlineStr"/>
-      <c r="L122" t="inlineStr"/>
+          <t>feel.</t>
+        </is>
+      </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>ライアー</t>
+        </is>
+      </c>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>Kucci</t>
+        </is>
+      </c>
+      <c r="K122" t="inlineStr">
+        <is>
+          <t>陽炎</t>
+        </is>
+      </c>
+      <c r="L122" t="inlineStr">
+        <is>
+          <t>サイダーガール</t>
+        </is>
+      </c>
       <c r="M122" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26933</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25058</t>
         </is>
       </c>
     </row>
@@ -6991,7 +7007,7 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>追放されたチート付与魔術師は気ままなセカンドライフを謳歌する。</t>
+          <t>超巡！超条先輩</t>
         </is>
       </c>
       <c r="E123" t="b">
@@ -7004,12 +7020,12 @@
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t>2026年10月～ テレ東系列にて</t>
+          <t>2026年10月～ カンテレ・フジテレビ系全国ネットにて</t>
         </is>
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>P.A.WORKS</t>
+          <t>アルボアニメーション</t>
         </is>
       </c>
       <c r="I123" t="inlineStr"/>
@@ -7018,7 +7034,7 @@
       <c r="L123" t="inlineStr"/>
       <c r="M123" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27631</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26933</t>
         </is>
       </c>
     </row>
@@ -7036,7 +7052,7 @@
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>てつりょー！meet with 鉄道むすめ</t>
+          <t>追放されたチート付与魔術師は気ままなセカンドライフを謳歌する。</t>
         </is>
       </c>
       <c r="E124" t="b">
@@ -7049,12 +7065,12 @@
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>2026年秋</t>
+          <t>2026年10月～ テレ東系列にて</t>
         </is>
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>イーストフィッシュスタジオ</t>
+          <t>P.A.WORKS</t>
         </is>
       </c>
       <c r="I124" t="inlineStr"/>
@@ -7063,7 +7079,7 @@
       <c r="L124" t="inlineStr"/>
       <c r="M124" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26895</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27631</t>
         </is>
       </c>
     </row>
@@ -7081,7 +7097,7 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>テムパル～アイテムの力～</t>
+          <t>てつりょー！meet with 鉄道むすめ</t>
         </is>
       </c>
       <c r="E125" t="b">
@@ -7094,12 +7110,12 @@
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
+          <t>2026年秋</t>
         </is>
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>J.C.STAFF</t>
+          <t>イーストフィッシュスタジオ</t>
         </is>
       </c>
       <c r="I125" t="inlineStr"/>
@@ -7108,7 +7124,7 @@
       <c r="L125" t="inlineStr"/>
       <c r="M125" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28478</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26895</t>
         </is>
       </c>
     </row>
@@ -7126,7 +7142,7 @@
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>デモンズ・クレスト</t>
+          <t>テムパル～アイテムの力～</t>
         </is>
       </c>
       <c r="E126" t="b">
@@ -7134,34 +7150,26 @@
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>配信</t>
+          <t>TVアニメ</t>
         </is>
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t>2026年11月6日（金） Prime Videoにて</t>
+          <t>2026年10月～</t>
         </is>
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>Production I.G</t>
-        </is>
-      </c>
-      <c r="I126" t="inlineStr">
-        <is>
-          <t>シンカ</t>
-        </is>
-      </c>
-      <c r="J126" t="inlineStr">
-        <is>
-          <t>Ado</t>
-        </is>
-      </c>
+          <t>J.C.STAFF</t>
+        </is>
+      </c>
+      <c r="I126" t="inlineStr"/>
+      <c r="J126" t="inlineStr"/>
       <c r="K126" t="inlineStr"/>
       <c r="L126" t="inlineStr"/>
       <c r="M126" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27189</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28478</t>
         </is>
       </c>
     </row>
@@ -7179,7 +7187,7 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>転生貴族、鑑定スキルで成り上がる 第3期</t>
+          <t>デモンズ・クレスト</t>
         </is>
       </c>
       <c r="E127" t="b">
@@ -7187,26 +7195,34 @@
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>TVアニメ</t>
+          <t>配信</t>
         </is>
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t>2026年秋 CBC/TBS系全国28局ネット「アガルアニメ」にて</t>
+          <t>2026年11月6日（金） Prime Videoにて</t>
         </is>
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>studio MOTHER</t>
-        </is>
-      </c>
-      <c r="I127" t="inlineStr"/>
-      <c r="J127" t="inlineStr"/>
+          <t>Production I.G</t>
+        </is>
+      </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>シンカ</t>
+        </is>
+      </c>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>Ado</t>
+        </is>
+      </c>
       <c r="K127" t="inlineStr"/>
       <c r="L127" t="inlineStr"/>
       <c r="M127" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25385</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27189</t>
         </is>
       </c>
     </row>
@@ -7224,7 +7240,7 @@
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>転生ゴブリンだけど質問ある？</t>
+          <t>転生貴族、鑑定スキルで成り上がる 第3期</t>
         </is>
       </c>
       <c r="E128" t="b">
@@ -7237,12 +7253,12 @@
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
+          <t>2026年秋 CBC/TBS系全国28局ネット「アガルアニメ」にて</t>
         </is>
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>BAKKKA</t>
+          <t>studio MOTHER</t>
         </is>
       </c>
       <c r="I128" t="inlineStr"/>
@@ -7251,7 +7267,7 @@
       <c r="L128" t="inlineStr"/>
       <c r="M128" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27909</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25385</t>
         </is>
       </c>
     </row>
@@ -7269,7 +7285,7 @@
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>転生した大聖女は、聖女であることをひた隠す</t>
+          <t>転生ゴブリンだけど質問ある？</t>
         </is>
       </c>
       <c r="E129" t="b">
@@ -7287,32 +7303,16 @@
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>FelixFilm</t>
-        </is>
-      </c>
-      <c r="I129" t="inlineStr">
-        <is>
-          <t>Flare of Soul</t>
-        </is>
-      </c>
-      <c r="J129" t="inlineStr">
-        <is>
-          <t>花耶</t>
-        </is>
-      </c>
-      <c r="K129" t="inlineStr">
-        <is>
-          <t>STELLAR</t>
-        </is>
-      </c>
-      <c r="L129" t="inlineStr">
-        <is>
-          <t>ウタヒメドリーム オールスターズ</t>
-        </is>
-      </c>
+          <t>BAKKKA</t>
+        </is>
+      </c>
+      <c r="I129" t="inlineStr"/>
+      <c r="J129" t="inlineStr"/>
+      <c r="K129" t="inlineStr"/>
+      <c r="L129" t="inlineStr"/>
       <c r="M129" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25630</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27909</t>
         </is>
       </c>
     </row>
@@ -7330,7 +7330,7 @@
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>転生したら剣でした 第2期</t>
+          <t>転生した大聖女は、聖女であることをひた隠す</t>
         </is>
       </c>
       <c r="E130" t="b">
@@ -7348,16 +7348,32 @@
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>C2C</t>
-        </is>
-      </c>
-      <c r="I130" t="inlineStr"/>
-      <c r="J130" t="inlineStr"/>
-      <c r="K130" t="inlineStr"/>
-      <c r="L130" t="inlineStr"/>
+          <t>FelixFilm</t>
+        </is>
+      </c>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>Flare of Soul</t>
+        </is>
+      </c>
+      <c r="J130" t="inlineStr">
+        <is>
+          <t>花耶</t>
+        </is>
+      </c>
+      <c r="K130" t="inlineStr">
+        <is>
+          <t>STELLAR</t>
+        </is>
+      </c>
+      <c r="L130" t="inlineStr">
+        <is>
+          <t>ウタヒメドリーム オールスターズ</t>
+        </is>
+      </c>
       <c r="M130" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=19149</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25630</t>
         </is>
       </c>
     </row>
@@ -7375,7 +7391,7 @@
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>とある暗部の少女共棲</t>
+          <t>転生したら剣でした 第2期</t>
         </is>
       </c>
       <c r="E131" t="b">
@@ -7388,37 +7404,21 @@
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>2026年10月9日（金）～ TOKYO MXほか</t>
+          <t>2026年10月～</t>
         </is>
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>J.C.STAFF</t>
-        </is>
-      </c>
-      <c r="I131" t="inlineStr">
-        <is>
-          <t>Ghost Sequence</t>
-        </is>
-      </c>
-      <c r="J131" t="inlineStr">
-        <is>
-          <t>East Of Eden</t>
-        </is>
-      </c>
-      <c r="K131" t="inlineStr">
-        <is>
-          <t>原子崩し(メルトダウナー)</t>
-        </is>
-      </c>
-      <c r="L131" t="inlineStr">
-        <is>
-          <t>岸田教団&amp;THE明星ロケッツ</t>
-        </is>
-      </c>
+          <t>C2C</t>
+        </is>
+      </c>
+      <c r="I131" t="inlineStr"/>
+      <c r="J131" t="inlineStr"/>
+      <c r="K131" t="inlineStr"/>
+      <c r="L131" t="inlineStr"/>
       <c r="M131" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25552</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=19149</t>
         </is>
       </c>
     </row>
@@ -7436,7 +7436,7 @@
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>東京リベンジャーズ 三天戦争編</t>
+          <t>とある暗部の少女共棲</t>
         </is>
       </c>
       <c r="E132" t="b">
@@ -7449,21 +7449,37 @@
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>2026年10月2日（金）～ MBS・TBS・CBC”アニメイズム”枠ほか</t>
+          <t>2026年10月9日（金）～ TOKYO MXほか</t>
         </is>
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>ライデンフィルム</t>
-        </is>
-      </c>
-      <c r="I132" t="inlineStr"/>
-      <c r="J132" t="inlineStr"/>
-      <c r="K132" t="inlineStr"/>
-      <c r="L132" t="inlineStr"/>
+          <t>J.C.STAFF</t>
+        </is>
+      </c>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>Ghost Sequence</t>
+        </is>
+      </c>
+      <c r="J132" t="inlineStr">
+        <is>
+          <t>East Of Eden</t>
+        </is>
+      </c>
+      <c r="K132" t="inlineStr">
+        <is>
+          <t>原子崩し(メルトダウナー)</t>
+        </is>
+      </c>
+      <c r="L132" t="inlineStr">
+        <is>
+          <t>岸田教団&amp;THE明星ロケッツ</t>
+        </is>
+      </c>
       <c r="M132" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=24207</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25552</t>
         </is>
       </c>
     </row>
@@ -7481,7 +7497,7 @@
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>桃源暗鬼 ～日光・華厳の滝編～</t>
+          <t>東京リベンジャーズ 三天戦争編</t>
         </is>
       </c>
       <c r="E133" t="b">
@@ -7494,17 +7510,21 @@
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>2026年10月～ 日本テレビ系「FRIDAY ANIME NIGHT（フラアニ）」枠にて</t>
-        </is>
-      </c>
-      <c r="H133" t="inlineStr"/>
+          <t>2026年10月2日（金）～ MBS・TBS・CBC”アニメイズム”枠ほか</t>
+        </is>
+      </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>ライデンフィルム</t>
+        </is>
+      </c>
       <c r="I133" t="inlineStr"/>
       <c r="J133" t="inlineStr"/>
       <c r="K133" t="inlineStr"/>
       <c r="L133" t="inlineStr"/>
       <c r="M133" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27376</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=24207</t>
         </is>
       </c>
     </row>
@@ -7522,7 +7542,7 @@
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>どうも、好きな人に惚れ薬を依頼された魔女です。</t>
+          <t>桃源暗鬼 ～日光・華厳の滝編～</t>
         </is>
       </c>
       <c r="E134" t="b">
@@ -7535,21 +7555,17 @@
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
-        </is>
-      </c>
-      <c r="H134" t="inlineStr">
-        <is>
-          <t>ディオメディア</t>
-        </is>
-      </c>
+          <t>2026年10月～ 日本テレビ系「FRIDAY ANIME NIGHT（フラアニ）」枠にて</t>
+        </is>
+      </c>
+      <c r="H134" t="inlineStr"/>
       <c r="I134" t="inlineStr"/>
       <c r="J134" t="inlineStr"/>
       <c r="K134" t="inlineStr"/>
       <c r="L134" t="inlineStr"/>
       <c r="M134" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27581</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27376</t>
         </is>
       </c>
     </row>
@@ -7567,7 +7583,7 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>ドラゴンボール超 ビルス</t>
+          <t>どうも、好きな人に惚れ薬を依頼された魔女です。</t>
         </is>
       </c>
       <c r="E135" t="b">
@@ -7580,17 +7596,21 @@
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>2026年秋 フジテレビにて</t>
-        </is>
-      </c>
-      <c r="H135" t="inlineStr"/>
+          <t>2026年10月～</t>
+        </is>
+      </c>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>ディオメディア</t>
+        </is>
+      </c>
       <c r="I135" t="inlineStr"/>
       <c r="J135" t="inlineStr"/>
       <c r="K135" t="inlineStr"/>
       <c r="L135" t="inlineStr"/>
       <c r="M135" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27491</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27581</t>
         </is>
       </c>
     </row>
@@ -7608,7 +7628,7 @@
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>鳴海の平日</t>
+          <t>ドラゴンボール超 ビルス</t>
         </is>
       </c>
       <c r="E136" t="b">
@@ -7616,26 +7636,22 @@
       </c>
       <c r="F136" t="inlineStr">
         <is>
-          <t>配信</t>
+          <t>TVアニメ</t>
         </is>
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>2026年秋</t>
-        </is>
-      </c>
-      <c r="H136" t="inlineStr">
-        <is>
-          <t>Production I.G</t>
-        </is>
-      </c>
+          <t>2026年秋 フジテレビにて</t>
+        </is>
+      </c>
+      <c r="H136" t="inlineStr"/>
       <c r="I136" t="inlineStr"/>
       <c r="J136" t="inlineStr"/>
       <c r="K136" t="inlineStr"/>
       <c r="L136" t="inlineStr"/>
       <c r="M136" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28465</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27491</t>
         </is>
       </c>
     </row>
@@ -7653,7 +7669,7 @@
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>バーテックスフォース</t>
+          <t>鳴海の平日</t>
         </is>
       </c>
       <c r="E137" t="b">
@@ -7661,17 +7677,17 @@
       </c>
       <c r="F137" t="inlineStr">
         <is>
-          <t>TVアニメ</t>
+          <t>配信</t>
         </is>
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>2026年10月〜</t>
+          <t>2026年秋</t>
         </is>
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>SMDE</t>
+          <t>Production I.G</t>
         </is>
       </c>
       <c r="I137" t="inlineStr"/>
@@ -7680,7 +7696,7 @@
       <c r="L137" t="inlineStr"/>
       <c r="M137" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27988</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28465</t>
         </is>
       </c>
     </row>
@@ -7698,7 +7714,7 @@
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>Battle Spirits [Re] 絶界の空</t>
+          <t>バーテックスフォース</t>
         </is>
       </c>
       <c r="E138" t="b">
@@ -7711,17 +7727,21 @@
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t>2026年秋</t>
-        </is>
-      </c>
-      <c r="H138" t="inlineStr"/>
+          <t>2026年10月〜</t>
+        </is>
+      </c>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>SMDE</t>
+        </is>
+      </c>
       <c r="I138" t="inlineStr"/>
       <c r="J138" t="inlineStr"/>
       <c r="K138" t="inlineStr"/>
       <c r="L138" t="inlineStr"/>
       <c r="M138" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27954</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27988</t>
         </is>
       </c>
     </row>
@@ -7739,7 +7759,7 @@
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>パンどろぼう</t>
+          <t>Battle Spirits [Re] 絶界の空</t>
         </is>
       </c>
       <c r="E139" t="b">
@@ -7752,7 +7772,7 @@
       </c>
       <c r="G139" t="inlineStr">
         <is>
-          <t>2026年10月〜 NHK Eテレにて</t>
+          <t>2026年秋</t>
         </is>
       </c>
       <c r="H139" t="inlineStr"/>
@@ -7762,7 +7782,7 @@
       <c r="L139" t="inlineStr"/>
       <c r="M139" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26163</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27954</t>
         </is>
       </c>
     </row>
@@ -7780,7 +7800,7 @@
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>百妖譜 京師篇</t>
+          <t>パンどろぼう</t>
         </is>
       </c>
       <c r="E140" t="b">
@@ -7793,7 +7813,7 @@
       </c>
       <c r="G140" t="inlineStr">
         <is>
-          <t>2026年10月〜 フジテレビ「B8station」にて</t>
+          <t>2026年10月〜 NHK Eテレにて</t>
         </is>
       </c>
       <c r="H140" t="inlineStr"/>
@@ -7803,7 +7823,7 @@
       <c r="L140" t="inlineStr"/>
       <c r="M140" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27781</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26163</t>
         </is>
       </c>
     </row>
@@ -7821,7 +7841,7 @@
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>冰剣の魔術師が世界を統べるⅡ</t>
+          <t>百妖譜 京師篇</t>
         </is>
       </c>
       <c r="E141" t="b">
@@ -7834,21 +7854,17 @@
       </c>
       <c r="G141" t="inlineStr">
         <is>
-          <t>2026年10月〜</t>
-        </is>
-      </c>
-      <c r="H141" t="inlineStr">
-        <is>
-          <t>ゼロジー</t>
-        </is>
-      </c>
+          <t>2026年10月〜 フジテレビ「B8station」にて</t>
+        </is>
+      </c>
+      <c r="H141" t="inlineStr"/>
       <c r="I141" t="inlineStr"/>
       <c r="J141" t="inlineStr"/>
       <c r="K141" t="inlineStr"/>
       <c r="L141" t="inlineStr"/>
       <c r="M141" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28403</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27781</t>
         </is>
       </c>
     </row>
@@ -7866,7 +7882,7 @@
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>ブラッククローバー 2nd Season</t>
+          <t>冰剣の魔術師が世界を統べるⅡ</t>
         </is>
       </c>
       <c r="E142" t="b">
@@ -7879,29 +7895,21 @@
       </c>
       <c r="G142" t="inlineStr">
         <is>
-          <t>2026年10月～ テレ東系列ほか</t>
+          <t>2026年10月〜</t>
         </is>
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>スタジオぴえろ</t>
-        </is>
-      </c>
-      <c r="I142" t="inlineStr">
-        <is>
-          <t>消えない理由</t>
-        </is>
-      </c>
-      <c r="J142" t="inlineStr">
-        <is>
-          <t>WANIMA</t>
-        </is>
-      </c>
+          <t>ゼロジー</t>
+        </is>
+      </c>
+      <c r="I142" t="inlineStr"/>
+      <c r="J142" t="inlineStr"/>
       <c r="K142" t="inlineStr"/>
       <c r="L142" t="inlineStr"/>
       <c r="M142" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26361</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28403</t>
         </is>
       </c>
     </row>
@@ -7919,7 +7927,7 @@
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>ホタルの嫁入り</t>
+          <t>ブラッククローバー 2nd Season</t>
         </is>
       </c>
       <c r="E143" t="b">
@@ -7932,21 +7940,29 @@
       </c>
       <c r="G143" t="inlineStr">
         <is>
-          <t>2026年10月～ 全国フジテレビ系“ ノイタミナ ”にて</t>
+          <t>2026年10月～ テレ東系列ほか</t>
         </is>
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>david production</t>
-        </is>
-      </c>
-      <c r="I143" t="inlineStr"/>
-      <c r="J143" t="inlineStr"/>
+          <t>スタジオぴえろ</t>
+        </is>
+      </c>
+      <c r="I143" t="inlineStr">
+        <is>
+          <t>消えない理由</t>
+        </is>
+      </c>
+      <c r="J143" t="inlineStr">
+        <is>
+          <t>WANIMA</t>
+        </is>
+      </c>
       <c r="K143" t="inlineStr"/>
       <c r="L143" t="inlineStr"/>
       <c r="M143" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27415</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26361</t>
         </is>
       </c>
     </row>
@@ -7964,7 +7980,7 @@
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>ポップパップポルターズ</t>
+          <t>ホタルの嫁入り</t>
         </is>
       </c>
       <c r="E144" t="b">
@@ -7977,12 +7993,12 @@
       </c>
       <c r="G144" t="inlineStr">
         <is>
-          <t>2026年10月～ テレビ朝日「PicoAniTime」にて</t>
+          <t>2026年10月～ 全国フジテレビ系“ ノイタミナ ”にて</t>
         </is>
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>MOZU STUDIOS</t>
+          <t>david production</t>
         </is>
       </c>
       <c r="I144" t="inlineStr"/>
@@ -7991,7 +8007,7 @@
       <c r="L144" t="inlineStr"/>
       <c r="M144" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27823</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27415</t>
         </is>
       </c>
     </row>
@@ -8009,7 +8025,7 @@
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>ホテル・インヒューマンズ 第2期</t>
+          <t>ポップパップポルターズ</t>
         </is>
       </c>
       <c r="E145" t="b">
@@ -8022,12 +8038,12 @@
       </c>
       <c r="G145" t="inlineStr">
         <is>
-          <t>2026年10月～ テレ東系列ほか</t>
+          <t>2026年10月～ テレビ朝日「PicoAniTime」にて</t>
         </is>
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>ブリッジ</t>
+          <t>MOZU STUDIOS</t>
         </is>
       </c>
       <c r="I145" t="inlineStr"/>
@@ -8036,7 +8052,7 @@
       <c r="L145" t="inlineStr"/>
       <c r="M145" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26870</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27823</t>
         </is>
       </c>
     </row>
@@ -8054,7 +8070,7 @@
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>マジカル★エクスプローラー</t>
+          <t>ホテル・インヒューマンズ 第2期</t>
         </is>
       </c>
       <c r="E146" t="b">
@@ -8067,12 +8083,12 @@
       </c>
       <c r="G146" t="inlineStr">
         <is>
-          <t>2026年秋</t>
+          <t>2026年10月～ テレ東系列ほか</t>
         </is>
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>WHITE FOX</t>
+          <t>ブリッジ</t>
         </is>
       </c>
       <c r="I146" t="inlineStr"/>
@@ -8081,7 +8097,7 @@
       <c r="L146" t="inlineStr"/>
       <c r="M146" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=23375</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26870</t>
         </is>
       </c>
     </row>
@@ -8099,7 +8115,7 @@
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>魔法騎士レイアース</t>
+          <t>マジカル★エクスプローラー</t>
         </is>
       </c>
       <c r="E147" t="b">
@@ -8112,12 +8128,12 @@
       </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t>2026年10月7日（水）～ テレビ朝日系列にて</t>
+          <t>2026年秋</t>
         </is>
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>E&amp;H production</t>
+          <t>WHITE FOX</t>
         </is>
       </c>
       <c r="I147" t="inlineStr"/>
@@ -8126,7 +8142,7 @@
       <c r="L147" t="inlineStr"/>
       <c r="M147" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=24301</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=23375</t>
         </is>
       </c>
     </row>
@@ -8144,7 +8160,7 @@
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>魔法少女育成計画restart</t>
+          <t>魔法騎士レイアース</t>
         </is>
       </c>
       <c r="E148" t="b">
@@ -8157,29 +8173,21 @@
       </c>
       <c r="G148" t="inlineStr">
         <is>
-          <t>2026年秋</t>
+          <t>2026年10月7日（水）～ テレビ朝日系列にて</t>
         </is>
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>SynergySP</t>
-        </is>
-      </c>
-      <c r="I148" t="inlineStr">
-        <is>
-          <t>No tears here</t>
-        </is>
-      </c>
-      <c r="J148" t="inlineStr">
-        <is>
-          <t>茅原実里</t>
-        </is>
-      </c>
+          <t>E&amp;H production</t>
+        </is>
+      </c>
+      <c r="I148" t="inlineStr"/>
+      <c r="J148" t="inlineStr"/>
       <c r="K148" t="inlineStr"/>
       <c r="L148" t="inlineStr"/>
       <c r="M148" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26693</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=24301</t>
         </is>
       </c>
     </row>
@@ -8197,7 +8205,7 @@
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>魔法の姉妹ルルットリリィ 第2クール</t>
+          <t>魔法少女育成計画restart</t>
         </is>
       </c>
       <c r="E149" t="b">
@@ -8210,37 +8218,29 @@
       </c>
       <c r="G149" t="inlineStr">
         <is>
-          <t>第1クール：2026年4月5日（日）～2026年6月21日（日） 第2クール：2026年10月～ TOKYO MX・ABCテレビほか</t>
+          <t>2026年秋</t>
         </is>
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>スタジオぴえろ</t>
+          <t>SynergySP</t>
         </is>
       </c>
       <c r="I149" t="inlineStr">
         <is>
-          <t>Bubee</t>
+          <t>No tears here</t>
         </is>
       </c>
       <c r="J149" t="inlineStr">
         <is>
-          <t>ILLIT</t>
-        </is>
-      </c>
-      <c r="K149" t="inlineStr">
-        <is>
-          <t>Calling</t>
-        </is>
-      </c>
-      <c r="L149" t="inlineStr">
-        <is>
-          <t>ルルットリリィ（こんぺとリリィ（CV.橘めい）、ましゅールル（CV.小鹿なお））</t>
-        </is>
-      </c>
+          <t>茅原実里</t>
+        </is>
+      </c>
+      <c r="K149" t="inlineStr"/>
+      <c r="L149" t="inlineStr"/>
       <c r="M149" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=24293</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26693</t>
         </is>
       </c>
     </row>
@@ -8258,7 +8258,7 @@
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>マロニエ王国の七人の騎士</t>
+          <t>魔法の姉妹ルルットリリィ 第2クール</t>
         </is>
       </c>
       <c r="E150" t="b">
@@ -8271,21 +8271,37 @@
       </c>
       <c r="G150" t="inlineStr">
         <is>
-          <t>2026年10月～ NHK Eテレにて</t>
+          <t>第1クール：2026年4月5日（日）～2026年6月21日（日） 第2クール：2026年10月～ TOKYO MX・ABCテレビほか</t>
         </is>
       </c>
       <c r="H150" t="inlineStr">
         <is>
-          <t>J.C.STAFF</t>
-        </is>
-      </c>
-      <c r="I150" t="inlineStr"/>
-      <c r="J150" t="inlineStr"/>
-      <c r="K150" t="inlineStr"/>
-      <c r="L150" t="inlineStr"/>
+          <t>スタジオぴえろ</t>
+        </is>
+      </c>
+      <c r="I150" t="inlineStr">
+        <is>
+          <t>Bubee</t>
+        </is>
+      </c>
+      <c r="J150" t="inlineStr">
+        <is>
+          <t>ILLIT</t>
+        </is>
+      </c>
+      <c r="K150" t="inlineStr">
+        <is>
+          <t>Calling</t>
+        </is>
+      </c>
+      <c r="L150" t="inlineStr">
+        <is>
+          <t>ルルットリリィ（こんぺとリリィ（CV.橘めい）、ましゅールル（CV.小鹿なお））</t>
+        </is>
+      </c>
       <c r="M150" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28456</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=24293</t>
         </is>
       </c>
     </row>
@@ -8303,7 +8319,7 @@
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>目覚めたら最強装備と宇宙船持ちだったので、一戸建て目指して傭兵として自由に生きたい</t>
+          <t>マロニエ王国の七人の騎士</t>
         </is>
       </c>
       <c r="E151" t="b">
@@ -8316,37 +8332,21 @@
       </c>
       <c r="G151" t="inlineStr">
         <is>
-          <t>2026年10月〜 TOKYO MX・読売テレビ・中京テレビほか</t>
+          <t>2026年10月～ NHK Eテレにて</t>
         </is>
       </c>
       <c r="H151" t="inlineStr">
         <is>
-          <t>studio A-CAT</t>
-        </is>
-      </c>
-      <c r="I151" t="inlineStr">
-        <is>
-          <t>UNSTOPPABLE</t>
-        </is>
-      </c>
-      <c r="J151" t="inlineStr">
-        <is>
-          <t>FLOW</t>
-        </is>
-      </c>
-      <c r="K151" t="inlineStr">
-        <is>
-          <t>MY WAY</t>
-        </is>
-      </c>
-      <c r="L151" t="inlineStr">
-        <is>
-          <t>ASTERISM</t>
-        </is>
-      </c>
+          <t>J.C.STAFF</t>
+        </is>
+      </c>
+      <c r="I151" t="inlineStr"/>
+      <c r="J151" t="inlineStr"/>
+      <c r="K151" t="inlineStr"/>
+      <c r="L151" t="inlineStr"/>
       <c r="M151" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25525</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28456</t>
         </is>
       </c>
     </row>
@@ -8364,7 +8364,7 @@
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>ゆるゆる図鑑</t>
+          <t>目覚めたら最強装備と宇宙船持ちだったので、一戸建て目指して傭兵として自由に生きたい</t>
         </is>
       </c>
       <c r="E152" t="b">
@@ -8377,17 +8377,37 @@
       </c>
       <c r="G152" t="inlineStr">
         <is>
-          <t>2026年10月～ テレ東系列6局ネット「アニもり！」内にて</t>
-        </is>
-      </c>
-      <c r="H152" t="inlineStr"/>
-      <c r="I152" t="inlineStr"/>
-      <c r="J152" t="inlineStr"/>
-      <c r="K152" t="inlineStr"/>
-      <c r="L152" t="inlineStr"/>
+          <t>2026年10月〜 TOKYO MX・読売テレビ・中京テレビほか</t>
+        </is>
+      </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>studio A-CAT</t>
+        </is>
+      </c>
+      <c r="I152" t="inlineStr">
+        <is>
+          <t>UNSTOPPABLE</t>
+        </is>
+      </c>
+      <c r="J152" t="inlineStr">
+        <is>
+          <t>FLOW</t>
+        </is>
+      </c>
+      <c r="K152" t="inlineStr">
+        <is>
+          <t>MY WAY</t>
+        </is>
+      </c>
+      <c r="L152" t="inlineStr">
+        <is>
+          <t>ASTERISM</t>
+        </is>
+      </c>
       <c r="M152" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28579</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25525</t>
         </is>
       </c>
     </row>
@@ -8405,7 +8425,7 @@
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>夜桜さんちの大作戦 第2期 第2クール</t>
+          <t>ゆるゆる図鑑</t>
         </is>
       </c>
       <c r="E153" t="b">
@@ -8418,37 +8438,17 @@
       </c>
       <c r="G153" t="inlineStr">
         <is>
-          <t>第1クール：2026年4月12日（日）～2026年6月28日（日） 第2クール：2026年10月〜 MBS／TBS系全国28局ネットにて</t>
-        </is>
-      </c>
-      <c r="H153" t="inlineStr">
-        <is>
-          <t>SILVER LINK.</t>
-        </is>
-      </c>
-      <c r="I153" t="inlineStr">
-        <is>
-          <t>What's "KAZOKU"</t>
-        </is>
-      </c>
-      <c r="J153" t="inlineStr">
-        <is>
-          <t>櫻坂46</t>
-        </is>
-      </c>
-      <c r="K153" t="inlineStr">
-        <is>
-          <t>Shalala</t>
-        </is>
-      </c>
-      <c r="L153" t="inlineStr">
-        <is>
-          <t>ピラフ星人</t>
-        </is>
-      </c>
+          <t>2026年10月～ テレ東系列6局ネット「アニもり！」内にて</t>
+        </is>
+      </c>
+      <c r="H153" t="inlineStr"/>
+      <c r="I153" t="inlineStr"/>
+      <c r="J153" t="inlineStr"/>
+      <c r="K153" t="inlineStr"/>
+      <c r="L153" t="inlineStr"/>
       <c r="M153" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25032</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28579</t>
         </is>
       </c>
     </row>
@@ -8466,7 +8466,7 @@
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>弱気MAX令嬢なのに、辣腕婚約者様の賭けに乗ってしまった</t>
+          <t>夜桜さんちの大作戦 第2期 第2クール</t>
         </is>
       </c>
       <c r="E154" t="b">
@@ -8479,21 +8479,37 @@
       </c>
       <c r="G154" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
+          <t>第1クール：2026年4月12日（日）～2026年6月28日（日） 第2クール：2026年10月〜 MBS／TBS系全国28局ネットにて</t>
         </is>
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>寿門堂</t>
-        </is>
-      </c>
-      <c r="I154" t="inlineStr"/>
-      <c r="J154" t="inlineStr"/>
-      <c r="K154" t="inlineStr"/>
-      <c r="L154" t="inlineStr"/>
+          <t>SILVER LINK.</t>
+        </is>
+      </c>
+      <c r="I154" t="inlineStr">
+        <is>
+          <t>What's "KAZOKU"</t>
+        </is>
+      </c>
+      <c r="J154" t="inlineStr">
+        <is>
+          <t>櫻坂46</t>
+        </is>
+      </c>
+      <c r="K154" t="inlineStr">
+        <is>
+          <t>Shalala</t>
+        </is>
+      </c>
+      <c r="L154" t="inlineStr">
+        <is>
+          <t>ピラフ星人</t>
+        </is>
+      </c>
       <c r="M154" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26947</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25032</t>
         </is>
       </c>
     </row>
@@ -8511,11 +8527,11 @@
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>ラブライブ！虹ヶ咲学園スクールアイドル同好会 第2期</t>
+          <t>弱気MAX令嬢なのに、辣腕婚約者様の賭けに乗ってしまった</t>
         </is>
       </c>
       <c r="E155" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F155" t="inlineStr">
         <is>
@@ -8524,12 +8540,12 @@
       </c>
       <c r="G155" t="inlineStr">
         <is>
-          <t>2022年4月2日（土）～2022年6月25日（土） TOKYO MXほか 【再放送】 2026年9月30日（水）〜 BS日テレにて</t>
+          <t>2026年10月～</t>
         </is>
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>サンライズ</t>
+          <t>寿門堂</t>
         </is>
       </c>
       <c r="I155" t="inlineStr"/>
@@ -8538,7 +8554,7 @@
       <c r="L155" t="inlineStr"/>
       <c r="M155" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=14120</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26947</t>
         </is>
       </c>
     </row>
@@ -8556,11 +8572,11 @@
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>らんま1/2 第3期</t>
+          <t>ラブライブ！虹ヶ咲学園スクールアイドル同好会 第2期</t>
         </is>
       </c>
       <c r="E156" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F156" t="inlineStr">
         <is>
@@ -8569,17 +8585,21 @@
       </c>
       <c r="G156" t="inlineStr">
         <is>
-          <t>2026年10月～ 日本テレビ系にて</t>
-        </is>
-      </c>
-      <c r="H156" t="inlineStr"/>
+          <t>2022年4月2日（土）～2022年6月25日（土） TOKYO MXほか 【再放送】 2026年9月30日（水）〜 BS日テレにて</t>
+        </is>
+      </c>
+      <c r="H156" t="inlineStr">
+        <is>
+          <t>サンライズ</t>
+        </is>
+      </c>
       <c r="I156" t="inlineStr"/>
       <c r="J156" t="inlineStr"/>
       <c r="K156" t="inlineStr"/>
       <c r="L156" t="inlineStr"/>
       <c r="M156" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28013</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=14120</t>
         </is>
       </c>
     </row>
@@ -8597,7 +8617,7 @@
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>LEGO® ONE PIECE</t>
+          <t>らんま1/2 第3期</t>
         </is>
       </c>
       <c r="E157" t="b">
@@ -8605,12 +8625,12 @@
       </c>
       <c r="F157" t="inlineStr">
         <is>
-          <t>配信</t>
+          <t>TVアニメ</t>
         </is>
       </c>
       <c r="G157" t="inlineStr">
         <is>
-          <t>2026年9月29日（火） Netflixにて</t>
+          <t>2026年10月～ 日本テレビ系にて</t>
         </is>
       </c>
       <c r="H157" t="inlineStr"/>
@@ -8619,6 +8639,47 @@
       <c r="K157" t="inlineStr"/>
       <c r="L157" t="inlineStr"/>
       <c r="M157" t="inlineStr">
+        <is>
+          <t>https://www.animatetimes.com/tag/details.php?id=28013</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C158" t="n">
+        <v>70</v>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>LEGO® ONE PIECE</t>
+        </is>
+      </c>
+      <c r="E158" t="b">
+        <v>0</v>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>配信</t>
+        </is>
+      </c>
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>2026年9月29日（火） Netflixにて</t>
+        </is>
+      </c>
+      <c r="H158" t="inlineStr"/>
+      <c r="I158" t="inlineStr"/>
+      <c r="J158" t="inlineStr"/>
+      <c r="K158" t="inlineStr"/>
+      <c r="L158" t="inlineStr"/>
+      <c r="M158" t="inlineStr">
         <is>
           <t>https://www.animatetimes.com/tag/details.php?id=28168</t>
         </is>
@@ -8635,7 +8696,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O177"/>
+  <dimension ref="A1:O179"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8917,13 +8978,37 @@
           <t>Lia</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=k2Gfd254sMg</t>
+        </is>
+      </c>
+      <c r="J5" t="n">
+        <v>15183</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>NBCUniversal Anime/Music</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=k2Gfd254sMg</t>
+        </is>
+      </c>
+      <c r="M5" t="n">
+        <v>15183</v>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>NBCUniversal Anime/Music</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>2026-07-14T09:00:19</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -9009,7 +9094,7 @@
         </is>
       </c>
       <c r="J7" t="n">
-        <v>9401</v>
+        <v>144449</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
@@ -9022,7 +9107,7 @@
         </is>
       </c>
       <c r="M7" t="n">
-        <v>9401</v>
+        <v>144449</v>
       </c>
       <c r="N7" t="inlineStr">
         <is>
@@ -9031,7 +9116,7 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>2026-07-06T09:00:34</t>
+          <t>2026-07-14T09:00:36</t>
         </is>
       </c>
     </row>
@@ -9076,7 +9161,7 @@
         </is>
       </c>
       <c r="J8" t="n">
-        <v>4198</v>
+        <v>13838</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
@@ -9089,7 +9174,7 @@
         </is>
       </c>
       <c r="M8" t="n">
-        <v>4198</v>
+        <v>13838</v>
       </c>
       <c r="N8" t="inlineStr">
         <is>
@@ -9098,7 +9183,7 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>2026-07-06T09:00:43</t>
+          <t>2026-07-14T09:00:46</t>
         </is>
       </c>
     </row>
@@ -9143,7 +9228,7 @@
         </is>
       </c>
       <c r="J9" t="n">
-        <v>30487</v>
+        <v>54112</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
@@ -9156,7 +9241,7 @@
         </is>
       </c>
       <c r="M9" t="n">
-        <v>30487</v>
+        <v>54112</v>
       </c>
       <c r="N9" t="inlineStr">
         <is>
@@ -9165,7 +9250,7 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>2026-07-07T09:00:36</t>
+          <t>2026-07-14T09:00:57</t>
         </is>
       </c>
     </row>
@@ -9210,7 +9295,7 @@
         </is>
       </c>
       <c r="J10" t="n">
-        <v>25246</v>
+        <v>27264</v>
       </c>
       <c r="K10" t="inlineStr">
         <is>
@@ -9223,7 +9308,7 @@
         </is>
       </c>
       <c r="M10" t="n">
-        <v>25246</v>
+        <v>27264</v>
       </c>
       <c r="N10" t="inlineStr">
         <is>
@@ -9232,7 +9317,7 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>2026-07-07T09:00:43</t>
+          <t>2026-07-14T09:01:05</t>
         </is>
       </c>
     </row>
@@ -9273,33 +9358,33 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
+          <t>https://www.youtube.com/watch?v=JNkPfX9bJ_k</t>
+        </is>
+      </c>
+      <c r="J11" t="n">
+        <v>490326</v>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>DISH// official YouTube channel</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
           <t>https://www.youtube.com/watch?v=X_knFby9AJc</t>
         </is>
       </c>
-      <c r="J11" t="n">
-        <v>80021</v>
-      </c>
-      <c r="K11" t="inlineStr">
+      <c r="M11" t="n">
+        <v>93656</v>
+      </c>
+      <c r="N11" t="inlineStr">
         <is>
           <t>アニプレックス チャンネル</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=X_knFby9AJc</t>
-        </is>
-      </c>
-      <c r="M11" t="n">
-        <v>80021</v>
-      </c>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t>アニプレックス チャンネル</t>
-        </is>
-      </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>2026-07-07T09:00:52</t>
+          <t>2026-07-14T09:01:14</t>
         </is>
       </c>
     </row>
@@ -9769,7 +9854,7 @@
         </is>
       </c>
       <c r="J19" t="n">
-        <v>47490</v>
+        <v>190362</v>
       </c>
       <c r="K19" t="inlineStr">
         <is>
@@ -9782,7 +9867,7 @@
         </is>
       </c>
       <c r="M19" t="n">
-        <v>47490</v>
+        <v>190362</v>
       </c>
       <c r="N19" t="inlineStr">
         <is>
@@ -9791,7 +9876,7 @@
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>2026-07-06T09:01:28</t>
+          <t>2026-07-14T09:01:26</t>
         </is>
       </c>
     </row>
@@ -9836,7 +9921,7 @@
         </is>
       </c>
       <c r="J20" t="n">
-        <v>20400</v>
+        <v>88640</v>
       </c>
       <c r="K20" t="inlineStr">
         <is>
@@ -9849,7 +9934,7 @@
         </is>
       </c>
       <c r="M20" t="n">
-        <v>20400</v>
+        <v>88640</v>
       </c>
       <c r="N20" t="inlineStr">
         <is>
@@ -9858,7 +9943,7 @@
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>2026-07-06T09:01:37</t>
+          <t>2026-07-14T09:01:36</t>
         </is>
       </c>
     </row>
@@ -10495,7 +10580,7 @@
         </is>
       </c>
       <c r="J31" t="n">
-        <v>6356365</v>
+        <v>6386624</v>
       </c>
       <c r="K31" t="inlineStr">
         <is>
@@ -10508,7 +10593,7 @@
         </is>
       </c>
       <c r="M31" t="n">
-        <v>6356365</v>
+        <v>6386624</v>
       </c>
       <c r="N31" t="inlineStr">
         <is>
@@ -10517,7 +10602,7 @@
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>2026-07-06T09:01:56</t>
+          <t>2026-07-14T09:01:45</t>
         </is>
       </c>
     </row>
@@ -11315,13 +11400,37 @@
           <t>名称非公開</t>
         </is>
       </c>
-      <c r="I45" t="inlineStr"/>
-      <c r="J45" t="inlineStr"/>
-      <c r="K45" t="inlineStr"/>
-      <c r="L45" t="inlineStr"/>
-      <c r="M45" t="inlineStr"/>
-      <c r="N45" t="inlineStr"/>
-      <c r="O45" t="inlineStr"/>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=UDD-U-c-m9Y</t>
+        </is>
+      </c>
+      <c r="J45" t="n">
+        <v>2391</v>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>GREE Entertainment ANIME &amp; GAME【公式】</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=UDD-U-c-m9Y</t>
+        </is>
+      </c>
+      <c r="M45" t="n">
+        <v>2391</v>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>GREE Entertainment ANIME &amp; GAME【公式】</t>
+        </is>
+      </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>2026-07-14T09:02:21</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -11612,7 +11721,7 @@
         </is>
       </c>
       <c r="J50" t="n">
-        <v>14061</v>
+        <v>78756</v>
       </c>
       <c r="K50" t="inlineStr">
         <is>
@@ -11625,7 +11734,7 @@
         </is>
       </c>
       <c r="M50" t="n">
-        <v>14061</v>
+        <v>78756</v>
       </c>
       <c r="N50" t="inlineStr">
         <is>
@@ -11634,7 +11743,7 @@
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>2026-07-06T09:02:54</t>
+          <t>2026-07-14T09:02:30</t>
         </is>
       </c>
     </row>
@@ -12706,7 +12815,7 @@
         </is>
       </c>
       <c r="J68" t="n">
-        <v>2364</v>
+        <v>14667</v>
       </c>
       <c r="K68" t="inlineStr">
         <is>
@@ -12719,7 +12828,7 @@
         </is>
       </c>
       <c r="M68" t="n">
-        <v>2364</v>
+        <v>14667</v>
       </c>
       <c r="N68" t="inlineStr">
         <is>
@@ -12728,7 +12837,7 @@
       </c>
       <c r="O68" t="inlineStr">
         <is>
-          <t>2026-07-06T09:03:37</t>
+          <t>2026-07-14T09:02:46</t>
         </is>
       </c>
     </row>
@@ -12773,7 +12882,7 @@
         </is>
       </c>
       <c r="J69" t="n">
-        <v>1321</v>
+        <v>5251</v>
       </c>
       <c r="K69" t="inlineStr">
         <is>
@@ -12786,7 +12895,7 @@
         </is>
       </c>
       <c r="M69" t="n">
-        <v>1321</v>
+        <v>5251</v>
       </c>
       <c r="N69" t="inlineStr">
         <is>
@@ -12795,7 +12904,7 @@
       </c>
       <c r="O69" t="inlineStr">
         <is>
-          <t>2026-07-06T09:03:46</t>
+          <t>2026-07-14T09:02:56</t>
         </is>
       </c>
     </row>
@@ -13579,7 +13688,7 @@
         </is>
       </c>
       <c r="J83" t="n">
-        <v>124925</v>
+        <v>726508</v>
       </c>
       <c r="K83" t="inlineStr">
         <is>
@@ -13592,7 +13701,7 @@
         </is>
       </c>
       <c r="M83" t="n">
-        <v>124925</v>
+        <v>726508</v>
       </c>
       <c r="N83" t="inlineStr">
         <is>
@@ -13601,7 +13710,7 @@
       </c>
       <c r="O83" t="inlineStr">
         <is>
-          <t>2026-07-06T09:04:33</t>
+          <t>2026-07-14T09:03:24</t>
         </is>
       </c>
     </row>
@@ -13646,7 +13755,7 @@
         </is>
       </c>
       <c r="J84" t="n">
-        <v>42587</v>
+        <v>155932</v>
       </c>
       <c r="K84" t="inlineStr">
         <is>
@@ -13659,7 +13768,7 @@
         </is>
       </c>
       <c r="M84" t="n">
-        <v>42587</v>
+        <v>155932</v>
       </c>
       <c r="N84" t="inlineStr">
         <is>
@@ -13668,7 +13777,7 @@
       </c>
       <c r="O84" t="inlineStr">
         <is>
-          <t>2026-07-06T09:04:42</t>
+          <t>2026-07-14T09:03:33</t>
         </is>
       </c>
     </row>
@@ -14019,7 +14128,7 @@
         </is>
       </c>
       <c r="J91" t="n">
-        <v>8471</v>
+        <v>73898</v>
       </c>
       <c r="K91" t="inlineStr">
         <is>
@@ -14032,7 +14141,7 @@
         </is>
       </c>
       <c r="M91" t="n">
-        <v>8471</v>
+        <v>73898</v>
       </c>
       <c r="N91" t="inlineStr">
         <is>
@@ -14041,7 +14150,7 @@
       </c>
       <c r="O91" t="inlineStr">
         <is>
-          <t>2026-07-06T09:05:07</t>
+          <t>2026-07-14T09:04:13</t>
         </is>
       </c>
     </row>
@@ -14694,23 +14803,33 @@
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=SN2CGcKOZuY</t>
+          <t>https://www.youtube.com/watch?v=6vv4mJOGoLg</t>
         </is>
       </c>
       <c r="J102" t="n">
-        <v>3525</v>
+        <v>24844</v>
       </c>
       <c r="K102" t="inlineStr">
         <is>
           <t>内田真礼（UCHIDA MAAYA）Official Channel</t>
         </is>
       </c>
-      <c r="L102" t="inlineStr"/>
-      <c r="M102" t="inlineStr"/>
-      <c r="N102" t="inlineStr"/>
+      <c r="L102" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=mGmKY-PB82o</t>
+        </is>
+      </c>
+      <c r="M102" t="n">
+        <v>12833</v>
+      </c>
+      <c r="N102" t="inlineStr">
+        <is>
+          <t>ぽにきゃん-Anime PONY CANYON</t>
+        </is>
+      </c>
       <c r="O102" t="inlineStr">
         <is>
-          <t>2026-07-06T09:05:39</t>
+          <t>2026-07-14T09:04:30</t>
         </is>
       </c>
     </row>
@@ -15554,11 +15673,11 @@
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=IJONbpfIlUg</t>
+          <t>https://www.youtube.com/watch?v=g2iWIWqJ39s</t>
         </is>
       </c>
       <c r="J116" t="n">
-        <v>740213</v>
+        <v>2024420</v>
       </c>
       <c r="K116" t="inlineStr">
         <is>
@@ -15571,7 +15690,7 @@
         </is>
       </c>
       <c r="M116" t="n">
-        <v>253343</v>
+        <v>264298</v>
       </c>
       <c r="N116" t="inlineStr">
         <is>
@@ -15580,7 +15699,7 @@
       </c>
       <c r="O116" t="inlineStr">
         <is>
-          <t>2026-07-06T09:06:00</t>
+          <t>2026-07-14T09:04:52</t>
         </is>
       </c>
     </row>
@@ -15960,23 +16079,33 @@
       </c>
       <c r="I124" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=udTJAApluV4</t>
+          <t>https://www.youtube.com/watch?v=S5BYg1_0u7M</t>
         </is>
       </c>
       <c r="J124" t="n">
-        <v>60</v>
+        <v>78041</v>
       </c>
       <c r="K124" t="inlineStr">
         <is>
-          <t>mogepuff rhythm channel</t>
-        </is>
-      </c>
-      <c r="L124" t="inlineStr"/>
-      <c r="M124" t="inlineStr"/>
-      <c r="N124" t="inlineStr"/>
+          <t>avex pictures</t>
+        </is>
+      </c>
+      <c r="L124" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=S5BYg1_0u7M</t>
+        </is>
+      </c>
+      <c r="M124" t="n">
+        <v>78041</v>
+      </c>
+      <c r="N124" t="inlineStr">
+        <is>
+          <t>avex pictures</t>
+        </is>
+      </c>
       <c r="O124" t="inlineStr">
         <is>
-          <t>2026-07-06T09:06:36</t>
+          <t>2026-07-14T09:05:24</t>
         </is>
       </c>
     </row>
@@ -16711,13 +16840,27 @@
           <t>風輪（徳間ジャパンコミュニケーションズ）</t>
         </is>
       </c>
-      <c r="I137" t="inlineStr"/>
-      <c r="J137" t="inlineStr"/>
-      <c r="K137" t="inlineStr"/>
+      <c r="I137" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=VYlvomHOnO4</t>
+        </is>
+      </c>
+      <c r="J137" t="n">
+        <v>10222</v>
+      </c>
+      <c r="K137" t="inlineStr">
+        <is>
+          <t>闇芝居チャンネル</t>
+        </is>
+      </c>
       <c r="L137" t="inlineStr"/>
       <c r="M137" t="inlineStr"/>
       <c r="N137" t="inlineStr"/>
-      <c r="O137" t="inlineStr"/>
+      <c r="O137" t="inlineStr">
+        <is>
+          <t>2026-07-14T09:05:59</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="n">
@@ -17595,7 +17738,7 @@
         </is>
       </c>
       <c r="J153" t="n">
-        <v>25023</v>
+        <v>548822</v>
       </c>
       <c r="K153" t="inlineStr">
         <is>
@@ -17608,7 +17751,7 @@
         </is>
       </c>
       <c r="M153" t="n">
-        <v>25023</v>
+        <v>548822</v>
       </c>
       <c r="N153" t="inlineStr">
         <is>
@@ -17617,7 +17760,7 @@
       </c>
       <c r="O153" t="inlineStr">
         <is>
-          <t>2026-07-06T09:07:31</t>
+          <t>2026-07-14T09:06:30</t>
         </is>
       </c>
     </row>
@@ -18225,7 +18368,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>デモンズ・クレスト</t>
+          <t>千歳くんはラムネ瓶のなか 第2クール</t>
         </is>
       </c>
       <c r="D165" t="b">
@@ -18241,21 +18384,45 @@
       </c>
       <c r="G165" t="inlineStr">
         <is>
-          <t>シンカ</t>
+          <t>ライアー</t>
         </is>
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>Ado</t>
-        </is>
-      </c>
-      <c r="I165" t="inlineStr"/>
-      <c r="J165" t="inlineStr"/>
-      <c r="K165" t="inlineStr"/>
-      <c r="L165" t="inlineStr"/>
-      <c r="M165" t="inlineStr"/>
-      <c r="N165" t="inlineStr"/>
-      <c r="O165" t="inlineStr"/>
+          <t>Kucci</t>
+        </is>
+      </c>
+      <c r="I165" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=pjGmDIrNgHw</t>
+        </is>
+      </c>
+      <c r="J165" t="n">
+        <v>674766</v>
+      </c>
+      <c r="K165" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="L165" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=pjGmDIrNgHw</t>
+        </is>
+      </c>
+      <c r="M165" t="n">
+        <v>674766</v>
+      </c>
+      <c r="N165" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="O165" t="inlineStr">
+        <is>
+          <t>2026-07-14T09:07:04</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" t="n">
@@ -18268,7 +18435,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>転生した大聖女は、聖女であることをひた隠す</t>
+          <t>千歳くんはラムネ瓶のなか 第2クール</t>
         </is>
       </c>
       <c r="D166" t="b">
@@ -18276,7 +18443,7 @@
       </c>
       <c r="E166" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F166" t="n">
@@ -18284,21 +18451,45 @@
       </c>
       <c r="G166" t="inlineStr">
         <is>
-          <t>Flare of Soul</t>
+          <t>陽炎</t>
         </is>
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>花耶</t>
-        </is>
-      </c>
-      <c r="I166" t="inlineStr"/>
-      <c r="J166" t="inlineStr"/>
-      <c r="K166" t="inlineStr"/>
-      <c r="L166" t="inlineStr"/>
-      <c r="M166" t="inlineStr"/>
-      <c r="N166" t="inlineStr"/>
-      <c r="O166" t="inlineStr"/>
+          <t>サイダーガール</t>
+        </is>
+      </c>
+      <c r="I166" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=ca7_nIyte3I</t>
+        </is>
+      </c>
+      <c r="J166" t="n">
+        <v>367168</v>
+      </c>
+      <c r="K166" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="L166" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=ca7_nIyte3I</t>
+        </is>
+      </c>
+      <c r="M166" t="n">
+        <v>367168</v>
+      </c>
+      <c r="N166" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="O166" t="inlineStr">
+        <is>
+          <t>2026-07-14T09:07:13</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="n">
@@ -18311,7 +18502,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>転生した大聖女は、聖女であることをひた隠す</t>
+          <t>デモンズ・クレスト</t>
         </is>
       </c>
       <c r="D167" t="b">
@@ -18319,7 +18510,7 @@
       </c>
       <c r="E167" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F167" t="n">
@@ -18327,12 +18518,12 @@
       </c>
       <c r="G167" t="inlineStr">
         <is>
-          <t>STELLAR</t>
+          <t>シンカ</t>
         </is>
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>ウタヒメドリーム オールスターズ</t>
+          <t>Ado</t>
         </is>
       </c>
       <c r="I167" t="inlineStr"/>
@@ -18354,7 +18545,7 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>とある暗部の少女共棲</t>
+          <t>転生した大聖女は、聖女であることをひた隠す</t>
         </is>
       </c>
       <c r="D168" t="b">
@@ -18370,12 +18561,12 @@
       </c>
       <c r="G168" t="inlineStr">
         <is>
-          <t>Ghost Sequence</t>
+          <t>Flare of Soul</t>
         </is>
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>East Of Eden</t>
+          <t>花耶</t>
         </is>
       </c>
       <c r="I168" t="inlineStr"/>
@@ -18397,7 +18588,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>とある暗部の少女共棲</t>
+          <t>転生した大聖女は、聖女であることをひた隠す</t>
         </is>
       </c>
       <c r="D169" t="b">
@@ -18413,35 +18604,21 @@
       </c>
       <c r="G169" t="inlineStr">
         <is>
-          <t>原子崩し(メルトダウナー)</t>
+          <t>STELLAR</t>
         </is>
       </c>
       <c r="H169" t="inlineStr">
         <is>
-          <t>岸田教団&amp;THE明星ロケッツ</t>
-        </is>
-      </c>
-      <c r="I169" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=JH927fq9qaM</t>
-        </is>
-      </c>
-      <c r="J169" t="n">
-        <v>2148</v>
-      </c>
-      <c r="K169" t="inlineStr">
-        <is>
-          <t>Kisidakyoudan &amp; the Akebosi rockets official</t>
-        </is>
-      </c>
+          <t>ウタヒメドリーム オールスターズ</t>
+        </is>
+      </c>
+      <c r="I169" t="inlineStr"/>
+      <c r="J169" t="inlineStr"/>
+      <c r="K169" t="inlineStr"/>
       <c r="L169" t="inlineStr"/>
       <c r="M169" t="inlineStr"/>
       <c r="N169" t="inlineStr"/>
-      <c r="O169" t="inlineStr">
-        <is>
-          <t>2026-07-07T09:19:36</t>
-        </is>
-      </c>
+      <c r="O169" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" t="n">
@@ -18454,7 +18631,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>ブラッククローバー 2nd Season</t>
+          <t>とある暗部の少女共棲</t>
         </is>
       </c>
       <c r="D170" t="b">
@@ -18470,12 +18647,12 @@
       </c>
       <c r="G170" t="inlineStr">
         <is>
-          <t>消えない理由</t>
+          <t>Ghost Sequence</t>
         </is>
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>WANIMA</t>
+          <t>East Of Eden</t>
         </is>
       </c>
       <c r="I170" t="inlineStr"/>
@@ -18497,7 +18674,7 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>魔法少女育成計画restart</t>
+          <t>とある暗部の少女共棲</t>
         </is>
       </c>
       <c r="D171" t="b">
@@ -18505,7 +18682,7 @@
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F171" t="n">
@@ -18513,25 +18690,25 @@
       </c>
       <c r="G171" t="inlineStr">
         <is>
-          <t>No tears here</t>
+          <t>原子崩し(メルトダウナー)</t>
         </is>
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>茅原実里</t>
+          <t>岸田教団&amp;THE明星ロケッツ</t>
         </is>
       </c>
       <c r="I171" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=-PX7FqZ55tE</t>
+          <t>https://www.youtube.com/watch?v=JH927fq9qaM</t>
         </is>
       </c>
       <c r="J171" t="n">
-        <v>105963</v>
+        <v>2148</v>
       </c>
       <c r="K171" t="inlineStr">
         <is>
-          <t>TVアニメ「魔法少女育成計画restart」公式チャンネル</t>
+          <t>Kisidakyoudan &amp; the Akebosi rockets official</t>
         </is>
       </c>
       <c r="L171" t="inlineStr"/>
@@ -18539,7 +18716,7 @@
       <c r="N171" t="inlineStr"/>
       <c r="O171" t="inlineStr">
         <is>
-          <t>2026-07-07T09:19:53</t>
+          <t>2026-07-07T09:19:36</t>
         </is>
       </c>
     </row>
@@ -18554,7 +18731,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>魔法の姉妹ルルットリリィ 第2クール</t>
+          <t>ブラッククローバー 2nd Season</t>
         </is>
       </c>
       <c r="D172" t="b">
@@ -18570,45 +18747,21 @@
       </c>
       <c r="G172" t="inlineStr">
         <is>
-          <t>Bubee</t>
+          <t>消えない理由</t>
         </is>
       </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t>ILLIT</t>
-        </is>
-      </c>
-      <c r="I172" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
-        </is>
-      </c>
-      <c r="J172" t="n">
-        <v>290217</v>
-      </c>
-      <c r="K172" t="inlineStr">
-        <is>
-          <t>Bandai Namco Filmworks Channel</t>
-        </is>
-      </c>
-      <c r="L172" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
-        </is>
-      </c>
-      <c r="M172" t="n">
-        <v>290217</v>
-      </c>
-      <c r="N172" t="inlineStr">
-        <is>
-          <t>Bandai Namco Filmworks Channel</t>
-        </is>
-      </c>
-      <c r="O172" t="inlineStr">
-        <is>
-          <t>2026-07-10T09:07:47</t>
-        </is>
-      </c>
+          <t>WANIMA</t>
+        </is>
+      </c>
+      <c r="I172" t="inlineStr"/>
+      <c r="J172" t="inlineStr"/>
+      <c r="K172" t="inlineStr"/>
+      <c r="L172" t="inlineStr"/>
+      <c r="M172" t="inlineStr"/>
+      <c r="N172" t="inlineStr"/>
+      <c r="O172" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" t="n">
@@ -18621,7 +18774,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>魔法の姉妹ルルットリリィ 第2クール</t>
+          <t>魔法少女育成計画restart</t>
         </is>
       </c>
       <c r="D173" t="b">
@@ -18629,7 +18782,7 @@
       </c>
       <c r="E173" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F173" t="n">
@@ -18637,43 +18790,33 @@
       </c>
       <c r="G173" t="inlineStr">
         <is>
-          <t>Calling</t>
+          <t>No tears here</t>
         </is>
       </c>
       <c r="H173" t="inlineStr">
         <is>
-          <t>ルルットリリィ（こんぺとリリィ（CV.橘めい）、ましゅールル（CV.小鹿なお））</t>
+          <t>茅原実里</t>
         </is>
       </c>
       <c r="I173" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
+          <t>https://www.youtube.com/watch?v=-PX7FqZ55tE</t>
         </is>
       </c>
       <c r="J173" t="n">
-        <v>290217</v>
+        <v>105963</v>
       </c>
       <c r="K173" t="inlineStr">
         <is>
-          <t>Bandai Namco Filmworks Channel</t>
-        </is>
-      </c>
-      <c r="L173" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
-        </is>
-      </c>
-      <c r="M173" t="n">
-        <v>290217</v>
-      </c>
-      <c r="N173" t="inlineStr">
-        <is>
-          <t>Bandai Namco Filmworks Channel</t>
-        </is>
-      </c>
+          <t>TVアニメ「魔法少女育成計画restart」公式チャンネル</t>
+        </is>
+      </c>
+      <c r="L173" t="inlineStr"/>
+      <c r="M173" t="inlineStr"/>
+      <c r="N173" t="inlineStr"/>
       <c r="O173" t="inlineStr">
         <is>
-          <t>2026-07-10T09:07:56</t>
+          <t>2026-07-07T09:19:53</t>
         </is>
       </c>
     </row>
@@ -18688,7 +18831,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>目覚めたら最強装備と宇宙船持ちだったので、一戸建て目指して傭兵として自由に生きたい</t>
+          <t>魔法の姉妹ルルットリリィ 第2クール</t>
         </is>
       </c>
       <c r="D174" t="b">
@@ -18704,21 +18847,45 @@
       </c>
       <c r="G174" t="inlineStr">
         <is>
-          <t>UNSTOPPABLE</t>
+          <t>Bubee</t>
         </is>
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>FLOW</t>
-        </is>
-      </c>
-      <c r="I174" t="inlineStr"/>
-      <c r="J174" t="inlineStr"/>
-      <c r="K174" t="inlineStr"/>
-      <c r="L174" t="inlineStr"/>
-      <c r="M174" t="inlineStr"/>
-      <c r="N174" t="inlineStr"/>
-      <c r="O174" t="inlineStr"/>
+          <t>ILLIT</t>
+        </is>
+      </c>
+      <c r="I174" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
+        </is>
+      </c>
+      <c r="J174" t="n">
+        <v>290217</v>
+      </c>
+      <c r="K174" t="inlineStr">
+        <is>
+          <t>Bandai Namco Filmworks Channel</t>
+        </is>
+      </c>
+      <c r="L174" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
+        </is>
+      </c>
+      <c r="M174" t="n">
+        <v>290217</v>
+      </c>
+      <c r="N174" t="inlineStr">
+        <is>
+          <t>Bandai Namco Filmworks Channel</t>
+        </is>
+      </c>
+      <c r="O174" t="inlineStr">
+        <is>
+          <t>2026-07-10T09:07:47</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" t="n">
@@ -18731,7 +18898,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>目覚めたら最強装備と宇宙船持ちだったので、一戸建て目指して傭兵として自由に生きたい</t>
+          <t>魔法の姉妹ルルットリリィ 第2クール</t>
         </is>
       </c>
       <c r="D175" t="b">
@@ -18747,21 +18914,45 @@
       </c>
       <c r="G175" t="inlineStr">
         <is>
-          <t>MY WAY</t>
+          <t>Calling</t>
         </is>
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>ASTERISM</t>
-        </is>
-      </c>
-      <c r="I175" t="inlineStr"/>
-      <c r="J175" t="inlineStr"/>
-      <c r="K175" t="inlineStr"/>
-      <c r="L175" t="inlineStr"/>
-      <c r="M175" t="inlineStr"/>
-      <c r="N175" t="inlineStr"/>
-      <c r="O175" t="inlineStr"/>
+          <t>ルルットリリィ（こんぺとリリィ（CV.橘めい）、ましゅールル（CV.小鹿なお））</t>
+        </is>
+      </c>
+      <c r="I175" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
+        </is>
+      </c>
+      <c r="J175" t="n">
+        <v>290217</v>
+      </c>
+      <c r="K175" t="inlineStr">
+        <is>
+          <t>Bandai Namco Filmworks Channel</t>
+        </is>
+      </c>
+      <c r="L175" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
+        </is>
+      </c>
+      <c r="M175" t="n">
+        <v>290217</v>
+      </c>
+      <c r="N175" t="inlineStr">
+        <is>
+          <t>Bandai Namco Filmworks Channel</t>
+        </is>
+      </c>
+      <c r="O175" t="inlineStr">
+        <is>
+          <t>2026-07-10T09:07:56</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" t="n">
@@ -18774,7 +18965,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>夜桜さんちの大作戦 第2期 第2クール</t>
+          <t>目覚めたら最強装備と宇宙船持ちだったので、一戸建て目指して傭兵として自由に生きたい</t>
         </is>
       </c>
       <c r="D176" t="b">
@@ -18790,45 +18981,21 @@
       </c>
       <c r="G176" t="inlineStr">
         <is>
-          <t>What's "KAZOKU"</t>
+          <t>UNSTOPPABLE</t>
         </is>
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t>櫻坂46</t>
-        </is>
-      </c>
-      <c r="I176" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=4SdeuouXcWI</t>
-        </is>
-      </c>
-      <c r="J176" t="n">
-        <v>669793</v>
-      </c>
-      <c r="K176" t="inlineStr">
-        <is>
-          <t>櫻坂46 OFFICIAL YouTube CHANNEL</t>
-        </is>
-      </c>
-      <c r="L176" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=AIspds2UVts</t>
-        </is>
-      </c>
-      <c r="M176" t="n">
-        <v>347279</v>
-      </c>
-      <c r="N176" t="inlineStr">
-        <is>
-          <t>NBCUniversal Anime/Music</t>
-        </is>
-      </c>
-      <c r="O176" t="inlineStr">
-        <is>
-          <t>2026-07-07T09:20:03</t>
-        </is>
-      </c>
+          <t>FLOW</t>
+        </is>
+      </c>
+      <c r="I176" t="inlineStr"/>
+      <c r="J176" t="inlineStr"/>
+      <c r="K176" t="inlineStr"/>
+      <c r="L176" t="inlineStr"/>
+      <c r="M176" t="inlineStr"/>
+      <c r="N176" t="inlineStr"/>
+      <c r="O176" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" t="n">
@@ -18841,7 +19008,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>夜桜さんちの大作戦 第2期 第2クール</t>
+          <t>目覚めたら最強装備と宇宙船持ちだったので、一戸建て目指して傭兵として自由に生きたい</t>
         </is>
       </c>
       <c r="D177" t="b">
@@ -18857,41 +19024,151 @@
       </c>
       <c r="G177" t="inlineStr">
         <is>
+          <t>MY WAY</t>
+        </is>
+      </c>
+      <c r="H177" t="inlineStr">
+        <is>
+          <t>ASTERISM</t>
+        </is>
+      </c>
+      <c r="I177" t="inlineStr"/>
+      <c r="J177" t="inlineStr"/>
+      <c r="K177" t="inlineStr"/>
+      <c r="L177" t="inlineStr"/>
+      <c r="M177" t="inlineStr"/>
+      <c r="N177" t="inlineStr"/>
+      <c r="O177" t="inlineStr"/>
+    </row>
+    <row r="178">
+      <c r="A178" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>夜桜さんちの大作戦 第2期 第2クール</t>
+        </is>
+      </c>
+      <c r="D178" t="b">
+        <v>0</v>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>OP</t>
+        </is>
+      </c>
+      <c r="F178" t="n">
+        <v>1</v>
+      </c>
+      <c r="G178" t="inlineStr">
+        <is>
+          <t>What's "KAZOKU"</t>
+        </is>
+      </c>
+      <c r="H178" t="inlineStr">
+        <is>
+          <t>櫻坂46</t>
+        </is>
+      </c>
+      <c r="I178" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=4SdeuouXcWI</t>
+        </is>
+      </c>
+      <c r="J178" t="n">
+        <v>669793</v>
+      </c>
+      <c r="K178" t="inlineStr">
+        <is>
+          <t>櫻坂46 OFFICIAL YouTube CHANNEL</t>
+        </is>
+      </c>
+      <c r="L178" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=AIspds2UVts</t>
+        </is>
+      </c>
+      <c r="M178" t="n">
+        <v>347279</v>
+      </c>
+      <c r="N178" t="inlineStr">
+        <is>
+          <t>NBCUniversal Anime/Music</t>
+        </is>
+      </c>
+      <c r="O178" t="inlineStr">
+        <is>
+          <t>2026-07-07T09:20:03</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>夜桜さんちの大作戦 第2期 第2クール</t>
+        </is>
+      </c>
+      <c r="D179" t="b">
+        <v>0</v>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>ED</t>
+        </is>
+      </c>
+      <c r="F179" t="n">
+        <v>1</v>
+      </c>
+      <c r="G179" t="inlineStr">
+        <is>
           <t>Shalala</t>
         </is>
       </c>
-      <c r="H177" t="inlineStr">
+      <c r="H179" t="inlineStr">
         <is>
           <t>ピラフ星人</t>
         </is>
       </c>
-      <c r="I177" t="inlineStr">
+      <c r="I179" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=X6fNe1uPs9E</t>
         </is>
       </c>
-      <c r="J177" t="n">
+      <c r="J179" t="n">
         <v>369976</v>
       </c>
-      <c r="K177" t="inlineStr">
+      <c r="K179" t="inlineStr">
         <is>
           <t>NBCUniversal Anime/Music</t>
         </is>
       </c>
-      <c r="L177" t="inlineStr">
+      <c r="L179" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=X6fNe1uPs9E</t>
         </is>
       </c>
-      <c r="M177" t="n">
+      <c r="M179" t="n">
         <v>369976</v>
       </c>
-      <c r="N177" t="inlineStr">
+      <c r="N179" t="inlineStr">
         <is>
           <t>NBCUniversal Anime/Music</t>
         </is>
       </c>
-      <c r="O177" t="inlineStr">
+      <c r="O179" t="inlineStr">
         <is>
           <t>2026-07-07T09:20:12</t>
         </is>

</xml_diff>

<commit_message>
auto: anime list update (PC) 2026-07-16
</commit_message>
<xml_diff>
--- a/data/anime_list.xlsx
+++ b/data/anime_list.xlsx
@@ -10942,13 +10942,37 @@
           <t>前島麻由</t>
         </is>
       </c>
-      <c r="I36" t="inlineStr"/>
-      <c r="J36" t="inlineStr"/>
-      <c r="K36" t="inlineStr"/>
-      <c r="L36" t="inlineStr"/>
-      <c r="M36" t="inlineStr"/>
-      <c r="N36" t="inlineStr"/>
-      <c r="O36" t="inlineStr"/>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=SiTi3WCmzfc</t>
+        </is>
+      </c>
+      <c r="J36" t="n">
+        <v>6984</v>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=SiTi3WCmzfc</t>
+        </is>
+      </c>
+      <c r="M36" t="n">
+        <v>6984</v>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>2026-07-16T09:01:01</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -10985,13 +11009,37 @@
           <t>MYTH &amp; ROID</t>
         </is>
       </c>
-      <c r="I37" t="inlineStr"/>
-      <c r="J37" t="inlineStr"/>
-      <c r="K37" t="inlineStr"/>
-      <c r="L37" t="inlineStr"/>
-      <c r="M37" t="inlineStr"/>
-      <c r="N37" t="inlineStr"/>
-      <c r="O37" t="inlineStr"/>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=Tbyi0Tx1QLA</t>
+        </is>
+      </c>
+      <c r="J37" t="n">
+        <v>5191</v>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=Tbyi0Tx1QLA</t>
+        </is>
+      </c>
+      <c r="M37" t="n">
+        <v>5191</v>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>2026-07-16T09:01:09</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -17191,13 +17239,37 @@
           <t>MYTH &amp; ROID</t>
         </is>
       </c>
-      <c r="I139" t="inlineStr"/>
-      <c r="J139" t="inlineStr"/>
-      <c r="K139" t="inlineStr"/>
-      <c r="L139" t="inlineStr"/>
-      <c r="M139" t="inlineStr"/>
-      <c r="N139" t="inlineStr"/>
-      <c r="O139" t="inlineStr"/>
+      <c r="I139" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=IVyvkwvsqW0</t>
+        </is>
+      </c>
+      <c r="J139" t="n">
+        <v>43946</v>
+      </c>
+      <c r="K139" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="L139" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=IVyvkwvsqW0</t>
+        </is>
+      </c>
+      <c r="M139" t="n">
+        <v>43946</v>
+      </c>
+      <c r="N139" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="O139" t="inlineStr">
+        <is>
+          <t>2026-07-16T09:03:08</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="n">
@@ -17234,13 +17306,37 @@
           <t>ターニャ・デグレチャフ（CV：悠木碧）</t>
         </is>
       </c>
-      <c r="I140" t="inlineStr"/>
-      <c r="J140" t="inlineStr"/>
-      <c r="K140" t="inlineStr"/>
-      <c r="L140" t="inlineStr"/>
-      <c r="M140" t="inlineStr"/>
-      <c r="N140" t="inlineStr"/>
-      <c r="O140" t="inlineStr"/>
+      <c r="I140" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=x2k_iYCGKvE</t>
+        </is>
+      </c>
+      <c r="J140" t="n">
+        <v>24116</v>
+      </c>
+      <c r="K140" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="L140" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=x2k_iYCGKvE</t>
+        </is>
+      </c>
+      <c r="M140" t="n">
+        <v>24116</v>
+      </c>
+      <c r="N140" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="O140" t="inlineStr">
+        <is>
+          <t>2026-07-16T09:03:17</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="n">

</xml_diff>

<commit_message>
auto: anime list update (PC) 2026-07-17
</commit_message>
<xml_diff>
--- a/data/anime_list.xlsx
+++ b/data/anime_list.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M159"/>
+  <dimension ref="A1:M160"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5735,7 +5735,7 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>仮面ライダーマイス</t>
+          <t>彼方から</t>
         </is>
       </c>
       <c r="E95" t="b">
@@ -5743,22 +5743,26 @@
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>特撮</t>
+          <t>TVアニメ</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>2026年9月〜 テレビ朝日系列にて</t>
-        </is>
-      </c>
-      <c r="H95" t="inlineStr"/>
+          <t>2026年10⽉4⽇（⽇）～ TOKYO MXほか</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>スタジオディーン</t>
+        </is>
+      </c>
       <c r="I95" t="inlineStr"/>
       <c r="J95" t="inlineStr"/>
       <c r="K95" t="inlineStr"/>
       <c r="L95" t="inlineStr"/>
       <c r="M95" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28713</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27963</t>
         </is>
       </c>
     </row>
@@ -5776,7 +5780,7 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>帰還者の魔法は特別です 第2期</t>
+          <t>仮面ライダーマイス</t>
         </is>
       </c>
       <c r="E96" t="b">
@@ -5784,42 +5788,22 @@
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>TVアニメ</t>
+          <t>特撮</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>2026年10月〜 フジテレビ「＋Ultra」ほか</t>
-        </is>
-      </c>
-      <c r="H96" t="inlineStr">
-        <is>
-          <t>アルボアニメーション</t>
-        </is>
-      </c>
-      <c r="I96" t="inlineStr">
-        <is>
-          <t>Sorrow</t>
-        </is>
-      </c>
-      <c r="J96" t="inlineStr">
-        <is>
-          <t>FLOW</t>
-        </is>
-      </c>
-      <c r="K96" t="inlineStr">
-        <is>
-          <t>Everlasting</t>
-        </is>
-      </c>
-      <c r="L96" t="inlineStr">
-        <is>
-          <t>krage</t>
-        </is>
-      </c>
+          <t>2026年9月〜 テレビ朝日系列にて</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr"/>
+      <c r="I96" t="inlineStr"/>
+      <c r="J96" t="inlineStr"/>
+      <c r="K96" t="inlineStr"/>
+      <c r="L96" t="inlineStr"/>
       <c r="M96" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=23327</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28713</t>
         </is>
       </c>
     </row>
@@ -5837,7 +5821,7 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>傷だらけ聖女より報復をこめて Season2</t>
+          <t>帰還者の魔法は特別です 第2期</t>
         </is>
       </c>
       <c r="E97" t="b">
@@ -5850,21 +5834,37 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>2026年10月1日（木）〜 テレビ神奈川・CBCテレビにて</t>
+          <t>2026年10月〜 フジテレビ「＋Ultra」ほか</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>Imagica Infos</t>
-        </is>
-      </c>
-      <c r="I97" t="inlineStr"/>
-      <c r="J97" t="inlineStr"/>
-      <c r="K97" t="inlineStr"/>
-      <c r="L97" t="inlineStr"/>
+          <t>アルボアニメーション</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>Sorrow</t>
+        </is>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>FLOW</t>
+        </is>
+      </c>
+      <c r="K97" t="inlineStr">
+        <is>
+          <t>Everlasting</t>
+        </is>
+      </c>
+      <c r="L97" t="inlineStr">
+        <is>
+          <t>krage</t>
+        </is>
+      </c>
       <c r="M97" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25118</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=23327</t>
         </is>
       </c>
     </row>
@@ -5882,7 +5882,7 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>恐怖コレクター</t>
+          <t>傷だらけ聖女より報復をこめて Season2</t>
         </is>
       </c>
       <c r="E98" t="b">
@@ -5895,17 +5895,21 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>2026年10月～ NHK総合にて</t>
-        </is>
-      </c>
-      <c r="H98" t="inlineStr"/>
+          <t>2026年10月1日（木）〜 テレビ神奈川・CBCテレビにて</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>Imagica Infos</t>
+        </is>
+      </c>
       <c r="I98" t="inlineStr"/>
       <c r="J98" t="inlineStr"/>
       <c r="K98" t="inlineStr"/>
       <c r="L98" t="inlineStr"/>
       <c r="M98" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27214</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25118</t>
         </is>
       </c>
     </row>
@@ -5923,7 +5927,7 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>凶乱令嬢ニア・リストン 病弱令嬢に転生した神殺しの武人の華麗なる無双録</t>
+          <t>恐怖コレクター</t>
         </is>
       </c>
       <c r="E99" t="b">
@@ -5936,21 +5940,17 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
-        </is>
-      </c>
-      <c r="H99" t="inlineStr">
-        <is>
-          <t>KONAMI animation</t>
-        </is>
-      </c>
+          <t>2026年10月～ NHK総合にて</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr"/>
       <c r="I99" t="inlineStr"/>
       <c r="J99" t="inlineStr"/>
       <c r="K99" t="inlineStr"/>
       <c r="L99" t="inlineStr"/>
       <c r="M99" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27537</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27214</t>
         </is>
       </c>
     </row>
@@ -5968,7 +5968,7 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>薬屋のひとりごと 第3期</t>
+          <t>凶乱令嬢ニア・リストン 病弱令嬢に転生した神殺しの武人の華麗なる無双録</t>
         </is>
       </c>
       <c r="E100" t="b">
@@ -5981,17 +5981,21 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>第1クール：2026年10月～ 第2クール：2027年4月～ 日本テレビ系にて</t>
-        </is>
-      </c>
-      <c r="H100" t="inlineStr"/>
+          <t>2026年10月～</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>KONAMI animation</t>
+        </is>
+      </c>
       <c r="I100" t="inlineStr"/>
       <c r="J100" t="inlineStr"/>
       <c r="K100" t="inlineStr"/>
       <c r="L100" t="inlineStr"/>
       <c r="M100" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26369</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27537</t>
         </is>
       </c>
     </row>
@@ -6009,7 +6013,7 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>ケロロ軍曹☆</t>
+          <t>薬屋のひとりごと 第3期</t>
         </is>
       </c>
       <c r="E101" t="b">
@@ -6022,7 +6026,7 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>2026年秋</t>
+          <t>第1クール：2026年10月～ 第2クール：2027年4月～ 日本テレビ系にて</t>
         </is>
       </c>
       <c r="H101" t="inlineStr"/>
@@ -6032,7 +6036,7 @@
       <c r="L101" t="inlineStr"/>
       <c r="M101" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27337</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26369</t>
         </is>
       </c>
     </row>
@@ -6050,7 +6054,7 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>幻想水滸伝</t>
+          <t>ケロロ軍曹☆</t>
         </is>
       </c>
       <c r="E102" t="b">
@@ -6063,25 +6067,17 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>2026年10月～ TOKYO MX ほか</t>
+          <t>2026年秋</t>
         </is>
       </c>
       <c r="H102" t="inlineStr"/>
-      <c r="I102" t="inlineStr">
-        <is>
-          <t>悲しみさえ大人びて</t>
-        </is>
-      </c>
-      <c r="J102" t="inlineStr">
-        <is>
-          <t>amazarashi</t>
-        </is>
-      </c>
+      <c r="I102" t="inlineStr"/>
+      <c r="J102" t="inlineStr"/>
       <c r="K102" t="inlineStr"/>
       <c r="L102" t="inlineStr"/>
       <c r="M102" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25616</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27337</t>
         </is>
       </c>
     </row>
@@ -6099,7 +6095,7 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>氷の城壁 第2期</t>
+          <t>幻想水滸伝</t>
         </is>
       </c>
       <c r="E103" t="b">
@@ -6112,21 +6108,25 @@
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>2026年10月1日（木）～ TBS系28局にて</t>
-        </is>
-      </c>
-      <c r="H103" t="inlineStr">
-        <is>
-          <t>スタジオKAI</t>
-        </is>
-      </c>
-      <c r="I103" t="inlineStr"/>
-      <c r="J103" t="inlineStr"/>
+          <t>2026年10月～ TOKYO MX ほか</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr"/>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>悲しみさえ大人びて</t>
+        </is>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>amazarashi</t>
+        </is>
+      </c>
       <c r="K103" t="inlineStr"/>
       <c r="L103" t="inlineStr"/>
       <c r="M103" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25508</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25616</t>
         </is>
       </c>
     </row>
@@ -6144,7 +6144,7 @@
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>サイバーパンク：エッジランナーズ2</t>
+          <t>氷の城壁 第2期</t>
         </is>
       </c>
       <c r="E104" t="b">
@@ -6152,17 +6152,17 @@
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>配信</t>
+          <t>TVアニメ</t>
         </is>
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>2026年秋 Netflixにて</t>
+          <t>2026年10月1日（木）～ TBS系28局にて</t>
         </is>
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>TRIGGER</t>
+          <t>スタジオKAI</t>
         </is>
       </c>
       <c r="I104" t="inlineStr"/>
@@ -6171,7 +6171,7 @@
       <c r="L104" t="inlineStr"/>
       <c r="M104" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28680</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25508</t>
         </is>
       </c>
     </row>
@@ -6189,7 +6189,7 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>PSYREN -サイレン-</t>
+          <t>サイバーパンク：エッジランナーズ2</t>
         </is>
       </c>
       <c r="E105" t="b">
@@ -6197,17 +6197,17 @@
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>TVアニメ</t>
+          <t>配信</t>
         </is>
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>2026年10月～ TOKYO MX・BS11ほか</t>
+          <t>2026年秋 Netflixにて</t>
         </is>
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>サテライト</t>
+          <t>TRIGGER</t>
         </is>
       </c>
       <c r="I105" t="inlineStr"/>
@@ -6216,7 +6216,7 @@
       <c r="L105" t="inlineStr"/>
       <c r="M105" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27257</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28680</t>
         </is>
       </c>
     </row>
@@ -6234,7 +6234,7 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>佐々木とピーちゃん シーズン２</t>
+          <t>PSYREN -サイレン-</t>
         </is>
       </c>
       <c r="E106" t="b">
@@ -6247,12 +6247,12 @@
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
+          <t>2026年10月～ TOKYO MX・BS11ほか</t>
         </is>
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>SILVER LINK.</t>
+          <t>サテライト</t>
         </is>
       </c>
       <c r="I106" t="inlineStr"/>
@@ -6261,7 +6261,7 @@
       <c r="L106" t="inlineStr"/>
       <c r="M106" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=23804</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27257</t>
         </is>
       </c>
     </row>
@@ -6279,7 +6279,7 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>塩対応の佐藤さんが俺にだけ甘い</t>
+          <t>佐々木とピーちゃん シーズン２</t>
         </is>
       </c>
       <c r="E107" t="b">
@@ -6295,14 +6295,18 @@
           <t>2026年10月～</t>
         </is>
       </c>
-      <c r="H107" t="inlineStr"/>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>SILVER LINK.</t>
+        </is>
+      </c>
       <c r="I107" t="inlineStr"/>
       <c r="J107" t="inlineStr"/>
       <c r="K107" t="inlineStr"/>
       <c r="L107" t="inlineStr"/>
       <c r="M107" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27964</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=23804</t>
         </is>
       </c>
     </row>
@@ -6320,7 +6324,7 @@
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>紫禁・御猫房〜紫禁城猫警備室〜</t>
+          <t>塩対応の佐藤さんが俺にだけ甘い</t>
         </is>
       </c>
       <c r="E108" t="b">
@@ -6343,7 +6347,7 @@
       <c r="L108" t="inlineStr"/>
       <c r="M108" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28779</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27964</t>
         </is>
       </c>
     </row>
@@ -6361,7 +6365,7 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>ジャンケットバンク</t>
+          <t>紫禁・御猫房〜紫禁城猫警備室〜</t>
         </is>
       </c>
       <c r="E109" t="b">
@@ -6377,18 +6381,14 @@
           <t>2026年10月～</t>
         </is>
       </c>
-      <c r="H109" t="inlineStr">
-        <is>
-          <t>CUE</t>
-        </is>
-      </c>
+      <c r="H109" t="inlineStr"/>
       <c r="I109" t="inlineStr"/>
       <c r="J109" t="inlineStr"/>
       <c r="K109" t="inlineStr"/>
       <c r="L109" t="inlineStr"/>
       <c r="M109" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27908</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28779</t>
         </is>
       </c>
     </row>
@@ -6406,7 +6406,7 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>朱色の仮面</t>
+          <t>ジャンケットバンク</t>
         </is>
       </c>
       <c r="E110" t="b">
@@ -6419,17 +6419,21 @@
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>2026年10月～ 読売テレビ・日本テレビ系全国ネットにて</t>
-        </is>
-      </c>
-      <c r="H110" t="inlineStr"/>
+          <t>2026年10月～ テレ東系列にて</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>CUE</t>
+        </is>
+      </c>
       <c r="I110" t="inlineStr"/>
       <c r="J110" t="inlineStr"/>
       <c r="K110" t="inlineStr"/>
       <c r="L110" t="inlineStr"/>
       <c r="M110" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26362</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27908</t>
         </is>
       </c>
     </row>
@@ -6447,7 +6451,7 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>獣王武神ダンデヴァイン</t>
+          <t>朱色の仮面</t>
         </is>
       </c>
       <c r="E111" t="b">
@@ -6460,29 +6464,17 @@
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
-        </is>
-      </c>
-      <c r="H111" t="inlineStr">
-        <is>
-          <t>ライデンフィルム</t>
-        </is>
-      </c>
-      <c r="I111" t="inlineStr">
-        <is>
-          <t>曲名未発表</t>
-        </is>
-      </c>
-      <c r="J111" t="inlineStr">
-        <is>
-          <t>西川貴教</t>
-        </is>
-      </c>
+          <t>2026年10月～ 読売テレビ・日本テレビ系全国ネットにて</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr"/>
+      <c r="I111" t="inlineStr"/>
+      <c r="J111" t="inlineStr"/>
       <c r="K111" t="inlineStr"/>
       <c r="L111" t="inlineStr"/>
       <c r="M111" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28479</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26362</t>
         </is>
       </c>
     </row>
@@ -6500,7 +6492,7 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>しろたん</t>
+          <t>獣王武神ダンデヴァイン</t>
         </is>
       </c>
       <c r="E112" t="b">
@@ -6513,21 +6505,29 @@
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>2026年10月～ テレビ朝日にて</t>
+          <t>2026年10月～</t>
         </is>
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>レスプリ</t>
-        </is>
-      </c>
-      <c r="I112" t="inlineStr"/>
-      <c r="J112" t="inlineStr"/>
+          <t>ライデンフィルム</t>
+        </is>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>曲名未発表</t>
+        </is>
+      </c>
+      <c r="J112" t="inlineStr">
+        <is>
+          <t>西川貴教</t>
+        </is>
+      </c>
       <c r="K112" t="inlineStr"/>
       <c r="L112" t="inlineStr"/>
       <c r="M112" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27989</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28479</t>
         </is>
       </c>
     </row>
@@ -6545,7 +6545,7 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>信者ゼロの女神サマと始める異世界攻略</t>
+          <t>しろたん</t>
         </is>
       </c>
       <c r="E113" t="b">
@@ -6558,12 +6558,12 @@
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
+          <t>2026年10月～ テレビ朝日にて</t>
         </is>
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>HORNETS</t>
+          <t>レスプリ</t>
         </is>
       </c>
       <c r="I113" t="inlineStr"/>
@@ -6572,7 +6572,7 @@
       <c r="L113" t="inlineStr"/>
       <c r="M113" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27418</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27989</t>
         </is>
       </c>
     </row>
@@ -6590,7 +6590,7 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>新テニスの王子様 U-17 WORLD CUP 決勝メンバー決定戦</t>
+          <t>信者ゼロの女神サマと始める異世界攻略</t>
         </is>
       </c>
       <c r="E114" t="b">
@@ -6603,17 +6603,21 @@
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>2026年秋</t>
-        </is>
-      </c>
-      <c r="H114" t="inlineStr"/>
+          <t>2026年10月～</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>HORNETS</t>
+        </is>
+      </c>
       <c r="I114" t="inlineStr"/>
       <c r="J114" t="inlineStr"/>
       <c r="K114" t="inlineStr"/>
       <c r="L114" t="inlineStr"/>
       <c r="M114" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26829</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27418</t>
         </is>
       </c>
     </row>
@@ -6631,7 +6635,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>スティール・ボール・ラン ジョジョの奇妙な冒険 2nd &amp; 3rd STAGE</t>
+          <t>新テニスの王子様 U-17 WORLD CUP 決勝メンバー決定戦</t>
         </is>
       </c>
       <c r="E115" t="b">
@@ -6639,26 +6643,22 @@
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>配信</t>
+          <t>TVアニメ</t>
         </is>
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>1st STAGE：2026年3月19日（木）～ 2nd&amp;3rd STAGE：2026年9月25日（金）～ Netflixにて</t>
-        </is>
-      </c>
-      <c r="H115" t="inlineStr">
-        <is>
-          <t>david production</t>
-        </is>
-      </c>
+          <t>2026年秋</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr"/>
       <c r="I115" t="inlineStr"/>
       <c r="J115" t="inlineStr"/>
       <c r="K115" t="inlineStr"/>
       <c r="L115" t="inlineStr"/>
       <c r="M115" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25812</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26829</t>
         </is>
       </c>
     </row>
@@ -6676,7 +6676,7 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>生徒会にも穴はある！</t>
+          <t>スティール・ボール・ラン ジョジョの奇妙な冒険 2nd &amp; 3rd STAGE</t>
         </is>
       </c>
       <c r="E116" t="b">
@@ -6684,22 +6684,26 @@
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>TVアニメ</t>
+          <t>配信</t>
         </is>
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
-        </is>
-      </c>
-      <c r="H116" t="inlineStr"/>
+          <t>1st STAGE：2026年3月19日（木）～ 2nd&amp;3rd STAGE：2026年9月25日（金）～ Netflixにて</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>david production</t>
+        </is>
+      </c>
       <c r="I116" t="inlineStr"/>
       <c r="J116" t="inlineStr"/>
       <c r="K116" t="inlineStr"/>
       <c r="L116" t="inlineStr"/>
       <c r="M116" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25874</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25812</t>
         </is>
       </c>
     </row>
@@ -6717,7 +6721,7 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>世界最強の魔女、始めました</t>
+          <t>生徒会にも穴はある！</t>
         </is>
       </c>
       <c r="E117" t="b">
@@ -6733,18 +6737,14 @@
           <t>2026年10月～</t>
         </is>
       </c>
-      <c r="H117" t="inlineStr">
-        <is>
-          <t>ブリッジ</t>
-        </is>
-      </c>
+      <c r="H117" t="inlineStr"/>
       <c r="I117" t="inlineStr"/>
       <c r="J117" t="inlineStr"/>
       <c r="K117" t="inlineStr"/>
       <c r="L117" t="inlineStr"/>
       <c r="M117" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28288</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25874</t>
         </is>
       </c>
     </row>
@@ -6762,7 +6762,7 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>#ゾンビさがしてます</t>
+          <t>世界最強の魔女、始めました</t>
         </is>
       </c>
       <c r="E118" t="b">
@@ -6775,17 +6775,21 @@
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>2026年10月〜 テレビ朝日系にて</t>
-        </is>
-      </c>
-      <c r="H118" t="inlineStr"/>
+          <t>2026年10月～</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>ブリッジ</t>
+        </is>
+      </c>
       <c r="I118" t="inlineStr"/>
       <c r="J118" t="inlineStr"/>
       <c r="K118" t="inlineStr"/>
       <c r="L118" t="inlineStr"/>
       <c r="M118" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26825</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28288</t>
         </is>
       </c>
     </row>
@@ -6803,7 +6807,7 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>ダイヤのA actⅡ -Second Season- 第2クール</t>
+          <t>#ゾンビさがしてます</t>
         </is>
       </c>
       <c r="E119" t="b">
@@ -6816,37 +6820,17 @@
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>第1クール：2026年4月5日（日）～2026年6月28日（日） 第2クール：2026年10月～ テレビ東京ほか</t>
-        </is>
-      </c>
-      <c r="H119" t="inlineStr">
-        <is>
-          <t>OLM</t>
-        </is>
-      </c>
-      <c r="I119" t="inlineStr">
-        <is>
-          <t>Let's Go Crazy</t>
-        </is>
-      </c>
-      <c r="J119" t="inlineStr">
-        <is>
-          <t>Baby Canta</t>
-        </is>
-      </c>
-      <c r="K119" t="inlineStr">
-        <is>
-          <t>NUMBER</t>
-        </is>
-      </c>
-      <c r="L119" t="inlineStr">
-        <is>
-          <t>SUPER★DRAGON</t>
-        </is>
-      </c>
+          <t>2026年10月〜 テレビ朝日系にて</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr"/>
+      <c r="I119" t="inlineStr"/>
+      <c r="J119" t="inlineStr"/>
+      <c r="K119" t="inlineStr"/>
+      <c r="L119" t="inlineStr"/>
       <c r="M119" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=24072</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26825</t>
         </is>
       </c>
     </row>
@@ -6864,7 +6848,7 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>タヌキとキツネ</t>
+          <t>ダイヤのA actⅡ -Second Season- 第2クール</t>
         </is>
       </c>
       <c r="E120" t="b">
@@ -6877,17 +6861,37 @@
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
-        </is>
-      </c>
-      <c r="H120" t="inlineStr"/>
-      <c r="I120" t="inlineStr"/>
-      <c r="J120" t="inlineStr"/>
-      <c r="K120" t="inlineStr"/>
-      <c r="L120" t="inlineStr"/>
+          <t>第1クール：2026年4月5日（日）～2026年6月28日（日） 第2クール：2026年10月～ テレビ東京ほか</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>OLM</t>
+        </is>
+      </c>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>Let's Go Crazy</t>
+        </is>
+      </c>
+      <c r="J120" t="inlineStr">
+        <is>
+          <t>Baby Canta</t>
+        </is>
+      </c>
+      <c r="K120" t="inlineStr">
+        <is>
+          <t>NUMBER</t>
+        </is>
+      </c>
+      <c r="L120" t="inlineStr">
+        <is>
+          <t>SUPER★DRAGON</t>
+        </is>
+      </c>
       <c r="M120" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=6380</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=24072</t>
         </is>
       </c>
     </row>
@@ -6905,7 +6909,7 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>TANK CHAIR-戦車椅子-</t>
+          <t>タヌキとキツネ</t>
         </is>
       </c>
       <c r="E121" t="b">
@@ -6918,21 +6922,17 @@
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>2026年秋</t>
-        </is>
-      </c>
-      <c r="H121" t="inlineStr">
-        <is>
-          <t>ポリゴン・ピクチュアズ</t>
-        </is>
-      </c>
+          <t>2026年10月～</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr"/>
       <c r="I121" t="inlineStr"/>
       <c r="J121" t="inlineStr"/>
       <c r="K121" t="inlineStr"/>
       <c r="L121" t="inlineStr"/>
       <c r="M121" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27965</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=6380</t>
         </is>
       </c>
     </row>
@@ -6950,7 +6950,7 @@
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>探偵はもう、死んでいる。Season2</t>
+          <t>TANK CHAIR-戦車椅子-</t>
         </is>
       </c>
       <c r="E122" t="b">
@@ -6963,12 +6963,12 @@
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>2026年10月〜</t>
+          <t>2026年秋</t>
         </is>
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>ENGI</t>
+          <t>ポリゴン・ピクチュアズ</t>
         </is>
       </c>
       <c r="I122" t="inlineStr"/>
@@ -6977,7 +6977,7 @@
       <c r="L122" t="inlineStr"/>
       <c r="M122" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=16348</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27965</t>
         </is>
       </c>
     </row>
@@ -6995,7 +6995,7 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>千歳くんはラムネ瓶のなか 第2クール</t>
+          <t>探偵はもう、死んでいる。Season2</t>
         </is>
       </c>
       <c r="E123" t="b">
@@ -7008,37 +7008,21 @@
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t>第1クール：2025年10月7日（火）～ 2025年12月30日（火） AT-X・TOKYO MXほか 第2クール：2026年10月〜</t>
+          <t>2026年10月〜</t>
         </is>
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>feel.</t>
-        </is>
-      </c>
-      <c r="I123" t="inlineStr">
-        <is>
-          <t>ライアー</t>
-        </is>
-      </c>
-      <c r="J123" t="inlineStr">
-        <is>
-          <t>Kucci</t>
-        </is>
-      </c>
-      <c r="K123" t="inlineStr">
-        <is>
-          <t>陽炎</t>
-        </is>
-      </c>
-      <c r="L123" t="inlineStr">
-        <is>
-          <t>サイダーガール</t>
-        </is>
-      </c>
+          <t>ENGI</t>
+        </is>
+      </c>
+      <c r="I123" t="inlineStr"/>
+      <c r="J123" t="inlineStr"/>
+      <c r="K123" t="inlineStr"/>
+      <c r="L123" t="inlineStr"/>
       <c r="M123" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25058</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=16348</t>
         </is>
       </c>
     </row>
@@ -7056,7 +7040,7 @@
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>超巡！超条先輩</t>
+          <t>千歳くんはラムネ瓶のなか 第2クール</t>
         </is>
       </c>
       <c r="E124" t="b">
@@ -7069,21 +7053,37 @@
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>2026年10月～ カンテレ・フジテレビ系全国ネットにて</t>
+          <t>第1クール：2025年10月7日（火）～ 2025年12月30日（火） AT-X・TOKYO MXほか 第2クール：2026年10月〜</t>
         </is>
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>アルボアニメーション</t>
-        </is>
-      </c>
-      <c r="I124" t="inlineStr"/>
-      <c r="J124" t="inlineStr"/>
-      <c r="K124" t="inlineStr"/>
-      <c r="L124" t="inlineStr"/>
+          <t>feel.</t>
+        </is>
+      </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>ライアー</t>
+        </is>
+      </c>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>Kucci</t>
+        </is>
+      </c>
+      <c r="K124" t="inlineStr">
+        <is>
+          <t>陽炎</t>
+        </is>
+      </c>
+      <c r="L124" t="inlineStr">
+        <is>
+          <t>サイダーガール</t>
+        </is>
+      </c>
       <c r="M124" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26933</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25058</t>
         </is>
       </c>
     </row>
@@ -7101,7 +7101,7 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>追放されたチート付与魔術師は気ままなセカンドライフを謳歌する。</t>
+          <t>超巡！超条先輩</t>
         </is>
       </c>
       <c r="E125" t="b">
@@ -7114,12 +7114,12 @@
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>2026年10月～ テレ東系列にて</t>
+          <t>2026年10月～ カンテレ・フジテレビ系全国ネットにて</t>
         </is>
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>P.A.WORKS</t>
+          <t>アルボアニメーション</t>
         </is>
       </c>
       <c r="I125" t="inlineStr"/>
@@ -7128,7 +7128,7 @@
       <c r="L125" t="inlineStr"/>
       <c r="M125" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27631</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26933</t>
         </is>
       </c>
     </row>
@@ -7146,7 +7146,7 @@
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>てつりょー！meet with 鉄道むすめ</t>
+          <t>追放されたチート付与魔術師は気ままなセカンドライフを謳歌する。</t>
         </is>
       </c>
       <c r="E126" t="b">
@@ -7159,29 +7159,21 @@
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
+          <t>2026年10月～ テレ東系列にて</t>
         </is>
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>イーストフィッシュスタジオ</t>
+          <t>P.A.WORKS</t>
         </is>
       </c>
       <c r="I126" t="inlineStr"/>
       <c r="J126" t="inlineStr"/>
-      <c r="K126" t="inlineStr">
-        <is>
-          <t>わたし未来線</t>
-        </is>
-      </c>
-      <c r="L126" t="inlineStr">
-        <is>
-          <t>てつりょー会（橘めい・庄子真央・福嶋晴菜・月城日花）</t>
-        </is>
-      </c>
+      <c r="K126" t="inlineStr"/>
+      <c r="L126" t="inlineStr"/>
       <c r="M126" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26895</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27631</t>
         </is>
       </c>
     </row>
@@ -7199,7 +7191,7 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>テムパル～アイテムの力～</t>
+          <t>てつりょー！meet with 鉄道むすめ</t>
         </is>
       </c>
       <c r="E127" t="b">
@@ -7217,16 +7209,24 @@
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>J.C.STAFF</t>
+          <t>イーストフィッシュスタジオ</t>
         </is>
       </c>
       <c r="I127" t="inlineStr"/>
       <c r="J127" t="inlineStr"/>
-      <c r="K127" t="inlineStr"/>
-      <c r="L127" t="inlineStr"/>
+      <c r="K127" t="inlineStr">
+        <is>
+          <t>わたし未来線</t>
+        </is>
+      </c>
+      <c r="L127" t="inlineStr">
+        <is>
+          <t>てつりょー会（橘めい・庄子真央・福嶋晴菜・月城日花）</t>
+        </is>
+      </c>
       <c r="M127" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28478</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26895</t>
         </is>
       </c>
     </row>
@@ -7244,7 +7244,7 @@
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>デモンズ・クレスト</t>
+          <t>テムパル～アイテムの力～</t>
         </is>
       </c>
       <c r="E128" t="b">
@@ -7252,34 +7252,26 @@
       </c>
       <c r="F128" t="inlineStr">
         <is>
-          <t>配信</t>
+          <t>TVアニメ</t>
         </is>
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t>2026年11月6日（金） Prime Videoにて</t>
+          <t>2026年10月～</t>
         </is>
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>Production I.G</t>
-        </is>
-      </c>
-      <c r="I128" t="inlineStr">
-        <is>
-          <t>シンカ</t>
-        </is>
-      </c>
-      <c r="J128" t="inlineStr">
-        <is>
-          <t>Ado</t>
-        </is>
-      </c>
+          <t>J.C.STAFF</t>
+        </is>
+      </c>
+      <c r="I128" t="inlineStr"/>
+      <c r="J128" t="inlineStr"/>
       <c r="K128" t="inlineStr"/>
       <c r="L128" t="inlineStr"/>
       <c r="M128" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27189</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28478</t>
         </is>
       </c>
     </row>
@@ -7297,7 +7289,7 @@
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>転生貴族、鑑定スキルで成り上がる 第3期</t>
+          <t>デモンズ・クレスト</t>
         </is>
       </c>
       <c r="E129" t="b">
@@ -7305,26 +7297,34 @@
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>TVアニメ</t>
+          <t>配信</t>
         </is>
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>2026年秋 CBC/TBS系全国28局ネット「アガルアニメ」にて</t>
+          <t>2026年11月6日（金） Prime Videoにて</t>
         </is>
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>studio MOTHER</t>
-        </is>
-      </c>
-      <c r="I129" t="inlineStr"/>
-      <c r="J129" t="inlineStr"/>
+          <t>Production I.G</t>
+        </is>
+      </c>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>シンカ</t>
+        </is>
+      </c>
+      <c r="J129" t="inlineStr">
+        <is>
+          <t>Ado</t>
+        </is>
+      </c>
       <c r="K129" t="inlineStr"/>
       <c r="L129" t="inlineStr"/>
       <c r="M129" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25385</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27189</t>
         </is>
       </c>
     </row>
@@ -7342,7 +7342,7 @@
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>転生ゴブリンだけど質問ある？</t>
+          <t>転生貴族、鑑定スキルで成り上がる 第3期</t>
         </is>
       </c>
       <c r="E130" t="b">
@@ -7355,12 +7355,12 @@
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
+          <t>2026年秋 CBC/TBS系全国28局ネット「アガルアニメ」にて</t>
         </is>
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>BAKKKA</t>
+          <t>studio MOTHER</t>
         </is>
       </c>
       <c r="I130" t="inlineStr"/>
@@ -7369,7 +7369,7 @@
       <c r="L130" t="inlineStr"/>
       <c r="M130" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27909</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25385</t>
         </is>
       </c>
     </row>
@@ -7387,7 +7387,7 @@
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>転生した大聖女は、聖女であることをひた隠す</t>
+          <t>転生ゴブリンだけど質問ある？</t>
         </is>
       </c>
       <c r="E131" t="b">
@@ -7405,32 +7405,16 @@
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>FelixFilm</t>
-        </is>
-      </c>
-      <c r="I131" t="inlineStr">
-        <is>
-          <t>Flare of Soul</t>
-        </is>
-      </c>
-      <c r="J131" t="inlineStr">
-        <is>
-          <t>花耶</t>
-        </is>
-      </c>
-      <c r="K131" t="inlineStr">
-        <is>
-          <t>STELLAR</t>
-        </is>
-      </c>
-      <c r="L131" t="inlineStr">
-        <is>
-          <t>ウタヒメドリーム オールスターズ</t>
-        </is>
-      </c>
+          <t>BAKKKA</t>
+        </is>
+      </c>
+      <c r="I131" t="inlineStr"/>
+      <c r="J131" t="inlineStr"/>
+      <c r="K131" t="inlineStr"/>
+      <c r="L131" t="inlineStr"/>
       <c r="M131" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25630</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27909</t>
         </is>
       </c>
     </row>
@@ -7448,7 +7432,7 @@
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>転生したら剣でした 第2期</t>
+          <t>転生した大聖女は、聖女であることをひた隠す</t>
         </is>
       </c>
       <c r="E132" t="b">
@@ -7466,16 +7450,32 @@
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>C2C</t>
-        </is>
-      </c>
-      <c r="I132" t="inlineStr"/>
-      <c r="J132" t="inlineStr"/>
-      <c r="K132" t="inlineStr"/>
-      <c r="L132" t="inlineStr"/>
+          <t>FelixFilm</t>
+        </is>
+      </c>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>Flare of Soul</t>
+        </is>
+      </c>
+      <c r="J132" t="inlineStr">
+        <is>
+          <t>花耶</t>
+        </is>
+      </c>
+      <c r="K132" t="inlineStr">
+        <is>
+          <t>STELLAR</t>
+        </is>
+      </c>
+      <c r="L132" t="inlineStr">
+        <is>
+          <t>ウタヒメドリーム オールスターズ</t>
+        </is>
+      </c>
       <c r="M132" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=19149</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25630</t>
         </is>
       </c>
     </row>
@@ -7493,7 +7493,7 @@
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>とある暗部の少女共棲</t>
+          <t>転生したら剣でした 第2期</t>
         </is>
       </c>
       <c r="E133" t="b">
@@ -7506,37 +7506,21 @@
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>2026年10月9日（金）～ TOKYO MXほか</t>
+          <t>2026年10月～</t>
         </is>
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>J.C.STAFF</t>
-        </is>
-      </c>
-      <c r="I133" t="inlineStr">
-        <is>
-          <t>Ghost Sequence</t>
-        </is>
-      </c>
-      <c r="J133" t="inlineStr">
-        <is>
-          <t>East Of Eden</t>
-        </is>
-      </c>
-      <c r="K133" t="inlineStr">
-        <is>
-          <t>原子崩し(メルトダウナー)</t>
-        </is>
-      </c>
-      <c r="L133" t="inlineStr">
-        <is>
-          <t>岸田教団&amp;THE明星ロケッツ</t>
-        </is>
-      </c>
+          <t>C2C</t>
+        </is>
+      </c>
+      <c r="I133" t="inlineStr"/>
+      <c r="J133" t="inlineStr"/>
+      <c r="K133" t="inlineStr"/>
+      <c r="L133" t="inlineStr"/>
       <c r="M133" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25552</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=19149</t>
         </is>
       </c>
     </row>
@@ -7554,7 +7538,7 @@
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>東京リベンジャーズ 三天戦争編</t>
+          <t>とある暗部の少女共棲</t>
         </is>
       </c>
       <c r="E134" t="b">
@@ -7567,21 +7551,37 @@
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>2026年10月2日（金）～ MBS・TBS・CBC”アニメイズム”枠ほか</t>
+          <t>2026年10月9日（金）～ TOKYO MXほか</t>
         </is>
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>ライデンフィルム</t>
-        </is>
-      </c>
-      <c r="I134" t="inlineStr"/>
-      <c r="J134" t="inlineStr"/>
-      <c r="K134" t="inlineStr"/>
-      <c r="L134" t="inlineStr"/>
+          <t>J.C.STAFF</t>
+        </is>
+      </c>
+      <c r="I134" t="inlineStr">
+        <is>
+          <t>Ghost Sequence</t>
+        </is>
+      </c>
+      <c r="J134" t="inlineStr">
+        <is>
+          <t>East Of Eden</t>
+        </is>
+      </c>
+      <c r="K134" t="inlineStr">
+        <is>
+          <t>原子崩し(メルトダウナー)</t>
+        </is>
+      </c>
+      <c r="L134" t="inlineStr">
+        <is>
+          <t>岸田教団&amp;THE明星ロケッツ</t>
+        </is>
+      </c>
       <c r="M134" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=24207</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25552</t>
         </is>
       </c>
     </row>
@@ -7599,7 +7599,7 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>桃源暗鬼 ～日光・華厳の滝編～</t>
+          <t>東京リベンジャーズ 三天戦争編</t>
         </is>
       </c>
       <c r="E135" t="b">
@@ -7612,17 +7612,21 @@
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>2026年10月～ 日本テレビ系「FRIDAY ANIME NIGHT（フラアニ）」枠にて</t>
-        </is>
-      </c>
-      <c r="H135" t="inlineStr"/>
+          <t>2026年10月2日（金）～ MBS・TBS・CBC”アニメイズム”枠ほか</t>
+        </is>
+      </c>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>ライデンフィルム</t>
+        </is>
+      </c>
       <c r="I135" t="inlineStr"/>
       <c r="J135" t="inlineStr"/>
       <c r="K135" t="inlineStr"/>
       <c r="L135" t="inlineStr"/>
       <c r="M135" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27376</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=24207</t>
         </is>
       </c>
     </row>
@@ -7640,7 +7644,7 @@
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>どうも、好きな人に惚れ薬を依頼された魔女です。</t>
+          <t>桃源暗鬼 ～日光・華厳の滝編～</t>
         </is>
       </c>
       <c r="E136" t="b">
@@ -7653,21 +7657,17 @@
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
-        </is>
-      </c>
-      <c r="H136" t="inlineStr">
-        <is>
-          <t>ディオメディア</t>
-        </is>
-      </c>
+          <t>2026年10月～ 日本テレビ系「FRIDAY ANIME NIGHT（フラアニ）」枠にて</t>
+        </is>
+      </c>
+      <c r="H136" t="inlineStr"/>
       <c r="I136" t="inlineStr"/>
       <c r="J136" t="inlineStr"/>
       <c r="K136" t="inlineStr"/>
       <c r="L136" t="inlineStr"/>
       <c r="M136" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27581</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27376</t>
         </is>
       </c>
     </row>
@@ -7685,7 +7685,7 @@
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>ドラゴンボール超 ビルス</t>
+          <t>どうも、好きな人に惚れ薬を依頼された魔女です。</t>
         </is>
       </c>
       <c r="E137" t="b">
@@ -7698,17 +7698,21 @@
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>2026年秋 フジテレビにて</t>
-        </is>
-      </c>
-      <c r="H137" t="inlineStr"/>
+          <t>2026年10月～</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>ディオメディア</t>
+        </is>
+      </c>
       <c r="I137" t="inlineStr"/>
       <c r="J137" t="inlineStr"/>
       <c r="K137" t="inlineStr"/>
       <c r="L137" t="inlineStr"/>
       <c r="M137" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27491</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27581</t>
         </is>
       </c>
     </row>
@@ -7726,7 +7730,7 @@
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>鳴海の平日</t>
+          <t>ドラゴンボール超 ビルス</t>
         </is>
       </c>
       <c r="E138" t="b">
@@ -7734,26 +7738,22 @@
       </c>
       <c r="F138" t="inlineStr">
         <is>
-          <t>配信</t>
+          <t>TVアニメ</t>
         </is>
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t>2026年秋</t>
-        </is>
-      </c>
-      <c r="H138" t="inlineStr">
-        <is>
-          <t>Production I.G</t>
-        </is>
-      </c>
+          <t>2026年秋 フジテレビにて</t>
+        </is>
+      </c>
+      <c r="H138" t="inlineStr"/>
       <c r="I138" t="inlineStr"/>
       <c r="J138" t="inlineStr"/>
       <c r="K138" t="inlineStr"/>
       <c r="L138" t="inlineStr"/>
       <c r="M138" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28465</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27491</t>
         </is>
       </c>
     </row>
@@ -7771,7 +7771,7 @@
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>バーテックスフォース</t>
+          <t>鳴海の平日</t>
         </is>
       </c>
       <c r="E139" t="b">
@@ -7779,17 +7779,17 @@
       </c>
       <c r="F139" t="inlineStr">
         <is>
-          <t>TVアニメ</t>
+          <t>配信</t>
         </is>
       </c>
       <c r="G139" t="inlineStr">
         <is>
-          <t>2026年10月〜</t>
+          <t>2026年秋</t>
         </is>
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>SMDE</t>
+          <t>Production I.G</t>
         </is>
       </c>
       <c r="I139" t="inlineStr"/>
@@ -7798,7 +7798,7 @@
       <c r="L139" t="inlineStr"/>
       <c r="M139" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27988</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28465</t>
         </is>
       </c>
     </row>
@@ -7816,7 +7816,7 @@
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>Battle Spirits [Re] 絶界の空</t>
+          <t>バーテックスフォース</t>
         </is>
       </c>
       <c r="E140" t="b">
@@ -7829,17 +7829,21 @@
       </c>
       <c r="G140" t="inlineStr">
         <is>
-          <t>2026年秋</t>
-        </is>
-      </c>
-      <c r="H140" t="inlineStr"/>
+          <t>2026年10月〜</t>
+        </is>
+      </c>
+      <c r="H140" t="inlineStr">
+        <is>
+          <t>SMDE</t>
+        </is>
+      </c>
       <c r="I140" t="inlineStr"/>
       <c r="J140" t="inlineStr"/>
       <c r="K140" t="inlineStr"/>
       <c r="L140" t="inlineStr"/>
       <c r="M140" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27954</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27988</t>
         </is>
       </c>
     </row>
@@ -7857,7 +7861,7 @@
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>パンどろぼう</t>
+          <t>Battle Spirits [Re] 絶界の空</t>
         </is>
       </c>
       <c r="E141" t="b">
@@ -7870,7 +7874,7 @@
       </c>
       <c r="G141" t="inlineStr">
         <is>
-          <t>2026年10月〜 NHK Eテレにて</t>
+          <t>2026年秋</t>
         </is>
       </c>
       <c r="H141" t="inlineStr"/>
@@ -7880,7 +7884,7 @@
       <c r="L141" t="inlineStr"/>
       <c r="M141" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26163</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27954</t>
         </is>
       </c>
     </row>
@@ -7898,7 +7902,7 @@
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>百妖譜 京師篇</t>
+          <t>パンどろぼう</t>
         </is>
       </c>
       <c r="E142" t="b">
@@ -7911,7 +7915,7 @@
       </c>
       <c r="G142" t="inlineStr">
         <is>
-          <t>2026年10月〜 フジテレビ「B8station」にて</t>
+          <t>2026年10月〜 NHK Eテレにて</t>
         </is>
       </c>
       <c r="H142" t="inlineStr"/>
@@ -7921,7 +7925,7 @@
       <c r="L142" t="inlineStr"/>
       <c r="M142" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27781</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26163</t>
         </is>
       </c>
     </row>
@@ -7939,7 +7943,7 @@
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>冰剣の魔術師が世界を統べるⅡ</t>
+          <t>百妖譜 京師篇</t>
         </is>
       </c>
       <c r="E143" t="b">
@@ -7952,21 +7956,17 @@
       </c>
       <c r="G143" t="inlineStr">
         <is>
-          <t>2026年10月〜</t>
-        </is>
-      </c>
-      <c r="H143" t="inlineStr">
-        <is>
-          <t>ゼロジー</t>
-        </is>
-      </c>
+          <t>2026年10月〜 フジテレビ「B8station」にて</t>
+        </is>
+      </c>
+      <c r="H143" t="inlineStr"/>
       <c r="I143" t="inlineStr"/>
       <c r="J143" t="inlineStr"/>
       <c r="K143" t="inlineStr"/>
       <c r="L143" t="inlineStr"/>
       <c r="M143" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28403</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27781</t>
         </is>
       </c>
     </row>
@@ -7984,7 +7984,7 @@
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>ブラッククローバー 2nd Season</t>
+          <t>冰剣の魔術師が世界を統べるⅡ</t>
         </is>
       </c>
       <c r="E144" t="b">
@@ -7997,29 +7997,21 @@
       </c>
       <c r="G144" t="inlineStr">
         <is>
-          <t>2026年10月～ テレ東系列ほか</t>
+          <t>2026年10月〜</t>
         </is>
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>スタジオぴえろ</t>
-        </is>
-      </c>
-      <c r="I144" t="inlineStr">
-        <is>
-          <t>消えない理由</t>
-        </is>
-      </c>
-      <c r="J144" t="inlineStr">
-        <is>
-          <t>WANIMA</t>
-        </is>
-      </c>
+          <t>ゼロジー</t>
+        </is>
+      </c>
+      <c r="I144" t="inlineStr"/>
+      <c r="J144" t="inlineStr"/>
       <c r="K144" t="inlineStr"/>
       <c r="L144" t="inlineStr"/>
       <c r="M144" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26361</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28403</t>
         </is>
       </c>
     </row>
@@ -8037,7 +8029,7 @@
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>ホタルの嫁入り</t>
+          <t>ブラッククローバー 2nd Season</t>
         </is>
       </c>
       <c r="E145" t="b">
@@ -8050,21 +8042,29 @@
       </c>
       <c r="G145" t="inlineStr">
         <is>
-          <t>2026年10月～ 全国フジテレビ系“ ノイタミナ ”にて</t>
+          <t>2026年10月～ テレ東系列ほか</t>
         </is>
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>david production</t>
-        </is>
-      </c>
-      <c r="I145" t="inlineStr"/>
-      <c r="J145" t="inlineStr"/>
+          <t>スタジオぴえろ</t>
+        </is>
+      </c>
+      <c r="I145" t="inlineStr">
+        <is>
+          <t>消えない理由</t>
+        </is>
+      </c>
+      <c r="J145" t="inlineStr">
+        <is>
+          <t>WANIMA</t>
+        </is>
+      </c>
       <c r="K145" t="inlineStr"/>
       <c r="L145" t="inlineStr"/>
       <c r="M145" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27415</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26361</t>
         </is>
       </c>
     </row>
@@ -8082,7 +8082,7 @@
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>ポップパップポルターズ</t>
+          <t>ホタルの嫁入り</t>
         </is>
       </c>
       <c r="E146" t="b">
@@ -8095,12 +8095,12 @@
       </c>
       <c r="G146" t="inlineStr">
         <is>
-          <t>2026年10月～ テレビ朝日「PicoAniTime」にて</t>
+          <t>2026年10月～ 全国フジテレビ系“ ノイタミナ ”にて</t>
         </is>
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>MOZU STUDIOS</t>
+          <t>david production</t>
         </is>
       </c>
       <c r="I146" t="inlineStr"/>
@@ -8109,7 +8109,7 @@
       <c r="L146" t="inlineStr"/>
       <c r="M146" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=27823</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27415</t>
         </is>
       </c>
     </row>
@@ -8127,7 +8127,7 @@
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>ホテル・インヒューマンズ 第2期</t>
+          <t>ポップパップポルターズ</t>
         </is>
       </c>
       <c r="E147" t="b">
@@ -8140,12 +8140,12 @@
       </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t>2026年10月～ テレ東系列ほか</t>
+          <t>2026年10月～ テレビ朝日「PicoAniTime」にて</t>
         </is>
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>ブリッジ</t>
+          <t>MOZU STUDIOS</t>
         </is>
       </c>
       <c r="I147" t="inlineStr"/>
@@ -8154,7 +8154,7 @@
       <c r="L147" t="inlineStr"/>
       <c r="M147" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26870</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=27823</t>
         </is>
       </c>
     </row>
@@ -8172,7 +8172,7 @@
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>マジカル★エクスプローラー</t>
+          <t>ホテル・インヒューマンズ 第2期</t>
         </is>
       </c>
       <c r="E148" t="b">
@@ -8185,12 +8185,12 @@
       </c>
       <c r="G148" t="inlineStr">
         <is>
-          <t>2026年秋</t>
+          <t>2026年10月～ テレ東系列ほか</t>
         </is>
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>WHITE FOX</t>
+          <t>ブリッジ</t>
         </is>
       </c>
       <c r="I148" t="inlineStr"/>
@@ -8199,7 +8199,7 @@
       <c r="L148" t="inlineStr"/>
       <c r="M148" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=23375</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26870</t>
         </is>
       </c>
     </row>
@@ -8217,7 +8217,7 @@
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>魔法騎士レイアース</t>
+          <t>マジカル★エクスプローラー</t>
         </is>
       </c>
       <c r="E149" t="b">
@@ -8230,12 +8230,12 @@
       </c>
       <c r="G149" t="inlineStr">
         <is>
-          <t>2026年10月7日（水）～ テレビ朝日系列にて</t>
+          <t>2026年秋</t>
         </is>
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>E&amp;H production</t>
+          <t>WHITE FOX</t>
         </is>
       </c>
       <c r="I149" t="inlineStr"/>
@@ -8244,7 +8244,7 @@
       <c r="L149" t="inlineStr"/>
       <c r="M149" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=24301</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=23375</t>
         </is>
       </c>
     </row>
@@ -8262,7 +8262,7 @@
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>魔法少女育成計画restart</t>
+          <t>魔法騎士レイアース</t>
         </is>
       </c>
       <c r="E150" t="b">
@@ -8275,29 +8275,21 @@
       </c>
       <c r="G150" t="inlineStr">
         <is>
-          <t>2026年秋</t>
+          <t>2026年10月7日（水）～ テレビ朝日系列にて</t>
         </is>
       </c>
       <c r="H150" t="inlineStr">
         <is>
-          <t>SynergySP</t>
-        </is>
-      </c>
-      <c r="I150" t="inlineStr">
-        <is>
-          <t>No tears here</t>
-        </is>
-      </c>
-      <c r="J150" t="inlineStr">
-        <is>
-          <t>茅原実里</t>
-        </is>
-      </c>
+          <t>E&amp;H production</t>
+        </is>
+      </c>
+      <c r="I150" t="inlineStr"/>
+      <c r="J150" t="inlineStr"/>
       <c r="K150" t="inlineStr"/>
       <c r="L150" t="inlineStr"/>
       <c r="M150" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26693</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=24301</t>
         </is>
       </c>
     </row>
@@ -8315,7 +8307,7 @@
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>魔法の姉妹ルルットリリィ 第2クール</t>
+          <t>魔法少女育成計画restart</t>
         </is>
       </c>
       <c r="E151" t="b">
@@ -8328,37 +8320,29 @@
       </c>
       <c r="G151" t="inlineStr">
         <is>
-          <t>第1クール：2026年4月5日（日）～2026年6月21日（日） 第2クール：2026年10月～ TOKYO MX・ABCテレビほか</t>
+          <t>2026年秋</t>
         </is>
       </c>
       <c r="H151" t="inlineStr">
         <is>
-          <t>スタジオぴえろ</t>
+          <t>SynergySP</t>
         </is>
       </c>
       <c r="I151" t="inlineStr">
         <is>
-          <t>Bubee</t>
+          <t>No tears here</t>
         </is>
       </c>
       <c r="J151" t="inlineStr">
         <is>
-          <t>ILLIT</t>
-        </is>
-      </c>
-      <c r="K151" t="inlineStr">
-        <is>
-          <t>Calling</t>
-        </is>
-      </c>
-      <c r="L151" t="inlineStr">
-        <is>
-          <t>ルルットリリィ（こんぺとリリィ（CV.橘めい）、ましゅールル（CV.小鹿なお））</t>
-        </is>
-      </c>
+          <t>茅原実里</t>
+        </is>
+      </c>
+      <c r="K151" t="inlineStr"/>
+      <c r="L151" t="inlineStr"/>
       <c r="M151" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=24293</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26693</t>
         </is>
       </c>
     </row>
@@ -8376,7 +8360,7 @@
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>マロニエ王国の七人の騎士</t>
+          <t>魔法の姉妹ルルットリリィ 第2クール</t>
         </is>
       </c>
       <c r="E152" t="b">
@@ -8389,21 +8373,37 @@
       </c>
       <c r="G152" t="inlineStr">
         <is>
-          <t>2026年10月～ NHK Eテレにて</t>
+          <t>第1クール：2026年4月5日（日）～2026年6月21日（日） 第2クール：2026年10月～ TOKYO MX・ABCテレビほか</t>
         </is>
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>J.C.STAFF</t>
-        </is>
-      </c>
-      <c r="I152" t="inlineStr"/>
-      <c r="J152" t="inlineStr"/>
-      <c r="K152" t="inlineStr"/>
-      <c r="L152" t="inlineStr"/>
+          <t>スタジオぴえろ</t>
+        </is>
+      </c>
+      <c r="I152" t="inlineStr">
+        <is>
+          <t>Bubee</t>
+        </is>
+      </c>
+      <c r="J152" t="inlineStr">
+        <is>
+          <t>ILLIT</t>
+        </is>
+      </c>
+      <c r="K152" t="inlineStr">
+        <is>
+          <t>Calling</t>
+        </is>
+      </c>
+      <c r="L152" t="inlineStr">
+        <is>
+          <t>ルルットリリィ（こんぺとリリィ（CV.橘めい）、ましゅールル（CV.小鹿なお））</t>
+        </is>
+      </c>
       <c r="M152" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28456</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=24293</t>
         </is>
       </c>
     </row>
@@ -8421,7 +8421,7 @@
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>目覚めたら最強装備と宇宙船持ちだったので、一戸建て目指して傭兵として自由に生きたい</t>
+          <t>マロニエ王国の七人の騎士</t>
         </is>
       </c>
       <c r="E153" t="b">
@@ -8434,37 +8434,21 @@
       </c>
       <c r="G153" t="inlineStr">
         <is>
-          <t>2026年10月〜 TOKYO MX・読売テレビ・中京テレビほか</t>
+          <t>2026年10月～ NHK Eテレにて</t>
         </is>
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>studio A-CAT</t>
-        </is>
-      </c>
-      <c r="I153" t="inlineStr">
-        <is>
-          <t>UNSTOPPABLE</t>
-        </is>
-      </c>
-      <c r="J153" t="inlineStr">
-        <is>
-          <t>FLOW</t>
-        </is>
-      </c>
-      <c r="K153" t="inlineStr">
-        <is>
-          <t>MY WAY</t>
-        </is>
-      </c>
-      <c r="L153" t="inlineStr">
-        <is>
-          <t>ASTERISM</t>
-        </is>
-      </c>
+          <t>J.C.STAFF</t>
+        </is>
+      </c>
+      <c r="I153" t="inlineStr"/>
+      <c r="J153" t="inlineStr"/>
+      <c r="K153" t="inlineStr"/>
+      <c r="L153" t="inlineStr"/>
       <c r="M153" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25525</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28456</t>
         </is>
       </c>
     </row>
@@ -8482,7 +8466,7 @@
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>ゆるゆる図鑑</t>
+          <t>目覚めたら最強装備と宇宙船持ちだったので、一戸建て目指して傭兵として自由に生きたい</t>
         </is>
       </c>
       <c r="E154" t="b">
@@ -8495,17 +8479,37 @@
       </c>
       <c r="G154" t="inlineStr">
         <is>
-          <t>2026年10月～ テレ東系列6局ネット「アニもり！」内にて</t>
-        </is>
-      </c>
-      <c r="H154" t="inlineStr"/>
-      <c r="I154" t="inlineStr"/>
-      <c r="J154" t="inlineStr"/>
-      <c r="K154" t="inlineStr"/>
-      <c r="L154" t="inlineStr"/>
+          <t>2026年10月〜 TOKYO MX・読売テレビ・中京テレビほか</t>
+        </is>
+      </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>studio A-CAT</t>
+        </is>
+      </c>
+      <c r="I154" t="inlineStr">
+        <is>
+          <t>UNSTOPPABLE</t>
+        </is>
+      </c>
+      <c r="J154" t="inlineStr">
+        <is>
+          <t>FLOW</t>
+        </is>
+      </c>
+      <c r="K154" t="inlineStr">
+        <is>
+          <t>MY WAY</t>
+        </is>
+      </c>
+      <c r="L154" t="inlineStr">
+        <is>
+          <t>ASTERISM</t>
+        </is>
+      </c>
       <c r="M154" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28579</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25525</t>
         </is>
       </c>
     </row>
@@ -8523,7 +8527,7 @@
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>夜桜さんちの大作戦 第2期 第2クール</t>
+          <t>ゆるゆる図鑑</t>
         </is>
       </c>
       <c r="E155" t="b">
@@ -8536,37 +8540,21 @@
       </c>
       <c r="G155" t="inlineStr">
         <is>
-          <t>第1クール：2026年4月12日（日）～2026年6月28日（日） 第2クール：2026年10月〜 MBS／TBS系全国28局ネットにて</t>
+          <t>2026年10月～ テレ東系列6局ネット「アニもり！」内にて</t>
         </is>
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>SILVER LINK.</t>
-        </is>
-      </c>
-      <c r="I155" t="inlineStr">
-        <is>
-          <t>What's "KAZOKU"</t>
-        </is>
-      </c>
-      <c r="J155" t="inlineStr">
-        <is>
-          <t>櫻坂46</t>
-        </is>
-      </c>
-      <c r="K155" t="inlineStr">
-        <is>
-          <t>Shalala</t>
-        </is>
-      </c>
-      <c r="L155" t="inlineStr">
-        <is>
-          <t>ピラフ星人</t>
-        </is>
-      </c>
+          <t>Imagica Infos</t>
+        </is>
+      </c>
+      <c r="I155" t="inlineStr"/>
+      <c r="J155" t="inlineStr"/>
+      <c r="K155" t="inlineStr"/>
+      <c r="L155" t="inlineStr"/>
       <c r="M155" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=25032</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=28579</t>
         </is>
       </c>
     </row>
@@ -8584,7 +8572,7 @@
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>弱気MAX令嬢なのに、辣腕婚約者様の賭けに乗ってしまった</t>
+          <t>夜桜さんちの大作戦 第2期 第2クール</t>
         </is>
       </c>
       <c r="E156" t="b">
@@ -8597,21 +8585,37 @@
       </c>
       <c r="G156" t="inlineStr">
         <is>
-          <t>2026年10月～</t>
+          <t>第1クール：2026年4月12日（日）～2026年6月28日（日） 第2クール：2026年10月〜 MBS／TBS系全国28局ネットにて</t>
         </is>
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>寿門堂</t>
-        </is>
-      </c>
-      <c r="I156" t="inlineStr"/>
-      <c r="J156" t="inlineStr"/>
-      <c r="K156" t="inlineStr"/>
-      <c r="L156" t="inlineStr"/>
+          <t>SILVER LINK.</t>
+        </is>
+      </c>
+      <c r="I156" t="inlineStr">
+        <is>
+          <t>What's "KAZOKU"</t>
+        </is>
+      </c>
+      <c r="J156" t="inlineStr">
+        <is>
+          <t>櫻坂46</t>
+        </is>
+      </c>
+      <c r="K156" t="inlineStr">
+        <is>
+          <t>Shalala</t>
+        </is>
+      </c>
+      <c r="L156" t="inlineStr">
+        <is>
+          <t>ピラフ星人</t>
+        </is>
+      </c>
       <c r="M156" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=26947</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=25032</t>
         </is>
       </c>
     </row>
@@ -8629,11 +8633,11 @@
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>ラブライブ！虹ヶ咲学園スクールアイドル同好会 第2期</t>
+          <t>弱気MAX令嬢なのに、辣腕婚約者様の賭けに乗ってしまった</t>
         </is>
       </c>
       <c r="E157" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F157" t="inlineStr">
         <is>
@@ -8642,12 +8646,12 @@
       </c>
       <c r="G157" t="inlineStr">
         <is>
-          <t>2022年4月2日（土）～2022年6月25日（土） TOKYO MXほか 【再放送】 2026年9月30日（水）〜 BS日テレにて</t>
+          <t>2026年10月～</t>
         </is>
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>サンライズ</t>
+          <t>寿門堂</t>
         </is>
       </c>
       <c r="I157" t="inlineStr"/>
@@ -8656,7 +8660,7 @@
       <c r="L157" t="inlineStr"/>
       <c r="M157" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=14120</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=26947</t>
         </is>
       </c>
     </row>
@@ -8674,11 +8678,11 @@
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>らんま1/2 第3期</t>
+          <t>ラブライブ！虹ヶ咲学園スクールアイドル同好会 第2期</t>
         </is>
       </c>
       <c r="E158" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F158" t="inlineStr">
         <is>
@@ -8687,17 +8691,21 @@
       </c>
       <c r="G158" t="inlineStr">
         <is>
-          <t>2026年10月～ 日本テレビ系にて</t>
-        </is>
-      </c>
-      <c r="H158" t="inlineStr"/>
+          <t>2022年4月2日（土）～2022年6月25日（土） TOKYO MXほか 【再放送】 2026年9月30日（水）〜 BS日テレにて</t>
+        </is>
+      </c>
+      <c r="H158" t="inlineStr">
+        <is>
+          <t>サンライズ</t>
+        </is>
+      </c>
       <c r="I158" t="inlineStr"/>
       <c r="J158" t="inlineStr"/>
       <c r="K158" t="inlineStr"/>
       <c r="L158" t="inlineStr"/>
       <c r="M158" t="inlineStr">
         <is>
-          <t>https://www.animatetimes.com/tag/details.php?id=28013</t>
+          <t>https://www.animatetimes.com/tag/details.php?id=14120</t>
         </is>
       </c>
     </row>
@@ -8715,7 +8723,7 @@
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>LEGO® ONE PIECE</t>
+          <t>らんま1/2 第3期</t>
         </is>
       </c>
       <c r="E159" t="b">
@@ -8723,12 +8731,12 @@
       </c>
       <c r="F159" t="inlineStr">
         <is>
-          <t>配信</t>
+          <t>TVアニメ</t>
         </is>
       </c>
       <c r="G159" t="inlineStr">
         <is>
-          <t>2026年9月29日（火） Netflixにて</t>
+          <t>2026年10月～ 日本テレビ系にて</t>
         </is>
       </c>
       <c r="H159" t="inlineStr"/>
@@ -8737,6 +8745,47 @@
       <c r="K159" t="inlineStr"/>
       <c r="L159" t="inlineStr"/>
       <c r="M159" t="inlineStr">
+        <is>
+          <t>https://www.animatetimes.com/tag/details.php?id=28013</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C160" t="n">
+        <v>72</v>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>LEGO® ONE PIECE</t>
+        </is>
+      </c>
+      <c r="E160" t="b">
+        <v>0</v>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>配信</t>
+        </is>
+      </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>2026年9月29日（火） Netflixにて</t>
+        </is>
+      </c>
+      <c r="H160" t="inlineStr"/>
+      <c r="I160" t="inlineStr"/>
+      <c r="J160" t="inlineStr"/>
+      <c r="K160" t="inlineStr"/>
+      <c r="L160" t="inlineStr"/>
+      <c r="M160" t="inlineStr">
         <is>
           <t>https://www.animatetimes.com/tag/details.php?id=28168</t>
         </is>
@@ -9480,37 +9529,13 @@
           <t>汐れいら</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=6fUdDUk-FZQ</t>
-        </is>
-      </c>
-      <c r="J12" t="n">
-        <v>3706</v>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>アニプレックス チャンネル</t>
-        </is>
-      </c>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=6fUdDUk-FZQ</t>
-        </is>
-      </c>
-      <c r="M12" t="n">
-        <v>3706</v>
-      </c>
-      <c r="N12" t="inlineStr">
-        <is>
-          <t>アニプレックス チャンネル</t>
-        </is>
-      </c>
-      <c r="O12" t="inlineStr">
-        <is>
-          <t>2026-07-09T09:00:41</t>
-        </is>
-      </c>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -9677,19 +9702,29 @@
         </is>
       </c>
       <c r="J15" t="n">
-        <v>9108</v>
+        <v>170434</v>
       </c>
       <c r="K15" t="inlineStr">
         <is>
           <t>MARUMOCHI from HoneyWorks</t>
         </is>
       </c>
-      <c r="L15" t="inlineStr"/>
-      <c r="M15" t="inlineStr"/>
-      <c r="N15" t="inlineStr"/>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=waOUdRPozDY</t>
+        </is>
+      </c>
+      <c r="M15" t="n">
+        <v>10929</v>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>GOOD SMILE CHANNEL</t>
+        </is>
+      </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>2026-07-09T09:00:54</t>
+          <t>2026-07-17T09:00:31</t>
         </is>
       </c>
     </row>
@@ -9734,7 +9769,7 @@
         </is>
       </c>
       <c r="J16" t="n">
-        <v>14795</v>
+        <v>64180</v>
       </c>
       <c r="K16" t="inlineStr">
         <is>
@@ -9747,7 +9782,7 @@
         </is>
       </c>
       <c r="M16" t="n">
-        <v>14795</v>
+        <v>64180</v>
       </c>
       <c r="N16" t="inlineStr">
         <is>
@@ -9756,7 +9791,7 @@
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>2026-07-09T09:01:04</t>
+          <t>2026-07-17T09:00:40</t>
         </is>
       </c>
     </row>
@@ -9797,11 +9832,11 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=pU3P4At856Q</t>
+          <t>https://www.youtube.com/watch?v=0_xM9UeELDc</t>
         </is>
       </c>
       <c r="J17" t="n">
-        <v>7783</v>
+        <v>450371</v>
       </c>
       <c r="K17" t="inlineStr">
         <is>
@@ -9810,11 +9845,11 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=pU3P4At856Q</t>
+          <t>https://www.youtube.com/watch?v=0_xM9UeELDc</t>
         </is>
       </c>
       <c r="M17" t="n">
-        <v>7783</v>
+        <v>450371</v>
       </c>
       <c r="N17" t="inlineStr">
         <is>
@@ -9823,7 +9858,7 @@
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>2026-07-09T09:01:13</t>
+          <t>2026-07-17T09:00:50</t>
         </is>
       </c>
     </row>
@@ -10533,19 +10568,29 @@
         </is>
       </c>
       <c r="J29" t="n">
-        <v>38646</v>
+        <v>325501</v>
       </c>
       <c r="K29" t="inlineStr">
         <is>
           <t>ReoNa official YouTube channel</t>
         </is>
       </c>
-      <c r="L29" t="inlineStr"/>
-      <c r="M29" t="inlineStr"/>
-      <c r="N29" t="inlineStr"/>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=01Vgu7BIxmI</t>
+        </is>
+      </c>
+      <c r="M29" t="n">
+        <v>126318</v>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>2026-07-09T09:01:34</t>
+          <t>2026-07-17T09:01:02</t>
         </is>
       </c>
     </row>
@@ -11212,11 +11257,11 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=bYIT69zX8nE</t>
+          <t>https://www.youtube.com/watch?v=FhzaLI_Npg8</t>
         </is>
       </c>
       <c r="J40" t="n">
-        <v>503119</v>
+        <v>1336939</v>
       </c>
       <c r="K40" t="inlineStr">
         <is>
@@ -11229,7 +11274,7 @@
         </is>
       </c>
       <c r="M40" t="n">
-        <v>350764</v>
+        <v>1336939</v>
       </c>
       <c r="N40" t="inlineStr">
         <is>
@@ -11238,7 +11283,7 @@
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>2026-07-09T09:02:14</t>
+          <t>2026-07-17T09:01:21</t>
         </is>
       </c>
     </row>
@@ -15725,7 +15770,7 @@
         </is>
       </c>
       <c r="J113" t="n">
-        <v>219591</v>
+        <v>750794</v>
       </c>
       <c r="K113" t="inlineStr">
         <is>
@@ -15737,7 +15782,7 @@
       <c r="N113" t="inlineStr"/>
       <c r="O113" t="inlineStr">
         <is>
-          <t>2026-07-09T09:04:21</t>
+          <t>2026-07-17T09:02:42</t>
         </is>
       </c>
     </row>
@@ -16686,19 +16731,29 @@
         </is>
       </c>
       <c r="J130" t="n">
-        <v>10791</v>
+        <v>15823</v>
       </c>
       <c r="K130" t="inlineStr">
         <is>
           <t xml:space="preserve">Kaya Official YouTube Channel </t>
         </is>
       </c>
-      <c r="L130" t="inlineStr"/>
-      <c r="M130" t="inlineStr"/>
-      <c r="N130" t="inlineStr"/>
+      <c r="L130" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=TOj2RisiiwY</t>
+        </is>
+      </c>
+      <c r="M130" t="n">
+        <v>12311</v>
+      </c>
+      <c r="N130" t="inlineStr">
+        <is>
+          <t>【公式】アース・スター エンターテイメント</t>
+        </is>
+      </c>
       <c r="O130" t="inlineStr">
         <is>
-          <t>2026-07-09T09:05:08</t>
+          <t>2026-07-17T09:03:20</t>
         </is>
       </c>
     </row>
@@ -17005,13 +17060,37 @@
           <t>冨岡愛</t>
         </is>
       </c>
-      <c r="I135" t="inlineStr"/>
-      <c r="J135" t="inlineStr"/>
-      <c r="K135" t="inlineStr"/>
-      <c r="L135" t="inlineStr"/>
-      <c r="M135" t="inlineStr"/>
-      <c r="N135" t="inlineStr"/>
-      <c r="O135" t="inlineStr"/>
+      <c r="I135" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=00D8aV_cT6c</t>
+        </is>
+      </c>
+      <c r="J135" t="n">
+        <v>492</v>
+      </c>
+      <c r="K135" t="inlineStr">
+        <is>
+          <t>Project ANIMA チャンネル</t>
+        </is>
+      </c>
+      <c r="L135" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=00D8aV_cT6c</t>
+        </is>
+      </c>
+      <c r="M135" t="n">
+        <v>492</v>
+      </c>
+      <c r="N135" t="inlineStr">
+        <is>
+          <t>Project ANIMA チャンネル</t>
+        </is>
+      </c>
+      <c r="O135" t="inlineStr">
+        <is>
+          <t>2026-07-17T09:03:29</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="n">
@@ -18268,7 +18347,7 @@
         </is>
       </c>
       <c r="J156" t="n">
-        <v>1503</v>
+        <v>7403</v>
       </c>
       <c r="K156" t="inlineStr">
         <is>
@@ -18281,7 +18360,7 @@
         </is>
       </c>
       <c r="M156" t="n">
-        <v>1503</v>
+        <v>7403</v>
       </c>
       <c r="N156" t="inlineStr">
         <is>
@@ -18290,7 +18369,7 @@
       </c>
       <c r="O156" t="inlineStr">
         <is>
-          <t>2026-07-09T09:06:03</t>
+          <t>2026-07-17T09:03:50</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: anime list update (PC) 2026-07-18
</commit_message>
<xml_diff>
--- a/data/anime_list.xlsx
+++ b/data/anime_list.xlsx
@@ -9029,11 +9029,11 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=MGwURX7-Sas</t>
+          <t>https://www.youtube.com/watch?v=0BRjnQLg1nk</t>
         </is>
       </c>
       <c r="J4" t="n">
-        <v>3969358</v>
+        <v>600478</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -9045,7 +9045,7 @@
       <c r="N4" t="inlineStr"/>
       <c r="O4" t="inlineStr">
         <is>
-          <t>2026-07-10T09:00:44</t>
+          <t>2026-07-18T09:00:38</t>
         </is>
       </c>
     </row>
@@ -9631,33 +9631,33 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=_wL4-eA8JmU</t>
+          <t>https://www.youtube.com/watch?v=hFldDZZcrQo</t>
         </is>
       </c>
       <c r="J14" t="n">
-        <v>22799</v>
+        <v>67022</v>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>METANICK</t>
+          <t>GOOD SMILE CHANNEL</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=waOUdRPozDY</t>
+          <t>https://www.youtube.com/watch?v=wh36fOeXxqg</t>
         </is>
       </c>
       <c r="M14" t="n">
-        <v>1332</v>
+        <v>254165</v>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>GOOD SMILE CHANNEL</t>
+          <t>KADOKAWA Official Channel</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>2026-07-10T09:01:05</t>
+          <t>2026-07-18T09:01:01</t>
         </is>
       </c>
     </row>
@@ -10080,7 +10080,7 @@
         </is>
       </c>
       <c r="J21" t="n">
-        <v>6810695</v>
+        <v>6832555</v>
       </c>
       <c r="K21" t="inlineStr">
         <is>
@@ -10093,7 +10093,7 @@
         </is>
       </c>
       <c r="M21" t="n">
-        <v>73451</v>
+        <v>91671</v>
       </c>
       <c r="N21" t="inlineStr">
         <is>
@@ -10102,7 +10102,7 @@
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>2026-07-10T09:01:17</t>
+          <t>2026-07-18T09:01:14</t>
         </is>
       </c>
     </row>
@@ -10826,7 +10826,7 @@
         </is>
       </c>
       <c r="J33" t="n">
-        <v>1056</v>
+        <v>10735</v>
       </c>
       <c r="K33" t="inlineStr">
         <is>
@@ -10838,7 +10838,7 @@
       <c r="N33" t="inlineStr"/>
       <c r="O33" t="inlineStr">
         <is>
-          <t>2026-07-11T09:00:59</t>
+          <t>2026-07-18T09:01:42</t>
         </is>
       </c>
     </row>
@@ -11529,7 +11529,7 @@
         </is>
       </c>
       <c r="J44" t="n">
-        <v>7262</v>
+        <v>31702</v>
       </c>
       <c r="K44" t="inlineStr">
         <is>
@@ -11542,7 +11542,7 @@
         </is>
       </c>
       <c r="M44" t="n">
-        <v>7262</v>
+        <v>31702</v>
       </c>
       <c r="N44" t="inlineStr">
         <is>
@@ -11551,7 +11551,7 @@
       </c>
       <c r="O44" t="inlineStr">
         <is>
-          <t>2026-07-11T09:01:36</t>
+          <t>2026-07-18T09:02:00</t>
         </is>
       </c>
     </row>
@@ -12352,33 +12352,33 @@
       </c>
       <c r="I57" t="inlineStr">
         <is>
+          <t>https://www.youtube.com/watch?v=GnEgPPerpFc</t>
+        </is>
+      </c>
+      <c r="J57" t="n">
+        <v>51511</v>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>音羽-otoha-</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
           <t>https://www.youtube.com/watch?v=2SXzmgP26bk</t>
         </is>
       </c>
-      <c r="J57" t="n">
-        <v>2681</v>
-      </c>
-      <c r="K57" t="inlineStr">
+      <c r="M57" t="n">
+        <v>6837</v>
+      </c>
+      <c r="N57" t="inlineStr">
         <is>
           <t>【フジテレビ】アニメ公式チャンネル</t>
         </is>
       </c>
-      <c r="L57" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=2SXzmgP26bk</t>
-        </is>
-      </c>
-      <c r="M57" t="n">
-        <v>2681</v>
-      </c>
-      <c r="N57" t="inlineStr">
-        <is>
-          <t>【フジテレビ】アニメ公式チャンネル</t>
-        </is>
-      </c>
       <c r="O57" t="inlineStr">
         <is>
-          <t>2026-07-10T09:02:29</t>
+          <t>2026-07-18T09:02:15</t>
         </is>
       </c>
     </row>
@@ -12978,7 +12978,7 @@
         </is>
       </c>
       <c r="J67" t="n">
-        <v>96982</v>
+        <v>356566</v>
       </c>
       <c r="K67" t="inlineStr">
         <is>
@@ -12987,11 +12987,11 @@
       </c>
       <c r="L67" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=A6aH9jPW8ZY</t>
+          <t>https://www.youtube.com/watch?v=FlqDBh8QjZk</t>
         </is>
       </c>
       <c r="M67" t="n">
-        <v>289860</v>
+        <v>68342</v>
       </c>
       <c r="N67" t="inlineStr">
         <is>
@@ -13000,7 +13000,7 @@
       </c>
       <c r="O67" t="inlineStr">
         <is>
-          <t>2026-07-10T09:02:49</t>
+          <t>2026-07-18T09:02:25</t>
         </is>
       </c>
     </row>
@@ -13356,7 +13356,7 @@
         </is>
       </c>
       <c r="J73" t="n">
-        <v>100304</v>
+        <v>115779</v>
       </c>
       <c r="K73" t="inlineStr">
         <is>
@@ -13369,7 +13369,7 @@
         </is>
       </c>
       <c r="M73" t="n">
-        <v>100304</v>
+        <v>115779</v>
       </c>
       <c r="N73" t="inlineStr">
         <is>
@@ -13378,7 +13378,7 @@
       </c>
       <c r="O73" t="inlineStr">
         <is>
-          <t>2026-07-11T09:02:25</t>
+          <t>2026-07-18T09:02:37</t>
         </is>
       </c>
     </row>
@@ -13423,7 +13423,7 @@
         </is>
       </c>
       <c r="J74" t="n">
-        <v>131604</v>
+        <v>184427</v>
       </c>
       <c r="K74" t="inlineStr">
         <is>
@@ -13435,7 +13435,7 @@
       <c r="N74" t="inlineStr"/>
       <c r="O74" t="inlineStr">
         <is>
-          <t>2026-07-10T09:03:11</t>
+          <t>2026-07-18T09:02:47</t>
         </is>
       </c>
     </row>
@@ -13476,23 +13476,33 @@
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=j44OcUcmKCU</t>
+          <t>https://www.youtube.com/watch?v=wTQdf37-OBk</t>
         </is>
       </c>
       <c r="J75" t="n">
-        <v>47223</v>
+        <v>113128</v>
       </c>
       <c r="K75" t="inlineStr">
         <is>
-          <t>原因は自分にある。Official</t>
-        </is>
-      </c>
-      <c r="L75" t="inlineStr"/>
-      <c r="M75" t="inlineStr"/>
-      <c r="N75" t="inlineStr"/>
+          <t>NBCUniversal Anime/Music</t>
+        </is>
+      </c>
+      <c r="L75" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=wTQdf37-OBk</t>
+        </is>
+      </c>
+      <c r="M75" t="n">
+        <v>113128</v>
+      </c>
+      <c r="N75" t="inlineStr">
+        <is>
+          <t>NBCUniversal Anime/Music</t>
+        </is>
+      </c>
       <c r="O75" t="inlineStr">
         <is>
-          <t>2026-07-11T09:02:43</t>
+          <t>2026-07-18T09:02:56</t>
         </is>
       </c>
     </row>
@@ -13889,13 +13899,37 @@
           <t>清水美依紗</t>
         </is>
       </c>
-      <c r="I82" t="inlineStr"/>
-      <c r="J82" t="inlineStr"/>
-      <c r="K82" t="inlineStr"/>
-      <c r="L82" t="inlineStr"/>
-      <c r="M82" t="inlineStr"/>
-      <c r="N82" t="inlineStr"/>
-      <c r="O82" t="inlineStr"/>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=z0cYxw8Eifg</t>
+        </is>
+      </c>
+      <c r="J82" t="n">
+        <v>1958</v>
+      </c>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t>VAP Official</t>
+        </is>
+      </c>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=z0cYxw8Eifg</t>
+        </is>
+      </c>
+      <c r="M82" t="n">
+        <v>1958</v>
+      </c>
+      <c r="N82" t="inlineStr">
+        <is>
+          <t>VAP Official</t>
+        </is>
+      </c>
+      <c r="O82" t="inlineStr">
+        <is>
+          <t>2026-07-18T09:03:14</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -14068,33 +14102,33 @@
       </c>
       <c r="I85" t="inlineStr">
         <is>
+          <t>https://www.youtube.com/watch?v=TcMV9YeT9Sw</t>
+        </is>
+      </c>
+      <c r="J85" t="n">
+        <v>9108593</v>
+      </c>
+      <c r="K85" t="inlineStr">
+        <is>
+          <t>QWER</t>
+        </is>
+      </c>
+      <c r="L85" t="inlineStr">
+        <is>
           <t>https://www.youtube.com/watch?v=PVN8Pj_Ykyo</t>
         </is>
       </c>
-      <c r="J85" t="n">
-        <v>160213</v>
-      </c>
-      <c r="K85" t="inlineStr">
+      <c r="M85" t="n">
+        <v>181286</v>
+      </c>
+      <c r="N85" t="inlineStr">
         <is>
           <t>KADOKAWAanime</t>
         </is>
       </c>
-      <c r="L85" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=PVN8Pj_Ykyo</t>
-        </is>
-      </c>
-      <c r="M85" t="n">
-        <v>160213</v>
-      </c>
-      <c r="N85" t="inlineStr">
-        <is>
-          <t>KADOKAWAanime</t>
-        </is>
-      </c>
       <c r="O85" t="inlineStr">
         <is>
-          <t>2026-07-10T09:03:24</t>
+          <t>2026-07-18T09:03:24</t>
         </is>
       </c>
     </row>
@@ -14139,7 +14173,7 @@
         </is>
       </c>
       <c r="J86" t="n">
-        <v>160213</v>
+        <v>181286</v>
       </c>
       <c r="K86" t="inlineStr">
         <is>
@@ -14152,7 +14186,7 @@
         </is>
       </c>
       <c r="M86" t="n">
-        <v>160213</v>
+        <v>181286</v>
       </c>
       <c r="N86" t="inlineStr">
         <is>
@@ -14161,7 +14195,7 @@
       </c>
       <c r="O86" t="inlineStr">
         <is>
-          <t>2026-07-10T09:03:33</t>
+          <t>2026-07-18T09:03:33</t>
         </is>
       </c>
     </row>
@@ -14243,13 +14277,27 @@
           <t>櫻井優衣</t>
         </is>
       </c>
-      <c r="I88" t="inlineStr"/>
-      <c r="J88" t="inlineStr"/>
-      <c r="K88" t="inlineStr"/>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=_eUtav7vS38</t>
+        </is>
+      </c>
+      <c r="J88" t="n">
+        <v>48617</v>
+      </c>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>櫻井優衣 -SAKURAI YUI- (OFFICIAL)</t>
+        </is>
+      </c>
       <c r="L88" t="inlineStr"/>
       <c r="M88" t="inlineStr"/>
       <c r="N88" t="inlineStr"/>
-      <c r="O88" t="inlineStr"/>
+      <c r="O88" t="inlineStr">
+        <is>
+          <t>2026-07-18T09:04:00</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -14329,13 +14377,37 @@
           <t>中島健人</t>
         </is>
       </c>
-      <c r="I90" t="inlineStr"/>
-      <c r="J90" t="inlineStr"/>
-      <c r="K90" t="inlineStr"/>
-      <c r="L90" t="inlineStr"/>
-      <c r="M90" t="inlineStr"/>
-      <c r="N90" t="inlineStr"/>
-      <c r="O90" t="inlineStr"/>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=wp_4AThBtCA</t>
+        </is>
+      </c>
+      <c r="J90" t="n">
+        <v>61500</v>
+      </c>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>Kento Nakajima Official YouTube Channel</t>
+        </is>
+      </c>
+      <c r="L90" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=Dgj69Vqr120</t>
+        </is>
+      </c>
+      <c r="M90" t="n">
+        <v>52279</v>
+      </c>
+      <c r="N90" t="inlineStr">
+        <is>
+          <t>アニプレックス チャンネル</t>
+        </is>
+      </c>
+      <c r="O90" t="inlineStr">
+        <is>
+          <t>2026-07-18T09:04:15</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -14646,19 +14718,29 @@
         </is>
       </c>
       <c r="J95" t="n">
-        <v>2547</v>
+        <v>34408</v>
       </c>
       <c r="K95" t="inlineStr">
         <is>
           <t>shallm</t>
         </is>
       </c>
-      <c r="L95" t="inlineStr"/>
-      <c r="M95" t="inlineStr"/>
-      <c r="N95" t="inlineStr"/>
+      <c r="L95" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=CmP5HMtIOEY</t>
+        </is>
+      </c>
+      <c r="M95" t="n">
+        <v>4316</v>
+      </c>
+      <c r="N95" t="inlineStr">
+        <is>
+          <t>宝島社公式</t>
+        </is>
+      </c>
       <c r="O95" t="inlineStr">
         <is>
-          <t>2026-07-11T09:03:50</t>
+          <t>2026-07-18T09:04:24</t>
         </is>
       </c>
     </row>
@@ -15191,7 +15273,7 @@
         </is>
       </c>
       <c r="J104" t="n">
-        <v>916149</v>
+        <v>1346995</v>
       </c>
       <c r="K104" t="inlineStr">
         <is>
@@ -15204,7 +15286,7 @@
         </is>
       </c>
       <c r="M104" t="n">
-        <v>89187</v>
+        <v>386727</v>
       </c>
       <c r="N104" t="inlineStr">
         <is>
@@ -15213,7 +15295,7 @@
       </c>
       <c r="O104" t="inlineStr">
         <is>
-          <t>2026-07-10T09:04:36</t>
+          <t>2026-07-18T09:04:46</t>
         </is>
       </c>
     </row>
@@ -15258,7 +15340,7 @@
         </is>
       </c>
       <c r="J105" t="n">
-        <v>916149</v>
+        <v>1346995</v>
       </c>
       <c r="K105" t="inlineStr">
         <is>
@@ -15271,7 +15353,7 @@
         </is>
       </c>
       <c r="M105" t="n">
-        <v>89187</v>
+        <v>386727</v>
       </c>
       <c r="N105" t="inlineStr">
         <is>
@@ -15280,7 +15362,7 @@
       </c>
       <c r="O105" t="inlineStr">
         <is>
-          <t>2026-07-10T09:04:45</t>
+          <t>2026-07-18T09:04:55</t>
         </is>
       </c>
     </row>
@@ -15368,7 +15450,7 @@
         </is>
       </c>
       <c r="J107" t="n">
-        <v>495982</v>
+        <v>562336</v>
       </c>
       <c r="K107" t="inlineStr">
         <is>
@@ -15381,7 +15463,7 @@
         </is>
       </c>
       <c r="M107" t="n">
-        <v>495982</v>
+        <v>562336</v>
       </c>
       <c r="N107" t="inlineStr">
         <is>
@@ -15390,7 +15472,7 @@
       </c>
       <c r="O107" t="inlineStr">
         <is>
-          <t>2026-07-10T09:04:55</t>
+          <t>2026-07-18T09:05:07</t>
         </is>
       </c>
     </row>
@@ -15502,7 +15584,7 @@
         </is>
       </c>
       <c r="J109" t="n">
-        <v>17402</v>
+        <v>24509</v>
       </c>
       <c r="K109" t="inlineStr">
         <is>
@@ -15515,7 +15597,7 @@
         </is>
       </c>
       <c r="M109" t="n">
-        <v>10957</v>
+        <v>15643</v>
       </c>
       <c r="N109" t="inlineStr">
         <is>
@@ -15524,7 +15606,7 @@
       </c>
       <c r="O109" t="inlineStr">
         <is>
-          <t>2026-07-10T09:05:04</t>
+          <t>2026-07-18T09:05:16</t>
         </is>
       </c>
     </row>
@@ -15894,7 +15976,7 @@
         </is>
       </c>
       <c r="J115" t="n">
-        <v>266478</v>
+        <v>266997</v>
       </c>
       <c r="K115" t="inlineStr">
         <is>
@@ -15907,7 +15989,7 @@
         </is>
       </c>
       <c r="M115" t="n">
-        <v>16260</v>
+        <v>21316</v>
       </c>
       <c r="N115" t="inlineStr">
         <is>
@@ -15916,7 +15998,7 @@
       </c>
       <c r="O115" t="inlineStr">
         <is>
-          <t>2026-07-11T09:04:15</t>
+          <t>2026-07-18T09:05:26</t>
         </is>
       </c>
     </row>
@@ -16328,13 +16410,27 @@
           <t>The Canbellz</t>
         </is>
       </c>
-      <c r="I123" t="inlineStr"/>
-      <c r="J123" t="inlineStr"/>
-      <c r="K123" t="inlineStr"/>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=_EEMJOr1NLA</t>
+        </is>
+      </c>
+      <c r="J123" t="n">
+        <v>20179</v>
+      </c>
+      <c r="K123" t="inlineStr">
+        <is>
+          <t>神戸シンキ / The Canbellz</t>
+        </is>
+      </c>
       <c r="L123" t="inlineStr"/>
       <c r="M123" t="inlineStr"/>
       <c r="N123" t="inlineStr"/>
-      <c r="O123" t="inlineStr"/>
+      <c r="O123" t="inlineStr">
+        <is>
+          <t>2026-07-18T09:05:55</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="n">
@@ -17769,7 +17865,7 @@
         </is>
       </c>
       <c r="J146" t="n">
-        <v>13368</v>
+        <v>55063</v>
       </c>
       <c r="K146" t="inlineStr">
         <is>
@@ -17781,7 +17877,7 @@
       <c r="N146" t="inlineStr"/>
       <c r="O146" t="inlineStr">
         <is>
-          <t>2026-07-10T09:06:17</t>
+          <t>2026-07-18T09:06:30</t>
         </is>
       </c>
     </row>
@@ -18146,7 +18242,7 @@
         </is>
       </c>
       <c r="J153" t="n">
-        <v>60984</v>
+        <v>103834</v>
       </c>
       <c r="K153" t="inlineStr">
         <is>
@@ -18159,7 +18255,7 @@
         </is>
       </c>
       <c r="M153" t="n">
-        <v>60984</v>
+        <v>103834</v>
       </c>
       <c r="N153" t="inlineStr">
         <is>
@@ -18168,7 +18264,7 @@
       </c>
       <c r="O153" t="inlineStr">
         <is>
-          <t>2026-07-10T09:06:36</t>
+          <t>2026-07-18T09:06:42</t>
         </is>
       </c>
     </row>
@@ -18481,7 +18577,7 @@
         </is>
       </c>
       <c r="J158" t="n">
-        <v>261225</v>
+        <v>298375</v>
       </c>
       <c r="K158" t="inlineStr">
         <is>
@@ -18494,7 +18590,7 @@
         </is>
       </c>
       <c r="M158" t="n">
-        <v>261225</v>
+        <v>298375</v>
       </c>
       <c r="N158" t="inlineStr">
         <is>
@@ -18503,7 +18599,7 @@
       </c>
       <c r="O158" t="inlineStr">
         <is>
-          <t>2026-07-10T09:06:43</t>
+          <t>2026-07-18T09:06:52</t>
         </is>
       </c>
     </row>
@@ -19403,7 +19499,7 @@
         </is>
       </c>
       <c r="J176" t="n">
-        <v>290217</v>
+        <v>294655</v>
       </c>
       <c r="K176" t="inlineStr">
         <is>
@@ -19416,7 +19512,7 @@
         </is>
       </c>
       <c r="M176" t="n">
-        <v>290217</v>
+        <v>294655</v>
       </c>
       <c r="N176" t="inlineStr">
         <is>
@@ -19425,7 +19521,7 @@
       </c>
       <c r="O176" t="inlineStr">
         <is>
-          <t>2026-07-10T09:07:47</t>
+          <t>2026-07-18T09:08:01</t>
         </is>
       </c>
     </row>
@@ -19470,7 +19566,7 @@
         </is>
       </c>
       <c r="J177" t="n">
-        <v>290217</v>
+        <v>294656</v>
       </c>
       <c r="K177" t="inlineStr">
         <is>
@@ -19483,7 +19579,7 @@
         </is>
       </c>
       <c r="M177" t="n">
-        <v>290217</v>
+        <v>294656</v>
       </c>
       <c r="N177" t="inlineStr">
         <is>
@@ -19492,7 +19588,7 @@
       </c>
       <c r="O177" t="inlineStr">
         <is>
-          <t>2026-07-10T09:07:56</t>
+          <t>2026-07-18T09:08:11</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: anime list update (PC) 2026-07-21
</commit_message>
<xml_diff>
--- a/data/anime_list.xlsx
+++ b/data/anime_list.xlsx
@@ -8984,13 +8984,37 @@
           <t>橋本みゆき</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=0s8wRiSeKyg</t>
+        </is>
+      </c>
+      <c r="J3" t="n">
+        <v>5774</v>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>SHOCHIKU anime Channel</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=0s8wRiSeKyg</t>
+        </is>
+      </c>
+      <c r="M3" t="n">
+        <v>5774</v>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>SHOCHIKU anime Channel</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>2026-07-21T09:00:12</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -10769,7 +10793,7 @@
         </is>
       </c>
       <c r="J32" t="n">
-        <v>62831</v>
+        <v>84295</v>
       </c>
       <c r="K32" t="inlineStr">
         <is>
@@ -10781,7 +10805,7 @@
       <c r="N32" t="inlineStr"/>
       <c r="O32" t="inlineStr">
         <is>
-          <t>2026-07-12T09:00:45</t>
+          <t>2026-07-21T09:00:40</t>
         </is>
       </c>
     </row>
@@ -12116,13 +12140,27 @@
           <t>スキマスイッチ</t>
         </is>
       </c>
-      <c r="I53" t="inlineStr"/>
-      <c r="J53" t="inlineStr"/>
-      <c r="K53" t="inlineStr"/>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=xLU_wlNciSI</t>
+        </is>
+      </c>
+      <c r="J53" t="n">
+        <v>1041</v>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>【公式】石森プロ</t>
+        </is>
+      </c>
       <c r="L53" t="inlineStr"/>
       <c r="M53" t="inlineStr"/>
       <c r="N53" t="inlineStr"/>
-      <c r="O53" t="inlineStr"/>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>2026-07-21T09:01:04</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -12228,23 +12266,33 @@
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=H8BSBY59Dh0</t>
+          <t>https://www.youtube.com/watch?v=od3XN58Gnws</t>
         </is>
       </c>
       <c r="J55" t="n">
-        <v>1198</v>
+        <v>16719</v>
       </c>
       <c r="K55" t="inlineStr">
         <is>
-          <t>Hana Hope</t>
-        </is>
-      </c>
-      <c r="L55" t="inlineStr"/>
-      <c r="M55" t="inlineStr"/>
-      <c r="N55" t="inlineStr"/>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=od3XN58Gnws</t>
+        </is>
+      </c>
+      <c r="M55" t="n">
+        <v>16719</v>
+      </c>
+      <c r="N55" t="inlineStr">
+        <is>
+          <t>KADOKAWAanime</t>
+        </is>
+      </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>2026-07-13T09:01:34</t>
+          <t>2026-07-21T09:01:13</t>
         </is>
       </c>
     </row>
@@ -13541,13 +13589,37 @@
           <t>えむにみに</t>
         </is>
       </c>
-      <c r="I76" t="inlineStr"/>
-      <c r="J76" t="inlineStr"/>
-      <c r="K76" t="inlineStr"/>
-      <c r="L76" t="inlineStr"/>
-      <c r="M76" t="inlineStr"/>
-      <c r="N76" t="inlineStr"/>
-      <c r="O76" t="inlineStr"/>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=1tc784esysA</t>
+        </is>
+      </c>
+      <c r="J76" t="n">
+        <v>7476</v>
+      </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>NBCUniversal Anime/Music</t>
+        </is>
+      </c>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=1tc784esysA</t>
+        </is>
+      </c>
+      <c r="M76" t="n">
+        <v>7476</v>
+      </c>
+      <c r="N76" t="inlineStr">
+        <is>
+          <t>NBCUniversal Anime/Music</t>
+        </is>
+      </c>
+      <c r="O76" t="inlineStr">
+        <is>
+          <t>2026-07-21T09:01:25</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -13775,27 +13847,13 @@
           <t>harmoe</t>
         </is>
       </c>
-      <c r="I80" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=UTEjVKRw1Gs</t>
-        </is>
-      </c>
-      <c r="J80" t="n">
-        <v>4523</v>
-      </c>
-      <c r="K80" t="inlineStr">
-        <is>
-          <t>harmoeオフィシャルYouTubeチャンネル</t>
-        </is>
-      </c>
+      <c r="I80" t="inlineStr"/>
+      <c r="J80" t="inlineStr"/>
+      <c r="K80" t="inlineStr"/>
       <c r="L80" t="inlineStr"/>
       <c r="M80" t="inlineStr"/>
       <c r="N80" t="inlineStr"/>
-      <c r="O80" t="inlineStr">
-        <is>
-          <t>2026-07-12T09:02:10</t>
-        </is>
-      </c>
+      <c r="O80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -14647,33 +14705,33 @@
       </c>
       <c r="I94" t="inlineStr">
         <is>
+          <t>https://www.youtube.com/watch?v=k3NwKLjfEOw</t>
+        </is>
+      </c>
+      <c r="J94" t="n">
+        <v>178868</v>
+      </c>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>suis from Yorushika - Topic</t>
+        </is>
+      </c>
+      <c r="L94" t="inlineStr">
+        <is>
           <t>https://www.youtube.com/watch?v=ZH8xYK5vac0</t>
         </is>
       </c>
-      <c r="J94" t="n">
-        <v>72237</v>
-      </c>
-      <c r="K94" t="inlineStr">
+      <c r="M94" t="n">
+        <v>108510</v>
+      </c>
+      <c r="N94" t="inlineStr">
         <is>
           <t>宝島社公式</t>
         </is>
       </c>
-      <c r="L94" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=ZH8xYK5vac0</t>
-        </is>
-      </c>
-      <c r="M94" t="n">
-        <v>72237</v>
-      </c>
-      <c r="N94" t="inlineStr">
-        <is>
-          <t>宝島社公式</t>
-        </is>
-      </c>
       <c r="O94" t="inlineStr">
         <is>
-          <t>2026-07-12T09:02:53</t>
+          <t>2026-07-21T09:01:54</t>
         </is>
       </c>
     </row>
@@ -15139,7 +15197,7 @@
         </is>
       </c>
       <c r="J102" t="n">
-        <v>10238</v>
+        <v>36586</v>
       </c>
       <c r="K102" t="inlineStr">
         <is>
@@ -15152,7 +15210,7 @@
         </is>
       </c>
       <c r="M102" t="n">
-        <v>10238</v>
+        <v>36586</v>
       </c>
       <c r="N102" t="inlineStr">
         <is>
@@ -15161,7 +15219,7 @@
       </c>
       <c r="O102" t="inlineStr">
         <is>
-          <t>2026-07-13T09:02:41</t>
+          <t>2026-07-21T09:02:13</t>
         </is>
       </c>
     </row>
@@ -15909,7 +15967,7 @@
         </is>
       </c>
       <c r="J114" t="n">
-        <v>472908</v>
+        <v>501334</v>
       </c>
       <c r="K114" t="inlineStr">
         <is>
@@ -15922,7 +15980,7 @@
         </is>
       </c>
       <c r="M114" t="n">
-        <v>472908</v>
+        <v>501334</v>
       </c>
       <c r="N114" t="inlineStr">
         <is>
@@ -15931,7 +15989,7 @@
       </c>
       <c r="O114" t="inlineStr">
         <is>
-          <t>2026-07-12T09:03:19</t>
+          <t>2026-07-21T09:02:25</t>
         </is>
       </c>
     </row>
@@ -16306,7 +16364,7 @@
         </is>
       </c>
       <c r="J121" t="n">
-        <v>13869</v>
+        <v>17994</v>
       </c>
       <c r="K121" t="inlineStr">
         <is>
@@ -16319,7 +16377,7 @@
         </is>
       </c>
       <c r="M121" t="n">
-        <v>13869</v>
+        <v>17994</v>
       </c>
       <c r="N121" t="inlineStr">
         <is>
@@ -16328,7 +16386,7 @@
       </c>
       <c r="O121" t="inlineStr">
         <is>
-          <t>2026-07-12T09:03:41</t>
+          <t>2026-07-21T09:02:49</t>
         </is>
       </c>
     </row>
@@ -18004,23 +18062,33 @@
       </c>
       <c r="I149" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=ivJRaXk3GUw</t>
+          <t>https://www.youtube.com/watch?v=fCboU3XWuLU</t>
         </is>
       </c>
       <c r="J149" t="n">
-        <v>634</v>
+        <v>7627</v>
       </c>
       <c r="K149" t="inlineStr">
         <is>
-          <t>CROWN HEAD</t>
-        </is>
-      </c>
-      <c r="L149" t="inlineStr"/>
-      <c r="M149" t="inlineStr"/>
-      <c r="N149" t="inlineStr"/>
+          <t>NBCUniversal Anime/Music</t>
+        </is>
+      </c>
+      <c r="L149" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=fCboU3XWuLU</t>
+        </is>
+      </c>
+      <c r="M149" t="n">
+        <v>7627</v>
+      </c>
+      <c r="N149" t="inlineStr">
+        <is>
+          <t>NBCUniversal Anime/Music</t>
+        </is>
+      </c>
       <c r="O149" t="inlineStr">
         <is>
-          <t>2026-07-13T09:04:01</t>
+          <t>2026-07-21T09:03:18</t>
         </is>
       </c>
     </row>
@@ -18061,15 +18129,15 @@
       </c>
       <c r="I150" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=Wx9lV4C2ShU</t>
+          <t>https://www.youtube.com/watch?v=dhAKFhT6pno</t>
         </is>
       </c>
       <c r="J150" t="n">
-        <v>8320</v>
+        <v>55761</v>
       </c>
       <c r="K150" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kaya Official YouTube Channel </t>
+          <t>NBCUniversal Anime/Music</t>
         </is>
       </c>
       <c r="L150" t="inlineStr">
@@ -18078,7 +18146,7 @@
         </is>
       </c>
       <c r="M150" t="n">
-        <v>5403</v>
+        <v>55761</v>
       </c>
       <c r="N150" t="inlineStr">
         <is>
@@ -18087,7 +18155,7 @@
       </c>
       <c r="O150" t="inlineStr">
         <is>
-          <t>2026-07-12T09:04:43</t>
+          <t>2026-07-21T09:03:27</t>
         </is>
       </c>
     </row>
@@ -18175,7 +18243,7 @@
         </is>
       </c>
       <c r="J152" t="n">
-        <v>173757</v>
+        <v>186682</v>
       </c>
       <c r="K152" t="inlineStr">
         <is>
@@ -18188,7 +18256,7 @@
         </is>
       </c>
       <c r="M152" t="n">
-        <v>173757</v>
+        <v>186682</v>
       </c>
       <c r="N152" t="inlineStr">
         <is>
@@ -18197,7 +18265,7 @@
       </c>
       <c r="O152" t="inlineStr">
         <is>
-          <t>2026-07-12T09:04:54</t>
+          <t>2026-07-21T09:03:39</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: anime list update (PC) 2026-07-23
</commit_message>
<xml_diff>
--- a/data/anime_list.xlsx
+++ b/data/anime_list.xlsx
@@ -7636,8 +7636,16 @@
           <t>ライデンフィルム</t>
         </is>
       </c>
-      <c r="I135" t="inlineStr"/>
-      <c r="J135" t="inlineStr"/>
+      <c r="I135" t="inlineStr">
+        <is>
+          <t>IGNITE</t>
+        </is>
+      </c>
+      <c r="J135" t="inlineStr">
+        <is>
+          <t>JO1</t>
+        </is>
+      </c>
       <c r="K135" t="inlineStr"/>
       <c r="L135" t="inlineStr"/>
       <c r="M135" t="inlineStr">
@@ -8859,7 +8867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O184"/>
+  <dimension ref="A1:O185"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19441,7 +19449,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>ブラッククローバー 2nd Season</t>
+          <t>東京リベンジャーズ 三天戦争編</t>
         </is>
       </c>
       <c r="D177" t="b">
@@ -19457,45 +19465,21 @@
       </c>
       <c r="G177" t="inlineStr">
         <is>
-          <t>消えない理由</t>
+          <t>IGNITE</t>
         </is>
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>WANIMA</t>
-        </is>
-      </c>
-      <c r="I177" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=1BWy13nlY1A</t>
-        </is>
-      </c>
-      <c r="J177" t="n">
-        <v>2587</v>
-      </c>
-      <c r="K177" t="inlineStr">
-        <is>
-          <t>Anime Trailer アニメ</t>
-        </is>
-      </c>
-      <c r="L177" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=1BWy13nlY1A</t>
-        </is>
-      </c>
-      <c r="M177" t="n">
-        <v>2587</v>
-      </c>
-      <c r="N177" t="inlineStr">
-        <is>
-          <t>Anime Trailer アニメ</t>
-        </is>
-      </c>
-      <c r="O177" t="inlineStr">
-        <is>
-          <t>2026-07-22T09:17:34</t>
-        </is>
-      </c>
+          <t>JO1</t>
+        </is>
+      </c>
+      <c r="I177" t="inlineStr"/>
+      <c r="J177" t="inlineStr"/>
+      <c r="K177" t="inlineStr"/>
+      <c r="L177" t="inlineStr"/>
+      <c r="M177" t="inlineStr"/>
+      <c r="N177" t="inlineStr"/>
+      <c r="O177" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" t="n">
@@ -19508,7 +19492,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>魔法少女育成計画restart</t>
+          <t>ブラッククローバー 2nd Season</t>
         </is>
       </c>
       <c r="D178" t="b">
@@ -19524,33 +19508,43 @@
       </c>
       <c r="G178" t="inlineStr">
         <is>
-          <t>No tears here</t>
+          <t>消えない理由</t>
         </is>
       </c>
       <c r="H178" t="inlineStr">
         <is>
-          <t>茅原実里</t>
+          <t>WANIMA</t>
         </is>
       </c>
       <c r="I178" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=-PX7FqZ55tE</t>
+          <t>https://www.youtube.com/watch?v=1BWy13nlY1A</t>
         </is>
       </c>
       <c r="J178" t="n">
-        <v>106403</v>
+        <v>2587</v>
       </c>
       <c r="K178" t="inlineStr">
         <is>
-          <t>TVアニメ「魔法少女育成計画restart」公式チャンネル</t>
-        </is>
-      </c>
-      <c r="L178" t="inlineStr"/>
-      <c r="M178" t="inlineStr"/>
-      <c r="N178" t="inlineStr"/>
+          <t>Anime Trailer アニメ</t>
+        </is>
+      </c>
+      <c r="L178" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=1BWy13nlY1A</t>
+        </is>
+      </c>
+      <c r="M178" t="n">
+        <v>2587</v>
+      </c>
+      <c r="N178" t="inlineStr">
+        <is>
+          <t>Anime Trailer アニメ</t>
+        </is>
+      </c>
       <c r="O178" t="inlineStr">
         <is>
-          <t>2026-07-22T09:17:48</t>
+          <t>2026-07-22T09:17:34</t>
         </is>
       </c>
     </row>
@@ -19565,7 +19559,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>魔法の姉妹ルルットリリィ 第2クール</t>
+          <t>魔法少女育成計画restart</t>
         </is>
       </c>
       <c r="D179" t="b">
@@ -19581,43 +19575,33 @@
       </c>
       <c r="G179" t="inlineStr">
         <is>
-          <t>Bubee</t>
+          <t>No tears here</t>
         </is>
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>ILLIT</t>
+          <t>茅原実里</t>
         </is>
       </c>
       <c r="I179" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
+          <t>https://www.youtube.com/watch?v=-PX7FqZ55tE</t>
         </is>
       </c>
       <c r="J179" t="n">
-        <v>294655</v>
+        <v>106403</v>
       </c>
       <c r="K179" t="inlineStr">
         <is>
-          <t>Bandai Namco Filmworks Channel</t>
-        </is>
-      </c>
-      <c r="L179" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
-        </is>
-      </c>
-      <c r="M179" t="n">
-        <v>294655</v>
-      </c>
-      <c r="N179" t="inlineStr">
-        <is>
-          <t>Bandai Namco Filmworks Channel</t>
-        </is>
-      </c>
+          <t>TVアニメ「魔法少女育成計画restart」公式チャンネル</t>
+        </is>
+      </c>
+      <c r="L179" t="inlineStr"/>
+      <c r="M179" t="inlineStr"/>
+      <c r="N179" t="inlineStr"/>
       <c r="O179" t="inlineStr">
         <is>
-          <t>2026-07-18T09:08:01</t>
+          <t>2026-07-22T09:17:48</t>
         </is>
       </c>
     </row>
@@ -19640,7 +19624,7 @@
       </c>
       <c r="E180" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F180" t="n">
@@ -19648,12 +19632,12 @@
       </c>
       <c r="G180" t="inlineStr">
         <is>
-          <t>Calling</t>
+          <t>Bubee</t>
         </is>
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>ルルットリリィ（こんぺとリリィ（CV.橘めい）、ましゅールル（CV.小鹿なお））</t>
+          <t>ILLIT</t>
         </is>
       </c>
       <c r="I180" t="inlineStr">
@@ -19662,7 +19646,7 @@
         </is>
       </c>
       <c r="J180" t="n">
-        <v>294656</v>
+        <v>294655</v>
       </c>
       <c r="K180" t="inlineStr">
         <is>
@@ -19675,7 +19659,7 @@
         </is>
       </c>
       <c r="M180" t="n">
-        <v>294656</v>
+        <v>294655</v>
       </c>
       <c r="N180" t="inlineStr">
         <is>
@@ -19684,7 +19668,7 @@
       </c>
       <c r="O180" t="inlineStr">
         <is>
-          <t>2026-07-18T09:08:11</t>
+          <t>2026-07-18T09:08:01</t>
         </is>
       </c>
     </row>
@@ -19699,7 +19683,7 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>目覚めたら最強装備と宇宙船持ちだったので、一戸建て目指して傭兵として自由に生きたい</t>
+          <t>魔法の姉妹ルルットリリィ 第2クール</t>
         </is>
       </c>
       <c r="D181" t="b">
@@ -19707,7 +19691,7 @@
       </c>
       <c r="E181" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F181" t="n">
@@ -19715,21 +19699,45 @@
       </c>
       <c r="G181" t="inlineStr">
         <is>
-          <t>UNSTOPPABLE</t>
+          <t>Calling</t>
         </is>
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>FLOW</t>
-        </is>
-      </c>
-      <c r="I181" t="inlineStr"/>
-      <c r="J181" t="inlineStr"/>
-      <c r="K181" t="inlineStr"/>
-      <c r="L181" t="inlineStr"/>
-      <c r="M181" t="inlineStr"/>
-      <c r="N181" t="inlineStr"/>
-      <c r="O181" t="inlineStr"/>
+          <t>ルルットリリィ（こんぺとリリィ（CV.橘めい）、ましゅールル（CV.小鹿なお））</t>
+        </is>
+      </c>
+      <c r="I181" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
+        </is>
+      </c>
+      <c r="J181" t="n">
+        <v>294656</v>
+      </c>
+      <c r="K181" t="inlineStr">
+        <is>
+          <t>Bandai Namco Filmworks Channel</t>
+        </is>
+      </c>
+      <c r="L181" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=803SES0YVcM</t>
+        </is>
+      </c>
+      <c r="M181" t="n">
+        <v>294656</v>
+      </c>
+      <c r="N181" t="inlineStr">
+        <is>
+          <t>Bandai Namco Filmworks Channel</t>
+        </is>
+      </c>
+      <c r="O181" t="inlineStr">
+        <is>
+          <t>2026-07-18T09:08:11</t>
+        </is>
+      </c>
     </row>
     <row r="182">
       <c r="A182" t="n">
@@ -19750,7 +19758,7 @@
       </c>
       <c r="E182" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F182" t="n">
@@ -19758,12 +19766,12 @@
       </c>
       <c r="G182" t="inlineStr">
         <is>
-          <t>MY WAY</t>
+          <t>UNSTOPPABLE</t>
         </is>
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>ASTERISM</t>
+          <t>FLOW</t>
         </is>
       </c>
       <c r="I182" t="inlineStr"/>
@@ -19785,7 +19793,7 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>夜桜さんちの大作戦 第2期 第2クール</t>
+          <t>目覚めたら最強装備と宇宙船持ちだったので、一戸建て目指して傭兵として自由に生きたい</t>
         </is>
       </c>
       <c r="D183" t="b">
@@ -19793,7 +19801,7 @@
       </c>
       <c r="E183" t="inlineStr">
         <is>
-          <t>OP</t>
+          <t>ED</t>
         </is>
       </c>
       <c r="F183" t="n">
@@ -19801,45 +19809,21 @@
       </c>
       <c r="G183" t="inlineStr">
         <is>
-          <t>What's "KAZOKU"</t>
+          <t>MY WAY</t>
         </is>
       </c>
       <c r="H183" t="inlineStr">
         <is>
-          <t>櫻坂46</t>
-        </is>
-      </c>
-      <c r="I183" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=4SdeuouXcWI</t>
-        </is>
-      </c>
-      <c r="J183" t="n">
-        <v>776489</v>
-      </c>
-      <c r="K183" t="inlineStr">
-        <is>
-          <t>櫻坂46 OFFICIAL YouTube CHANNEL</t>
-        </is>
-      </c>
-      <c r="L183" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=AIspds2UVts</t>
-        </is>
-      </c>
-      <c r="M183" t="n">
-        <v>367020</v>
-      </c>
-      <c r="N183" t="inlineStr">
-        <is>
-          <t>NBCUniversal Anime/Music</t>
-        </is>
-      </c>
-      <c r="O183" t="inlineStr">
-        <is>
-          <t>2026-07-22T09:18:09</t>
-        </is>
-      </c>
+          <t>ASTERISM</t>
+        </is>
+      </c>
+      <c r="I183" t="inlineStr"/>
+      <c r="J183" t="inlineStr"/>
+      <c r="K183" t="inlineStr"/>
+      <c r="L183" t="inlineStr"/>
+      <c r="M183" t="inlineStr"/>
+      <c r="N183" t="inlineStr"/>
+      <c r="O183" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" t="n">
@@ -19860,7 +19844,7 @@
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>ED</t>
+          <t>OP</t>
         </is>
       </c>
       <c r="F184" t="n">
@@ -19868,41 +19852,108 @@
       </c>
       <c r="G184" t="inlineStr">
         <is>
+          <t>What's "KAZOKU"</t>
+        </is>
+      </c>
+      <c r="H184" t="inlineStr">
+        <is>
+          <t>櫻坂46</t>
+        </is>
+      </c>
+      <c r="I184" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=4SdeuouXcWI</t>
+        </is>
+      </c>
+      <c r="J184" t="n">
+        <v>776489</v>
+      </c>
+      <c r="K184" t="inlineStr">
+        <is>
+          <t>櫻坂46 OFFICIAL YouTube CHANNEL</t>
+        </is>
+      </c>
+      <c r="L184" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=AIspds2UVts</t>
+        </is>
+      </c>
+      <c r="M184" t="n">
+        <v>367020</v>
+      </c>
+      <c r="N184" t="inlineStr">
+        <is>
+          <t>NBCUniversal Anime/Music</t>
+        </is>
+      </c>
+      <c r="O184" t="inlineStr">
+        <is>
+          <t>2026-07-22T09:18:09</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="n">
+        <v>5947</v>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>2026秋アニメ</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>夜桜さんちの大作戦 第2期 第2クール</t>
+        </is>
+      </c>
+      <c r="D185" t="b">
+        <v>0</v>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>ED</t>
+        </is>
+      </c>
+      <c r="F185" t="n">
+        <v>1</v>
+      </c>
+      <c r="G185" t="inlineStr">
+        <is>
           <t>Shalala</t>
         </is>
       </c>
-      <c r="H184" t="inlineStr">
+      <c r="H185" t="inlineStr">
         <is>
           <t>ピラフ星人</t>
         </is>
       </c>
-      <c r="I184" t="inlineStr">
+      <c r="I185" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=X6fNe1uPs9E</t>
         </is>
       </c>
-      <c r="J184" t="n">
+      <c r="J185" t="n">
         <v>384697</v>
       </c>
-      <c r="K184" t="inlineStr">
+      <c r="K185" t="inlineStr">
         <is>
           <t>NBCUniversal Anime/Music</t>
         </is>
       </c>
-      <c r="L184" t="inlineStr">
+      <c r="L185" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=X6fNe1uPs9E</t>
         </is>
       </c>
-      <c r="M184" t="n">
+      <c r="M185" t="n">
         <v>384697</v>
       </c>
-      <c r="N184" t="inlineStr">
+      <c r="N185" t="inlineStr">
         <is>
           <t>NBCUniversal Anime/Music</t>
         </is>
       </c>
-      <c r="O184" t="inlineStr">
+      <c r="O185" t="inlineStr">
         <is>
           <t>2026-07-22T09:18:19</t>
         </is>

</xml_diff>

<commit_message>
auto: anime list update (PC) 2026-07-24
</commit_message>
<xml_diff>
--- a/data/anime_list.xlsx
+++ b/data/anime_list.xlsx
@@ -11077,7 +11077,7 @@
         </is>
       </c>
       <c r="J37" t="n">
-        <v>6984</v>
+        <v>50264</v>
       </c>
       <c r="K37" t="inlineStr">
         <is>
@@ -11090,7 +11090,7 @@
         </is>
       </c>
       <c r="M37" t="n">
-        <v>6984</v>
+        <v>50264</v>
       </c>
       <c r="N37" t="inlineStr">
         <is>
@@ -11099,7 +11099,7 @@
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>2026-07-16T09:01:01</t>
+          <t>2026-07-24T09:00:42</t>
         </is>
       </c>
     </row>
@@ -11140,33 +11140,33 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
+          <t>https://www.youtube.com/watch?v=9hrlfMldegI</t>
+        </is>
+      </c>
+      <c r="J38" t="n">
+        <v>228049</v>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>MYTH &amp; ROID Official Channel</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
           <t>https://www.youtube.com/watch?v=Tbyi0Tx1QLA</t>
         </is>
       </c>
-      <c r="J38" t="n">
-        <v>5191</v>
-      </c>
-      <c r="K38" t="inlineStr">
+      <c r="M38" t="n">
+        <v>21447</v>
+      </c>
+      <c r="N38" t="inlineStr">
         <is>
           <t>KADOKAWAanime</t>
         </is>
       </c>
-      <c r="L38" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=Tbyi0Tx1QLA</t>
-        </is>
-      </c>
-      <c r="M38" t="n">
-        <v>5191</v>
-      </c>
-      <c r="N38" t="inlineStr">
-        <is>
-          <t>KADOKAWAanime</t>
-        </is>
-      </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>2026-07-16T09:01:09</t>
+          <t>2026-07-24T09:00:51</t>
         </is>
       </c>
     </row>
@@ -17442,7 +17442,7 @@
         </is>
       </c>
       <c r="J140" t="n">
-        <v>43946</v>
+        <v>334778</v>
       </c>
       <c r="K140" t="inlineStr">
         <is>
@@ -17455,7 +17455,7 @@
         </is>
       </c>
       <c r="M140" t="n">
-        <v>43946</v>
+        <v>334778</v>
       </c>
       <c r="N140" t="inlineStr">
         <is>
@@ -17464,7 +17464,7 @@
       </c>
       <c r="O140" t="inlineStr">
         <is>
-          <t>2026-07-16T09:03:08</t>
+          <t>2026-07-24T09:02:09</t>
         </is>
       </c>
     </row>
@@ -17505,33 +17505,33 @@
       </c>
       <c r="I141" t="inlineStr">
         <is>
+          <t>https://www.youtube.com/watch?v=_werYjm5BmY</t>
+        </is>
+      </c>
+      <c r="J141" t="n">
+        <v>11469371</v>
+      </c>
+      <c r="K141" t="inlineStr">
+        <is>
+          <t>ターニャ・デグレチャフ（CV：悠木碧） - Topic</t>
+        </is>
+      </c>
+      <c r="L141" t="inlineStr">
+        <is>
           <t>https://www.youtube.com/watch?v=x2k_iYCGKvE</t>
         </is>
       </c>
-      <c r="J141" t="n">
-        <v>24116</v>
-      </c>
-      <c r="K141" t="inlineStr">
+      <c r="M141" t="n">
+        <v>107568</v>
+      </c>
+      <c r="N141" t="inlineStr">
         <is>
           <t>KADOKAWAanime</t>
         </is>
       </c>
-      <c r="L141" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=x2k_iYCGKvE</t>
-        </is>
-      </c>
-      <c r="M141" t="n">
-        <v>24116</v>
-      </c>
-      <c r="N141" t="inlineStr">
-        <is>
-          <t>KADOKAWAanime</t>
-        </is>
-      </c>
       <c r="O141" t="inlineStr">
         <is>
-          <t>2026-07-16T09:03:17</t>
+          <t>2026-07-24T09:02:18</t>
         </is>
       </c>
     </row>

</xml_diff>